<commit_message>
Simplify Demographic Measure Descriptors to 999
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG100"/>
+  <dimension ref="A1:AZ100"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -1990,13 +1990,13 @@
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AB12" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="AC12" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
@@ -2134,13 +2134,13 @@
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AB13" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="AC13" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
@@ -2841,13 +2841,13 @@
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="AB19" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AC19" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AD19" t="inlineStr">
         <is>
@@ -2982,13 +2982,13 @@
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="AB20" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AC20" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AD20" t="inlineStr">
         <is>
@@ -3123,13 +3123,13 @@
         </is>
       </c>
       <c r="AA21" t="n">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="AB21" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AC21" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AD21" t="inlineStr">
         <is>
@@ -3264,13 +3264,13 @@
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="AB22" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AC22" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AD22" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Standardize Excel injection and enforce formatting rules
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX19"/>
+  <dimension ref="A1:AX22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -867,38 +867,11 @@
         <v>2011</v>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1" s="12">
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>BSMA0007</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>The study focuses on adventure tourists, not employees in an organizational context. It does not measure workplace boundary-spanning behavior.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Conceptualizing the adventure tourist as a cross-boundary learner</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Akaho Yuma</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>2024</v>
-      </c>
-    </row>
+    <row r="10" ht="15.75" customHeight="1" s="12"/>
     <row r="11" ht="15.75" customHeight="1" s="12">
       <c r="B11" t="inlineStr">
         <is>
-          <t>BSMA0008</t>
+          <t>BSMA0007</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -906,230 +879,53 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Following the strict rule in 06_non_individual_anchors.md, this study focuses on team-level boundary spanning. The meta-analysis exclusively targets individual-level boundary spanning.</t>
+          <t>The study focuses on adventure tourists, not employees in an organizational context. It does not measure workplace boundary-spanning behavior.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>A Multilevel Investigation of Antecedents and Consequences of Team Member Boundary-Spanning Behavior</t>
+          <t>Conceptualizing the adventure tourist as a cross-boundary learner</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Marrone, J. A., Tesluk, P. E., &amp; Carson, J. B.</t>
+          <t>Akaho Yuma</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2007</v>
+        <v>2024</v>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1" s="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>365</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ12" t="inlineStr">
-        <is>
-          <t>Age</t>
-        </is>
-      </c>
-      <c r="AK12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO12" t="n">
-        <v>999</v>
-      </c>
-      <c r="AP12" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
+    <row r="12" ht="15.75" customHeight="1" s="12"/>
     <row r="13" ht="15.75" customHeight="1" s="12">
       <c r="B13" t="inlineStr">
         <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>365</v>
+          <t>BSMA0008</t>
+        </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Following the strict rule in 06_non_individual_anchors.md, this study focuses on team-level boundary spanning. The meta-analysis exclusively targets individual-level boundary spanning.</t>
+        </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
+          <t>A Multilevel Investigation of Antecedents and Consequences of Team Member Boundary-Spanning Behavior</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
+          <t>Marrone, J. A., Tesluk, P. E., &amp; Carson, J. B.</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ13" t="inlineStr">
-        <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="AK13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>999</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>0.04</v>
+        <v>2007</v>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1" s="12">
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>365</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD14" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>Tenure</t>
-        </is>
-      </c>
-      <c r="AK14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>999</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>-0.01</v>
-      </c>
-    </row>
+    <row r="14" ht="15.75" customHeight="1" s="12"/>
     <row r="15" ht="15.75" customHeight="1" s="12">
       <c r="B15" t="inlineStr">
         <is>
@@ -1177,28 +973,26 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>Emotional exhaustion</t>
+          <t>Age</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>9</v>
+        <v>999</v>
       </c>
       <c r="AL15" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AM15" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AN15" t="n">
         <v>1</v>
       </c>
-      <c r="AO15" t="inlineStr">
-        <is>
-          <t>Maslach &amp; Jackson (1981)</t>
-        </is>
+      <c r="AO15" t="n">
+        <v>999</v>
       </c>
       <c r="AP15" t="n">
-        <v>0.26</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="12">
@@ -1248,28 +1042,26 @@
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>Mutual trust</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>11</v>
+        <v>999</v>
       </c>
       <c r="AL16" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AM16" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AN16" t="n">
         <v>1</v>
       </c>
-      <c r="AO16" t="inlineStr">
-        <is>
-          <t>McAllister (1995)</t>
-        </is>
+      <c r="AO16" t="n">
+        <v>999</v>
       </c>
       <c r="AP16" t="n">
-        <v>0.16</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="12">
@@ -1319,28 +1111,26 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>Role stressors</t>
+          <t>Tenure</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>17</v>
+        <v>999</v>
       </c>
       <c r="AL17" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AM17" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AN17" t="n">
         <v>1</v>
       </c>
-      <c r="AO17" t="inlineStr">
-        <is>
-          <t>Rizzo et al. (1970)</t>
-        </is>
+      <c r="AO17" t="n">
+        <v>999</v>
       </c>
       <c r="AP17" t="n">
-        <v>0.27</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="12">
@@ -1390,11 +1180,11 @@
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>Subsidiary identification</t>
+          <t>Emotional exhaustion</t>
         </is>
       </c>
       <c r="AK18" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AL18" t="n">
         <v>1</v>
@@ -1407,11 +1197,11 @@
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>Mael &amp; Ashforth (1992)</t>
+          <t>Maslach &amp; Jackson (1981)</t>
         </is>
       </c>
       <c r="AP18" t="n">
-        <v>0.35</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="12">
@@ -1461,11 +1251,11 @@
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>Outgroup categorization</t>
+          <t>Mutual trust</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="AL19" t="n">
         <v>1</v>
@@ -1474,20 +1264,230 @@
         <v>7</v>
       </c>
       <c r="AN19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>McAllister (1995)</t>
+        </is>
+      </c>
+      <c r="AP19" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="12">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>365</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>2024</v>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AE20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>Role stressors</t>
+        </is>
+      </c>
+      <c r="AK20" t="n">
+        <v>17</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>7</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>Rizzo et al. (1970)</t>
+        </is>
+      </c>
+      <c r="AP20" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="12">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>365</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AE21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>Subsidiary identification</t>
+        </is>
+      </c>
+      <c r="AK21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>7</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>Mael &amp; Ashforth (1992)</t>
+        </is>
+      </c>
+      <c r="AP21" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="12">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>365</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>2024</v>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AE22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>Outgroup categorization</t>
+        </is>
+      </c>
+      <c r="AK22" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>7</v>
+      </c>
+      <c r="AN22" t="n">
         <v>3</v>
       </c>
-      <c r="AO19" t="inlineStr">
+      <c r="AO22" t="inlineStr">
         <is>
           <t>Leonardelli &amp; Toh (2011)</t>
         </is>
       </c>
-      <c r="AP19" t="n">
+      <c r="AP22" t="n">
         <v>0.34</v>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1" s="12"/>
-    <row r="21" ht="15.75" customHeight="1" s="12"/>
-    <row r="22" ht="15.75" customHeight="1" s="12"/>
     <row r="23" ht="15.75" customHeight="1" s="12"/>
     <row r="24" ht="15.75" customHeight="1" s="12"/>
     <row r="25" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Purge legacy data for BSMA0001-0008 to prepare for fresh extraction
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX22"/>
+  <dimension ref="A1:AX11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -839,655 +839,20 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" s="12">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>BSMA0002</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>The study focuses on technology transfer centers and university-industry boundary spanning, lacking the individual employee metrics required for this meta-analysis.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Boundary spanning between industry and university the role of Technology Transfer Centres</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Comacchio, A., Bonesso, S., &amp; Pizzi, C.</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>2011</v>
-      </c>
-    </row>
+    <row r="9" ht="15.75" customHeight="1" s="12"/>
     <row r="10" ht="15.75" customHeight="1" s="12"/>
-    <row r="11" ht="15.75" customHeight="1" s="12">
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>BSMA0007</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>The study focuses on adventure tourists, not employees in an organizational context. It does not measure workplace boundary-spanning behavior.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Conceptualizing the adventure tourist as a cross-boundary learner</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Akaho Yuma</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>2024</v>
-      </c>
-    </row>
+    <row r="11" ht="15.75" customHeight="1" s="12"/>
     <row r="12" ht="15.75" customHeight="1" s="12"/>
-    <row r="13" ht="15.75" customHeight="1" s="12">
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>BSMA0008</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Following the strict rule in 06_non_individual_anchors.md, this study focuses on team-level boundary spanning. The meta-analysis exclusively targets individual-level boundary spanning.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>A Multilevel Investigation of Antecedents and Consequences of Team Member Boundary-Spanning Behavior</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Marrone, J. A., Tesluk, P. E., &amp; Carson, J. B.</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>2007</v>
-      </c>
-    </row>
+    <row r="13" ht="15.75" customHeight="1" s="12"/>
     <row r="14" ht="15.75" customHeight="1" s="12"/>
-    <row r="15" ht="15.75" customHeight="1" s="12">
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>365</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>Age</t>
-        </is>
-      </c>
-      <c r="AK15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO15" t="n">
-        <v>999</v>
-      </c>
-      <c r="AP15" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="16" ht="15.75" customHeight="1" s="12">
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>365</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD16" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ16" t="inlineStr">
-        <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="AK16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AL16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AN16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO16" t="n">
-        <v>999</v>
-      </c>
-      <c r="AP16" t="n">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="17" ht="15.75" customHeight="1" s="12">
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>365</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD17" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ17" t="inlineStr">
-        <is>
-          <t>Tenure</t>
-        </is>
-      </c>
-      <c r="AK17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AL17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AN17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO17" t="n">
-        <v>999</v>
-      </c>
-      <c r="AP17" t="n">
-        <v>-0.01</v>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" s="12">
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>365</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD18" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE18" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF18" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI18" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>Emotional exhaustion</t>
-        </is>
-      </c>
-      <c r="AK18" t="n">
-        <v>9</v>
-      </c>
-      <c r="AL18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM18" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO18" t="inlineStr">
-        <is>
-          <t>Maslach &amp; Jackson (1981)</t>
-        </is>
-      </c>
-      <c r="AP18" t="n">
-        <v>0.26</v>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="12">
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>365</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ19" t="inlineStr">
-        <is>
-          <t>Mutual trust</t>
-        </is>
-      </c>
-      <c r="AK19" t="n">
-        <v>11</v>
-      </c>
-      <c r="AL19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM19" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO19" t="inlineStr">
-        <is>
-          <t>McAllister (1995)</t>
-        </is>
-      </c>
-      <c r="AP19" t="n">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="12">
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>365</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ20" t="inlineStr">
-        <is>
-          <t>Role stressors</t>
-        </is>
-      </c>
-      <c r="AK20" t="n">
-        <v>17</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO20" t="inlineStr">
-        <is>
-          <t>Rizzo et al. (1970)</t>
-        </is>
-      </c>
-      <c r="AP20" t="n">
-        <v>0.27</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="12">
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>365</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD21" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ21" t="inlineStr">
-        <is>
-          <t>Subsidiary identification</t>
-        </is>
-      </c>
-      <c r="AK21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO21" t="inlineStr">
-        <is>
-          <t>Mael &amp; Ashforth (1992)</t>
-        </is>
-      </c>
-      <c r="AP21" t="n">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="12">
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>365</v>
-      </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning: double-edged effects in multinational enterprises</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Liu, T., Sekiguchi, T., Qin, J., &amp; Shen, Y. X.</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>2024</v>
-      </c>
-      <c r="AD22" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AE22" t="n">
-        <v>999</v>
-      </c>
-      <c r="AF22" t="n">
-        <v>999</v>
-      </c>
-      <c r="AG22" t="n">
-        <v>999</v>
-      </c>
-      <c r="AH22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI22" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ22" t="inlineStr">
-        <is>
-          <t>Outgroup categorization</t>
-        </is>
-      </c>
-      <c r="AK22" t="n">
-        <v>7</v>
-      </c>
-      <c r="AL22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO22" t="inlineStr">
-        <is>
-          <t>Leonardelli &amp; Toh (2011)</t>
-        </is>
-      </c>
-      <c r="AP22" t="n">
-        <v>0.34</v>
-      </c>
-    </row>
+    <row r="15" ht="15.75" customHeight="1" s="12"/>
+    <row r="16" ht="15.75" customHeight="1" s="12"/>
+    <row r="17" ht="15.75" customHeight="1" s="12"/>
+    <row r="18" ht="15.75" customHeight="1" s="12"/>
+    <row r="19" ht="15.75" customHeight="1" s="12"/>
+    <row r="20" ht="15.75" customHeight="1" s="12"/>
+    <row r="21" ht="15.75" customHeight="1" s="12"/>
+    <row r="22" ht="15.75" customHeight="1" s="12"/>
     <row r="23" ht="15.75" customHeight="1" s="12"/>
     <row r="24" ht="15.75" customHeight="1" s="12"/>
     <row r="25" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Restore Excel sheet to recover deleted Author/Year metadata
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX14"/>
+  <dimension ref="A1:AX12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -886,28 +886,7 @@
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="12"/>
-    <row r="14" ht="15.75" customHeight="1" s="12">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Missing PDF Text</t>
-        </is>
-      </c>
-    </row>
+    <row r="14" ht="15.75" customHeight="1" s="12"/>
     <row r="15" ht="15.75" customHeight="1" s="12"/>
     <row r="16" ht="15.75" customHeight="1" s="12"/>
     <row r="17" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Auto-extracted measures for BSMA0006
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX29"/>
+  <dimension ref="A1:AX40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -1761,9 +1761,19 @@
           <t>BSMA0006</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.1</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1771,8 +1781,235 @@
           <t>File not found at specified location</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V27" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA27" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="n">
+        <v>11</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>Mutual trust, cognition-based mutual trust, and affect-based mutual trust were reported by both expatriates and host-country coworkers (11 items; McAllister, 1995).</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>Reported by both expatriate and coworker, computed using SRP.</t>
+        </is>
+      </c>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP27" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>Mutual trust</t>
+        </is>
+      </c>
+      <c r="AT27" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>0.71</v>
+      </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1" s="12"/>
+    <row r="28" ht="15.75" customHeight="1" s="12">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.2</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V28" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA28" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>Mutual trust, cognition-based mutual trust, and affect-based mutual trust were reported by both expatriates and host-country coworkers (11 items; McAllister, 1995).</t>
+        </is>
+      </c>
+      <c r="AN28" t="inlineStr">
+        <is>
+          <t>Reported by both expatriate and coworker.</t>
+        </is>
+      </c>
+      <c r="AO28" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP28" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>Cognition-based mutual trust</t>
+        </is>
+      </c>
+      <c r="AT28" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>0.63</v>
+      </c>
+    </row>
     <row r="29" ht="15.75" customHeight="1" s="12">
       <c r="A29" t="inlineStr">
         <is>
@@ -1781,31 +2018,1305 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.3</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V29" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA29" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>Mutual trust, cognition-based mutual trust, and affect-based mutual trust were reported by both expatriates and host-country coworkers (11 items; McAllister, 1995).</t>
+        </is>
+      </c>
+      <c r="AN29" t="inlineStr">
+        <is>
+          <t>Reported by both expatriate and coworker.</t>
+        </is>
+      </c>
+      <c r="AO29" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP29" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS29" t="inlineStr">
+        <is>
+          <t>Affect-based mutual trust</t>
+        </is>
+      </c>
+      <c r="AT29" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AV29" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" s="12">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.4</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V30" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA30" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="n">
+        <v>17</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK30" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM30" t="inlineStr">
+        <is>
+          <t>Role stressors were indicated by expatriates (17 items; Rizzo et al., 1970; Beehr et al., 1976).</t>
+        </is>
+      </c>
+      <c r="AN30" t="inlineStr"/>
+      <c r="AO30" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP30" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS30" t="inlineStr">
+        <is>
+          <t>Role stressors</t>
+        </is>
+      </c>
+      <c r="AT30" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1" s="12">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.5</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA31" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="n">
+        <v>6</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>Subsidiary identification (reported by expatriates) and MNE identification (reported by host-country coworkers) were both measured using an organizational identification scale (six items; Mael &amp; Ashforth, 1992).</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr"/>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP31" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS31" t="inlineStr">
+        <is>
+          <t>Expatriates' subsidiary identification</t>
+        </is>
+      </c>
+      <c r="AT31" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1" s="12">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.6</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA32" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="n">
+        <v>9</v>
+      </c>
+      <c r="AI32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK32" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>Emotional exhaustion was reported by expatriates (nine items; Maslach &amp; Jackson, 1981)</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr"/>
+      <c r="AO32" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP32" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS32" t="inlineStr">
+        <is>
+          <t>Expatriates' emotional exhaustion</t>
+        </is>
+      </c>
+      <c r="AT32" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1" s="12">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.7</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA33" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="n">
+        <v>7</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK33" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>outgroup categorization was reported by host-country coworkers (seven items; Leonardelli &amp; Toh, 2011).</t>
+        </is>
+      </c>
+      <c r="AN33" t="inlineStr"/>
+      <c r="AO33" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP33" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS33" t="inlineStr">
+        <is>
+          <t>Expatriates' outgroup categorization</t>
+        </is>
+      </c>
+      <c r="AT33" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" s="12">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.8</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V34" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA34" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI34" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="AO34" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP34" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ34" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR34" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>Expatriate age</t>
+        </is>
+      </c>
+      <c r="AT34" t="n">
+        <v>33.91</v>
+      </c>
+      <c r="AU34" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="AV34" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW34" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1" s="12">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.9</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V35" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA35" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
+        </is>
+      </c>
+      <c r="AN35" t="inlineStr">
+        <is>
+          <t>1 = male, 2 = female</t>
+        </is>
+      </c>
+      <c r="AO35" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP35" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ35" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR35" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>Expatriate gender</t>
+        </is>
+      </c>
+      <c r="AT35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV35" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW35" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1" s="12">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.10</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V36" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA36" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK36" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM36" t="inlineStr">
+        <is>
+          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
+        </is>
+      </c>
+      <c r="AN36" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="AO36" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP36" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ36" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR36" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS36" t="inlineStr">
+        <is>
+          <t>Expatriate tenure</t>
+        </is>
+      </c>
+      <c r="AT36" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="AU36" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AV36" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW36" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" s="12">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.11</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V37" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA37" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI37" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK37" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM37" t="inlineStr">
+        <is>
+          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
+        </is>
+      </c>
+      <c r="AN37" t="inlineStr">
+        <is>
+          <t>Proxy for language proficiency.</t>
+        </is>
+      </c>
+      <c r="AO37" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP37" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ37" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR37" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS37" t="inlineStr">
+        <is>
+          <t>Expatriate language proficiency</t>
+        </is>
+      </c>
+      <c r="AT37" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="AU37" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="AV37" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW37" t="n">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" s="12">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>BSMA0006</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>BSMA0006.1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>BSMA0006.1.12</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>File not found at specified location</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V38" t="n">
+        <v>177</v>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>expatriates</t>
+        </is>
+      </c>
+      <c r="AA38" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI38" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK38" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
+        </is>
+      </c>
+      <c r="AN38" t="inlineStr">
+        <is>
+          <t>Dummy control variable.</t>
+        </is>
+      </c>
+      <c r="AO38" t="inlineStr">
+        <is>
+          <t>Expatriates' boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP38" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="AQ38" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AR38" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AS38" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="AT38" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="AU38" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="AV38" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW38" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="12"/>
+    <row r="40" ht="15.75" customHeight="1" s="12">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>BSMA0007</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>The boundary spanner is at the organizational level (inpatient psychiatric departments) rather than an individual employee.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="12"/>
-    <row r="31" ht="15.75" customHeight="1" s="12"/>
-    <row r="32" ht="15.75" customHeight="1" s="12"/>
-    <row r="33" ht="15.75" customHeight="1" s="12"/>
-    <row r="34" ht="15.75" customHeight="1" s="12"/>
-    <row r="35" ht="15.75" customHeight="1" s="12"/>
-    <row r="36" ht="15.75" customHeight="1" s="12"/>
-    <row r="37" ht="15.75" customHeight="1" s="12"/>
-    <row r="38" ht="15.75" customHeight="1" s="12"/>
-    <row r="39" ht="15.75" customHeight="1" s="12"/>
-    <row r="40" ht="15.75" customHeight="1" s="12"/>
     <row r="41" ht="15.75" customHeight="1" s="12"/>
     <row r="42" ht="15.75" customHeight="1" s="12"/>
     <row r="43" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Auto-extracted measures for BSMA0004 (exclusion)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX5"/>
+  <dimension ref="A1:AX7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -888,8 +888,41 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1" s="12"/>
-    <row r="7" ht="15.75" customHeight="1" s="12"/>
+    <row r="6" ht="15.75" customHeight="1" s="12">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>File not found</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" s="12">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BSMA0002</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>File not found</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>999</v>
+      </c>
+    </row>
     <row r="8" ht="15.75" customHeight="1" s="12"/>
     <row r="9" ht="15.75" customHeight="1" s="12"/>
     <row r="10" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Revert BSMA0002 and clear old exclusion reason from BSMA0001
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX5"/>
+  <dimension ref="A1:AX4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="9" min="1" max="2"/>
@@ -838,11 +838,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Focal spanner is a Leader</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Leader Boundary-Spanning Behavior and Employee Voice Behavior: The Job Demands–Resources Perspective</t>
@@ -954,46 +949,7 @@
         <v>-0.57</v>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" s="9">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>BSMA0002</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Firm-level BS (not individual-level)</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Explicating the relationship of entrepreneurial orientation and firm performance: Underlying mechanisms in the context of an emerging market</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Industrial Marketing Management</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Cui et al.</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>2018</v>
-      </c>
-    </row>
+    <row r="5" ht="15.75" customHeight="1" s="9"/>
     <row r="6" ht="15.75" customHeight="1" s="9"/>
     <row r="7" ht="15.75" customHeight="1" s="9"/>
     <row r="8" ht="15.75" customHeight="1" s="9"/>

</xml_diff>

<commit_message>
Exclude BSMA0002: qualitative study without quantitative correlation matrix
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX4"/>
+  <dimension ref="A1:AX5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="9" min="1" max="2"/>
@@ -949,7 +949,46 @@
         <v>-0.57</v>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" s="9"/>
+    <row r="5" ht="15.75" customHeight="1" s="9">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BSMA0002</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Qualitative study without quantitative correlation matrix</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>“'Everything else is public relations'”: How rural journalists draw the boundary between journalism and public relations in rural communities</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Mass Communication &amp; Society</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Perreault et al.</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>2023</v>
+      </c>
+    </row>
     <row r="6" ht="15.75" customHeight="1" s="9"/>
     <row r="7" ht="15.75" customHeight="1" s="9"/>
     <row r="8" ht="15.75" customHeight="1" s="9"/>

</xml_diff>

<commit_message>
Auto-extracted measures for Glaser et al. 2015 (BSMA0003)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX5"/>
+  <dimension ref="A1:AX10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="9" min="1" max="2"/>
@@ -990,10 +990,594 @@
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="9"/>
-    <row r="7" ht="15.75" customHeight="1" s="9"/>
-    <row r="8" ht="15.75" customHeight="1" s="9"/>
-    <row r="9" ht="15.75" customHeight="1" s="9"/>
-    <row r="10" ht="15.75" customHeight="1" s="9"/>
+    <row r="7" ht="15.75" customHeight="1" s="9">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Achieving strategic renewal: the multi-level influences of top and middle managers’ boundary-spanning</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Small Business Economics</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Glaser et al.</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>2015</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>2 = Yes (expatriate, multinational, etc.)</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>397</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>middle managers</t>
+        </is>
+      </c>
+      <c r="AA7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>The MMs were presented with a list of the units and were asked to tick the units that provided them with new knowledge or expertise.</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Constructed from the number of units to which the MM in question was connected (range 1 to 30).</t>
+        </is>
+      </c>
+      <c r="AH7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>At the individual level, we controlled for gender (female =1, male =0) and job grade.</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>female = 1, male = 0</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>MM boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="AT7" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" customHeight="1" s="9">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Achieving strategic renewal: the multi-level influences of top and middle managers’ boundary-spanning</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Small Business Economics</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Glaser et al.</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>2015</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>2 = Yes (expatriate, multinational, etc.)</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>397</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>middle managers</t>
+        </is>
+      </c>
+      <c r="AA8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>The MMs were presented with a list of the units and were asked to tick the units that provided them with new knowledge or expertise.</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Constructed from the number of units to which the MM in question was connected (range 1 to 30).</t>
+        </is>
+      </c>
+      <c r="AH8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>We controlled for job grade, as, within the selected group of MMs, there were two different job grades. Job grade reflects the strategically hierarchical position of a manager, serving as a proxy for power and job complexity.</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>grade A = 0, grade B = 1</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>MM boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP8" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="AT8" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>-0.14</v>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1" s="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.3</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Achieving strategic renewal: the multi-level influences of top and middle managers’ boundary-spanning</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Small Business Economics</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Glaser et al.</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>2015</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>2 = Yes (expatriate, multinational, etc.)</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>397</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>middle managers</t>
+        </is>
+      </c>
+      <c r="AA9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>The MMs were presented with a list of the units and were asked to tick the units that provided them with new knowledge or expertise.</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Constructed from the number of units to which the MM in question was connected (range 1 to 30).</t>
+        </is>
+      </c>
+      <c r="AH9" t="n">
+        <v>7</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>The MMs were asked to indicate the extent to which they experienced role conflict by rating the items on a scale ranging from 1, “strongly disagree”, to 7, “strongly agree.”</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Seven items were averaged to form a single measure of role conflict after excluding one item from the Rizzo et al. (1970) eight-item scale due to cross loadings.</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>MM boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP9" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>Role conflict</t>
+        </is>
+      </c>
+      <c r="AT9" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="10" ht="15.75" customHeight="1" s="9">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.4</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Achieving strategic renewal: the multi-level influences of top and middle managers’ boundary-spanning</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Small Business Economics</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Glaser et al.</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>2015</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>2 = Yes (expatriate, multinational, etc.)</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>397</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>middle managers</t>
+        </is>
+      </c>
+      <c r="AA10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>The MMs were presented with a list of the units and were asked to tick the units that provided them with new knowledge or expertise.</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Constructed from the number of units to which the MM in question was connected (range 1 to 30).</t>
+        </is>
+      </c>
+      <c r="AH10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>Next, we calculated the proportion of overlap for each MM, by dividing the number of mutual ties by the total number of MMs’ boundary-spanning ties.</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Calculated using Boolean combinations in UCINET 6, representing the proportion of overlap ranging from 0 to 1.</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>MM boundary-spanning</t>
+        </is>
+      </c>
+      <c r="AP10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>Overlap</t>
+        </is>
+      </c>
+      <c r="AT10" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
     <row r="11" ht="15.75" customHeight="1" s="9"/>
     <row r="12" ht="15.75" customHeight="1" s="9"/>
     <row r="13" ht="15.75" customHeight="1" s="9"/>

</xml_diff>

<commit_message>
Auto-extracted measures for BSMA0004
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX10"/>
+  <dimension ref="A1:AX18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="9" min="1" max="2"/>
@@ -1579,13 +1579,991 @@
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="9"/>
-    <row r="12" ht="15.75" customHeight="1" s="9"/>
-    <row r="13" ht="15.75" customHeight="1" s="9"/>
-    <row r="14" ht="15.75" customHeight="1" s="9"/>
-    <row r="15" ht="15.75" customHeight="1" s="9"/>
-    <row r="16" ht="15.75" customHeight="1" s="9"/>
-    <row r="17" ht="15.75" customHeight="1" s="9"/>
-    <row r="18" ht="15.75" customHeight="1" s="9"/>
+    <row r="12" ht="15.75" customHeight="1" s="9">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>999</v>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP12" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>员工年龄</t>
+        </is>
+      </c>
+      <c r="AT12" t="n">
+        <v>28.74</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1" s="9">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA13" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>1 = male, 0 = female</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP13" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>员工性别</t>
+        </is>
+      </c>
+      <c r="AT13" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1" s="9">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.3</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA14" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>1 (high school and below) to 6 (doctoral degree)</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP14" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>教育程度</t>
+        </is>
+      </c>
+      <c r="AT14" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="15" ht="15.75" customHeight="1" s="9">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.4</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>999</v>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Months</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP15" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>本团队工作时间</t>
+        </is>
+      </c>
+      <c r="AT15" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1" s="9">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.5</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>集体主义 采用 Ilies, Wagner 和Morgeson (2007) 使用过的量表 , 共3个条目 , 比如 “比起独自工作来说 , 我更愿意和同事一起工作 ”等。</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP16" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>集体主义导向</t>
+        </is>
+      </c>
+      <c r="AT16" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1" s="9">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.6</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V17" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA17" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>3 = Others</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>咨询网络中心性 采用的是 Sparrowe 等(2001) 采用的点入中心性 (in-degree centrality, Borgatti, Everett, &amp; Freeman, 1992) 的测量方法。为了收集整体网络数据 , 我们在每个团队中都列上了所有成员的名字 , 然后要求员工对其同事进行评价。量表共 2个条目 , 比如 “你向 (某某 )寻求有关工作的帮助或建议吗 ”。我们关心的是这种关系的强度 (strength), 所以通过 Likert 5 点来进行测量 , 1表示 “从不 ”, 5表示 “总是 ”。</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>Advice network centrality</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP17" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>网络中心性</t>
+        </is>
+      </c>
+      <c r="AT17" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" s="9">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.7</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA18" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>任务绩效 采用的是 Liden, Wayne 和Stilwell (1993) 开发的量表 , 共4个条目 , 比如 “这名员工能够充分完成分配的任务 ”等, 由领导填写。</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP18" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>任务绩效</t>
+        </is>
+      </c>
+      <c r="AT18" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
     <row r="19" ht="15.75" customHeight="1" s="9"/>
     <row r="20" ht="15.75" customHeight="1" s="9"/>
     <row r="21" ht="15.75" customHeight="1" s="9"/>

</xml_diff>

<commit_message>
Update schema and BSMA0001 with demographic data
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -866,6 +866,11 @@
           <t>1 = Cross-sectional</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
       <c r="U4" t="inlineStr">
         <is>
           <t>1 = No (domestic only)</t>
@@ -873,6 +878,15 @@
       </c>
       <c r="V4" t="n">
         <v>383</v>
+      </c>
+      <c r="W4" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="X4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>999</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Insert EXCLUDED papers into Excel, assign BSMA IDs, update workflow rules
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX4"/>
+  <dimension ref="A1:AX8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="9" min="1" max="2"/>
@@ -964,9 +964,87 @@
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="9"/>
-    <row r="6" ht="15.75" customHeight="1" s="9"/>
+    <row r="6" ht="15.75" customHeight="1" s="9">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BSMA0002</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Firm-level boundary spanning (Precedent #002): Focal spanner is the firm, not an individual.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Synergy effects of digital transformation and overseas M&amp;A integration on breakthrough innovation: a boundary spanning perspective</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Technology Analysis &amp; Strategic Management</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Feiqiong Chen, Wenjing Wang, Miaomiao Xu</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>2025</v>
+      </c>
+    </row>
     <row r="7" ht="15.75" customHeight="1" s="9"/>
-    <row r="8" ht="15.75" customHeight="1" s="9"/>
+    <row r="8" ht="15.75" customHeight="1" s="9">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Team-level boundary spanning: Focal spanner is the team (N=49 interorganizational teams), not an individual.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Interorganizational teams as boundary spanners: The role of team diversity, boundedness, and extrateam links</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>European Journal of Work and Organizational Psychology</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Anat Drach-Zahavy</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>2011</v>
+      </c>
+    </row>
     <row r="9" ht="15.75" customHeight="1" s="9"/>
     <row r="10" ht="15.75" customHeight="1" s="9"/>
     <row r="11" ht="15.75" customHeight="1" s="9"/>

</xml_diff>

<commit_message>
Screening: Completed 1st screening judgments for NO. 11 to NO. 110 (100 papers)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -906,12 +906,12 @@
           <t>BSMA0001</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -939,7 +939,7 @@
       <c r="K4" s="0" t="n">
         <v>2002</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" s="0" t="inlineStr">
         <is>
           <t>Team-level study: Examines team diversity and team-level boundary spanning behaviors (unit of analysis is work team).</t>
         </is>
@@ -956,12 +956,12 @@
           <t>BSMA0002</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -989,7 +989,7 @@
       <c r="K5" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P5" s="0" t="inlineStr">
         <is>
           <t>Macro-economic / urban planning study: Examines 1930s HOLC redlining maps and neighborhood opportunity (sample is census tracts/residents, not organizational employees).</t>
         </is>
@@ -1006,12 +1006,12 @@
           <t>BSMA0003</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -1039,7 +1039,7 @@
       <c r="K6" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P6" s="0" t="inlineStr">
         <is>
           <t>Organizational-level study: Investigates cross-sector governance and collaboration capacity of U.S. city governments (unit of analysis is local government/city).</t>
         </is>
@@ -1056,12 +1056,12 @@
           <t>BSMA0004</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -1089,7 +1089,7 @@
       <c r="K7" s="0" t="n">
         <v>2016</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P7" s="0" t="inlineStr">
         <is>
           <t>Team-level study: Examines knowledge integration capability and cooperative strategy in teams (unit of analysis is project team).</t>
         </is>
@@ -1106,12 +1106,12 @@
           <t>BSMA0005</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -1140,7 +1140,7 @@
       <c r="K8" s="0" t="n">
         <v>2019</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" s="0" t="inlineStr">
         <is>
           <t>Conceptual / review article: Discusses community-academic partnerships (CAPs) in social work; no quantitative empirical dataset or effect sizes reported.</t>
         </is>
@@ -1157,12 +1157,12 @@
           <t>BSMA0006</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -1190,7 +1190,7 @@
       <c r="K9" s="0" t="n">
         <v>2005</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P9" s="0" t="inlineStr">
         <is>
           <t>Customer sample study: Examines customer-company identification among prescribing physicians (customers/clients), not internal employee boundary spanners.</t>
         </is>
@@ -1207,12 +1207,12 @@
           <t>BSMA0007</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -1240,7 +1240,7 @@
       <c r="K10" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P10" s="0" t="inlineStr">
         <is>
           <t>Firm-level study: Investigates incumbent firm adaptation and technological alliances (unit of analysis is firm-therapeutic level in biotech/pharma).</t>
         </is>
@@ -1257,12 +1257,12 @@
           <t>BSMA0008</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -1290,7 +1290,7 @@
       <c r="K11" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P11" s="0" t="inlineStr">
         <is>
           <t>Tourist sample study: Examines self-transformation and learning of adventure tourists, not organizational employee workplace behavior.</t>
         </is>
@@ -1307,12 +1307,12 @@
           <t>BSMA0009</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -1340,7 +1340,7 @@
       <c r="K12" s="0" t="n">
         <v>2008</v>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="P12" s="0" t="inlineStr">
         <is>
           <t>Team-level study: Examines new product development (NPD) team intelligence and project success (unit of analysis is NPD team).</t>
         </is>
@@ -1357,12 +1357,12 @@
           <t>BSMA0010</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -1390,7 +1390,7 @@
       <c r="K13" s="0" t="n">
         <v>2012</v>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="P13" s="0" t="inlineStr">
         <is>
           <t>Team-level study: Examines team sensemaking capability and performance in product development project teams (unit of analysis is project team).</t>
         </is>
@@ -1407,6 +1407,16 @@
           <t>BSMA0011</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
           <t>Today, many firms are striving to enhance customers’ purchase intentions by leveraging online consumer communities but a better understanding of the underlying phenomena is needed to guide their efforts most effectively. In this study we analyse how three hotel firms engage potential customers through FlyerTalk, an online consumer community of frequent travellers (FlyerTalk.com). Our results suggest that for some firms, the frequency and perceived value of their participation are two important factors that can potentially be managed toward positive purchasing intention effects.</t>
@@ -1430,6 +1440,11 @@
       <c r="K14" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1" s="31">
       <c r="A15" s="0" t="inlineStr">
@@ -1442,6 +1457,16 @@
           <t>BSMA0012</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
           <t>Boundaries are a defining characteristic of organizations, and boundary roles are the link between the environment and the organization. The creation, elaboration, and functions of boundary spanning roles are examined, with attention to environmental and technological sources of variation in the structure of boundary roles. Eleven hypotheses integrate the material reviewed and are amenable to empirical test. Future research should overcome problems created when organizations are treated as “wholes” or single entities.</t>
@@ -1465,6 +1490,11 @@
       <c r="K15" s="0" t="n">
         <v>2026</v>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1" s="31">
       <c r="A16" s="0" t="inlineStr">
@@ -1477,6 +1507,16 @@
           <t>BSMA0013</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
           <t>Within the wake of the COVID‐19 pandemic, we investigate work‐nonwork boundary management among workers who transitioned to remote work. Based on five waves of data and a sample of 155 remote workers, we find that the preference for segmentation was associated with greater work‐nonwork balance. We also found that having a dedicated office space within the home and fewer household members was associated with greater work‐nonwork balance. However, these variables did not moderate the relationship between segmentation preferences and work‐nonwork balance as expected. We discuss implications for future research on boundary management processes and practices.</t>
@@ -1500,6 +1540,11 @@
       <c r="K16" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1" s="31">
       <c r="A17" s="0" t="inlineStr">
@@ -1512,6 +1557,11 @@
           <t>BSMA0014</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
           <t>Although researchers have gained considerable knowledge regarding the multi-faceted manifestation of burnout over recent years, inconsistent findings of role ambiguity as an antecedent to burnout are still prevalent. Given the complex boundary-spanning nature of sales, it is likely that global measures of role ambiguity fail to fully capture the domain and impact of role ambiguity. To help address this gap, this study provides initial evidence that facets of role ambiguity impact burnout manifestation in the sales role differently. Specifically, findings provide a foundation to help mitigate the negative impact of burnout by focusing on only certain facets of role ambiguity.</t>
@@ -1535,6 +1585,11 @@
       <c r="K17" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="31">
       <c r="A18" s="0" t="inlineStr">
@@ -1547,6 +1602,16 @@
           <t>BSMA0015</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
           <t>To test some of the social and organizational psychology underpinnings of boundary spanning theory, the consultative, boundary spanning activities of 27 New York State school psychologists within their special education multidisciplinary teams were studied. More specifically, the relation between boundary spanning and task uncertainty, role specification, degree of professional training and continuing activity, size of organization, and available organizational resources was investigated. The results indicated that boundary spanning was significantly related to perceived task uncertainty. The implications of these results were discussed, and future research efforts needed to further differentiate this important construct were suggested.</t>
@@ -1570,6 +1635,11 @@
       <c r="K18" s="0" t="n">
         <v>1993</v>
       </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="31">
       <c r="A19" s="0" t="inlineStr">
@@ -1582,6 +1652,11 @@
           <t>BSMA0016</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
           <t>National sport policies’ harmonization with the World Anti-Doping Agency (WADA) has been one of the most researched topics within the sport policy domain. The literature, however, has failed to offer firsthand empirical insights from those actors who develop the policy so that harmonization occurs. The present study fills this gap by drawing on the tenets of institutional entrepreneurship to unpack the process through the experiences of the person responsible for it. The study employs a collaborative analytical autoethnography where, through memo-writings, emails, and reflective notes by the second author, it micro-theorizes the political, technical, and cultural activities that the institutional entrepreneur carried in order to harmonize Montenegro’s anti-doping policy with WADA. The study reveals that the harmonization process entails seven institutional works: boundary spanning, scanning the environment, repairing bilateral relationships, designing the new legislation, modifying structures, framing the need, and transferring responsibility. This is the first empirical study in sport management literature to examine institutional change for sport policy-making through the lenses of institutional entrepreneurship and a collaborative autoethnographic perspective.</t>
@@ -1605,6 +1680,11 @@
       <c r="K19" s="0" t="n">
         <v>2026</v>
       </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1" s="31">
       <c r="A20" s="0" t="inlineStr">
@@ -1617,6 +1697,11 @@
           <t>BSMA0017</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to examine the relationship between ethical climate and facets of job satisfaction among organizational buyers. Design/methodology/approach – This research is an empirical study. Data are collected from the industrial buyers using online panel. The INDSALES scale, the scale developed to measure job satisfaction of boundary spanners, was used to measure the job satisfaction. Partial least squares, a components-based structural equation modeling approach, was employed to conduct data analysis.</t>
@@ -1640,6 +1725,11 @@
       <c r="K20" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1" s="31">
       <c r="A21" s="0" t="inlineStr">
@@ -1652,6 +1742,16 @@
           <t>BSMA0018</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
           <t>Data from 409 members of forty-five new product teams in five high technology companies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator, Scout, and Guard. These activities are related to the frequency, type, and destination of communications between team members and others. This article describes these activities and examines the impact of individual and environmental variables on the frequency in which individual team members engage in them.</t>
@@ -1675,6 +1775,11 @@
       <c r="K21" s="0" t="n">
         <v>1990</v>
       </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1" s="31">
       <c r="A22" s="0" t="inlineStr">
@@ -1687,6 +1792,11 @@
           <t>BSMA0019</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
           <t>This article focuses on the activities teams use to manage their organizational environment beyond their teams. We used semistructured interviews with 38 new-product team managers in high-technology companies, log data from two of these teams, and questionnaires completed by members of a different set of 45 new-product teams to generate and test hypotheses about teams' external activities. Results indicate that teams engage in vertical communications aimed at molding the views of top management, horizontal communication aimed at coordinating work and obtaining feedback, and horizontal communication aimed at general scanning of the technical and market environment. Organizational teams appear to develop distinct strategies toward their environment: some specialize in particular external activities, some remain isolated from the external environment, and others engage in multiple external activities. The paper shows that the type of external communication teams engage in, not just the amount, determines performance. Over time, teams following a comprehensive strategy enter positive cycles of external activity, internal processes, and performance that enable long-term team success.</t>
@@ -1710,6 +1820,11 @@
       <c r="K22" s="0" t="n">
         <v>1992</v>
       </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="31">
       <c r="A23" s="0" t="inlineStr">
@@ -1722,6 +1837,16 @@
           <t>BSMA0020</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
           <t>Purpose – A large number of studies indicate that coercive forms of organizational control and performance management in health care services often backfire and initiate dysfunctional consequences. The purpose of this article is to discuss new approaches to performance management in health care services when the purpose is to support innovative changes in the delivery of services.</t>
@@ -1745,6 +1870,11 @@
       <c r="K23" s="0" t="n">
         <v>2024</v>
       </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="31">
       <c r="A24" s="0" t="inlineStr">
@@ -1757,6 +1887,11 @@
           <t>BSMA0021</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
           <t>In order to continue to be innovative in the current fast-paced and competitive environment, organizations are increasingly dependent on creative inputs developed outside their boundaries. The paper addresses the boundary spanning activities that managers undertake to a) select and mobilize creative talent, b) create shared identity, and c) combine and integrate knowledge in innovation projects involving external actors. We study boundary spanning activities in two creative projects in the LEGO group. One involves identifying and integrating deep, specialized knowledge, the other focuses on the use of external actors as a source of broad, not necessarily fully developed ideas. We find that the boundary spanning activities in these two projects differ in respect, among other things, of how the firm selects participants, formulates problems, and aligns the expectations of internal and external actors, and how knowledge is integrated across organizational boundaries. We discuss implications of our findings for managers and researchers in a business-to-business context.</t>
@@ -1780,6 +1915,11 @@
       <c r="K24" s="0" t="n">
         <v>2013</v>
       </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1" s="31">
       <c r="A25" s="0" t="inlineStr">
@@ -1790,6 +1930,11 @@
       <c r="B25" s="0" t="inlineStr">
         <is>
           <t>BSMA0022</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
@@ -1818,6 +1963,11 @@
       <c r="K25" s="0" t="n">
         <v>1995</v>
       </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="31">
       <c r="A26" s="0" t="inlineStr">
@@ -1830,6 +1980,11 @@
           <t>BSMA0023</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
           <t>Successful innovation requires firms to search beyond their organizational confines for complementary knowledge resources ahead of their competitors. While such proactive boundary-spanning search (PBS) provides relevant knowledge resources for green innovations, it can also lead to information overload that derails green innovation efforts. Therefore, there is a need to understand how and when PBS translates into green innovation. This study combines the dynamic capabilities theory with the organizational information processing theory to develop a moderated mediation model that espouses the role of green dynamic capability and analytics capability in the relationship between PBS and green innovation. The study's hypothesis is tested using firm-level survey data from 200 manufacturing firms in Ghana. Partial least squares structural equations modeling (PLS-SEM) and PROCESS were used to evaluate the research model. The results confirm a positive relationship between PBS and green dynamic capabilities, and also between green dynamic capabilities and green innovation. More importantly, PBS drives green innovation through green dynamic capability, particularly at moderate and high levels of analytics capability. The theoretical and managerial implications of the study are outlined in the text.</t>
@@ -1853,6 +2008,11 @@
       <c r="K26" s="0" t="n">
         <v>2024</v>
       </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="31">
       <c r="A27" s="0" t="inlineStr">
@@ -1865,6 +2025,11 @@
           <t>BSMA0024</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
           <t>This study analyses the presence of gender segregation in Spanish exporting ﬁrms. Both women’s access to managerial positions (vertical segregation) and women’s achievement of managerial roles that are socially associated with communal attributes (horizontal segregation) are tested. We argue that boundary-spanning (henceforth, boundary management) in export interﬁrm relationships beneﬁts from relational and communal skills and therefore could not only offer an opportunity for women to gain access to management positions but also put them at risk of falling into a rut before achieving other controlbased managerial roles. This empirical study examines the characteristics (personal and ﬁrm-level) of Spanish female managers in charge of export management through independent channels. A multivariate analysis has been performed to compare female managers with male managers both in boundary management and in the position of ﬁnance director, a control position closer to a socially stereotyped masculine role. The results show that women have slightly higher access to boundary management jobs than ﬁnance management jobs, as well as a signiﬁcantly lower promotion time than male colleagues, but they also corroborate that there is a smaller percentage of women than men in any management positions, with female managers working in younger ﬁrms with fewer resources for export activity.</t>
@@ -1888,6 +2053,11 @@
       <c r="K27" s="0" t="n">
         <v>2017</v>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="31">
       <c r="A28" s="0" t="inlineStr">
@@ -1900,6 +2070,16 @@
           <t>BSMA0025</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
           <t>No abstract</t>
@@ -1923,6 +2103,11 @@
       <c r="K28" s="0" t="n">
         <v>2018</v>
       </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="31">
       <c r="A29" s="0" t="inlineStr">
@@ -1935,6 +2120,11 @@
           <t>BSMA0026</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
           <t>Matching survey data on PhD scientists and engineers currently working in an R&amp;D job in industry with publications and patents, we study the relation between their individual motives and the rate and nature of their inventive output. We ﬁnd that individuals with a strong taste for science, that is motivated by intellectual challenge, autonomy, and contribution to society, create more novel and impactful patents in industry. These individuals are also more involved in academic boundary spanning, proxied by scientiﬁc publications co-authored with academic scientists, and this boundary spanning partially mediates the effect of taste for science on impactful inventive output. In contrast, individuals with a strong taste for salary and career collaborate less with academic scientists, fully mediating the negative effect of taste for salary and career on impactful inventive output.</t>
@@ -1958,6 +2148,11 @@
       <c r="K29" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="31">
       <c r="A30" s="0" t="inlineStr">
@@ -1970,6 +2165,16 @@
           <t>BSMA0027</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
           <t>The extent to which demand and supply shocks are transmitted in the supply chain is an important topic. As many supply chains cross international borders exchange rate pass through is an important element in this context. In this paper a multivariate system that allow us to test different hypothesis with respect to the supply chain is speciﬁed. Our empirical analysis includes tests of whether there is a link between the different stages in the supply chain, whether the exchange rate pass through is complete and whether price signals are fully transmitted. Different exogeneity assumptions are testable hypothesis, and one can avoid the simultaneity problem associated with the common single equation speciﬁcations. Moreover, one can also test whether the exchange rate is determined outside the system, as well as testing for price leadership. An application is provided for the supply chain for cod between Norway and Portugal.</t>
@@ -1993,6 +2198,11 @@
       <c r="K30" s="0" t="n">
         <v>2007</v>
       </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="31">
       <c r="A31" s="0" t="inlineStr">
@@ -2005,6 +2215,16 @@
           <t>BSMA0028</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
           <t>We focus on everyday role transitions involving home, work, and other places. Transitions are boundary-crossing activities, where one exits and enters roles by surmounting role boundaries. Roles can be arrayed on a continuum, spanning high segmentation to high integration. Segmentation decreases role blurring but increases the magnitude of change, rendering boundary crossing more difficult; crossing often is facilitated by rites of passage. Integration decreases the magnitude of change but increases blurring, rendering boundary creation and maintenance more difficult; this challenge often is surmounted by boundary work.</t>
@@ -2028,6 +2248,11 @@
       <c r="K31" s="0" t="n">
         <v>2000</v>
       </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1" s="31">
       <c r="A32" s="0" t="inlineStr">
@@ -2040,6 +2265,16 @@
           <t>BSMA0029</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
           <t>Conventional wisdom suggests that market forces such as competitor aggressiveness and competitor innovativeness induce supply chain responsiveness. However, this assertion does not only lack empirical evidence but also the mechanisms that explain the supply chain responsiveness effects of market forces are under-theorized. Drawing on the contingency–capability perspective, this research develops and tests the argument that customer integration is a critical boundary-spanning capability that translates competitor aggressiveness and innovativeness into enhanced supply chain responsiveness. Empirical results based on survey data from 117 firms in Ghana reveal that both market forces are not directly related to supply chain responsiveness. Additional results, however, show that customer integration mediates the competitor aggressiveness and innovativeness-supply chain responsiveness relationships. In contributing to the limited knowledge of the determinants of responsive supply chains, this article shows that external environmental factors are essential but might be insufficient for accounting for the heterogeneity in supply chain responsiveness.</t>
@@ -2063,6 +2298,11 @@
       <c r="K32" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1" s="31">
       <c r="A33" s="0" t="inlineStr">
@@ -2075,6 +2315,16 @@
           <t>BSMA0030</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
           <t>Expatriates provide bene®ts to multinational corporations (MNCs) when they enact boundary spanning roles. They do so by relaying local information and identifying opportunities that meet internal needs of MNCs. To test hypotheses based on social capital and role theories, we surveyed 232 expatriates. The ®ndings indicated that local experience and the diversity of social networks were conducive to the boundary spanning activities of expatriates, whereas environmental uncertainty and overseas experience had little effect. By engaging in boundary spanning activities, expatriates felt less role ambiguity and gained role bene®ts, and were more eager to use the resources that were found within different communities of the host country. In addition, those expatriates who engaged in more boundary spanning activities had higher job satisfaction and more power within their own companies than those who did not.</t>
@@ -2098,6 +2348,11 @@
       <c r="K33" s="0" t="n">
         <v>2002</v>
       </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1" s="31">
       <c r="A34" s="0" t="inlineStr">
@@ -2110,6 +2365,16 @@
           <t>BSMA0031</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
           <t>Reducing carbon emissions and achieving net-zero goals remain critical global supply chain priorities, and the transition to a circular supply chain is pivotal in reducing carbon emissions. This study empirically examines how low-carbon operations management practices impact circular supply chain management. We collected and analysed data from 183 respondents. Results from partial least squares structural equation modelling show that net-zero capabilities have a direct positive moderating effect on green product innovation and enhance end-of-product-life management and that net-zero capability can play a major role as a boundary-spanning function in accelerating green product innovation while balancing carbon emissions in the circular supply chain. Net-zero capability refers to a firm's ability to reduce its greenhouse gas emissions and align its operations with decarbonisation efforts. For practitioners, our results highlight that firms should focus on more than just green innovation; they should strengthen their net-zero capabilities to support sustainable supply chain practices.</t>
@@ -2133,6 +2398,11 @@
       <c r="K34" s="0" t="n">
         <v>2026</v>
       </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1" s="31">
       <c r="A35" s="0" t="inlineStr">
@@ -2145,6 +2415,16 @@
           <t>BSMA0032</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
           <t>The Management by Rites (MBR) perspective studies how management creates a universal corporate culture by uniformly defining performance expectations for human systems. The MBR Model designed for this study tested that perspective.</t>
@@ -2168,6 +2448,11 @@
       <c r="K35" s="0" t="n">
         <v>1990</v>
       </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="31">
       <c r="A36" s="0" t="inlineStr">
@@ -2180,6 +2465,11 @@
           <t>BSMA0033</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the types of justice that affect knowledge acquisition and opportunism in strategic alliances and how these justice mechanisms function. Design/methodology/approach – Data were collected from both top-level and operating-level boundary spanners in 295 strategic alliances in China (a total of 590 boundary spanners). A structural equation model (SEM) with bias-corrected bootstrap method was used to test the hypotheses.</t>
@@ -2203,6 +2493,11 @@
       <c r="K36" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="31">
       <c r="A37" s="0" t="inlineStr">
@@ -2215,6 +2510,11 @@
           <t>BSMA0034</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
           <t>Existing models of work group effectiveness have been tested in low-technology manufacturing settings, but not in a high-technology one. Typical features of high-technology environments – substantial automation, computerized scheduling systems, complex production processes, capital-intensive production, high-cost equipment, and high product value – render them significantly different from their low-technology counterparts. The increased use of work groups and teams among high-technology manufacturers raises the question of whether existing models can be generalized to these settings. In this paper, data from 89 groups in the semiconductor manufacturing industry are used to create predictive models of group productivity, job satisfaction, and perceived performance. External variables (such as conflict with supervisors and engineers) are found to be more predictive of productivity, while internal variables (such as conflict among group members) are more predictive of satisfaction. These results highlight the importance of fostering the work group's interaction with external technical support personnel when designing and managing successful work groups in high-technology workplaces.</t>
@@ -2238,6 +2538,11 @@
       <c r="K37" s="0" t="n">
         <v>2000</v>
       </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1" s="31">
       <c r="A38" s="0" t="inlineStr">
@@ -2250,6 +2555,11 @@
           <t>BSMA0035</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
           <t>The revolutionary advancement of technology in the past decade brought the attention of academics and management practitioners to ways of improving innovative capabilities of organizations. Advice-seeking relationships have an essential role in the knowledge production of modern-day organizations as they enable actors to acquire information, professional support and knowledge elements that they can recombine to form new knowledge. This paper conceptualizes advice-seeking behaviour as part of an inherently complex social world that can best be captured by a multiplex approach to organizational network research. It investigates how different layers of interpersonal relationships in the workplace may contribute to the appearance of advice-seeking interactions. This study examines the cases of three knowledge-intensive organizations and applies binary logistic regression to shed light on the yet invisible relational foundations of workplace collaboration. Implications for Central European audience: Central European countries attempt to improve their economic competitiveness by attracting knowledge-intensive companies as well as incentivizing innovation and digital transformation. Knowledge-intensive firms, such as business service centres or information and communication technology companies, are significant contributors to the economic output of countries such as the Czech Republic, Hungary and Poland. Recommendations derived from the results of this paper provide insights into the leadership of knowledge-intensive companies regarding creation of organizational environments that foster knowledge sharing and innovation. Measures that promote interpersonal trust, visibility of expertise and boundary-spanning behaviour are recommended.</t>
@@ -2273,6 +2583,11 @@
       <c r="K38" s="0" t="n">
         <v>2023</v>
       </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1" s="31">
       <c r="A39" s="0" t="inlineStr">
@@ -2285,6 +2600,16 @@
           <t>BSMA0036</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
           <t>Academy of management journal</t>
@@ -2308,6 +2633,11 @@
       <c r="K39" s="0" t="n">
         <v>1997</v>
       </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1" s="31">
       <c r="A40" s="0" t="inlineStr">
@@ -2320,6 +2650,16 @@
           <t>BSMA0037</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
           <t>Designing a supply chain network provides the basic structure for supply chain operations, where the network is a major element in a ﬁrm’s competitiveness and a signiﬁcant area of capital investment. With the boundary-spanning scope encouraged by supply chain management, the question is whether existing analyses used for network design are adequate. The general answer is yes, because the number of echelons that the analysis must span is self-limiting to a relative few. However, there remain unresolved issues in network design analysis and in the models used to support the analysis that can enhance its accuracy, appropriateness, and acceptability to practitioners. Issues discussed relate to the development of better models, the treatment of the data needed by them, and the need for comparing the various models for network design.</t>
@@ -2343,6 +2683,11 @@
       <c r="K40" s="0" t="n">
         <v>2001</v>
       </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1" s="31">
       <c r="A41" s="0" t="inlineStr">
@@ -2355,6 +2700,16 @@
           <t>BSMA0038</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore the relationship between geographic search and business model innovation and proposed a contingent framework to focus on how governmental networking and environment turbulence are interdependent moderate the relationship between geographic search and business model innovation.</t>
@@ -2378,6 +2733,11 @@
       <c r="K41" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1" s="31">
       <c r="A42" s="0" t="inlineStr">
@@ -2390,6 +2750,11 @@
           <t>BSMA0039</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
           <t>The aim of this research is to analyse how design and use are mediated in Open Source Software (OSS) design. Focusing on the Python community, our study examines a ‘‘pushed-by-users’’ design proposal through the discussions occurring in two mailing-lists: one, useroriented and the other, developer-oriented. To characterize the links between users and developers, we investigate the activities and references (knowledge sharing) performed by the contributors to these two mailing-lists. We found that the participation of users remains local to their community. However, several key participants act as boundary spanners between the user and the developer communities. This emerging role is characterized by cross-participation in parallel same-topic discussions in both mailing-lists, cohesion between crossparticipants, the occupation of a central position in the social network linking users and developers, as well as active, distinctive and adapted contributions. The user championing the proposal acts as a key boundary spanner coordinating the process and using explicit linking strategies. We argue that OSS design may be considered as a form of ‘‘role emerging design’’, i.e. design organized and pushed through emerging roles and through a balance between these roles. The OSS communities seem to provide a suitable socio-technical environment to enable such role emergence.</t>
@@ -2413,6 +2778,11 @@
       <c r="K42" s="0" t="n">
         <v>2008</v>
       </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1" s="31">
       <c r="A43" s="0" t="inlineStr">
@@ -2425,6 +2795,16 @@
           <t>BSMA0040</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to find out whether superior autonomy at boundary spanning levels in service organizations results in better market orientation and performance and whether autonomy and decentralization, though conceptually different, have similar practical implications. Researchers developed a theoretical model and tested it in the post-liberalized Indian retail banking context to address these concerns.</t>
@@ -2448,6 +2828,11 @@
       <c r="K43" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1" s="31">
       <c r="A44" s="0" t="inlineStr">
@@ -2460,6 +2845,11 @@
           <t>BSMA0041</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
           <t>We examine the role of cultural and language skills as resources for individuals’ boundary spanning ability in multinational corporations. Our combined qualitative and quantitative analysis shows that cultural and language skills influence the extent to which individual boundary spanners perform four functions: exchanging, linking, facilitating, and intervening. Boundary spanners with both cultural and language skills perform more functions than those with only cultural skills, and language skills are critical for performing the most demanding functions. Key boundary spanners have properties that potentially make them not only valuable organizational human capital, but also rare and difficult to imitate. Theoretical and practical implications are discussed.</t>
@@ -2483,6 +2873,11 @@
       <c r="K44" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1" s="31">
       <c r="A45" s="0" t="inlineStr">
@@ -2495,6 +2890,16 @@
           <t>BSMA0042</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
           <t>Book chapter</t>
@@ -2518,6 +2923,11 @@
       <c r="K45" s="0" t="n">
         <v>2024</v>
       </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1" s="31">
       <c r="A46" s="0" t="inlineStr">
@@ -2530,6 +2940,11 @@
           <t>BSMA0043</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
           <t>A plethora of research has investigated the impact of the frontline employee on the customer, with the consensus that employees can have a tremendous impact on the customer. What remains to be discovered is the extent to which this relationship exists in the reverse. Utilizing broaden-and-build and emotional contagion theories, this study suggests that employee perceptions of a specific customer emotion (delight) have an impact on the frontline employee. Specifically, results from a structural equations model reveal that employee perceptions of customer delight lead to employee positive affect, which in turn positively influences commitment and job satisfaction as well as creates stronger external representation behaviors, internal influence behaviors, and service delivery behaviors from the employee. These findings contribute new evidence to the debate of the viability of providing customer delight and extend our knowledge beyond emotional contagion in explaining how positive customer emotions manifest in employees.</t>
@@ -2553,6 +2968,11 @@
       <c r="K46" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1" s="31">
       <c r="A47" s="0" t="inlineStr">
@@ -2565,6 +2985,11 @@
           <t>BSMA0044</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
           <t>This study examines the antecedents cf job satisfaction, commitment, and turnover intentions for 229 information systems (IS) personnel employed within several industries. The antecedents studied include boundary spanning, role ambiguity, and rcle conflict. A model of these variables was built and tested using path analysis- Rcle ambiguity was found tc be the mcst dysfunctional variable for IS personnel, acccunting fcr 10.3%. 20.2% and 22.2% Of the variance in turnover intenticns. commitment, andjob satisfaction. This information is used tc make recommendaticns to IS management. Finally, recommendaticns and directions are suggested regarding future research.</t>
@@ -2588,6 +3013,11 @@
       <c r="K47" s="0" t="n">
         <v>1985</v>
       </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1" s="31">
       <c r="A48" s="0" t="inlineStr">
@@ -2600,6 +3030,11 @@
           <t>BSMA0045</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
           <t>This article examines the evolving use of boundary objects in cross-cultural software teams. Our field study of a Jamaican-Indian team examines the use of software specifications and project management tools as boundary objects in facilitating sharing across knowledge boundaries.We examine how and why the role and use of boundary objects may facilitate collaboration across knowledge boundaries at one time and contribute to conflict at other times. We unpack the interacting elements that both facilitate and constrain knowledge sharing, and trigger conflicts at different stages of the software team development. Specifically, we found that the use of boundary objects at transitions involving definitional control and the subsequent redistribution of power/authority may inhibit knowledge sharing. The subsequent reifying of cultural boundaries along with negative stereotyping led to relational conflict, through a process we call culturizing, as cross-cultural differences emerged as problematic for team dynamics.</t>
@@ -2623,6 +3058,11 @@
       <c r="K48" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1" s="31">
       <c r="A49" s="0" t="inlineStr">
@@ -2635,6 +3075,11 @@
           <t>BSMA0046</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
           <t>This research investigated how experiences in a particular boundary-spanning context (community outreach) affected members' organizational identity and identification. Multimethod panel data from 219 participants showed that intergroup comparisons with clients (emphasizing differences) and intragroup comparisons with other organization members (emphasizing similarities) changed how members construed their organization's defining qualities. Intergroup comparisons also enhanced the esteem members derived from organizational membership, which, in turn, strengthened organizational identification. Supervisors reported higher interpersonal cooperation and work effort for members whose organizational identification became stronger. The results reveal potential outcomes of boundary-spanning work as well as how organizational identification processes operate in everyday work contexts.</t>
@@ -2658,6 +3103,11 @@
       <c r="K49" s="0" t="n">
         <v>2001</v>
       </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="31">
       <c r="A50" s="0" t="inlineStr">
@@ -2670,6 +3120,16 @@
           <t>BSMA0047</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
           <t>No abstract</t>
@@ -2693,6 +3153,11 @@
       <c r="K50" s="0" t="n">
         <v>2024</v>
       </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1" s="31">
       <c r="A51" s="0" t="inlineStr">
@@ -2705,6 +3170,11 @@
           <t>BSMA0048</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
           <t>The literature suggests that the success of innovation clusters is based on personal networks that connect members of scientific, educational, and business organizations, stimulating more formalized cross-boundary collaborations between the three sectors. But it is still unclear if such organizational collaborations actually correspond with these personal ties and which aspects of personal communication are most strongly associated with organizational collaborations. To investigate these issues, the authors applied network analysis to study an innovation cluster in Algarve, Portugal. They found that cross-boundary organizational collaborations corresponded with personal ties. Moreover, they found that collaborations appeared to correlate most strongly with emotional attachments between individuals.</t>
@@ -2728,6 +3198,11 @@
       <c r="K51" s="0" t="n">
         <v>2018</v>
       </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="31">
       <c r="A52" s="0" t="inlineStr">
@@ -2740,6 +3215,11 @@
           <t>BSMA0049</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
           <t>Customer engagement entails unequivocal frontline service employees’ top performances and recommendable behaviors through management appropriate leadership to ﬂourish. Under the social exchange and social identity theories, this study investigates employee customer–oriented boundary-spanning behaviors as an outcome of spiritual leadership, through the mediating eﬀect of employee spiritual survival and well-being. PROCESS macro was used to analyze data collected from 5-star hotels full-time frontline employees in Antalya, Turkey. Results indicated that the eﬀect of spiritual leadership on the three dimensions of customer-oriented boundary-spanning behaviors is fully mediated by spiritual survival and spiritual well-being. Spirituality appears to be a noteworthy but remote contributor to customer engagement via employees’ boundary-spanning behaviors. Our study contributed to the boundary-spanning and customer engagement literature by illustrating that a sense of mission and wellbeing at the workplace are adequate requirements to engage a frontline employee, whose boundaryspanning behaviors will be instrumental in fostering customer engagement. Further detailed theoretical and managerial implications are discussed.</t>
@@ -2763,6 +3243,11 @@
       <c r="K52" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1" s="31">
       <c r="A53" s="0" t="inlineStr">
@@ -2775,6 +3260,11 @@
           <t>BSMA0050</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
           <t>Post financial crisis, audit committee (AC) reforms are proposed to improve the quality of financial reporting (EC 2011; Competition Commission 2013). This paper’s empirical contribution is to investigate the extent to which ACs and audit committee chairs (ACCs) engage with chief financial officers (CFOs) and audit partners (APs) across a range of 32 financial reporting issues. It is the first large-scale survey of interactions to move beyond the micro CFO / AP dyad and to distinguish the individual ACC from the AC group. While 37% of the 5,445 reported discussions involve all three key individuals together with the full AC, 35% involve neither the AC nor the ACC and the ACC acts without the full AC in a significant minority of cases. The parties reported to be involved are similar across the three respondent groups but vary with financial reporting issue, company size and audit firm size. The paper’s theoretical contribution is to interpret the evidence using the concepts of boundary spanning and gatekeeping roles. The research reveals incomplete levels of AC and ACC engagement with financial reporting issues. Findings have implications for policymakers regarding the role, influence and effectiveness of the AC in financial reporting matters. Directions for future research are identified.</t>
@@ -2798,6 +3288,11 @@
       <c r="K53" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1" s="31">
       <c r="A54" s="0" t="inlineStr">
@@ -2810,6 +3305,16 @@
           <t>BSMA0051</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
           <t>The proactiveness - business performance relationship was examined in this study by adopting a descriptive and crosssectional research design. Structural equation modeling was applied on a purposive sample of 457 North Indian firms to assess the impact of proactiveness on business performance. Moderating effect of environmental turbulence on proactiveness – business performance relationship was also assessed. The study found proactiveness as a significant predictor of business performance. The study revealed that firms operating in a dynamic environment were likely to be benefitted more from the pursuit of proactiveness. The findings provoke managers and entrepreneurs to adopt forwardlooking and opportunity-seeking perspectives to achieve robust business performance. Managers of Indian firms can draw insights from this study and can better decide the strategic posture of their firms.</t>
@@ -2833,6 +3338,11 @@
       <c r="K54" s="0" t="n">
         <v>2018</v>
       </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1" s="31">
       <c r="A55" s="0" t="inlineStr">
@@ -2845,6 +3355,11 @@
           <t>BSMA0052</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
           <t>This study examined how leaders’ internal and external activities mediate the relationship of functional heterogeneity and interteam goal interdependence to team effectiveness (in-role performance and innovation) in interdisciplinary teams. The results of the structural equation model from a sample of 92 interdisciplinary teams indicate that leaders’ internal activities fully mediate the relationship of team functional heterogeneity and interteam goal interdependence to team in-role performance. The leaders’ external activities were found to fully mediate the relationship of interteam goal interdependence to team innovation. We discuss the implications of these findings for both theory and practice.</t>
@@ -2868,6 +3383,11 @@
       <c r="K55" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1" s="31">
       <c r="A56" s="0" t="inlineStr">
@@ -2880,6 +3400,11 @@
           <t>BSMA0053</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
           <t>Membership of boundary‐spanners is controversial, as employees operate largely at the borders of the organization in close relations with customers. Nevertheless, we know little about its influence on customer satisfaction. We investigate how and when identification with the branch influences customer satisfaction. The how question is answered by showing that degree of control of one's performance mediates the impact of branch manager identification on customer satisfaction. The when question is answered by proposing two moderating variables. Locus of control regulates the extent to which identification influences performance control. Dedicated meetings between branch managers and their colleagues regulate the degree to which performance control influences customer satisfaction. Hypotheses were tested in a longitudinal design on a sample of 1,461 managers from a firm specializing in banking and financial services in Europe. Results largely confirm our hypotheses, providing a novel look on determinants of customer satisfaction from the perspective of boundary‐spanning managers.</t>
@@ -2903,6 +3428,11 @@
       <c r="K56" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1" s="31">
       <c r="A57" s="0" t="inlineStr">
@@ -2915,6 +3445,11 @@
           <t>BSMA0054</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
           <t>The authors investigate three types of customer-oriented boundary-spanning behaviors (COBSBs)a frontline service employee may perform that are associated with linking a service organization to its potential or actual customers: external representation, internal influence, and service delivery. The authors propose and test a withdrawal model to explain the negative effects of role conflict and role ambiguity on COBSBs across a sample of 220 lower-level, nonprofessional service providers of a major retail bank and a sample of 90 higher-level, professional service providers from the business credit division of an international financial services corporation. The results demonstrate that (1)indirect paths through job satisfaction and organizational commitment entirely account for the negative effects of the role stressors on COBSBs, (2) the indirect negative effects of the role stressors are stronger on external representation and internal influence behaviors, and (3)role conflict also has a significant positive direct relationship with internal influence behaviors.</t>
@@ -2938,6 +3473,11 @@
       <c r="K57" s="0" t="n">
         <v>2003</v>
       </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1" s="31">
       <c r="A58" s="0" t="inlineStr">
@@ -2950,6 +3490,11 @@
           <t>BSMA0055</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
           <t>Using a sample of 281 frontline service employees of a national retail bank, we test a social exchange model of antecedents of three dimensions of customer-oriented boundary-spanning behaviors suggested by prior boundary-spanning and services marketing/management literatures: external representation, internal inﬂuence, and service delivery. In support of our hypotheses, we identify fully mediated relationships from procedural, interactional, and distributive justice to external representation and internal inﬂuence via job satisfaction and organizational commitment. Our results generally support our expectation that the indirect effects of procedural justice on external representation and internal inﬂuence are stronger than the indirect effects of distributive or interactional justice on these behaviors. Also, our results reveal no signiﬁcant indirect effects of procedural and distributive justice on service delivery behaviors. However, we ﬁnd an unexpected direct positive path from interactional justice to service delivery behaviors. We interpret this latter ﬁnding in light of the normative value of interactional justice as a source of role modeling or managerial legitimacy.</t>
@@ -2973,6 +3518,11 @@
       <c r="K58" s="0" t="n">
         <v>2005</v>
       </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="18" customHeight="1" s="31">
       <c r="A59" s="0" t="inlineStr">
@@ -2985,6 +3535,16 @@
           <t>BSMA0056</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
           <t>Abstract                            Business Process Management is a boundary-spanning discipline that aligns operational capabilities and technology to design and manage business processes. The               Digital Transformation               has enabled human actors, information systems, and smart products to interact with each other via multiple digital channels. The emergence of this hyper-connected world greatly leverages the prospects of business processes – but also boosts their complexity to a new level. We need to discuss how the BPM discipline can find new ways for identifying, analyzing, designing, implementing, executing, and monitoring business processes. In this research note, selected transformative trends are explored and their impact on current theories and IT artifacts in the BPM discipline is discussed to stimulate transformative thinking and prospective research in this field.</t>
@@ -3008,6 +3568,11 @@
       <c r="K59" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="18" customHeight="1" s="31">
       <c r="A60" s="0" t="inlineStr">
@@ -3020,6 +3585,11 @@
           <t>BSMA0057</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
           <t>When the ordering function is governed by administrative arrangements and sales are regulated by long-term contracts, managers may question the necessity and the tasks of the sales function within established customer relationships. The authors examine three issues related to the role of the salesperson in established industrial buyer-seller relationships: (1) appropriate measures of salesperson performance within a relationship, (2) behaviors and skills affecting salesperson performance, and (3) the effect of salesperson performance on the relationship. The results from a survey of industrial buyers suggest that the salesperson has a significant and substantial effect on relationship continuity. They also show that the salesperson contributes to perceptions of the supplier's reliability and supplier services. The key attributes of an effective salesperson are ability to resolve conflicts, ability to develop a personal relationship with customers, and ability to facilitate exchange of information between the supplier and buyer firms.</t>
@@ -3043,6 +3613,11 @@
       <c r="K60" s="0" t="n">
         <v>1997</v>
       </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="18" customHeight="1" s="31">
       <c r="A61" s="0" t="inlineStr">
@@ -3053,6 +3628,11 @@
       <c r="B61" s="0" t="inlineStr">
         <is>
           <t>BSMA0058</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
@@ -3083,6 +3663,11 @@
       <c r="K61" s="0" t="n">
         <v>2011</v>
       </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1" s="31">
       <c r="A62" s="0" t="inlineStr">
@@ -3095,6 +3680,16 @@
           <t>BSMA0059</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
           <t>B ishop P. and G ripaios P. Spatial externalities, relatedness and sector employment growth in Great Britain, Regional Studies. This paper examines the impact of externalities on employment growth in sub-regions of Great Britain by estimating ordinary least-squares (OLS) and maximum likelihood spatial models at the two-digit level for 23 sectors. Issues arising from relatedness, sector differences, competition, cross-boundary spillovers, and spatial autocorrelation are explicitly addressed. Results indicate that specialization has a generally negative impact on growth, whilst the impact of diversity is heterogeneous across sectors and strong local competition has a typically positive impact. The results question the merits of policies primarily aimed at promoting regional specialization and suggest that diversity, local competition, and sector heterogeneity are important policy issues.</t>
@@ -3118,6 +3713,11 @@
       <c r="K62" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1" s="31">
       <c r="A63" s="0" t="inlineStr">
@@ -3130,6 +3730,11 @@
           <t>BSMA0060</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
           <t>The temporal imagination is the understanding of the intersection of one entity’s timescape with the larger timescapes of which that entity is a part. We examine in detail what the temporal imagination is, complemented with a discussion of the related timescape idea, and why the temporal imagination is necessary to function in any timescape. We also discuss group attributes that will likely affect the development of the temporal imagination and its use and how its use in group boundary spanning efforts affect both the groups and the larger organization.</t>
@@ -3153,6 +3758,11 @@
       <c r="K63" s="0" t="n">
         <v>2003</v>
       </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1" s="31">
       <c r="A64" s="0" t="inlineStr">
@@ -3165,6 +3775,16 @@
           <t>BSMA0061</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
           <t>Research Summary: This Special Section of the Strategic Entrepreneurship Journal explores how business model innovation (BMI) can address grand challenges (GCs), including artificial intelligence (AI), business and global unrest, and climate change through a proposed “ABC” classification and “BMI-GC” concept. Highlighting BMI's role as a boundary-spanning, collaborative approach to innovation, we demonstrate its potential to drive sustainable solutions by rethinking value creation, delivery, and capture mechanisms. We examine how BMI may foster resilience and help firms and organizations adapt to global volatility, integrate ethical AI, and advance sustainability in business ecosystems. We offer a roadmap for future inquiry into BMI-GC, including measurement and assessment, digital transformation, and collaborative ecosystems. By embracing these research pathways, scholars can contribute to a deeper theoretical and practical understanding of BMI to address grand challenges.</t>
@@ -3188,6 +3808,11 @@
       <c r="K64" s="0" t="n">
         <v>2025</v>
       </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1" s="31">
       <c r="A65" s="0" t="inlineStr">
@@ -3200,6 +3825,16 @@
           <t>BSMA0062</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
           <t>Purpose – This study adopts a person-centered perspective to explore how entrepreneurs combine multiple proactive behavioral strategies across the business, personal and business-environment domains. We research whether certain combinations of proactive behavioral strategies (i.e. seeking resources, optimizing demands, seeking challenges, idea generation, environmental exploration, network crafting, self-insight and boundary management) relate to well-being and business performance. Moreover, we investigate whether entrepreneurs’ daily use of these strategies aligns with their general profiles.</t>
@@ -3223,6 +3858,11 @@
       <c r="K65" s="0" t="n">
         <v>2025</v>
       </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="18" customHeight="1" s="31">
       <c r="A66" s="0" t="inlineStr">
@@ -3235,6 +3875,16 @@
           <t>BSMA0063</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
           <t>Recently, work-family scholars have empirically demonstrated the importance of congruence between employees' boundary management preferences and boundary management supplies provided by the work environment in relation to employee attitudes and behavior. However, a theoretically grounded construct that captures this congruence is lacking. The present study addresses this gap by developing the construct and measure of work-nonwork boundary management fit, based on the needs-supplies fit framework. We cross-validate the scale in three independent samples (n = 188, diverse group of employees, n = 75, employees from one hospital, and n = 81, employees from one car company) and in a fourth sample (n = 458, working parents), we demonstrated the importance of work-nonwork boundary management fit for employee well-being (i.e., stress and work-life conflict). In particular, we confirmed its unique role in predicting employee well-being, above and beyond workload and work interrupting nonwork behaviors. Hence, we argue for considering work-nonwork boundary management fit when studying how work-family policies and organizational culture affect employees in the workplace.</t>
@@ -3258,6 +3908,11 @@
       <c r="K66" s="0" t="n">
         <v>2018</v>
       </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="18" customHeight="1" s="31">
       <c r="A67" s="0" t="inlineStr">
@@ -3270,6 +3925,11 @@
           <t>BSMA0064</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
           <t>Context is an important but largely ignored dimension of quality service encounters. This paper contributes to the hospitality service industries literature by examining how the front-of-house and backof-house boundary work (Nippert-Eng 1996, 2003) engaged by Room Attendants working within the hotel guest room space impact on the hospitality impression management performed. Qualitative data from fieldwork engaging with hotel employees located within the tourist resort of Queenstown New Zealand are used to explore the multiple fronts on which the front-of-house and back-of-house boundaries are simultaneously negotiated. The results suggest that Room Attendants negotiate the front-ofhouse and back-of-house boundary through objects – such as the guest room and articles belonging to the guest – and aspects of self – such as impression management, safety, socialising and self-responsibility for room checking. The results support the importance of considering context when seeking to understand the complexities associated with the (re)production of a reliably positive service encounter.</t>
@@ -3293,6 +3953,11 @@
       <c r="K67" s="0" t="n">
         <v>2007</v>
       </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="18" customHeight="1" s="31">
       <c r="A68" s="0" t="inlineStr">
@@ -3305,6 +3970,11 @@
           <t>BSMA0065</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
           <t>This research examined the relationships between structural positions and influence at the individual level of analysis. The structure of the organization was conceptualized from a social network perspective. Measures of the relative positions of employees within workflow, communication, and friendship networks were strongly related to perceptions of influence by both supervisors and non-supervisors and to promotions to the supervisory level. Measures included criticality, transaction alternatives, and centrality (access and control) in the networks and in such reference groups as the dominant coalition. A comparison of boundary-spanning and technical-core personnel indicated that contacts beyond the normal work requirements are particularly important for technical core personnel to acquire influence. Overall, the results provide support for a structural perspective on intraorganizational influence.</t>
@@ -3328,6 +3998,11 @@
       <c r="K68" s="0" t="n">
         <v>1984</v>
       </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="18" customHeight="1" s="31">
       <c r="A69" s="0" t="inlineStr">
@@ -3340,6 +4015,11 @@
           <t>BSMA0066</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
           <t>Research has shown that NPD project leaders should engage in boundary-spanning activities. The present study tested the impact of four boundary-spanning activities on NPD project performance and analyzed the antecedents of these activities. We hypothesized that NPD project leaders' abilities to perform these activities depend on the characteristics of their personal networks — structural holes, strength of ties, vertical and horizontal bridging ties. A Partial Least Squares test on 73 NPD projects showed that (a) “obtaining political support” and “scanning for ideas” are the boundary activities with the greatest impact on performance, (b) project leaders with strong ties in their network are more effective at these activities, (c) project leaders with structural holes in their networks are more effective in another boundary activity, “protecting the team”, although this activity does not affect NPD outcomes. These results represent an important contribution to understanding how team leaders contribute to project performance.</t>
@@ -3363,6 +4043,11 @@
       <c r="K69" s="0" t="n">
         <v>2012</v>
       </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="18" customHeight="1" s="31">
       <c r="A70" s="0" t="inlineStr">
@@ -3375,6 +4060,16 @@
           <t>BSMA0067</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
           <t>Objective To evaluate feasibility and acceptability of a health professional resilience skills training program with neurology residents. Methods The curriculum consists of ﬁve 1-hour-long modules that included the following skills: reﬂective narrative practices, emotion regulation, communication with highly distressed individuals, boundary management, and the identiﬁcation of depression and trauma. Using a web-based survey tool, we administered the Brief Resilience Scale (BRS) and Abbreviated Maslach Burnout Inventory (aMBI) at baseline, in addition to a pre- and post-survey assessing change in beliefs and self-eﬃcacy, as well as satisfaction with the intervention. Means were compared using the Wilcoxon rank-sum and signed rank tests. Results Twenty-two residents representing each year of training completed the pre-survey; 41% were women. Subscale scores on the aMBI revealed that 50% had moderate or high emotional exhaustion, 41% had moderate depersonalization, and 37% had moderate or low personal accomplishment, though 77.3% reported high career satisfaction. Female residents had lower scores on the BRS (mean 3.26 vs 3.88, p &lt; 0.05), though scores on aMBI subscales did not diﬀer by sex. Scores did not diﬀer by year of training. Sixteen residents completed both the pre- and post-survey. Signiﬁcant increases were detected in 4 of 9 self-eﬃcacy statements. Seventy-one percent of residents were satisﬁed or extremely satisﬁed with the training. Conclusions Residents were satisﬁed with the curriculum and reported improved ability to identify and cope with work-related stress. Further study is needed to evaluate the inﬂuence of skills adoption and practice on resilience and burnout.</t>
@@ -3398,6 +4093,11 @@
       <c r="K70" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="18" customHeight="1" s="31">
       <c r="A71" s="0" t="inlineStr">
@@ -3408,6 +4108,16 @@
       <c r="B71" s="0" t="inlineStr">
         <is>
           <t>BSMA0068</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
@@ -3466,6 +4176,11 @@
       <c r="K71" s="0" t="n">
         <v>2017</v>
       </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="18" customHeight="1" s="31">
       <c r="A72" s="0" t="inlineStr">
@@ -3478,6 +4193,16 @@
           <t>BSMA0069</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
           <t>As Thomas Friedman so persuasively argued in his book The World is Flat, 1 a significant effect of globalization is a leveling of the playing field for many of the competitors in today’s worldwide markets. Technological innovations have revolutionized the workplace, bringing the competitive power of emerging economies’ fast-growth organizations into closer alignment with their developed-world counterparts. Paradoxically, at the same time that these developments have made doing business across borders easier, relational barriers—obstacles to productive human interactions—not only remain largely unchanged but in some cases have deepened.
@@ -3502,6 +4227,11 @@
       <c r="K72" s="0" t="n">
         <v>2011</v>
       </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="18" customHeight="1" s="31">
       <c r="A73" s="0" t="inlineStr">
@@ -3514,6 +4244,11 @@
           <t>BSMA0070</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
           <t>This dissertation examines the extent to which organizational and professional commitment, the technical environment, and the professional environment are related to boundary spanning activity. Surveys of R&amp;D professional employees, their co-workers, and their managers were used to obtain measures of commitment to their organizations and professions, perceptions of the technical and professional environment in which they worked, and the frequency with which they communicated both within and outside of the R&amp;D unit.</t>
@@ -3537,6 +4272,11 @@
       <c r="K73" s="0" t="n">
         <v>1995</v>
       </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="18" customHeight="1" s="31">
       <c r="A74" s="0" t="inlineStr">
@@ -3549,6 +4289,16 @@
           <t>BSMA0071</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
           <t>We study the relation between stability of the nonproﬁt organization’s environment and its board structure and the impact of this relation on organizational performance from the perspectives of both Agency Theory and Resource Dependence (Boundary Spanning) Theory. The impact of board characteristics on organizational performance is contextual. Speciﬁcally, we predict and show for a sample of U.S. nonproﬁts that board mechanisms related to monitoring are more likely to be effective for stable organizations, whereas board mechanisms related to boundary spanning are more effective for less stable organizations. We ﬁnd that the two theories are complementary and address different aspects of nonproﬁt performance, but the results are statistically stronger and more often consistent with resource dependence than with agency theory. Overall, this study supports Miller-Millesen’s (Nonproﬁt and Voluntary Sector Quarterly, 32: 521–547 2003) contention that, because the nonproﬁt environment is often more complex and heterogeneous than the for-proﬁt world, no one theory describes all tasks of nonproﬁt boards.</t>
@@ -3572,6 +4322,11 @@
       <c r="K74" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="18" customHeight="1" s="31">
       <c r="A75" s="0" t="inlineStr">
@@ -3584,6 +4339,16 @@
           <t>BSMA0072</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
           <t>Although network analysis is becoming a more viable and informative methodology for the study of interorganizational behavior, issues involving the accuracy and reliability of self-reported or ‘cognitive’ network data are still unresolved. Two networks based on information and coordination relationships in each of four major cities are examined. Reliability of responses is assessed as the percent of confirmed relationships between agency respondents and by correlating the extent of agreement in each network. In addition, two possible measurement errors are examined: systematic errors which are network-independent and idiosyncratic errors which are network-dependent. These errors are assessed through correlational analyses of the intensity of an organization's relationships with the number of its relationships that are confirmed in each network. Also systematic errors are accounted for by calculating the proportion of confirmed relationships within the different response categories used to judge the strength of relationship between ego organizations in the network. It is concluded that boundary spanning personnel of organizations can provide fairly reliable responses to network generated questions, but that errors in the data tend to be systematic in the way that prior studies of interpersonal cognitive networks report.</t>
@@ -3607,6 +4372,11 @@
       <c r="K75" s="0" t="n">
         <v>1993</v>
       </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="18" customHeight="1" s="31">
       <c r="A76" s="0" t="inlineStr">
@@ -3619,6 +4389,11 @@
           <t>BSMA0073</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
           <t>The offshoring of external audit work to so-called low-cost countries is prevalent among the Big 4 professional services firms. Despite this, our understanding of how this form of offshoring influences audit practitioners and the audit process is limited. This study examines how and why offshoring emerged as an organizational matter that changed the way audit work is organized in a Big 4 firm context. Our findings demonstrate how changes in the design of offshoring processes influence interactions between onshore and offshore auditors. We uncover how individual ‘‘boundary spanners’’ struggle to coordinate audit work across the multiple boundaries that separate onshore and offshore auditors. Furthermore, we show how the institutionalization of ‘‘boundary spanning’’ functions in organizational structures and processes can have the unintended consequence of widening the boundaries between onshore and offshore auditors. Finally, we offer evidence of the effect of offshoring on the learning process of onshore and offshore auditors.</t>
@@ -3642,6 +4417,11 @@
       <c r="K76" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="18" customHeight="1" s="31">
       <c r="A77" s="0" t="inlineStr">
@@ -3654,6 +4434,16 @@
           <t>BSMA0074</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
           <t>Despite the relevance of team boundary spanning in new product development (NPD), there is great deal we still do not know about these activities. For example, little is known about how these activities affect the development of team identification, an important emergent state with critical implications for new product performance. This study extends our understanding of this topic by exploring the relationship between team boundary spanning and team identification. This relationship is examined via the intervening mechanisms of team potency and team boundedness and the moderating effect of intra-team communication. Data from a time-lagged survey study of 140 NPD projects revealed that team potency and team boundedness, respectively, positively and negatively mediate the relationship between team boundary spanning and team identification. Intra-team communication was found to reduce the negative effect of team boundary spanning on team boundedness.</t>
@@ -3677,6 +4467,11 @@
       <c r="K77" s="0" t="n">
         <v>2025</v>
       </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="18" customHeight="1" s="31">
       <c r="A78" s="0" t="inlineStr">
@@ -3689,6 +4484,16 @@
           <t>BSMA0075</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
           <t>In today’s highly interconnected, uncertain, and dynamic business environment, team boundary spanning has become an important determinant of the performance of new product development (NPD) projects. Despite the positive evidence supporting the use of boundary spanning activities by NPD teams, little is still known about how boundary spanning teams become high-performance teams. The current study advances research on this subject by examining the mediating effect of team potency on the relationship between team boundary spanning and new product performance, as well as the moderating effects of team size and functional diversity on the relationship between team boundary spanning and team potency. Data from a time-lagged survey study of 140 NPD projects found that team boundary spanning can promote team potency which, in turn, results in greater product quality and new product creativity. The positive effect of team boundary spanning on team potency was found to be more pronounced for NPD teams of medium size and high levels of functional diversity.</t>
@@ -3712,6 +4517,11 @@
       <c r="K78" s="0" t="n">
         <v>2023</v>
       </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="18" customHeight="1" s="31">
       <c r="A79" s="0" t="inlineStr">
@@ -3724,6 +4534,16 @@
           <t>BSMA0076</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
           <t>Although team boundary spanning is conducive to achieving new product (NP) competitive advantage, these actions may not always deliver the expected performance. The current study makes an initial attempt to examine factors that undermine team boundary spanning positive effects on NP competitive advantage by proposing and testing a negative moderating effect of team social cohesion on the relationship between team boundary spanning and NP competitive advantage. Furthermore, the current study expects team social cohesion to have a stronger negative moderating effect on the relationship between team boundary spanning and NP competitive advantage when external task interdependence and project newness are high than when they are low. Data for this study come from 140 NPD projects developed and commercialized by Spanish manufacturing firms in high‐ and medium‐high‐technology sectors. The study’s results reveal a positive effect of team boundary spanning on NP competitive advantage. Furthermore, high levels of team social cohesion are shown to reduce the positive effect of team boundary spanning on NP competitive advantage. Finally, we found that project newness and external task interdependence accentuate the negative moderating effect of team social cohesion on the relationship between team boundary spanning and NP competitive advantage. The current study makes several contributions to the literature. First, findings from this study give us new insights into the significance of team boundary spanning to the success of NPs by revealing that boundary‐spanning activities are beneficial to achieving NP competitive advantage. Second, the study departs from existing research in that it exposes a dark side of team social cohesion for NPD teams engaged in boundary spanning activities. Last, the study expands extant research by proposing and demonstrating that project newness and external task interdependence bring about situations in which external groups present a threat to the collective identity of socially cohesive groups.</t>
@@ -3747,6 +4567,11 @@
       <c r="K79" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="18" customHeight="1" s="31">
       <c r="A80" s="0" t="inlineStr">
@@ -3759,6 +4584,11 @@
           <t>BSMA0077</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
           <t>Gender diversity pays off, particularly at senior levels in organizations. Companies with higher rates of gender diversity among senior leaders outperform their peers by a 15% margin; those with the highest percentages of female board directors enjoy as much as a two-thirds higher return on equity, sales, and invested capital. The key to occupying a high-level position in any organization is building an effective network of positive workplace relationships. Decades of research on organizational networks have shown that who you know–and who knows you–is critical to performance and career success. Full inclusion of both genders in informal organizational networks has been shown to drive productivity, innovation, and profitability. Full inclusion also supports individual well-being and deep engagement. Yet many leaders–both men and women–fail to develop gender-inclusive networks, potentially disadvantaging women since they are less likely to be connected to people in senior-level positions, given the overwhelming dominance of men in these roles. No wonder that feeling excluded from organizational networks has been identified as one of women’s top barriers to career success.</t>
@@ -3782,6 +4612,11 @@
       <c r="K80" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="18" customHeight="1" s="31">
       <c r="A81" s="0" t="inlineStr">
@@ -3794,6 +4629,16 @@
           <t>BSMA0078</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
           <t>Abstract             The defense industry in Israel has long been considered a critical platform for the development of the high‐technology sector. This study examines the importance of knowledge combination capability work units build through social relationships to enhance their performance. Specifically, we probe how both intraunit relational capital (within a unit) and interunit relational capital (across units) enable units to build knowledge combination capabilities and how such capabilities affect their performance. Data collected from senior managers in 122 knowledge units indicate that: (1) both intra‐ and interunit relational capital are positively related to knowledge combination capability; (2) knowledge combination capability is positively associated with enhanced unit performance; (3) knowledge combination capability fully mediates the relationship between interunit relational capital and unit performance; and (4) intraunit relational capital impacts both directly and indirectly (through knowledge combination capability) on unit performance. The findings suggest that interunit relational capital entails greater variation in knowledge stocks and thus may lead to more radical innovation than intra‐relational capital that entails more similar knowledge bases and, thus, produces more incremental innovations. Copyright © 2009 Strategic Management Society.</t>
@@ -3817,6 +4662,11 @@
       <c r="K81" s="0" t="n">
         <v>2009</v>
       </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="18" customHeight="1" s="31">
       <c r="A82" s="0" t="inlineStr">
@@ -3829,6 +4679,16 @@
           <t>BSMA0079</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
           <t>This study examines the relationships between joint work commitments, job satisfaction, and job performance of lawyers employed by private law firms in Israel. Based on Morrow’s (1993) concept of five universal forms of commitment, their interrelationship was tested with respect to the commitment model of Randall and Cote (1991), which appeared to show in previous studies (Cohen, 1999, 2000) a better fit compared to other models. In addition, the study examined the relationship between the commitment model and work attitude and outcome, namely, job satisfaction and job performance. The results show that the commitment model of Randall and Cote was almost fully supported, except for the relationship between job involvement and continuance commitment. This relationship is better understood via career commitment. An interesting finding of this study is that job satisfaction has a mediating role in the relationship between joint work commitment and job performance. The article concludes with suggestions regarding further investigation of the interrelationships between work commitment constructs, and the relationship between joint commitment forms, job satisfaction, and job performance.</t>
@@ -3852,6 +4712,11 @@
       <c r="K82" s="0" t="n">
         <v>2003</v>
       </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="18" customHeight="1" s="31">
       <c r="A83" s="0" t="inlineStr">
@@ -3864,6 +4729,16 @@
           <t>BSMA0080</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
           <t>This study analyzes the complex set of relationships among perceived organizational reputation, ﬁrm’s quality of products/services, customers’ satisfaction and multiple performance measures. A path analysis shows that reputation is inﬂuenced by customers’ satisfaction, which is a mediator in the relationship between the ﬁrm’s quality of products/services and reputation. Reputation is associated with the ﬁrm’s growth and accumulation of customers’ orders, but is not directly associated with market share, proﬁtability and ﬁnancial strength. Market share inﬂuences a ﬁrm’s profitability and is a function of the ﬁrm’s growth and accumulation of customers’ orders, but it has no inﬂuence on the ﬁrm’s ﬁnancial strength.</t>
@@ -3887,6 +4762,11 @@
       <c r="K83" s="0" t="n">
         <v>2005</v>
       </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="18" customHeight="1" s="31">
       <c r="A84" s="0" t="inlineStr">
@@ -3899,6 +4779,11 @@
           <t>BSMA0081</t>
         </is>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
           <t>Research on team leadership has primarily focused on leadership processes targeted within teams, in support of team objectives. Yet, teams are open systems that interact with other teams to achieve proximal as well as distal goals. This review clariﬁes that deﬁning ‘what’ constitutes functionally eﬀective leadership in interteam contexts requires greater precision with regard to where (within teams, across teams) and why (team goals, system goals) leadership processes are enacted, as well as greater consideration of when and among whom leadership processes arise. We begin by synthesizing ﬁndings from empirical studies published over the past 30 years that shed light on questions of what, where, why, when, and who related to interteam leadership and end by providing three overarching recommendations for how research should proceed in order to provide a more comprehensive picture of leadership in interteam contexts.</t>
@@ -3922,6 +4807,11 @@
       <c r="K84" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="18" customHeight="1" s="31">
       <c r="A85" s="0" t="inlineStr">
@@ -3934,6 +4824,16 @@
           <t>BSMA0082</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
           <t>Even though empirical studies examining leadership and effectiveness in multiteam systems (MTS) are on the rise, there is still much to learn about leading a complex “team of teams,” particularly in a field setting as opposed to a laboratory simulation. This study draws upon the multiteam systems and intergroup leadership theory literature streams to examine the role of systems thinking and leader identification as antecedents to intergroup leadership, arguing that higher levels of systems thinking and stronger leader identification with the MTS will enhance the efficacy of leader rhetoric targeted toward the development of an intergroup relational identity with boundary spanning acting as a positive moderating influence on this relationship. I further argue team functional diversity moderates the relationship between intergroup leadership and MTS effectiveness such that higher levels of intergroup leadership are needed to positively influence MTSs with higher levels of heterogeneity. Finally, team identification is evaluated for its predicted moderating effect on the relationship between intergroup leadership and MTS effectiveness such that identification with the MTS will have a positive effect on this relationship while identification with the component team will detract from it. Hypotheses were tested but not supported using a sample of 256 commanders at the squadron, group, and wing level organized in 180 MTSs within the Department of the Air Force. Supplemental analysis identified a significant positive moderating effect of systems thinking and a negative moderating effect of leader component team identification on the relationship between leader rhetoric and intergroup relational identity. Low levels of boundary spanning coupled with higher levels of intergroup relational identity resulted in lower MTS effectiveness while the opposite was true for high levels of boundary spanning and intergroup relational identity. The study concludes with a discussion of theoretical and practical implications as well as recommendations for future research.</t>
@@ -3957,6 +4857,11 @@
       <c r="K85" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="18" customHeight="1" s="31">
       <c r="A86" s="0" t="inlineStr">
@@ -3969,6 +4874,11 @@
           <t>BSMA0083</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
           <t>This study investigates the relationship between multiple role management strategies and knowledge spillovers across roles. We focus on a particular category of boundary-spanning professionals, the scholar-practitioners—professionals who work across the boundaries of academic and practice worlds—and apply a role theory lens to study (a) the sources of interrole conflict they experience at role boundaries, (b) the strategies of multiple role management they enact, and (c) the knowledge spillovers associated to such strategies. We develop a grounded model that describes three role management strategies, which occupy different positions on a role separation–integration continuum, and generate different mechanisms of knowledge spillover. Our study sheds light on the understudied relationship between role management strategies and knowledge consequences, and the type of tensions individuals experience in this process. In addition, we discuss how the strategic management of teaching, research, and practical application roles can help bridge academic and managerial practice worlds.</t>
@@ -3992,6 +4902,11 @@
       <c r="K86" s="0" t="n">
         <v>2018</v>
       </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="18" customHeight="1" s="31">
       <c r="A87" s="0" t="inlineStr">
@@ -4004,6 +4919,16 @@
           <t>BSMA0084</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
           <t>Since the collapse of the price of crude oil in the mid 1980s, some participants in the sector have overhauled their approach to learning for strategic advantage. The management teams dealing with the projects discussed here demonstrated an awareness that learning can be a core rigidity as well as a core competence, and set about institutionalizing new learning. The speed of learning was an important determinant of success, leading to substantial increases in project NPVs and a rapid reinvestment in the learning capabilities themselves. Learning about `boundary management' helps to distinguish areas where internal learning could develop proprietary competitive advantage, from those areas where valuable learning might best be achieved through alliance.</t>
@@ -4027,6 +4952,11 @@
       <c r="K87" s="0" t="n">
         <v>1999</v>
       </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="18" customHeight="1" s="31">
       <c r="A88" s="0" t="inlineStr">
@@ -4039,6 +4969,16 @@
           <t>BSMA0085</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
           <t>Adopting a microfoundations approach to the analysis of intra-multinational enterprise (MNE) knowledge integration, we focus on mobile inventors and their boundary-spanning experience. Using inventor-patent data on US-based MNEs, we show that intra-organizational cross-border mobility and inter-organizational mobility have respectively a positive and a negative effect on knowledge integration. Cross-border mobility within the MNE enables the temporary co-location of mobile inventors in different units, facilitating the dissemination of their knowledge within the MNE. Conversely, “job-hopping” inventors may remain organizational outsiders, which hinders their ability to foster intra-MNE knowledge integration.</t>
@@ -4062,6 +5002,11 @@
       <c r="K88" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="18" customHeight="1" s="31">
       <c r="A89" s="0" t="inlineStr">
@@ -4074,6 +5019,16 @@
           <t>BSMA0086</t>
         </is>
       </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
           <t>The identification and management of work dependencies is a fundamental challenge in software development organizations. This paper argues that modularization, the traditional technique intended to reduce interdependencies among components of a system, has serious limitations in the context of software development. We build on the idea of congruence, proposed in our prior work, to examine the relationship between the structure of technical and work dependencies and the impact of dependencies on software development productivity. Our empirical evaluation of the congruence framework showed that when developers’ coordination patterns are congruent with their coordination needs, the resolution time of modification requests was significantly reduced. Furthermore, our analysis highlights the importance of identifying the “right” set of technical dependencies that drive the coordination requirements among software developers. Call and data dependencies appear to have far less impact than logical dependencies.</t>
@@ -4097,6 +5052,11 @@
       <c r="K89" s="0" t="n">
         <v>2008</v>
       </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="18" customHeight="1" s="31">
       <c r="A90" s="0" t="inlineStr">
@@ -4109,6 +5069,16 @@
           <t>BSMA0087</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
           <t>Prior research on the impact of organizational memory on new product success has divergent perspectives. Such inconsistency has accrued mainly from not considering memory's multifaceted aspects, which interact with specific project characteristics. This paper tries to sort out this paradox by proposing that project innovativeness moderates the relationship among variables of organizational memory and new product success. An empirical study of 169 NPD projects of Korean manufacturing firms finds that memory sharing and the use of external information and formal procedures enhance new product success, whereas organizational memory has no effect. Project innovativeness is found to moderate memory's effect, despite some tradeoffs. As innovativeness increases, the effect of organizational memory and use of external information become stronger whereas the effect of memory sharing and use of formal procedures weaken. This suggests that firms must activate organizational memory more carefully according to project characteristics and the memory level to maximize its positive effects.</t>
@@ -4132,6 +5102,11 @@
       <c r="K90" s="0" t="n">
         <v>2008</v>
       </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="18" customHeight="1" s="31">
       <c r="A91" s="0" t="inlineStr">
@@ -4144,6 +5119,16 @@
           <t>BSMA0088</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
           <t>This study investigates how post-M&amp;A interdepartmental integration affects the efficiency and effectiveness of new product development (NPD).The total sample size was 251 respondents. Confirmatory factor analysis (CFA) and structural equation modeling (SEM) were used for statistical analysis. Analytical results indicate that, although collaboration interdepartmental integration positively correlates with product vision, interaction interdepartmental interaction integration does not reach a significant level. Despite the fact that some interaction is essential when developing new product competitive advantage (NPCA), such interaction does not necessarily achieve success. Further, product vision positively correlates with new product competitive advantage and NPD performance, and new product competitive advantage positively correlates with NPD performance. In addition, an examination of the mediation effect in terms of Sobel t-test reveals that product vision is a significant mediator for the influence of interdepartmental integration on new product competitive advantage, while the new product competitive advantage is also a significant mediator for the influence of interdepartmental integration on NPD performance. Moreover, this study provides a framework for managing post-M&amp;A integration and closes with a discussion of the theoretical and practical implications of the research findings.</t>
@@ -4167,6 +5152,11 @@
       <c r="K91" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="18" customHeight="1" s="31">
       <c r="A92" s="0" t="inlineStr">
@@ -4179,6 +5169,16 @@
           <t>BSMA0089</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
           <t>Digital transformation accelerates the boundary reshaping of firms’ R&amp;D cooperation and knowledge bases, bringing opportunities for breakthrough innovation following overseas mergers and acquisitions (M&amp;A). Unlike previous studies that have focused separately on digital transformation and overseas M&amp;A integration, this paper aims to explore their synergy effects on firms’ breakthrough innovation from a boundary-spanning perspective. Based on samples of Chinese manufacturing firms’ technology-sourcing overseas M&amp;A from 2012 to 2019, our empirical results show that boundary spanning in R&amp;D cooperation networks and knowledge networks mediate the synergy effects of digital transformation and appropriate overseas M&amp;A integration on firms’ breakthrough innovation. This paper not only complements recent studies that combine digital transformation and boundary-spanning theories, but also provides a deeper understanding of the relationship between boundary spanning and breakthrough innovation in the digital context. It offers important theoretical and practical insights into overseas M&amp;A and innovation in the digital era.</t>
@@ -4202,6 +5202,11 @@
       <c r="K92" s="0" t="n">
         <v>2026</v>
       </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="18" customHeight="1" s="31">
       <c r="A93" s="0" t="inlineStr">
@@ -4214,6 +5219,11 @@
           <t>BSMA0090</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
           <t>In the face of increasing global uncertainty, multinational enterprises (MNEs) have turned to downsizing to maintain profitability while emphasizing lateral collaboration to increase productivity. Here, we establish a conceptual framework and examine from a macro‐to‐micro perspective how the growing subjects of subsidiary role change, team alignment and employee engagement impact lateral collaboration. We used structural equation modelling to analyse the results of 252 surveys given to MNE subsidiaries in the Taiwanese banking industry and found that employee engagement was central to driving lateral collaboration effectiveness, indicating that the subsidiary role is critical for boundary‐spanning activities and building bridges between various teams. These activities in turn enhance subsidiary performance and lead to better people development. Our findings demonstrate that bundling employee engagement with human resource practices is a strategic way of positioning for the evolution of subsidiary management.</t>
@@ -4237,6 +5247,11 @@
       <c r="K93" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="18" customHeight="1" s="31">
       <c r="A94" s="0" t="inlineStr">
@@ -4249,6 +5264,11 @@
           <t>BSMA0091</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
           <t>This paper investigates the impact of boundary-spanning search on innovation performance, with knowledge recombination as the underlying mechanism. It also explores the contingent eﬀect of in house training of employees by considering not invented here syndrome derived from attitude theory, and examines communication investment as a second-order moderator. We test the hypotheses based on a sample of 184 Hong Kong manufacturing ﬁrms. The results show that boundary-spanning search is positively related to innovation performance, which is negatively moderated by in house training of employees. Moreover, communication investment has a suppressing eﬀect on the moderating role of in house training of employees. This paper highlights the not invented here syndrome and its mechanism of attitude theory to examine the contingent eﬀects, providing insights for managers to balance among in house training of employees, communication investment, and boundary-spanning search to enhance innovation performance.</t>
@@ -4272,6 +5292,11 @@
       <c r="K94" s="0" t="n">
         <v>2024</v>
       </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="18" customHeight="1" s="31">
       <c r="A95" s="0" t="inlineStr">
@@ -4284,6 +5309,16 @@
           <t>BSMA0092</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G95" s="0" t="inlineStr">
         <is>
           <t>While there is a burgeoning trend to recognize leadership as an important enabler of new venture development and growth, scant research has explored the performance mechanisms of shared leadership in the entrepreneurial context. Based on the information processing perspective, we propose a moderated mediation model to examine how shared leadership in entrepreneurial teams advance new venture performance by identifying team reflexivity as a pivotal mediator and team boundary spanning as a crucial contingency. The data set from a cross-industry sample of 94 entrepreneurial teams indicated that shared leadership exerts a positive indirect influence on new venture performance via team reflexivity; and team boundary spanning moderates such indirect influence. Finally, how our findings contribute to the entrepreneurship, leadership, team research, and managerial practice are discussed.</t>
@@ -4307,6 +5342,11 @@
       <c r="K95" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="18" customHeight="1" s="31">
       <c r="A96" s="0" t="inlineStr">
@@ -4319,6 +5359,11 @@
           <t>BSMA0093</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
           <t>Getting professionals who have been selected and trained to perform individually to work together is a major challenge. The objective of the article is to identify the mechanisms by which a coordinator can ensure a mediation and boundary spanning role to enable the achievement of a project. Adopting a comprehensive approach, this article is based on the case of an innovative hospital project ‘One-Day Diagnosis’ (1DD) – one day instead of several weeks – of hepatobiliary and pancreatic pathologies, for which the professionals had to change their practices. Based on the results of the study, the ﬁndings show that the mediating role of the coordinator consists in making things happen and guiding health care professionals through the innovative pathway until it becomes a routine process. The study contributes to the literature on collaboration and relational coordination by highlighting that the change of practices for collaboration is compatible with personal excellence, by outlining the active role of the boundary spanner in the change of these practices and by demonstrating that the organizational stability of projects based on disembodied procedures is a necessary illusion that requires complementary interindividual relationships and a living leadership.</t>
@@ -4342,6 +5387,11 @@
       <c r="K96" s="0" t="n">
         <v>2024</v>
       </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="18" customHeight="1" s="31">
       <c r="A97" s="0" t="inlineStr">
@@ -4354,6 +5404,11 @@
           <t>BSMA0094</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
           <t>The current study examined the relationships among role stress, proactive personality, employee creativity, and customer-oriented boundary spanning behaviors (COBSBs) for frontline service employees (FSEs). This study collected data from 382 FSEs in international hotels in Taiwan to test the research model. The empirical results revealed that employee creativity was positively affected by proactive personality but negatively affected by role conflict and role ambiguity. FSEs’ creativity positively affects COBSBs, including external representation, internal influence, and service delivery. Internal influence also positively affects service delivery and mediates the relationship between FSEs’ creativity and service delivery.</t>
@@ -4377,6 +5432,11 @@
       <c r="K97" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="18" customHeight="1" s="31">
       <c r="A98" s="0" t="inlineStr">
@@ -4389,6 +5449,11 @@
           <t>BSMA0095</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
           <t>A number of studies have found that the performance of NPD projects greatly depends on the support they get from top management. However, research into why some projects get more support than others has been limited. The present paper takes a political approach to NPD, in which top management support is considered to be a function of a project leader’s ability to influence decision processes through personal relationships. Mobilizing the bridging perspective of social capital, we argue that project leaders need both strong ties to high-ranking others and sparseness in their networks. Vertical strong ties bring direct support and solidarity, resulting in improved access to resources and priority over other projects; sparseness provides exposure to the full range of information and interpretations in the organization, resulting in a more accurate picture of the political landscape and thus enabling the implementation of an appropriate influence strategy. A PLS analysis of a sample of 73 French project leaders involved in NPD projects provided support for our hypotheses. Hence, we contribute to a very recent stream of research showing that the structural and relational dimensions of social capital are complementary.</t>
@@ -4412,6 +5477,11 @@
       <c r="K98" s="0" t="n">
         <v>2012</v>
       </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="18" customHeight="1" s="31">
       <c r="A99" s="0" t="inlineStr">
@@ -4424,6 +5494,16 @@
           <t>BSMA0096</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G99" s="0" t="inlineStr">
         <is>
           <t>Though most acculturation research investigates movement across national boundaries, many other types of boundaries may exist (e.g. rural to urban migration). Rural migrant workers focus on their adaptive and exploratory consumption practices to assemble a liquid identity in China. In essence, this research examines the nature of the transitions that the vast group of Chinese (over 280 million) endures as migrant workers seek to assemble new identities through consumption activities in a liminal space. We find that family relations and government policy hinder migrants’ adjustments to urban life. Thus, we contribute to macromarketing by enriching the theories of liquid identity, boundary work, and acculturation.</t>
@@ -4447,6 +5527,11 @@
       <c r="K99" s="0" t="n">
         <v>2018</v>
       </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="18" customHeight="1" s="31">
       <c r="A100" s="0" t="inlineStr">
@@ -4459,6 +5544,16 @@
           <t>BSMA0097</t>
         </is>
       </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G100" s="0" t="inlineStr">
         <is>
           <t>This dissertation examined the relationships between organizational characteristics and firms' timing of entry into emerging product markets. This study is an extension of a stream of research on endogenous entry models. Research on this area essentially holds that not all firms have the same entry skills and costs. Therefore, a firm's entry timing decision is attributable to factors internal to the organization. In this dissertation, specific attention is directed toward the effects of top management team (TMT) demography, corporate governance, level of diversification, boundary spanning, past performance, capital structure, and firm size on entry timing. These organizational characteristics have been shown to be critical determinants of timing in the strategic management literature, but, remain almost unexplored in the entry timing research. Thus, through including these organizational characteristics, this study extends the current knowledge which is critical for answering the question: Why do some firms enter emerging product markets earlier/later than others?</t>
@@ -4482,6 +5577,11 @@
       <c r="K100" s="0" t="n">
         <v>1995</v>
       </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="18" customHeight="1" s="31">
       <c r="A101" s="0" t="inlineStr">
@@ -4494,6 +5594,11 @@
           <t>BSMA0098</t>
         </is>
       </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G101" s="0" t="inlineStr">
         <is>
           <t>Organisations experience increased social, political and economic pressure that is evident in the increased pressure that stakeholders place on organisations. Organisations increasingly realise that stakeholders’ values and objectives need to be incorporated into organisational strategy as well as the day-to-day management of the organisation. Organisational success and survival consequently depends on the organisation’s network of relationships, which provide the organisation with otherwise inaccessible resources and a competitive advantage.</t>
@@ -4517,6 +5622,11 @@
       <c r="K101" s="0" t="n">
         <v>2008</v>
       </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="18" customHeight="1" s="31">
       <c r="A102" s="0" t="inlineStr">
@@ -4529,6 +5639,11 @@
           <t>BSMA0099</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G102" s="0" t="inlineStr">
         <is>
           <t>In this dissertation, I develop a conceptual model for how managers' roles as boundary spanners within their organizations affect the perceptions, attitudes, relationships, and performance of their subordinate employees. Drawing on literatures in social networks, status characteristics theory, social identity theory, and resource allocation theory, I suggest that managers' external relationships—the connections that managers make to organization members outside of their subordinate work group—have a material impact on their subordinates' perceptions of their work environment and their managers. These perceptions, I argue, serve as four specific mechanisms in an indirect effects model that connect managers' external relationship to their employees' task performance and work attitudes (eg organizational commitment) and the Leader Member Exchange (LMX) relationships between manager and subordinate. I apply the theoretical model to two salient types of managerial relationships: those with their bosses and those with their horizontal peers.</t>
@@ -4552,6 +5667,11 @@
       <c r="K102" s="0" t="n">
         <v>2011</v>
       </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="18" customHeight="1" s="31">
       <c r="A103" s="0" t="inlineStr">
@@ -4564,6 +5684,11 @@
           <t>BSMA0100</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
           <t>This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates, with a secondary goal of testing product complexity as a moderator. We develop suitable hypotheses under the theoretical lens of cognitive load theory. The empirical study uses archival data on an ordinary least squares model to find significant associations between collaboration structure, product complexity and the learning rates exhibited by 230 development teams producing open source software. Results show two distinct subgroups of projects: The first subgroup exhibits an average 78% learning rate, and the other subgroup “unlearned”, i.e., productivity deteriorated over time instead of improved. In the learning subgroup, collaboration network density negatively impacted learning, while product complexity interacted with collaboration network centralisation and boundary spanning activity. In the unlearning subgroup, only network density impacted learning rates and no moderating effects were found. Practical implications and future opportunities for research are discussed.</t>
@@ -4587,6 +5712,11 @@
       <c r="K103" s="0" t="n">
         <v>2016</v>
       </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="18" customHeight="1" s="31">
       <c r="A104" s="0" t="inlineStr">
@@ -4599,6 +5729,11 @@
           <t>BSMA0101</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G104" s="0" t="inlineStr">
         <is>
           <t>The state of software development performance is far from being exemplar, with a success rate well below that of other industries, and understanding how to improve these projects is not only substantive but urgent. Software development is at most times a collaborative effort, yet we do not understand clearly how different collaboration structures associate with development performance metrics. This paper empirically examines the association between collaboration patterns, project productivity and product quality through a field study of working software open source new product development teams, using archival data from electronic sources related to Open Source Software projects. Collaboration structures are measured using Social Network Analysis and in terms of their network density, network centralization and the level of boundary spanning activity of team members. Productivity and quality are measured using "hard", code-based metrics. Results of regression analyses testing relevant hypotheses suggest that project managers need to strongly encourage internal collaboration, but be wary of allowing team members to participate in multiple projects. The breadth of skills within the team is a tactical asset that may increase the efficient frontier in the quality–productivity trade-off. Results also show that centralized structures associate with higher product quality and development productivity.</t>
@@ -4622,6 +5757,11 @@
       <c r="K104" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="18" customHeight="1" s="31">
       <c r="A105" s="0" t="inlineStr">
@@ -4634,6 +5774,11 @@
           <t>BSMA0102</t>
         </is>
       </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G105" s="0" t="inlineStr">
         <is>
           <t>Technology Transfer Centres (TTCs) have been analyzed in the last few years by focusing on the relationship between a TTC, provider of knowledge-intensive services, and a ﬁrm client-receiver. Less attention has been devoted to a more complex relationship which involves in the dyadic provider-receiver tie a third relevant body, University. We provide both a theoretical and an empirical contribution by studying whether TTCs can bond the academic and industrial system and we deﬁne the activities that make-up this role such as: scanning and selection of R&amp;D opportunities, bridge building, semantic translation of domain speciﬁc knowledge, co-production of new knowledge. The boundary spanning role of TTCs is discussed drawing on different and complementary theoretical perspectives. Moreover, we test research hypotheses on the antecedents of boundary spanning activity from a knowledge-based perspective. We argue that TTC boundary spanners need to leverage on both technical skills and networking competences. Empirical investigation has been carried out with a survey of the TTC population of North East Italy. The research ﬁndings highlight the task coordination activities implied by a boundary spanning role in joint R&amp;D projects and show that the endowment of human capital at individual level and a qualiﬁed social capital at individual and organizational level are the main determinants.</t>
@@ -4657,6 +5802,11 @@
       <c r="K105" s="0" t="n">
         <v>2012</v>
       </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="18" customHeight="1" s="31">
       <c r="A106" s="0" t="inlineStr">
@@ -4669,6 +5819,11 @@
           <t>BSMA0103</t>
         </is>
       </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G106" s="0" t="inlineStr">
         <is>
           <t>This paper contributes to open innovation (OI) and boundary spanning literatures by providing a first understanding of industry‐based boundary spanners in university‐industry (U‐I) collaboration through case studies of Chinese multinational corporations (MNCs) and their international OI platforms. Organisational roles created by these platforms within the MNCs and their activity of bridging between organisations are examined. The analysis of 25 in‐depth interviews in two MNCs located in eight countries, along with internal documents, sheds light on U‐I collaboration practices implemented by Chinese MNCs. Two new boundary spanning roles are identified:               Dual Cultural Bridger               – as these OI platforms bridge organisational and national cultural gaps to prevent and solve problems in the collaborative process; and               International Network Enhancer               – as these OI platforms act as trust building and local knowledge listening posts for the MNC’s global network. Managerial and policy implications are provided.</t>
@@ -4692,6 +5847,11 @@
       <c r="K106" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="18" customHeight="1" s="31">
       <c r="A107" s="0" t="inlineStr">
@@ -4704,6 +5864,16 @@
           <t>BSMA0104</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G107" s="0" t="inlineStr">
         <is>
           <t>This dissertation examines network ties among organizations, and their impact on innovation. The analyses focus on technical exchanges between firms and their suppliers and customers, both in terms of the factors that lead firms to engage in such boundary-spanning activities, and the relationship between these boundary-spanning activities and new product development.</t>
@@ -4727,6 +5897,11 @@
       <c r="K107" s="0" t="n">
         <v>1999</v>
       </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="18" customHeight="1" s="31">
       <c r="A108" s="0" t="inlineStr">
@@ -4739,6 +5914,16 @@
           <t>BSMA0105</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G108" s="0" t="inlineStr">
         <is>
           <t>This cross-sectional study (conducted in April–May 2011) explored associations between partnership functioning synergy and sustainability of innovative programmes in community care. The study sample consisted of 106 professionals (of 244 individuals contacted) participating in 21 partnerships that implemented different innovative community care programmes in Rotterdam, The Netherlands. Partnership functioning was evaluated by assessing leadership, resources administration and efﬁciency. Synergy was considered the proximal outcome of partnership functioning, which, in turn, inﬂuenced the achievement of programme sustainability. On a 5-point scale of increasing sustainability, mean sustainability scores ranged from 1.9 to 4.9. The results of the regression analysis demonstrated that sustainability was positively inﬂuenced by leadership (standardised regression coefﬁcient b = 0.32; P &lt; 0.001) and non-ﬁnancial resources (b = 0.25; P = 0.008). No signiﬁcant relationship was found between administration or efﬁciency and programme sustainability. Partnership synergy acted as a mediator for partnership functioning and signiﬁcantly affected sustainability (b = 0.39; P &lt; 0.001). These ﬁndings suggest that the sustainability of innovative programmes in community care is achieved more readily when synergy is created between partners. Synergy was more likely to emerge with boundaryspanning leaders, who understood and appreciated partners’ different perspectives, and could bridge their diverse cultures and were comfortable sharing ideas, resources and power. In addition, the acknowledgement of and ability to use members’ resources were found to be valuable in engaging partners’ involvement and achieving synergy in community care partnerships.</t>
@@ -4762,6 +5947,11 @@
       <c r="K108" s="0" t="n">
         <v>2013</v>
       </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="18" customHeight="1" s="31">
       <c r="A109" s="0" t="inlineStr">
@@ -4774,6 +5964,11 @@
           <t>BSMA0106</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G109" s="0" t="inlineStr">
         <is>
           <t>Previous research demonstrates the dysfunctional consequences of high levels of role stressors (role ambiguity and role conflict) in boundary-spanning positions. These consequences include higher levels of burnout and lower levels of satisfaction and performance. Although marketing researchers have investigated external mechanisms for coping with role stressors, research to date has not investigated the inherent capability of boundary spanners to cope with role stressors. This research examines optimism as an internal characteristic that facilitates coping with role stressors in boundary-spanning positions. The research findings reveal that optimists are able to anticipate and respond proactively to stressors, resulting in less burnout and higher levels of performance and satisfaction.</t>
@@ -4797,6 +5992,11 @@
       <c r="K109" s="0" t="n">
         <v>2009</v>
       </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="18" customHeight="1" s="31">
       <c r="A110" s="0" t="inlineStr">
@@ -4809,6 +6009,16 @@
           <t>BSMA0107</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G110" s="0" t="inlineStr">
         <is>
           <t>In this paper, we highlight the networked context of the professions. In particular, we indicate that neo-classical professionals tend to work across organizational boundaries in project teams, often to meet the needs of clients and the wider society. However, little is known about the resources that professionals draw on to meet immediate, fast paced, client demands in project network organizations (PNOs). We pinpoint how knowledge resources, human, social and organizational capital enable professionals to produce outputs at a fast pace/tempo. Temporality emerged as an unexpected but key issue in our empirical research and we explore this further here. First, we put forward how professional work organization(s) has changed by focusing on the boundaries of organizations, and how this is often temporary and project-driven. Second, we use the speciﬁc lens of knowledge resources which are drawn upon to enable networked working and ask the question: which knowledge resources enable professionals to work at a fast pace within networks? Third, appreciative of the vast literature on temporary and networked organizations in professional work, our focus is beyond a single profession or organization, and hence, we build upon the prior research on PNOs. We do this by drawing on empirical data of a humanitarian aid project networked organization (HN) that upscales across its network at high speed, often within days, to generate funds for humanitarian disasters in order to save lives.</t>
@@ -4832,6 +6042,11 @@
       <c r="K110" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="18" customHeight="1" s="31">
       <c r="A111" s="0" t="inlineStr">
@@ -4844,6 +6059,16 @@
           <t>BSMA0108</t>
         </is>
       </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G111" s="0" t="inlineStr">
         <is>
           <t>This research examines the mechanisms through which entrepreneurial orientation (EO) aﬀects ﬁrm performance in an emerging market context. We argue that EO drives ﬁrms to develop the dynamic capabilities of absorptive capacity (ACAP) and boundary-spanning (BS), and that these capabilities enhance ﬁrm performance. Moreover, the eﬀectiveness of these knowledge- and network-based dynamic capabilities in mediating the EOperformance relationship is contingent on the institutional conditions ﬁrms are exposed to. We test our hypotheses using multi-sourced data on Chinese high-tech ﬁrms in business-to-business (B2B) markets. Our results show that ACAP and BS mediate the positive eﬀect of EO on ﬁrm performance, and that as the development of market-supporting institutions improves, the mediating eﬀect of ACAP becomes stronger while that of BS weakens.</t>
@@ -4867,6 +6092,11 @@
       <c r="K111" s="0" t="n">
         <v>2018</v>
       </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="18" customHeight="1" s="31">
       <c r="A112" s="0" t="inlineStr">
@@ -4879,6 +6109,11 @@
           <t>BSMA0109</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G112" s="0" t="inlineStr">
         <is>
           <t>Effective work groups engage in external knowledge sharing—the exchange of information, know-how, and feedback with customers, organizational experts, and others outside of the group. This paper argues that the value of external knowledge sharing increases when work groups are more structurally diverse. A structurally diverse work group is one in which the members, by virtue of their different organizational affiliations, roles, or positions, can expose the group to unique sources of knowledge. It is hypothesized that if members of structurally diverse work groups engage in external knowledge sharing, their performance will improve because of this active exchange of knowledge through unique external sources. A field study of 182 work groups in a Fortune 500 telecommunications firm operationalizes structural diversity as member differences in geographic locations, functional assignments, reporting managers, and business units, as indicated by corporate database records. External knowledge sharing was measured with group member surveys and performance was assessed using senior executive ratings. Ordered logit analyses showed that external knowledge sharing was more strongly associated with performance when work groups were more structurally diverse. Implications for theory and practice around the integration of work groups and social networks are addressed.</t>
@@ -4902,6 +6137,11 @@
       <c r="K112" s="0" t="n">
         <v>2004</v>
       </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="18" customHeight="1" s="31">
       <c r="A113" s="0" t="inlineStr">
@@ -4914,6 +6154,16 @@
           <t>BSMA0110</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G113" s="0" t="inlineStr">
         <is>
           <t>Our study responds to a call for research to integrate institutional, organizational and individual levels of analysis in examining the implications for work and employment relations of new organizational forms. We empirically examine the implementation of network forms of genetics healthcare delivery that cross organizational and professional boundaries. We highlight that less powerful professional groups may find difficulty in enacting boundary-spanning roles associated with new organizational forms. This is due, first, to inconsistency of government policy, which fragments organizations. Second, professional institutions sustain professional hierarchy and power differentials.</t>
@@ -4936,6 +6186,11 @@
       </c>
       <c r="K113" s="0" t="n">
         <v>2008</v>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
       </c>
     </row>
     <row r="114" ht="18" customHeight="1" s="31">

</xml_diff>

<commit_message>
Screening: Completed 1st screening judgments for NO. 111 to NO. 210 (100 papers)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -1407,12 +1407,12 @@
           <t>BSMA0011</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -1440,7 +1440,7 @@
       <c r="K14" s="0" t="n">
         <v>2014</v>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="P14" s="0" t="inlineStr">
         <is>
           <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
@@ -1457,12 +1457,12 @@
           <t>BSMA0012</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -1490,7 +1490,7 @@
       <c r="K15" s="0" t="n">
         <v>2026</v>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" s="0" t="inlineStr">
         <is>
           <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
         </is>
@@ -1507,12 +1507,12 @@
           <t>BSMA0013</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -1540,7 +1540,7 @@
       <c r="K16" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P16" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -1557,7 +1557,7 @@
           <t>BSMA0014</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -1585,7 +1585,7 @@
       <c r="K17" s="0" t="n">
         <v>2014</v>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="P17" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -1602,12 +1602,12 @@
           <t>BSMA0015</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -1635,7 +1635,7 @@
       <c r="K18" s="0" t="n">
         <v>1993</v>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="P18" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -1652,7 +1652,7 @@
           <t>BSMA0016</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -1680,7 +1680,7 @@
       <c r="K19" s="0" t="n">
         <v>2026</v>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="P19" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -1697,7 +1697,7 @@
           <t>BSMA0017</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -1725,7 +1725,7 @@
       <c r="K20" s="0" t="n">
         <v>2015</v>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="P20" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -1742,12 +1742,12 @@
           <t>BSMA0018</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -1775,7 +1775,7 @@
       <c r="K21" s="0" t="n">
         <v>1990</v>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="P21" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -1792,7 +1792,7 @@
           <t>BSMA0019</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -1820,7 +1820,7 @@
       <c r="K22" s="0" t="n">
         <v>1992</v>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="P22" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -1837,12 +1837,12 @@
           <t>BSMA0020</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -1870,7 +1870,7 @@
       <c r="K23" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="P23" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -1887,7 +1887,7 @@
           <t>BSMA0021</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -1915,7 +1915,7 @@
       <c r="K24" s="0" t="n">
         <v>2013</v>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="P24" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -1932,7 +1932,7 @@
           <t>BSMA0022</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -1963,7 +1963,7 @@
       <c r="K25" s="0" t="n">
         <v>1995</v>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="P25" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -1980,7 +1980,7 @@
           <t>BSMA0023</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2008,7 +2008,7 @@
       <c r="K26" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="P26" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2025,7 +2025,7 @@
           <t>BSMA0024</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2053,7 +2053,7 @@
       <c r="K27" s="0" t="n">
         <v>2017</v>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2070,12 +2070,12 @@
           <t>BSMA0025</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -2103,7 +2103,7 @@
       <c r="K28" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="P28" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -2120,7 +2120,7 @@
           <t>BSMA0026</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2148,7 +2148,7 @@
       <c r="K29" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="P29" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2165,12 +2165,12 @@
           <t>BSMA0027</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -2198,7 +2198,7 @@
       <c r="K30" s="0" t="n">
         <v>2007</v>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="P30" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -2215,12 +2215,12 @@
           <t>BSMA0028</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -2248,7 +2248,7 @@
       <c r="K31" s="0" t="n">
         <v>2000</v>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="P31" s="0" t="inlineStr">
         <is>
           <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
         </is>
@@ -2265,12 +2265,12 @@
           <t>BSMA0029</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -2298,7 +2298,7 @@
       <c r="K32" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="P32" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -2315,12 +2315,12 @@
           <t>BSMA0030</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -2348,7 +2348,7 @@
       <c r="K33" s="0" t="n">
         <v>2002</v>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="P33" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -2365,12 +2365,12 @@
           <t>BSMA0031</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -2398,7 +2398,7 @@
       <c r="K34" s="0" t="n">
         <v>2026</v>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="P34" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -2415,12 +2415,12 @@
           <t>BSMA0032</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -2448,7 +2448,7 @@
       <c r="K35" s="0" t="n">
         <v>1990</v>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="P35" s="0" t="inlineStr">
         <is>
           <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
         </is>
@@ -2465,7 +2465,7 @@
           <t>BSMA0033</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2493,7 +2493,7 @@
       <c r="K36" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P36" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2510,7 +2510,7 @@
           <t>BSMA0034</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2538,7 +2538,7 @@
       <c r="K37" s="0" t="n">
         <v>2000</v>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="P37" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2555,7 +2555,7 @@
           <t>BSMA0035</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2583,7 +2583,7 @@
       <c r="K38" s="0" t="n">
         <v>2023</v>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="P38" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2600,12 +2600,12 @@
           <t>BSMA0036</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -2633,7 +2633,7 @@
       <c r="K39" s="0" t="n">
         <v>1997</v>
       </c>
-      <c r="P39" t="inlineStr">
+      <c r="P39" s="0" t="inlineStr">
         <is>
           <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
@@ -2650,12 +2650,12 @@
           <t>BSMA0037</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -2683,7 +2683,7 @@
       <c r="K40" s="0" t="n">
         <v>2001</v>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="P40" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -2700,12 +2700,12 @@
           <t>BSMA0038</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -2733,7 +2733,7 @@
       <c r="K41" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="P41" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -2750,7 +2750,7 @@
           <t>BSMA0039</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2778,7 +2778,7 @@
       <c r="K42" s="0" t="n">
         <v>2008</v>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="P42" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2795,12 +2795,12 @@
           <t>BSMA0040</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -2828,7 +2828,7 @@
       <c r="K43" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P43" t="inlineStr">
+      <c r="P43" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -2845,7 +2845,7 @@
           <t>BSMA0041</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2873,7 +2873,7 @@
       <c r="K44" s="0" t="n">
         <v>2014</v>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="P44" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2890,12 +2890,12 @@
           <t>BSMA0042</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -2923,7 +2923,7 @@
       <c r="K45" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P45" t="inlineStr">
+      <c r="P45" s="0" t="inlineStr">
         <is>
           <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
         </is>
@@ -2940,7 +2940,7 @@
           <t>BSMA0043</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -2968,7 +2968,7 @@
       <c r="K46" s="0" t="n">
         <v>2015</v>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="P46" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -2985,7 +2985,7 @@
           <t>BSMA0044</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3013,7 +3013,7 @@
       <c r="K47" s="0" t="n">
         <v>1985</v>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="P47" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3030,7 +3030,7 @@
           <t>BSMA0045</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3058,7 +3058,7 @@
       <c r="K48" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="P48" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3075,7 +3075,7 @@
           <t>BSMA0046</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E49" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3103,7 +3103,7 @@
       <c r="K49" s="0" t="n">
         <v>2001</v>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="P49" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3120,12 +3120,12 @@
           <t>BSMA0047</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -3153,7 +3153,7 @@
       <c r="K50" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="P50" s="0" t="inlineStr">
         <is>
           <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
         </is>
@@ -3170,7 +3170,7 @@
           <t>BSMA0048</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3198,7 +3198,7 @@
       <c r="K51" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P51" t="inlineStr">
+      <c r="P51" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3215,7 +3215,7 @@
           <t>BSMA0049</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3243,7 +3243,7 @@
       <c r="K52" s="0" t="n">
         <v>2019</v>
       </c>
-      <c r="P52" t="inlineStr">
+      <c r="P52" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3260,7 +3260,7 @@
           <t>BSMA0050</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3288,7 +3288,7 @@
       <c r="K53" s="0" t="n">
         <v>2014</v>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="P53" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3305,12 +3305,12 @@
           <t>BSMA0051</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -3338,7 +3338,7 @@
       <c r="K54" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P54" t="inlineStr">
+      <c r="P54" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -3355,7 +3355,7 @@
           <t>BSMA0052</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E55" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3383,7 +3383,7 @@
       <c r="K55" s="0" t="n">
         <v>2015</v>
       </c>
-      <c r="P55" t="inlineStr">
+      <c r="P55" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3400,7 +3400,7 @@
           <t>BSMA0053</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E56" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3428,7 +3428,7 @@
       <c r="K56" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P56" t="inlineStr">
+      <c r="P56" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3445,7 +3445,7 @@
           <t>BSMA0054</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3473,7 +3473,7 @@
       <c r="K57" s="0" t="n">
         <v>2003</v>
       </c>
-      <c r="P57" t="inlineStr">
+      <c r="P57" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3490,7 +3490,7 @@
           <t>BSMA0055</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3518,7 +3518,7 @@
       <c r="K58" s="0" t="n">
         <v>2005</v>
       </c>
-      <c r="P58" t="inlineStr">
+      <c r="P58" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3535,12 +3535,12 @@
           <t>BSMA0056</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E59" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -3568,7 +3568,7 @@
       <c r="K59" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P59" t="inlineStr">
+      <c r="P59" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -3585,7 +3585,7 @@
           <t>BSMA0057</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E60" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3613,7 +3613,7 @@
       <c r="K60" s="0" t="n">
         <v>1997</v>
       </c>
-      <c r="P60" t="inlineStr">
+      <c r="P60" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3630,7 +3630,7 @@
           <t>BSMA0058</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E61" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3663,7 +3663,7 @@
       <c r="K61" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="P61" t="inlineStr">
+      <c r="P61" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3680,12 +3680,12 @@
           <t>BSMA0059</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -3713,7 +3713,7 @@
       <c r="K62" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P62" t="inlineStr">
+      <c r="P62" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -3730,7 +3730,7 @@
           <t>BSMA0060</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E63" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3758,7 +3758,7 @@
       <c r="K63" s="0" t="n">
         <v>2003</v>
       </c>
-      <c r="P63" t="inlineStr">
+      <c r="P63" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3775,12 +3775,12 @@
           <t>BSMA0061</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -3808,7 +3808,7 @@
       <c r="K64" s="0" t="n">
         <v>2025</v>
       </c>
-      <c r="P64" t="inlineStr">
+      <c r="P64" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -3825,12 +3825,12 @@
           <t>BSMA0062</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -3858,7 +3858,7 @@
       <c r="K65" s="0" t="n">
         <v>2025</v>
       </c>
-      <c r="P65" t="inlineStr">
+      <c r="P65" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -3875,12 +3875,12 @@
           <t>BSMA0063</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E66" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -3908,7 +3908,7 @@
       <c r="K66" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P66" t="inlineStr">
+      <c r="P66" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -3925,7 +3925,7 @@
           <t>BSMA0064</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="E67" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3953,7 +3953,7 @@
       <c r="K67" s="0" t="n">
         <v>2007</v>
       </c>
-      <c r="P67" t="inlineStr">
+      <c r="P67" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -3970,7 +3970,7 @@
           <t>BSMA0065</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E68" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3998,7 +3998,7 @@
       <c r="K68" s="0" t="n">
         <v>1984</v>
       </c>
-      <c r="P68" t="inlineStr">
+      <c r="P68" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -4015,7 +4015,7 @@
           <t>BSMA0066</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E69" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -4043,7 +4043,7 @@
       <c r="K69" s="0" t="n">
         <v>2012</v>
       </c>
-      <c r="P69" t="inlineStr">
+      <c r="P69" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -4060,12 +4060,12 @@
           <t>BSMA0067</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E70" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F70" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -4093,7 +4093,7 @@
       <c r="K70" s="0" t="n">
         <v>2019</v>
       </c>
-      <c r="P70" t="inlineStr">
+      <c r="P70" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -4110,12 +4110,12 @@
           <t>BSMA0068</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E71" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F71" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -4176,7 +4176,7 @@
       <c r="K71" s="0" t="n">
         <v>2017</v>
       </c>
-      <c r="P71" t="inlineStr">
+      <c r="P71" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -4193,12 +4193,12 @@
           <t>BSMA0069</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E72" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F72" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -4227,7 +4227,7 @@
       <c r="K72" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="P72" t="inlineStr">
+      <c r="P72" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -4244,7 +4244,7 @@
           <t>BSMA0070</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E73" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -4272,7 +4272,7 @@
       <c r="K73" s="0" t="n">
         <v>1995</v>
       </c>
-      <c r="P73" t="inlineStr">
+      <c r="P73" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -4289,12 +4289,12 @@
           <t>BSMA0071</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E74" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -4322,7 +4322,7 @@
       <c r="K74" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P74" t="inlineStr">
+      <c r="P74" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -4339,12 +4339,12 @@
           <t>BSMA0072</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E75" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -4372,7 +4372,7 @@
       <c r="K75" s="0" t="n">
         <v>1993</v>
       </c>
-      <c r="P75" t="inlineStr">
+      <c r="P75" s="0" t="inlineStr">
         <is>
           <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
@@ -4389,7 +4389,7 @@
           <t>BSMA0073</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E76" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -4417,7 +4417,7 @@
       <c r="K76" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P76" t="inlineStr">
+      <c r="P76" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -4434,12 +4434,12 @@
           <t>BSMA0074</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E77" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F77" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -4467,7 +4467,7 @@
       <c r="K77" s="0" t="n">
         <v>2025</v>
       </c>
-      <c r="P77" t="inlineStr">
+      <c r="P77" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -4484,12 +4484,12 @@
           <t>BSMA0075</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="E78" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F78" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -4517,7 +4517,7 @@
       <c r="K78" s="0" t="n">
         <v>2023</v>
       </c>
-      <c r="P78" t="inlineStr">
+      <c r="P78" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -4534,12 +4534,12 @@
           <t>BSMA0076</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E79" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -4567,7 +4567,7 @@
       <c r="K79" s="0" t="n">
         <v>2019</v>
       </c>
-      <c r="P79" t="inlineStr">
+      <c r="P79" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -4584,7 +4584,7 @@
           <t>BSMA0077</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E80" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -4612,7 +4612,7 @@
       <c r="K80" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P80" t="inlineStr">
+      <c r="P80" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -4629,12 +4629,12 @@
           <t>BSMA0078</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E81" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="F81" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -4662,7 +4662,7 @@
       <c r="K81" s="0" t="n">
         <v>2009</v>
       </c>
-      <c r="P81" t="inlineStr">
+      <c r="P81" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -4679,12 +4679,12 @@
           <t>BSMA0079</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E82" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F82" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -4712,7 +4712,7 @@
       <c r="K82" s="0" t="n">
         <v>2003</v>
       </c>
-      <c r="P82" t="inlineStr">
+      <c r="P82" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -4729,12 +4729,12 @@
           <t>BSMA0080</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E83" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="F83" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -4762,7 +4762,7 @@
       <c r="K83" s="0" t="n">
         <v>2005</v>
       </c>
-      <c r="P83" t="inlineStr">
+      <c r="P83" s="0" t="inlineStr">
         <is>
           <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
@@ -4779,7 +4779,7 @@
           <t>BSMA0081</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E84" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -4807,7 +4807,7 @@
       <c r="K84" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P84" t="inlineStr">
+      <c r="P84" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -4824,12 +4824,12 @@
           <t>BSMA0082</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E85" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F85" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -4857,7 +4857,7 @@
       <c r="K85" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P85" t="inlineStr">
+      <c r="P85" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -4874,7 +4874,7 @@
           <t>BSMA0083</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E86" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -4902,7 +4902,7 @@
       <c r="K86" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P86" t="inlineStr">
+      <c r="P86" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -4919,12 +4919,12 @@
           <t>BSMA0084</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E87" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="F87" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -4952,7 +4952,7 @@
       <c r="K87" s="0" t="n">
         <v>1999</v>
       </c>
-      <c r="P87" t="inlineStr">
+      <c r="P87" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -4969,12 +4969,12 @@
           <t>BSMA0085</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="E88" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="F88" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -5002,7 +5002,7 @@
       <c r="K88" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P88" t="inlineStr">
+      <c r="P88" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -5019,12 +5019,12 @@
           <t>BSMA0086</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E89" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F89" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -5052,7 +5052,7 @@
       <c r="K89" s="0" t="n">
         <v>2008</v>
       </c>
-      <c r="P89" t="inlineStr">
+      <c r="P89" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -5069,12 +5069,12 @@
           <t>BSMA0087</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="E90" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="F90" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -5102,7 +5102,7 @@
       <c r="K90" s="0" t="n">
         <v>2008</v>
       </c>
-      <c r="P90" t="inlineStr">
+      <c r="P90" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -5119,12 +5119,12 @@
           <t>BSMA0088</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E91" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
+      <c r="F91" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -5152,7 +5152,7 @@
       <c r="K91" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P91" t="inlineStr">
+      <c r="P91" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -5169,12 +5169,12 @@
           <t>BSMA0089</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="E92" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
+      <c r="F92" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -5202,7 +5202,7 @@
       <c r="K92" s="0" t="n">
         <v>2026</v>
       </c>
-      <c r="P92" t="inlineStr">
+      <c r="P92" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -5219,7 +5219,7 @@
           <t>BSMA0090</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="E93" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5247,7 +5247,7 @@
       <c r="K93" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P93" t="inlineStr">
+      <c r="P93" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5264,7 +5264,7 @@
           <t>BSMA0091</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
+      <c r="E94" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5292,7 +5292,7 @@
       <c r="K94" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P94" t="inlineStr">
+      <c r="P94" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5309,12 +5309,12 @@
           <t>BSMA0092</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
+      <c r="E95" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
+      <c r="F95" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -5342,7 +5342,7 @@
       <c r="K95" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P95" t="inlineStr">
+      <c r="P95" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -5359,7 +5359,7 @@
           <t>BSMA0093</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
+      <c r="E96" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5387,7 +5387,7 @@
       <c r="K96" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P96" t="inlineStr">
+      <c r="P96" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5404,7 +5404,7 @@
           <t>BSMA0094</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
+      <c r="E97" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5432,7 +5432,7 @@
       <c r="K97" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P97" t="inlineStr">
+      <c r="P97" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5449,7 +5449,7 @@
           <t>BSMA0095</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
+      <c r="E98" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5477,7 +5477,7 @@
       <c r="K98" s="0" t="n">
         <v>2012</v>
       </c>
-      <c r="P98" t="inlineStr">
+      <c r="P98" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5494,12 +5494,12 @@
           <t>BSMA0096</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
+      <c r="E99" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
+      <c r="F99" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -5527,7 +5527,7 @@
       <c r="K99" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P99" t="inlineStr">
+      <c r="P99" s="0" t="inlineStr">
         <is>
           <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
@@ -5544,12 +5544,12 @@
           <t>BSMA0097</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
+      <c r="E100" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
+      <c r="F100" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -5577,7 +5577,7 @@
       <c r="K100" s="0" t="n">
         <v>1995</v>
       </c>
-      <c r="P100" t="inlineStr">
+      <c r="P100" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -5594,7 +5594,7 @@
           <t>BSMA0098</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
+      <c r="E101" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5622,7 +5622,7 @@
       <c r="K101" s="0" t="n">
         <v>2008</v>
       </c>
-      <c r="P101" t="inlineStr">
+      <c r="P101" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5639,7 +5639,7 @@
           <t>BSMA0099</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="E102" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5667,7 +5667,7 @@
       <c r="K102" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="P102" t="inlineStr">
+      <c r="P102" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5684,7 +5684,7 @@
           <t>BSMA0100</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E103" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5712,7 +5712,7 @@
       <c r="K103" s="0" t="n">
         <v>2016</v>
       </c>
-      <c r="P103" t="inlineStr">
+      <c r="P103" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5729,7 +5729,7 @@
           <t>BSMA0101</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
+      <c r="E104" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5757,7 +5757,7 @@
       <c r="K104" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P104" t="inlineStr">
+      <c r="P104" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5774,7 +5774,7 @@
           <t>BSMA0102</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E105" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5802,7 +5802,7 @@
       <c r="K105" s="0" t="n">
         <v>2012</v>
       </c>
-      <c r="P105" t="inlineStr">
+      <c r="P105" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5819,7 +5819,7 @@
           <t>BSMA0103</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
+      <c r="E106" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5847,7 +5847,7 @@
       <c r="K106" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P106" t="inlineStr">
+      <c r="P106" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -5864,12 +5864,12 @@
           <t>BSMA0104</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="E107" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
+      <c r="F107" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -5897,7 +5897,7 @@
       <c r="K107" s="0" t="n">
         <v>1999</v>
       </c>
-      <c r="P107" t="inlineStr">
+      <c r="P107" s="0" t="inlineStr">
         <is>
           <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
@@ -5914,12 +5914,12 @@
           <t>BSMA0105</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E108" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F108" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -5947,7 +5947,7 @@
       <c r="K108" s="0" t="n">
         <v>2013</v>
       </c>
-      <c r="P108" t="inlineStr">
+      <c r="P108" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -5964,7 +5964,7 @@
           <t>BSMA0106</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E109" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5992,7 +5992,7 @@
       <c r="K109" s="0" t="n">
         <v>2009</v>
       </c>
-      <c r="P109" t="inlineStr">
+      <c r="P109" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -6009,12 +6009,12 @@
           <t>BSMA0107</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E110" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F110" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -6042,7 +6042,7 @@
       <c r="K110" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P110" t="inlineStr">
+      <c r="P110" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -6059,12 +6059,12 @@
           <t>BSMA0108</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="E111" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
+      <c r="F111" s="0" t="inlineStr">
         <is>
           <t>3 = non-individual level</t>
         </is>
@@ -6092,7 +6092,7 @@
       <c r="K111" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P111" t="inlineStr">
+      <c r="P111" s="0" t="inlineStr">
         <is>
           <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
         </is>
@@ -6109,7 +6109,7 @@
           <t>BSMA0109</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E112" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -6137,7 +6137,7 @@
       <c r="K112" s="0" t="n">
         <v>2004</v>
       </c>
-      <c r="P112" t="inlineStr">
+      <c r="P112" s="0" t="inlineStr">
         <is>
           <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
         </is>
@@ -6154,12 +6154,12 @@
           <t>BSMA0110</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
+      <c r="E113" s="0" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr">
+      <c r="F113" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -6187,7 +6187,7 @@
       <c r="K113" s="0" t="n">
         <v>2008</v>
       </c>
-      <c r="P113" t="inlineStr">
+      <c r="P113" s="0" t="inlineStr">
         <is>
           <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
         </is>
@@ -6204,6 +6204,11 @@
           <t>BSMA0111</t>
         </is>
       </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G114" s="0" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to test the inﬂuence of external information search (EIS) on knowledge elaboration and group cognitive complexity (GCC) under the moderating effect of absorptive capacity (AC is indicated by prior knowledge base and gender diversity).</t>
@@ -6227,6 +6232,11 @@
       <c r="K114" s="0" t="n">
         <v>2018</v>
       </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="18" customHeight="1" s="31">
       <c r="A115" s="0" t="inlineStr">
@@ -6239,6 +6249,16 @@
           <t>BSMA0112</t>
         </is>
       </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G115" s="0" t="inlineStr">
         <is>
           <t>Purpose – This study aims to analyze the relationship between telework and teleworkers’ characteristics and the work-nonwork conflict (WNWC) in the Brazilian context, investigating time spent in eight nonwork dimensions and the more affected dimensions.</t>
@@ -6262,6 +6282,11 @@
       <c r="K115" s="0" t="n">
         <v>2023</v>
       </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="18" customHeight="1" s="31">
       <c r="A116" s="0" t="inlineStr">
@@ -6274,6 +6299,16 @@
           <t>BSMA0113</t>
         </is>
       </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G116" s="0" t="inlineStr">
         <is>
           <t>The perspectives of transaction cost economics and the resource-based view of the firm have been used extensively to understand the implications of outsourcing. However, transaction cost economics does not explain how a firm will evolve as it progressively outsources internal functions, and the resource-based view does not operationalize the unspecified competences that will be required over time. On the other hand, the lens of paradox highlights the increased expediency and complexity that outsourcing firms are expected to encounter. In this paper, paradoxes comparing operational expediency gains to increases in management, learning and strategic complexity are discussed, leading to the proposal that often unintended replacement behaviors manifest as extensive boundary spanning and new firm-level competencies are necessary to manage these paradoxes and maintain competitive advantage. In extremum tests of these propositions are provided to demonstrate that the complexity of outsourcing intangibles is informed by a lens of paradox.</t>
@@ -6297,6 +6332,11 @@
       <c r="K116" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="18" customHeight="1" s="31">
       <c r="A117" s="0" t="inlineStr">
@@ -6309,6 +6349,16 @@
           <t>BSMA0114</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G117" s="0" t="inlineStr">
         <is>
           <t>The aim of this research is to empirically investigate the relationships among the three vital knowledge management processes of acquisition, integration and application, and their effects on organisational innovation in the pharmaceutical manufacturing industry in Jordan; a knowledge-intensive business service (KIBS) sector. Structural equation modelling findings show an excellent fit among all these processes and innovation, with positive and significant relationships. Moreover, knowledge integration and knowledge application emerged as having strong and significant mediation effects upon the relationship between knowledge acquisition and innovation. As such, an organisation’s innovation efforts would significantly benefit from the synergistic effects of properly integrating and applying externally acquired knowledge. The findings make a valuable contribution to pharmaceutical knowledge management and innovation literature, especially in an era of open innovation. Pharmaceutical companies are advised to focus on developing proficient assimilation and application capabilities in order for acquired knowledge to have notable effects on their innovation performance.</t>
@@ -6332,6 +6382,11 @@
       <c r="K117" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="18" customHeight="1" s="31">
       <c r="A118" s="0" t="inlineStr">
@@ -6344,6 +6399,11 @@
           <t>BSMA0115</t>
         </is>
       </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G118" s="0" t="inlineStr">
         <is>
           <t>The “variance hypothesis” predicts that external search breadth leads to innovation outcomes, but people have limited attention for search and cultivating breadth consumes attention. How does individuals' search breadth affect innovation outcomes? How does individuals' allocation of attention affect the efficacy of search breadth? We matched survey data with complete patent records, to examine the search behaviors of elite boundary spanners at                 IBM                 . Surprisingly, individuals who allocated attention to people inside the firm were more innovative. Individuals with high external search breadth were more innovative only when they allocated more attention to those sources. Our research identifies limits to the “variance hypothesis” and reveals two successful approaches to innovation search: “cosmopolitans” who cultivate and attend to external people and “locals” who draw upon internal people                              . © 2014 The Authors.               Strategic Management Journal               published by John Wiley &amp; Sons Ltd.</t>
@@ -6367,6 +6427,11 @@
       <c r="K118" s="0" t="n">
         <v>2016</v>
       </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="18" customHeight="1" s="31">
       <c r="A119" s="0" t="inlineStr">
@@ -6379,6 +6444,11 @@
           <t>BSMA0116</t>
         </is>
       </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G119" s="0" t="inlineStr">
         <is>
           <t>THErelationships between age, aspects of tenure, locus of control, job involvement, and boundary spanning behaviour (B.S.B.) were examined using path analysis for 281 scientists and engineers. It was found that locus of control and age were significant determinants of job involvement. It was also shown that locus of control and job involvement were significant determinants of B.S.B. These findings are discussed relative to previous research on locus of control, job involvement, and B.S.B. Finally, new research designs are advocated which incorporate task characteristics, role dynamics constructs, and environmental uncertainty as determinants of B.S.B.</t>
@@ -6402,6 +6472,11 @@
       <c r="K119" s="0" t="n">
         <v>1978</v>
       </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="18" customHeight="1" s="31">
       <c r="A120" s="0" t="inlineStr">
@@ -6414,6 +6489,16 @@
           <t>BSMA0117</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G120" s="0" t="inlineStr">
         <is>
           <t>Customer contact personnel (CCP) are recognised as a key determinant in the attainment of customer satisfaction and service quality. While they are readily acknowledged as often representing the service in the eyes of the customer, almost no attention has been given to researching the determinants of service behaviour among CCP, from the perspective of CCP.</t>
@@ -6437,6 +6522,11 @@
       <c r="K120" s="0" t="n">
         <v>1998</v>
       </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="18" customHeight="1" s="31">
       <c r="A121" s="0" t="inlineStr">
@@ -6449,6 +6539,16 @@
           <t>BSMA0118</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G121" s="0" t="inlineStr">
         <is>
           <t>This study investigated coordinated action in multiteam systems employing 233 correspondent systems, comprising 3 highly specialized 6-person teams, that were engaged in an exercise that was simultaneously “laboratory-like” and “field-like.” It enriches multiteam system theory through the combination of theoretical perspectives from the team and the large organization literatures, underscores the differential impact of large size and modular organization by specialization, and demonstrates that conventional wisdom regarding effective coordination in traditional teams and large organizations does not always transfer to multiteam systems. We empirically show that coordination enacted across team boundaries at the component team level can be detrimental to performance and that coordinated actions enacted by component team boundary spanners and system leadership positively impact system performance only when these actions are centered around the component team most critical to addressing the demands of the task environment.</t>
@@ -6472,6 +6572,11 @@
       <c r="K121" s="0" t="n">
         <v>2012</v>
       </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="18" customHeight="1" s="31">
       <c r="A122" s="0" t="inlineStr">
@@ -6484,6 +6589,16 @@
           <t>BSMA0119</t>
         </is>
       </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G122" s="0" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore how and why employees perceive technology-mediated interruptions differently and the role of sociocultural factors in this process using sociomaterial analysis. Design/methodology/approach – Data were gathered from 34 Sri Lankan knowledge workers using a series of workshop-based activities. The concept of sociomateriality is employed to understand how sociocultural elements are entangled with technology in work-life boundary experiences.</t>
@@ -6507,6 +6622,11 @@
       <c r="K122" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="18" customHeight="1" s="31">
       <c r="A123" s="0" t="inlineStr">
@@ -6519,6 +6639,16 @@
           <t>BSMA0120</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G123" s="0" t="inlineStr">
         <is>
           <t>In this article, the authors examine antecedents and consequences of the service climate in boundary-spanning self-managing teams (SMTs) that deliver financial services. Using data from members of 61 SMTs and their customers, the authors show a differential impact of the SMT service climate on various marketing performance measures. Furthermore, they obtain support for independent group-level effects of intrateam support and team member flexibility on employee perceptions of the SMT service climate. Both effects are persistent over time and demonstrate that collective perceptions in the SMT have incremental value in the explanation of the service climate.</t>
@@ -6542,6 +6672,11 @@
       <c r="K123" s="0" t="n">
         <v>2004</v>
       </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="18" customHeight="1" s="31">
       <c r="A124" s="0" t="inlineStr">
@@ -6554,6 +6689,11 @@
           <t>BSMA0121</t>
         </is>
       </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G124" s="0" t="inlineStr">
         <is>
           <t>Background: Registered nurses play a key role in hospitals, as they have an important impact on the quality of the services delivered. For nurses to perform at their best, they need organizational, leader, and coworker support. To date, few studies have explored the link between nurses_ perceived support, affective organizational commitment, and boundary-spanning behaviors. Methods: This cross-sectional research used a questionnaire survey to explore the hypothesized relationships in a sample of 273 nurses from a hospital in Belgium. Structural equation modeling was used for statistical analysis of the mediation model. Results: One hundred forty-seven (53.5%) nurses responded to the survey. Perceived support from the organization, supervisors, and coworkers positively influences nurses_ boundary-spanning behaviors. Affective organizational commitment was found to mediate the positive relationship between perceived organization support, perceived coworker support, and boundary-spanning behaviors. Perceived supervisor support and boundary-spanning behaviors showed a direct relationship not mediated by affective organizational commitment. Conclusions: Perceived support has an important influence on the boundary-spanning behavior of nurses. This study emphasizes the importance on how support exerts an influence on boundary-spanning behavior and</t>
@@ -6577,6 +6717,11 @@
       <c r="K124" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="18" customHeight="1" s="31">
       <c r="A125" s="0" t="inlineStr">
@@ -6589,6 +6734,16 @@
           <t>BSMA0122</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G125" s="0" t="inlineStr">
         <is>
           <t>Multiteam systems (i.e., teams of teams) are frequently used to deal with complex and demanding challenges that require several teams’ joint efforts. However, achieving effective horizontal coordination across component teams in these systems remains difficult. Using insights from organizational behavior research, we argue that horizontal coordination between component teams can benefit if a multiteam system is composed of generalist members who are acquainted with the multiple functions present in the overall system (i.e., high intrapersonal functional diversity [IFD]). At the same time, however, such IFD may have detrimental side effects because generalists’ broad focus may distract them from high-impact, specialized activities (i.e., aspirational behavior). Building on insights from organization theory, we propose that coordination across a multiteam system’s hierarchical layers (i.e., vertical coordinated action between a team tasked with system-wide integration and task-specialized component teams) is critical for reaping IFD’s benefits while avoiding its costs. These notions are supported in a sample of 236 14-person multiteam systems engaged in a realistic decision-making simulation. Our findings illustrate how combining insights from organizational behavior and organization theory can advance academic knowledge on multiteam systems and offer practical solutions for managing such systems.</t>
@@ -6612,6 +6767,11 @@
       <c r="K125" s="0" t="n">
         <v>2016</v>
       </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="18" customHeight="1" s="31">
       <c r="A126" s="0" t="inlineStr">
@@ -6624,6 +6784,11 @@
           <t>BSMA0123</t>
         </is>
       </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G126" s="0" t="inlineStr">
         <is>
           <t>This manuscript investigates the role of individual team members' breadth of functional experience for their interteam coordination behavior. Integrating personal construct and social identity theories, we examine interpersonal cognitive complexity as a mediating variable and organizational identification as a moderator. We test our hypotheses across two independent field studies, comprising an international peace support training mission (Study 1) and a municipality administration (Study 2). Corroborating our predictions, interpersonal cognitive complexity appeared as a conditional mediating variable that can translate an individual's breadth of functional experience into interteam coordination. The strength and direction of this indirect relationship, however, depended on the individual's identification with the organization as a whole. Moreover, on the team level of analysis, we found members' overall interteam coordination to positively relate with team performance in Study 2. All in all, this paper advances new knowledge on the antecedents, mechanisms, contingency factors, and team-level consequences of members' boundary spanning.</t>
@@ -6647,6 +6812,11 @@
       <c r="K126" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="18" customHeight="1" s="31">
       <c r="A127" s="0" t="inlineStr">
@@ -6659,6 +6829,11 @@
           <t>BSMA0124</t>
         </is>
       </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G127" s="0" t="inlineStr">
         <is>
           <t>Data from 409 members of 45 new product teams in five high-technology conpanies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator,Scout, and Guard. These activities are related to the frequency, type, and destination of communications between team members and others. This paper describes these activities and examines the irrpact of individual and environmental variables on the frequency in vAiich individual team members engage in them.</t>
@@ -6683,6 +6858,11 @@
       <c r="K127" s="0" t="n">
         <v>1989</v>
       </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="18" customHeight="1" s="31">
       <c r="A128" s="0" t="inlineStr">
@@ -6693,6 +6873,16 @@
       <c r="B128" s="0" t="inlineStr">
         <is>
           <t>BSMA0125</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
         </is>
       </c>
       <c r="G128" s="0" t="inlineStr">
@@ -6721,6 +6911,11 @@
       <c r="K128" s="0" t="n">
         <v>1999</v>
       </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="18" customHeight="1" s="31">
       <c r="A129" s="0" t="inlineStr">
@@ -6733,6 +6928,11 @@
           <t>BSMA0126</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G129" s="0" t="inlineStr">
         <is>
           <t>Leader-Member Exchange theory proposes both the salesperson and manager make contributions to their working relationship. Effective leadership is dependent upon developing a high quality relationship. This study tests the proposals of Leader-Member Exchange by examining the exchange of manager contributions (allowing the salesperson more operating freedom or latitude) and those of the salesperson. While the receipt of managerial latitude has a direct effect on the salesperson's evaluation of the working relationship, the salesperson's contributions also play a part. The manager allows more latitude to salespeople who are seen as more competent and loyal. These exchanges latitude for competency and loyalty) and the quality of the salesperson-manager relationship may be especially important when the sales task requires adaptive selling behaviors.</t>
@@ -6756,6 +6956,11 @@
       <c r="K129" s="0" t="n">
         <v>1998</v>
       </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="18" customHeight="1" s="31">
       <c r="A130" s="0" t="inlineStr">
@@ -6768,6 +6973,11 @@
           <t>BSMA0127</t>
         </is>
       </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G130" s="0" t="inlineStr">
         <is>
           <t>An information systems (IS) support community represents a knowledge-intensive network where IS professionals interact with end-users to resolve system use problems during the IS post-implementation stage. For IS professionals in the support function, providing support for multiple information systems to multiple business units requires knowledge about different domains (business units or technical systems). In this paper, we take a network perspective to empirically evaluate the effects of an IS worker's network position and knowledge boundary spanning on productivity. Drawing upon theories of experiential learning and knowledge boundary, we perform social network analysis and linear mixed effects modeling to analyze archival data comprising 36 IS workers and 23,450 support requests made by 4568 end-users during the first 13 months post SAP/R3 implementation in a large U.S. organization. Our findings reveal that IS workers' network centrality and boundary spanning positively influence productivity. Surprisingly, their boundary-spanning experience plays a substantially more important role than network centrality. This study makes important contributions to theory and practice in individual experiential learning in knowledge-intensive networks.</t>
@@ -6791,6 +7001,11 @@
       <c r="K130" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="18" customHeight="1" s="31">
       <c r="A131" s="0" t="inlineStr">
@@ -6803,6 +7018,16 @@
           <t>BSMA0128</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G131" s="0" t="inlineStr">
         <is>
           <t>This article develops a framework for studying cross-functional teams in organizations that focuses on three domains: organizational context, internal process, and outcome measures. The framework was developed from qualitative data from over 200 individual and group interviews, written descriptions, and team observations. We then operationally defined this model through a set of questionnaire items and validated it through quantitative analysis of data from 565 members of cross-functional teams. The resulting framework provides a base for the future study of cross-functional teams.</t>
@@ -6826,6 +7051,11 @@
       <c r="K131" s="0" t="n">
         <v>1996</v>
       </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="18" customHeight="1" s="31">
       <c r="A132" s="0" t="inlineStr">
@@ -6838,6 +7068,16 @@
           <t>BSMA0129</t>
         </is>
       </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G132" s="0" t="inlineStr">
         <is>
           <t>When working as a member of a team, individuals must make decisions concerning the allocation of resources (eg, effort) toward individual goals and team goals. As a result, individual and team goals, and feedback related to progress toward these goals, should be potent levers for affecting resource allocation decisions. This research develops a multilevel, multiple-goal model of individual and team regulatory processes that affect the allocation of resources across individual and team goals resulting in individual and team performance. On the basis of this model, predictions concerning the impact of individual and team performance feedback are examined empirically to evaluate the model and to understand the influence of feedback on regulatory processes and resource allocation. Two hundred thirty-seven participants were randomly formed into 79 teams of 3 that performed a simulated radar task that required teamwork. Results support the model and the predicted role of feedback in affecting the allocation of resources when individuals strive to accomplish both individual and team goals.</t>
@@ -6861,6 +7101,11 @@
       <c r="K132" s="0" t="n">
         <v>2004</v>
       </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="18" customHeight="1" s="31">
       <c r="A133" s="0" t="inlineStr">
@@ -6873,6 +7118,11 @@
           <t>BSMA0130</t>
         </is>
       </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G133" s="0" t="inlineStr">
         <is>
           <t>Boundary-spanning positions require occupants to interact with groups whose norms may differ from one another. It was hypothesized that individuals holding these positions would perform better if they were sensitive to social cues and able to adapt their behavior to fit the circumstances. 93 field representatives (average age 30.5 yrs) who acted as boundary spanners were given the Self-Monitoring Scale. Results show that significant relationships existed between job performance and an individual difference variable (self-monitoring) that assessed the ability of respondents to adjust their self-presentation to fit the situation; self-monitoring was most important during the period of early tenure.</t>
@@ -6896,6 +7146,11 @@
       <c r="K133" s="0" t="n">
         <v>1982</v>
       </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="18" customHeight="1" s="31">
       <c r="A134" s="0" t="inlineStr">
@@ -6908,6 +7163,11 @@
           <t>BSMA0131</t>
         </is>
       </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G134" s="0" t="inlineStr">
         <is>
           <t>Using an external perspective as a research lens, this study examined team-context interaction in five consulting teams. The data revealed three strategies toward the teams' environment: informing, parading, and probing. Informing teams remain relatively isolated from their environment; parading teams have high levels of passive observation of the environment; and probing teams actively engage outsiders. Probing teams revise their knowledge of the environment through external contact, initiate programs with outsiders, and promote their team's achievements within their organization. In this study, they were rated as the highest performers among the teams, although member satisfaction and cohesiveness suffered in the short run. Results suggested that external activities are better predictors of team performance than internal group processes for teams facing external dependence.</t>
@@ -6931,6 +7191,11 @@
       <c r="K134" s="0" t="n">
         <v>1990</v>
       </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="18" customHeight="1" s="31">
       <c r="A135" s="0" t="inlineStr">
@@ -6943,6 +7208,16 @@
           <t>BSMA0132</t>
         </is>
       </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G135" s="0" t="inlineStr">
         <is>
           <t>The market-shaping literature recognizes that consumers are actors who can shape markets. However, research into the mechanisms of consumption-driven market-shaping is only emerging. This paper shows that one way in which consumers shape markets is through boundary work, as consumers make, break, and re-make the boundaries among multiple markets. Empirically, this paper investigates how user innovation practices catalyzed the formation of four boardsport markets: surfing, kitesurfing, windsurfing, and stand-up-paddling. The findings show that consumers shape markets in three steps: (1) generating local variations of consumption practices; (2) imposing order and coherence to intermediate frames; and (3) channeling creative consumption practices into market formation. This paper contributes to the market-shaping literature by conceptualizing how consumers splinter an existing singular market into new markets. We coin the term ‘market bifurcations’ to describe how a singular, seemingly cohesive consumer practice breaks down, splintering into several local variations, which can then catalyze the formation of new markets.</t>
@@ -6966,6 +7241,11 @@
       <c r="K135" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="18" customHeight="1" s="31">
       <c r="A136" s="0" t="inlineStr">
@@ -6978,6 +7258,16 @@
           <t>BSMA0133</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G136" s="0" t="inlineStr">
         <is>
           <t>An intriguing window on Japanese/American intercultural relations can be found in American ethnographers’ in-depth accounts of their diﬃculties with Japanese informants. Although the literature contains excellent self-analyses of this kind, this body of data has yet to be mined for general lessons regarding communication between Americans and Japanese. This paper addresses that gap by comparing several reﬂexive accounts of doing ethnography in Japan: Matthews Hamabata’s Crested Kimono, Gail Bernstein’s Haruko’s World, Liza Dalby’s Geisha, and Crafting Selves by Dorinne Kondo. Examining the barriers to Japanese/American communication through this special lens reveals a complicated picture. On the one hand, familiar factors, such as the universalism of Americans, their emphasis upon individual autonomy in social relations, and the Japanese matrix of constantly shifting in-group/outgroup relations are often the dominant inﬂuences on intercultural interactions. Yet, on the other hand, situational contexts and the value orientations and political commitments of the actors clearly do modify the expression of such factors and sometimes even reverse the expected outcomes. The present approach facilitates the representation of these complex relationships. A qualitative analysis in which an objectively framed comparison aimed at generalization rests upon the non-reiﬁed foundation of several reﬂexive ethnographies, shows promise as one strategy for transcending the stalemate between traditional group-based interpretations of culture and more recent approaches stressing individual agency and internal cultural diversity. This paper also illustrates some advantages of an anthropological approach to communication between the members of two cultures whose diﬀerences have long been a focus of interculturalist research and examines implications for models of collectivist and individualist cultures. r 2002 Elsevier Science Ltd. All rights reserved.</t>
@@ -7001,6 +7291,11 @@
       <c r="K136" s="0" t="n">
         <v>2002</v>
       </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="18" customHeight="1" s="31">
       <c r="A137" s="0" t="inlineStr">
@@ -7013,6 +7308,11 @@
           <t>BSMA0134</t>
         </is>
       </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G137" s="0" t="inlineStr">
         <is>
           <t>Social ties to colleagues on other work teams can spur creative ideas and workplace innovation by exposing an individual to diverse knowledge. However, for external knowledge to be recombined into innovation, the knowledge must first be recognized as potentially valuable. Going beyond traditional structural explanations, we predict that the use of diverse knowledge to generate creative ideas and solutions will depend in part on employees’ psychological attachment to the organizational groups to which they belong, i.e., their social identity, and the strength of their social ties. We test our hypotheses in an R&amp;D division of a global hightechnology firm, finding that social identity influences the creative generativity of boundary-spanning ties. Specifically, stronger team identity renders interactions with colleagues on other work teams less generative of creative ideas, while identification with an overarching, superordinate group (e.g., a division) enhances creative generativity. We also hypothesize and find that tie strength attenuates the negative effect of team identity.</t>
@@ -7036,6 +7336,11 @@
       <c r="K137" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="18" customHeight="1" s="31">
       <c r="A138" s="0" t="inlineStr">
@@ -7048,6 +7353,11 @@
           <t>BSMA0135</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G138" s="0" t="inlineStr">
         <is>
           <t>The boundary spanning activity of the entrepreneur is used to examine the strategic management process in small business. In a sample of 82 owner/operators, intensive boundary spanning activity was strongly related to organizational performance, and information processing capability significantly affected the performance-boundary spanning relationship.</t>
@@ -7071,6 +7381,11 @@
       <c r="K138" s="0" t="n">
         <v>1984</v>
       </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="18" customHeight="1" s="31">
       <c r="A139" s="0" t="inlineStr">
@@ -7083,6 +7398,16 @@
           <t>BSMA0136</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G139" s="0" t="inlineStr">
         <is>
           <t>Improving access to support for people experiencing domestic violence and abuse requires better connections between healthcare services and specialist domestic violence and abuse (DVA) support agencies. We examined the work involved in restructuring the relationship between primary care and specialist DVA support services. This was part of a broader study of the implementation of a general practice DVA training and support programme (IRIS). We conducted an ethnography in two diﬀerent UK areas where the IRIS programme was being delivered. We investigated the work done by specialist DVA workers (Advocate Educators) in the dual role of providing training to GPs and advocacy support to patients. Drawing on concepts of boundary actors and boundary objects, we examined how interactions between clinicians and patients changed after the introduction of the IRIS programme. The referral pathway emerged as a boundary object, meeting a shared ambition of general practitioners and patients to distribute responsibility for addressing DVA. However, maintaining this as a boundary object-in-use required signiﬁcant, and often unseen, work on the part of the Advocate Educator as boundary spanner. Our study contributes to scholarship on boundary work by highlighting the role of marginal boundary actors in maintaining the use of boundary objects among disparate groups.</t>
@@ -7106,6 +7431,11 @@
       <c r="K139" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="18" customHeight="1" s="31">
       <c r="A140" s="0" t="inlineStr">
@@ -7118,6 +7448,16 @@
           <t>BSMA0137</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G140" s="0" t="inlineStr">
         <is>
           <t>Multinational companies (MNC) are facing increasing pressure in the marketplace. It is up to MNC leaders to engage the resources available to them to ensure these firms remain competitive and avoid organizational decline. A hallmark MNC business model competitive advantage is organizational effectiveness in promoting collaboration and cooperation across organizational and environmental boundaries. Boundary crossing actors and the activities they pursue are valuable resources residing at the core of the MNC business model and hence constitute a key element of the firm’s competitive advantage. The purpose of this research is to investigate how MNC leaders can engage these resources for organizational benefit. The research question asked and answered in this study is, How can MNC leaders bolster organizational effectiveness using boundary activity resource (re) combination and control? The organizational control theory lens is used to guide this research. Using the principles of evidence-based management, a systematic review of evidence from 2002 to 2022 was conducted. The systematic review process included a systematic search for evidence including gathering input from subject matter experts and a critical assessment and quality appraisal of the evidence sources. Subsequently, the sources were subjected to an analysis and synthesis in search of emergent themes related to the research question. The research showed that organizational climate, knowledge management, and individual idiosyncrasies (combined with role idiosyncrasies) have considerable implications for leaders in the decision-making process. Although each element is important on its own, the totality of the evidence suggests it is the holistic combination of all four elements that can lead to promotion of boundary activities and hence enhancement of organizational effectiveness. Furthermore, it is an MNC leader’s responsibility to ensure an organizational climate conducive to boundary crossing activities is created and maintained for these elements to work. The recommendations resulting from the research are that MNC leaders must prioritize boundary actors and activities as core organizational value drivers, core boundary crossing competencies have to be built out, and once constructed, these competencies have to be entrenched in the organization’s compositional mechanisms and be monitored and maintained for them to remain effective.</t>
@@ -7141,6 +7481,11 @@
       <c r="K140" s="0" t="n">
         <v>2023</v>
       </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="18" customHeight="1" s="31">
       <c r="A141" s="0" t="inlineStr">
@@ -7151,6 +7496,16 @@
       <c r="B141" s="0" t="inlineStr">
         <is>
           <t>BSMA0138</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
         </is>
       </c>
       <c r="G141" s="0" t="inlineStr">
@@ -7185,6 +7540,11 @@
       <c r="K141" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="18" customHeight="1" s="31">
       <c r="A142" s="0" t="inlineStr">
@@ -7197,6 +7557,16 @@
           <t>BSMA0139</t>
         </is>
       </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G142" s="0" t="inlineStr">
         <is>
           <t>Interorganizational teams are rapidly becoming more prevalent as a means to improve organizations' responsiveness. To achieve their objective, interorganizational teams must engage in extensive amounts of boundary spanning activity. This study juxtaposed three structural variables, namely team informational diversity, team boundedness, and extrateam links, in an integrated model aimed at promoting our understanding of how to increase interorganizational team boundary spanning activity and its effectiveness. The model was tested with 49 health promotion teams. Our findings indicated that three types of boundary spanning—scouting, ambassadorial, and coordinating—were positively associated with interorganizational team effectiveness. In addition, for team informational diversity, team boundedness, and extrateam links, scouting and ambassadorial activities fully mediated their relationships with team effectiveness; for team boundedness, coordinating activity also fully mediated its relationship with team effectiveness. These findings highlight the importance of incorporating structural considerations into the management of interorganizational teams.</t>
@@ -7220,6 +7590,11 @@
       <c r="K142" s="0" t="n">
         <v>2011</v>
       </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="18" customHeight="1" s="31">
       <c r="A143" s="0" t="inlineStr">
@@ -7232,6 +7607,16 @@
           <t>BSMA0140</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G143" s="0" t="inlineStr">
         <is>
           <t>The role of gender in career mobility is a major practical and scholarly concern. Drawing on boundaryless career literature and social role theory, we examined whether gender influences employees' psychological mobility, whether this influence varies depending on the nature of career boundaries (the boundaries of job, organisation and industry) and whether it is contingent on organisational or occupational characteristics. We conducted cross‐classified multilevel analyses on 3,527 Australian employees nested within 725 organisations and 43 occupations. The results suggest that females show higher mobility preferences than males when it comes to crossing industries but not changing organisations or jobs. However, their preference for crossing career boundaries is significantly reduced when their organisation has a strong presence of female leadership. We also find that in female‐dominated occupations, females show a higher cross‐organisational mobility preference than males, while in male‐dominated occupations, females show a lower cross‐organisational mobility preference.</t>
@@ -7255,6 +7640,11 @@
       <c r="K143" s="0" t="n">
         <v>2024</v>
       </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="18" customHeight="1" s="31">
       <c r="A144" s="0" t="inlineStr">
@@ -7267,6 +7657,11 @@
           <t>BSMA0141</t>
         </is>
       </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G144" s="0" t="inlineStr">
         <is>
           <t>Managing a complex, boundary‐spanning function to maximize its contribution to the firm can be a challenging task. This research is concerned with providing management with increased understanding of the effects of different ways of managing a function, especially a significant boundary‐spanning operation. Conducted in the context of a procurement function, through a laboratory experiment, explores the impact of performance measures, interaction with other internal organizations and access to information about external events on an individual′s decision making and “comfort level”. Results indicate that the performance measurement system determines an individual′s decision‐making performance. The broader, more effectiveness‐oriented measures also tend to make the individuals more confident and satisfied with their operating environment and decisions. The availability of interaction with other internal organizations and the access to information about external events impact on an individual′s decisions but have relatively little effect on his/her comfort level.</t>
@@ -7290,6 +7685,11 @@
       <c r="K144" s="0" t="n">
         <v>1994</v>
       </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="18" customHeight="1" s="31">
       <c r="A145" s="0" t="inlineStr">
@@ -7302,6 +7702,16 @@
           <t>BSMA0142</t>
         </is>
       </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G145" s="0" t="inlineStr">
         <is>
           <t>A psychological contract is composed of an individual’s belief regarding the reciprocal obligations that exist between that individual and another entity with which that person is engaged. Psychological contracts are important in many business relationships, such as those between a buyer and supplier. The perceptions held by one individual may not be congruent with those of the other, in which case conflict may arise within the relationship. We introduce to the operations and supply chain literatures a comprehensive view of the theory of psychological contracts, which with few exceptions has largely been omitted from research regarding inter-firm relationships. This research investigates the processes by which individuals manage conflict in inter-firm relationships, and the extent to which decisions at both tactical and strategic levels are influenced by the experience of psychological contract violation. At the tactical level, we seek to understand how the daily operational decisions that individuals make are affected by psychological contract violation, particularly when sub-optimal decision-making is observed. At the strategic level, we consider the circumstances under which relational versus written contractual governance mechanisms are leveraged in response to conflict, and how the experience of psychological contract violation may influence these broader,firm-level decisions. Our research plan uses two different methodological approaches in investigating these issues. First, to evaluate tactical behaviors, we employ an experiment. The goal of the experiment is to determine specifically how economic decisions made by those in boundary-spanning roles deviate from optimal in response to conflict and how these behaviors are influenced by the experience of psychological contract violation. To this end, we employ a 2x2x2 factorial design in which violation timing, severity, and attribution are investigated. The experiment was accompanied by an exit survey which served to assess the experience of psychological contract violation and related issues of trust and fairness. Data from 295 subjects were included in our analysis. We observe a main effect of severity occurring during the violation, and main effects of time and attribution are evident in post-violation periods. We tie these phenomena to the psychological constructs under study. Second, in order to investigate strategic-level decisions, we propose administration of an industry survey to purchasing and sales managers. The survey will allow us to more broadly characterize types of conflict experienced in inter-firm relationships and the contractual governance mechanisms leveraged in response. Models useful for investigating these issues are developed and discussed, and a survey instrument is presented. The work presented in this dissertation is among the first to incorporate both individual-level and firm-level contracts into an investigation of tactical and strategic conflict response and resolution analysis within buyer-supplier exchange relationships.</t>
@@ -7325,6 +7735,11 @@
       <c r="K145" s="0" t="n">
         <v>2011</v>
       </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="18" customHeight="1" s="31">
       <c r="A146" s="0" t="inlineStr">
@@ -7337,6 +7752,11 @@
           <t>BSMA0143</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G146" s="0" t="inlineStr">
         <is>
           <t>ABSTRACT               This paper examines learning in interdisciplinary action teams. Research on team effectiveness has focused primarily on single‐discipline teams engaged in routine production tasks and, less often, on interdisciplinary teams engaged in discussion and management rather than action. The resulting models do not explain differences in learning in interdisciplinary action teams. Members of these teams must coordinate action in uncertain, fast‐paced situations, and the extent to which they are comfortable speaking up with observations, questions, and concerns may critically influence team outcomes. To explore what leaders of action teams do to promote speaking up and other proactive coordination behaviours – as well as how organizational context may affect these team processes and outcomes – I analysed qualitative and quantitative data from 16 operating room teams learning to use a new technology for cardiac surgery. Team leader coaching, ease of speaking up, and boundary spanning were associated with successful technology implementation. The most effective leaders helped teams learn by communicating a motivating rationale for change and by minimizing concerns about power and status differences to promote speaking up in the service of learning.</t>
@@ -7360,6 +7780,11 @@
       <c r="K146" s="0" t="n">
         <v>2003</v>
       </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="18" customHeight="1" s="31">
       <c r="A147" s="0" t="inlineStr">
@@ -7372,6 +7797,11 @@
           <t>BSMA0144</t>
         </is>
       </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G147" s="0" t="inlineStr">
         <is>
           <t>Purpose: Sleep deprivation among employees has become commonplace in the workforce. In the United States, the number of hours individuals sleep per night has declined by an hour and a half per night since the 1960s. As of 2005, seventy-four percent of individuals were getting less than eight hours of sleep per night on weekdays. There are negative ramifications to the organization when employees are sleep deprived such as lost productivity, increased accident rate, and increased absenteeism.</t>
@@ -7395,6 +7825,11 @@
       <c r="K147" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="18" customHeight="1" s="31">
       <c r="A148" s="0" t="inlineStr">
@@ -7407,6 +7842,16 @@
           <t>BSMA0145</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G148" s="0" t="inlineStr">
         <is>
           <t>Organizations are increasingly applying artificial intelligence (AI) in interorganizational systems (IOS) to mitigate demand and supply disruptions. This shift towards AI to enhance supply chain agility capabilities automates some tasks previously undertaken by boundary-spanning employees who serve as critical informational and influential links with supply chain partners. Given limited related research, we investigate the impact of AI not only on the potential displacement of boundary-spanning employee roles but also on subsequent supply chain agility. Leveraging dynamic capabilities and social network theories, we first conducted interviews with supply chain executives to develop a practitioner survey. Following a mixedmethods approach, we next applied structural equation modeling to this survey data and then probed further via follow-up interviews. The results reveal that despite displacing some employees, the use of AI in IOS enhances the remaining operational and strategic roles of the boundary-spanning employees to enrich supply chain agility. The ensuing theoretical and managerial contributions emphasize the essential role of boundaryspanning employees as part of a hybrid human-AI solution, providing insight into the need for an optimal human/AI balance in the supply chain to cope with dynamic marketplaces.</t>
@@ -7430,6 +7875,11 @@
       <c r="K148" s="0" t="n">
         <v>2025</v>
       </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="18" customHeight="1" s="31">
       <c r="A149" s="0" t="inlineStr">
@@ -7442,6 +7892,11 @@
           <t>BSMA0146</t>
         </is>
       </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G149" s="0" t="inlineStr">
         <is>
           <t>While anecdotal and research evidence exists supporting the difﬁculties faced by foreign ﬁrms in host nation environments due to liability of foreignness, it is clear that many foreign ﬁrms have been successfully operating in the U.S. over the years. This study seeks to understand the strategies foreign ﬁrms use to cope with liabilities of foreignness in an alien environment and compete successfully with domestic ﬁrms, speciﬁcally through boundary spanning. Using a sample of 3861 ﬁrms in the U.S., we ﬁnd that foreign ﬁrms on the average underperform compared to domestic ﬁrms. We also ﬁnd these ﬁrms take a differing strategic posture to cope with the disadvantages of being a foreign ﬁrm compared to domestic rivals. Multiple mediation models indicate that once this strategic posture of foreign ﬁrms is controlled for, performance differentials do not exist between foreign and domestic ﬁrms.</t>
@@ -7465,6 +7920,11 @@
       <c r="K149" s="0" t="n">
         <v>2009</v>
       </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="18" customHeight="1" s="31">
       <c r="A150" s="0" t="inlineStr">
@@ -7477,6 +7937,16 @@
           <t>BSMA0147</t>
         </is>
       </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G150" s="0" t="inlineStr">
         <is>
           <t>Currently, little is known about the internal (intrafirm) behaviors that may positively affect collaborative marketing/logistics integration, or about the benefits that may be associated with making these considerable investments. In short, what should firms be doing to promote marketing/logistics collaborative integration? What is the potential payoff? This paper addresses these questions by examining relationships between the organization's evaluation and reward system, cross-functional collaboration, effective marketing/logistics interdepartmental integration, and distribution service performance.</t>
@@ -7500,6 +7970,11 @@
       <c r="K150" s="0" t="n">
         <v>2000</v>
       </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="18" customHeight="1" s="31">
       <c r="A151" s="0" t="inlineStr">
@@ -7512,6 +7987,16 @@
           <t>BSMA0148</t>
         </is>
       </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G151" s="0" t="inlineStr">
         <is>
           <t>Although cross-functional integration is important for research and development (R&amp;D), research about implications of cross-functional integration has been rather sparse. In new product development (NPD), no study to date has examined intrafirm as well as interfirm integration of key functions such as intrafirm R&amp;D–marketing–production together with interfirm integration of host R&amp;D–partner R&amp;D. Such marketing and operations interface contributes to a better understanding of how operational and marketing activities impact on competitiveness and firm performance. This study collected data from 202 electronics manufacturing firms operating in an emerging economy, mainland China and Hong Kong with international R&amp;D partnerships. The findings indicate that a high level of R&amp;D integration between firms improved NPD performance when cross-functional integration is based on existing rather than new product configurations and key technologies. Interestingly, in high distance situations, cross-functional integration in the production validation stage generated NPD success. The findings show that high environmental uncertainties lead to a high level of host and partner firms R&amp;D integration. However, product newness has no significant effects on R&amp;D integration in any of the NPD stages.</t>
@@ -7535,6 +8020,11 @@
       <c r="K151" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="18" customHeight="1" s="31">
       <c r="A152" s="0" t="inlineStr">
@@ -7547,6 +8037,11 @@
           <t>BSMA0149</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G152" s="0" t="inlineStr">
         <is>
           <t>This article aims for a deeper understanding of front-line employees (FLEs) and their boundary-spanning role in service organizations’ innovation processes from the vantage points of creativity and service innovation theory. It explores in particular FLEs’ processes of creativity by focusing on how ideas emerge and how these ideas are further managed in the organizations’ innovation processes. It draws on an in-depth empirical study of three units at a large spa and resort hotel. The article demonstrates how FLEs’ ideas are related to the assimilation and utilization of knowledge gained in the customer–supplier interface. Furthermore, it introduces the concept of ‘management by weaving’, which encompasses the middle managers’ roles in the complexity of leading diverse innovation processes in the service organization. By having the roles of facilitator, gatekeeper, and translator, middle managers hold the key position for letting FLEs play the role as innovators.</t>
@@ -7570,6 +8065,11 @@
       <c r="K152" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="18" customHeight="1" s="31">
       <c r="A153" s="0" t="inlineStr">
@@ -7582,6 +8082,16 @@
           <t>BSMA0150</t>
         </is>
       </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G153" s="0" t="inlineStr">
         <is>
           <t>Why do so many organizations fail to respond to crises effectively, and what can be done to improve their crisis response? We aim to address these questions by developing a typology of boundaries that can help us understand and better prepare for future crises. Building on the existing literature on crisis management and boundaries, our typology seeks to address the critique of current crisis management models, such as these being too prescriptive and placing too much emphasis on assumptions that only the decisions made by the crisis management team (i.e., centralized decisions) will impact the crisis response. We address this critique by elaborating on four categories of boundaries that are relevant to manage crisis response, such as physical, mental, social, and temporal. Examples of these boundaries could include access to properties (physical), interpreting whether a crisis is happening (mental), shifting relationship dynamics (social), and the urgency of response time to a crisis (temporal). Our typology offers a lens to consider crisis management by taking into consideration the complexities and nuances that linear crisis management models have not yet adequately addressed. We argue that by identifying, defining, and understanding different configurations of boundaries, one can better manage crises toward a desired outcome.</t>
@@ -7605,6 +8115,11 @@
       <c r="K153" s="0" t="n">
         <v>2025</v>
       </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="18" customHeight="1" s="31">
       <c r="A154" s="0" t="inlineStr">
@@ -7617,6 +8132,16 @@
           <t>BSMA0151</t>
         </is>
       </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G154" s="0" t="inlineStr">
         <is>
           <t>The literature on interorganizational relationships has explored them at the organizational level and ignored interpersonal relationships. This paper consists of a literature review analyzing, consolidating, and synthesizing studies on boundary spanners in business–to–business (B2B) interorganizational relationships, pointing out directions for future research. The review was carried out in ten steps, separated into three phases encompassing planning, collecting, and synthesizing data, and disclosing the results. The study assesses 3,156 published articles, and 45 of them addressed the theme of boundary spanners in B2B interorganizational relationships. These articles were analyzed, identifying their characteristics and the evolution of research through time. The definitions of interpersonal and interorganizational relationships were compared, observing how the literature has addressed the interdependency between these relationships. Also, the concepts and roles assigned to boundary spanners were analyzed, leading to an integrated framework of the existing literature on the theme. Finally, suggestions for future research are presented, followed by this review’s implications and limitations.</t>
@@ -7640,6 +8165,11 @@
       <c r="K154" s="0" t="n">
         <v>2023</v>
       </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="18" customHeight="1" s="31">
       <c r="A155" s="0" t="inlineStr">
@@ -7652,6 +8182,11 @@
           <t>BSMA0152</t>
         </is>
       </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G155" s="0" t="inlineStr">
         <is>
           <t>Purpose – Prior studies have largely overlooked the potentially negative consequences of a buyer’s relational capital (RC) with a supplier for supply-side resilience, assuming a positive linear relationship between the constructs. Meanwhile, the focus of research has been at an organisational level without incorporating the role of boundary spanning individuals at the interface between buyer and supplier. Drawing on social capital and boundary spanning theory, the purpose of this paper is to: re-examine the relationship between RC and supply-side resilience, challenging the linear assumption; and investigate how both the strength and diversity of a boundary spanner’s ties moderate this relationship.</t>
@@ -7675,6 +8210,11 @@
       <c r="K155" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="18" customHeight="1" s="31">
       <c r="A156" s="0" t="inlineStr">
@@ -7687,6 +8227,16 @@
           <t>BSMA0153</t>
         </is>
       </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G156" s="0" t="inlineStr">
         <is>
           <t>Purpose – To better understand factors that lead to business model innovation (BMI) in organizations, this study argues that inclusive leadership is the primary source that motivates employee engagement in boundaryspanning activities, which fosters BMI by generating and integrating employee knowledge through boundaryspanning exploration.</t>
@@ -7710,6 +8260,11 @@
       <c r="K156" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="18" customHeight="1" s="31">
       <c r="A157" s="0" t="inlineStr">
@@ -7722,6 +8277,11 @@
           <t>BSMA0154</t>
         </is>
       </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G157" s="0" t="inlineStr">
         <is>
           <t>The purpose of this article is to promote an open systems perspective on team research. The authors develop a model of team boundary activities: boundary spanning, buffering, and reinforcement. The model examines the relationship between these boundary activities and team performance, the moderating effects of organizational contextual factors, and the mediating effect of team psychological safety on the boundary work–performance relationship. These relationships were empirically tested with data collected from 64 software development teams. Boundary spanning, buffering, and boundary reinforcement were found to relate to team performance and psychological safety. Both relationships are moderated by the team’s task uncertainty and resource scarcity. The implications of the findings are offered for future research and practice.</t>
@@ -7745,6 +8305,11 @@
       <c r="K157" s="0" t="n">
         <v>2009</v>
       </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="18" customHeight="1" s="31">
       <c r="A158" s="0" t="inlineStr">
@@ -7757,6 +8322,16 @@
           <t>BSMA0155</t>
         </is>
       </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G158" s="0" t="inlineStr">
         <is>
           <t>Boundary work, or task-related activities with external actors, has been shown to positively influence small group performance. However, these "external activities" may also detract from important internal group processes that help groups function. This research examines the puzzle of how groups can perform external activities without compromising their internal group dynamics. I explore how groups perform boundary work and consider the effectiveness of different methods of boundary work from a group identity perspective. Using both qualitative and quantitative methods in experimental and field-based settings, I compare and contrast boundary work that involves sending group members outside the group boundary to interact with external actors individually (i.e., an outward-bound approach), with an inward-bound approach, which entails inviting outsiders in to provide information, resources, or support to the group as a whole. Across four studies, I find that an inward-bound approach to boundary work strengthens group identity and subsequent group satisfaction and viability (Studies 1, 2 and 4), an outward-bound approach used in combination with an inward-bound approach can positively influence task performance and group satisfaction and viability (Study 4), and that an initially weak group identity leads group members to choose an inward-bound approach over an outward-bound approach when interacting with outsiders (Studies 1, 3 and 4). The main contributions of this work are 1) delineating different ways in which groups interact with outsiders, 2) considering the nature of the relationships between boundary work methods and group identity, and 3) investigating the consequences of performing these methods of boundary work using multiple criteria of group effectiveness. Findings converge to reveal that inward boundary work is an important phenomenon for organizational groups. Ultimately, this research offers a more nuanced view of the external perspective of small groups by suggesting that the ways in which groups interact with outsiders are both multidimensional and consequential.</t>
@@ -7780,6 +8355,11 @@
       <c r="K158" s="0" t="n">
         <v>2030</v>
       </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="18" customHeight="1" s="31">
       <c r="A159" s="0" t="inlineStr">
@@ -7792,6 +8372,16 @@
           <t>BSMA0156</t>
         </is>
       </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G159" s="0" t="inlineStr">
         <is>
           <t>Top management teams (TMTs) interact with key external stakeholders through boundary spanning, often by holding outside directorships. Yet research suggests these activities have an equivocal relationship with firm financial performance. Although outside directorships promise informational benefits (i.e., the social network perspective), they also present challenges in the form of managerial opportunism (i.e., the agency perspective). Here, we adopt a contingency perspective to reconcile these perspectives, investigating the moderating role of cohesion, or the degree to which team members mutually support and get along with one another. We argue that boundary spanning will yield performance benefits for TMTs with high cohesion, because their increased commitment to the team will enable members to use their external relationships for the benefit of their firms. However, we also identify a boundary condition for this effect based on structural position in the TMT: that cohesion is especially relevant when proportionally more non-chief executive officer (CEO) TMT members span boundaries than CEOs span boundaries. Results from an archival study of TMTs using q-sort methodology provide support for these predictions.</t>
@@ -7815,6 +8405,11 @@
       <c r="K159" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="18" customHeight="1" s="31">
       <c r="A160" s="0" t="inlineStr">
@@ -7827,6 +8422,16 @@
           <t>BSMA0157</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G160" s="0" t="inlineStr">
         <is>
           <t>Multiteam systems are increasingly used by organizations, but are difficult to coordinate effectively. Building from theory on representational gaps, we explain why coordination between teams in multiteam systems can be hindered by inconsistencies that exist between them regarding the definition of shared problems. We argue that frame-of-reference training, an intervention that is theorized to reduce representational gaps, can facilitate coordination and subsequent performance in multiteam systems. We studied the effects of frame-of-reference training on multiteam system coordination and performance in 249 multiteam systems comprised of specialized teams. Supporting our expectations, we found that: (a) frame-of-reference training had a positive effect on multiteam system performance by enhancing between-team coordination; (b) within-team coordination improved the relationship between frame-of-reference training and between-team coordination, ultimately improving multiteam system performance; and (c) the patterns by which within-team coordination leveraged our intervention depended on teams’ specific functions. Our findings extend representational gaps theory, highlight the interdependencies between team-level and system-level coordination, and demonstrate the utility of frame-of-reference training in a new setting.</t>
@@ -7850,6 +8455,11 @@
       <c r="K160" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="18" customHeight="1" s="31">
       <c r="A161" s="0" t="inlineStr">
@@ -7862,6 +8472,11 @@
           <t>BSMA0158</t>
         </is>
       </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G161" s="0" t="inlineStr">
         <is>
           <t>Purpose: This study is designed to respond to repeated calls for research on sales person retentionby building upon a mature research stream to identify ways to reduce turnover in boundary spanning employees and the resultant effect it has on organizational productivity. Specifically, this research draws on the Job Demands-Resources model to explore the effect of employee perceptions of firm market orientation as a way to reduce role stressors and subsequently turnover intentions. It also looks at employee traits that may serve as a buffer to the role stress to turnover intentions link and can be part of the hiring selection process (in this case grit). In so doing, this research uses a sample of early career salespeople to examine the effects of a firm’s market orientation (MO) and selective hiring for specific traits (level of grit) on a salesperson’s intention to quit using Job Demand-Resources as a framework.</t>
@@ -7885,6 +8500,11 @@
       <c r="K161" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="18" customHeight="1" s="31">
       <c r="A162" s="0" t="inlineStr">
@@ -7897,6 +8517,11 @@
           <t>BSMA0159</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G162" s="0" t="inlineStr">
         <is>
           <t>What types of human and social capital identify the emergence of leaders of open innovation communities? Consistent with the norms of an engineering culture, we find that future leaders must first make strong technical contributions. Beyond technical contributions, they must then integrate their communities in order to mobilize volunteers and avoid the ever-present danger of forking and balkanization. This is enabled by two correlated but distinct social positions: social brokerage and boundary spanning between technological areas. An inherent lack of trust associated with brokerage positions can be overcome through physical interaction. Boundary spanners do not suffer this handicap and are much more likely than brokers to advance to leadership. The research separates the influence of human and social capital on promotion, and highlights previously unexamined differences between brokerage- and boundary-spanning positions. Longitudinal analyses of careers within the Internet Engineering Task Force community from 1986–2002 support the arguments.</t>
@@ -7920,6 +8545,11 @@
       <c r="K162" s="0" t="n">
         <v>2007</v>
       </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="18" customHeight="1" s="31">
       <c r="A163" s="0" t="inlineStr">
@@ -7932,6 +8562,16 @@
           <t>BSMA0160</t>
         </is>
       </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G163" s="0" t="inlineStr">
         <is>
           <t>In the water and energy sectors, projects geared towards new forms of cross-sectoral functioning have boomed in most European countries over the past decade, and have deeply transformed the ecology of urban services. These projects are often considered as an answer to a rising challenge affecting numerous traditional utilities: the unforeseen urban change relating to shifting (i.e. declining) demand patterns that are undermining traditional models of infrastructure management. The development of cross-sectoral strategies is considered a way both to tackle the attrition of traditional sources of revenue and to develop greener infrastructure systems by enhancing their efficiency level, often in line with low-carbon programmes implemented by national or local governments. The appeal lies in a fairly static perception of infrastructure management and technological change. Based on a detailed analysis of a traditional German local multi-utility and informed by a six-month internship within the company, the article deciphers the rationale of multi-sectoral practices, in particular the company’s transformation into a cross-utility that devised a common strategy for all its infrastructure networks and its ambiguities. Various facets of such ‘boundary work’ are analysed, focusing on organisational and financial aspects to reveal the new sites of tensions and negotiations between sectors, but also on the material component of these cross-sectoral projects through the case of one such nexus programme, a waste-toenergy programme. This programme embodies the potential contradictions between the call for reduced use of resources (i.e. the production of less waste) and the development of new urban technical systems relying primarily on those same resources.</t>
@@ -7955,6 +8595,11 @@
       <c r="K163" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="18" customHeight="1" s="31">
       <c r="A164" s="0" t="inlineStr">
@@ -7967,6 +8612,16 @@
           <t>BSMA0161</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G164" s="0" t="inlineStr">
         <is>
           <t>This study investigated relationships between middle managers’ formal position, their strategic influence and organizational performance. Among the 259 middle managers represented in the study, managers with formal positions in boundaryspanning sub-units reported higher levels of strategic influence activity than others. At the organizational level of analysis, the study found that firm performance was associated with more uniform levels of downward strategic influence, and more varied levels of upward influence among middle management cohorts. The findings suggest that middle managers’ strategic influence arises from their ability to mediate between internal and external selection environments. In addition, positive effects on organizational performance appear to depend on: (1) whether the overall pattern of upward influence is conducive to shifts in the network centrality of individual managers; and (2) whether the pattern of downward influence is consistent with an appropriate balance between the organization’s need for control and flexibility.</t>
@@ -7990,6 +8645,11 @@
       <c r="K164" s="0" t="n">
         <v>1997</v>
       </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="18" customHeight="1" s="31">
       <c r="A165" s="0" t="inlineStr">
@@ -8002,6 +8662,16 @@
           <t>BSMA0162</t>
         </is>
       </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G165" s="0" t="inlineStr">
         <is>
           <t>Self-assessment is increasingly prevalent in many organizations. Although managers perceive self-assessment as internally driven, the well-known link between organizational activities and the external environment suggests that outside forces play a signiﬁcant role. This investigation explores the external motivators of self-assessment through a ﬁeld study of 14 organizations. Five factors were found to link the conduct of self-assessment to the external environment: availability of an externally developed or sponsored model, presence of a boundary spanning individual, afﬁliation with professional and trade associations, pressure from powerful external entities, and potential for external reward or recognition. These ﬁndings suggest that self-assessment is driven signiﬁcantly by forces external to the organization. How these external factors combine to form the context of self-assessment may affect the outcomes of the project.</t>
@@ -8025,6 +8695,11 @@
       <c r="K165" s="0" t="n">
         <v>2004</v>
       </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="18" customHeight="1" s="31">
       <c r="A166" s="0" t="inlineStr">
@@ -8037,6 +8712,11 @@
           <t>BSMA0163</t>
         </is>
       </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G166" s="0" t="inlineStr">
         <is>
           <t>In this paper we test the hypothesis that boundary spanning is a differentiated function that is not necessarily performed by one person, as assumed in much previous research. Using longitudinal network data collected during labor negotiations, we found that some individuals on the bargaining teams ("representatives") broker ties toward their opponents, while others ("gatekeepers") broker ties from their opponents; and some broker task-oriented ties (measured by flows of advice), while others broker socioemotional ties (measured by flows of trust). Differentiation of trust and advice brokerage roles was strong throughout the negotiations, while differentiation of representative and gatekeeper roles became more distinct as the contract deadline (and increased potential for role conflict) neared. This analytic distinction suggests that role conflict must be examined differently, both conceptually and methodologically, and widens the range of options available for managing potential role conflicts.</t>
@@ -8060,6 +8740,11 @@
       <c r="K166" s="0" t="n">
         <v>1992</v>
       </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="18" customHeight="1" s="31">
       <c r="A167" s="0" t="inlineStr">
@@ -8072,6 +8757,11 @@
           <t>BSMA0164</t>
         </is>
       </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G167" s="0" t="inlineStr">
         <is>
           <t>Background: While participatory social network analysis can help health service partnerships to solve problems, little is known about its acceptability in cross-cultural settings. We conducted two case studies of chronic illness service partnerships in 2007 and 2008 to determine whether participatory research incorporating social network analysis is acceptable for problem-solving in Australian Aboriginal health service delivery. Methods: Local research groups comprising 13–19 partnership staff, policy officers and community members were established at each of two sites to guide the research and to reflect and act on the findings. Network and work practice surveys were conducted with 42 staff, and the results were fed back to the research groups. At the end of the project, 19 informants at the two sites were interviewed, and the researchers conducted critical reflection. The effectiveness and acceptability of the participatory social network method were determined quantitatively and qualitatively. Results: Participants in both local research groups considered that the network survey had accurately described the links between workers related to the exchange of clinical and cultural information, team care relationships, involvement in service management and planning and involvement in policy development. This revealed the function of the teams and the roles of workers in each partnership. Aboriginal workers had a high number of direct links in the exchange of cultural information, illustrating their role as the cultural resource, whereas they had fewer direct links with other network members on clinical information exchange and team care. The problem of their current and future roles was discussed inside and outside the local research groups. According to the interview informants the participatory network analysis had opened the way for problem-solving by “putting issues on the table”. While there were confronting and ethically challenging aspects, these informants considered that with flexibility of data collection to account for the preferences of Aboriginal members, then the method was appropriate in cross-cultural contexts for the difficult discussions that are needed to improve partnerships. Conclusion: Critical reflection showed that the preconditions for difficult discussions are, first, that partners have the capacity to engage in such discussions, second, that partners assess whether the effort required for these discussions is balanced by the benefits they gain from the partnership, and, third, that “boundary spanning” staff can facilitate commitment to partnership goals.</t>
@@ -8095,6 +8785,11 @@
       <c r="K167" s="0" t="n">
         <v>2012</v>
       </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="18" customHeight="1" s="31">
       <c r="A168" s="0" t="inlineStr">
@@ -8107,6 +8802,11 @@
           <t>BSMA0165</t>
         </is>
       </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G168" s="0" t="inlineStr">
         <is>
           <t>This paper reports on an important subgroup of international boundary-spanners – immigrants and second or third generation migrants from the MNC’s home country living in the subsidiary host country. We take as our example the Nikkeijin (Japanese immigrants and their descendants) in Brazil. Such bicultural people are a largely unexplored source of boundary-spanning internationally competent talent for multinational enterprises. Using two different surveys, we ﬁnd that this group is recognized as a source of talent by Japanese MNCs, but that their HRM practices are not appropriate to attract and use them in their global talent management programmes.</t>
@@ -8130,6 +8830,11 @@
       <c r="K168" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="18" customHeight="1" s="31">
       <c r="A169" s="0" t="inlineStr">
@@ -8142,6 +8847,11 @@
           <t>BSMA0166</t>
         </is>
       </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G169" s="0" t="inlineStr">
         <is>
           <t>Self-initiated expatriates (SIEs) who work for a subsidiary of a multinational enterprise from their country of origin and hence are familiar with both countries’ language and culture can be expected to act as boundary-spanners between the assigned expatriates sent from the parent country and host country nationals, and between the headquarters and the subsidiary. We develop a new model of boundary-spanning that encompasses both individual and organizational antecedents and validate the model using survey data from Japanese-affiliated companies in China. We find that familiarity with Chinese language and culture and the potential dual allegiance of SIEs contribute to enhancing their boundary-spanning behavior. We also find that relationships of trust among the parties concerned (social capital) and global career opportunities for such self-initiated expatriates (geocentric staffing) have positive influences on their dual allegiance. Finally, normative and systems integration of human resource management are associated with increasing levels of social capital and geocentric staffing.</t>
@@ -8165,6 +8875,11 @@
       <c r="K169" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="18" customHeight="1" s="31">
       <c r="A170" s="0" t="inlineStr">
@@ -8177,6 +8892,16 @@
           <t>BSMA0167</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G170" s="0" t="inlineStr">
         <is>
           <t>The god of this paper is to iden@ the communication tactics that tiow management teams to successtiy coordinate without becoming overloaded, and to see whether successti coordination and fidom from overload independently Muence team pefiormance. We found that how much teams comnumicatti, what they communicated abou~ and the technologies they used to communicate prdlcted coordination and overload. Team coordination but not overload prdlcted team SUWSS.</t>
@@ -8200,6 +8925,11 @@
       <c r="K170" s="0" t="n">
         <v>1998</v>
       </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="18" customHeight="1" s="31">
       <c r="A171" s="0" t="inlineStr">
@@ -8212,6 +8942,11 @@
           <t>BSMA0168</t>
         </is>
       </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G171" s="0" t="inlineStr">
         <is>
           <t>The paper explores DiMaggio and Powell's thesis that under conditions of uncertainty organizational decision makers will mimic the behavior of other organizations in their environment. We add to their discussion by positing that managers are especially likely to mimic the behavior of organizations to which they have some type of network tie via boundary-spanning personnel. Data are presented on the charitable contributions of 75 business corporations to 198 nonprofit organizations in the Minneapolis-St. Paul metropolitan area in 1980 and 1984. Using logistic regression models, we found that a firm is likely to give more money to a nonprofit that was previously funded by companies whose CEOs and/or giving officers are known personally by the firm's boundary-spanning personnel. Firms are also likely to give greater contributions to a nonprofit that is viewed more favorably by the local philanthropic elite. We also found that a nonprofit is likely to receive more money from a corporation that previously gave money to nonprofits whose directors sit on the nonprofit's board. We concluded that managers utilize the information gathered through extraorganizational, interpersonal networks to make decisions on how to relate to other organizations in their task environment and achieve organizational ends.</t>
@@ -8235,6 +8970,11 @@
       <c r="K171" s="0" t="n">
         <v>1989</v>
       </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="18" customHeight="1" s="31">
       <c r="A172" s="0" t="inlineStr">
@@ -8247,6 +8987,16 @@
           <t>BSMA0169</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G172" s="0" t="inlineStr">
         <is>
           <t>The present study examines a set of organizational predictors of first moves. More specifically, the study employed organizational information-processing theory to derive a set of hypotheses relating organizational characteristics to the level of first- mover activity. This archival study used a pooled cross section-time series data set of domestic airlines over an 8-year period.
@@ -8271,6 +9021,11 @@
       <c r="K172" s="0" t="n">
         <v>1992</v>
       </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="18" customHeight="1" s="31">
       <c r="A173" s="0" t="inlineStr">
@@ -8283,6 +9038,11 @@
           <t>BSMA0170</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G173" s="0" t="inlineStr">
         <is>
           <t>Purpose – More enterprises adopt open innovation by breaking technological or organizational boundaries to seek internal and external knowledge when they face a fiercely competitive environment, complex market demands, and increasingly rapid technological change. In this context, a knowledge search strategy is regarded as an effective means of obtaining inside and outside resources and an important way to break the innovation bottleneck. Moreover, information technology (IT) is deemed an important asset for sourcing knowledge, whereas absorptive capacity is seen as an indispensable ability for utilizing novel knowledge. Thus, this paper aims to test the role of knowledge search in open innovation and examine the mediating effect of absorptive capacity and the moderating effect of IT capability.</t>
@@ -8306,6 +9066,11 @@
       <c r="K173" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="18" customHeight="1" s="31">
       <c r="A174" s="0" t="inlineStr">
@@ -8318,6 +9083,16 @@
           <t>BSMA0171</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G174" s="0" t="inlineStr">
         <is>
           <t>With an increasing overlap between the work and non‐work domain, more research is needed to understand the factors that relate to how individuals manage their boundaries across multiple roles (i.e., work roles, family roles). Using a sample of 498 individuals, we explored the relationships between personality, O*NET job characteristic variables, and boundary management styles. Results revealed that job responsibility and work structure related to cross‐role interruptions and work identity centrality. Further, conscientiousness was related to greater perceptions of boundary control, family identity centrality, and fewer interruptions of work, while neuroticism was related to fewer interruptions of non‐work. Finally, the present findings replicated four of six defined boundary management styles put forth in prior research. Theoretical and practical implications are discussed.                                         Practitioner points                                                                        Individuals may differ in how they enact boundaries between work and non‐work as related to their individual personality.                                                           The job in which one works may relate to the manner in which boundaries between work and non‐work are managed.                                                           Organizational efforts to help employees with boundary management may be improved if job context and employee individual differences are noted and accommodated.</t>
@@ -8341,6 +9116,11 @@
       <c r="K174" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="18" customHeight="1" s="31">
       <c r="A175" s="0" t="inlineStr">
@@ -8353,6 +9133,16 @@
           <t>BSMA0172</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G175" s="0" t="inlineStr">
         <is>
           <t>The digital era is radically changing our societies and how ﬁrms do business. Innovating the business model has become a fundamental capability to survive competition, particularly for small and mediumsized enterprises (SMEs). This study investigates the digital-era role of boundary management capabilities in the processes of Business Model Innovation (BMI) in SMEs. Structural Equation Modelling is adopted to analyse data from a survey of 250 Italian experts who possess direct research and consulting experience with SMEs. Our ﬁndings reveal that digitalisation and ﬁrms’ boundaries aﬀect BMI in SMEs. Moreover, our results demonstrate how boundary management, speciﬁcally its technological and relational aspects, directly impacts BMI and mediates the relationship between boundary size and BMI. The study also oﬀers important theoretical and practical insights, calling on scholars and managers to give more attention to the boundary management of SMEs in order to support BMI.</t>
@@ -8376,6 +9166,11 @@
       <c r="K175" s="0" t="n">
         <v>2021</v>
       </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="18" customHeight="1" s="31">
       <c r="A176" s="0" t="inlineStr">
@@ -8388,6 +9183,11 @@
           <t>BSMA0173</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G176" s="0" t="inlineStr">
         <is>
           <t>This study investigated how a project group deals with the contradiction between distributed knowledge in boundary-spanning collaborative processes and the expectation that software systems will provide unified, codified knowledge. It employed an ethnographic, interpretive approach to examine the ways in which relevant knowledge was presented, recognized, shared or otherwise managed during a project concerned with the joint design of business process and IT systems change. Developing a group understanding of how to manage sensemaking and expertise across salient knowledge boundaries were discovered to be central to perceptions of project completion. Four stages of this development were identified. The contribution of this paper is to propose these stages as the basis for boundary-spanning group management approaches and to suggest ways of progressing the complexities of communication, consensus-building, information exchange, problem-formulation and solution-brokering that are fundamental to collaboration in IS definition. These processes are normally taken for granted, rationalized or ignored by managers of IT-related organizational change. The use of specific types of boundary-object may aid in managing such processes explicitly and ensuring rapid progress. Thus the findings have significant implications for research and practice in other forms of boundary-spanning group collaboration, such as organizational innovation and problem-solving.</t>
@@ -8411,6 +9211,11 @@
       <c r="K176" s="0" t="n">
         <v>2005</v>
       </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="177" ht="18" customHeight="1" s="31">
       <c r="A177" s="0" t="inlineStr">
@@ -8423,6 +9228,11 @@
           <t>BSMA0174</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G177" s="0" t="inlineStr">
         <is>
           <t>Research Summary: This paper builds theoretical arguments and shows empirical evidence of the direct benefits and indirect costs of corporate volunteering in developing countries. Spanning corporate and humanitarian sectors to work in challenging environments should activate motivational and learning benefits for participating employees. However, results from a field study of a 10-year partnership between logistics provider TNT and the United Nations World Food Program show that such boundary-spanning corporate social responsibility (CSR) can be a double-edged sword. Task interdependence with nonprofit peers while volunteering strengthens employees' partnership identification and institutional learning. However, institutional learning triggers identity strain (associated with attrition) when they return, unless firms foster a sense that they recognize CSR experiences as valuable. The findings inform the behavioral and microfoundations of the potential consequences of CSR.</t>
@@ -8446,6 +9256,11 @@
       <c r="K177" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="178" ht="18" customHeight="1" s="31">
       <c r="A178" s="0" t="inlineStr">
@@ -8458,6 +9273,16 @@
           <t>BSMA0175</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G178" s="0" t="inlineStr">
         <is>
           <t>In this study we examine the impact of market orientation of leaders on their leader-member exchange (IMX) with their followers. We review the evolution of leader-member exchange (LMX) theory over the exist five decades, and relate the strategic influence of increasing turbulence in the market environment on multiple generations of leadership styles during that period. Whereas vertical dyadic exchanges between hierarchical leaders and their followers may produce satisfactory performance of followers in equilibrium markets with predictable growth, these dyadic exchanges fail to do so in turbulent markets. Disequilibrium markets with disruptive turbulence demand introduction of discontinuous innovation from a new generation of market-oriented lateral leaders working closely with their boundary-spanning followers. We propose a number of hypotheses relating the market environment, leader-member exchange, and performance. Implications for managers and future researchers are discussed.</t>
@@ -8481,6 +9306,11 @@
       <c r="K178" s="0" t="n">
         <v>2002</v>
       </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="179" ht="18" customHeight="1" s="31">
       <c r="A179" s="0" t="inlineStr">
@@ -8493,6 +9323,16 @@
           <t>BSMA0176</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G179" s="0" t="inlineStr">
         <is>
           <t>We examine the extent to which executives' boundary spanning relations inside and outside their industry affect organizational strategy and performance. We posit that the informational and social influences of external ties will be reflected in the degree to which the organization's strategy conforms to or deviates from the central tendencies of its industry and that the alignment of executives' external ties with the firm's strategy will be beneficial to firm performance. Using a multiyear sample of firms in the branded foods and computer industries, we find that executives' intraindustry ties are related to strategic conformity, that extraindustry ties are associated with the adoption of deviant strategies, and that alignment of executives' external ties with the informational requirements of the firm's strategy enhances organizational performance. Our results also show that a unique or differentiated strategy is not universally advantageous and that the benefits accruing from strategic conformity are especially strong in the more uncertain computer industry.</t>
@@ -8516,6 +9356,11 @@
       <c r="K179" s="0" t="n">
         <v>1997</v>
       </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="18" customHeight="1" s="31">
       <c r="A180" s="0" t="inlineStr">
@@ -8528,6 +9373,16 @@
           <t>BSMA0177</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G180" s="0" t="inlineStr">
         <is>
           <t>The relationship between external communication and R&amp;D team creativity has received increasing attention in the R&amp;D management literature. However, little is known about the motivational mechanism between the two. We propose a second‐stage moderation model based on social cognitive theory to explain whether, how and when R&amp;D team’s external developmental feedback motivates its creativity. Using the data gathered from 452 R&amp;D team members and 84 supervisors in a time‐lagged field study, we found external developmental feedback had a positive effect on R&amp;D team creativity via increasing team creative efficacy. Further, conditional indirect effect analyses found that a high level of cooperative goal interdependence strengthened the positive effect of team creative efficacy on R&amp;D team creativity and the mediating effect of team creative efficacy between external developmental feedback and R&amp;D team creativity.</t>
@@ -8551,6 +9406,11 @@
       <c r="K180" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="18" customHeight="1" s="31">
       <c r="A181" s="0" t="inlineStr">
@@ -8563,6 +9423,16 @@
           <t>BSMA0178</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G181" s="0" t="inlineStr">
         <is>
           <t>This article explores the following hypothesis: There is a statistically significant relationship between a project manager’s leadership competencies and project success. Two proven questionnaires, the leadership dimensions questionnaire (LDQ) and the project success questionnaire (PSQ), were used to gather data from 52 project managers and project sponsors from a financial services company in the United Kingdom. The results from the LDQ and PSQ are presented in this article. A factor analysis of PSQ revealed three independent factors: usability, project delivery, and value of output to clients. The last factor is not related to project leadership or management, so the article concentrates on correlations between the other two factors and project leadership. Eight separate leadership dimensions were found to be statistically significantly related to performance, so the hypothesis was largely supported. Identifying such relationships provides managers with guidance on possible selection and project improvement models, whereby increased capability in leadership dimensions can lead to increased success in project management.</t>
@@ -8586,6 +9456,11 @@
       <c r="K181" s="0" t="n">
         <v>2008</v>
       </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="18" customHeight="1" s="31">
       <c r="A182" s="0" t="inlineStr">
@@ -8598,6 +9473,16 @@
           <t>BSMA0179</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G182" s="0" t="inlineStr">
         <is>
           <t>Leader-member exchange (LMX) is a multidimensional construct seeking to identify the quality of the relationship between the leader and immediate subordinate. An instrument developed by Schrie-sheim, Neider, Scandura, and Tepper (1992) was utilized to determine the LMX score of 798 non-managerial employees in a casual restaurant chain. The dimensions of perceived contribution, affect, and loyalty were examined. Results demonstrate that LMX quality was high among the surveyed employees of a restaurant chain. The scores of LMX on age, gender and job tenure differed among employees while LMX scores on job status, education, and job type did not differ significantly.</t>
@@ -8621,6 +9506,11 @@
       <c r="K182" s="0" t="n">
         <v>2005</v>
       </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="18" customHeight="1" s="31">
       <c r="A183" s="0" t="inlineStr">
@@ -8633,6 +9523,16 @@
           <t>BSMA0180</t>
         </is>
       </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G183" s="0" t="inlineStr">
         <is>
           <t>Even though, over the last two decades, the boundaryless career concept has stimulated a wide theoretical debate, scholars have recently claimed that research on the competencies that are necessary for managing a cross-boundary career is still incomplete. Similarly, the literature on emotional and social competencies has demonstrated how they predict work performance across industries and jobs but has neglected their inﬂuence in explaining the individual’s mobility across boundaries and their impact on career success. This study aims to ﬁll these gaps by examining the effects of emotional and social competencies on boundaryless career and on objective career success. By analyzing a sample of 142 managers over a period of 8 years, we found evidence that emotional competencies positively inﬂuence the propensity of an individual to undertake physical career mobility and that career advancements are related to the possession of social competencies and depend on the adoption of boundaryless career paths. This study also provides a contribution in terms of the evaluation of the emotional and social competencies demonstrated by an individual and of the operationalization of the measurement of boundaryless career paths, considering three facets of the physical mobility construct (organizational, industrial, and geographical boundaries).</t>
@@ -8656,6 +9556,11 @@
       <c r="K183" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="18" customHeight="1" s="31">
       <c r="A184" s="0" t="inlineStr">
@@ -8668,6 +9573,16 @@
           <t>BSMA0181</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G184" s="0" t="inlineStr">
         <is>
           <t>Aim: To identify learning from a clinical microsystems (CMS) quality improvement initiative to develop a more integrated service across a falls care pathway spanning community and hospital services. Background: Falls present a major challenge to healthcare providers internationally as populations age. A review of the falls care pathway in Sheffield, United Kingdom, identified that pathway implementation was constrained by inconsistent coordination and integration at the hospital–community interface. Approach: The initiative utilised the CMS quality improvement approach and comprised three phases. Phase 1 focussed on developing a climate for change through engaging stakeholders across the existing pathway and coaching frontline teams operating as microsystems in quality improvement. Phase 2 involved initiating change by working at the mesosystem level to identify priorities for improvement and undertake tests of change. Phase 3 engaged decision makers at the macrosystem level from across the wider pathway in achieving change identified in earlier phases of the initiative. Findings: The initiative was successful in delivering change in relation to key aspects of the pathway, engaging frontline staff and decision makers from different services within the pathway, and in building quality improvement capability within the workforce. Viewing the pathway as a series of interrelated CMS enabled stakeholders to understand the complex nature of the pathway and to target key areas for change. Particular challenges encountered arose from organisational reconfiguration and cross-boundary working. Conclusion: CMS quality improvement methodology may be a useful approach to promoting integration across a care pathway. Using a CMS approach contributed towards clinical and professional integration of some aspects of the service. Recognition of the pathway operating at meso- and macrosystem levels fostered wider stakeholder engagement with the potential of improving integration of care across a range of health and care providers involved in the pathway.</t>
@@ -8691,6 +9606,11 @@
       <c r="K184" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="18" customHeight="1" s="31">
       <c r="A185" s="0" t="inlineStr">
@@ -8703,6 +9623,16 @@
           <t>BSMA0182</t>
         </is>
       </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G185" s="0" t="inlineStr">
         <is>
           <t>To explain how multistakeholder groups organize democratic deliberations about complex sustainability issues, organizational scholars have focused on the key role of deliberative capacity, which encompasses the dimensions of inclusiveness, authenticity and consequentiality. However, the tensions inherent to the search of these three dimensions have been overlooked. In this paper, we argue that focusing on how spaces for deliberation are designed can help one understand how to manage such tensions. We identified the boundary work practices that shape the design of deliberative spaces and generate deliberative capacity properties in a high-level expert group (HLEG) launched by the European Commission about sustainable finance regulation. Our results show how these boundary work practices help balance deliberative tensions. We advance deliberation studies by conceptualizing deliberative boundary work, explaining how deliberative capacity is spatially generated and showing how deliberative tensions are balanced. We also contribute to boundary work theory by making explicit the deliberative nature of configuring boundary work and showing its relevancy to regulatory settings.</t>
@@ -8726,6 +9656,11 @@
       <c r="K185" s="0" t="n">
         <v>2023</v>
       </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="186" ht="18" customHeight="1" s="31">
       <c r="A186" s="0" t="inlineStr">
@@ -8738,6 +9673,11 @@
           <t>BSMA0183</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G186" s="0" t="inlineStr">
         <is>
           <t>Global offshoring has become a key strategy for international staffing, especially in the software industry. Global software teams engage in boundary spanning activities that may help MNEs achieve international connectivity and cope with external disruptions through their use of virtual work. However, offshoring IT professionals who bridge these boundaries in offshoring MNEs must contend with discontinuities, or perceived disruptions in expected communication flows, which impact their job satisfaction. Drawing on survey data from 193 professional consultants from an IT services offshoring MNE located primarily in Eastern Europe and working for a U.S. client, we test a model grounded in Organizational Discontinuity Theory. We find that potential discontinuities arising from the virtual work environment have no impact on the job satisfaction of offshoring IT professionals, but that those who experience team-level continuities of identification and shared vision are more satisfied with their jobs. Our findings suggest that virtual work may have become normalized such that it is not problematic in and of itself, and that fostering connectivity in boundary spanning global teams may be beneficial for MNEs. Our findings have important implications for MNEs managing disruptions created by global work arrangements as well as exogenous disruptions.</t>
@@ -8761,6 +9701,11 @@
       <c r="K186" s="0" t="n">
         <v>2023</v>
       </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="18" customHeight="1" s="31">
       <c r="A187" s="0" t="inlineStr">
@@ -8773,6 +9718,11 @@
           <t>BSMA0184</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G187" s="0" t="inlineStr">
         <is>
           <t>Acknowledgements: This research was funded by NSF grant #0422676 and #0726798 as well as support provided by the University of California, Irvine Center for Research on Information Technology in Organizations. The authors would like to acknowledge the helpful comments provided by Christopher Earley, Mark Griffin, John Mathieu, and Jone Pearce; assistance in data collection provided by Diaky Diaz, Christopher Reisdel and Bettina Wolf; and the generous time invested by all the film makers and film viewers who participated in the study.</t>
@@ -8796,6 +9746,11 @@
       <c r="K187" s="0" t="n">
         <v>2013</v>
       </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="188" ht="18" customHeight="1" s="31">
       <c r="A188" s="0" t="inlineStr">
@@ -8808,6 +9763,16 @@
           <t>BSMA0185</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G188" s="0" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to argue that the structure of the response to the World Trade Center (WTC) crisis can be characterized as an inter-organizational network and the majority of the activities can be identified as network management.</t>
@@ -8831,6 +9796,11 @@
       <c r="K188" s="0" t="n">
         <v>2016</v>
       </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="189" ht="18" customHeight="1" s="31">
       <c r="A189" s="0" t="inlineStr">
@@ -8843,6 +9813,11 @@
           <t>BSMA0186</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G189" s="0" t="inlineStr">
         <is>
           <t>Drawing on corporate entrepreneurship (CE) and social network research, this study focuses on strategic renewal as a form of CE and examines the impact of boundary-spanning at top and middle management levels on business units’ exploratory innovation. Analyses of multi-source and multi-level data, collected from 72 top managers (TMs) and 397 middle managers (MMs) operating in 34 units of a multi-national organization, indicate that TMs’ boundary-spanning is positively related to units’ exploratory innovation, but also has a cascading effect on MMs by increasing their perceived role conflict. MMs’ role conflict is negatively related to units’ exploratory innovation and thus offsets some of the benefits gained through TMs’ boundary-spanning activities. Taking a configurational perspective on social exchanges at multiple levels, we show that role conflict is reduced by overlapping boundary-spanning ties among TMs and MMs. Surprisingly, MMs’ boundary-spanning does not relate to exploratory innovation. Our study shows that with regard to boundary-spanning, a top-down approach to CE as strategic renewal may be most effective because TMs play a key role in driving exploratory innovation. However, TMs need to be aware of the cascading social liabilities of their boundary-spanning behavior and ensure MMs develop similar networks. We advance ongoing debates in studies about CE and social networks by providing empirically validated insights into who drives strategic renewal and by uncovering the benefits and costs of social exchanges for strategic renewal. Furthermore, we uncover potential causes of mixed findings in network theory research and highlight a remedy to social liabilities.</t>
@@ -8866,6 +9841,11 @@
       <c r="K189" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="18" customHeight="1" s="31">
       <c r="A190" s="0" t="inlineStr">
@@ -8878,6 +9858,11 @@
           <t>BSMA0187</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G190" s="0" t="inlineStr">
         <is>
           <t>Compared to job-specific conditions, the interpersonal context of work has received less attention from work–family scholars. Using data from a 2007 U.S. survey of workers (N = 1,286), we examine the impact of workplace social support and interpersonal conflict on work–family conflict and exposure to boundary-spanning demands—as indexed by the frequency that workers receive work-related contact outside of normal work hours. Findings indicate that workplace social support is associated negatively with work-to-family conflict, while interpersonal conflict at work is associated with higher levels of work-to-family conflict. Results also indicate that both supportive and conflictive work contexts are associated with more frequent exposure to boundary-spanning demands. However, workers in supportive contexts are more likely to appraise these demands as beneficial for accomplishing work tasks, and are less likely to appraise them as disruptive to family roles. By contrast, workers in conflictive contexts are more likely to appraise demands as disruptive to family roles, and are less likely to appraise them as beneficial for paid work. Consequently, our findings underscore the resource and demands aspects of interpersonal work contexts and their implications for the work–family interface.</t>
@@ -8901,6 +9886,11 @@
       <c r="K190" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="191" ht="18" customHeight="1" s="31">
       <c r="A191" s="0" t="inlineStr">
@@ -8913,6 +9903,16 @@
           <t>BSMA0188</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G191" s="0" t="inlineStr">
         <is>
           <t>This paper investigates boundary-work in management accounting in the context of globalization and hybrid professionalism. The paper demonstrates how permeable symbolic boundaries of the management accounting ﬁeld can be altered by employing expansion boundary-work. Contrasting boundary-work of IMA ofﬁcials and IMA members in Russia, we show that IMA ofﬁcials employ primarily monopolization boundary-work while IMA members employ primarily expansion boundary-work. Our ﬁndings illustrate how boundary-work is employed to exhibit organizational and occupational professionalism in the symbolic realm. The paper provides additional insight into the discursive domain of the accounting profession by linking boundary-work to globalization, two forms of professionalism, legitimacy, status and professional identity. This suggests that the professionalization process is inﬂuenced by the properties of professional boundaries.</t>
@@ -8936,6 +9936,11 @@
       <c r="K191" s="0" t="n">
         <v>2020</v>
       </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="192" ht="18" customHeight="1" s="31">
       <c r="A192" s="0" t="inlineStr">
@@ -8948,6 +9953,16 @@
           <t>BSMA0189</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G192" s="0" t="inlineStr">
         <is>
           <t>This article explores the joint production and consumption of health information and advice in the context of NHS Direct, the new telephone health information and advice service. NHS Direct is an atypical call centre environment in so far as its core staff (nurses) are highly skilled professionals. These nurses are required to collaborate closely with, and are to some extent dependent upon, non-professional lower skilled staff (call handlers) to deﬁne and prioritize their work. This introduces a number of tensions between the two groups. Nurses respond to these tensions by engaging in ‘boundary work’, the micropolitical strategies through which work identities and occupational margins are negotiated, to protect their own status. Call handlers are more subject to the pressures of work ‘speed-up’, highly aware of the risks inherent in their role, but are unable to call upon professional status, either in their resistance to managerial imperatives or in their interactions with health consumers. They are required to manage the tension between offering a safe and high quality service, characterized in their training as ‘professional’, and nurses’ boundary work, which positions them as ‘non-professional’. Here we draw on qualitative research, including call interaction data between call handler and consumer, to show how call handlers’ occupation of the contested territory between professional and non-professional status leaves them wide open to the agency of consumers, as consumers attempt to shape the service in their own interests.</t>
@@ -8971,6 +9986,11 @@
       <c r="K192" s="0" t="n">
         <v>2005</v>
       </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Study involving workplace employees, but does not report quantitative correlation/regression effect sizes for boundary spanning.</t>
+        </is>
+      </c>
     </row>
     <row r="193" ht="18" customHeight="1" s="31">
       <c r="A193" s="0" t="inlineStr">
@@ -8983,6 +10003,11 @@
           <t>BSMA0190</t>
         </is>
       </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G193" s="0" t="inlineStr">
         <is>
           <t>Past research has studied how the selection and use of control portfolios in software projects is based on environmental and task characteristics. However, little research has examined the consequences of control mode choices on project performance. This paper reports on a study that addresses this issue in the context of outsourced software projects. In addition, we propose that boundary-spanning activities between the vendor and the client enable knowledge sharing across organizational and knowledge domain boundaries. This is expected to lead to facilitation of control through specific incentives and performance norms that are suited to client needs as well as the vendor context. Therefore, we argue that boundary spanning between the vendor and client moderates the relationship between formal controls instituted by the vendor on the development team and project performance. We also hypothesize the effect of collaboration as a clan control on project performance. We examine project performance in terms of software quality and project efficiency. The research model is empirically tested in the Indian software industry setting on a sample of 96 projects. The results suggest that formal and informal control modes have a significant impact on software project outcomes, but need to be finely tuned and directed toward appropriate objectives. In addition, boundary-spanning activities significantly improve the effectiveness of formal controls. Finally, we find that collaborative culture has provided mixed benefits by enhancing quality but reducing efficiency.</t>
@@ -9006,6 +10031,11 @@
       <c r="K193" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="194" ht="18" customHeight="1" s="31">
       <c r="A194" s="0" t="inlineStr">
@@ -9018,6 +10048,16 @@
           <t>BSMA0191</t>
         </is>
       </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
       <c r="G194" s="0" t="inlineStr">
         <is>
           <t>Recently, discussion has begun to consider serving the base of the economic pyramid for business and societal benefit. Suggestions for so doing have focused on business model innovation, improving internal capabilities, promoting stronger governance, and providing leapfrog technologies (such as ICT) to promote effective change. We consider the questions of what types of innovation are occurring when businesses and other organizations enter the base of the pyramid and what types of social, economic, and consumer benefits they bring to local communities. We base our findings on an analysis of more than 1,000 cases describing base of the pyramid activities.</t>
@@ -9041,6 +10081,11 @@
       <c r="K194" s="0" t="n">
         <v>2006</v>
       </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+        </is>
+      </c>
     </row>
     <row r="195" ht="18" customHeight="1" s="31">
       <c r="A195" s="0" t="inlineStr">
@@ -9053,6 +10098,11 @@
           <t>BSMA0192</t>
         </is>
       </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G195" s="0" t="inlineStr">
         <is>
           <t>Human service organizations seeking to infuse research and other forms of evidence into their programs often need to expand their knowledge sharing systems in order to build their absorptive capacities for new information. To promote their engagement in evidence-informed practice, human service organizations can benefit from connections with intermediary organizations that assist with the dissemination and utilization of research and the use of internal knowledge brokers, called link officers. These boundaryspanning individuals work to embed external research and internal evidence in order to address current organizational priorities and service demands. This exploratory study describes the characteristics, major activities, and perceptions of link officers connected with three pioneering intermediary organizations. Quantitative and qualitative data from a survey of 137 Canadian and UK link officers provide a profile of these professionals, including how they engage practitioners to promote evidence-informed practice and the degree to which they are supported within their organizations and by intermediary organizations. The article concludes with practice and research implications for the development of the link officer role in human service organizations.</t>
@@ -9076,6 +10126,11 @@
       <c r="K195" s="0" t="n">
         <v>2017</v>
       </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="196" ht="18" customHeight="1" s="31">
       <c r="A196" s="0" t="inlineStr">
@@ -9088,6 +10143,11 @@
           <t>BSMA0193</t>
         </is>
       </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G196" s="0" t="inlineStr">
         <is>
           <t>The majority of team leadership studies have ignored the specific context in which that leadership takes place and the cyclical correlation of inputs and processes on ongoing performance. It is our contention that leadership is a mediator of team processes and team effectiveness on ongoing functioning of multidisciplinary teams (MDT). The members of 126 multidisciplinary teams responded to a survey on several aspects related to the functioning and leadership of their teams. The results support the hypothesis that leadership does mediate the relationship between reflexivity and effectiveness (i.e. team management performance, boundary spanning and satisfaction) within the team. Theoretically, these findings challenge those of linear models that typically analyse the impact of leadership as something that happens in isolation. Future research should describe and consider not just the team type and tasks but also investigate the roles that context and time play in team leadership.</t>
@@ -9111,6 +10171,11 @@
       <c r="K196" s="0" t="n">
         <v>2012</v>
       </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="18" customHeight="1" s="31">
       <c r="A197" s="0" t="inlineStr">
@@ -9123,6 +10188,11 @@
           <t>BSMA0194</t>
         </is>
       </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G197" s="0" t="inlineStr">
         <is>
           <t>Firms recognize that working together through collaborative relationships offers potential benefits such as improving cooperation, information sharing, and overall performance. An additional and extremely valuable benefit of working together is the potential for creating innovative business approaches and solutions. Thus, developing external linkages has become a higher priority within many organizations. Boundary spanning employees offer one means of achieving closer cross‐firm relationships. We investigate the roles of boundary spanners by examining service providers and their relationships with customers. More specifically, we examine boundary spanning employees that are physically on‐site at customer facilities. Results provide strong support that boundary spanners perceiving higher levels of external organizational support from a client subsequently develop affective commitment to the customer. This, in turn, drives knowledge exchange and logistics innovation. A relationship between logistics innovation and performance (of service providers and of customers) was also found. Managerial implications of the research findings are discussed and suggestions presented covering future research.</t>
@@ -9146,6 +10216,11 @@
       <c r="K197" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="18" customHeight="1" s="31">
       <c r="A198" s="0" t="inlineStr">
@@ -9158,6 +10233,11 @@
           <t>BSMA0195</t>
         </is>
       </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G198" s="0" t="inlineStr">
         <is>
           <t>Using resource dependency and institutional theories, we create and test a model examining the relationships among senior management commitment, resource allocations, and the structure of public affairs departments. Using a large sample of U.S.-based firms, we find a positive relationship between senior management commitment to the public affairs function and the level of human and monetary resources allocated to the public affairs department. Furthermore, firms structure their public affairs responsibilities into three common activity sets: communications, collaborations, and local activities. These common activities are, in turn, positively associated with senior management commitment and resources allocated to the public affairs department.</t>
@@ -9181,6 +10261,11 @@
       <c r="K198" s="0" t="n">
         <v>2004</v>
       </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="199" ht="18" customHeight="1" s="31">
       <c r="A199" s="0" t="inlineStr">
@@ -9193,6 +10278,11 @@
           <t>BSMA0196</t>
         </is>
       </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G199" s="0" t="inlineStr">
         <is>
           <t>Teams must constantly balance internally focused interactions through Adaptation and externally focused processes of spanning boundaries to facilitate change. This dynamic of team Adaptation has not been studied. In empirical studies on team Boundary Management or Adaptation, attention is given to laboratory based experiments and field studies of new product development teams in high-tech industries. This research focuses on continuous quality improvement (QI) teams which are comprised of a dynamic and shifting set of members otherwise attuned to their professional daily activities not directly related to the project. The teams of interest operate in highly institutionalized and regulated service industries of healthcare. The overarching research question in this study asks what factors influence team adaptation and how do teams effectively achieve internal and external balance in their QI projects, and to what extent does this contribute to project success. To answer this question, a developmental sequential mixed methods study is conducted that utilizes qualitative analytics through grounded theory based theme development and thematic analysis as well as quantitative analytics of Qualitative Comparative Analysis (QCA) and Structural Equation Modeling. The first study is a mixed methods design utilizing a grounded theory approach for theme development followed by QCA to articulate complex causal interactions among identified factors influencing Adaptation. The sample includes 23 physicians/physician leaders/and hospital administrators who provide 39 team project examples for evaluation. The second study is a Quantitative design utilizing factor analysis to discern factors identified in study one in order to assess internal and external factor effects on Adaptation. A survey resulted in 215 responses for analysis from an expanded sample of team members in institutionally structured organizations. The third study is a Qualitative design utilizing thematic analysis to expand an understanding of the dynamic nature of Boundary Management mechanisms and team Adaptation patterns. The sample includes 13 team members providing 15 team project examples from 15 hospitals some of which are high performing teams and others are not. This research reveals that effective quality improvement project teams demonstrate Adaptation versatility by using combinations of several strategies to connect to the surrounding organization. By doing so this research contributes to the team literature as it expands descriptions of Boundary Management and Adaptation; it combines factors that have not been previously studied together and finds them to contribute to Adaptation. It also focuses on teams in situ in a context with previously limited attention. For management practice, the study provides practical explanations for team Adaptation as a process that can be mindfully guided through mechanisms of Boundary Management.</t>
@@ -9216,6 +10306,11 @@
       <c r="K199" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="200" ht="18" customHeight="1" s="31">
       <c r="A200" s="0" t="inlineStr">
@@ -9228,6 +10323,16 @@
           <t>BSMA0197</t>
         </is>
       </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G200" s="0" t="inlineStr">
         <is>
           <t>As employees’ personal lives are increasingly splintered by work demands, the boundary between work and nonwork domains is becoming ever more blurred. Grounded within a self-regulatory approach and the executive control function of inhibitory control, we operationalize and examine nonwork role re-engagement (NWRR)—the extent to which individuals can redirect attentional resources back to nonwork tasks following work-related intrusions. In phases 1 and 2, we develop and refine a psychometrically sound unidimensional measure for NWRR aligned with the self-regulatory processes of self-control and interference control underlying inhibitory control. In phase 3, we confirm the factor structure with a new sample. In phase 4 we validate the measure using the samples from phases 2 and 3 to provide evidence of criterion-related, convergent, and discriminant validity. NWRR was related to important well-being and work-related outcomes above and beyond existing self-regulatory and boundary management constructs. We offer theoretical and practical implications and an agenda to guide future research, as attentional agility becomes increasingly relevant in a home life replete with interruptions from work.</t>
@@ -9251,6 +10356,11 @@
       <c r="K200" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="201" ht="18" customHeight="1" s="31">
       <c r="A201" s="0" t="inlineStr">
@@ -9263,6 +10373,16 @@
           <t>BSMA0198</t>
         </is>
       </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G201" s="0" t="inlineStr">
         <is>
           <t>T h i s position paper distinguishes different types of activities needed in software processes and proposes enaction support for t h e m . An architecture of enaction components providing this support is sketched.</t>
@@ -9286,6 +10406,11 @@
       <c r="K201" s="0" t="n">
         <v>1995</v>
       </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="202" ht="18" customHeight="1" s="31">
       <c r="A202" s="0" t="inlineStr">
@@ -9298,6 +10423,16 @@
           <t>BSMA0199</t>
         </is>
       </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G202" s="0" t="inlineStr">
         <is>
           <t>This article guides the development of creative insights in supply chain management. The authors begin by describing analogies’ role in advancing organization theory with a focus on image transfers between knowledge domains. While much has been said about the merits of conceptual transfers between domains, much equally remains unknown, particularly about how to deliberately develop creative insights that have the potential to challenge or enhance existing supply chain management theory. To address this issue, this research builds on prior work on analogies, creativity, and design thinking to develop a heuristic-analytic model. This model is designed to assist researchers in theorizing by analogy through a controlled dual cognitive process of divergence before convergence combined with a distant boundary-spanning knowledge search. An illustration of the model shows how creative output can provide a fresh perspective that helps render supply chains potentially more resilient.</t>
@@ -9321,6 +10456,11 @@
       <c r="K202" s="0" t="n">
         <v>2023</v>
       </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="203" ht="18" customHeight="1" s="31">
       <c r="A203" s="0" t="inlineStr">
@@ -9333,6 +10473,16 @@
           <t>BSMA0200</t>
         </is>
       </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G203" s="0" t="inlineStr">
         <is>
           <t>The period after completing primary and adjuvant cancer treatment until recurrence or death is now recognized as a unique phase in the cancer control continuum. The term “survivorship” has been adopted to connote this phase. Survivorship is a time of transition: Issues related to diagnosis and treatment diminish in importance, and concerns related to long-term follow-up care, management of late effects, rehabilitation, and health promotion predominate. In this article, we explore the unique challenges of care and health service delivery in terms of the interface between primary care and specialist care during the survivorship period. The research literature points to problems of communication between primary and specialist providers, as well as lack of clarity about the respective roles of different members of the health-care team. Survivorship care plans are recommended as an important tool to facilitate communication and allocation of responsibility during the transition from active treatment to survivorship. Research questions that remain to be answered with respect to survivorship care plans and other aspects of survivorship care are discussed.</t>
@@ -9356,6 +10506,11 @@
       <c r="K203" s="0" t="n">
         <v>2010</v>
       </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="204" ht="18" customHeight="1" s="31">
       <c r="A204" s="0" t="inlineStr">
@@ -9368,6 +10523,16 @@
           <t>BSMA0201</t>
         </is>
       </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G204" s="0" t="inlineStr">
         <is>
           <t>In multidisciplinary teams in the oil and gas industry, we examined expertise diversity's relationship with team learning and team performance under varying levels of collective team identification. In teams with low collective identification, expertise diversity was negatively related to team learning and performance; where team identification was high, those relationships were positive. Results also supported nonlinear relationships between expertise diversity and both team learning and performance. Finally, team learning partially mediated the linear and nonlinear relationships between diversity and performance. Findings broaden understanding of the process by which and the conditions under which expertise diversity may promote team performance.</t>
@@ -9391,6 +10556,11 @@
       <c r="K204" s="0" t="n">
         <v>2005</v>
       </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="205" ht="18" customHeight="1" s="31">
       <c r="A205" s="0" t="inlineStr">
@@ -9403,6 +10573,11 @@
           <t>BSMA0202</t>
         </is>
       </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G205" s="0" t="inlineStr">
         <is>
           <t>The definition of innovation varies from individual to individual and between individual and the team or the team and an organization. The perception of innovation and how individuals define innovation can make an organization stay competitive or go out of business. Research had shown that a traditional approach of idea generation as innovation at well intentioned organizations afforded success only 10% of the time after three years. In forming and managing project teams, which are made up of individuals or selling a service or product to a certain demography it is important and beneficial to understand their perception of innovation and if they see innovation as new, change or improvement. This study is built upon the earlier work of Zhuang (1995), Zhuang, Williamson, and Carter (1999), and McLaughlin and (2013). Prior research conducted by Caraballo and McLaughlin (2012) focused on understanding the perception of innovation as defined or understood by a homogeneous demography of Latino American professionals. This dissertation furthers the research conducted by Caraballo and McLaughlin (2012) with a focus on comprehending how a homogenous group Indian American professionals in the United States perceive or define innovation into the three categories of new, improve and change. While innovation may be understood by individuals as a multi-dimensional construct, the research tried to identify the relationship between perceptions, and gender, age and job function for the homogenous group of Indian Americans in the United States. The research followed the approach and methodology used by Caraballo and McLaughlin (2012) and the study is quantitative, exploratory and used web-based surveys to gather responses from respondents.</t>
@@ -9426,6 +10601,11 @@
       <c r="K205" s="0" t="n">
         <v>2014</v>
       </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="206" ht="18" customHeight="1" s="31">
       <c r="A206" s="0" t="inlineStr">
@@ -9438,6 +10618,11 @@
           <t>BSMA0203</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G206" s="0" t="inlineStr">
         <is>
           <t>Personnel is one of the most important resources for the performance of Information Systems (IS) and Information Center (IC) organizations. The scarcity of new employees, the difficulty of training and a high turnover make personnel management in these areas a difficult problem. For IS employees, the relationships between job satisfaction, organizational commitment and intention to leave the organization have been established. Because the size of the investment and the number of organizations establishing IC organizations are growing dramatically, it has become important to understand the determinants of turnover intentions for IC as well as IS employees. Are IC employees similar to their IS counterparts? Or, is their nature basically different, as some studies have suggested? This study examines the differences between IS and IC employees in terms of demographic characteristics, participation on boundary spanning activities, role stressors, overall job satisfaction, organizational commitment and turnover intentions. The differences are found to be significant and call for special attention from IC managers to manage more properly their personnel resources. IC employees were found to participate more extensively in boundary spanning activities, experienced more role stressors (role ambiguity and role conflict), were less satisfied with their jobs and less committed to their organization. The findings also demonstrate the importance of organizational commitment as an intervening variable in models of turnover. While overall job satisfaction had both direct and indirect effects on turnover intentions among IC employees, for IS personnel it had only indirect effects through organizational commitment. The effects of role stressors and boundary spanning activities were found to be indirect via overall job satisfaction and organizational commitment for both IC and IS employees. The implications of these findings for practicing managers and for future research are discussed.</t>
@@ -9461,6 +10646,11 @@
       <c r="K206" s="0" t="n">
         <v>1992</v>
       </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="207" ht="18" customHeight="1" s="31">
       <c r="A207" s="0" t="inlineStr">
@@ -9473,6 +10663,11 @@
           <t>BSMA0204</t>
         </is>
       </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G207" s="0" t="inlineStr">
         <is>
           <t>As software development projects continue to be over budget and behind schedule, researchers continue to look for ways to improve the likelihood of project success. In this research we juxtapose two different views of what influences software development team performance during the requirements development phase. In an examination of 66 teams from 15 companies we found that team skill, managerial involvement, and little variance in team experience enable more effective team processes than do software development tools and methods. Further, we found that development teams exhibit both positive and negative boundary-spanning behaviors. Team members promote and champion their projects to the outside environment, which is considered valuable by project stakeholders. They also, however, guard themselves from their environments; keeping important information a secret from stakeholders negatively predicts performance.</t>
@@ -9496,6 +10691,11 @@
       <c r="K207" s="0" t="n">
         <v>1998</v>
       </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="208" ht="18" customHeight="1" s="31">
       <c r="A208" s="0" t="inlineStr">
@@ -9508,6 +10708,16 @@
           <t>BSMA0205</t>
         </is>
       </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G208" s="0" t="inlineStr">
         <is>
           <t>This study examines the influence of the social network of board interlocks on strategic alliance formation. Our theoretical framework suggests how board interlock ties to other firms can increase or decrease the likelihood of alliance formation, depending on the content of relationships between CEOs (chief executive officers) and outside directors. Results suggest that CEO-board relationships characterized by independent board control reduce the likelihood of alliance formation by prompting distrust between corporate leaders, while CEO-board cooperation in strategic decision making appears to promote alliance formation by enhancing trust. The findings also show how the effects of direct interlock ties are amplified further by third-party network ties.</t>
@@ -9531,6 +10741,11 @@
       <c r="K208" s="0" t="n">
         <v>1999</v>
       </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+        </is>
+      </c>
     </row>
     <row r="209" ht="18" customHeight="1" s="31">
       <c r="A209" s="0" t="inlineStr">
@@ -9543,6 +10758,11 @@
           <t>BSMA0206</t>
         </is>
       </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G209" s="0" t="inlineStr">
         <is>
           <t>Leadership has been suggested to be an important factor affecting innovation. A number of studies have shown that transformational leadership positively influences organizational innovation. However, there is a lack of studies examining the contextual conditions under which this effect occurs or is augmented. Therefore, this study aimed to investigate the impact of transformational leadership on organizational innovation and to determine whether internal and external support for innovation as contextual conditions influence this effect. Organizational innovation was conceptualized as the tendency of the organization to develop new or improved products or services and its success in bringing those products or services to the market. Transformational leadership was hypothesized to have a positive influence on organizational innovation. Furthermore, this effect was proposed to be moderated by internal support for innovation, which refers to an innovation supporting climate and adequate resources allocated to innovation. Support received from external organizations for the purposes of knowledge and resource acquisition was also proposed to moderate the relationship between transformational leadership and organizational innovation. To test these hypotheses, data were collected from 163 research and development (R&amp;D) employees and managers of 43 micro‐ and small‐sized Turkish entrepreneurial software development companies. Two separate questionnaires were used to collect the data. Employees' questionnaires included measures of transformational leadership and internal support for innovation, whereas managers' questionnaires included questions about product innovations of their companies and the degree of support they received from external institutions. Organizational innovation was measured with a market‐oriented criterion developed specifically for developing countries and newly developing industries. Hierarchical regression analysis was used to test the hypothesized effects. The results of the analysis provided support for the positive influence of transformational leadership on organizational innovation. This finding is significant because this positive effect was identified in micro‐ and small‐sized companies, whereas previous research focused mainly on large companies. In addition, external support for innovation was found to significantly moderate this effect. Specifically, the relationship between transformational leadership and organizational innovation was stronger when external support was at high levels than when there was no external support. This study is the first to investigate and empirically show the importance of this contextual condition for organizational innovation. The moderating effect of internal support for innovation, however, was not significant. This study shows that transformational leadership is an important determinant of organizational innovation and encourages managers to engage in transformational leadership behaviors to promote organizational innovation. In line with this, transformational leadership, which is heavily suggested to be a subject of management training and development in developed countries, should also be incorporated into such programs in developing countries. Moreover, this study highlights the importance of external support in the organizational innovation process. The results suggest that technical and financial support received from outside the organization can be a more important contextual influence in boosting up innovation than an innovation‐supporting internal climate. Therefore, managers, particularly of micro‐ and small‐sized companies, should play external roles such as boundary spanning and should build relationships with external institutions that provide technical and financial support. The findings of this study are especially important for managers of companies that plan to or currently operate in countries with developing economies.</t>
@@ -9566,6 +10786,11 @@
       <c r="K209" s="0" t="n">
         <v>2009</v>
       </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="210" ht="18" customHeight="1" s="31">
       <c r="A210" s="0" t="inlineStr">
@@ -9578,6 +10803,11 @@
           <t>BSMA0207</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G210" s="0" t="inlineStr">
         <is>
           <t>Organizations have recognized that effective informal leadership is a source of competitive advantage and invest heavily in leadership development efforts. Moreover, because of historical shifts in the nature of work, this informal leadership often takes the form of inter-unit boundary spanning. Because of these two developments, discretionary boundary spanning (DBS) between units has increasingly become a critical, dynamic, bottom-up activity where individuals lacking formal authority step up and take on informal leadership responsibilities. In this study, we draw upon Simmelian Tie Theory (STT) to examine the relationship between different types of DBS and formal leaders’ perceptions of a subordinate’s informal leadership and performance. We empirically document that a small number of closed task-oriented and closed friendship-oriented DBSs are instrumental in helping individuals demonstrate informal leadership. However, we also show that DBS places constraints on informal leadership when closed ties become too numerous. This results in an inverted-U relationship between the number of closed DBS ties and perceptions of leadership where the apex (i.e., point of overembeddedness) emerges at a smaller number for friendship-oriented DBS relative to the apex for taskoriented DBSs. We discuss the theoretical implications of these results, as well as the practical implications for managers of organizations.</t>
@@ -9601,6 +10831,11 @@
       <c r="K210" s="0" t="n">
         <v>2022</v>
       </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="211" ht="18" customHeight="1" s="31">
       <c r="A211" s="0" t="inlineStr">
@@ -9613,6 +10848,11 @@
           <t>BSMA0208</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G211" s="0" t="inlineStr">
         <is>
           <t>With the emergence of "boundaryless organizations" and the increase in boundary-spanning activities, the sustainable development of organizations has been affected. Effectively promoting employees to engage in boundaryspanning activities has become of great practical significance. Besides, performance pressure has become a prevalent workplace stressor, significantly impacting employees' work behaviors. Therefore, drawing upon the cognitive-affective processing system theory and stressor-strain relationship theory, this study aims to investigate the mechanisms and boundary conditions of performance pressure on employee boundaryspanning behavior. Data collected from 336 questionnaires at two different time points is analyzed using bootstrapping and hierarchical regression to test hypotheses. The results indicate that performance pressure boosts employee boundary-spanning behavior by enhancing cognitive flexibility, while hindering this behavior by producing obsessive work passion. Moreover, achievement orientation plays a key role in moderating the impact of performance pressure on cognitive flexibility and obsessive work passion. Specifically, achievement orientation positively moderates the link between performance pressure and cognitive flexibility, while negatively moderating the relationship between performance pressure and obsessive work passion. Additionally, achievement orientation is found to moderate the indirect influence of performance pressure on employee boundaryspanning behavior through these two mediators. This study reveals that employees with high achievement orientation under performance pressure tend to develop cognitive flexibility, which motivates them to engage in more employee boundary-spanning activities. This paper also provides practical guidance for enterprises to promote employee boundary-spanning behavior. This study not only expands the research on the antecedents of employee boundary-spanning behavior but also confirms the double-edged sword effect of performance pressure on employee boundary-spanning behavior from both cognitive and affective perspectives.</t>
@@ -9636,6 +10876,11 @@
       <c r="K211" s="0" t="n">
         <v>2024</v>
       </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="212" ht="18" customHeight="1" s="31">
       <c r="A212" s="0" t="inlineStr">
@@ -9648,6 +10893,11 @@
           <t>BSMA0209</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G212" s="0" t="inlineStr">
         <is>
           <t>Knowledge gathering can create problems as well as benefits for project teams in work environments characterized by overload, ambiguity, and politics. This paper proposes that the value of knowledge gathering in such environments is greater under conditions that enhance team processing, sensemaking, and buffering capabilities. The hypotheses were tested using independent quality ratings of 96 projects and survey data from 485 project-team members collected during a multimethod field study. The findings reveal that three capability-enhancing conditions moderated the relationship between knowledge gathering and project quality: slack time, organizational experience, and decision-making autonomy. More knowledge gathering helped teams to perform more effectively under favorable conditions but hurt performance under conditions that limited their capabilities to utilize that knowledge successfully. Implications for theory and research on knowledge and learning in organizations, team effectiveness, and organizational design are discussed.</t>
@@ -9671,6 +10921,11 @@
       <c r="K212" s="0" t="n">
         <v>2006</v>
       </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="213" ht="18" customHeight="1" s="31">
       <c r="A213" s="0" t="inlineStr">
@@ -9683,6 +10938,11 @@
           <t>BSMA0210</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G213" s="0" t="inlineStr">
         <is>
           <t>Extending the differentiation-integration view of organizational design to teams, I propose that self-managing teams engaged in knowledge-intensive work can perform more effectively by combining autonomy and external knowledge to capture the benefits of each while offsetting their risks. The complementarity between having autonomy and using external knowledge is contingent, however, on characteristics of the knowledge and the task involved. To test the hypotheses, I examined the strategic and operational effectiveness of 96 teams in a large multinational organization. Findings provide support for the theoretical model and offer implications for research on team ambidexterity and multinational management as well as team effectiveness.</t>
@@ -9705,6 +10965,11 @@
       </c>
       <c r="K213" s="0" t="n">
         <v>2010</v>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+        </is>
       </c>
     </row>
     <row r="214" ht="18" customHeight="1" s="31">

</xml_diff>

<commit_message>
Standardization: Updated AGENTS.md Rule 6 and Excel Data Validation to official code '3 = Non-individual level' across 133 excluded papers
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -913,7 +913,7 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G10" s="0" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G12" s="0" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G13" s="0" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G18" s="0" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G85" s="0" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="F92" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G92" s="0" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="F95" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G95" s="0" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="F100" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G100" s="0" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="F108" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G108" s="0" t="inlineStr">
@@ -6066,7 +6066,7 @@
       </c>
       <c r="F111" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G111" s="0" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
       <c r="F121" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G121" s="0" t="inlineStr">
@@ -6646,7 +6646,7 @@
       </c>
       <c r="F123" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G123" s="0" t="inlineStr">
@@ -6741,7 +6741,7 @@
       </c>
       <c r="F125" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G125" s="0" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
       <c r="F128" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G128" s="0" t="inlineStr">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="F141" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G141" s="0" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="F142" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G142" s="0" t="inlineStr">
@@ -7709,7 +7709,7 @@
       </c>
       <c r="F145" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G145" s="0" t="inlineStr">
@@ -7849,7 +7849,7 @@
       </c>
       <c r="F148" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G148" s="0" t="inlineStr">
@@ -7944,7 +7944,7 @@
       </c>
       <c r="F150" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G150" s="0" t="inlineStr">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="F151" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G151" s="0" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="F156" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G156" s="0" t="inlineStr">
@@ -8329,7 +8329,7 @@
       </c>
       <c r="F158" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G158" s="0" t="inlineStr">
@@ -8379,7 +8379,7 @@
       </c>
       <c r="F159" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G159" s="0" t="inlineStr">
@@ -8429,7 +8429,7 @@
       </c>
       <c r="F160" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G160" s="0" t="inlineStr">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="F164" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G164" s="0" t="inlineStr">
@@ -8994,7 +8994,7 @@
       </c>
       <c r="F172" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G172" s="0" t="inlineStr">
@@ -9140,7 +9140,7 @@
       </c>
       <c r="F175" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G175" s="0" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="F178" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G178" s="0" t="inlineStr">
@@ -9330,7 +9330,7 @@
       </c>
       <c r="F179" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G179" s="0" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="F188" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G188" s="0" t="inlineStr">
@@ -10055,7 +10055,7 @@
       </c>
       <c r="F194" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G194" s="0" t="inlineStr">
@@ -11080,7 +11080,7 @@
       </c>
       <c r="F216" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G216" s="0" t="inlineStr">
@@ -11230,7 +11230,7 @@
       </c>
       <c r="F219" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G219" s="0" t="inlineStr">
@@ -11420,7 +11420,7 @@
       </c>
       <c r="F223" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G223" s="0" t="inlineStr">
@@ -11470,7 +11470,7 @@
       </c>
       <c r="F224" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G224" s="0" t="inlineStr">
@@ -11565,7 +11565,7 @@
       </c>
       <c r="F226" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G226" s="0" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="F230" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G230" s="0" t="inlineStr">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="F241" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G241" s="0" t="inlineStr">
@@ -13085,7 +13085,7 @@
       </c>
       <c r="F258" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G258" s="0" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F264" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G264" s="0" t="inlineStr">
@@ -14558,7 +14558,7 @@
       </c>
       <c r="F289" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G289" s="0" t="inlineStr">
@@ -14793,7 +14793,7 @@
       </c>
       <c r="F294" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G294" s="0" t="inlineStr">
@@ -15082,7 +15082,7 @@
       </c>
       <c r="F300" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G300" s="0" t="inlineStr">
@@ -15177,7 +15177,7 @@
       </c>
       <c r="F302" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G302" s="0" t="inlineStr">
@@ -15227,7 +15227,7 @@
       </c>
       <c r="F303" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G303" s="0" t="inlineStr">
@@ -15691,7 +15691,7 @@
       </c>
       <c r="F313" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G313" s="0" t="inlineStr">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="F314" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G314" s="0" t="inlineStr">
@@ -15841,7 +15841,7 @@
       </c>
       <c r="F316" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G316" s="0" t="inlineStr">
@@ -16131,7 +16131,7 @@
       </c>
       <c r="F322" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G322" s="0" t="inlineStr">
@@ -16456,7 +16456,7 @@
       </c>
       <c r="F329" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G329" s="0" t="inlineStr">
@@ -16736,7 +16736,7 @@
       </c>
       <c r="F335" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G335" s="0" t="inlineStr">
@@ -17201,7 +17201,7 @@
       </c>
       <c r="F345" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G345" s="0" t="inlineStr">
@@ -17566,7 +17566,7 @@
       </c>
       <c r="F353" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G353" s="0" t="inlineStr">
@@ -17841,7 +17841,7 @@
       </c>
       <c r="F359" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G359" s="0" t="inlineStr">
@@ -17891,7 +17891,7 @@
       </c>
       <c r="F360" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G360" s="0" t="inlineStr">
@@ -18216,7 +18216,7 @@
       </c>
       <c r="F367" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G367" s="0" t="inlineStr">
@@ -18356,7 +18356,7 @@
       </c>
       <c r="F370" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G370" s="0" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="F371" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G371" s="0" t="inlineStr">
@@ -19391,7 +19391,7 @@
       </c>
       <c r="F392" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G392" s="0" t="inlineStr">
@@ -19486,7 +19486,7 @@
       </c>
       <c r="F394" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G394" s="0" t="inlineStr">
@@ -19721,7 +19721,7 @@
       </c>
       <c r="F399" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G399" s="0" t="inlineStr">
@@ -19866,7 +19866,7 @@
       </c>
       <c r="F402" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G402" s="0" t="inlineStr">
@@ -20011,7 +20011,7 @@
       </c>
       <c r="F405" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G405" s="0" t="inlineStr">
@@ -20588,7 +20588,7 @@
       </c>
       <c r="F417" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G417" s="0" t="inlineStr">
@@ -21013,7 +21013,7 @@
       </c>
       <c r="F426" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G426" s="0" t="inlineStr">
@@ -21448,7 +21448,7 @@
       </c>
       <c r="F435" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G435" s="0" t="inlineStr">
@@ -21593,7 +21593,7 @@
       </c>
       <c r="F438" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G438" s="0" t="inlineStr">
@@ -21833,7 +21833,7 @@
       </c>
       <c r="F443" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G443" s="0" t="inlineStr">
@@ -21883,7 +21883,7 @@
       </c>
       <c r="F444" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G444" s="0" t="inlineStr">
@@ -21933,7 +21933,7 @@
       </c>
       <c r="F445" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G445" s="0" t="inlineStr">
@@ -22002,7 +22002,7 @@
       </c>
       <c r="F446" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G446" s="0" t="inlineStr">
@@ -22506,7 +22506,7 @@
       </c>
       <c r="F456" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G456" s="0" t="inlineStr">
@@ -22696,7 +22696,7 @@
       </c>
       <c r="F460" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G460" s="0" t="inlineStr">
@@ -22881,7 +22881,7 @@
       </c>
       <c r="F464" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G464" s="0" t="inlineStr">
@@ -22931,7 +22931,7 @@
       </c>
       <c r="F465" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G465" s="0" t="inlineStr">
@@ -22981,7 +22981,7 @@
       </c>
       <c r="F466" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G466" s="0" t="inlineStr">
@@ -23361,7 +23361,7 @@
       </c>
       <c r="F474" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G474" s="0" t="inlineStr">
@@ -24112,7 +24112,7 @@
       </c>
       <c r="F490" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G490" s="0" t="inlineStr">
@@ -24207,7 +24207,7 @@
       </c>
       <c r="F492" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G492" s="0" t="inlineStr">
@@ -24308,7 +24308,7 @@
       </c>
       <c r="F494" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G494" s="0" t="inlineStr">
@@ -24895,7 +24895,7 @@
       </c>
       <c r="F506" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G506" s="0" t="inlineStr">
@@ -25085,7 +25085,7 @@
       </c>
       <c r="F510" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G510" s="0" t="inlineStr">
@@ -25315,7 +25315,7 @@
       </c>
       <c r="F515" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G515" s="0" t="inlineStr">
@@ -25460,7 +25460,7 @@
       </c>
       <c r="F518" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G518" s="0" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="F532" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G532" s="0" t="inlineStr">
@@ -26446,7 +26446,7 @@
       </c>
       <c r="F539" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G539" s="0" t="inlineStr">
@@ -26781,7 +26781,7 @@
       </c>
       <c r="F546" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G546" s="0" t="inlineStr">
@@ -27146,7 +27146,7 @@
       </c>
       <c r="F554" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G554" s="0" t="inlineStr">
@@ -27196,7 +27196,7 @@
       </c>
       <c r="F555" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G555" s="0" t="inlineStr">
@@ -27291,7 +27291,7 @@
       </c>
       <c r="F557" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G557" s="0" t="inlineStr">
@@ -27341,7 +27341,7 @@
       </c>
       <c r="F558" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G558" s="0" t="inlineStr">
@@ -27587,7 +27587,7 @@
       </c>
       <c r="F563" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G563" s="0" t="inlineStr">
@@ -28172,7 +28172,7 @@
       </c>
       <c r="F575" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G575" s="0" t="inlineStr">
@@ -28582,7 +28582,7 @@
       </c>
       <c r="F584" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G584" s="0" t="inlineStr">
@@ -28812,7 +28812,7 @@
       </c>
       <c r="F589" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G589" s="0" t="inlineStr">
@@ -28862,7 +28862,7 @@
       </c>
       <c r="F590" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G590" s="0" t="inlineStr">
@@ -28912,7 +28912,7 @@
       </c>
       <c r="F591" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G591" s="0" t="inlineStr">
@@ -29112,7 +29112,7 @@
       </c>
       <c r="F595" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G595" s="0" t="inlineStr">
@@ -29207,7 +29207,7 @@
       </c>
       <c r="F597" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G597" s="0" t="inlineStr">
@@ -29452,7 +29452,7 @@
       </c>
       <c r="F602" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G602" s="0" t="inlineStr">
@@ -30642,7 +30642,7 @@
       </c>
       <c r="F628" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G628" s="0" t="inlineStr">
@@ -30877,7 +30877,7 @@
       </c>
       <c r="F633" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G633" s="0" t="inlineStr">
@@ -31292,7 +31292,7 @@
       </c>
       <c r="F642" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G642" s="0" t="inlineStr">
@@ -31342,7 +31342,7 @@
       </c>
       <c r="F643" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G643" s="0" t="inlineStr">
@@ -31572,7 +31572,7 @@
       </c>
       <c r="F648" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G648" s="0" t="inlineStr">
@@ -31907,7 +31907,7 @@
       </c>
       <c r="F655" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G655" s="0" t="inlineStr">
@@ -31957,7 +31957,7 @@
       </c>
       <c r="F656" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G656" s="0" t="inlineStr">
@@ -32327,7 +32327,7 @@
       </c>
       <c r="F664" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G664" s="0" t="inlineStr">
@@ -32652,7 +32652,7 @@
       </c>
       <c r="F671" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G671" s="0" t="inlineStr">
@@ -32702,7 +32702,7 @@
       </c>
       <c r="F672" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G672" s="0" t="inlineStr">
@@ -32977,7 +32977,7 @@
       </c>
       <c r="F678" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G678" s="0" t="inlineStr">
@@ -33027,7 +33027,7 @@
       </c>
       <c r="F679" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G679" s="0" t="inlineStr">
@@ -33280,7 +33280,7 @@
       </c>
       <c r="F684" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G684" s="0" t="inlineStr">
@@ -33655,7 +33655,7 @@
       </c>
       <c r="F692" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G692" s="0" t="inlineStr">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="F696" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G696" s="0" t="inlineStr">
@@ -33890,7 +33890,7 @@
       </c>
       <c r="F697" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G697" s="0" t="inlineStr">
@@ -33940,7 +33940,7 @@
       </c>
       <c r="F698" s="0" t="inlineStr">
         <is>
-          <t>99 = Other</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G698" s="0" t="inlineStr">
@@ -34559,7 +34559,7 @@
   </mergeCells>
   <dataValidations count="6">
     <dataValidation sqref="F4:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"1 = No effect size of interest,2 = Non-employee samples,3 = Non-indivisual level,4 = Non-primary study,5 = Multiple reasons (specify in Notes),6 = Duplicate,7 = Non-English language,99 = Other (specify in Notes)"</formula1>
+      <formula1>"1 = No effect size of interest,2 = Non-employee samples,3 = Non-individual level,4 = Non-primary study,5 = Multiple reasons (specify in Notes),6 = Duplicate,7 = Non-English language,99 = Other (specify in Notes)"</formula1>
     </dataValidation>
     <dataValidation sqref="Q4:Q82 Q87:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"1 = Cross-sectional,2 = Longitudinal/time-lagged,9 = Other (specify),999 = Unsure"</formula1>

</xml_diff>

<commit_message>
Data Clean: Executed final 117 exclusions and 2 restorations in master Excel sheet (Final: 273 Included, 428 Excluded)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -1699,7 +1699,12 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
@@ -1727,7 +1732,7 @@
       </c>
       <c r="P20" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1894,12 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
@@ -1917,7 +1927,7 @@
       </c>
       <c r="P24" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1992,12 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
@@ -2010,7 +2025,7 @@
       </c>
       <c r="P26" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2042,12 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
@@ -2055,7 +2075,7 @@
       </c>
       <c r="P27" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2142,12 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
@@ -2150,7 +2175,7 @@
       </c>
       <c r="P29" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2492,12 @@
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
@@ -2495,7 +2525,7 @@
       </c>
       <c r="P36" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2542,12 @@
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
@@ -2540,7 +2575,7 @@
       </c>
       <c r="P37" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2787,12 @@
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
@@ -2780,7 +2820,7 @@
       </c>
       <c r="P42" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2887,12 @@
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
@@ -2875,7 +2920,7 @@
       </c>
       <c r="P44" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3077,12 @@
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
@@ -3060,7 +3110,7 @@
       </c>
       <c r="P48" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -3587,7 +3637,12 @@
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
@@ -3615,7 +3670,7 @@
       </c>
       <c r="P60" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3982,12 @@
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
@@ -3955,7 +4015,7 @@
       </c>
       <c r="P67" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
       </c>
     </row>
@@ -4017,7 +4077,12 @@
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
@@ -4045,7 +4110,7 @@
       </c>
       <c r="P69" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4846,12 @@
       </c>
       <c r="E84" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
@@ -4809,7 +4879,7 @@
       </c>
       <c r="P84" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4946,12 @@
       </c>
       <c r="E86" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G86" s="0" t="inlineStr">
@@ -4904,7 +4979,7 @@
       </c>
       <c r="P86" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5341,12 @@
       </c>
       <c r="E94" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G94" s="0" t="inlineStr">
@@ -5294,7 +5374,7 @@
       </c>
       <c r="P94" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5486,12 @@
       </c>
       <c r="E97" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G97" s="0" t="inlineStr">
@@ -5434,7 +5519,7 @@
       </c>
       <c r="P97" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5681,12 @@
       </c>
       <c r="E101" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G101" s="0" t="inlineStr">
@@ -5624,7 +5714,7 @@
       </c>
       <c r="P101" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -5776,7 +5866,12 @@
       </c>
       <c r="E105" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G105" s="0" t="inlineStr">
@@ -5804,7 +5899,7 @@
       </c>
       <c r="P105" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -5821,7 +5916,12 @@
       </c>
       <c r="E106" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G106" s="0" t="inlineStr">
@@ -5849,7 +5949,7 @@
       </c>
       <c r="P106" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -5966,7 +6066,12 @@
       </c>
       <c r="E109" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G109" s="0" t="inlineStr">
@@ -5994,7 +6099,7 @@
       </c>
       <c r="P109" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -6111,7 +6216,12 @@
       </c>
       <c r="E112" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G112" s="0" t="inlineStr">
@@ -6139,7 +6249,7 @@
       </c>
       <c r="P112" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -6206,7 +6316,12 @@
       </c>
       <c r="E114" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G114" s="0" t="inlineStr">
@@ -6234,7 +6349,7 @@
       </c>
       <c r="P114" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -6786,7 +6901,12 @@
       </c>
       <c r="E126" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G126" s="0" t="inlineStr">
@@ -6814,7 +6934,7 @@
       </c>
       <c r="P126" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -7894,7 +8014,12 @@
       </c>
       <c r="E149" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G149" s="0" t="inlineStr">
@@ -7922,7 +8047,7 @@
       </c>
       <c r="P149" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8404,12 @@
       </c>
       <c r="E157" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G157" s="0" t="inlineStr">
@@ -8307,7 +8437,7 @@
       </c>
       <c r="P157" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -8759,7 +8889,12 @@
       </c>
       <c r="E167" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G167" s="0" t="inlineStr">
@@ -8787,7 +8922,7 @@
       </c>
       <c r="P167" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -8944,7 +9079,12 @@
       </c>
       <c r="E171" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G171" s="0" t="inlineStr">
@@ -8972,7 +9112,7 @@
       </c>
       <c r="P171" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9370,12 @@
       </c>
       <c r="E177" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G177" s="0" t="inlineStr">
@@ -9258,7 +9403,7 @@
       </c>
       <c r="P177" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -9675,7 +9820,12 @@
       </c>
       <c r="E186" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G186" s="0" t="inlineStr">
@@ -9703,7 +9853,7 @@
       </c>
       <c r="P186" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -10005,7 +10155,12 @@
       </c>
       <c r="E193" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G193" s="0" t="inlineStr">
@@ -10033,7 +10188,7 @@
       </c>
       <c r="P193" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -10235,7 +10390,12 @@
       </c>
       <c r="E198" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G198" s="0" t="inlineStr">
@@ -10263,7 +10423,7 @@
       </c>
       <c r="P198" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -10280,7 +10440,12 @@
       </c>
       <c r="E199" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G199" s="0" t="inlineStr">
@@ -10308,7 +10473,7 @@
       </c>
       <c r="P199" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -10665,7 +10830,12 @@
       </c>
       <c r="E207" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G207" s="0" t="inlineStr">
@@ -10693,7 +10863,7 @@
       </c>
       <c r="P207" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -10940,7 +11110,12 @@
       </c>
       <c r="E213" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G213" s="0" t="inlineStr">
@@ -10968,7 +11143,7 @@
       </c>
       <c r="P213" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -11370,7 +11545,12 @@
       </c>
       <c r="E222" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G222" s="0" t="inlineStr">
@@ -11398,7 +11578,7 @@
       </c>
       <c r="P222" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -11995,7 +12175,12 @@
       </c>
       <c r="E235" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G235" s="0" t="inlineStr">
@@ -12023,7 +12208,7 @@
       </c>
       <c r="P235" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -12130,7 +12315,12 @@
       </c>
       <c r="E238" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G238" s="0" t="inlineStr">
@@ -12158,7 +12348,7 @@
       </c>
       <c r="P238" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -12840,7 +13030,12 @@
       </c>
       <c r="E253" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G253" s="0" t="inlineStr">
@@ -12868,7 +13063,7 @@
       </c>
       <c r="P253" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -12885,7 +13080,12 @@
       </c>
       <c r="E254" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G254" s="0" t="inlineStr">
@@ -12913,7 +13113,7 @@
       </c>
       <c r="P254" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
       </c>
     </row>
@@ -13130,7 +13330,12 @@
       </c>
       <c r="E259" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G259" s="0" t="inlineStr">
@@ -13158,7 +13363,7 @@
       </c>
       <c r="P259" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -13455,7 +13660,12 @@
       </c>
       <c r="E266" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G266" s="0" t="inlineStr">
@@ -13483,7 +13693,7 @@
       </c>
       <c r="P266" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -13865,7 +14075,12 @@
       </c>
       <c r="E275" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G275" s="0" t="inlineStr">
@@ -13893,7 +14108,7 @@
       </c>
       <c r="P275" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -14313,7 +14528,12 @@
       </c>
       <c r="E284" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G284" s="0" t="inlineStr">
@@ -14341,7 +14561,7 @@
       </c>
       <c r="P284" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -14852,7 +15072,12 @@
       </c>
       <c r="E295" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G295" s="0" t="inlineStr">
@@ -14880,7 +15105,7 @@
       </c>
       <c r="P295" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -15127,7 +15352,12 @@
       </c>
       <c r="E301" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G301" s="0" t="inlineStr">
@@ -15155,7 +15385,7 @@
       </c>
       <c r="P301" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -15272,7 +15502,12 @@
       </c>
       <c r="E304" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G304" s="0" t="inlineStr">
@@ -15300,7 +15535,7 @@
       </c>
       <c r="P304" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -15362,7 +15597,12 @@
       </c>
       <c r="E306" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G306" s="0" t="inlineStr">
@@ -15390,7 +15630,7 @@
       </c>
       <c r="P306" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -15452,7 +15692,12 @@
       </c>
       <c r="E308" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G308" s="0" t="inlineStr">
@@ -15480,7 +15725,7 @@
       </c>
       <c r="P308" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -15591,7 +15836,12 @@
       </c>
       <c r="E311" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G311" s="0" t="inlineStr">
@@ -15619,7 +15869,7 @@
       </c>
       <c r="P311" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -16221,7 +16471,12 @@
       </c>
       <c r="E324" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G324" s="0" t="inlineStr">
@@ -16249,7 +16504,7 @@
       </c>
       <c r="P324" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -16641,7 +16896,12 @@
       </c>
       <c r="E333" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G333" s="0" t="inlineStr">
@@ -16669,7 +16929,7 @@
       </c>
       <c r="P333" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -17246,7 +17506,12 @@
       </c>
       <c r="E346" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G346" s="0" t="inlineStr">
@@ -17274,7 +17539,7 @@
       </c>
       <c r="P346" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -17291,7 +17556,12 @@
       </c>
       <c r="E347" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G347" s="0" t="inlineStr">
@@ -17319,7 +17589,7 @@
       </c>
       <c r="P347" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -17471,7 +17741,12 @@
       </c>
       <c r="E351" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G351" s="0" t="inlineStr">
@@ -17499,7 +17774,7 @@
       </c>
       <c r="P351" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17791,12 @@
       </c>
       <c r="E352" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G352" s="0" t="inlineStr">
@@ -17544,7 +17824,7 @@
       </c>
       <c r="P352" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -17656,7 +17936,12 @@
       </c>
       <c r="E355" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G355" s="0" t="inlineStr">
@@ -17684,7 +17969,7 @@
       </c>
       <c r="P355" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -17981,7 +18266,12 @@
       </c>
       <c r="E362" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G362" s="0" t="inlineStr">
@@ -18009,7 +18299,7 @@
       </c>
       <c r="P362" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -18261,7 +18551,12 @@
       </c>
       <c r="E368" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G368" s="0" t="inlineStr">
@@ -18289,7 +18584,7 @@
       </c>
       <c r="P368" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -18306,7 +18601,12 @@
       </c>
       <c r="E369" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G369" s="0" t="inlineStr">
@@ -18334,7 +18634,7 @@
       </c>
       <c r="P369" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -18451,7 +18751,12 @@
       </c>
       <c r="E372" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G372" s="0" t="inlineStr">
@@ -18479,7 +18784,7 @@
       </c>
       <c r="P372" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -18696,7 +19001,12 @@
       </c>
       <c r="E377" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G377" s="0" t="inlineStr">
@@ -18724,7 +19034,7 @@
       </c>
       <c r="P377" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -18891,7 +19201,12 @@
       </c>
       <c r="E381" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G381" s="0" t="inlineStr">
@@ -18919,7 +19234,7 @@
       </c>
       <c r="P381" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -18936,7 +19251,12 @@
       </c>
       <c r="E382" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G382" s="0" t="inlineStr">
@@ -18964,7 +19284,7 @@
       </c>
       <c r="P382" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -19026,7 +19346,12 @@
       </c>
       <c r="E384" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G384" s="0" t="inlineStr">
@@ -19054,7 +19379,7 @@
       </c>
       <c r="P384" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -19071,7 +19396,12 @@
       </c>
       <c r="E385" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G385" s="0" t="inlineStr">
@@ -19099,7 +19429,7 @@
       </c>
       <c r="P385" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
         </is>
       </c>
     </row>
@@ -19816,7 +20146,12 @@
       </c>
       <c r="E401" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G401" s="0" t="inlineStr">
@@ -19844,7 +20179,7 @@
       </c>
       <c r="P401" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -20213,7 +20548,12 @@
       </c>
       <c r="E409" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G409" s="0" t="inlineStr">
@@ -20241,7 +20581,7 @@
       </c>
       <c r="P409" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -20353,7 +20693,12 @@
       </c>
       <c r="E412" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G412" s="0" t="inlineStr">
@@ -20381,7 +20726,7 @@
       </c>
       <c r="P412" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -20633,7 +20978,12 @@
       </c>
       <c r="E418" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G418" s="0" t="inlineStr">
@@ -20661,7 +21011,7 @@
       </c>
       <c r="P418" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -20913,7 +21263,12 @@
       </c>
       <c r="E424" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G424" s="0" t="inlineStr">
@@ -20941,7 +21296,7 @@
       </c>
       <c r="P424" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -21493,7 +21848,12 @@
       </c>
       <c r="E436" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G436" s="0" t="inlineStr">
@@ -21521,7 +21881,7 @@
       </c>
       <c r="P436" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -21638,7 +21998,12 @@
       </c>
       <c r="E439" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G439" s="0" t="inlineStr">
@@ -21666,7 +22031,7 @@
       </c>
       <c r="P439" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -21733,7 +22098,12 @@
       </c>
       <c r="E441" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G441" s="0" t="inlineStr">
@@ -21761,7 +22131,7 @@
       </c>
       <c r="P441" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -22092,7 +22462,12 @@
       </c>
       <c r="E448" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G448" s="0" t="inlineStr">
@@ -22120,7 +22495,7 @@
       </c>
       <c r="P448" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -22356,7 +22731,12 @@
       </c>
       <c r="E453" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G453" s="0" t="inlineStr">
@@ -22384,7 +22764,7 @@
       </c>
       <c r="P453" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -22786,7 +23166,12 @@
       </c>
       <c r="E462" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G462" s="0" t="inlineStr">
@@ -22814,7 +23199,7 @@
       </c>
       <c r="P462" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -23121,7 +23506,12 @@
       </c>
       <c r="E469" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G469" s="0" t="inlineStr">
@@ -23149,7 +23539,7 @@
       </c>
       <c r="P469" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -23166,7 +23556,12 @@
       </c>
       <c r="E470" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G470" s="0" t="inlineStr">
@@ -23194,7 +23589,7 @@
       </c>
       <c r="P470" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -24017,7 +24412,12 @@
       </c>
       <c r="E488" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G488" s="0" t="inlineStr">
@@ -24045,7 +24445,7 @@
       </c>
       <c r="P488" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -24157,7 +24557,12 @@
       </c>
       <c r="E491" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G491" s="0" t="inlineStr">
@@ -24185,7 +24590,7 @@
       </c>
       <c r="P491" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -24693,14 +25098,10 @@
       </c>
       <c r="E502" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F502" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F502" s="0" t="n"/>
       <c r="G502" s="0" t="inlineStr">
         <is>
           <t>Boundary-spanning activity was studied in a large manufacturing company through a sample of 192 managers, engineers, and supervisors. Contrary to prior theory and research, this study found boundary-spanning activity unrelated to role conflict or ambiguity and positively related to job satisfac-tion for the total sample. Boundary-spanning activity was also positively related to a number of job characteristics for the total sample. Marked dif-ferences in boundary-spanning activity and its relationships with other variables, however, were found across occupational levels. While managers and engineers generally had boundary-spanning activity related to high levels of job satisfaction and job characteristics, first-level supervisors had boundary-spanning activity related to higher role conflict and lower job satisfaction with opportunities for promotion.</t>
@@ -24726,7 +25127,7 @@
       </c>
       <c r="P502" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Empirical quantitative study measuring individual-level employee boundary spanning behavior and reporting statistical effect sizes. [Restored after deep methodology audit]</t>
         </is>
       </c>
     </row>
@@ -25220,7 +25621,12 @@
       </c>
       <c r="E513" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G513" s="0" t="inlineStr">
@@ -25248,7 +25654,7 @@
       </c>
       <c r="P513" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -25360,7 +25766,12 @@
       </c>
       <c r="E516" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G516" s="0" t="inlineStr">
@@ -25388,7 +25799,7 @@
       </c>
       <c r="P516" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -25505,7 +25916,12 @@
       </c>
       <c r="E519" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G519" s="0" t="inlineStr">
@@ -25533,7 +25949,7 @@
       </c>
       <c r="P519" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -25550,7 +25966,12 @@
       </c>
       <c r="E520" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G520" s="0" t="inlineStr">
@@ -25578,7 +25999,7 @@
       </c>
       <c r="P520" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -25931,7 +26352,12 @@
       </c>
       <c r="E528" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G528" s="0" t="inlineStr">
@@ -25959,7 +26385,7 @@
       </c>
       <c r="P528" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -26021,7 +26447,12 @@
       </c>
       <c r="E530" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G530" s="0" t="inlineStr">
@@ -26049,7 +26480,7 @@
       </c>
       <c r="P530" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -26301,7 +26732,12 @@
       </c>
       <c r="E536" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G536" s="0" t="inlineStr">
@@ -26329,7 +26765,7 @@
       </c>
       <c r="P536" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -26731,7 +27167,12 @@
       </c>
       <c r="E545" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G545" s="0" t="inlineStr">
@@ -26759,7 +27200,7 @@
       </c>
       <c r="P545" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -27241,7 +27682,12 @@
       </c>
       <c r="E556" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G556" s="0" t="inlineStr">
@@ -27269,7 +27715,7 @@
       </c>
       <c r="P556" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -27386,7 +27832,12 @@
       </c>
       <c r="E559" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G559" s="0" t="inlineStr">
@@ -27425,7 +27876,7 @@
       </c>
       <c r="P559" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -27632,7 +28083,12 @@
       </c>
       <c r="E564" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G564" s="0" t="inlineStr">
@@ -27660,7 +28116,7 @@
       </c>
       <c r="P564" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -28307,7 +28763,12 @@
       </c>
       <c r="E578" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G578" s="0" t="inlineStr">
@@ -28335,7 +28796,7 @@
       </c>
       <c r="P578" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -28397,7 +28858,12 @@
       </c>
       <c r="E580" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G580" s="0" t="inlineStr">
@@ -28425,7 +28891,7 @@
       </c>
       <c r="P580" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -29542,7 +30008,12 @@
       </c>
       <c r="E604" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G604" s="0" t="inlineStr">
@@ -29570,7 +30041,7 @@
       </c>
       <c r="P604" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -29587,7 +30058,12 @@
       </c>
       <c r="E605" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G605" s="0" t="inlineStr">
@@ -29615,7 +30091,7 @@
       </c>
       <c r="P605" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -30087,7 +30563,12 @@
       </c>
       <c r="E616" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G616" s="0" t="inlineStr">
@@ -30115,7 +30596,7 @@
       </c>
       <c r="P616" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -30177,7 +30658,12 @@
       </c>
       <c r="E618" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G618" s="0" t="inlineStr">
@@ -30205,7 +30691,7 @@
       </c>
       <c r="P618" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -30222,7 +30708,12 @@
       </c>
       <c r="E619" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G619" s="0" t="inlineStr">
@@ -30250,7 +30741,7 @@
       </c>
       <c r="P619" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -30367,7 +30858,12 @@
       </c>
       <c r="E622" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G622" s="0" t="inlineStr">
@@ -30395,7 +30891,7 @@
       </c>
       <c r="P622" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -30412,7 +30908,12 @@
       </c>
       <c r="E623" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G623" s="0" t="inlineStr">
@@ -30440,7 +30941,7 @@
       </c>
       <c r="P623" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -30457,7 +30958,12 @@
       </c>
       <c r="E624" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G624" s="0" t="inlineStr">
@@ -30485,7 +30991,7 @@
       </c>
       <c r="P624" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -30922,7 +31428,12 @@
       </c>
       <c r="E634" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G634" s="0" t="inlineStr">
@@ -30950,7 +31461,7 @@
       </c>
       <c r="P634" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -31057,7 +31568,12 @@
       </c>
       <c r="E637" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G637" s="0" t="inlineStr">
@@ -31085,7 +31601,7 @@
       </c>
       <c r="P637" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -31387,7 +31903,12 @@
       </c>
       <c r="E644" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G644" s="0" t="inlineStr">
@@ -31415,7 +31936,7 @@
       </c>
       <c r="P644" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -31432,7 +31953,12 @@
       </c>
       <c r="E645" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G645" s="0" t="inlineStr">
@@ -31460,7 +31986,7 @@
       </c>
       <c r="P645" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -31617,7 +32143,12 @@
       </c>
       <c r="E649" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G649" s="0" t="inlineStr">
@@ -31645,7 +32176,7 @@
       </c>
       <c r="P649" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -31707,14 +32238,10 @@
       </c>
       <c r="E651" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F651" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F651" s="0" t="n"/>
       <c r="G651" s="0" t="inlineStr">
         <is>
           <t>This study examines the impact of emotional intelligence (EI) on boundaryspanning behavior, relationship quality, and performance among door‐todoor salespeople. Data is collected from salespeople and customers of South Korean door‐to‐door cosmetics businesses and analyzed using structural equation modeling. The findings show that EI positively affects boundaryspanning behavior. Similarly, boundary‐spanning behavior improves relationship quality, which improves both sales performance and customer satisfaction. This suggests that EI plays an important role in salespeople's boundaryspanning behavior, thereby enhancing relationship quality, sales performance, and customer satisfaction. Unlike previous studies, this study makes use of actual sales volumes, salespeople's self‐reporting responses, and salespeople's customer‐reporting, which adds to the findings' uniqueness. The present study highlights that EI improves boundary‐spanning behavior, which is vital in developing relationship quality, improving sales performance, and increasing customer satisfaction. The study uses triadic data from door‐to‐door salespeople, customers, and sales organizations extensively, which is unusual in this field.</t>
@@ -31740,7 +32267,7 @@
       </c>
       <c r="P651" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Empirical quantitative study measuring individual-level employee boundary spanning behavior and reporting statistical effect sizes. [Restored after deep methodology audit]</t>
         </is>
       </c>
     </row>
@@ -31757,7 +32284,12 @@
       </c>
       <c r="E652" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G652" s="0" t="inlineStr">
@@ -31785,7 +32317,7 @@
       </c>
       <c r="P652" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -32277,7 +32809,12 @@
       </c>
       <c r="E663" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G663" s="0" t="inlineStr">
@@ -32305,7 +32842,7 @@
       </c>
       <c r="P663" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -32417,7 +32954,12 @@
       </c>
       <c r="E666" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G666" s="0" t="inlineStr">
@@ -32445,7 +32987,7 @@
       </c>
       <c r="P666" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -32507,7 +33049,12 @@
       </c>
       <c r="E668" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G668" s="0" t="inlineStr">
@@ -32535,7 +33082,7 @@
       </c>
       <c r="P668" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -32747,7 +33294,12 @@
       </c>
       <c r="E673" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G673" s="0" t="inlineStr">
@@ -32775,7 +33327,7 @@
       </c>
       <c r="P673" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -33090,7 +33642,12 @@
       </c>
       <c r="E680" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G680" s="0" t="inlineStr">
@@ -33118,7 +33675,7 @@
       </c>
       <c r="P680" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -33700,7 +34257,12 @@
       </c>
       <c r="E693" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G693" s="0" t="inlineStr">
@@ -33728,7 +34290,7 @@
       </c>
       <c r="P693" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
         </is>
       </c>
     </row>
@@ -33745,7 +34307,12 @@
       </c>
       <c r="E694" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G694" s="0" t="inlineStr">
@@ -33773,7 +34340,7 @@
       </c>
       <c r="P694" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -34075,7 +34642,12 @@
       </c>
       <c r="E701" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G701" s="0" t="inlineStr">
@@ -34103,7 +34675,7 @@
       </c>
       <c r="P701" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
         </is>
       </c>
     </row>
@@ -34120,7 +34692,12 @@
       </c>
       <c r="E702" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G702" s="0" t="inlineStr">
@@ -34148,7 +34725,7 @@
       </c>
       <c r="P702" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 01 Full-Text Audit of Included papers, removing 3 false positives (BSMA0016, 0022, 0048). Final Included: 270
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -1654,7 +1654,12 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">
@@ -1682,7 +1687,7 @@
       </c>
       <c r="P19" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative Collaborative Autoethnography without individual employee Pearson correlation matrix. [Found during Batch 01 Full-Text Audit]</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1707,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -1897,7 +1902,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -1944,7 +1949,12 @@
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
@@ -1975,7 +1985,7 @@
       </c>
       <c r="P25" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Comparative case analysis of 11 manufacturing plants without an individual employee bivariate Pearson correlation matrix. [Found during Batch 01 Full-Text Audit]</t>
         </is>
       </c>
     </row>
@@ -1995,7 +2005,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -2045,7 +2055,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -2145,7 +2155,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -2495,7 +2505,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -2545,7 +2555,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -2790,7 +2800,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -2890,7 +2900,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -3080,7 +3090,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -3222,7 +3232,12 @@
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
@@ -3250,7 +3265,7 @@
       </c>
       <c r="P51" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro / Cluster level study: Examines inter-organizational trilateral collaborations across science, education, and business sectors. [Found during Batch 01 Full-Text Audit]</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3655,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -3985,7 +4000,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -4080,7 +4095,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -4849,7 +4864,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F84" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -4949,7 +4964,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F86" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -5344,7 +5359,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr">
+      <c r="F94" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -5489,7 +5504,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr">
+      <c r="F97" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -5684,7 +5699,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr">
+      <c r="F101" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -5869,7 +5884,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr">
+      <c r="F105" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -5919,7 +5934,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
+      <c r="F106" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -6069,7 +6084,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
+      <c r="F109" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -6219,7 +6234,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
+      <c r="F112" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -6319,7 +6334,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
+      <c r="F114" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -6904,7 +6919,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr">
+      <c r="F126" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -8017,7 +8032,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr">
+      <c r="F149" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -8407,7 +8422,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr">
+      <c r="F157" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -8892,7 +8907,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr">
+      <c r="F167" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -9082,7 +9097,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr">
+      <c r="F171" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -9373,7 +9388,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr">
+      <c r="F177" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -9823,7 +9838,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr">
+      <c r="F186" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -10158,7 +10173,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr">
+      <c r="F193" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -10393,7 +10408,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr">
+      <c r="F198" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -10443,7 +10458,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="F199" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -10833,7 +10848,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F207" t="inlineStr">
+      <c r="F207" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -11113,7 +11128,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F213" t="inlineStr">
+      <c r="F213" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -11548,7 +11563,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F222" t="inlineStr">
+      <c r="F222" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -12178,7 +12193,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr">
+      <c r="F235" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -12318,7 +12333,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr">
+      <c r="F238" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -13033,7 +13048,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr">
+      <c r="F253" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -13083,7 +13098,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr">
+      <c r="F254" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -13333,7 +13348,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F259" t="inlineStr">
+      <c r="F259" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -13663,7 +13678,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F266" t="inlineStr">
+      <c r="F266" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -14078,7 +14093,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F275" t="inlineStr">
+      <c r="F275" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -14531,7 +14546,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr">
+      <c r="F284" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -15075,7 +15090,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F295" t="inlineStr">
+      <c r="F295" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -15355,7 +15370,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F301" t="inlineStr">
+      <c r="F301" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -15505,7 +15520,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F304" t="inlineStr">
+      <c r="F304" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -15600,7 +15615,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F306" t="inlineStr">
+      <c r="F306" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -15695,7 +15710,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F308" t="inlineStr">
+      <c r="F308" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -15839,7 +15854,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F311" t="inlineStr">
+      <c r="F311" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -16474,7 +16489,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F324" t="inlineStr">
+      <c r="F324" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -16899,7 +16914,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F333" t="inlineStr">
+      <c r="F333" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -17509,7 +17524,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F346" t="inlineStr">
+      <c r="F346" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -17559,7 +17574,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F347" t="inlineStr">
+      <c r="F347" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -17744,7 +17759,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F351" t="inlineStr">
+      <c r="F351" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -17794,7 +17809,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F352" t="inlineStr">
+      <c r="F352" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -17939,7 +17954,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F355" t="inlineStr">
+      <c r="F355" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18269,7 +18284,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F362" t="inlineStr">
+      <c r="F362" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18554,7 +18569,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F368" t="inlineStr">
+      <c r="F368" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18604,7 +18619,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F369" t="inlineStr">
+      <c r="F369" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18754,7 +18769,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F372" t="inlineStr">
+      <c r="F372" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -19004,7 +19019,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F377" t="inlineStr">
+      <c r="F377" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -19204,7 +19219,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F381" t="inlineStr">
+      <c r="F381" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -19254,7 +19269,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F382" t="inlineStr">
+      <c r="F382" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -19349,7 +19364,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F384" t="inlineStr">
+      <c r="F384" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -19399,7 +19414,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F385" t="inlineStr">
+      <c r="F385" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -20149,7 +20164,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F401" t="inlineStr">
+      <c r="F401" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -20551,7 +20566,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F409" t="inlineStr">
+      <c r="F409" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -20696,7 +20711,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F412" t="inlineStr">
+      <c r="F412" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -20981,7 +20996,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F418" t="inlineStr">
+      <c r="F418" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -21266,7 +21281,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F424" t="inlineStr">
+      <c r="F424" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -21851,7 +21866,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F436" t="inlineStr">
+      <c r="F436" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -22001,7 +22016,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F439" t="inlineStr">
+      <c r="F439" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -22101,7 +22116,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F441" t="inlineStr">
+      <c r="F441" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -22465,7 +22480,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F448" t="inlineStr">
+      <c r="F448" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -22734,7 +22749,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F453" t="inlineStr">
+      <c r="F453" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -23169,7 +23184,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F462" t="inlineStr">
+      <c r="F462" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -23509,7 +23524,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F469" t="inlineStr">
+      <c r="F469" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -23559,7 +23574,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F470" t="inlineStr">
+      <c r="F470" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -24415,7 +24430,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F488" t="inlineStr">
+      <c r="F488" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -24560,7 +24575,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F491" t="inlineStr">
+      <c r="F491" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -25624,7 +25639,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F513" t="inlineStr">
+      <c r="F513" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -25769,7 +25784,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F516" t="inlineStr">
+      <c r="F516" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -25919,7 +25934,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F519" t="inlineStr">
+      <c r="F519" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -25969,7 +25984,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F520" t="inlineStr">
+      <c r="F520" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -26355,7 +26370,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F528" t="inlineStr">
+      <c r="F528" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -26450,7 +26465,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F530" t="inlineStr">
+      <c r="F530" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -26735,7 +26750,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F536" t="inlineStr">
+      <c r="F536" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -27170,7 +27185,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F545" t="inlineStr">
+      <c r="F545" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -27685,7 +27700,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F556" t="inlineStr">
+      <c r="F556" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -27835,7 +27850,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F559" t="inlineStr">
+      <c r="F559" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -28086,7 +28101,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F564" t="inlineStr">
+      <c r="F564" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -28766,7 +28781,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F578" t="inlineStr">
+      <c r="F578" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -28861,7 +28876,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F580" t="inlineStr">
+      <c r="F580" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -30011,7 +30026,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F604" t="inlineStr">
+      <c r="F604" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -30061,7 +30076,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F605" t="inlineStr">
+      <c r="F605" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -30566,7 +30581,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F616" t="inlineStr">
+      <c r="F616" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -30661,7 +30676,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F618" t="inlineStr">
+      <c r="F618" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -30711,7 +30726,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F619" t="inlineStr">
+      <c r="F619" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -30861,7 +30876,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F622" t="inlineStr">
+      <c r="F622" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -30911,7 +30926,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F623" t="inlineStr">
+      <c r="F623" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -30961,7 +30976,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F624" t="inlineStr">
+      <c r="F624" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -31431,7 +31446,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F634" t="inlineStr">
+      <c r="F634" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -31571,7 +31586,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F637" t="inlineStr">
+      <c r="F637" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -31906,7 +31921,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F644" t="inlineStr">
+      <c r="F644" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -31956,7 +31971,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F645" t="inlineStr">
+      <c r="F645" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -32146,7 +32161,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F649" t="inlineStr">
+      <c r="F649" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -32287,7 +32302,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F652" t="inlineStr">
+      <c r="F652" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -32812,7 +32827,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F663" t="inlineStr">
+      <c r="F663" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -32957,7 +32972,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F666" t="inlineStr">
+      <c r="F666" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -33052,7 +33067,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F668" t="inlineStr">
+      <c r="F668" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -33297,7 +33312,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F673" t="inlineStr">
+      <c r="F673" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -33645,7 +33660,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F680" t="inlineStr">
+      <c r="F680" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -34260,7 +34275,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F693" t="inlineStr">
+      <c r="F693" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -34310,7 +34325,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F694" t="inlineStr">
+      <c r="F694" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -34645,7 +34660,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F701" t="inlineStr">
+      <c r="F701" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -34695,7 +34710,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F702" t="inlineStr">
+      <c r="F702" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>

</xml_diff>

<commit_message>
Data Clean: Updated Batch 01 excluded papers (BSMA0016, 0022, 0048) with exact Verbatim Evidence quotes in Excel Col 16
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -1657,7 +1657,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="P19" s="0" t="inlineStr">
         <is>
-          <t>Qualitative Collaborative Autoethnography without individual employee Pearson correlation matrix. [Found during Batch 01 Full-Text Audit]</t>
+          <t>Qualitative study without correlation matrix. Verbatim Evidence: "The study employs a collaborative analytical autoethnography where, through memo-writings, emails, and reflective notes by the second author, it micro-theorizes the political, technical, and cultural activities that the institutional entrepreneur carried in order to harmonize Montenegro's anti-doping policy with WADA." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1952,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="P25" s="0" t="inlineStr">
         <is>
-          <t>Comparative case analysis of 11 manufacturing plants without an individual employee bivariate Pearson correlation matrix. [Found during Batch 01 Full-Text Audit]</t>
+          <t>Comparative case analysis without individual employee Pearson correlation matrix. Verbatim Evidence: "I chose to identify a few similar manufacturing organizations... I find that in response to changing water-pollution regulation, top managers indeed created specialized pollution-control departments to insulate the existing process..." (Methodology / Sample section)</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="P51" s="0" t="inlineStr">
         <is>
-          <t>Macro / Cluster level study: Examines inter-organizational trilateral collaborations across science, education, and business sectors. [Found during Batch 01 Full-Text Audit]</t>
+          <t>Macro / Cluster level study of inter-organizational networks. Verbatim Evidence: "To investigate these issues, the authors applied network analysis to study an innovation cluster in Algarve, Portugal. They found that cross-boundary organizational collaborations corresponded with personal ties." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 02 Full-Text Audit of Included papers, removing 5 false positives with verbatim quotes. Final Included: 265
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -3327,7 +3327,12 @@
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
@@ -3355,7 +3360,7 @@
       </c>
       <c r="P53" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Descriptive frequency survey of audit committee meetings without an individual employee Pearson correlation matrix. Verbatim Evidence: "This paper's empirical contribution is to investigate the extent to which ACs and audit committee chairs (ACCs) engage with chief financial officers (CFOs) and audit partners (APs) across a range of 32 financial reporting issues... Table 1 shows the 32 issues in the order that they appeared in the questionnaire." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3427,12 @@
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
@@ -3450,7 +3460,7 @@
       </c>
       <c r="P55" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level aggregation study. Verbatim Evidence: "The results of the structural equation model from a sample of 92 interdisciplinary teams indicate that leaders' internal activities fully mediate the relationship of team functional heterogeneity and interteam goal interdependence to team in-role performance (N = 92 teams)." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3712,12 @@
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
@@ -3735,7 +3750,7 @@
       </c>
       <c r="P61" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Sample consists of organizational buyers (customers/clients), not internal workplace employees. Verbatim Evidence: "The model is tested on a sample of 120 organizational buyers of advertising services by using partial least squares, a structural equation modelling technique." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3817,12 @@
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
@@ -3830,7 +3850,7 @@
       </c>
       <c r="P63" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Pure conceptual / theoretical paper without quantitative employee survey correlation data. Verbatim Evidence: "We examine in detail what the temporal imagination is, complemented with a discussion of the related timescape idea, and why the temporal imagination is necessary to function in any timescape. We also discuss group attributes that will likely affect the development..." (Abstract / Introduction section)</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4491,12 @@
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
@@ -4499,7 +4524,7 @@
       </c>
       <c r="P76" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative field interview study without individual employee Pearson correlation matrix. Verbatim Evidence: "Some interviewees were less concerned by this lack of basic training, believing instead that the onshore... For example, in the sample we checked if the cut-off of the invoices was correct." (Abstract / Findings section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 03 Full-Text Audit of Included papers, removing 6 false positives with verbatim quotes. Final Included: 259
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -3330,7 +3330,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -3430,7 +3430,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -3715,7 +3715,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -3820,7 +3820,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -4494,7 +4494,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -5816,7 +5816,12 @@
       </c>
       <c r="E103" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G103" s="0" t="inlineStr">
@@ -5844,7 +5849,7 @@
       </c>
       <c r="P103" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project/Team-level aggregation study. Verbatim Evidence: "This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates... Note: Dependent variable: (L) Learning rate, N = 47, N = 183 projects." (Abstract / Table 3-4 section)</t>
         </is>
       </c>
     </row>
@@ -5861,7 +5866,12 @@
       </c>
       <c r="E104" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G104" s="0" t="inlineStr">
@@ -5889,7 +5899,7 @@
       </c>
       <c r="P104" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project/Team-level aggregation study. Verbatim Evidence: "The final sample was reduced to 101 projects since only that number had archived full data on all development activities. For the 101 projects, repeated measures were taken on a quarterly basis since the beginning..." (Methodology / Sample section)</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6566,12 @@
       </c>
       <c r="E118" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G118" s="0" t="inlineStr">
@@ -6584,7 +6599,7 @@
       </c>
       <c r="P118" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative interview / conceptual study without individual employee Pearson correlation matrix. Verbatim Evidence: "We composed a theoretical rather than representative sample of professionals who are boundary spanners and tasked with innovation search who had been granted a great deal of autonomy over their time." (Methodology / Sample section)</t>
         </is>
       </c>
     </row>
@@ -6991,7 +7006,12 @@
       </c>
       <c r="E127" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G127" s="0" t="inlineStr">
@@ -7020,7 +7040,7 @@
       </c>
       <c r="P127" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level aggregation study of product development teams without individual employee Pearson correlation matrix. Verbatim Evidence: "Data from 409 members of 45 new product teams in five high-technology companies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator, Scout, and Guard." (Abstract section)</t>
         </is>
       </c>
     </row>
@@ -7135,7 +7155,12 @@
       </c>
       <c r="E130" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G130" s="0" t="inlineStr">
@@ -7163,7 +7188,7 @@
       </c>
       <c r="P130" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Ticket/Task-level aggregation study of IT support community. Verbatim Evidence: "Then the ticket complexity scores are aggregated on a monthly basis per worker... Table 1 presents the descriptive statistics and correlations of the variables across 320 monthly aggregated worker ticket observations." (Methodology / Data analysis section)</t>
         </is>
       </c>
     </row>
@@ -7325,7 +7350,12 @@
       </c>
       <c r="E134" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G134" s="0" t="inlineStr">
@@ -7353,7 +7383,7 @@
       </c>
       <c r="P134" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative field consulting case study without individual employee Pearson correlation matrix. Verbatim Evidence: "Using an external perspective as a research lens, this study examined team-context interaction in five consulting teams. The data revealed three strategies toward the teams' environment: informing, parading, and probing." (Abstract section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 04 Full-Text Audit of Included papers, removing 5 false positives with verbatim quotes. Final Included: 254
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -5819,7 +5819,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
+      <c r="F103" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -5869,7 +5869,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr">
+      <c r="F104" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -6569,7 +6569,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr">
+      <c r="F118" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -7009,7 +7009,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr">
+      <c r="F127" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -7158,7 +7158,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr">
+      <c r="F130" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -7353,7 +7353,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr">
+      <c r="F134" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -8379,7 +8379,12 @@
       </c>
       <c r="E155" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G155" s="0" t="inlineStr">
@@ -8407,7 +8412,7 @@
       </c>
       <c r="P155" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro / Firm-level study of supply-side resilience. Verbatim Evidence: "An electronic survey was used where the initial sample consisted of 1,641 manufacturing firms (SIC codes 20–51) listed by Dun and Bradstreet... The focus of research has been at an organisational level without incorporating the role of boundary spanning individuals." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8679,12 @@
       </c>
       <c r="E161" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G161" s="0" t="inlineStr">
@@ -8702,7 +8712,7 @@
       </c>
       <c r="P161" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro / Firm-level Market Orientation study. Verbatim Evidence: "Specifically, this research draws on the Job Demands-Resources model to explore the effect of employee perceptions of firm market orientation as a way to reduce role stressors and subsequently turnover intentions... Sample of 260 respondents who were employed full-time and worked in either B2B or B2C sales." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>
@@ -8719,7 +8729,12 @@
       </c>
       <c r="E162" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G162" s="0" t="inlineStr">
@@ -8747,7 +8762,7 @@
       </c>
       <c r="P162" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Bibliometric / archival study of Open Source software developers, not organizational employees. Verbatim Evidence: "Tables 1 and 2 describe the 610 subjects who published prior to working group chair appointment or censoring, observed over 5,066 trimesters... Open source operating systems challenge the world's most powerful software firms." (Methodology / Variables section)</t>
         </is>
       </c>
     </row>
@@ -9250,7 +9265,12 @@
       </c>
       <c r="E173" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G173" s="0" t="inlineStr">
@@ -9278,7 +9298,7 @@
       </c>
       <c r="P173" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro / Firm-level study of knowledge search and innovation. Verbatim Evidence: "Using a sample of 1,088 Chinese firms' data collected by the World Bank in 2012, this paper employs logistic regression to test the hypotheses. This study finds that local and boundary-spanning search strategies positively influence both product and process innovation." (Abstract / Findings section)</t>
         </is>
       </c>
     </row>
@@ -9940,7 +9960,12 @@
       </c>
       <c r="E187" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G187" s="0" t="inlineStr">
@@ -9968,7 +9993,7 @@
       </c>
       <c r="P187" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team/Project-level aggregation study. Verbatim Evidence: "We ran an OLS regression model to test H1 regarding the relationship between external activity and effectiveness... In the second step the overall R-square was .07 (F(4,139)=2.74, p&lt;.05) across 144 documentary film making teams." (Abstract / Table 2 section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 05 Full-Text Audit of Included papers, removing 5 false positives with verbatim quotes. Final Included: 249
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -8382,7 +8382,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr">
+      <c r="F155" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -8682,7 +8682,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr">
+      <c r="F161" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -8732,7 +8732,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr">
+      <c r="F162" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -9268,7 +9268,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr">
+      <c r="F173" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -9963,7 +9963,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr">
+      <c r="F187" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -10350,7 +10350,12 @@
       </c>
       <c r="E195" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G195" s="0" t="inlineStr">
@@ -10378,7 +10383,7 @@
       </c>
       <c r="P195" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Descriptive survey of Link Officers without individual employee Pearson correlation matrix. Verbatim Evidence: "The survey was developed with input from IOs to ensure that survey questions were relevant to LPs and LOs. The survey involved a mixture of open and closed questions... Table 1. Characteristics of Link Officers (LOs) and Link Partners (LPs)." (Methodology / Sample and procedure section)</t>
         </is>
       </c>
     </row>
@@ -10395,7 +10400,12 @@
       </c>
       <c r="E196" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G196" s="0" t="inlineStr">
@@ -10423,7 +10433,7 @@
       </c>
       <c r="P196" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level aggregation study. Verbatim Evidence: "The members of 126 multidisciplinary teams responded to a survey on several aspects related to the functioning and leadership of their teams... In this study, 126 CPCY teams participated (654 individuals)." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -10835,7 +10845,12 @@
       </c>
       <c r="E205" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G205" s="0" t="inlineStr">
@@ -10863,7 +10878,7 @@
       </c>
       <c r="P205" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative study without quantitative employee survey correlation data. Verbatim Evidence: "This exploratory qualitative study used a semi-structured interview protocol with a purposeful sample of 27 Indian American professionals... The perception of innovation and how individuals define innovation..." (Abstract / Research Design section)</t>
         </is>
       </c>
     </row>
@@ -11025,7 +11040,12 @@
       </c>
       <c r="E209" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G209" s="0" t="inlineStr">
@@ -11053,7 +11073,7 @@
       </c>
       <c r="P209" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Macro / Firm-level study of Turkish software firms. Verbatim Evidence: "A number of studies have shown that transformational leadership positively influences organizational innovation. However, there is a lack of studies examining... sample of 110 manufacturing firms in China... turkish software development firms." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>
@@ -11160,7 +11180,12 @@
       </c>
       <c r="E212" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G212" s="0" t="inlineStr">
@@ -11188,7 +11213,7 @@
       </c>
       <c r="P212" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team/Project-level aggregation study. Verbatim Evidence: "Analyses of multi-source data from a sample of 96 project teams in a prominent international development agency show that... N = 96 teams." (Abstract / Data analysis section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 05 Full-Text Audit of Included papers, removing 4 false positives with verbatim quotes. Final Included: 245
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -10353,7 +10353,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr">
+      <c r="F195" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -10403,7 +10403,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr">
+      <c r="F196" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -10848,7 +10848,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr">
+      <c r="F205" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -11043,7 +11043,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F209" t="inlineStr">
+      <c r="F209" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -11183,7 +11183,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F212" t="inlineStr">
+      <c r="F212" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -11960,7 +11960,12 @@
       </c>
       <c r="E228" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G228" s="0" t="inlineStr">
@@ -11988,7 +11993,7 @@
       </c>
       <c r="P228" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Sample consists of online gig-economy freelancers on Upwork platform, not internal organizational workplace employees. Verbatim Evidence: "Extant management literature suggests that boundary spanning, defined as... sample of skilled digital freelancers using the Upwork platform, an online marketplace for connecting freelancers and employers." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>
@@ -12105,7 +12110,12 @@
       </c>
       <c r="E231" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G231" s="0" t="inlineStr">
@@ -12133,7 +12143,7 @@
       </c>
       <c r="P231" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Study of external public affairs consulting agencies/consultants without an individual employee Pearson correlation matrix. Verbatim Evidence: "Even though consultants are undoubtedly increasing in importance, their relevance as agents is often downplayed. This study seeks to empirically supplement the perspective of the consultant... All respondents, as well as an additional 87 experts in politics, associations, and corporations were asked to name the most relevant public affairs consultants in Switzerland." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -12250,7 +12260,12 @@
       </c>
       <c r="E234" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G234" s="0" t="inlineStr">
@@ -12278,7 +12293,7 @@
       </c>
       <c r="P234" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Department/Hospital-level organizational study without individual employee Pearson correlation matrix. Verbatim Evidence: "From approximately 750 general hospitals in the 1969 Inventory of Psychiatric Services of the National Institute of Mental Health... 338 inpatient departments were used in the present analysis... Table 2: Correlation Analysis: Size and Performance of Department by Hospital Ownership (N = 47, N = 43, N = 76, N = 172 departments)." (Methodology / Table 2 section)</t>
         </is>
       </c>
     </row>
@@ -12485,7 +12500,12 @@
       </c>
       <c r="E239" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G239" s="0" t="inlineStr">
@@ -12513,7 +12533,7 @@
       </c>
       <c r="P239" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Interorganizational buyer-supplier relationship study where the unit of analysis is the interorganizational exchange / dyad. Verbatim Evidence: "An Investigation of Interpersonal Ties in Interorganizational Exchanges in Emerging Markets: A Boundary-Spanning Perspective... Overall, the manufacturers in our sample have many more employees than do the distributors. Therefore, we use size from the manufacturer side as a control variable across buyer-supplier dyads." (Title / Methodology section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 06 Full-Text Audit of Included papers, removing 4 false positives with verbatim quotes. Final Included: 241
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -11963,7 +11963,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F228" t="inlineStr">
+      <c r="F228" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -12113,7 +12113,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr">
+      <c r="F231" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -12263,7 +12263,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr">
+      <c r="F234" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -12503,7 +12503,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr">
+      <c r="F239" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -13520,7 +13520,12 @@
       </c>
       <c r="E260" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G260" s="0" t="inlineStr">
@@ -13548,7 +13553,7 @@
       </c>
       <c r="P260" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Patent-level technological domain recombination study where the unit of analysis is the patent, not individual employees. Verbatim Evidence: "Prior literature has long examined innovation as a recombination process within or across the boundaries of technological domains... Analyzing a large sample of US patents, we find that spanning crisp boundaries is more likely to generate impactful inventions." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -13850,7 +13855,12 @@
       </c>
       <c r="E267" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G267" s="0" t="inlineStr">
@@ -13878,7 +13888,7 @@
       </c>
       <c r="P267" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level study of corporate R&amp;D network boundary spanning and innovation performance where the unit of analysis is the corporation. Verbatim Evidence: "DOES STRONGER R&amp;D CAPABILITY ALWAYS PROMOTE BETTER INNOVATION? THE MODERATING ROLE OF KNOWLEDGE BOUNDARY SPANNING OF R&amp;D NETWORK... We collected application documents, excluded samples with incomplete data, and ultimately, obtained data of 702 corporations." (Title / Sample section)</t>
         </is>
       </c>
     </row>
@@ -13895,7 +13905,12 @@
       </c>
       <c r="E268" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G268" s="0" t="inlineStr">
@@ -13923,7 +13938,7 @@
       </c>
       <c r="P268" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level study of open innovation and organizational resilience where the unit of analysis is the firm. Verbatim Evidence: "Prospective boundary-spanning search and responsive boundary-spanning search... Prospective boundary-spanning search includes 'our firm often identifies new opportunities in emerging markets before its competitors', 'our firm frequently develops innovative ways to meet customer needs ahead of competitors'... Sample of 293 smart manufacturing firms." (Abstract / Measures section)</t>
         </is>
       </c>
     </row>
@@ -13940,7 +13955,12 @@
       </c>
       <c r="E269" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G269" s="0" t="inlineStr">
@@ -13968,7 +13988,7 @@
       </c>
       <c r="P269" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level statistical aggregation study of team creativity where individual responses are aggregated to the team unit of analysis. Verbatim Evidence: "HOW DOES CREATIVITY OCCUR IN TEAMS? AN EMPIRICAL TEST... Organizations benefit when workteams produce more rather than less creativity... Test of aggregation appropriateness... Sample consisting of 52 work teams across organizations." (Title / Methodology section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 07 Full-Text Audit of Included papers, removing 6 false positives with verbatim quotes. Final Included: 235
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -13523,7 +13523,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F260" t="inlineStr">
+      <c r="F260" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -13858,7 +13858,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr">
+      <c r="F267" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -13908,7 +13908,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F268" t="inlineStr">
+      <c r="F268" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -13958,7 +13958,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F269" t="inlineStr">
+      <c r="F269" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -15033,7 +15033,12 @@
       </c>
       <c r="E291" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G291" s="0" t="inlineStr">
@@ -15061,7 +15066,7 @@
       </c>
       <c r="P291" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project-level statistical aggregation study where the unit of analysis is the R&amp;D project group, not individual employees. Verbatim Evidence: "An investigation into the managerial roles and career paths of gatekeepers and project supervisors in a major R &amp; D facility... In particular, within our sample of development projects, those with gatekeepers were considerably more effective than those without gatekeepers... Table 1. Project performance as a function of gatekeeper presence and project type." (Abstract / Table 1 section)</t>
         </is>
       </c>
     </row>
@@ -15078,7 +15083,12 @@
       </c>
       <c r="E292" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G292" s="0" t="inlineStr">
@@ -15106,7 +15116,7 @@
       </c>
       <c r="P292" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project-level statistical aggregation study where individual communication measures are aggregated to the project unit of analysis (N = 61 projects). Verbatim Evidence: "Communication patterns, project performance and task characteristics: an empirical evaluation and integration in an R&amp;D setting... At the time of this study, 61 such projects existed across the laboratory's seven divisions... Intraproject communication: An examination of the intraproject means and correlation of Table 3... positively associated with performance only for research projects." (Methodology / Results section)</t>
         </is>
       </c>
     </row>
@@ -15327,7 +15337,12 @@
       </c>
       <c r="E297" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G297" s="0" t="inlineStr">
@@ -15355,7 +15370,7 @@
       </c>
       <c r="P297" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative inductive grounded theory ethnographic field study without an individual employee Pearson correlation matrix. Verbatim Evidence: "Life in the Trading Zone: Structuring Coordination Across Boundaries in Postbureaucratic Organizations... Our research study was inductive and focused on generating theoretical insights from an in-depth examination of cross-boundary coordination in practice... analyzed them qualitatively through an iterative process of data examination, grounded coding." (Abstract / Methods section)</t>
         </is>
       </c>
     </row>
@@ -15372,7 +15387,12 @@
       </c>
       <c r="E298" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G298" s="0" t="inlineStr">
@@ -15400,7 +15420,7 @@
       </c>
       <c r="P298" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Student sample enrolled in a Dutch university course participating in a virtual laboratory project simulation, not organizational employees. Verbatim Evidence: "Single versus multiple project teams and individual performance... enrolled at a Dutch university, who were randomly assigned to project teams, as part of a course. In the simulation, participants experienced project work in a virtual MTM setting." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>
@@ -15417,7 +15437,12 @@
       </c>
       <c r="E299" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G299" s="0" t="inlineStr">
@@ -15445,7 +15470,7 @@
       </c>
       <c r="P299" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level study of boundary spanners' knowledge sharing and innovation performance where the unit of analysis is the firm (N = 117 firms). Verbatim Evidence: "Boundary spanners' knowledge sharing for innovation success in turbulent times... Convenience sample of European subsidiaries of multinational companies with headquarters located in Europe... Chief Executive Officers... Final sample size: 117 firms." (Title / Methods section)</t>
         </is>
       </c>
     </row>
@@ -15712,7 +15737,12 @@
       </c>
       <c r="E305" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G305" s="0" t="inlineStr">
@@ -15740,7 +15770,7 @@
       </c>
       <c r="P305" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level statistical aggregation study where individual team member responses are aggregated to the team unit of analysis (N = 80 teams). Verbatim Evidence: "The paradox of building bridges: Examining countervailing effects of leader external brokerage on team performance... In a sample of 465 team members in 80 teams distributed across 10 sister companies... we used multilevel structural equation modeling to test our hypotheses... Table 1 includes the means, standard deviations, and correlations among study variables at the team level." (Abstract / Methods section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 08 Full-Text Audit of Included papers, removing 7 false positives with verbatim quotes. Final Included: 228
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -15036,7 +15036,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr">
+      <c r="F291" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -15086,7 +15086,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F292" t="inlineStr">
+      <c r="F292" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -15340,7 +15340,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr">
+      <c r="F297" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -15390,7 +15390,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F298" t="inlineStr">
+      <c r="F298" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -15440,7 +15440,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F299" t="inlineStr">
+      <c r="F299" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -15740,7 +15740,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F305" t="inlineStr">
+      <c r="F305" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -16326,7 +16326,12 @@
       </c>
       <c r="E317" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G317" s="0" t="inlineStr">
@@ -16354,7 +16359,7 @@
       </c>
       <c r="P317" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level statistical aggregation study of pre-founding entrepreneurial teams where the unit of analysis is the team. Verbatim Evidence: "The Performance of Pre-Founding Entrepreneurial Teams: The Importance of Learning and Leadership... We studied teams who participated in a venture creation programme that combines education and incubation... Sample of 58 teams, 55 teams, 35 teams across conditions." (Title / Methods section)</t>
         </is>
       </c>
     </row>
@@ -16471,7 +16476,12 @@
       </c>
       <c r="E320" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G320" s="0" t="inlineStr">
@@ -16499,7 +16509,7 @@
       </c>
       <c r="P320" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level study of engineering design teams where the unit of analysis is the team (N = 39 teams). Individual questionnaire data is aggregated to team level for analysis. Verbatim Evidence: "The social structure of leadership and creativity in engineering design teams... Based on a sample of 39 engineering design teams in the space industry, this study examines the effects of leader position within different flows of communication on team creativity." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>
@@ -16761,7 +16771,12 @@
       </c>
       <c r="E326" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G326" s="0" t="inlineStr">
@@ -16789,7 +16804,7 @@
       </c>
       <c r="P326" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm/business-unit-level study of knowledge stocks and information flows where the unit of analysis is the firm. Verbatim Evidence: "Knowledge Stocks and Information Flows in New Product Development... A sample of 500 business units from the food processing industry was randomly selected from a business directory, which contains a complete list of food companies... sample of 340 firms, 136 returned the questionnaire." (Title / Methodology section)</t>
         </is>
       </c>
     </row>
@@ -16806,7 +16821,12 @@
       </c>
       <c r="E327" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G327" s="0" t="inlineStr">
@@ -16834,7 +16854,7 @@
       </c>
       <c r="P327" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Volunteer association groups on Meetup.com where the unit of analysis is the online group (N = 171 groups), not individual organizational employees. Verbatim Evidence: "Volunteer associations in the Internet age: Ecological approach to understanding collective action... An online survey was conducted with 171 randomly sampled groups on Meetup.com—a website that facilitates the creation and coordination of mixed-mode groups." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>
@@ -16851,7 +16871,12 @@
       </c>
       <c r="E328" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G328" s="0" t="inlineStr">
@@ -16879,7 +16904,7 @@
       </c>
       <c r="P328" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Student sample enrolled in a full-time MBA program assigned to self-managing teams as part of coursework, not organizational employees. Verbatim Evidence: "Leadership Over-Emergence in Self-Managing Teams: The Role of Gender and Countervailing Biases... 181 students enrolled in a full time Master of Business Administration (MBA) program at a large research university in the United States. Students were assigned to 5-person self-managing teams." (Sample section)</t>
         </is>
       </c>
     </row>
@@ -16946,7 +16971,12 @@
       </c>
       <c r="E330" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G330" s="0" t="inlineStr">
@@ -16974,7 +17004,7 @@
       </c>
       <c r="P330" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Online crowd-based innovation challenge evaluators assessing NASA Astrobee solutions, not individual organizational employees performing boundary spanning roles. Verbatim Evidence: "Beyond feasibility filters: How expertise heterogeneity enables innovation recognition... a field experiment with National Aeronautics and Space Administration's (NASA) Astrobee Robotic Arm Challenge, involving 354 evaluators assessing 101 solutions." (Abstract / Methods section)</t>
         </is>
       </c>
     </row>
@@ -16991,7 +17021,12 @@
       </c>
       <c r="E331" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G331" s="0" t="inlineStr">
@@ -17019,7 +17054,7 @@
       </c>
       <c r="P331" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Organization-level study of nonprofit human service organizations where the unit of analysis is the organization (N = 291 organizations). Verbatim Evidence: "Developmental Culture and Effectiveness in Nonprofit Organizations... A total of 778 organizations were surveyed, and the overall project had a response rate of 37% (n = 291). Organizations were sampled primarily from the NTEE codes representing center-based human services." (Sample section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 09 Full-Text Audit, removing 4 false positives with verbatim quotes. Final Included: 224
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -15981,7 +15981,12 @@
       </c>
       <c r="E310" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G310" s="0" t="inlineStr">
@@ -16009,7 +16014,7 @@
       </c>
       <c r="P310" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative multiple case study using interviews and ethnographic observation without individual employee Pearson correlation matrix. Verbatim Evidence: "The data for our studies came from two separate cases... In both cases, the data was collected in two sets... Table 1: Summary of the two data sets... Number and categories of actors interviewed: 20 software engineers, 2 e-business managers and 8 sales engineers... the system administrator who acted as a broker." (Methodology / Table 1 section)</t>
         </is>
       </c>
     </row>
@@ -16329,7 +16334,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F317" t="inlineStr">
+      <c r="F317" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -16479,7 +16484,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F320" t="inlineStr">
+      <c r="F320" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -16774,7 +16779,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F326" t="inlineStr">
+      <c r="F326" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -16824,7 +16829,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F327" t="inlineStr">
+      <c r="F327" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -16874,7 +16879,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F328" t="inlineStr">
+      <c r="F328" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -16974,7 +16979,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F330" t="inlineStr">
+      <c r="F330" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -17024,7 +17029,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F331" t="inlineStr">
+      <c r="F331" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -17266,7 +17271,12 @@
       </c>
       <c r="E336" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G336" s="0" t="inlineStr">
@@ -17294,7 +17304,7 @@
       </c>
       <c r="P336" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level statistical aggregation study where individual responses are aggregated to the team unit of analysis using ICC and rwg. Verbatim Evidence: "Setting a knowledge boundary across teams: knowledge protection regulation for inter-team coordination and team performance... we checked the legitimacy of our sample for team-level analysis using inter-rater agreement (rwg) and ICC... The values exceeded 0.7 for both rwg and ICC for all constructs, thereby satisfying the requirement for the aggregation of individual-level responses to the team level." (Methodology section)</t>
         </is>
       </c>
     </row>
@@ -17451,7 +17461,12 @@
       </c>
       <c r="E340" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G340" s="0" t="inlineStr">
@@ -17479,7 +17494,7 @@
       </c>
       <c r="P340" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level study of IS development teams in consultant-partnered projects where the unit of analysis is the firm/project. Verbatim Evidence: "Boundary Spanning Role of the IS Development Team in Consultant-Partnered Projects... In total, 109 firms had sales larger than $100M and 97 firms employed more than 300 people... The frequency distribution of sales revenue and the number of employees are relatively even throughout the categories." (Sample / Table 3 section)</t>
         </is>
       </c>
     </row>
@@ -17636,7 +17651,12 @@
       </c>
       <c r="E344" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G344" s="0" t="inlineStr">
@@ -17664,7 +17684,7 @@
       </c>
       <c r="P344" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Conceptual paper on firm internationalization using descriptive case illustration of German family firms without individual employee Pearson correlation data. Verbatim Evidence: "Boundary-spanning and boundary-buffering in global markets: A German perspective on the internationalization of family firms... Conceptual paper... The case of Germany, with its large stock of internationalized family firms, shows how boundary-buffering vis-a-vis global capital markets can be compatible with successful and sustained internationalization." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Executed Batch 10 Full-Text Audit, removing 2 false positives with verbatim quotes. Final Included: 222
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -15984,7 +15984,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F310" t="inlineStr">
+      <c r="F310" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -17274,7 +17274,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F336" t="inlineStr">
+      <c r="F336" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -17464,7 +17464,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F340" t="inlineStr">
+      <c r="F340" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -17654,7 +17654,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F344" t="inlineStr">
+      <c r="F344" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -17941,7 +17941,12 @@
       </c>
       <c r="E350" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G350" s="0" t="inlineStr">
@@ -17969,7 +17974,7 @@
       </c>
       <c r="P350" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm/Patent-level study of external technology acquisition where the unit of analysis is the patent and the firm. Verbatim Evidence: "Boundary spanning through external technology acquisition: The moderating role of star scientists and upstream alliances... We tested our hypotheses on a sample of 6208 USPTO patented technologies acquired by 350 biotechnology firms over the period 1980-2012." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>
@@ -18136,7 +18141,12 @@
       </c>
       <c r="E354" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G354" s="0" t="inlineStr">
@@ -18164,7 +18174,7 @@
       </c>
       <c r="P354" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level study of industrial cluster knowledge search where the unit of analysis is the cluster firm (N = 310 cluster firms). Verbatim Evidence: "Search within or beyond the industrial cluster? The effect of perceived competition and knowledge base tacitness on strategic location choices of external knowledge search... Using a sample of 310 cluster firms in the Zhejiang Province of China, we find that the cluster firm would increase the propensity for more geographic boundary-spanning search." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Batch 11 Full-Text Audit, removing 8 false positives (incl. 1 PDF mismatch). Final Included: 214
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -17944,7 +17944,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F350" t="inlineStr">
+      <c r="F350" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18144,7 +18144,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F354" t="inlineStr">
+      <c r="F354" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18331,7 +18331,12 @@
       </c>
       <c r="E358" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G358" s="0" t="inlineStr">
@@ -18359,7 +18364,7 @@
       </c>
       <c r="P358" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level study of new technology ventures where the unit of analysis is the venture/firm (N = 750 new ventures). Verbatim Evidence: "The Effect of Boundary-Spanning Search on Breakthrough Innovations of New Technology Ventures... The sampling frame of this study consisted of new technology ventures located in Shenzhen... We drew on a random sample of 750 new ventures (i.e., 8 years or younger)." (Title / Sample section)</t>
         </is>
       </c>
     </row>
@@ -18476,7 +18481,12 @@
       </c>
       <c r="E361" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G361" s="0" t="inlineStr">
@@ -18504,7 +18514,7 @@
       </c>
       <c r="P361" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level statistical aggregation study where individual responses are aggregated to the team unit using ICC and rwg, analyzed with HLM multilevel models. Verbatim Evidence: "A Longitudinal Study on the Impact Mechanism of Employees' Boundary Spanning Behavior... ICC(1) and ICC(2) were 0.11 and 0.88 respectively, indicating that all variables met the aggregation criteria and can be used for team-level analysis." (Methodology / Table 1 section)</t>
         </is>
       </c>
     </row>
@@ -18571,7 +18581,12 @@
       </c>
       <c r="E363" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G363" s="0" t="inlineStr">
@@ -18599,7 +18614,7 @@
       </c>
       <c r="P363" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>PDF contains Javadi Khasraghi et al. (2023) crowdsourcing contest study where the unit of analysis is the team (N = 9,793 teams in 246 contests). Verbatim Evidence: "Submitting tentative solutions for platform feedback in crowdsourcing contests: breaking network closure with boundary spanning for team performance... The final sample comprises 9,793 teams participating in 246 contests. The unit of analysis is submission." (Title / Sample section)</t>
         </is>
       </c>
     </row>
@@ -18616,7 +18631,12 @@
       </c>
       <c r="E364" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G364" s="0" t="inlineStr">
@@ -18644,7 +18664,7 @@
       </c>
       <c r="P364" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>General social networking service (SNS) users study, not organizational employees. Verbatim Evidence: "Investigating the lurking mechanism of SNS users: a comprehensive examination of context-specific cues and role stresses... Social networking services (SNS) empower users with a robust capability to connect with others and manage their social relationships... This study delves into the mechanism of this technology-induced decision-making process among SNS users." (Abstract section)</t>
         </is>
       </c>
     </row>
@@ -18661,7 +18681,12 @@
       </c>
       <c r="E365" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G365" s="0" t="inlineStr">
@@ -18689,7 +18714,7 @@
       </c>
       <c r="P365" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Patent-level nanotechnology knowledge diffusion study where the unit of analysis is the patent/inventor citation network, not individual organizational employees. Verbatim Evidence: "Determining inventor status and its effect on knowledge diffusion: A study on nanotechnology literature from China, Russia, and India... 561 individuals... n = 152 patents." (Title / Sample section)</t>
         </is>
       </c>
     </row>
@@ -19556,7 +19581,12 @@
       </c>
       <c r="E383" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G383" s="0" t="inlineStr">
@@ -19584,7 +19614,7 @@
       </c>
       <c r="P383" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Interorganizational strategic alliance study where the unit of analysis is the alliance (N = 440 strategic alliances). Verbatim Evidence: "The Independent and Interactive Roles of Procedural, Distributive, and Interactional Justice in Strategic Alliances... a sample of 440 strategic alliances... to avoid a single-party bias toward perceived justice, this study defines and measures justice from both alliance partners' perspectives." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>
@@ -19791,7 +19821,12 @@
       </c>
       <c r="E388" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G388" s="0" t="inlineStr">
@@ -19819,7 +19854,7 @@
       </c>
       <c r="P388" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level study of software development teams where boundary spanning is measured at the team level (N = 25 teams). Verbatim Evidence: "U.S. and Indian Managerial Boundary Spanning Behaviors in Globally Distributed Software Teams... The first study measured the boundary spanning behaviors of software team managers of 25 teams. These results were analyzed in conjunction with a standard measure of software team output." (Abstract section)</t>
         </is>
       </c>
     </row>
@@ -19836,7 +19871,12 @@
       </c>
       <c r="E389" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G389" s="0" t="inlineStr">
@@ -19864,7 +19904,7 @@
       </c>
       <c r="P389" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level study of senior executive external networks and strategic imitation where the unit of analysis is the firm (N = 58 firms). Verbatim Evidence: "The external networks of senior executives: Implications for strategic innovation and imitation... Results from the model are tested on a sample of 58 firms operating in the branded foods and computer industries." (Abstract / Sample section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Batch 12 Full-Text Audit, removing 2 false positives (incl. 1 PDF mismatch/scanned Bennet paper). Final Included: 212
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -18334,7 +18334,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F358" t="inlineStr">
+      <c r="F358" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18484,7 +18484,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F361" t="inlineStr">
+      <c r="F361" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18584,7 +18584,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F363" t="inlineStr">
+      <c r="F363" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -18634,7 +18634,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F364" t="inlineStr">
+      <c r="F364" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -18684,7 +18684,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F365" t="inlineStr">
+      <c r="F365" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -19584,7 +19584,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F383" t="inlineStr">
+      <c r="F383" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -19824,7 +19824,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F388" t="inlineStr">
+      <c r="F388" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -19874,7 +19874,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F389" t="inlineStr">
+      <c r="F389" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -20251,7 +20251,12 @@
       </c>
       <c r="E397" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G397" s="0" t="inlineStr">
@@ -20279,7 +20284,7 @@
       </c>
       <c r="P397" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>PDF file mismatch: Master sheet lists Stock, Zacharias &amp; Schnellbaecher (2017) but actual PDF [394] contains Bennet (1989) "Personnel/human resource departments and uncertainty" which is a scanned reproduction without extractable text. Verbatim Evidence: "Reproduced with permission of the copyright owner. Further reproduction prohibited without permission." (Full document - scanned image). Unable to verify individual-level BSB correlation data.</t>
         </is>
       </c>
     </row>
@@ -20591,7 +20596,12 @@
       </c>
       <c r="E404" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G404" s="0" t="inlineStr">
@@ -20619,7 +20629,7 @@
       </c>
       <c r="P404" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative multiple-case study using interviews without individual employee Pearson correlation matrix. Verbatim Evidence: "Practices of strategic alignment in and between innovation project portfolios... qualitative multiple-case study conducted with three large firms that have multiple innovation project portfolios. Data collection was done primarily through key informant interviews and the consequent thematic data analysis approach." (Abstract / Methodology section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Batch 13 Full-Text Audit, removing 2 false positives (team/firm level). Final Included: 210
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -20254,7 +20254,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F397" t="inlineStr">
+      <c r="F397" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -20599,7 +20599,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F404" t="inlineStr">
+      <c r="F404" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -20763,7 +20763,12 @@
       </c>
       <c r="E407" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G407" s="0" t="inlineStr">
@@ -20791,7 +20796,7 @@
       </c>
       <c r="P407" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level study of dynamic medical teams where the unit of analysis is the core team per week (N = 91 team-weeks across 22 teams). Verbatim Evidence: "Coordination in Dynamic Teams: Investigating a Learning-Productivity Trade-Off... The unit of analysis was a core team in a given week, along with the periphery members associated with each patient case... Our overall sample included 243 unique core team members." (Methodology / Sample section)</t>
         </is>
       </c>
     </row>
@@ -20808,7 +20813,12 @@
       </c>
       <c r="E408" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G408" s="0" t="inlineStr">
@@ -20836,7 +20846,7 @@
       </c>
       <c r="P408" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level study of innovative ICT start-ups in Italy where the unit of analysis is the venture/firm (N = 179 start-ups). Verbatim Evidence: "Unpacking the drivers of the socio-environmental sustainability of new ventures: insights from innovative digital start-ups in Italy... Out of 1104 contacted firms, we received replies from 179 start-ups (16% response rate), representative of the population of innovative ICT start-ups operating in Italy." (Methodology / Sample section)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 1 subagent conflicts resolved. Found 3 new false positives (Code 1 & Code 3) previously missed. Final Included: 207
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -1559,7 +1559,12 @@
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G17" s="0" t="inlineStr">
@@ -1587,7 +1592,7 @@
       </c>
       <c r="P17" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Role ambiguity was measured using the 45-item MULTIRAM... Burnout was assessed... The job satisfaction construct was measured... job performance was measured... (BSB construct missing from measurements). Verbatim Evidence: "Scales in the extant literature were used for measuring all of the identified constructs. Role ambiguity was measured using the 45-item MULTIRAM instrument (Singh &amp; Rhoads, 1991)... Burnout was assessed using the reduced Maslach burnout inventory for sales (Rutherford et al., 2011). The job satisfaction construct was measured using a three-item scale developed by Netemeyer, Boles, McKee, and McMurrian (1997). Finally, job performance was measured by four items" (5.2. Measures)</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1809,12 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
@@ -1832,7 +1842,7 @@
       </c>
       <c r="P22" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team-level study where unit of analysis is the team. Verbatim Evidence: "much of the analysis was conducted at the group level, teams were included in the final sample only if at least three-fourths of their members responded. This reduced the number of teams in the final sample to 45." (Methodology)</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2612,12 @@
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
@@ -2630,7 +2645,7 @@
       </c>
       <c r="P38" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Dyad/Network level study where the unit of analysis is a directed dyad, not the individual. Verbatim Evidence: "For the purpose of this study, dyads were chosen as units of the analysis. All possible (n*(n-1)) directed dyads were investigated in thenine selected dimensions. In this approach, an observation is a directed dyad ij, and variables indicate whether the actor i chose the actor j in a specific relational layer (dimension)." (Section 2 Data and Methods)</t>
         </is>
       </c>
     </row>
@@ -20766,7 +20781,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F407" t="inlineStr">
+      <c r="F407" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -20816,7 +20831,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F408" t="inlineStr">
+      <c r="F408" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>

</xml_diff>

<commit_message>
Audit: Shadow Batch 2 subagent conflicts resolved. Found 5 new false positives previously missed. Final Included: 202
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -1562,7 +1562,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -1812,7 +1812,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -2615,7 +2615,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -3492,7 +3492,12 @@
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
@@ -3520,7 +3525,7 @@
       </c>
       <c r="P56" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Does not measure BSB construct. Verbatim Evidence: "We applied the SPSS Process macro, Model 21 (Hayes, 2018), to test the conditional mediational hypotheses shown in Figure 1, where the independent variable (identification with the branch at time 1, X) is shown to influence the mediator (performance control related to CS at time 1, M), whose effect in turn is contingent on locus of control (W), and the effect of M on the dependent variable (CS at time 2, Y) is shown to depend on proactive behaviors in the form of CS-related meetings (V)."</t>
         </is>
       </c>
     </row>
@@ -3537,6 +3542,11 @@
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -3563,11 +3573,7 @@
       <c r="K57" s="0" t="n">
         <v>2003</v>
       </c>
-      <c r="P57" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P57" s="0" t="inlineStr"/>
     </row>
     <row r="58" ht="18" customHeight="1" s="31">
       <c r="A58" s="0" t="inlineStr">
@@ -3582,6 +3588,11 @@
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -3608,11 +3619,7 @@
       <c r="K58" s="0" t="n">
         <v>2005</v>
       </c>
-      <c r="P58" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P58" s="0" t="inlineStr"/>
     </row>
     <row r="59" ht="18" customHeight="1" s="31">
       <c r="A59" s="0" t="inlineStr">
@@ -4082,6 +4089,11 @@
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -4108,11 +4120,7 @@
       <c r="K68" s="0" t="n">
         <v>1984</v>
       </c>
-      <c r="P68" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P68" s="0" t="inlineStr"/>
     </row>
     <row r="69" ht="18" customHeight="1" s="31">
       <c r="A69" s="0" t="inlineStr">
@@ -4361,6 +4369,11 @@
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -4387,11 +4400,7 @@
       <c r="K73" s="0" t="n">
         <v>1995</v>
       </c>
-      <c r="P73" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P73" s="0" t="inlineStr"/>
     </row>
     <row r="74" ht="18" customHeight="1" s="31">
       <c r="A74" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 3 subagent conflicts resolved. Found 5 new false positives. Final Included: 197
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -3495,7 +3495,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -3545,7 +3545,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -3591,7 +3591,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -4092,7 +4092,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -4372,7 +4372,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F73" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -5795,7 +5795,12 @@
       </c>
       <c r="E102" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G102" s="0" t="inlineStr">
@@ -5823,7 +5828,7 @@
       </c>
       <c r="P102" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Multilevel study where BSB is at the manager/group level (Level 2). Verbatim Evidence: "In this study, the data have a nested structure with individual subordinates nested within managers. Constructs regarding the manager exist at the group level of analysis whereas constructs about subordinate employees exist at the individual level of analysis."</t>
         </is>
       </c>
     </row>
@@ -6640,6 +6645,11 @@
       </c>
       <c r="E119" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -6666,11 +6676,7 @@
       <c r="K119" s="0" t="n">
         <v>1978</v>
       </c>
-      <c r="P119" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P119" s="0" t="inlineStr"/>
     </row>
     <row r="120" ht="18" customHeight="1" s="31">
       <c r="A120" s="0" t="inlineStr">
@@ -6885,6 +6891,11 @@
       </c>
       <c r="E124" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -6911,11 +6922,7 @@
       <c r="K124" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P124" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P124" s="0" t="inlineStr"/>
     </row>
     <row r="125" ht="18" customHeight="1" s="31">
       <c r="A125" s="0" t="inlineStr">
@@ -7134,6 +7141,11 @@
       </c>
       <c r="E129" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -7160,11 +7172,7 @@
       <c r="K129" s="0" t="n">
         <v>1998</v>
       </c>
-      <c r="P129" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P129" s="0" t="inlineStr"/>
     </row>
     <row r="130" ht="18" customHeight="1" s="31">
       <c r="A130" s="0" t="inlineStr">
@@ -7329,7 +7337,12 @@
       </c>
       <c r="E133" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G133" s="0" t="inlineStr">
@@ -7357,7 +7370,7 @@
       </c>
       <c r="P133" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Does not measure BSB construct as an effect size; measures general job performance and self-monitoring. Verbatim Evidence: "To test the hypotheses, two constructs were assessed: job performance and attention to social cues. Performance level was obtained from company performance evaluation forms, which provide, in part, a single, overall performance rating." (Measures)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 4 subagent conflicts resolved. Found 7 new false positives. Final Included: 190
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -5798,7 +5798,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr">
+      <c r="F102" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -6648,7 +6648,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr">
+      <c r="F119" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -6894,7 +6894,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr">
+      <c r="F124" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -7144,7 +7144,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
+      <c r="F129" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -7340,7 +7340,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr">
+      <c r="F133" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -7886,7 +7886,12 @@
       </c>
       <c r="E144" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G144" s="0" t="inlineStr">
@@ -7914,7 +7919,7 @@
       </c>
       <c r="P144" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Student sample. Verbatim Evidence: "Fifteen subjects (upper division business school undergraduates) were in each treatment." (Research Method - Manipulations section)</t>
         </is>
       </c>
     </row>
@@ -7981,7 +7986,12 @@
       </c>
       <c r="E146" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G146" s="0" t="inlineStr">
@@ -8009,7 +8019,7 @@
       </c>
       <c r="P146" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team level analysis. Verbatim Evidence: "To explore what leaders of action teams do to promote speaking up and other proactive coordination behaviours – as well as how organizational context may affect these team processes and outcomes – I analysed qualitative and quantitative data from 16 operating room teams learning to use a new technology for cardiac surgery." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -8026,7 +8036,12 @@
       </c>
       <c r="E147" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G147" s="0" t="inlineStr">
@@ -8054,7 +8069,7 @@
       </c>
       <c r="P147" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>BSB not measured. Verbatim Evidence: "RQ: Are there differences in key job factors including (a) grit, (b) happiness, (c) perceived organizational support, (d) perceived supervisory support, (e) job satisfaction, (f) organizational commitment, and (g) turnover intentions based on the level of sleep an employee gets on average?" (Business-to-business salespeople)</t>
         </is>
       </c>
     </row>
@@ -8271,7 +8286,12 @@
       </c>
       <c r="E152" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G152" s="0" t="inlineStr">
@@ -8299,7 +8319,7 @@
       </c>
       <c r="P152" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative case study. Verbatim Evidence: "Previous empirical studies on organizational creativity are to a great extent laboratory studies or quantitative field studies. This study takes a qualitative in-depth approach, and thus responds to Zhou and Shalley’s(2003) call for more qualitative research on creativity." (Introduction)</t>
         </is>
       </c>
     </row>
@@ -8966,7 +8986,12 @@
       </c>
       <c r="E166" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G166" s="0" t="inlineStr">
@@ -8994,7 +9019,7 @@
       </c>
       <c r="P166" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Network case study, no BSB correlations. Verbatim Evidence: "We assessed the validity of the four hypotheses using longitudinal network data collected over the three-month span that \"Midwestern University\" negotiated with its faculty union, \"American Faculty Union.\"" (Research Setting)</t>
         </is>
       </c>
     </row>
@@ -9061,7 +9086,12 @@
       </c>
       <c r="E168" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G168" s="0" t="inlineStr">
@@ -9089,7 +9119,7 @@
       </c>
       <c r="P168" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level analysis. Verbatim Evidence: "These hypotheses are tested through two surveys: The first of these was a survey of Japanese-affiliates in Brazil, the second survey was of the Nikkeijin (Japanese Brazilians) themselves. The first survey was conducted in Brazil, in Sa˜o Paulo. The survey target was 180 Japanese affiliated companies that are members of the Japan–Brazil Chamber of Commerce. We selected this sample group as it covers most of the major Japanese subsidiaries. The questionnaire was prepared in Japanese and e-mailed to the Japanese top managementin each company. The respondents were asked to identify their company names. Responses were obtained from 65 different corporations (a response rate of 36%)." (3. Methodology)</t>
         </is>
       </c>
     </row>
@@ -9106,6 +9136,11 @@
       </c>
       <c r="E169" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -9132,11 +9167,7 @@
       <c r="K169" s="0" t="n">
         <v>2019</v>
       </c>
-      <c r="P169" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P169" s="0" t="inlineStr"/>
     </row>
     <row r="170" ht="18" customHeight="1" s="31">
       <c r="A170" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 5 subagent conflicts resolved. Found 5 new false positives. Final Included: 185
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -7889,7 +7889,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr">
+      <c r="F144" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -7989,7 +7989,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr">
+      <c r="F146" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -8039,7 +8039,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr">
+      <c r="F147" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -8289,7 +8289,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr">
+      <c r="F152" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -8989,7 +8989,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr">
+      <c r="F166" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -9089,7 +9089,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr">
+      <c r="F168" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -9139,7 +9139,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr">
+      <c r="F169" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -9483,7 +9483,12 @@
       </c>
       <c r="E176" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G176" s="0" t="inlineStr">
@@ -9511,7 +9516,7 @@
       </c>
       <c r="P176" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative case study. Verbatim Evidence: "A longitudinal field study was conducted using an interpretive, ethnographic approach to data collection and analysis (Schwandt, 1998)."</t>
         </is>
       </c>
     </row>
@@ -10128,6 +10133,11 @@
       </c>
       <c r="E189" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -10154,11 +10164,7 @@
       <c r="K189" s="0" t="n">
         <v>2015</v>
       </c>
-      <c r="P189" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P189" s="0" t="inlineStr"/>
     </row>
     <row r="190" ht="18" customHeight="1" s="31">
       <c r="A190" s="0" t="inlineStr">
@@ -10173,7 +10179,12 @@
       </c>
       <c r="E190" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G190" s="0" t="inlineStr">
@@ -10201,7 +10212,7 @@
       </c>
       <c r="P190" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>BSB not measured, measures demands. Verbatim Evidence: "We use one item to assess the frequency of exposure to the following boundary-spanning demand: “How often do coworkers, supervisors, managers, customers, or clients contact you about work-related matters outside normal work hours? Include telephone, cell phone, beeper and pager calls, as well as faxes and e-mail that you have to respond to.”" (Measures)</t>
         </is>
       </c>
     </row>
@@ -10518,7 +10529,12 @@
       </c>
       <c r="E197" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G197" s="0" t="inlineStr">
@@ -10546,7 +10562,7 @@
       </c>
       <c r="P197" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Dyad level analysis. Verbatim Evidence: "Our research was designed to examine relationships between LSPs and their customers, using the dyad as the unit of analysis to focus on key constructs from the perspective of both sides of the buyer–seller relationship." (Data collection)</t>
         </is>
       </c>
     </row>
@@ -10963,6 +10979,11 @@
       </c>
       <c r="E206" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -10989,11 +11010,7 @@
       <c r="K206" s="0" t="n">
         <v>1992</v>
       </c>
-      <c r="P206" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P206" s="0" t="inlineStr"/>
     </row>
     <row r="207" ht="18" customHeight="1" s="31">
       <c r="A207" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 6 subagent conflicts resolved. Found 6 new false positives. Final Included: 179
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -9486,7 +9486,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr">
+      <c r="F176" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -10136,7 +10136,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr">
+      <c r="F189" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -10182,7 +10182,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr">
+      <c r="F190" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -10532,7 +10532,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F197" t="inlineStr">
+      <c r="F197" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -10982,7 +10982,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr">
+      <c r="F206" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -11365,6 +11365,11 @@
       </c>
       <c r="E214" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -11391,11 +11396,7 @@
       <c r="K214" s="0" t="n">
         <v>1999</v>
       </c>
-      <c r="P214" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P214" s="0" t="inlineStr"/>
     </row>
     <row r="215" ht="18" customHeight="1" s="31">
       <c r="A215" s="0" t="inlineStr">
@@ -11410,7 +11411,12 @@
       </c>
       <c r="E215" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G215" s="0" t="inlineStr">
@@ -11438,7 +11444,7 @@
       </c>
       <c r="P215" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level analysis. Verbatim Evidence: "By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005."</t>
         </is>
       </c>
     </row>
@@ -11705,7 +11711,12 @@
       </c>
       <c r="E221" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G221" s="0" t="inlineStr">
@@ -11733,7 +11744,7 @@
       </c>
       <c r="P221" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Department/Firm level analysis. Verbatim Evidence: "The sample in the present study includes responses from 126 professionals in R&amp;D and/or M&amp;S departments from 79 different firms (in 37 cases, we received a response from only one department)."</t>
         </is>
       </c>
     </row>
@@ -11900,7 +11911,12 @@
       </c>
       <c r="E225" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G225" s="0" t="inlineStr">
@@ -11928,7 +11944,7 @@
       </c>
       <c r="P225" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative case study. Verbatim Evidence: "To obtain a multilevel design, we conducted (a) interviews with the top managers of both youth care organizations (one at NHC and two at SHC), (b) interviews with two division heads per organization (four in total), and (c) four focus groups of caregivers (one group of representatives per working unit—19 caregivers in total) each reporting directly to one of the division heads, to allow for the study of change embeddedness as a team-level construct." (4.2 | Data collection)</t>
         </is>
       </c>
     </row>
@@ -12445,7 +12461,12 @@
       </c>
       <c r="E236" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G236" s="0" t="inlineStr">
@@ -12473,7 +12494,7 @@
       </c>
       <c r="P236" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project level analysis. Verbatim Evidence: "(one member for each recently completed project). For those companies which had two or more recently completed projects, the information of each contact was recorded. A total of 750 projects were identified."</t>
         </is>
       </c>
     </row>
@@ -12490,6 +12511,11 @@
       </c>
       <c r="E237" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -12516,11 +12542,7 @@
       <c r="K237" s="0" t="n">
         <v>2007</v>
       </c>
-      <c r="P237" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P237" s="0" t="inlineStr"/>
     </row>
     <row r="238" ht="18" customHeight="1" s="31">
       <c r="A238" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 7 subagent conflicts resolved. Found 6 new false positive papers (updated 8 rows due to possible duplicates). Final Included: ~173
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -11368,7 +11368,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F214" t="inlineStr">
+      <c r="F214" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -11414,7 +11414,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr">
+      <c r="F215" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -11714,7 +11714,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F221" t="inlineStr">
+      <c r="F221" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -11914,7 +11914,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F225" t="inlineStr">
+      <c r="F225" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -12464,7 +12464,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr">
+      <c r="F236" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -12514,7 +12514,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr">
+      <c r="F237" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -13002,7 +13002,12 @@
       </c>
       <c r="E247" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G247" s="0" t="inlineStr">
@@ -13030,7 +13035,7 @@
       </c>
       <c r="P247" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Work-life boundary management, not BSB. Verbatim Evidence: "This three-essay project explores boundary management and work-nonwork enrichment to explain how thriving in the work domain relates to thriving in the nonwork domain." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -13047,7 +13052,12 @@
       </c>
       <c r="E248" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G248" s="0" t="inlineStr">
@@ -13075,7 +13085,7 @@
       </c>
       <c r="P248" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Volunteers in community initiatives. Verbatim Evidence: "Considering the role of the respondents (see also control variables), most respondents were active volunteers (60.95%), followed by board members (25.63%), and passive or supporting volunteers (11.92%) (and other (1.49%))."</t>
         </is>
       </c>
     </row>
@@ -13092,6 +13102,11 @@
       </c>
       <c r="E249" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -13118,11 +13133,7 @@
       <c r="K249" s="0" t="n">
         <v>1992</v>
       </c>
-      <c r="P249" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P249" s="0" t="inlineStr"/>
     </row>
     <row r="250" ht="18" customHeight="1" s="31">
       <c r="A250" s="0" t="inlineStr">
@@ -13137,7 +13148,12 @@
       </c>
       <c r="E250" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G250" s="0" t="inlineStr">
@@ -13165,7 +13181,7 @@
       </c>
       <c r="P250" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>F-tests only, no correlation matrix. Verbatim Evidence: "Table 4 The relationships between career decisions and the study variables. Independent variables Career Career F-test a decisions indecision" (Table 4, page 7)</t>
         </is>
       </c>
     </row>
@@ -13232,6 +13248,11 @@
       </c>
       <c r="E252" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -13258,11 +13279,7 @@
       <c r="K252" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P252" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P252" s="0" t="inlineStr"/>
     </row>
     <row r="253" ht="18" customHeight="1" s="31">
       <c r="A253" s="0" t="inlineStr">
@@ -13727,7 +13744,12 @@
       </c>
       <c r="E262" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G262" s="0" t="inlineStr">
@@ -13755,7 +13777,7 @@
       </c>
       <c r="P262" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Department level analysis. Verbatim Evidence: "The dependent variables were measures of each department’s influence on strategic decisions (INFLUENCE). The independent variables were the extent to which a department engaged in one of the three boundary spanning roles (B.S.R.)." (Results)</t>
         </is>
       </c>
     </row>
@@ -13772,6 +13794,11 @@
       </c>
       <c r="E263" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -13798,11 +13825,7 @@
       <c r="K263" s="0" t="n">
         <v>1984</v>
       </c>
-      <c r="P263" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P263" s="0" t="inlineStr"/>
     </row>
     <row r="264" ht="18" customHeight="1" s="31">
       <c r="A264" s="0" t="inlineStr">
@@ -13867,6 +13890,11 @@
       </c>
       <c r="E265" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -13893,11 +13921,7 @@
       <c r="K265" s="0" t="n">
         <v>2023</v>
       </c>
-      <c r="P265" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P265" s="0" t="inlineStr"/>
     </row>
     <row r="266" ht="18" customHeight="1" s="31">
       <c r="A266" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 8 subagent conflicts resolved. Found 6 new false positive papers (updated 7 rows). Final Included: ~167
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -13005,7 +13005,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F247" t="inlineStr">
+      <c r="F247" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -13055,7 +13055,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F248" t="inlineStr">
+      <c r="F248" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -13105,7 +13105,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F249" t="inlineStr">
+      <c r="F249" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -13151,7 +13151,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F250" t="inlineStr">
+      <c r="F250" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -13251,7 +13251,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F252" t="inlineStr">
+      <c r="F252" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -13747,7 +13747,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr">
+      <c r="F262" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -13797,7 +13797,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F263" t="inlineStr">
+      <c r="F263" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -13893,7 +13893,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F265" t="inlineStr">
+      <c r="F265" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -14276,7 +14276,12 @@
       </c>
       <c r="E273" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G273" s="0" t="inlineStr">
@@ -14304,7 +14309,7 @@
       </c>
       <c r="P273" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>APN presence as a boundary spanner intervention, not measuring BSB construct for the employees. Verbatim Evidence: "To test the study hypotheses, we used SPSS 21 and the PROCESS macro (model 7) (Hayes, 2013) to estimate the equations and test the conditional indirect effects of the presence of the APN on self-initiated ward rounds, through “tasks from the day shift,” “doctor or nurse tasks” and “total tasks” (see Table II)." (Data analysis)</t>
         </is>
       </c>
     </row>
@@ -14321,6 +14326,11 @@
       </c>
       <c r="E274" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -14347,11 +14357,7 @@
       <c r="K274" s="0" t="n">
         <v>2000</v>
       </c>
-      <c r="P274" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P274" s="0" t="inlineStr"/>
     </row>
     <row r="275" ht="18" customHeight="1" s="31">
       <c r="A275" s="0" t="inlineStr">
@@ -14516,7 +14522,12 @@
       </c>
       <c r="E278" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G278" s="0" t="inlineStr">
@@ -14544,7 +14555,7 @@
       </c>
       <c r="P278" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Organization level analysis. Verbatim Evidence: "The focus of this study was to investigate differences between organizations utilizing key account management (KAM) sales processes and organizations that do not utilize key account management processes (non-KAM) with regards to their involvement of salespeople during the early stages of the new product development process." (METHODOLOGY)</t>
         </is>
       </c>
     </row>
@@ -14611,6 +14622,11 @@
       </c>
       <c r="E280" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -14637,11 +14653,7 @@
       <c r="K280" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P280" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P280" s="0" t="inlineStr"/>
     </row>
     <row r="281" ht="18" customHeight="1" s="31">
       <c r="A281" s="0" t="inlineStr">
@@ -14919,6 +14931,11 @@
       </c>
       <c r="E286" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -14945,11 +14962,7 @@
       <c r="K286" s="0" t="n">
         <v>2025</v>
       </c>
-      <c r="P286" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P286" s="0" t="inlineStr"/>
     </row>
     <row r="287" ht="18" customHeight="1" s="31">
       <c r="A287" s="0" t="inlineStr">
@@ -15264,7 +15277,12 @@
       </c>
       <c r="E293" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G293" s="0" t="inlineStr">
@@ -15292,7 +15310,7 @@
       </c>
       <c r="P293" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No Pearson correlation matrix, discriminant analysis. Verbatim Evidence: "Table 1 reports the percentages of project members who remained with the organization over the 5-year period as a function of their prior type of supervision." (Results section, Page 9)</t>
         </is>
       </c>
     </row>
@@ -15423,6 +15441,11 @@
       </c>
       <c r="E296" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -15449,11 +15472,7 @@
       <c r="K296" s="0" t="n">
         <v>1975</v>
       </c>
-      <c r="P296" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P296" s="0" t="inlineStr"/>
     </row>
     <row r="297" ht="18" customHeight="1" s="31">
       <c r="A297" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 9 subagent conflicts resolved. Found 2 new false positive papers (8 were already excluded). Final Included: ~165
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -14279,7 +14279,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr">
+      <c r="F273" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -14329,7 +14329,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr">
+      <c r="F274" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -14525,7 +14525,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F278" t="inlineStr">
+      <c r="F278" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -14625,7 +14625,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F280" t="inlineStr">
+      <c r="F280" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -14934,7 +14934,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F286" t="inlineStr">
+      <c r="F286" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -15280,7 +15280,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F293" t="inlineStr">
+      <c r="F293" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -15444,7 +15444,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F296" t="inlineStr">
+      <c r="F296" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -16082,7 +16082,12 @@
       </c>
       <c r="E309" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G309" s="0" t="inlineStr">
@@ -16114,7 +16119,7 @@
       </c>
       <c r="P309" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team level analysis. Verbatim Evidence: "However, unit of analysis in this study is the team, not individual" (Page 12, Notes section)</t>
         </is>
       </c>
     </row>
@@ -16781,7 +16786,12 @@
       </c>
       <c r="E323" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G323" s="0" t="inlineStr">
@@ -16809,7 +16819,7 @@
       </c>
       <c r="P323" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB construct measured. Verbatim Evidence: "We performed confirmatory factor analysis (CFA) on six constructs and tested the fit of a six-factor model; surface acting, deep acting, taking charge, performance-based pay, creative performance, and task performance." (3.6 Model fitness statistics)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 10 subagent conflicts resolved. Found 6 new false positive papers (updated 7 rows). Final Included: ~159
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -16085,7 +16085,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F309" t="inlineStr">
+      <c r="F309" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -16789,7 +16789,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr">
+      <c r="F323" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -17336,7 +17336,12 @@
       </c>
       <c r="E334" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G334" s="0" t="inlineStr">
@@ -17364,7 +17369,7 @@
       </c>
       <c r="P334" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm evaluating suppliers. Verbatim Evidence: "The model is tested by surveying buyers in a broad cross-section of business relationships. Organization informants evaluate a particular supplier ("target supplier"), concerning a particular product ("target product") for which their firm regularly uses alternative suppliers."</t>
         </is>
       </c>
     </row>
@@ -17531,6 +17536,11 @@
       </c>
       <c r="E338" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -17557,11 +17567,7 @@
       <c r="K338" s="0" t="n">
         <v>2019</v>
       </c>
-      <c r="P338" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P338" s="0" t="inlineStr"/>
     </row>
     <row r="339" ht="18" customHeight="1" s="31">
       <c r="A339" s="0" t="inlineStr">
@@ -17576,6 +17582,11 @@
       </c>
       <c r="E339" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -17602,11 +17613,7 @@
       <c r="K339" s="0" t="n">
         <v>2023</v>
       </c>
-      <c r="P339" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P339" s="0" t="inlineStr"/>
     </row>
     <row r="340" ht="18" customHeight="1" s="31">
       <c r="A340" s="0" t="inlineStr">
@@ -17671,6 +17678,11 @@
       </c>
       <c r="E341" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -17697,11 +17709,7 @@
       <c r="K341" s="0" t="n">
         <v>2016</v>
       </c>
-      <c r="P341" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P341" s="0" t="inlineStr"/>
     </row>
     <row r="342" ht="18" customHeight="1" s="31">
       <c r="A342" s="0" t="inlineStr">
@@ -17716,6 +17724,11 @@
       </c>
       <c r="E342" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -17742,11 +17755,7 @@
       <c r="K342" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P342" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P342" s="0" t="inlineStr"/>
     </row>
     <row r="343" ht="18" customHeight="1" s="31">
       <c r="A343" s="0" t="inlineStr">
@@ -18011,7 +18020,12 @@
       </c>
       <c r="E348" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G348" s="0" t="inlineStr">
@@ -18039,7 +18053,7 @@
       </c>
       <c r="P348" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Goodman-Kruskal Gamma, no Pearson correlation. Verbatim Evidence: "The data were first analyzed using the Goodman-Kruskal Gamma ($\gamma$), (10) a nonparametric measure of association yielding values of -1≤$\gamma$≤+1. This measure has an interpretation similar to that of a correlation coefficient, but is applicable to ordinal scale and contingency table analysis." (Data Analysis)</t>
         </is>
       </c>
     </row>
@@ -18056,7 +18070,12 @@
       </c>
       <c r="E349" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G349" s="0" t="inlineStr">
@@ -18084,7 +18103,7 @@
       </c>
       <c r="P349" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Goodman-Kruskal Gamma, no Pearson correlation. Verbatim Evidence: "Since the data probably pos sessed only ordinal scale properties, they were first analyzed using the Goodman-Kruskal (1954) Gamma, y, a nonparametric measure of association yielding values of - 1 &lt;y&lt; + 1 • This measure has an interpretation similar to that of a correlation coefficient, but is applicable to ordinal scale" (Data Analysis)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 11 subagent conflicts resolved. Found 2 new false positive papers (5 were already excluded). Final Included: ~157
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -17339,7 +17339,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F334" t="inlineStr">
+      <c r="F334" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -17539,7 +17539,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F338" t="inlineStr">
+      <c r="F338" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -17585,7 +17585,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr">
+      <c r="F339" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -17681,7 +17681,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F341" t="inlineStr">
+      <c r="F341" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -17727,7 +17727,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr">
+      <c r="F342" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -18023,7 +18023,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F348" t="inlineStr">
+      <c r="F348" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -18073,7 +18073,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F349" t="inlineStr">
+      <c r="F349" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -19910,6 +19910,11 @@
       </c>
       <c r="E386" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -19936,11 +19941,7 @@
       <c r="K386" s="0" t="n">
         <v>1985</v>
       </c>
-      <c r="P386" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P386" s="0" t="inlineStr"/>
     </row>
     <row r="387" ht="18" customHeight="1" s="31">
       <c r="A387" s="0" t="inlineStr">
@@ -19955,6 +19956,11 @@
       </c>
       <c r="E387" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -19981,11 +19987,7 @@
       <c r="K387" s="0" t="n">
         <v>1988</v>
       </c>
-      <c r="P387" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P387" s="0" t="inlineStr"/>
     </row>
     <row r="388" ht="18" customHeight="1" s="31">
       <c r="A388" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 12 subagent conflicts resolved. Found 6 new false positive papers. Final Included: ~151
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -19913,7 +19913,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F386" t="inlineStr">
+      <c r="F386" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -19959,7 +19959,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F387" t="inlineStr">
+      <c r="F387" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -20242,7 +20242,12 @@
       </c>
       <c r="E393" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G393" s="0" t="inlineStr">
@@ -20270,7 +20275,7 @@
       </c>
       <c r="P393" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative interviews. Verbatim Evidence: "Our empirical study builds on 145 qualitative interviews with 118 individuals, yielding circa 1800 single-spaced pages of transcripts and 936,000 words." (Section 3. Data and methods)</t>
         </is>
       </c>
     </row>
@@ -20337,6 +20342,11 @@
       </c>
       <c r="E395" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -20363,11 +20373,7 @@
       <c r="K395" s="0" t="n">
         <v>2001</v>
       </c>
-      <c r="P395" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P395" s="0" t="inlineStr"/>
     </row>
     <row r="396" ht="18" customHeight="1" s="31">
       <c r="A396" s="0" t="inlineStr">
@@ -20482,7 +20488,12 @@
       </c>
       <c r="E398" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G398" s="0" t="inlineStr">
@@ -20510,7 +20521,7 @@
       </c>
       <c r="P398" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>rwg aggregation. Verbatim Evidence: "A check of the subordinate data tested whether aggregating the assessments by groups of subordinates for each senior manager was appropriate, according to the index of within-group interrater reliability (rwg)... Thus the averaged subordinate responses for each senior manager formed a single-group composite value"</t>
         </is>
       </c>
     </row>
@@ -20899,7 +20910,12 @@
       </c>
       <c r="E406" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G406" s="0" t="inlineStr">
@@ -20927,7 +20943,7 @@
       </c>
       <c r="P406" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter-organizational conflict" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -21094,7 +21110,12 @@
       </c>
       <c r="E410" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G410" s="0" t="inlineStr">
@@ -21122,7 +21143,7 @@
       </c>
       <c r="P410" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No Pearson correlation matrix. Verbatim Evidence: "Bivariate Pearson, Spearman, and phi correlation tests did not indicate any problematic collinearity among independent variables (e.g., &gt;0.33). Nor were the dependent variables highly correlated with any of the independent or control variables (i.e., all &gt;0.21)." (Analyses)</t>
         </is>
       </c>
     </row>
@@ -21289,6 +21310,11 @@
       </c>
       <c r="E414" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -21315,11 +21341,7 @@
       <c r="K414" s="0" t="n">
         <v>2008</v>
       </c>
-      <c r="P414" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P414" s="0" t="inlineStr"/>
     </row>
     <row r="415" ht="18" customHeight="1" s="31">
       <c r="A415" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 13 subagent conflicts resolved. Found 8 new false positive papers. Final Included: ~143
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -20245,7 +20245,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F393" t="inlineStr">
+      <c r="F393" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -20345,7 +20345,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F395" t="inlineStr">
+      <c r="F395" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -20491,7 +20491,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F398" t="inlineStr">
+      <c r="F398" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -20913,7 +20913,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F406" t="inlineStr">
+      <c r="F406" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -21113,7 +21113,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F410" t="inlineStr">
+      <c r="F410" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -21313,7 +21313,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F414" t="inlineStr">
+      <c r="F414" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -21596,7 +21596,12 @@
       </c>
       <c r="E420" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G420" s="0" t="inlineStr">
@@ -21624,7 +21629,7 @@
       </c>
       <c r="P420" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Group level analysis. Verbatim Evidence: "These two levels of analysis are hereafter identified as level-1 for nurses (at the individual level) and level-2 for managers (at the group level)." (Sample)</t>
         </is>
       </c>
     </row>
@@ -21641,7 +21646,12 @@
       </c>
       <c r="E421" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G421" s="0" t="inlineStr">
@@ -21669,7 +21679,7 @@
       </c>
       <c r="P421" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Unit level boundary spanning. Verbatim Evidence: "Employees in your unit frequently meet with individuals from other companies or organizations" and "Because the supervisors are most likely to have an accurate understanding of the organizational structures, the following measures are based on responses from supervisors."</t>
         </is>
       </c>
     </row>
@@ -21736,7 +21746,12 @@
       </c>
       <c r="E423" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G423" s="0" t="inlineStr">
@@ -21764,7 +21779,7 @@
       </c>
       <c r="P423" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "Table 1. Means, Standard Deviations, and Correlation Coefficients... 1. Workplace bullying, 2. Turnover intention, 3. Negative emotions, 4. Workplace unfairness"</t>
         </is>
       </c>
     </row>
@@ -21931,7 +21946,12 @@
       </c>
       <c r="E427" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G427" s="0" t="inlineStr">
@@ -21959,7 +21979,7 @@
       </c>
       <c r="P427" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project level aggregation. Verbatim Evidence: "Since the unit of analysis in Hypothesis 4 is the project, individual responses must be pooled to get project scores."</t>
         </is>
       </c>
     </row>
@@ -22176,7 +22196,12 @@
       </c>
       <c r="E432" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G432" s="0" t="inlineStr">
@@ -22204,7 +22229,7 @@
       </c>
       <c r="P432" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>General consumers. Verbatim Evidence: "There were only two requirements for participation: prospective samples must have been at least 18 years of age as well as having dined in a full-service restaurant in the previous 1 year."</t>
         </is>
       </c>
     </row>
@@ -22271,7 +22296,12 @@
       </c>
       <c r="E434" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G434" s="0" t="inlineStr">
@@ -22299,7 +22329,7 @@
       </c>
       <c r="P434" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project level. Verbatim Evidence: "To investigate this issue, we examine 6081 research projects in the Life Sciences, Physical &amp; Engineering, and Social Sciences &amp; Humanities sectors funded by the European Research Council"</t>
         </is>
       </c>
     </row>
@@ -22935,7 +22965,12 @@
       </c>
       <c r="E447" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G447" s="0" t="inlineStr">
@@ -22963,7 +22998,7 @@
       </c>
       <c r="P447" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "Design/methodology/approach – The authors utilized regression analytical technique and categorical moderation analytical technique to test their hypotheses on survey data of 579 firms."</t>
         </is>
       </c>
     </row>
@@ -23030,6 +23065,11 @@
       </c>
       <c r="E449" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -23056,11 +23096,7 @@
       <c r="K449" s="0" t="n">
         <v>2016</v>
       </c>
-      <c r="P449" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P449" s="0" t="inlineStr"/>
     </row>
     <row r="450" ht="18" customHeight="1" s="31">
       <c r="A450" s="0" t="inlineStr">
@@ -23075,6 +23111,11 @@
       </c>
       <c r="E450" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -23101,11 +23142,7 @@
       <c r="K450" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P450" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P450" s="0" t="inlineStr"/>
     </row>
     <row r="451" ht="18" customHeight="1" s="31">
       <c r="A451" s="0" t="inlineStr">
@@ -23120,7 +23157,12 @@
       </c>
       <c r="E451" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G451" s="0" t="inlineStr">
@@ -23182,7 +23224,7 @@
       </c>
       <c r="P451" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "The primary purpose of this study was to (1) construct a measure of WTNW segmentation behaviors, (2) to examine the relationship between these segmentation behaviors and WTNC" (CHAPTER 10 GENERAL DISCUSSION)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 14 subagent conflicts resolved. Found 6 new false positive papers. Final Included: ~137
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -21599,7 +21599,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F420" t="inlineStr">
+      <c r="F420" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -21649,7 +21649,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F421" t="inlineStr">
+      <c r="F421" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -21749,7 +21749,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F423" t="inlineStr">
+      <c r="F423" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -21949,7 +21949,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F427" t="inlineStr">
+      <c r="F427" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -22199,7 +22199,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F432" t="inlineStr">
+      <c r="F432" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -22299,7 +22299,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F434" t="inlineStr">
+      <c r="F434" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -22968,7 +22968,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F447" t="inlineStr">
+      <c r="F447" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -23068,7 +23068,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F449" t="inlineStr">
+      <c r="F449" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -23114,7 +23114,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F450" t="inlineStr">
+      <c r="F450" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -23160,7 +23160,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F451" t="inlineStr">
+      <c r="F451" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -23681,7 +23681,12 @@
       </c>
       <c r="E461" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G461" s="0" t="inlineStr">
@@ -23709,7 +23714,7 @@
       </c>
       <c r="P461" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative interviews. Verbatim Evidence: "Over the course of the study, I conducted 14 semi-structured meetings on Zoom."</t>
         </is>
       </c>
     </row>
@@ -23776,7 +23781,12 @@
       </c>
       <c r="E463" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G463" s="0" t="inlineStr">
@@ -23804,7 +23814,7 @@
       </c>
       <c r="P463" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Moderator only, no zero-order correlation. Verbatim Evidence: "The moderator variable in this research is involvement in boundary spanning activity. Again, boundary spanning activity is defined as job-related interaction with an individual or individuals who are not members of the same organization. Boundary spanning activity is a moderator since it is hypothesized as affecting the strength of the relationship between the nature of an individual's work setting and his or her behavior." (Page 36)</t>
         </is>
       </c>
     </row>
@@ -24021,6 +24031,11 @@
       </c>
       <c r="E468" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -24047,11 +24062,7 @@
       <c r="K468" s="0" t="n">
         <v>2012</v>
       </c>
-      <c r="P468" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P468" s="0" t="inlineStr"/>
     </row>
     <row r="469" ht="18" customHeight="1" s="31">
       <c r="A469" s="0" t="inlineStr">
@@ -24216,7 +24227,12 @@
       </c>
       <c r="E472" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G472" s="0" t="inlineStr">
@@ -24244,7 +24260,7 @@
       </c>
       <c r="P472" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team level analysis. Verbatim Evidence: "We chose the ‘group’ (or team) as the unit of analysis for practical reasons that ideate, plan, and execute the change." (Page 50)</t>
         </is>
       </c>
     </row>
@@ -24361,7 +24377,12 @@
       </c>
       <c r="E475" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G475" s="0" t="inlineStr">
@@ -24389,7 +24410,7 @@
       </c>
       <c r="P475" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "The main objective of this article is to explore the concomitant role of the HCI variables such as CSE, technology-training efficacy, perceived control over technology, and intrinsic motivation as moderators in the relationship between occupational stress and work exhaustion among software professionals." (4. HYPOTHESES)</t>
         </is>
       </c>
     </row>
@@ -24406,6 +24427,11 @@
       </c>
       <c r="E476" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -24432,11 +24458,7 @@
       <c r="K476" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="P476" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P476" s="0" t="inlineStr"/>
     </row>
     <row r="477" ht="18" customHeight="1" s="31">
       <c r="A477" s="0" t="inlineStr">
@@ -24551,6 +24573,11 @@
       </c>
       <c r="E479" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -24577,11 +24604,7 @@
       <c r="K479" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="P479" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P479" s="0" t="inlineStr"/>
     </row>
     <row r="480" ht="18" customHeight="1" s="31">
       <c r="A480" s="0" t="inlineStr">
@@ -24596,6 +24619,11 @@
       </c>
       <c r="E480" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -24622,11 +24650,7 @@
       <c r="K480" s="0" t="n">
         <v>1976</v>
       </c>
-      <c r="P480" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P480" s="0" t="inlineStr"/>
     </row>
     <row r="481" ht="18" customHeight="1" s="31">
       <c r="A481" s="0" t="inlineStr">
@@ -24641,7 +24665,12 @@
       </c>
       <c r="E481" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G481" s="0" t="inlineStr">
@@ -24669,7 +24698,7 @@
       </c>
       <c r="P481" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Group level aggregation. Verbatim Evidence: "Aggregation of data at the group level requires both a theoretical basis and empirical justification (Kozlowski &amp; Klein, 2000). [...] Therefore, both intergroup conflict scales were aggregated by groups."</t>
         </is>
       </c>
     </row>
@@ -24736,7 +24765,12 @@
       </c>
       <c r="E483" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G483" s="0" t="inlineStr">
@@ -24764,7 +24798,7 @@
       </c>
       <c r="P483" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Bibliometric WoS Data. Verbatim Evidence: "Bibliometric Web of Science data, enriched with National Science Founda- tion (NSF) journal classifications, formed the foundation from which a seed-and-expand dataset were created from journals containing the string cogni* and their cited articles for the years 2006-2016." (Abstract)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 15 subagent conflicts resolved. Found 4 new false positive papers. Final Included: ~133
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -23684,7 +23684,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F461" t="inlineStr">
+      <c r="F461" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -23784,7 +23784,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F463" t="inlineStr">
+      <c r="F463" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -24034,7 +24034,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F468" t="inlineStr">
+      <c r="F468" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -24230,7 +24230,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F472" t="inlineStr">
+      <c r="F472" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -24380,7 +24380,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F475" t="inlineStr">
+      <c r="F475" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -24430,7 +24430,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F476" t="inlineStr">
+      <c r="F476" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -24576,7 +24576,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F479" t="inlineStr">
+      <c r="F479" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -24622,7 +24622,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F480" t="inlineStr">
+      <c r="F480" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -24668,7 +24668,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F481" t="inlineStr">
+      <c r="F481" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -24768,7 +24768,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F483" t="inlineStr">
+      <c r="F483" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -25547,7 +25547,12 @@
       </c>
       <c r="E499" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G499" s="0" t="inlineStr">
@@ -25575,7 +25580,7 @@
       </c>
       <c r="P499" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm/Patent level. Verbatim Evidence: "The basic unit of analysis is the individual patent and its associated content, and the level of the analysis is the firm."</t>
         </is>
       </c>
     </row>
@@ -25692,10 +25697,14 @@
       </c>
       <c r="E502" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F502" s="0" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F502" s="0" t="n"/>
       <c r="G502" s="0" t="inlineStr">
         <is>
           <t>Boundary-spanning activity was studied in a large manufacturing company through a sample of 192 managers, engineers, and supervisors. Contrary to prior theory and research, this study found boundary-spanning activity unrelated to role conflict or ambiguity and positively related to job satisfac-tion for the total sample. Boundary-spanning activity was also positively related to a number of job characteristics for the total sample. Marked dif-ferences in boundary-spanning activity and its relationships with other variables, however, were found across occupational levels. While managers and engineers generally had boundary-spanning activity related to high levels of job satisfaction and job characteristics, first-level supervisors had boundary-spanning activity related to higher role conflict and lower job satisfaction with opportunities for promotion.</t>
@@ -25719,11 +25728,7 @@
       <c r="K502" s="0" t="n">
         <v>1976</v>
       </c>
-      <c r="P502" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee boundary spanning behavior and reporting statistical effect sizes. [Restored after deep methodology audit]</t>
-        </is>
-      </c>
+      <c r="P502" s="0" t="inlineStr"/>
     </row>
     <row r="503" ht="18" customHeight="1" s="31">
       <c r="A503" s="0" t="inlineStr">
@@ -25788,7 +25793,12 @@
       </c>
       <c r="E504" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G504" s="0" t="inlineStr">
@@ -25818,7 +25828,7 @@
       </c>
       <c r="P504" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Measures Boundary-Spanning Leadership (BSL), not BSB. Verbatim Evidence: "An autoregressive cross-lagged model was employed to examine the causal relationships among BSL, ACAP, and JE. Data were collected through three waves of surveys conducted at three-month intervals, with a final sample of 297 nurses in Chinese hospitals." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -25935,7 +25945,12 @@
       </c>
       <c r="E507" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G507" s="0" t="inlineStr">
@@ -25963,7 +25978,7 @@
       </c>
       <c r="P507" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative study. Verbatim Evidence: "Real time data, in the form of in-depth interviews (9 in total), was collected between 2001 and 2005, and included key boundary spanners from both organisations." (3. Method)</t>
         </is>
       </c>
     </row>
@@ -26030,6 +26045,11 @@
       </c>
       <c r="E509" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -26056,11 +26076,7 @@
       <c r="K509" s="0" t="n">
         <v>1989</v>
       </c>
-      <c r="P509" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P509" s="0" t="inlineStr"/>
     </row>
     <row r="510" ht="18" customHeight="1" s="31">
       <c r="A510" s="0" t="inlineStr">
@@ -26125,6 +26141,11 @@
       </c>
       <c r="E511" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -26151,11 +26172,7 @@
       <c r="K511" s="0" t="n">
         <v>2025</v>
       </c>
-      <c r="P511" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P511" s="0" t="inlineStr"/>
     </row>
     <row r="512" ht="18" customHeight="1" s="31">
       <c r="A512" s="0" t="inlineStr">
@@ -26170,6 +26187,11 @@
       </c>
       <c r="E512" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -26196,11 +26218,7 @@
       <c r="K512" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P512" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P512" s="0" t="inlineStr"/>
     </row>
     <row r="513" ht="18" customHeight="1" s="31">
       <c r="A513" s="0" t="inlineStr">
@@ -26265,6 +26283,11 @@
       </c>
       <c r="E514" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -26291,11 +26314,7 @@
       <c r="K514" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P514" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P514" s="0" t="inlineStr"/>
     </row>
     <row r="515" ht="18" customHeight="1" s="31">
       <c r="A515" s="0" t="inlineStr">
@@ -26610,7 +26629,12 @@
       </c>
       <c r="E521" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G521" s="0" t="inlineStr">
@@ -26638,7 +26662,7 @@
       </c>
       <c r="P521" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Organization level. Verbatim Evidence: "Our measure of collaboration identifies an organiza tion’s level of activity in joint projects."</t>
         </is>
       </c>
     </row>
@@ -26655,6 +26679,11 @@
       </c>
       <c r="E522" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -26681,11 +26710,7 @@
       <c r="K522" s="0" t="n">
         <v>2019</v>
       </c>
-      <c r="P522" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P522" s="0" t="inlineStr"/>
     </row>
     <row r="523" ht="18" customHeight="1" s="31">
       <c r="A523" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 16 subagent conflicts resolved. Found 8 new false positive papers. Final Included: ~125
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -25550,7 +25550,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F499" t="inlineStr">
+      <c r="F499" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -25796,7 +25796,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F504" t="inlineStr">
+      <c r="F504" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -25948,7 +25948,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F507" t="inlineStr">
+      <c r="F507" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -26048,7 +26048,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F509" t="inlineStr">
+      <c r="F509" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -26144,7 +26144,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F511" t="inlineStr">
+      <c r="F511" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -26190,7 +26190,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F512" t="inlineStr">
+      <c r="F512" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -26286,7 +26286,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F514" t="inlineStr">
+      <c r="F514" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -26632,7 +26632,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F521" t="inlineStr">
+      <c r="F521" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -26682,7 +26682,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F522" t="inlineStr">
+      <c r="F522" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -27256,7 +27256,12 @@
       </c>
       <c r="E534" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G534" s="0" t="inlineStr">
@@ -27284,7 +27289,7 @@
       </c>
       <c r="P534" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "Our initial sample contained 2,427 house-season observations, but due to the need to accommodate lags of the variables which we needed to instrument, we performed our regressions on the remaining sample of 2,023 observations."</t>
         </is>
       </c>
     </row>
@@ -27451,7 +27456,12 @@
       </c>
       <c r="E538" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G538" s="0" t="inlineStr">
@@ -27479,7 +27489,7 @@
       </c>
       <c r="P538" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Dyad level. Verbatim Evidence: "The unit of analysis for this study is a manufacturer (buyer)–supplier dyad." (Page 8, 4.1. Data Collection and Sample Characteristics)</t>
         </is>
       </c>
     </row>
@@ -27546,6 +27556,11 @@
       </c>
       <c r="E540" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -27572,11 +27587,7 @@
       <c r="K540" s="0" t="n">
         <v>1988</v>
       </c>
-      <c r="P540" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P540" s="0" t="inlineStr"/>
     </row>
     <row r="541" ht="18" customHeight="1" s="31">
       <c r="A541" s="0" t="inlineStr">
@@ -27641,6 +27652,11 @@
       </c>
       <c r="E542" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -27667,11 +27683,7 @@
       <c r="K542" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P542" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P542" s="0" t="inlineStr"/>
     </row>
     <row r="543" ht="18" customHeight="1" s="31">
       <c r="A543" s="0" t="inlineStr">
@@ -27886,7 +27898,12 @@
       </c>
       <c r="E547" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G547" s="0" t="inlineStr">
@@ -27914,7 +27931,7 @@
       </c>
       <c r="P547" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Work unit level. Verbatim Evidence: "For inter-unit analysis (H1 and H2), the unit of analysis is at the work unit level. Network structure, as described earlier, was measured at the work unit level by collecting responses from unit leaders." (3.4 Levels of analysis)</t>
         </is>
       </c>
     </row>
@@ -27931,7 +27948,12 @@
       </c>
       <c r="E548" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G548" s="0" t="inlineStr">
@@ -27959,7 +27981,7 @@
       </c>
       <c r="P548" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "Attributed Power—The power construct (a = .78) focused on the degree to which the purchasing agent was perceived by his constituents to influence the purchasing decision making process." (Measures)</t>
         </is>
       </c>
     </row>
@@ -27976,7 +27998,12 @@
       </c>
       <c r="E549" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G549" s="0" t="inlineStr">
@@ -28004,7 +28031,7 @@
       </c>
       <c r="P549" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Regression only, no correlation matrix. Verbatim Evidence: "I ran five different generalized linear models (GLM) with CS as the dependent variable, using the “quasibinomial” family to account for CS being a proportion." (2.4 Analysis)</t>
         </is>
       </c>
     </row>
@@ -28021,7 +28048,12 @@
       </c>
       <c r="E550" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G550" s="0" t="inlineStr">
@@ -28049,7 +28081,15 @@
       </c>
       <c r="P550" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "Table I Mean, standard deviation, correlations and reliability among major variables 
+Variables M SD 1 2 3 4 5 6 
+1 Age 44.82 11.13 
+2 Gender (% Male) 0.84 0.95 0.16** 
+3 Problem-focused coping 3.72 0.64 0.02  0.05 (0.77) 
+4 Emotion-focused coping 2.24 0.90  0.05  0.01  0.10** (0.65) 
+5 Life satisfaction 3.40 0.64 0.09* 0.04 0.31**  0.14** (0.86) 
+6 Job satisfaction 3.87 0.68 0.16** 0.02 0.38**  0.27** 0.43** (0.89) 
+7 Sales commission 11,946.00 8,297.00 0.10 0.06 0.05 0.07 0.18** 0.11*" (5.1 Descriptive statistics)</t>
         </is>
       </c>
     </row>
@@ -28066,7 +28106,12 @@
       </c>
       <c r="E551" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G551" s="0" t="inlineStr">
@@ -28094,7 +28139,7 @@
       </c>
       <c r="P551" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "The components of Coping Intelligence, problem-focused coping (CI-P), action-focused coping (CI-A), and emotion-focused coping (CI-E), were measured using 33 items adapted from Folkman and Lazarus (1988) Ways of Coping Checklist." (Measure)</t>
         </is>
       </c>
     </row>
@@ -28111,7 +28156,12 @@
       </c>
       <c r="E552" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G552" s="0" t="inlineStr">
@@ -28139,7 +28189,7 @@
       </c>
       <c r="P552" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "The current study draws upon socialization theory to investigate both antecedents and outcomes of support service utilization within a sales employee context." (Abstract)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 17 subagent conflicts resolved. Found 8 new false positive papers. Final Included: ~117
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -27259,7 +27259,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F534" t="inlineStr">
+      <c r="F534" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -27459,7 +27459,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F538" t="inlineStr">
+      <c r="F538" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -27559,7 +27559,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F540" t="inlineStr">
+      <c r="F540" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -27655,7 +27655,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F542" t="inlineStr">
+      <c r="F542" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -27901,7 +27901,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F547" t="inlineStr">
+      <c r="F547" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -27951,7 +27951,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F548" t="inlineStr">
+      <c r="F548" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -28001,7 +28001,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F549" t="inlineStr">
+      <c r="F549" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -28051,7 +28051,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F550" t="inlineStr">
+      <c r="F550" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -28109,7 +28109,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F551" t="inlineStr">
+      <c r="F551" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -28159,7 +28159,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F552" t="inlineStr">
+      <c r="F552" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -28657,6 +28657,11 @@
       </c>
       <c r="E562" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -28683,11 +28688,7 @@
       <c r="K562" s="0" t="n">
         <v>2000</v>
       </c>
-      <c r="P562" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P562" s="0" t="inlineStr"/>
     </row>
     <row r="563" ht="18" customHeight="1" s="31">
       <c r="A563" s="0" t="inlineStr">
@@ -28802,7 +28803,12 @@
       </c>
       <c r="E565" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G565" s="0" t="inlineStr">
@@ -28830,7 +28836,7 @@
       </c>
       <c r="P565" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "In addition, drawing on the practice of previous literature (Hu &amp; Yu, 2017; Xu &amp; Yu, 2020), this paper incorporates the control variables firm age, firm size, ownership nature, and industry distribution into the research model." (Variable Measurement)</t>
         </is>
       </c>
     </row>
@@ -28847,7 +28853,12 @@
       </c>
       <c r="E566" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G566" s="0" t="inlineStr">
@@ -28875,7 +28886,7 @@
       </c>
       <c r="P566" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>ERGM, no correlation matrix. Verbatim Evidence: "Across the two samples, we report estimates of models for the probability of observing ties between members as a function of (i) dyadic covariate-based network statistics, based on actor-specific variables, or “covariate effects,” (ii) dyadic dependencies between network ties and (iii) extra-dyadic endogenous network statistics. The dependent variables of the study (advice ties) take the form of binary tie variables." (Methods -&gt; Variables and measures -&gt; Dependent variable)</t>
         </is>
       </c>
     </row>
@@ -28892,7 +28903,12 @@
       </c>
       <c r="E567" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G567" s="0" t="inlineStr">
@@ -28920,7 +28936,7 @@
       </c>
       <c r="P567" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Dyadic level. Verbatim Evidence: "Because we are interested in investigating the determinants of communication ties and vocabulary similarity between pairs of managers, our data set is dyadic—that is, observations are of type (i, j)." (Empirical Model Specification and Estimation)</t>
         </is>
       </c>
     </row>
@@ -28937,7 +28953,12 @@
       </c>
       <c r="E568" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G568" s="0" t="inlineStr">
@@ -28965,7 +28986,7 @@
       </c>
       <c r="P568" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "Purpose – The aim of this paper is to investigate the link between store managers’ evaluation of how customers assess a shopping centre and their own evaluation of the centre and, based on that, the relevance of store managers in reflecting on and informing the management and marketing practices of the local shopping centre management." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -28982,7 +29003,12 @@
       </c>
       <c r="E569" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G569" s="0" t="inlineStr">
@@ -29040,7 +29066,7 @@
       </c>
       <c r="P569" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project level. Verbatim Evidence: "This dissertation explores the development of core competence in emerging technology innovation projects, and the level of analysis is at the project level." (5.4.1 Level of Analysis)</t>
         </is>
       </c>
     </row>
@@ -29057,7 +29083,12 @@
       </c>
       <c r="E570" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G570" s="0" t="inlineStr">
@@ -29085,7 +29116,7 @@
       </c>
       <c r="P570" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Categorical, no correlation. Verbatim Evidence: "Shop Steward. This is a categorical, dichotomous variable to be used in a logistics regression equation." (Measurements)</t>
         </is>
       </c>
     </row>
@@ -29102,7 +29133,12 @@
       </c>
       <c r="E571" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G571" s="0" t="inlineStr">
@@ -29130,7 +29166,7 @@
       </c>
       <c r="P571" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Students. Verbatim Evidence: "Study participants consisted of primarily upper-level undergraduate students from a large university in the south-west United States."</t>
         </is>
       </c>
     </row>
@@ -29197,7 +29233,12 @@
       </c>
       <c r="E573" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G573" s="0" t="inlineStr">
@@ -29225,7 +29266,7 @@
       </c>
       <c r="P573" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project level. Verbatim Evidence: "A distinct feature of investigating problem solving processes is using the problem solving project as the level of analysis (Obstfeld, 2012)."</t>
         </is>
       </c>
     </row>
@@ -29342,6 +29383,11 @@
       </c>
       <c r="E576" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -29368,11 +29414,7 @@
       <c r="K576" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P576" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P576" s="0" t="inlineStr"/>
     </row>
     <row r="577" ht="18" customHeight="1" s="31">
       <c r="A577" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 18 subagent conflicts resolved. Found 8 new false positive papers. Final Included: ~109
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -28660,7 +28660,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F562" t="inlineStr">
+      <c r="F562" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -28806,7 +28806,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F565" t="inlineStr">
+      <c r="F565" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -28856,7 +28856,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F566" t="inlineStr">
+      <c r="F566" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -28906,7 +28906,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F567" t="inlineStr">
+      <c r="F567" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -28956,7 +28956,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F568" t="inlineStr">
+      <c r="F568" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -29006,7 +29006,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F569" t="inlineStr">
+      <c r="F569" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -29086,7 +29086,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F570" t="inlineStr">
+      <c r="F570" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -29136,7 +29136,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F571" t="inlineStr">
+      <c r="F571" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>
@@ -29236,7 +29236,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F573" t="inlineStr">
+      <c r="F573" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -29386,7 +29386,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F576" t="inlineStr">
+      <c r="F576" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -29619,7 +29619,12 @@
       </c>
       <c r="E581" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G581" s="0" t="inlineStr">
@@ -29647,7 +29652,7 @@
       </c>
       <c r="P581" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Discriminant analysis, no Pearson matrix. Verbatim Evidence: "A stepwise discriminant analysis indicates that hierarchical level is the most powerful determinant of intra-departmental communication, and that professional orientation and laboratory tenure are other important determinants of internal communication" (RESULTS)</t>
         </is>
       </c>
     </row>
@@ -29664,7 +29669,12 @@
       </c>
       <c r="E582" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G582" s="0" t="inlineStr">
@@ -29692,7 +29702,7 @@
       </c>
       <c r="P582" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "This paper focuses on entrepreneurial enterprises in the Internet industry." (Section 4.2. Sample and data collection)</t>
         </is>
       </c>
     </row>
@@ -29709,6 +29719,11 @@
       </c>
       <c r="E583" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -29735,11 +29750,7 @@
       <c r="K583" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P583" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P583" s="0" t="inlineStr"/>
     </row>
     <row r="584" ht="18" customHeight="1" s="31">
       <c r="A584" s="0" t="inlineStr">
@@ -29804,7 +29815,12 @@
       </c>
       <c r="E585" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G585" s="0" t="inlineStr">
@@ -29832,7 +29848,7 @@
       </c>
       <c r="P585" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "The remainder of the study addresses these focal relationships, namely corporate ethics, including codes and corporate ethical values (CEVs), workplace bullying, and job satisfaction." (Page 144)</t>
         </is>
       </c>
     </row>
@@ -29849,7 +29865,12 @@
       </c>
       <c r="E586" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G586" s="0" t="inlineStr">
@@ -29877,7 +29898,7 @@
       </c>
       <c r="P586" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative case study. Verbatim Evidence: "To study in-depth the micro-interactions of boundary management and explore boundary actions and configurations of actions over time we use a single longitudinal case study design." (3. Methods)</t>
         </is>
       </c>
     </row>
@@ -29894,7 +29915,12 @@
       </c>
       <c r="E587" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G587" s="0" t="inlineStr">
@@ -29922,7 +29948,7 @@
       </c>
       <c r="P587" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No BSB measure. Verbatim Evidence: "In this study (N = 213), we demonstrate that intergroup leadership is linked to employee psycho logical empowerment via intergroup relational identification and access to resources." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -29939,7 +29965,12 @@
       </c>
       <c r="E588" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G588" s="0" t="inlineStr">
@@ -29967,7 +29998,7 @@
       </c>
       <c r="P588" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team level aggregation. Verbatim Evidence: "The individual responses are aggregated to the team level, for which intraclass correlation coefficients are calculated in the analysis section." (Methods and procedures for data collection)</t>
         </is>
       </c>
     </row>
@@ -30334,7 +30365,12 @@
       </c>
       <c r="E596" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G596" s="0" t="inlineStr">
@@ -30362,7 +30398,7 @@
       </c>
       <c r="P596" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>SEM betas only, no Pearson matrix, no BSB. Verbatim Evidence: "Table 1 presents the structural parameter estimates and R2 values." (Results)</t>
         </is>
       </c>
     </row>
@@ -30429,6 +30465,11 @@
       </c>
       <c r="E598" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -30455,11 +30496,7 @@
       <c r="K598" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P598" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P598" s="0" t="inlineStr"/>
     </row>
     <row r="599" ht="18" customHeight="1" s="31">
       <c r="A599" s="0" t="inlineStr">
@@ -30674,7 +30711,12 @@
       </c>
       <c r="E603" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G603" s="0" t="inlineStr">
@@ -30702,7 +30744,7 @@
       </c>
       <c r="P603" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Literature review. Verbatim Evidence: "Table 1 summarizes our synthesis of the literature on boundary-spanning processes in social movements."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 19 subagent conflicts resolved. Found 6 new false positive papers. Final Included: ~103
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -29622,7 +29622,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F581" t="inlineStr">
+      <c r="F581" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -29672,7 +29672,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F582" t="inlineStr">
+      <c r="F582" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -29722,7 +29722,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F583" t="inlineStr">
+      <c r="F583" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -29818,7 +29818,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F585" t="inlineStr">
+      <c r="F585" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -29868,7 +29868,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F586" t="inlineStr">
+      <c r="F586" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -29918,7 +29918,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F587" t="inlineStr">
+      <c r="F587" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -29968,7 +29968,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F588" t="inlineStr">
+      <c r="F588" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -30368,7 +30368,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F596" t="inlineStr">
+      <c r="F596" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -30468,7 +30468,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F598" t="inlineStr">
+      <c r="F598" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -30714,7 +30714,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F603" t="inlineStr">
+      <c r="F603" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -30951,7 +30951,12 @@
       </c>
       <c r="E608" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G608" s="0" t="inlineStr">
@@ -30979,7 +30984,7 @@
       </c>
       <c r="P608" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Squared correlations lose sign. Verbatim Evidence: "As shown in Table 3, AVE scores for all dimensions, presented in the diagonal of the matrix, exceeded the squares of paired correlation coefficients, shown in the off-diagonal of the matrix, satisfying discriminant validity (Chin, 1998)." (Section 4.2 Measurement model)</t>
         </is>
       </c>
     </row>
@@ -30996,6 +31001,11 @@
       </c>
       <c r="E609" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -31022,11 +31032,7 @@
       <c r="K609" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P609" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P609" s="0" t="inlineStr"/>
     </row>
     <row r="610" ht="18" customHeight="1" s="31">
       <c r="A610" s="0" t="inlineStr">
@@ -31091,7 +31097,12 @@
       </c>
       <c r="E611" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G611" s="0" t="inlineStr">
@@ -31119,7 +31130,7 @@
       </c>
       <c r="P611" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "Survey data are collected from 218 manufacturing firms in China" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -31136,7 +31147,12 @@
       </c>
       <c r="E612" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G612" s="0" t="inlineStr">
@@ -31164,7 +31180,7 @@
       </c>
       <c r="P612" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Enterprise level. Verbatim Evidence: "110 service-oriented manufacturing enterprises as research samples"</t>
         </is>
       </c>
     </row>
@@ -31181,7 +31197,12 @@
       </c>
       <c r="E613" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G613" s="0" t="inlineStr">
@@ -31209,7 +31230,7 @@
       </c>
       <c r="P613" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Department level. Verbatim Evidence: "The boundary spanning and boundary buffering scales were measured using four items adopted by Faraj and Yan (2009), and were mainly concerned with the boundary spanning and boundary buffering behavior of IT departments with the IT department as the boundary."</t>
         </is>
       </c>
     </row>
@@ -31226,6 +31247,11 @@
       </c>
       <c r="E614" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -31252,11 +31278,7 @@
       <c r="K614" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P614" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P614" s="0" t="inlineStr"/>
     </row>
     <row r="615" ht="18" customHeight="1" s="31">
       <c r="A615" s="0" t="inlineStr">
@@ -31271,6 +31293,11 @@
       </c>
       <c r="E615" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -31297,11 +31324,7 @@
       <c r="K615" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P615" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P615" s="0" t="inlineStr"/>
     </row>
     <row r="616" ht="18" customHeight="1" s="31">
       <c r="A616" s="0" t="inlineStr">
@@ -31366,6 +31389,11 @@
       </c>
       <c r="E617" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -31392,11 +31420,7 @@
       <c r="K617" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P617" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P617" s="0" t="inlineStr"/>
     </row>
     <row r="618" ht="18" customHeight="1" s="31">
       <c r="A618" s="0" t="inlineStr">
@@ -31761,7 +31785,12 @@
       </c>
       <c r="E625" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G625" s="0" t="inlineStr">
@@ -31789,7 +31818,7 @@
       </c>
       <c r="P625" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative. Verbatim Evidence: "The find ings from Phase 1 were used to inform the topic guide for a series of in depth and semi-structured interviews. Topics covered included motivations for partnership working; the management of boundary spanning roles; per sonal skills and competencies for collaborative working; evidencing effec tiveness through critical incidents; barriers and problems in cross-boundary activity; and training and development."</t>
         </is>
       </c>
     </row>
@@ -31806,7 +31835,12 @@
       </c>
       <c r="E626" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G626" s="0" t="inlineStr">
@@ -31834,7 +31868,7 @@
       </c>
       <c r="P626" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project group level. Verbatim Evidence: "Since the project group is the unit of analysis in the present study, all variables were aggregated to group means." (Page 16)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit: Shadow Batch 20 subagent conflicts resolved. Found 7 new false positive papers. Final Included: ~96
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -30954,7 +30954,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F608" t="inlineStr">
+      <c r="F608" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -31004,7 +31004,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F609" t="inlineStr">
+      <c r="F609" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -31100,7 +31100,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F611" t="inlineStr">
+      <c r="F611" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -31150,7 +31150,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F612" t="inlineStr">
+      <c r="F612" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -31200,7 +31200,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F613" t="inlineStr">
+      <c r="F613" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -31250,7 +31250,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F614" t="inlineStr">
+      <c r="F614" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -31296,7 +31296,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F615" t="inlineStr">
+      <c r="F615" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -31392,7 +31392,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F617" t="inlineStr">
+      <c r="F617" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -31788,7 +31788,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F625" t="inlineStr">
+      <c r="F625" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -31838,7 +31838,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F626" t="inlineStr">
+      <c r="F626" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -32265,7 +32265,12 @@
       </c>
       <c r="E635" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G635" s="0" t="inlineStr">
@@ -32293,7 +32298,7 @@
       </c>
       <c r="P635" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team/Project level. Verbatim Evidence: "The unit of analysis is the new product design team considered at the project level." (Section 2.2 External uncertainty and internal complexity)</t>
         </is>
       </c>
     </row>
@@ -32310,7 +32315,12 @@
       </c>
       <c r="E636" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G636" s="0" t="inlineStr">
@@ -32338,7 +32348,7 @@
       </c>
       <c r="P636" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Organizational network. Verbatim Evidence: "Our dependent variable is whether an organization seeks out information from another via social media, and we operationalize it as whether an emergency management organization follows the Twitter account of another emergency management organization in a foreign country. Thus, our unit of analysis is the directional dyad." (Data Collection)</t>
         </is>
       </c>
     </row>
@@ -32405,6 +32415,11 @@
       </c>
       <c r="E638" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -32431,11 +32446,7 @@
       <c r="K638" s="0" t="n">
         <v>2023</v>
       </c>
-      <c r="P638" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P638" s="0" t="inlineStr"/>
     </row>
     <row r="639" ht="18" customHeight="1" s="31">
       <c r="A639" s="0" t="inlineStr">
@@ -32500,7 +32511,12 @@
       </c>
       <c r="E640" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G640" s="0" t="inlineStr">
@@ -32528,7 +32544,7 @@
       </c>
       <c r="P640" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "Based on data collected from 294 manufacturing firms in China, the results show that both value-chain-based proactive search and industry–university-based proactive search positively influence radical green innovation." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -32545,7 +32561,12 @@
       </c>
       <c r="E641" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G641" s="0" t="inlineStr">
@@ -32573,7 +32594,7 @@
       </c>
       <c r="P641" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team level. Verbatim Evidence: "Team boundary-spanning behavior (short as TBB) was usually defined as teams’ activities of continuously establishing, managing relations, and interacting with external for accomplishing specific goals (Choi, 2002)."</t>
         </is>
       </c>
     </row>
@@ -32790,7 +32811,12 @@
       </c>
       <c r="E646" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G646" s="0" t="inlineStr">
@@ -32818,7 +32844,7 @@
       </c>
       <c r="P646" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "This study selected China’s advanced manufacturing firms as the research sample" (Section 3.1 Sample and data collection)</t>
         </is>
       </c>
     </row>
@@ -32835,7 +32861,12 @@
       </c>
       <c r="E647" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G647" s="0" t="inlineStr">
@@ -32863,7 +32894,7 @@
       </c>
       <c r="P647" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "To guarantee the typicality of samples, we randomly selected 100 firms in each region referring to the local business directory, a total of 600 firms." (Section 3.1. Sampling and data collection)</t>
         </is>
       </c>
     </row>
@@ -32980,7 +33011,12 @@
       </c>
       <c r="E650" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G650" s="0" t="inlineStr">
@@ -33008,7 +33044,7 @@
       </c>
       <c r="P650" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Team level aggregation. Verbatim Evidence: "Before aggregating individual-level data into founding team-level variables, we computed well-accepted statistical indexes such as the Index of Within-Group Interrater Agreement (Rwg) (James et al., 1993) and Interclass Correlation Coefficient (ICC (1) and ICC (2))."</t>
         </is>
       </c>
     </row>
@@ -33025,10 +33061,14 @@
       </c>
       <c r="E651" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F651" s="0" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F651" s="0" t="n"/>
       <c r="G651" s="0" t="inlineStr">
         <is>
           <t>This study examines the impact of emotional intelligence (EI) on boundaryspanning behavior, relationship quality, and performance among door‐todoor salespeople. Data is collected from salespeople and customers of South Korean door‐to‐door cosmetics businesses and analyzed using structural equation modeling. The findings show that EI positively affects boundaryspanning behavior. Similarly, boundary‐spanning behavior improves relationship quality, which improves both sales performance and customer satisfaction. This suggests that EI plays an important role in salespeople's boundaryspanning behavior, thereby enhancing relationship quality, sales performance, and customer satisfaction. Unlike previous studies, this study makes use of actual sales volumes, salespeople's self‐reporting responses, and salespeople's customer‐reporting, which adds to the findings' uniqueness. The present study highlights that EI improves boundary‐spanning behavior, which is vital in developing relationship quality, improving sales performance, and increasing customer satisfaction. The study uses triadic data from door‐to‐door salespeople, customers, and sales organizations extensively, which is unusual in this field.</t>
@@ -33052,11 +33092,7 @@
       <c r="K651" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P651" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee boundary spanning behavior and reporting statistical effect sizes. [Restored after deep methodology audit]</t>
-        </is>
-      </c>
+      <c r="P651" s="0" t="inlineStr"/>
     </row>
     <row r="652" ht="18" customHeight="1" s="31">
       <c r="A652" s="0" t="inlineStr">
@@ -33321,6 +33357,11 @@
       </c>
       <c r="E657" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -33347,11 +33388,7 @@
       <c r="K657" s="0" t="n">
         <v>2013</v>
       </c>
-      <c r="P657" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P657" s="0" t="inlineStr"/>
     </row>
     <row r="658" ht="18" customHeight="1" s="31">
       <c r="A658" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 21 subagent conflicts resolved. Found 8 new false positive papers. Final Included: ~88
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -32268,7 +32268,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F635" t="inlineStr">
+      <c r="F635" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -32318,7 +32318,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F636" t="inlineStr">
+      <c r="F636" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -32418,7 +32418,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F638" t="inlineStr">
+      <c r="F638" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -32514,7 +32514,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F640" t="inlineStr">
+      <c r="F640" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -32564,7 +32564,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F641" t="inlineStr">
+      <c r="F641" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -32814,7 +32814,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F646" t="inlineStr">
+      <c r="F646" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -32864,7 +32864,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F647" t="inlineStr">
+      <c r="F647" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -33014,7 +33014,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F650" t="inlineStr">
+      <c r="F650" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -33360,7 +33360,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F657" t="inlineStr">
+      <c r="F657" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -33588,7 +33588,12 @@
       </c>
       <c r="E662" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G662" s="0" t="inlineStr">
@@ -33616,7 +33621,7 @@
       </c>
       <c r="P662" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "A total of 270 non-core firms whose senior managers agreed to take part in the survey were finally identified as the sample firms, and a roster was made." (Sample and Data Collection)</t>
         </is>
       </c>
     </row>
@@ -33733,7 +33738,12 @@
       </c>
       <c r="E665" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G665" s="0" t="inlineStr">
@@ -33761,7 +33771,7 @@
       </c>
       <c r="P665" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level employee/leader boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>t-test and ANOVA only. Verbatim Evidence: "In analyzing the research question and hypothesis, the overall mean score was used as a basis to determine the orientation towards innovative work behavior and to test the differences in the contexts of demographic factors the t-test and ANOVA analyses were used." (3. METHODOLOGY)</t>
         </is>
       </c>
     </row>
@@ -33828,7 +33838,12 @@
       </c>
       <c r="E667" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G667" s="0" t="inlineStr">
@@ -33856,7 +33871,7 @@
       </c>
       <c r="P667" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>ERGM network tie parameters, no Pearson matrix. Verbatim Evidence: "To do this, we apply Multilevel Exponential Random Graph Models on data collected in a multiunit government institution in Italy."</t>
         </is>
       </c>
     </row>
@@ -33923,7 +33938,12 @@
       </c>
       <c r="E669" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G669" s="0" t="inlineStr">
@@ -33951,7 +33971,7 @@
       </c>
       <c r="P669" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative. Verbatim Evidence: "Taking a practice-based theoretical stance, the paper presents findings of qualitative research on the nature and genesis of design boundaries and their relation to the strategic decision-making on a transportation infrastructure project." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -34168,7 +34188,12 @@
       </c>
       <c r="E674" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G674" s="0" t="inlineStr">
@@ -34196,7 +34221,7 @@
       </c>
       <c r="P674" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level patent network. Verbatim Evidence: "The sample consists of 103 listed firms with more than 500 invention patents and a 5-year R&amp;D history." (6 | CONCLUSION)</t>
         </is>
       </c>
     </row>
@@ -34213,7 +34238,12 @@
       </c>
       <c r="E675" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G675" s="0" t="inlineStr">
@@ -34241,7 +34271,7 @@
       </c>
       <c r="P675" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Manufacturing plants. Verbatim Evidence: "The data were collected from 288 manufacturing plants located in 13 different countries and three different industrial sectors (electronics, machinery and transportation equipment)." (Section 3.1 Data)</t>
         </is>
       </c>
     </row>
@@ -34258,6 +34288,11 @@
       </c>
       <c r="E676" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -34284,11 +34319,7 @@
       <c r="K676" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P676" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P676" s="0" t="inlineStr"/>
     </row>
     <row r="677" ht="18" customHeight="1" s="31">
       <c r="A677" s="0" t="inlineStr">
@@ -34303,7 +34334,12 @@
       </c>
       <c r="E677" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G677" s="0" t="inlineStr">
@@ -34331,7 +34367,7 @@
       </c>
       <c r="P677" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>MNC-country-year. Verbatim Evidence: "We eventually obtained 97 MNCs involving 60,185 patents, whose overseas research operations are located across 24 host countries, comprising an unbalanced panel of 1954 MNC-country-year observations."</t>
         </is>
       </c>
     </row>
@@ -34516,7 +34552,12 @@
       </c>
       <c r="E681" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G681" s="0" t="inlineStr">
@@ -34544,7 +34585,7 @@
       </c>
       <c r="P681" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm level. Verbatim Evidence: "Specifically, the authors collected a sample composed of 150 high-tech manufacturing Chinese firms."</t>
         </is>
       </c>
     </row>
@@ -34611,6 +34652,11 @@
       </c>
       <c r="E683" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -34637,11 +34683,7 @@
       <c r="K683" s="0" t="n">
         <v>2025</v>
       </c>
-      <c r="P683" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P683" s="0" t="inlineStr"/>
     </row>
     <row r="684" ht="18" customHeight="1" s="31">
       <c r="A684" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Audit: Shadow Batch 22 subagent conflicts resolved. Found 2 new false positive papers. Final Included: ~86
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -33591,7 +33591,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F662" t="inlineStr">
+      <c r="F662" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -33741,7 +33741,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F665" t="inlineStr">
+      <c r="F665" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -33841,7 +33841,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F667" t="inlineStr">
+      <c r="F667" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -33941,7 +33941,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F669" t="inlineStr">
+      <c r="F669" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -34191,7 +34191,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F674" t="inlineStr">
+      <c r="F674" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -34241,7 +34241,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F675" t="inlineStr">
+      <c r="F675" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -34291,7 +34291,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F676" t="inlineStr">
+      <c r="F676" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -34337,7 +34337,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F677" t="inlineStr">
+      <c r="F677" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -34555,7 +34555,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F681" t="inlineStr">
+      <c r="F681" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -34655,7 +34655,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F683" t="inlineStr">
+      <c r="F683" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -34838,6 +34838,11 @@
       </c>
       <c r="E687" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -34864,11 +34869,7 @@
       <c r="K687" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P687" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P687" s="0" t="inlineStr"/>
     </row>
     <row r="688" ht="18" customHeight="1" s="31">
       <c r="A688" s="0" t="inlineStr">
@@ -34883,6 +34884,11 @@
       </c>
       <c r="E688" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -34909,11 +34915,7 @@
       <c r="K688" s="0" t="n">
         <v>2023</v>
       </c>
-      <c r="P688" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P688" s="0" t="inlineStr"/>
     </row>
     <row r="689" ht="18" customHeight="1" s="31">
       <c r="A689" s="0" t="inlineStr">
@@ -35028,6 +35030,11 @@
       </c>
       <c r="E691" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -35054,11 +35061,7 @@
       <c r="K691" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P691" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P691" s="0" t="inlineStr"/>
     </row>
     <row r="692" ht="18" customHeight="1" s="31">
       <c r="A692" s="0" t="inlineStr">
@@ -35223,6 +35226,11 @@
       </c>
       <c r="E695" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -35249,11 +35257,7 @@
       <c r="K695" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P695" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P695" s="0" t="inlineStr"/>
     </row>
     <row r="696" ht="18" customHeight="1" s="31">
       <c r="A696" s="0" t="inlineStr">
@@ -35418,6 +35422,11 @@
       </c>
       <c r="E699" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -35444,11 +35453,7 @@
       <c r="K699" s="0" t="n">
         <v>2017</v>
       </c>
-      <c r="P699" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P699" s="0" t="inlineStr"/>
     </row>
     <row r="700" ht="18" customHeight="1" s="31">
       <c r="A700" s="0" t="inlineStr">
@@ -35463,7 +35468,12 @@
       </c>
       <c r="E700" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G700" s="0" t="inlineStr">
@@ -35491,7 +35501,7 @@
       </c>
       <c r="P700" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Correlation table in online appendix. Verbatim Evidence: "Details on all measures and descriptive statistics can be found in the online appendix (Tables A1–A3 and Figures A1 and A2). The correlation table and an estimation of variance inflation factors indicate that our estimations are not subject to multicollinearity issues." (Methods - Control Variables)</t>
         </is>
       </c>
     </row>
@@ -35608,6 +35618,11 @@
       </c>
       <c r="E703" s="0" t="inlineStr">
         <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
           <t>1 = Include</t>
         </is>
       </c>
@@ -35634,11 +35649,7 @@
       <c r="K703" s="0" t="n">
         <v>2013</v>
       </c>
-      <c r="P703" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P703" s="0" t="inlineStr"/>
     </row>
     <row r="704" ht="18" customHeight="1" s="31">
       <c r="A704" s="0" t="inlineStr">
@@ -35653,7 +35664,12 @@
       </c>
       <c r="E704" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G704" s="0" t="inlineStr">
@@ -35681,7 +35697,7 @@
       </c>
       <c r="P704" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>701-page Dissertation. Verbatim Evidence: "This manuscript has been reproduced from the microfilm master. U M I films the text directly from the original or copy submitted. Thus, some thesis and dissertation copies are in typewriter face" (Page 1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Recover 65 falsely excluded papers due to apply_shadow_batch script bug. Final Included: 114
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -3347,7 +3347,7 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="P53" s="0" t="inlineStr">
         <is>
-          <t>Descriptive frequency survey of audit committee meetings without an individual employee Pearson correlation matrix. Verbatim Evidence: "This paper's empirical contribution is to investigate the extent to which ACs and audit committee chairs (ACCs) engage with chief financial officers (CFOs) and audit partners (APs) across a range of 32 financial reporting issues... Table 1 shows the 32 issues in the order that they appeared in the questionnaire." (Abstract / Methodology section)</t>
+          <t>No correlation matrix, only ANOVA/Chi-square. Verbatim Evidence: "Across all potential discussion issues, the combined sample reported 5,445 discussions. The parties involved in these discussions are shown in Table 5, which reports frequencies for the 15 combinations."</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="P55" s="0" t="inlineStr">
         <is>
-          <t>Team-level aggregation study. Verbatim Evidence: "The results of the structural equation model from a sample of 92 interdisciplinary teams indicate that leaders' internal activities fully mediate the relationship of team functional heterogeneity and interteam goal interdependence to team in-role performance (N = 92 teams)." (Abstract / Methodology section)</t>
+          <t>Team level analysis. Verbatim Evidence: "In the research hypotheses, the team is identified as the unit of analysis. Therefore, team innovation and team in-role performance were assessed by the team leader, the principal. Interteam goal interdependence and leader internal and external activities were represented by an aggregate of team member responses." (Level of Analysis, page 18)</t>
         </is>
       </c>
     </row>
@@ -3542,14 +3542,10 @@
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F57" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F57" s="0" t="inlineStr"/>
       <c r="G57" s="0" t="inlineStr">
         <is>
           <t>The authors investigate three types of customer-oriented boundary-spanning behaviors (COBSBs)a frontline service employee may perform that are associated with linking a service organization to its potential or actual customers: external representation, internal influence, and service delivery. The authors propose and test a withdrawal model to explain the negative effects of role conflict and role ambiguity on COBSBs across a sample of 220 lower-level, nonprofessional service providers of a major retail bank and a sample of 90 higher-level, professional service providers from the business credit division of an international financial services corporation. The results demonstrate that (1)indirect paths through job satisfaction and organizational commitment entirely account for the negative effects of the role stressors on COBSBs, (2) the indirect negative effects of the role stressors are stronger on external representation and internal influence behaviors, and (3)role conflict also has a significant positive direct relationship with internal influence behaviors.</t>
@@ -3588,14 +3584,10 @@
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F58" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F58" s="0" t="inlineStr"/>
       <c r="G58" s="0" t="inlineStr">
         <is>
           <t>Using a sample of 281 frontline service employees of a national retail bank, we test a social exchange model of antecedents of three dimensions of customer-oriented boundary-spanning behaviors suggested by prior boundary-spanning and services marketing/management literatures: external representation, internal inﬂuence, and service delivery. In support of our hypotheses, we identify fully mediated relationships from procedural, interactional, and distributive justice to external representation and internal inﬂuence via job satisfaction and organizational commitment. Our results generally support our expectation that the indirect effects of procedural justice on external representation and internal inﬂuence are stronger than the indirect effects of distributive or interactional justice on these behaviors. Also, our results reveal no signiﬁcant indirect effects of procedural and distributive justice on service delivery behaviors. However, we ﬁnd an unexpected direct positive path from interactional justice to service delivery behaviors. We interpret this latter ﬁnding in light of the normative value of interactional justice as a source of role modeling or managerial legitimacy.</t>
@@ -3739,7 +3731,7 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
@@ -3772,7 +3764,7 @@
       </c>
       <c r="P61" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of organizational buyers (customers/clients), not internal workplace employees. Verbatim Evidence: "The model is tested on a sample of 120 organizational buyers of advertising services by using partial least squares, a structural equation modelling technique." (Abstract / Methodology section)</t>
+          <t>Firm/inter-organizational level. Verbatim Evidence: "The model is tested on a sample of 120 organizational buyers of advertising services by using partial last squares, a structural equation modelling technique." (Abstract, p. 223)</t>
         </is>
       </c>
     </row>
@@ -3872,7 +3864,7 @@
       </c>
       <c r="P63" s="0" t="inlineStr">
         <is>
-          <t>Pure conceptual / theoretical paper without quantitative employee survey correlation data. Verbatim Evidence: "We examine in detail what the temporal imagination is, complemented with a discussion of the related timescape idea, and why the temporal imagination is necessary to function in any timescape. We also discuss group attributes that will likely affect the development..." (Abstract / Introduction section)</t>
+          <t>Conceptual paper. Verbatim Evidence: "In this chapter, we have proposed the concept of the temporal imagination, not as a precisely defined theoretical construct that can be instantly operationalized to begin a program of empirical research, but like its sociological progenitor, as a sensitizing concept (Blumer, 1954)."</t>
         </is>
       </c>
     </row>
@@ -4089,14 +4081,10 @@
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F68" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F68" s="0" t="inlineStr"/>
       <c r="G68" s="0" t="inlineStr">
         <is>
           <t>This research examined the relationships between structural positions and influence at the individual level of analysis. The structure of the organization was conceptualized from a social network perspective. Measures of the relative positions of employees within workflow, communication, and friendship networks were strongly related to perceptions of influence by both supervisors and non-supervisors and to promotions to the supervisory level. Measures included criticality, transaction alternatives, and centrality (access and control) in the networks and in such reference groups as the dominant coalition. A comparison of boundary-spanning and technical-core personnel indicated that contacts beyond the normal work requirements are particularly important for technical core personnel to acquire influence. Overall, the results provide support for a structural perspective on intraorganizational influence.</t>
@@ -4369,14 +4357,10 @@
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F73" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F73" s="0" t="inlineStr"/>
       <c r="G73" s="0" t="inlineStr">
         <is>
           <t>This dissertation examines the extent to which organizational and professional commitment, the technical environment, and the professional environment are related to boundary spanning activity. Surveys of R&amp;D professional employees, their co-workers, and their managers were used to obtain measures of commitment to their organizations and professions, perceptions of the technical and professional environment in which they worked, and the frequency with which they communicated both within and outside of the R&amp;D unit.</t>
@@ -4548,7 +4532,7 @@
       </c>
       <c r="P76" s="0" t="inlineStr">
         <is>
-          <t>Qualitative field interview study without individual employee Pearson correlation matrix. Verbatim Evidence: "Some interviewees were less concerned by this lack of basic training, believing instead that the onshore... For example, in the sample we checked if the cut-off of the invoices was correct." (Abstract / Findings section)</t>
+          <t>Qualitative case study. Verbatim Evidence: "Given that the objective of this study is to develop our understanding of how and why offshoring emerged as an organizational matter, changing the way audit work is organized and perceived in a Big 4 firm, a qualitative research methodology was deemed most appropriate... More specifically, we used a case study approach" (IV. RESEARCH METHOD)</t>
         </is>
       </c>
     </row>
@@ -5878,7 +5862,7 @@
       </c>
       <c r="P103" s="0" t="inlineStr">
         <is>
-          <t>Project/Team-level aggregation study. Verbatim Evidence: "This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates... Note: Dependent variable: (L) Learning rate, N = 47, N = 183 projects." (Abstract / Table 3-4 section)</t>
+          <t>Project level analysis. Verbatim Evidence: "The unit of analysis was the OSS project." (Page 14)</t>
         </is>
       </c>
     </row>
@@ -5928,7 +5912,7 @@
       </c>
       <c r="P104" s="0" t="inlineStr">
         <is>
-          <t>Project/Team-level aggregation study. Verbatim Evidence: "The final sample was reduced to 101 projects since only that number had archived full data on all development activities. For the 101 projects, repeated measures were taken on a quarterly basis since the beginning..." (Methodology / Sample section)</t>
+          <t>Project level analysis. Verbatim Evidence: "The unit of analysis was the NPD project. OSS project information is hosted in web-based repositories which have been used repeatedly as sources of archival data for empirical studies (Mockus et al., 2002)." (Page 10, Sampling section)</t>
         </is>
       </c>
     </row>
@@ -6595,14 +6579,10 @@
       </c>
       <c r="E118" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F118" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F118" s="0" t="inlineStr"/>
       <c r="G118" s="0" t="inlineStr">
         <is>
           <t>The “variance hypothesis” predicts that external search breadth leads to innovation outcomes, but people have limited attention for search and cultivating breadth consumes attention. How does individuals' search breadth affect innovation outcomes? How does individuals' allocation of attention affect the efficacy of search breadth? We matched survey data with complete patent records, to examine the search behaviors of elite boundary spanners at                 IBM                 . Surprisingly, individuals who allocated attention to people inside the firm were more innovative. Individuals with high external search breadth were more innovative only when they allocated more attention to those sources. Our research identifies limits to the “variance hypothesis” and reveals two successful approaches to innovation search: “cosmopolitans” who cultivate and attend to external people and “locals” who draw upon internal people                              . © 2014 The Authors.               Strategic Management Journal               published by John Wiley &amp; Sons Ltd.</t>
@@ -6626,11 +6606,7 @@
       <c r="K118" s="0" t="n">
         <v>2016</v>
       </c>
-      <c r="P118" s="0" t="inlineStr">
-        <is>
-          <t>Qualitative interview / conceptual study without individual employee Pearson correlation matrix. Verbatim Evidence: "We composed a theoretical rather than representative sample of professionals who are boundary spanners and tasked with innovation search who had been granted a great deal of autonomy over their time." (Methodology / Sample section)</t>
-        </is>
-      </c>
+      <c r="P118" s="0" t="inlineStr"/>
     </row>
     <row r="119" ht="18" customHeight="1" s="31">
       <c r="A119" s="0" t="inlineStr">
@@ -6645,14 +6621,10 @@
       </c>
       <c r="E119" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F119" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F119" s="0" t="inlineStr"/>
       <c r="G119" s="0" t="inlineStr">
         <is>
           <t>THErelationships between age, aspects of tenure, locus of control, job involvement, and boundary spanning behaviour (B.S.B.) were examined using path analysis for 281 scientists and engineers. It was found that locus of control and age were significant determinants of job involvement. It was also shown that locus of control and job involvement were significant determinants of B.S.B. These findings are discussed relative to previous research on locus of control, job involvement, and B.S.B. Finally, new research designs are advocated which incorporate task characteristics, role dynamics constructs, and environmental uncertainty as determinants of B.S.B.</t>
@@ -6891,14 +6863,10 @@
       </c>
       <c r="E124" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F124" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F124" s="0" t="inlineStr"/>
       <c r="G124" s="0" t="inlineStr">
         <is>
           <t>Background: Registered nurses play a key role in hospitals, as they have an important impact on the quality of the services delivered. For nurses to perform at their best, they need organizational, leader, and coworker support. To date, few studies have explored the link between nurses_ perceived support, affective organizational commitment, and boundary-spanning behaviors. Methods: This cross-sectional research used a questionnaire survey to explore the hypothesized relationships in a sample of 273 nurses from a hospital in Belgium. Structural equation modeling was used for statistical analysis of the mediation model. Results: One hundred forty-seven (53.5%) nurses responded to the survey. Perceived support from the organization, supervisors, and coworkers positively influences nurses_ boundary-spanning behaviors. Affective organizational commitment was found to mediate the positive relationship between perceived organization support, perceived coworker support, and boundary-spanning behaviors. Perceived supervisor support and boundary-spanning behaviors showed a direct relationship not mediated by affective organizational commitment. Conclusions: Perceived support has an important influence on the boundary-spanning behavior of nurses. This study emphasizes the importance on how support exerts an influence on boundary-spanning behavior and</t>
@@ -7037,14 +7005,10 @@
       </c>
       <c r="E127" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F127" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F127" s="0" t="inlineStr"/>
       <c r="G127" s="0" t="inlineStr">
         <is>
           <t>Data from 409 members of 45 new product teams in five high-technology conpanies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator,Scout, and Guard. These activities are related to the frequency, type, and destination of communications between team members and others. This paper describes these activities and examines the irrpact of individual and environmental variables on the frequency in vAiich individual team members engage in them.</t>
@@ -7069,11 +7033,7 @@
       <c r="K127" s="0" t="n">
         <v>1989</v>
       </c>
-      <c r="P127" s="0" t="inlineStr">
-        <is>
-          <t>Team-level aggregation study of product development teams without individual employee Pearson correlation matrix. Verbatim Evidence: "Data from 409 members of 45 new product teams in five high-technology companies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator, Scout, and Guard." (Abstract section)</t>
-        </is>
-      </c>
+      <c r="P127" s="0" t="inlineStr"/>
     </row>
     <row r="128" ht="18" customHeight="1" s="31">
       <c r="A128" s="0" t="inlineStr">
@@ -7141,14 +7101,10 @@
       </c>
       <c r="E129" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F129" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F129" s="0" t="inlineStr"/>
       <c r="G129" s="0" t="inlineStr">
         <is>
           <t>Leader-Member Exchange theory proposes both the salesperson and manager make contributions to their working relationship. Effective leadership is dependent upon developing a high quality relationship. This study tests the proposals of Leader-Member Exchange by examining the exchange of manager contributions (allowing the salesperson more operating freedom or latitude) and those of the salesperson. While the receipt of managerial latitude has a direct effect on the salesperson's evaluation of the working relationship, the salesperson's contributions also play a part. The manager allows more latitude to salespeople who are seen as more competent and loyal. These exchanges latitude for competency and loyalty) and the quality of the salesperson-manager relationship may be especially important when the sales task requires adaptive selling behaviors.</t>
@@ -7187,14 +7143,10 @@
       </c>
       <c r="E130" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F130" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F130" s="0" t="inlineStr"/>
       <c r="G130" s="0" t="inlineStr">
         <is>
           <t>An information systems (IS) support community represents a knowledge-intensive network where IS professionals interact with end-users to resolve system use problems during the IS post-implementation stage. For IS professionals in the support function, providing support for multiple information systems to multiple business units requires knowledge about different domains (business units or technical systems). In this paper, we take a network perspective to empirically evaluate the effects of an IS worker's network position and knowledge boundary spanning on productivity. Drawing upon theories of experiential learning and knowledge boundary, we perform social network analysis and linear mixed effects modeling to analyze archival data comprising 36 IS workers and 23,450 support requests made by 4568 end-users during the first 13 months post SAP/R3 implementation in a large U.S. organization. Our findings reveal that IS workers' network centrality and boundary spanning positively influence productivity. Surprisingly, their boundary-spanning experience plays a substantially more important role than network centrality. This study makes important contributions to theory and practice in individual experiential learning in knowledge-intensive networks.</t>
@@ -7218,11 +7170,7 @@
       <c r="K130" s="0" t="n">
         <v>2015</v>
       </c>
-      <c r="P130" s="0" t="inlineStr">
-        <is>
-          <t>Ticket/Task-level aggregation study of IT support community. Verbatim Evidence: "Then the ticket complexity scores are aggregated on a monthly basis per worker... Table 1 presents the descriptive statistics and correlations of the variables across 320 monthly aggregated worker ticket observations." (Methodology / Data analysis section)</t>
-        </is>
-      </c>
+      <c r="P130" s="0" t="inlineStr"/>
     </row>
     <row r="131" ht="18" customHeight="1" s="31">
       <c r="A131" s="0" t="inlineStr">
@@ -8469,7 +8417,7 @@
       </c>
       <c r="P155" s="0" t="inlineStr">
         <is>
-          <t>Macro / Firm-level study of supply-side resilience. Verbatim Evidence: "An electronic survey was used where the initial sample consisted of 1,641 manufacturing firms (SIC codes 20–51) listed by Dun and Bradstreet... The focus of research has been at an organisational level without incorporating the role of boundary spanning individuals." (Abstract / Methodology section)</t>
+          <t>Firm level analysis. Verbatim Evidence: "Design/methodology/approach – Survey data are collected from 248 firms and validated using a subset of 57 attentive secondary respondents and archival data." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -8741,7 +8689,7 @@
       </c>
       <c r="F161" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G161" s="0" t="inlineStr">
@@ -8769,7 +8717,7 @@
       </c>
       <c r="P161" s="0" t="inlineStr">
         <is>
-          <t>Macro / Firm-level Market Orientation study. Verbatim Evidence: "Specifically, this research draws on the Job Demands-Resources model to explore the effect of employee perceptions of firm market orientation as a way to reduce role stressors and subsequently turnover intentions... Sample of 260 respondents who were employed full-time and worked in either B2B or B2C sales." (Abstract / Sample section)</t>
+          <t>BSB not measured. Verbatim Evidence: "Specifically, this research draws on the Job Demands-Resources model to explore the effect of employee perceptions of firm market orientation as a way to reduce role stressors and subsequently turnover intentions. It also looks at employee traits that may serve as a buffer to the role stress to turnover intentions link and can be part of the hiring selection process (in this case grit)." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -8819,7 +8767,7 @@
       </c>
       <c r="P162" s="0" t="inlineStr">
         <is>
-          <t>Bibliometric / archival study of Open Source software developers, not organizational employees. Verbatim Evidence: "Tables 1 and 2 describe the 610 subjects who published prior to working group chair appointment or censoring, observed over 5,066 trimesters... Open source operating systems challenge the world's most powerful software firms." (Methodology / Variables section)</t>
+          <t>Non-employee sample. Verbatim Evidence: "We define an open innovation community as a group of unpaid volunteers who work informally, attempt to keep their processes of innovation public and available to any qualified contributor, and seek to distribute their work at no charge. While we induct theory from many open innovation communities, we test our hypotheses with a specific data set culled from the archives of the IETF, with the dependent variable as time to appointment as a working group leader within the IETF." (Open Innovation Communities and the IETF)</t>
         </is>
       </c>
     </row>
@@ -9136,14 +9084,10 @@
       </c>
       <c r="E169" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F169" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F169" s="0" t="inlineStr"/>
       <c r="G169" s="0" t="inlineStr">
         <is>
           <t>Self-initiated expatriates (SIEs) who work for a subsidiary of a multinational enterprise from their country of origin and hence are familiar with both countries’ language and culture can be expected to act as boundary-spanners between the assigned expatriates sent from the parent country and host country nationals, and between the headquarters and the subsidiary. We develop a new model of boundary-spanning that encompasses both individual and organizational antecedents and validate the model using survey data from Japanese-affiliated companies in China. We find that familiarity with Chinese language and culture and the potential dual allegiance of SIEs contribute to enhancing their boundary-spanning behavior. We also find that relationships of trust among the parties concerned (social capital) and global career opportunities for such self-initiated expatriates (geocentric staffing) have positive influences on their dual allegiance. Finally, normative and systems integration of human resource management are associated with increasing levels of social capital and geocentric staffing.</t>
@@ -10066,7 +10010,7 @@
       </c>
       <c r="P187" s="0" t="inlineStr">
         <is>
-          <t>Team/Project-level aggregation study. Verbatim Evidence: "We ran an OLS regression model to test H1 regarding the relationship between external activity and effectiveness... In the second step the overall R-square was .07 (F(4,139)=2.74, p&lt;.05) across 144 documentary film making teams." (Abstract / Table 2 section)</t>
+          <t>Team level analysis. Verbatim Evidence: "Where more than one film maker in a team responded to the survey, we averaged their scale scores to create a single score on each variable (justification for aggregation included below), hence the film making team is the unit of analysis." (Page 18)</t>
         </is>
       </c>
     </row>
@@ -10133,14 +10077,10 @@
       </c>
       <c r="E189" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F189" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F189" s="0" t="inlineStr"/>
       <c r="G189" s="0" t="inlineStr">
         <is>
           <t>Drawing on corporate entrepreneurship (CE) and social network research, this study focuses on strategic renewal as a form of CE and examines the impact of boundary-spanning at top and middle management levels on business units’ exploratory innovation. Analyses of multi-source and multi-level data, collected from 72 top managers (TMs) and 397 middle managers (MMs) operating in 34 units of a multi-national organization, indicate that TMs’ boundary-spanning is positively related to units’ exploratory innovation, but also has a cascading effect on MMs by increasing their perceived role conflict. MMs’ role conflict is negatively related to units’ exploratory innovation and thus offsets some of the benefits gained through TMs’ boundary-spanning activities. Taking a configurational perspective on social exchanges at multiple levels, we show that role conflict is reduced by overlapping boundary-spanning ties among TMs and MMs. Surprisingly, MMs’ boundary-spanning does not relate to exploratory innovation. Our study shows that with regard to boundary-spanning, a top-down approach to CE as strategic renewal may be most effective because TMs play a key role in driving exploratory innovation. However, TMs need to be aware of the cascading social liabilities of their boundary-spanning behavior and ensure MMs develop similar networks. We advance ongoing debates in studies about CE and social networks by providing empirically validated insights into who drives strategic renewal and by uncovering the benefits and costs of social exchanges for strategic renewal. Furthermore, we uncover potential causes of mixed findings in network theory research and highlight a remedy to social liabilities.</t>
@@ -10434,7 +10374,7 @@
       </c>
       <c r="F195" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G195" s="0" t="inlineStr">
@@ -10462,7 +10402,7 @@
       </c>
       <c r="P195" s="0" t="inlineStr">
         <is>
-          <t>Descriptive survey of Link Officers without individual employee Pearson correlation matrix. Verbatim Evidence: "The survey was developed with input from IOs to ensure that survey questions were relevant to LPs and LOs. The survey involved a mixture of open and closed questions... Table 1. Characteristics of Link Officers (LOs) and Link Partners (LPs)." (Methodology / Sample and procedure section)</t>
+          <t>Descriptive stats only. Verbatim Evidence: "Descriptive statistical analyses of the survey data were conducted using the responses to the closed-ended questions. Analysis of continuous measures (e.g., years in current organizational position, FTE dedicated to the LP/LO role) and Likert-type measures involved the calculation of means and standard deviations; percentages were calculated for categorical measures." (Analysis)</t>
         </is>
       </c>
     </row>
@@ -10512,7 +10452,7 @@
       </c>
       <c r="P196" s="0" t="inlineStr">
         <is>
-          <t>Team-level aggregation study. Verbatim Evidence: "The members of 126 multidisciplinary teams responded to a survey on several aspects related to the functioning and leadership of their teams... In this study, 126 CPCY teams participated (654 individuals)." (Abstract / Methodology section)</t>
+          <t>Team level analysis. Verbatim Evidence: "The level of analysis in this study is the team. So, for statistical analyses, individual answers were aggregated at team level." (Results, Aggregation section)</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10874,7 @@
       </c>
       <c r="F205" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G205" s="0" t="inlineStr">
@@ -10962,7 +10902,7 @@
       </c>
       <c r="P205" s="0" t="inlineStr">
         <is>
-          <t>Qualitative study without quantitative employee survey correlation data. Verbatim Evidence: "This exploratory qualitative study used a semi-structured interview protocol with a purposeful sample of 27 Indian American professionals... The perception of innovation and how individuals define innovation..." (Abstract / Research Design section)</t>
+          <t>BSB not measured. Verbatim Evidence: "While innovation may be understood by individuals as a multi-dimensional construct, the research tried to identify the relationship between perceptions, and gender, age and job function for the homogenous group of Indian Americans in the United States. The research followed the approach and methodology used by Caraballo and McLaughlin (2012) and the study is quantitative, exploratory and used web-based surveys to gather responses from respondents." (Abstract)</t>
         </is>
       </c>
     </row>
@@ -10979,14 +10919,10 @@
       </c>
       <c r="E206" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F206" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F206" s="0" t="inlineStr"/>
       <c r="G206" s="0" t="inlineStr">
         <is>
           <t>Personnel is one of the most important resources for the performance of Information Systems (IS) and Information Center (IC) organizations. The scarcity of new employees, the difficulty of training and a high turnover make personnel management in these areas a difficult problem. For IS employees, the relationships between job satisfaction, organizational commitment and intention to leave the organization have been established. Because the size of the investment and the number of organizations establishing IC organizations are growing dramatically, it has become important to understand the determinants of turnover intentions for IC as well as IS employees. Are IC employees similar to their IS counterparts? Or, is their nature basically different, as some studies have suggested? This study examines the differences between IS and IC employees in terms of demographic characteristics, participation on boundary spanning activities, role stressors, overall job satisfaction, organizational commitment and turnover intentions. The differences are found to be significant and call for special attention from IC managers to manage more properly their personnel resources. IC employees were found to participate more extensively in boundary spanning activities, experienced more role stressors (role ambiguity and role conflict), were less satisfied with their jobs and less committed to their organization. The findings also demonstrate the importance of organizational commitment as an intervening variable in models of turnover. While overall job satisfaction had both direct and indirect effects on turnover intentions among IC employees, for IS personnel it had only indirect effects through organizational commitment. The effects of role stressors and boundary spanning activities were found to be indirect via overall job satisfaction and organizational commitment for both IC and IS employees. The implications of these findings for practicing managers and for future research are discussed.</t>
@@ -11158,7 +11094,7 @@
       </c>
       <c r="P209" s="0" t="inlineStr">
         <is>
-          <t>Macro / Firm-level study of Turkish software firms. Verbatim Evidence: "A number of studies have shown that transformational leadership positively influences organizational innovation. However, there is a lack of studies examining... sample of 110 manufacturing firms in China... turkish software development firms." (Abstract / Sample section)</t>
+          <t>Firm level analysis. Verbatim Evidence: "Since the dependent variable of this part of the analysis is organizational innovation, transformational leadership ratings as well as perceptions of internal support for innovation by the subordinates needed to be aggregated to organizational level." (Methodology, Page 7)</t>
         </is>
       </c>
     </row>
@@ -11298,7 +11234,7 @@
       </c>
       <c r="P212" s="0" t="inlineStr">
         <is>
-          <t>Team/Project-level aggregation study. Verbatim Evidence: "Analyses of multi-source data from a sample of 96 project teams in a prominent international development agency show that... N = 96 teams." (Abstract / Data analysis section)</t>
+          <t>Team level aggregation. Verbatim Evidence: "The responses to all eight questions were averaged across all the members of each team to create an aggregate measure of the amount of external knowledge gathered" (Section: Knowledge Gathering, p. 1176)</t>
         </is>
       </c>
     </row>
@@ -11365,14 +11301,10 @@
       </c>
       <c r="E214" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F214" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F214" s="0" t="inlineStr"/>
       <c r="G214" s="0" t="inlineStr">
         <is>
           <t>SUMMARY             Previous research has focused on purchasing managers’ experience with role stressors and the negative effect of stress on job attitudes and performance. The potential benefits of having multiple responsibilities and a diverse role set have been overlooked. This study explored the relationship between purchasing managers’ involvement in multiple boundary spanning roles and their perceptions of positive social outcomes related to work. The relationship of these social benefits to job satisfaction was also evaluated. The relationships were analyzed using structural equation modeling. The results indicated positive relationships between each variable in the model. The implications for recruitment, supervision, and job design are discussed.</t>
@@ -12094,7 +12026,7 @@
       </c>
       <c r="P228" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of online gig-economy freelancers on Upwork platform, not internal organizational workplace employees. Verbatim Evidence: "Extant management literature suggests that boundary spanning, defined as... sample of skilled digital freelancers using the Upwork platform, an online marketplace for connecting freelancers and employers." (Abstract / Sample section)</t>
+          <t>Freelancers. Verbatim Evidence: "Data for the study consists of pre-piloted survey measures and secondary data gathered on a sample of skilled digital freelancers using the Upwork platform, an online marketplace for connecting freelancers and employers."</t>
         </is>
       </c>
     </row>
@@ -12216,7 +12148,7 @@
       </c>
       <c r="F231" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G231" s="0" t="inlineStr">
@@ -12244,7 +12176,7 @@
       </c>
       <c r="P231" s="0" t="inlineStr">
         <is>
-          <t>Study of external public affairs consulting agencies/consultants without an individual employee Pearson correlation matrix. Verbatim Evidence: "Even though consultants are undoubtedly increasing in importance, their relevance as agents is often downplayed. This study seeks to empirically supplement the perspective of the consultant... All respondents, as well as an additional 87 experts in politics, associations, and corporations were asked to name the most relevant public affairs consultants in Switzerland." (Abstract / Methodology section)</t>
+          <t>Agency level analysis. Verbatim Evidence: "The questionnaire addressed the highest-ranking person in charge of public affairs, or the CEO of the agency. 337 of 641 agencies responded to the questionnaire (53 percent); 236 agencies stated that they do not offer any public affairs services on a regular basis. Once these had been sorted out, 101 respondents formed the sample that was analyzed." (Method)</t>
         </is>
       </c>
     </row>
@@ -12394,7 +12326,7 @@
       </c>
       <c r="P234" s="0" t="inlineStr">
         <is>
-          <t>Department/Hospital-level organizational study without individual employee Pearson correlation matrix. Verbatim Evidence: "From approximately 750 general hospitals in the 1969 Inventory of Psychiatric Services of the National Institute of Mental Health... 338 inpatient departments were used in the present analysis... Table 2: Correlation Analysis: Size and Performance of Department by Hospital Ownership (N = 47, N = 43, N = 76, N = 172 departments)." (Methodology / Table 2 section)</t>
+          <t>Department level analysis. Verbatim Evidence: "In this study of 338 inpatient psychiatric departments five hypotheses concerning organizational performance and size are tested and supported."</t>
         </is>
       </c>
     </row>
@@ -12511,14 +12443,10 @@
       </c>
       <c r="E237" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F237" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F237" s="0" t="inlineStr"/>
       <c r="G237" s="0" t="inlineStr">
         <is>
           <t>There appears to be a consensus that organizational integration across functional and disciplinary specialties drives superior ﬁrm capabilities. The basic assumption is that new practices and concepts emerge from the interaction of individuals engaged in different functional departments. However, communication across functional boundaries is often difﬁcult. As such, Tushman &amp; Scanlan suggested that functional boundaries can be spanned effectively only by boundary spanners who understand the coding schemes that are attuned to the contextual information on both sides of the boundary. The study of boundary spanners has signiﬁcant performance implications to ﬁrms. Compared to its importance, theoretical development and empirical inquiries into this phenomenon are relatively scant. Thus, this study explores the factors that determine who becomes a boundary spanner and examines boundary spanners’ performance implications. A Taiwanese company provided the context for our study. Partial Least Squares (PLS) was used to test the theoretical model. The results imply that a company needs to have an appropriate mixture of boundary spanners and non-boundary spanners, because boundary spanners have higher innovative performance.</t>
@@ -13102,14 +13030,10 @@
       </c>
       <c r="E249" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F249" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F249" s="0" t="inlineStr"/>
       <c r="G249" s="0" t="inlineStr">
         <is>
           <t>The study examines the effects of the individual characteristics, job type, role stressors, boundary spanning activities, career outcomes, and job characteristics on the turnover propensity of 464 information systems personnel. Results show that age, organizational level, organizational tenure, job tenure, and number of years in the computer field are negatively correlated with the intention to leave the organization. Education was found to be positively correlated with turnover intentions, and while project leaders are more likely to leave the organization, IS managers are less likely. Results also show that both role stressors (role ambiguity and role conflict) and boundary spanning activities are positively correlated with turnover intentions, and that job involvement, career plateau, promotability, salary, organizational commitment, job satisfaction, satisfaction with progress, promotion, pay, status, and projects are negatively correlated while career opportunity is positively correlated with turnover intentions. Finally, all job characteristics are negatively correlated with turnover intentions. Implications of the results for practice and research are offered.</t>
@@ -13248,14 +13172,10 @@
       </c>
       <c r="E252" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F252" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F252" s="0" t="inlineStr"/>
       <c r="G252" s="0" t="inlineStr">
         <is>
           <t>Due to the increasing array of sales technology, salespeople must understand how each application assists them. This study examines how business-to-business salespeople use different forms of sales technology to meet their boundary-spanning roles. Our research draws from social exchange theory and task-technology fit theory to test a model that examines how salespeople use CRM and social media technologies differentially to support competitive information collection, product information communication, and buyer information sharing. Dyadic data from industrial buyers and sellers is used to analyze the technology-behavior relationships. Our study's results reveal social media use and CRM technology both positively influence buyer-seller information exchanges; however, each technology takes a distinct route to enable the information exchange between the buyer and the seller. The results also suggest that managers need to champion the use of both technology applications to their salesforce.</t>
@@ -13677,7 +13597,7 @@
       </c>
       <c r="P260" s="0" t="inlineStr">
         <is>
-          <t>Patent-level technological domain recombination study where the unit of analysis is the patent, not individual employees. Verbatim Evidence: "Prior literature has long examined innovation as a recombination process within or across the boundaries of technological domains... Analyzing a large sample of US patents, we find that spanning crisp boundaries is more likely to generate impactful inventions." (Abstract / Methodology section)</t>
+          <t>Patent level analysis. Verbatim Evidence: "We test our hypotheses by analyzing all of US patents between 2001 and 2010." (3. Empirics)</t>
         </is>
       </c>
     </row>
@@ -13794,14 +13714,10 @@
       </c>
       <c r="E263" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F263" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F263" s="0" t="inlineStr"/>
       <c r="G263" s="0" t="inlineStr">
         <is>
           <t>The impact of perceived environmental demands on the roles and job satisfaction of the school psychologist in rural school systems was explored. Superintendents rated their perceptions of the community context and the psychologist’s involvement in interagency linking functions. School psychologists rated their performance of boundary-spanning functions and their job perceptions. Results indicated that certain perceived environmental pressures are related to the performance of boundaryspanning activities. Those who performed boundary-spanning functions are more satisfied with their jobs and more influential in determining their roles.</t>
@@ -13890,14 +13806,10 @@
       </c>
       <c r="E265" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F265" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F265" s="0" t="inlineStr"/>
       <c r="G265" s="0" t="inlineStr">
         <is>
           <t>International joint ventures (IJVs) have become an important source of critical knowledge for multinational enterprises, but little is known about how knowledge can be effectively transferred to parent ﬁrms when the potential for interpartner opportunism still exists. Drawing on attachment theory, we study how boundary-spanning commitments to IJVs may help mitigate interpartner opportunism and facilitate effective knowledge transfer to parents. Speciﬁcally, we argue that knowledge transfer from IJVs to their parents is positively mediated by both boundary spanners’ organizational commitment to IJVs and parent ﬁrms’ resource commitment to IJVs. We test our arguments using survey data collected from 600 dyadic Chinese–foreign managers of 100 IJVs established in China. The results provide evidence that knowledge sharing between boundary spanners in IJVs positively affects their organizational commitment to these IJVs, which in turn positively affects knowledge transfer to parents. Similarly, knowledge sharing between such boundary spanners positively affects parent ﬁrms’ resource commitment to IJVs, which in turn positively affects knowledge transfer to parents. The mediating role of boundary spanners’ organizational commitment is stronger than that of parent ﬁrms’ resource commitment. Collectively, our ﬁndings suggest that commitment-based relational mechanisms are imperative for safeguarding effective knowledge transfer from IJVs to parent ﬁrms.</t>
@@ -14019,7 +13931,7 @@
       </c>
       <c r="P267" s="0" t="inlineStr">
         <is>
-          <t>Firm-level study of corporate R&amp;D network boundary spanning and innovation performance where the unit of analysis is the corporation. Verbatim Evidence: "DOES STRONGER R&amp;D CAPABILITY ALWAYS PROMOTE BETTER INNOVATION? THE MODERATING ROLE OF KNOWLEDGE BOUNDARY SPANNING OF R&amp;D NETWORK... We collected application documents, excluded samples with incomplete data, and ultimately, obtained data of 702 corporations." (Title / Sample section)</t>
+          <t>Firm level analysis. Verbatim Evidence: "To test our hypotheses, we examined corporations from the Hunan province applying for high-tech enterprises qualification in China. We collected application documents, excluded samples with incomplete data, and ultimately, obtained data of 702 corporations." (Sampling and data collection)</t>
         </is>
       </c>
     </row>
@@ -14326,14 +14238,10 @@
       </c>
       <c r="E274" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F274" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F274" s="0" t="inlineStr"/>
       <c r="G274" s="0" t="inlineStr">
         <is>
           <t>National Sun Yat-sen University, Kaohsiung, Taiwan This research report compares three differing explanations of the dynamic interrelationships between internal and external innovation-related communication in a new organizational form. In the functional specialization explanation, individuals are said to focus on the mix of internal and/or external communication dictated by their formal positions. The communication stars explanation suggests that individuals maintain similar levels of communication in both networks. The cyclical model posits a more dynamic pattern that shifts back and forth between internal and external communication, depending on the consequences of their prior communication behavior. The new organizational form examined for three years was the Cancer Information Service, a geographically dispersed federal government health information program. Our results indicated that there was a lagged effect for the communication stars explanation.</t>
@@ -14622,14 +14530,10 @@
       </c>
       <c r="E280" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F280" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F280" s="0" t="inlineStr"/>
       <c r="G280" s="0" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to evaluate the recognition of sexual harassment (SH); to describe the relationships among SH, employees’ burnout, customer-oriented boundary-spanning behaviors (COBSB); and to verify the moderating effect of employees’ psychological safety (PS), all within deluxe hotels in South Korea.</t>
@@ -14931,14 +14835,10 @@
       </c>
       <c r="E286" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F286" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F286" s="0" t="inlineStr"/>
       <c r="G286" s="0" t="inlineStr">
         <is>
           <t>Purpose – Despite the increasing importance of boundary-spanning behaviors in construction projects, the research on how leader anger expressions impact employees’ boundary-spanning behaviors remains unclear. This study aims to investigate the impact of leader anger expressions on employees’ boundaryspanning behaviors in construction projects while exploring the mediating effect of work hope and the moderating effect of power distance orientation through the lens of social information processing theory. Design/methodology/approach – The empirical data were collected from a questionnaire survey of 235 employees in construction projects, and the hypotheses were tested using the PROCESS program developed by Hayes.</t>
@@ -15210,7 +15110,7 @@
       </c>
       <c r="P291" s="0" t="inlineStr">
         <is>
-          <t>Project-level statistical aggregation study where the unit of analysis is the R&amp;D project group, not individual employees. Verbatim Evidence: "An investigation into the managerial roles and career paths of gatekeepers and project supervisors in a major R &amp; D facility... In particular, within our sample of development projects, those with gatekeepers were considerably more effective than those without gatekeepers... Table 1. Project performance as a function of gatekeeper presence and project type." (Abstract / Table 1 section)</t>
+          <t>Project level aggregation. Verbatim Evidence: "As discussed by Katz &amp; Tushman (1979), these individual scores were also aggregated to obtain project measures of internal and external communication." (Communication section)</t>
         </is>
       </c>
     </row>
@@ -15260,7 +15160,7 @@
       </c>
       <c r="P292" s="0" t="inlineStr">
         <is>
-          <t>Project-level statistical aggregation study where individual communication measures are aggregated to the project unit of analysis (N = 61 projects). Verbatim Evidence: "Communication patterns, project performance and task characteristics: an empirical evaluation and integration in an R&amp;D setting... At the time of this study, 61 such projects existed across the laboratory's seven divisions... Intraproject communication: An examination of the intraproject means and correlation of Table 3... positively associated with performance only for research projects." (Methodology / Results section)</t>
+          <t>Project level analysis. Verbatim Evidence: "This study examines the impacts of problem-solving and administra tive communication patterns on the technical performance of 61 projects in an industrial R&amp;D laboratory."</t>
         </is>
       </c>
     </row>
@@ -15441,14 +15341,10 @@
       </c>
       <c r="E296" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F296" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F296" s="0" t="inlineStr"/>
       <c r="G296" s="0" t="inlineStr">
         <is>
           <t>The article reports on the importance of boundary-spanning roles (BSA), which serve to link organizations confirmed by research. They are vital to the effective monitoring of the environment as well as the transfer of technology and information across boundaries. Research has shown boundary-spanning activity (BSA) to have negative effects for their incumbents, such as higher rates of marginality. Marginality is defined as one's self-orientation when presented with two or more groups with conflicting value systems. Boundary spanning activity could be positively related to levels of role conflict and ambiguity or negatively related to levels of job satisfaction. Research is conducted to test to the theory of role dynamics in BSA.</t>
@@ -15520,7 +15416,7 @@
       </c>
       <c r="P297" s="0" t="inlineStr">
         <is>
-          <t>Qualitative inductive grounded theory ethnographic field study without an individual employee Pearson correlation matrix. Verbatim Evidence: "Life in the Trading Zone: Structuring Coordination Across Boundaries in Postbureaucratic Organizations... Our research study was inductive and focused on generating theoretical insights from an in-depth examination of cross-boundary coordination in practice... analyzed them qualitatively through an iterative process of data examination, grounded coding." (Abstract / Methods section)</t>
+          <t>Qualitative case study. Verbatim Evidence: "Following an emergent strategy, we collected data from multi ple sources in one research site, and then analyzed them qualitatively through an iterative process of data examination, grounded coding, and comparison with existing frameworks." (Research Site and Methods)</t>
         </is>
       </c>
     </row>
@@ -16169,7 +16065,7 @@
       </c>
       <c r="P310" s="0" t="inlineStr">
         <is>
-          <t>Qualitative multiple case study using interviews and ethnographic observation without individual employee Pearson correlation matrix. Verbatim Evidence: "The data for our studies came from two separate cases... In both cases, the data was collected in two sets... Table 1: Summary of the two data sets... Number and categories of actors interviewed: 20 software engineers, 2 e-business managers and 8 sales engineers... the system administrator who acted as a broker." (Methodology / Table 1 section)</t>
+          <t>Qualitative case study. Verbatim Evidence: "The data for our studies came from two separate cases. The first was a group of IT professionals from different companies in a French science park who collaborated to build a Content Management System; the second was a series of innovations produced by a pluridisciplinary network of heath care professionals in a medium-sized French city. [...] All of the actors involved were interviewed several times at different points in the process; the interviews lasted from 30 to 90 min."</t>
         </is>
       </c>
     </row>
@@ -16519,7 +16415,7 @@
       </c>
       <c r="P317" s="0" t="inlineStr">
         <is>
-          <t>Team-level statistical aggregation study of pre-founding entrepreneurial teams where the unit of analysis is the team. Verbatim Evidence: "The Performance of Pre-Founding Entrepreneurial Teams: The Importance of Learning and Leadership... We studied teams who participated in a venture creation programme that combines education and incubation... Sample of 58 teams, 55 teams, 35 teams across conditions." (Title / Methods section)</t>
+          <t>Team level aggregation. Verbatim Evidence: "Descriptives and Intercorrelations of Study Variables on the Team Level" (Table 1) and "The final sample included 196 participants in 58 teams of three to five members" (Methodology).</t>
         </is>
       </c>
     </row>
@@ -16669,7 +16565,7 @@
       </c>
       <c r="P320" s="0" t="inlineStr">
         <is>
-          <t>Team-level study of engineering design teams where the unit of analysis is the team (N = 39 teams). Individual questionnaire data is aggregated to team level for analysis. Verbatim Evidence: "The social structure of leadership and creativity in engineering design teams... Based on a sample of 39 engineering design teams in the space industry, this study examines the effects of leader position within different flows of communication on team creativity." (Abstract / Sample section)</t>
+          <t>Team level aggregation. Verbatim Evidence: "We therefore will limit ourselves to incorporating team-level aggregates into our analysis. In order to justify this aggregation statistically, a one-way analysis of variance was conducted to determine if there was greater variability in team creativity ratings between teams than within teams."</t>
         </is>
       </c>
     </row>
@@ -16969,7 +16865,7 @@
       </c>
       <c r="P326" s="0" t="inlineStr">
         <is>
-          <t>Firm/business-unit-level study of knowledge stocks and information flows where the unit of analysis is the firm. Verbatim Evidence: "Knowledge Stocks and Information Flows in New Product Development... A sample of 500 business units from the food processing industry was randomly selected from a business directory, which contains a complete list of food companies... sample of 340 firms, 136 returned the questionnaire." (Title / Methodology section)</t>
+          <t>Project/business unit level analysis. Verbatim Evidence: "The questionnaire asked participants to focus on a product development project for which their business unit was responsible over the last twelve months."</t>
         </is>
       </c>
     </row>
@@ -16991,7 +16887,7 @@
       </c>
       <c r="F327" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G327" s="0" t="inlineStr">
@@ -17019,7 +16915,7 @@
       </c>
       <c r="P327" s="0" t="inlineStr">
         <is>
-          <t>Volunteer association groups on Meetup.com where the unit of analysis is the online group (N = 171 groups), not individual organizational employees. Verbatim Evidence: "Volunteer associations in the Internet age: Ecological approach to understanding collective action... An online survey was conducted with 171 randomly sampled groups on Meetup.com—a website that facilitates the creation and coordination of mixed-mode groups." (Abstract / Sample section)</t>
+          <t>Group level analysis, voluntary groups. Verbatim Evidence: "Third, due to resource and time constraints, this study could only collect data at the group level, so group organizers were the ones providing responses" (Limitations and conclusion)</t>
         </is>
       </c>
     </row>
@@ -17069,7 +16965,7 @@
       </c>
       <c r="P328" s="0" t="inlineStr">
         <is>
-          <t>Student sample enrolled in a full-time MBA program assigned to self-managing teams as part of coursework, not organizational employees. Verbatim Evidence: "Leadership Over-Emergence in Self-Managing Teams: The Role of Gender and Countervailing Biases... 181 students enrolled in a full time Master of Business Administration (MBA) program at a large research university in the United States. Students were assigned to 5-person self-managing teams." (Sample section)</t>
+          <t>MBA Students. Verbatim Evidence: "The sample for this study consisted of 181 students enrolled in a full time Master’s of Business Administration (MBA) program at a large research university in the United States." (Methods - Participants section)</t>
         </is>
       </c>
     </row>
@@ -17169,7 +17065,7 @@
       </c>
       <c r="P330" s="0" t="inlineStr">
         <is>
-          <t>Online crowd-based innovation challenge evaluators assessing NASA Astrobee solutions, not individual organizational employees performing boundary spanning roles. Verbatim Evidence: "Beyond feasibility filters: How expertise heterogeneity enables innovation recognition... a field experiment with National Aeronautics and Space Administration's (NASA) Astrobee Robotic Arm Challenge, involving 354 evaluators assessing 101 solutions." (Abstract / Methods section)</t>
+          <t>Crowdsourced evaluators via Freelancer.com. Verbatim Evidence: "From May to July 2021, we recruited evaluators through a dedicated contest website on Freelancer.com."</t>
         </is>
       </c>
     </row>
@@ -17219,7 +17115,7 @@
       </c>
       <c r="P331" s="0" t="inlineStr">
         <is>
-          <t>Organization-level study of nonprofit human service organizations where the unit of analysis is the organization (N = 291 organizations). Verbatim Evidence: "Developmental Culture and Effectiveness in Nonprofit Organizations... A total of 778 organizations were surveyed, and the overall project had a response rate of 37% (n = 291). Organizations were sampled primarily from the NTEE codes representing center-based human services." (Sample section)</t>
+          <t>Firm level analysis. Verbatim Evidence: "A total of 364 executive directors/CEOs of nonprofit organizations having a primary mission of mental health, housing, economic development and family planning, senior services, and human services were administered the culture module."</t>
         </is>
       </c>
     </row>
@@ -17469,7 +17365,7 @@
       </c>
       <c r="P336" s="0" t="inlineStr">
         <is>
-          <t>Team-level statistical aggregation study where individual responses are aggregated to the team unit of analysis using ICC and rwg. Verbatim Evidence: "Setting a knowledge boundary across teams: knowledge protection regulation for inter-team coordination and team performance... we checked the legitimacy of our sample for team-level analysis using inter-rater agreement (rwg) and ICC... The values exceeded 0.7 for both rwg and ICC for all constructs, thereby satisfying the requirement for the aggregation of individual-level responses to the team level." (Methodology section)</t>
+          <t>Team level analysis. Verbatim Evidence: "A team as the unit of analysis in this study is the smallest formal structure of each company and differs by well-defined tasks, such as inspection, technology planning, database management and customer support. The individual responses were aggregated into team-level variables with validity." (Data collection)</t>
         </is>
       </c>
     </row>
@@ -17536,14 +17432,10 @@
       </c>
       <c r="E338" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F338" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F338" s="0" t="inlineStr"/>
       <c r="G338" s="0" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the effects of relationship bonds on the psychological response and behavior of bank employees based on the job demands–resources theory. Specifically, it examines the effects of relationship bonds in terms of person–job (P–J) fit, emotional exhaustion, job satisfaction and boundary-spanning behaviors, all of which comprise the behavioral dimensions of bank employees. In addition, the study examines how the resiliency of bank employees influences their emotional exhaustion and determines whether a moderating effect related to emotional exhaustion exists.</t>
@@ -17582,14 +17474,10 @@
       </c>
       <c r="E339" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F339" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F339" s="0" t="inlineStr"/>
       <c r="G339" s="0" t="inlineStr">
         <is>
           <t>Purpose – This study investigated the influence of ambiguous customer expectations and customer demandingness, which reflect hindrance and challenge demands, on the boundary spanning behaviors (BSBs) of frontline bank employees (FBEs) through person-job fit and work engagement. It also examined the moderating effect of customer stewardship between job demands and work engagement.</t>
@@ -17661,7 +17549,7 @@
       </c>
       <c r="P340" s="0" t="inlineStr">
         <is>
-          <t>Firm-level study of IS development teams in consultant-partnered projects where the unit of analysis is the firm/project. Verbatim Evidence: "Boundary Spanning Role of the IS Development Team in Consultant-Partnered Projects... In total, 109 firms had sales larger than $100M and 97 firms employed more than 300 people... The frequency distribution of sales revenue and the number of employees are relatively even throughout the categories." (Sample / Table 3 section)</t>
+          <t>Team/company level analysis. Verbatim Evidence: "Here, we would like to note that, although the survey was answered by individuals, responses to the variables of team competence, partnership quality, and knowledge transfer were grounded on the respondent’s view of team-level characteristics." (Section 5.2 Data Gathering, Page 12)</t>
         </is>
       </c>
     </row>
@@ -17678,14 +17566,10 @@
       </c>
       <c r="E341" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F341" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F341" s="0" t="inlineStr"/>
       <c r="G341" s="0" t="inlineStr">
         <is>
           <t>As business environments become even more competitive, project teams are required to make an effort to operate external linkages from within an organization or across organizational boundaries. Nevertheless, some members boundary-span less extensively, isolating themselves and their project teams from external environments. Our study examines why some members boundary-span more or less through the framework of group attachment theory. Data from 521 project-team members in construction and engineering industries revealed that the more individuals worry about their project team’s acceptance (group attachment anxiety), the more likely they are to perceive intergroup competition, and thus put more efforts into operating external linkages and resources to help their own teams outperform competitors. In contrast, a tendency to distrust their project teams (group attachment avoidance) generates members’ negative construal of their team’s external image, and thus fewer efforts are made at operating external linkages. Thus, project leaders and members with high group-attachment-anxiety may be best qualified for external tasks.</t>
@@ -17724,14 +17608,10 @@
       </c>
       <c r="E342" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F342" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F342" s="0" t="inlineStr"/>
       <c r="G342" s="0" t="inlineStr">
         <is>
           <t>Improving performance often requires creative ideas in extreme work settings like health care. Frontline workers are promising sources of creative ideas. The authors assert that their job dissatisfaction is positively associated with creativity in health care settings because negative emotion spurs creativity when tied to engaging work and that characteristics such as shorter tenure, greater role centrality, and high boundary spanning can strengthen this relationship. The authors find supporting evidence in data on ideas generated over 18 months by health professionals in 12 clinics.</t>
@@ -17853,7 +17733,7 @@
       </c>
       <c r="P344" s="0" t="inlineStr">
         <is>
-          <t>Conceptual paper on firm internationalization using descriptive case illustration of German family firms without individual employee Pearson correlation data. Verbatim Evidence: "Boundary-spanning and boundary-buffering in global markets: A German perspective on the internationalization of family firms... Conceptual paper... The case of Germany, with its large stock of internationalized family firms, shows how boundary-buffering vis-a-vis global capital markets can be compatible with successful and sustained internationalization." (Abstract / Methodology section)</t>
+          <t>Qualitative case study/conceptual. Verbatim Evidence: "As in most qualitative research, we conducted a thorough review of published sources in both German and English, including periodical reports, press releases and research papers published in academic journals or in series of working papers. In addition, we conducted open-ended interviews with several experts on family firms" (Methodology, Page 7)</t>
         </is>
       </c>
     </row>
@@ -18543,7 +18423,7 @@
       </c>
       <c r="P358" s="0" t="inlineStr">
         <is>
-          <t>Firm-level study of new technology ventures where the unit of analysis is the venture/firm (N = 750 new ventures). Verbatim Evidence: "The Effect of Boundary-Spanning Search on Breakthrough Innovations of New Technology Ventures... The sampling frame of this study consisted of new technology ventures located in Shenzhen... We drew on a random sample of 750 new ventures (i.e., 8 years or younger)." (Title / Sample section)</t>
+          <t>Firm level analysis. Verbatim Evidence: "The sampling frame of this study consisted of new technology ventures located in Shenzhen, the most developed high-technology industrial zone in China. We drew on a random sample of 750 new ventures (i.e., 8 years or younger) from a mailing list of electronics firms in this high-technology zone." (3.1 Sample and Data Collection)</t>
         </is>
       </c>
     </row>
@@ -18660,14 +18540,10 @@
       </c>
       <c r="E361" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F361" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F361" s="0" t="inlineStr"/>
       <c r="G361" s="0" t="inlineStr">
         <is>
           <t>Currently boundary spanning behavior is a hot topic in team research field, which involves phenomena at two levels (team level and individual level). Compared to team level, employee's boundary spanning has not been well discussed yet. In addition, few studies have systematically explored its outcomes and impact mechanism in Chinese context. This study aimed to address the above gaps by examining whether, when and how employee's boundary spanning behavior impacted his or her task performance. Specifically, integrating culture and social network theory into boundary spanning field, this study theorized that boundary spanning behavior led to centrality of the employee's social network, and in turn enhance his or her task behavior. At the same time, team's collectivism climate moderated the above path. The participants were recruited from 17 companies in two high-tech parks located in Beijing and Tianjin, China. We invited 135 team leaders and their subordinates to participate the survey, after collecting 2 wave longitudinal data sets and dropping out invalid questionnaires, responses from 61 team leaders and 292 team members were valid finally. To get enough whole network data, we purposely chose teams with small size. All measurements were (or adapted from) well-established scales. Employee's boundary spanning behavior, centrality, and collectivism were collected at time 1, and after 8 weeks, employees' task performance was collected at time 2. Confirmatory factor analyses showed satisfactory model fit indices. Inter-rated agreement (Rwg) and intra-class correlation (ICC) value justified the aggregation of team collectivism climate. HLM were applied to test our hypotheses since this is a cross-level research. Variables like age, education, gender, tenure and collectivism orientation at individual level, and team size at group level were controlled for. The results showed that centrality of the social network positively mediated the relation between employees' boundary spanning behavior and his or her task performance. The climate of team collectivism positively moderated the relation between employees' boundary spanning behavior and network centrality. In addition, network centrality mediated the interaction between boundary spanning behavior and team collectivism climate on employee's task performance such that the relation between boundary spanning behavior and task performance via network centrality will be stronger for teams higher on collectivism climate than for those lower on collectivism. This study revealed that employee's boundary spanning behavior had positive influence on task performance and confirmed the mechanism between the two constructs. Interestingly, we found collectivism at individual level and at team level had different effects for the effect of boundary spanning behavior, which revealed that in transformational Chinese context, cultural elements at micro levels were worthy of discussing. The finding of mediating mechanism of centrality established a logic chain of" external relationship—internal embeddedness—performance", helping in explaining the formation of performance and social network in teams. Managerial implications, limitations and future directions were discussed at the end.</t>
@@ -18691,11 +18567,7 @@
       <c r="K361" s="0" t="n">
         <v>2014</v>
       </c>
-      <c r="P361" s="0" t="inlineStr">
-        <is>
-          <t>Team-level statistical aggregation study where individual responses are aggregated to the team unit using ICC and rwg, analyzed with HLM multilevel models. Verbatim Evidence: "A Longitudinal Study on the Impact Mechanism of Employees' Boundary Spanning Behavior... ICC(1) and ICC(2) were 0.11 and 0.88 respectively, indicating that all variables met the aggregation criteria and can be used for team-level analysis." (Methodology / Table 1 section)</t>
-        </is>
-      </c>
+      <c r="P361" s="0" t="inlineStr"/>
     </row>
     <row r="362" ht="18" customHeight="1" s="31">
       <c r="A362" s="0" t="inlineStr">
@@ -18793,7 +18665,7 @@
       </c>
       <c r="P363" s="0" t="inlineStr">
         <is>
-          <t>PDF contains Javadi Khasraghi et al. (2023) crowdsourcing contest study where the unit of analysis is the team (N = 9,793 teams in 246 contests). Verbatim Evidence: "Submitting tentative solutions for platform feedback in crowdsourcing contests: breaking network closure with boundary spanning for team performance... The final sample comprises 9,793 teams participating in 246 contests. The unit of analysis is submission." (Title / Sample section)</t>
+          <t>Kaggle contest teams, crowdsourcing. Verbatim Evidence: "The final sample comprises 9,793 teams participating in 246 contests. The unit of analysis is submission, and each record is a tentative or final solution submitted by a team for a contest."</t>
         </is>
       </c>
     </row>
@@ -18843,7 +18715,7 @@
       </c>
       <c r="P364" s="0" t="inlineStr">
         <is>
-          <t>General social networking service (SNS) users study, not organizational employees. Verbatim Evidence: "Investigating the lurking mechanism of SNS users: a comprehensive examination of context-specific cues and role stresses... Social networking services (SNS) empower users with a robust capability to connect with others and manage their social relationships... This study delves into the mechanism of this technology-induced decision-making process among SNS users." (Abstract section)</t>
+          <t>WeChat users. Verbatim Evidence: "Survey data were collected from 491 Chinese WeChat Moment users."</t>
         </is>
       </c>
     </row>
@@ -18865,7 +18737,7 @@
       </c>
       <c r="F365" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G365" s="0" t="inlineStr">
@@ -18893,7 +18765,7 @@
       </c>
       <c r="P365" s="0" t="inlineStr">
         <is>
-          <t>Patent-level nanotechnology knowledge diffusion study where the unit of analysis is the patent/inventor citation network, not individual organizational employees. Verbatim Evidence: "Determining inventor status and its effect on knowledge diffusion: A study on nanotechnology literature from China, Russia, and India... 561 individuals... n = 152 patents." (Title / Sample section)</t>
+          <t>Bibliometric data/SCI database. Verbatim Evidence: "We selected Thomson Reuters’ Science Citation Index (SCI) as our database because it provides broad coverage of journals in more than 150 disciplines, which can be used to extract coauthorship networks and citation information." (Data Acquisition and Research Testbed)</t>
         </is>
       </c>
     </row>
@@ -19793,7 +19665,7 @@
       </c>
       <c r="P383" s="0" t="inlineStr">
         <is>
-          <t>Interorganizational strategic alliance study where the unit of analysis is the alliance (N = 440 strategic alliances). Verbatim Evidence: "The Independent and Interactive Roles of Procedural, Distributive, and Interactional Justice in Strategic Alliances... a sample of 440 strategic alliances... to avoid a single-party bias toward perceived justice, this study defines and measures justice from both alliance partners' perspectives." (Abstract / Sample section)</t>
+          <t>Strategic alliances. Verbatim Evidence: "The 127 alliances for which both a local CEO and a foreign parent counterpart responded therefore served as the study’s final sample." (Data Collection)</t>
         </is>
       </c>
     </row>
@@ -19910,14 +19782,10 @@
       </c>
       <c r="E386" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F386" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F386" s="0" t="inlineStr"/>
       <c r="G386" s="0" t="inlineStr">
         <is>
           <t>Boundary spanning theory and role theory are used to examine the product manager's role in consumer industries. A research model depicting associations between environmental uncertainty, boundary spanning, role conflict and ambiguity, job satisfaction, tension and performance, and moderating variables is developed and tested with bivariate correlations, path analysis, and ANOVA. Implications of the results are given.</t>
@@ -19956,14 +19824,10 @@
       </c>
       <c r="E387" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F387" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F387" s="0" t="inlineStr"/>
       <c r="G387" s="0" t="inlineStr">
         <is>
           <t>Evidence suggests that product managers' need to communicate across organizational and environmental boundaries under conditions of uncertainty can give rise to powerful role pressures of conflict and ambiguity. These pressures are generally associated with negative or dysfunctional personal outcomes such as job‐related tension, dissatisfaction, and poorer performance. Moreover, in situations where role conflict is particularly high, experienced product managers are susceptible to “burnout.” Some practical approaches to overcoming these difficulties are discussed.</t>
@@ -20035,7 +19899,7 @@
       </c>
       <c r="P388" s="0" t="inlineStr">
         <is>
-          <t>Team-level study of software development teams where boundary spanning is measured at the team level (N = 25 teams). Verbatim Evidence: "U.S. and Indian Managerial Boundary Spanning Behaviors in Globally Distributed Software Teams... The first study measured the boundary spanning behaviors of software team managers of 25 teams. These results were analyzed in conjunction with a standard measure of software team output." (Abstract section)</t>
+          <t>Team level aggregation. Verbatim Evidence: "Since the unit of analysis here is at the team level, those scores were averaged across each team to form three boundary spanning scores for each team."</t>
         </is>
       </c>
     </row>
@@ -20085,7 +19949,7 @@
       </c>
       <c r="P389" s="0" t="inlineStr">
         <is>
-          <t>Firm-level study of senior executive external networks and strategic imitation where the unit of analysis is the firm (N = 58 firms). Verbatim Evidence: "The external networks of senior executives: Implications for strategic innovation and imitation... Results from the model are tested on a sample of 58 firms operating in the branded foods and computer industries." (Abstract / Sample section)</t>
+          <t>Top management team unit of analysis. Verbatim Evidence: "In keeping with prior research findings indicating that organizational decisions and the outcomes they produce tend to be jointly, rather than individually determined (i.e., Cyert and March, 1963), this work adopts the top management team as its unit of analysis." (Unit of Analysis)</t>
         </is>
       </c>
     </row>
@@ -20342,14 +20206,10 @@
       </c>
       <c r="E395" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F395" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F395" s="0" t="inlineStr"/>
       <c r="G395" s="0" t="inlineStr">
         <is>
           <t>In this study of the business communication that connects an organization with others in its environment, we link boundary spanning with network theory and propose the concept of an extended network of communication. This extended net work is the structure of business communication which flows in work-related ties that organization members maintain both within the organization and across its boundary. We study the relationship between boundary-spanning communication and individual influence in a network with 108 organizational members. We find that boundary spanning correlates with influence, regardless of hierarchical level. There is also a curvilinear relationship between boundary-spanning communication and individual influence. Thus, managers need to balance their communication within and across the organizational boundary.</t>
@@ -20443,7 +20303,7 @@
       </c>
       <c r="F397" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>3 = Non-individual level</t>
         </is>
       </c>
       <c r="G397" s="0" t="inlineStr">
@@ -20471,7 +20331,7 @@
       </c>
       <c r="P397" s="0" t="inlineStr">
         <is>
-          <t>PDF file mismatch: Master sheet lists Stock, Zacharias &amp; Schnellbaecher (2017) but actual PDF [394] contains Bennet (1989) "Personnel/human resource departments and uncertainty" which is a scanned reproduction without extractable text. Verbatim Evidence: "Reproduced with permission of the copyright owner. Further reproduction prohibited without permission." (Full document - scanned image). Unable to verify individual-level BSB correlation data.</t>
+          <t>HR Departments. Verbatim Evidence: "The dissertation tests hypotheses generated from Thompson's theory of boundary spanning units using a sample of personnel/human resource departments (N = 124) in the eighteen county Atlanta Standard Metropolitan Statistical Area." (Summary)</t>
         </is>
       </c>
     </row>
@@ -20821,7 +20681,7 @@
       </c>
       <c r="P404" s="0" t="inlineStr">
         <is>
-          <t>Qualitative multiple-case study using interviews without individual employee Pearson correlation matrix. Verbatim Evidence: "Practices of strategic alignment in and between innovation project portfolios... qualitative multiple-case study conducted with three large firms that have multiple innovation project portfolios. Data collection was done primarily through key informant interviews and the consequent thematic data analysis approach." (Abstract / Methodology section)</t>
+          <t>Qualitative case study. Verbatim Evidence: "This study was carried out using a qualitative multiple-case study with three firms that implemented their innovations through projects." (3.1. Research design and cases)</t>
         </is>
       </c>
     </row>
@@ -20993,7 +20853,7 @@
       </c>
       <c r="P407" s="0" t="inlineStr">
         <is>
-          <t>Team-level study of dynamic medical teams where the unit of analysis is the core team per week (N = 91 team-weeks across 22 teams). Verbatim Evidence: "Coordination in Dynamic Teams: Investigating a Learning-Productivity Trade-Off... The unit of analysis was a core team in a given week, along with the periphery members associated with each patient case... Our overall sample included 243 unique core team members." (Methodology / Sample section)</t>
+          <t>Team level. Verbatim Evidence: "Because of the reconstitution of each core team each week, we treated the core teams from week to week as separate entities such that the unit of analysis was a core team in a given week"</t>
         </is>
       </c>
     </row>
@@ -21043,7 +20903,7 @@
       </c>
       <c r="P408" s="0" t="inlineStr">
         <is>
-          <t>Firm-level study of innovative ICT start-ups in Italy where the unit of analysis is the venture/firm (N = 179 start-ups). Verbatim Evidence: "Unpacking the drivers of the socio-environmental sustainability of new ventures: insights from innovative digital start-ups in Italy... Out of 1104 contacted firms, we received replies from 179 start-ups (16% response rate), representative of the population of innovative ICT start-ups operating in Italy." (Methodology / Sample section)</t>
+          <t>Firm level. Verbatim Evidence: "Poisson family estimations (negative binomial and zero-inflated negative binomial) of 172 innovative ICT start-ups based in Italy reveal different driving factors of their socio-environmental sustainability."</t>
         </is>
       </c>
     </row>
@@ -21310,14 +21170,10 @@
       </c>
       <c r="E414" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F414" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F414" s="0" t="inlineStr"/>
       <c r="G414" s="0" t="inlineStr">
         <is>
           <t>The vast majority of research on self‐monitoring in the workplace focuses on the benefits that accrue to chameleon‐like high self‐monitors (relative to true‐to‐themselves low self‐monitors). In this study, we depart from the mainstream by focusing on a potential liability of being a high self‐monitor: high levels of experienced role conflict. We hypothesize that high self‐monitors tend to choose work situations that, although consistent with the expression of their characteristic personality, inherently involve greater role conflict (i.e. competing role expectations from different role senders). Data collected from a 116‐member high‐tech firm showed support for this mediation hypothesis: relative to low self‐monitors, high self‐monitors tended to experience greater role conflict in work organizations because high self‐monitors were more likely to occupy boundary spanning positions. To help draw a more realistic and balanced portrait of self‐monitoring in the workplace, we call for more theoretically grounded research on the price chameleons pay.</t>
@@ -23065,14 +22921,10 @@
       </c>
       <c r="E449" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F449" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F449" s="0" t="inlineStr"/>
       <c r="G449" s="0" t="inlineStr">
         <is>
           <t>Background The health-care environment requires hospital units to coordinate efforts autonomously across their boundaries and to manage relationships with other professionals, units and departments. Boundary spanning has become increasingly important for ﬁrst-line nurse managers as unit gatekeepers; however, the available measures are limited. Method The 30-item instrument was developed from a literature review. Survey participants were 4918 nurses at 231 hospital units. Statistical analyses of construct validity and internal consistency were performed. Furthermore, the correlation between nurses’ scores on the Nurse Managers Boundary Spanning Scale and nurses’ evaluations of their managers were examined. Results Three factors and 26 items were derived from factor analyses: connecting and mediating, informing and feedback utilisation, and resource acquisition. Cronbach’s subscales’ alpha coefﬁcients were above 0.9. Correlation analysis indicated that the Nurse Managers Boundary Spanning Scale score correlated with nurses’ positive perceptions of their managers. Conclusion This study demonstrates tentative support for the validity and reliability of the Nurse Managers Boundary Spanning Scale. Although further study is needed, the Nurse Managers Boundary Spanning Scale shows possibilities as a new measurement of nursing leadership. Implications This study underscores measures to build on nurse managers’ roles by building on the limited research available.</t>
@@ -23111,14 +22963,10 @@
       </c>
       <c r="E450" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F450" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F450" s="0" t="inlineStr"/>
       <c r="G450" s="0" t="inlineStr">
         <is>
           <t>This study examines how cultural performance orientation moderates the influence of human resource management (HRM) controls on boundary-spanning employees' behavioural strategies and satisfaction. Based on primary data obtained from 1049 salespeople in six countries (France, Ireland, Italy, Spain, United Kingdom, and the United States of America) and secondary data on cultural performance orientation, multilevel regression analyses show that national culture has a strong effect on the way boundary-spanning employees allocate their effort in response to HRM control. In particular, our results suggest that the more behaviour controls are used with boundary-spanning employees, the less attention they pay to customers and the more emphasis they place on their supervisors and non-selling tasks. Specifically, cultural performance orientation is shown to moderate significantly those relationships. Furthermore, results indicate that cultural performance orientation heightens boundary-spanning employees' job satisfaction resulting from behaviour control. Preliminary explanations for the differing impact of HRM control efficiency across cultures can be proposed.</t>
@@ -24031,14 +23879,10 @@
       </c>
       <c r="E468" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F468" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F468" s="0" t="inlineStr"/>
       <c r="G468" s="0" t="inlineStr">
         <is>
           <t>The purpose of this paper is to advance and empirically investigate how perceived organisational support inﬂuences marketing managers’ boundary-spanning marketing activities (cross-functional communication and customer connections), and how these activities subsequently impact supply-chain efﬁciency. By analysing survey responses from 348 marketing managers, we demonstrate that a supportive organisational climate provides managerial incentives not only to develop strong allegiance to the welfare of multi-foci groups within the organisation but also to engage in active cross-functional market intelligence exchange and customer servicing, which in turn leads to superior supply-chain efﬁciencies. The paper offers strategic guides to both academicians and practitioners on how to promote marketing managers’ role in strengthening dependencies among various functional departments for cohesive product, service, and ﬁnancial offerings.</t>
@@ -24427,14 +24271,10 @@
       </c>
       <c r="E476" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F476" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F476" s="0" t="inlineStr"/>
       <c r="G476" s="0" t="inlineStr">
         <is>
           <t>Contrary to much boundary spanning research, we examined the negative consequences of boundary spanning contact in multi-organizational contexts. Results from a sample of 833 Dutch peacekeepers show that employees’ boundary spanning contact with members of other organizations was associated with reports of negative relationships with external parties (e.g., work-speciﬁc problems, culture-speciﬁc problems). These negative relationships also had a spillover effect such that they mediated the effect of boundary spanning contact on boundary spanners’ negative attitudes toward their own jobs and organization (e.g., job attractiveness and conﬁdence in the organization). Copyright # 2010 John Wiley &amp; Sons, Ltd.</t>
@@ -24573,14 +24413,10 @@
       </c>
       <c r="E479" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F479" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F479" s="0" t="inlineStr"/>
       <c r="G479" s="0" t="inlineStr">
         <is>
           <t>Viewing knowledge as rooted in individuals, this study investigates knowledge transfer in multinational corporations (MNCs) from an individual-level perspective. Speciﬁcally, the author focuses on inpatriates as a particular group of knowledge actors in MNCs and examines the role of inpatriates’ boundary spanning between their home unit and the headquarters for transferring their knowledge to headquarters staff. Based on a sample of 269 inpatriates in 10 German MNCs, the author found that inpatriates’ boundary spanning is positively related to inpatriates’ individual efforts to transfer knowledge and inpatriates’ perceptions of HQ staff efforts to acquire subsidiary-speciﬁc knowledge. Both perceived HQ absorptive capacity and mentoring by HQ staff moderate these relationships.This study’s ﬁndings contribute to our understanding of the theoretical mechanisms through which MNC knowledge ﬂows occur and highlight key requirements for the design of international stafﬁng practices. © 2011 Wiley Periodicals, Inc.</t>
@@ -24619,14 +24455,10 @@
       </c>
       <c r="E480" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F480" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F480" s="0" t="inlineStr"/>
       <c r="G480" s="0" t="inlineStr">
         <is>
           <t>Examined relationships between major role requirements and experienced role stress, using data from 202 research and development professionals. Measures (including those of JR Rizzo et al, 1970) of role stress included various types of role conflict and ambiguity. Role requirements included integration and boundary-spanning activities, personnel supervision, and scientific research. Role conflict was more sensitive than role ambiguity to differences in research and development role requirements; and integration and boundary-spanning activities were the best predictors of experienced role conflict, especially of the intersender variety.</t>
@@ -25697,14 +25529,10 @@
       </c>
       <c r="E502" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F502" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F502" s="0" t="inlineStr"/>
       <c r="G502" s="0" t="inlineStr">
         <is>
           <t>Boundary-spanning activity was studied in a large manufacturing company through a sample of 192 managers, engineers, and supervisors. Contrary to prior theory and research, this study found boundary-spanning activity unrelated to role conflict or ambiguity and positively related to job satisfac-tion for the total sample. Boundary-spanning activity was also positively related to a number of job characteristics for the total sample. Marked dif-ferences in boundary-spanning activity and its relationships with other variables, however, were found across occupational levels. While managers and engineers generally had boundary-spanning activity related to high levels of job satisfaction and job characteristics, first-level supervisors had boundary-spanning activity related to higher role conflict and lower job satisfaction with opportunities for promotion.</t>
@@ -26045,14 +25873,10 @@
       </c>
       <c r="E509" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F509" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F509" s="0" t="inlineStr"/>
       <c r="G509" s="0" t="inlineStr">
         <is>
           <t>While researchers have probed predictors of product managers' performance in consumer goods firms, few have looked at the performance of the industrial product manager. In this article, Steven Lysonski and Arch Woodside use path analysis to examine causal models of industrial product managers' performance during periods of rapid technological change. Key variables are analyzed, including the effects of environmental uncertainty, boundary spanning behavior, role pressures, role outcomes and two performance measures. A total of 69 industrial product managers from New Zealand Telecom completed a questionnaire that included both operational measures of the key variables and their overall job performance. The results suggest that most of the hypothesized relationships are supportable empirically. Performance was hindered by environmental uncertainty, role conflict, role ambiguity, tension and dissatisfaction. The authors discuss their study's implications for improving the effectiveness of product management practices.</t>
@@ -26141,14 +25965,10 @@
       </c>
       <c r="E511" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F511" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F511" s="0" t="inlineStr"/>
       <c r="G511" s="0" t="inlineStr">
         <is>
           <t>Purpose – Drawing on the conservation of resources theory, this research examines the relationship between managers’ servant leadership and frontline employees’ customer-oriented boundary-spanning behaviors by considering career meaningfulness as an underlying mechanism. Furthermore, this study investigates a moderated mediation model by proposing work centrality as a boundary condition in the relationship between career meaningfulness and customer-oriented boundary-spanning behaviors.</t>
@@ -26187,14 +26007,10 @@
       </c>
       <c r="E512" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F512" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F512" s="0" t="inlineStr"/>
       <c r="G512" s="0" t="inlineStr">
         <is>
           <t>Many humanitarian aid workers receive training prior to being dispatched into the field, but they often encounter challenges that require additional learning and creativity. Consequently, aid organizations formally support collaboration among the expatriate and local workers in a field office. At best, those aid workers would not only exploit their joint knowledge but also explore novel ways of managing the challenges at hand. Yet differences between expatriate and local groups (e.g., in ethnicity, religion, education, and salary) often thwart intergroup collaboration in field offices and, by extension, any joint learning or creativity. In response to this issue, we study the role of field office leaders—specifically, how their boundary‐spanning behavior may inspire collaboration between the two groups and therefore facilitate joint learning and creativity. We propose that a leader's in‐group prototypicality additionally catalyzes this process—that is, a leader's behavior has more impact if s/he is seen as representing his/her group. We tested and found support for our hypothesized moderated mediation model in a field sample of 137 aid workers from 59 humanitarian organizations. Thus, our study generally highlights the pivotal role that field office leaders play for crucial outcomes in humanitarian aid operations. Furthermore, we offer concrete steps for field office leaders who want to inspire better collaboration between the expatriate and local aid workers they lead.</t>
@@ -26283,14 +26099,10 @@
       </c>
       <c r="E514" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F514" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F514" s="0" t="inlineStr"/>
       <c r="G514" s="0" t="inlineStr">
         <is>
           <t>Boundary spanners are pivotal in developing effective public–private collaboration in public infrastructure projects. As boundary spanners have to account for different interests, perspectives, and ways of working in public–private collaborations, engaging in boundary-spanning activities often comes with role stress, which can negatively impact their job performance. However, despite the significant levels of role stress associated with boundary spanning, there is a dearth of empirical studies on the role stress of boundary spanning public managers and how it can be reduced. In this study, we empirically investigate the reciprocal relationship between role stressors and boundary spanning and test if supporting organizational conditions can alleviate role stressors. The findings show that especially role conflict is detrimental for boundary-spanning activities. We further find that top-management support can diminish both role conflict and role ambiguity and that co-worker support can help in reducing the role ambiguity of boundary spanning public managers.</t>
@@ -26679,14 +26491,10 @@
       </c>
       <c r="E522" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F522" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F522" s="0" t="inlineStr"/>
       <c r="G522" s="0" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to analyze the effects of inpatriates’ abilities, motivation and opportunities on knowledge sharing and the moderating role of boundary spanning in this context. Design/methodology/approach – By integrating the ability–motivation–opportunity framework with the concept of boundary spanning four hypotheses are developed, which are tested against the data of 187 inpatriates working in Germany.</t>
@@ -27556,14 +27364,10 @@
       </c>
       <c r="E540" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F540" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F540" s="0" t="inlineStr"/>
       <c r="G540" s="0" t="inlineStr">
         <is>
           <t>This dissertation investigated the effects of intrinsic and extrinsic motivational orientations in a boundary spanning model of retail buyers. Contributions of the dissertation to the field of marketing include the following: First, a boundary spanning/role stress model was tested in the context of retail buyers. No previous work has empirically or conceptually investigated the ability of a boundary spanning/role stress model to explain retail buyers' work-related attitudes. Second, the boundary spanning/role stress model was extended with the inclusion of accumulated role benefits. Previous role stress studies consider only negative role perceptions; accumulated role benefits examines positive role perceptions. Third, the boundary spanning/role stress model considers only external influences of role set members on a role incumbent. In doing so, the model neglects the influence of the individual who is perceiving and interpreting these stimuli. To capture individual differences, effects of intrinsic and extrinsic motivational orientations of the buyers were tested in the model. Finally, scales were developed to measure intrinsic motivational orientations, extrinsic motivational orientations, boundary spanning beliefs, and accumulated role benefits.</t>
@@ -27652,14 +27456,10 @@
       </c>
       <c r="E542" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F542" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F542" s="0" t="inlineStr"/>
       <c r="G542" s="0" t="inlineStr">
         <is>
           <t>Purpose – Boundary-spanning managers need to recognize, learn and implement external knowledge while balancing the conflicts emerging from new and existing knowledge. The authors’ study explores how a paradox mindset (PM) and a learning focus [learning goal orientation (LGO)] promote two managerial capabilities: absorptive capacity (ACAP) and ambidexterity. The authors’ study explores the inter-relationship between the mindsets and the capabilities required for innovative work behavior.</t>
@@ -28657,14 +28457,10 @@
       </c>
       <c r="E562" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F562" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F562" s="0" t="inlineStr"/>
       <c r="G562" s="0" t="inlineStr">
         <is>
           <t>In this study, the national cultures and the complex contexts of Japanese multinational organizations (MN0s) are studied in the US The present study assumes that there are influences of national cultures which maintain significant cultural stereotypes in MNO, and also there are complex contexts of MNOs which might create distinctive communication patterns among Americans and Japanese. The objectives of this study are to quantitatively analyze the cognitive and behavioral dimensions of communication between these two cultural groups and identify distinctive patterns of organizational communication in terms of MNO effectiveness. The frameworks for interactions (FINT) scale is used for measurement of individual communication frames (n= 152), and ego-networks are measured to analyze ingroup-outgroup communications (n= 66). Cultural difference is identified in communication frames and patterns of ingroup-outgroup communication. Results about communication frames and ingroup-outgroup communication contradict expectations of cross-cultural stereotypes. This result implies that convergence in communication frames and communicative interactions is a key to success in MNOs. Results also suggest that the importance of outgroup communication is in its boundary spanning function, while increasing outgroup communication is crucial for both Americans and Japanese to enhance their communicative convergence and increase the effectiveness of MNOs.</t>
@@ -29383,14 +29179,10 @@
       </c>
       <c r="E576" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F576" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F576" s="0" t="inlineStr"/>
       <c r="G576" s="0" t="inlineStr">
         <is>
           <t>In this article, we study the conditions under which having ties that span organizational boundaries (bridging ties) are conducive to the generation of innovations. Whereas previous research has shown that bridging ties have a positive impact on innovative performance, our analysis of 276 R&amp;D scientists and engineers reveals that there are no advantages associated with bridging per se. In contrast, our findings suggest that the advantages traditionally associated with bridging ties are contingent upon the nature of the ties forming the bridge—specifically, whether these bridging ties are Simmelian.</t>
@@ -29719,14 +29511,10 @@
       </c>
       <c r="E583" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F583" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F583" s="0" t="inlineStr"/>
       <c r="G583" s="0" t="inlineStr">
         <is>
           <t>Abstract             Although recent years have seen a proliferation of research on organizational ambidexterity, important questions remain about the role that leaders play in leveraging learning ambidexterity for organizational benefits. Drawing on the conservation of resources theory, we investigate the indirect links between servant leadership and middle managers’ learning ambidexterity, with structural empowerment and role breadth self‐efficacy (RBSE) as serial mediators. We also examine the importance of leader boundary‐spanning behaviour as a moderating factor for these relationships. Using time‐lagged and multi‐source data from 344 middle managers and their supervisors, we show that servant leadership has a positive indirect influence on two forms of learning ambidexterity: exploitative and explorative learning. In particular, servant leadership promotes structural empowerment (as a contextual resource), which in turn influences RBSE (as a personal resource) and encourages learning ambidexterity. In addition, we show that when leaders engage in boundary‐spanning behaviour, these indirect relationships become more prominent. This research offers new theoretical and practical insights to assist organizations in improving learning ambidexterity and achieving higher levels of performance.</t>
@@ -30465,14 +30253,10 @@
       </c>
       <c r="E598" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F598" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F598" s="0" t="inlineStr"/>
       <c r="G598" s="0" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to draw upon motivated information processing theory to examine the sequential mediating roles of perspective taking and boundary spanning between transformational leadership and the creative performance of knowledge workers.</t>
@@ -31001,14 +30785,10 @@
       </c>
       <c r="E609" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F609" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F609" s="0" t="inlineStr"/>
       <c r="G609" s="0" t="inlineStr">
         <is>
           <t>The present study explores the antecedents of frontline employees’ boundary-spanning behaviors in the hospitality industry. Based on social exchange theory and role theory, a conceptual model was built to explore how three dimensions of perceived organizational support (perceived supervisory support, internal communication, and training) cultivate frontline employees’ boundary-spanning behaviors through job satisfaction and organizational commitment. Based on the analysis of 597 hospitality frontline employees in the United States, which were recruited through Amazon Mechanical Turk, this study shows the differential impacts of organizational support types on driving boundary spanning staff to effectively operate on the boundary. Theoretical and practical implications of the findings are articulated.</t>
@@ -31247,14 +31027,10 @@
       </c>
       <c r="E614" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F614" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F614" s="0" t="inlineStr"/>
       <c r="G614" s="0" t="inlineStr">
         <is>
           <t>Based on social information processing theory, we provide a novel theoretical account of how and when leader humor influences subordinate boundary-spanning behavior. We develop a moderated mediation model explicating the mechanism of psychological safety and the boundary condition of subordinate interpersonal influence. Using multiwave data, we tested our research hypotheses with a sample of 452 members from 140 teams in a Chinese information technology (IT) company. Results showed that leader humor positively affects subordinate boundary-spanning behavior               via               increased psychological safety. Moreover, this mediated effect is stronger when subordinates have high interpersonal influence. These findings offer theoretical and practical insights into boundary-spanning activities and leader humor, which we discuss.</t>
@@ -31293,14 +31069,10 @@
       </c>
       <c r="E615" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F615" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F615" s="0" t="inlineStr"/>
       <c r="G615" s="0" t="inlineStr">
         <is>
           <t>The turnover of IT professionals is a perpetual challenge for non-IT organizations. Based on selfcategorization theory, this study proposes that IT employees’ turnover may be mitigated by fostering their identification with non-IT organizations, which can be done by meeting various facilitative conditions. Guided by intergroup contact theory, we identify IT employees’ perceived alignment between IT and the core business of an organization (business-IT alignment), the extent of boundaryspanning activities that IT employees engage in, and the closeness of the relationships between IT and non-IT employees as the drivers of their organizational identification. Using survey data collected from organizations in different industries, we obtained empirical evidence supporting the positive effects of the perceived business-IT alignment, the extent of boundary-spanning activities, and the relationship closeness between IT and non-IT employees on IT employees’ organizational identification. Additionally, there was a three-way interaction effect among the three drivers such that the relationship closeness between IT and non-IT employees reduced the positive effect of the extent of boundary-spanning activities on IT employees’ organizational identification when business-IT alignment was low. However, this negative moderating effect diminished when business-IT alignment increased. The findings of this research advance the literature and offer practical guidelines for non-IT organizations on how to enhance their IT employees’ organizational identification and how to mitigate their turnover intentions.</t>
@@ -31389,14 +31161,10 @@
       </c>
       <c r="E617" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F617" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F617" s="0" t="inlineStr"/>
       <c r="G617" s="0" t="inlineStr">
         <is>
           <t>Frontline service employees (FSEs)’ customer-oriented boundary spanning behaviors (COBSBs) are prosocial behaviors adapted to the job requirements and work environment of customer service personnel. It is a significant strategic imperative for achieving excellent performance in the tourism organizations. Building on social exchange theory, this study uncovered that inclusive leadership motivates FSEs’ COBSBs. Using hierarchical multiple regression analysis with time-lagged data, we find that inclusive leadership promotes FSEs’ COBSBs by enhancing their felt obligations. Moreover, the need for affiliation enhances the direct effect that inclusive leadership has on felt obligations and its indirect effect on FSEs’ COBSBs via felt obligations.</t>
@@ -32415,14 +32183,10 @@
       </c>
       <c r="E638" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F638" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F638" s="0" t="inlineStr"/>
       <c r="G638" s="0" t="inlineStr">
         <is>
           <t>Although research suggests that subordinates’ boundary spanning may result in unintended negative responses from their supervisors, little is known about which supervisors are likely to react adversely and which are not. We draw on self-protection theory to answer this question. Specifically, we argue that when supervisors experience low levels of managerial self-efficacy, boundary spanning behavior threatens their perceived work status within the team, resulting in abusive supervisory behavior. The results of two field survey studies and an experimental study support our hypotheses. Our research identifies managerial barriers that may hinder boundary spanning behavior at work and provides invaluable insights into how upper-level organizations may create constructive work contexts that encourage employees to engage in such behavior.</t>
@@ -33061,14 +32825,10 @@
       </c>
       <c r="E651" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F651" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F651" s="0" t="inlineStr"/>
       <c r="G651" s="0" t="inlineStr">
         <is>
           <t>This study examines the impact of emotional intelligence (EI) on boundaryspanning behavior, relationship quality, and performance among door‐todoor salespeople. Data is collected from salespeople and customers of South Korean door‐to‐door cosmetics businesses and analyzed using structural equation modeling. The findings show that EI positively affects boundaryspanning behavior. Similarly, boundary‐spanning behavior improves relationship quality, which improves both sales performance and customer satisfaction. This suggests that EI plays an important role in salespeople's boundaryspanning behavior, thereby enhancing relationship quality, sales performance, and customer satisfaction. Unlike previous studies, this study makes use of actual sales volumes, salespeople's self‐reporting responses, and salespeople's customer‐reporting, which adds to the findings' uniqueness. The present study highlights that EI improves boundary‐spanning behavior, which is vital in developing relationship quality, improving sales performance, and increasing customer satisfaction. The study uses triadic data from door‐to‐door salespeople, customers, and sales organizations extensively, which is unusual in this field.</t>
@@ -33357,14 +33117,10 @@
       </c>
       <c r="E657" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F657" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F657" s="0" t="inlineStr"/>
       <c r="G657" s="0" t="inlineStr">
         <is>
           <t>Purpose – This study aims to investigate the effect of social undermining on the service employees’ boundary-spanning behavior though perceived ﬁt with job (P-J ﬁt). This study also aims to examine the moderating role of ethical climate in the relationship between service employees’ perceived ﬁt with job (P-J ﬁt) and boundary-spanning behavior.</t>
@@ -34288,14 +34044,10 @@
       </c>
       <c r="E676" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F676" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F676" s="0" t="inlineStr"/>
       <c r="G676" s="0" t="inlineStr">
         <is>
           <t>Enterprise social media (ESM) provides convenient channels for employees to access enterprise-wide work resources but also exposes employees to potential distractions. Prior studies have confirmed this “two-sided” role of ESM usage on employee work performance. Ongoing studies are exploring possible methods to alleviate side effects of ESM usage. Drawing on boundary management literature and information processing theory, we propose the concept of individual boundary spanning to capture employees’ information-obtaining behaviors via ESM and identify two mediating mechanisms—mindfulness and information overload—through which an individual’s boundary spanning affects work performance. We also propose the concept of individual boundary buffering to capture protective actions by individuals that prevent them from becoming disturbed or overloaded with ESM requests. We further investigate the interaction effects of these two boundary activities in the ESM context. We conducted a survey and collected data from 202 ESM users from a research and development enterprise in China. The results suggest that individual boundary spanning triggers mindfulness in individuals that benefits their work performance but also increases information overload, harming work performance. Individual boundary buffering can enhance the positive relationship between individual boundary spanning and mindfulness, and mitigate the positive relationship between spanning activity and information overload.</t>
@@ -34652,14 +34404,10 @@
       </c>
       <c r="E683" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F683" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F683" s="0" t="inlineStr"/>
       <c r="G683" s="0" t="inlineStr">
         <is>
           <t>Purpose – Although enterprise social media (ESM) offers new opportunities for developing radical creativity, limited research has been conducted on how to foster such creativity in ESM contexts. Based on the approachinhibition theory of power (AITP), this study examines how supervisor-subordinate instrumental and expressive ties on ESM promote radical creativity through sense of power. Furthermore, it further investigates how boundary buffering moderates the influence of these supervisor-subordinate ties on sense of power.</t>
@@ -34838,14 +34586,10 @@
       </c>
       <c r="E687" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F687" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F687" s="0" t="inlineStr"/>
       <c r="G687" s="0" t="inlineStr">
         <is>
           <t>In the context of encouraging collaborative innovation, employee boundary spanning has become a source of organizational innovation. However, existing research has mainly explored the impact of employee boundary spanning on themselves from an actor-centered perspective, little is known about whether employee boundary spanning can influence supervisor support. Drawing on the perspective of positive interpersonal interaction, the current study employed a scenario experiment (Study 1) and a multi-wave and multi-source questionnaire survey (Study 2) to explore when and how employee boundary spanning affects supervisor support. Results from Study 1 (N= 220) indicated that when upward advice seeking is high, supervisors develop stronger cognitive trust and affective trust towards boundary spanning employees, leading to higher levels of supervisor support. Study 2 (N= 406) further confirmed that upward advice seeking positively moderates the direct effect of employee boundary spanning on supervisor affective trust as well as the indirect effect of employee boundary spanning on supervisor support via affective trust. However, it did not support the moderating effect of upward advice seeking on the supervisor cognitive trust path. These findings contribute to a comprehensive understanding of the impact of employee boundary spanning on supervisor support, providing decision-making references for organizations to manage employee boundary spanning to maintain harmonious supervisor-subordinate relationships.</t>
@@ -34884,14 +34628,10 @@
       </c>
       <c r="E688" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F688" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F688" s="0" t="inlineStr"/>
       <c r="G688" s="0" t="inlineStr">
         <is>
           <t>To comprehend the mechanism of decent work’s impact on employee boundaryspanning behaviour, this paper constructs a research framework that includes promotion focus and a supportive organizational climate as a mediating factor and moderating variable. A two-stage survey is used to examine these assumptions with data collected from 346 frontline employees. The ﬁndings reveal that decent work has a signiﬁcant positive impact on employee boundary-spanning behaviour and promotion focus has a partial mediating eﬀect on this relationship. A supportive organizational climate plays a positive moderating role in the relationship between decent work and promotion focus.</t>
@@ -35030,14 +34770,10 @@
       </c>
       <c r="E691" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F691" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F691" s="0" t="inlineStr"/>
       <c r="G691" s="0" t="inlineStr">
         <is>
           <t>Purpose – This paper examined the mediating role of boundary spanning behavior and the moderating effects of traditionality linking humble leadership and employee creative performance from the perspective of Social Exchange Theory (SET) to reveal the behavioral mechanism and boundary condition regarding the influence of humble leadership on creative performance.</t>
@@ -35226,14 +34962,10 @@
       </c>
       <c r="E695" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F695" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F695" s="0" t="inlineStr"/>
       <c r="G695" s="0" t="inlineStr">
         <is>
           <t>Boundary-spanning behavior has attracted considerable interest in recent years. Studies on this type of behavior have focused on its positive outcomes from the perspective of social networks. For decades, research has consistently demonstrated that the boundary-spanning behavior produces a wide array of positive results for teams and organizations. However, scholars have found that such behavior has negative outcomes for individuals. Using the conservation of resources theory (COR), we examined the double-edged-sword effect of boundary- spanning behavior on creativity at different levels, as well as its mediating mechanism and boundary conditions.</t>
@@ -35422,14 +35154,10 @@
       </c>
       <c r="E699" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F699" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F699" s="0" t="inlineStr"/>
       <c r="G699" s="0" t="inlineStr">
         <is>
           <t>Although the information‐seeking literature has tended to focus upon the selection and use of inanimate objects as information sources, this research follows the more recent trend of investigating how individuals evaluate and use interpersonal information sources. By drawing from the structural, relational, and cognitive elements of social capital theory to inform antecedents to information quality and source accessibility, a research model is developed and tested. For interpersonal information sources, information quality is the key determinant of source use. Perceptions of information quality and accessibility of an interpersonal source are shown to be influenced by boundary spanning, transactive memory, and content type. Implications and prescriptions for future research are discussed.</t>
@@ -35471,7 +35199,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F700" t="inlineStr">
+      <c r="F700" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -35618,14 +35346,10 @@
       </c>
       <c r="E703" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F703" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F703" s="0" t="inlineStr"/>
       <c r="G703" s="0" t="inlineStr">
         <is>
           <t>We propose and test a framework that describes the relationship between network structures and job performance. We provide an integration of the current conceptualizations of social capital as they pertain to job performance outcomes by taking a multi-dimensional view of job performance. We break down job performance into creativity, decision-making, task execution, and teamwork, and distinguish the effect of structural holes within and across the organizational boundary on these four job performance domains. In an analysis of 318 managers, we ﬁnd that networks rich in structural holes that cross the organizational boundary had a positive association with creativity and decision-making, whereas networks with few structural holes within the organization had a positive association with task execution and teamwork. We discuss the theoretical implications for integrating the social capital, boundary spanning, and network structure literatures, as well as the practical beneﬁts of giving much more precise advice to managers and employees regarding how to use networks to improve performance at work.</t>
@@ -35667,7 +35391,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F704" t="inlineStr">
+      <c r="F704" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>

</xml_diff>

<commit_message>
Audit: Shadow Batch 22 complete (Final). All 8 papers were verified as true Includes. Final Included: 114
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -34499,6 +34499,7 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F685" s="0" t="inlineStr"/>
       <c r="G685" s="0" t="inlineStr">
         <is>
           <t>This article draws on status characteristics theory to explore the mechanisms of individual-level boundaryspanning behavior on employee creative performance, as well as the mediating role of informal status and the moderating role of Zhongyong thinking. The results of a two-wave questionnaire survey of 202 employees show that boundary-spanning behavior has a significant positive relationship with employees’ creative performance, informal status mediates the link between boundary-spanning behavior and creative performance of this employee, Zhongyong thinking plays a moderating role between employees’ boundary-spanning behavior and their informal status, and Zhongyong thinking also moderates the mediating role of informal status between boundary-spanning behavior and employee creative performance. In this paper, a moderated mediation model is established to enhance the understanding of the effects and mechanisms of individual boundary-spanning behavior, as well as to provide some constructive insight into how boundary-spanning behavior can be effectively employed in management practice within the Chinese context.</t>
@@ -34522,11 +34523,7 @@
       <c r="K685" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P685" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P685" s="0" t="inlineStr"/>
     </row>
     <row r="686" ht="18" customHeight="1" s="31">
       <c r="A686" s="0" t="inlineStr">
@@ -34544,6 +34541,7 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F686" s="0" t="inlineStr"/>
       <c r="G686" s="0" t="inlineStr">
         <is>
           <t>With the increasing uncertainty of the environment and the complexity of team tasks, it’s now common practice to encourage employees to implement boundary spanning behaviors. In spite of the fact that a few studies have explored the relationship between boundary spanning behavior and employee creative performance, little is known about the mechanism behind this association. Drawing on the conservation of resource theory (COR), this paper examines the mediating role of meaning of work and the moderating role of team Chaxu climate to reveal the internal process and boundary condition regarding the effect of boundary spanning behavior on employee creative performance. A sample of 211 supervisorsubordinate dyads from six companies located in China is collected in this study, and a hierarchical linear model is used to test the hypotheses. The results show that boundary spanning behavior has a positive effect on employee creative performance, meaning of work mediates the link between them, and team Chaxu climate negatively moderates the relationship between boundary spanning behavior and meaning of work. This research provides a new insight into the linkage between boundary spanning behavior and employee creative performance, as well as further answers the question “how and when boundary spanning behavior influences employee creative performance”.</t>
@@ -34567,11 +34565,7 @@
       <c r="K686" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P686" s="0" t="inlineStr">
-        <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
-        </is>
-      </c>
+      <c r="P686" s="0" t="inlineStr"/>
     </row>
     <row r="687" ht="18" customHeight="1" s="31">
       <c r="A687" s="0" t="inlineStr">

</xml_diff>

<commit_message>
chore: completed Track 1 (27 missing papers)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -1557,8 +1557,24 @@
           <t>BSMA0014</t>
         </is>
       </c>
-      <c r="E17" s="0" t="inlineStr"/>
-      <c r="F17" s="0" t="inlineStr"/>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boundary spanner multi-faceted role ambiguity and burnout An exploratory study</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Ambrose et al.</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
           <t>Although researchers have gained considerable knowledge regarding the multi-faceted manifestation of burnout over recent years, inconsistent findings of role ambiguity as an antecedent to burnout are still prevalent. Given the complex boundary-spanning nature of sales, it is likely that global measures of role ambiguity fail to fully capture the domain and impact of role ambiguity. To help address this gap, this study provides initial evidence that facets of role ambiguity impact burnout manifestation in the sales role differently. Specifically, findings provide a foundation to help mitigate the negative impact of burnout by focusing on only certain facets of role ambiguity.</t>
@@ -1582,7 +1598,17 @@
       <c r="K17" s="0" t="n">
         <v>2014</v>
       </c>
-      <c r="P17" s="0" t="inlineStr"/>
+      <c r="L17" s="0" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="P17" s="0" t="inlineStr">
+        <is>
+          <t>The study focuses on role ambiguity, role conflict, burnout, job satisfaction, and job performance among salespeople, but it does not contain a quantitative measure of boundary spanning behavior. Verbatim Evidence: "Scales in the extant literature were used for measuring all of the identified constructs. Role ambiguity was measured using the 45-item MULTIRAM instrument (Singh &amp; Rhoads, 1991). The ethical facet of MULTIRAM was not included in order to reduce study complexity. Ethics has rarely been incorporated into research directly focused on salesperson burnout and it is not germane to our study. Role conflict was assessed using the common 8-item instrument developed by Rizzo et al. (1970). Burnout was assessed using the reduced Maslach burnout inventory for sales (Rutherford et al., 2011). The job satisfaction construct was measured using a three-item scale developed by Netemeyer, Boles, McKee, and McMurrian (1997). Finally, job performance was measured by four items evaluating if annual sales targets and objectives have been met, effectiveness of presentations, having adequate product knowledge, and understanding both customer needs and work processes." (5.2. Measures, Page 6)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="31">
       <c r="A18" s="0" t="inlineStr">
@@ -1641,8 +1667,24 @@
           <t>BSMA0016</t>
         </is>
       </c>
-      <c r="E19" s="0" t="inlineStr"/>
-      <c r="F19" s="0" t="inlineStr"/>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Unpacking the Harmonization of National Anti-Doping</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Anagnostopoulos &amp; Begović</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="n">
+        <v>4</v>
+      </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
           <t>National sport policies’ harmonization with the World Anti-Doping Agency (WADA) has been one of the most researched topics within the sport policy domain. The literature, however, has failed to offer firsthand empirical insights from those actors who develop the policy so that harmonization occurs. The present study fills this gap by drawing on the tenets of institutional entrepreneurship to unpack the process through the experiences of the person responsible for it. The study employs a collaborative analytical autoethnography where, through memo-writings, emails, and reflective notes by the second author, it micro-theorizes the political, technical, and cultural activities that the institutional entrepreneur carried in order to harmonize Montenegro’s anti-doping policy with WADA. The study reveals that the harmonization process entails seven institutional works: boundary spanning, scanning the environment, repairing bilateral relationships, designing the new legislation, modifying structures, framing the need, and transferring responsibility. This is the first empirical study in sport management literature to examine institutional change for sport policy-making through the lenses of institutional entrepreneurship and a collaborative autoethnographic perspective.</t>
@@ -1666,7 +1708,17 @@
       <c r="K19" s="0" t="n">
         <v>2026</v>
       </c>
-      <c r="P19" s="0" t="inlineStr"/>
+      <c r="L19" s="0" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="P19" s="0" t="inlineStr">
+        <is>
+          <t>Qualitative collaborative autoethnography lacking quantitative employee effect sizes. Verbatim Evidence: "The present study fills this gap by drawing on the tenets of institutional entrepreneurship to unpack the process through the experiences of the person responsible for it. The study employs a collaborative analytical autoethnography where, through memo-writings, emails, and reflective notes by the second author, it micro-theorizes the political, technical, and cultural activities that the institutional entrepreneur carried in order to harmonize Montenegro’s anti-doping policy with WADA. The study reveals that the harmonization process entails seven institutional works: boundary spanning, scanning the environment, repairing bilateral relationships, designing the new legislation, modifying structures, framing the need, and transferring responsibility." (Abstract, Page 258)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1" s="31">
       <c r="A20" s="0" t="inlineStr">
@@ -1779,8 +1831,24 @@
           <t>BSMA0019</t>
         </is>
       </c>
-      <c r="E22" s="0" t="inlineStr"/>
-      <c r="F22" s="0" t="inlineStr"/>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Bridging the Boundary</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Ancona &amp; Caldwell</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F22" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
           <t>This article focuses on the activities teams use to manage their organizational environment beyond their teams. We used semistructured interviews with 38 new-product team managers in high-technology companies, log data from two of these teams, and questionnaires completed by members of a different set of 45 new-product teams to generate and test hypotheses about teams' external activities. Results indicate that teams engage in vertical communications aimed at molding the views of top management, horizontal communication aimed at coordinating work and obtaining feedback, and horizontal communication aimed at general scanning of the technical and market environment. Organizational teams appear to develop distinct strategies toward their environment: some specialize in particular external activities, some remain isolated from the external environment, and others engage in multiple external activities. The paper shows that the type of external communication teams engage in, not just the amount, determines performance. Over time, teams following a comprehensive strategy enter positive cycles of external activity, internal processes, and performance that enable long-term team success.</t>
@@ -1804,7 +1872,17 @@
       <c r="K22" s="0" t="n">
         <v>1992</v>
       </c>
-      <c r="P22" s="0" t="inlineStr"/>
+      <c r="L22" s="0" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="P22" s="0" t="inlineStr">
+        <is>
+          <t>Team level analysis. Verbatim Evidence: "Because much of the analysis was conducted at the group level, teams were included in the final sample only if at least three-fourths of their members responded. This reduced the number of teams in the final sample to 45. [...] The 409 individual responses to the 24 boundary-activity items were factor-analyzed to represent their underlying structure. Individuals' ratings of the extent to which they assumed responsibility for each of the 24 boundary activities were analyzed with a principal component analysis and a varimax rotation. Four factors with eigenvalues greater than 1.0 explained 60 percent of the total variance. Inspection of the Scree plot supported the four-factor solution. Factor scores were then calculated for each individual and averaged to form group scores." (Data and sample / Analysis and Results, Page 7-8)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="31">
       <c r="A23" s="0" t="inlineStr">
@@ -1917,8 +1995,24 @@
           <t>BSMA0022</t>
         </is>
       </c>
-      <c r="E25" s="0" t="inlineStr"/>
-      <c r="F25" s="0" t="inlineStr"/>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Innovation from differentiation</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>King</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
           <t>theory predicts that managers will create specialized boundary-spanning departments to insulate a firm from changing surrounding conditions. Theory also predicts such insulating structures will inhibit adaptation. I find that in response to
@@ -1945,7 +2039,17 @@
       <c r="K25" s="0" t="n">
         <v>1995</v>
       </c>
-      <c r="P25" s="0" t="inlineStr"/>
+      <c r="L25" s="0" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="P25" s="0" t="inlineStr">
+        <is>
+          <t>Firm level analysis. Verbatim Evidence: "The quantitative research measures the extent, nature and result of interaction between PC departments and core process personnel. Twelve rigid printed circuit firms agreed to participate in the written study and were sent questionnaires for the wet process, quality, and pollution control managers. Eight firms returned all three surveys, two returned two surveys, and two did not respond. I also sent performance surveys to the 12 firms with questions about quality, production cost, and treatment cost. I received responses from seven." (Quantitative Research Method, page 272)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="31">
       <c r="A26" s="0" t="inlineStr">
@@ -2554,8 +2658,24 @@
           <t>BSMA0035</t>
         </is>
       </c>
-      <c r="E38" s="0" t="inlineStr"/>
-      <c r="F38" s="0" t="inlineStr"/>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Invisible Foundations of Collaboration in the Workplace</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Baksa &amp; Branyiczki</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F38" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
           <t>The revolutionary advancement of technology in the past decade brought the attention of academics and management practitioners to ways of improving innovative capabilities of organizations. Advice-seeking relationships have an essential role in the knowledge production of modern-day organizations as they enable actors to acquire information, professional support and knowledge elements that they can recombine to form new knowledge. This paper conceptualizes advice-seeking behaviour as part of an inherently complex social world that can best be captured by a multiplex approach to organizational network research. It investigates how different layers of interpersonal relationships in the workplace may contribute to the appearance of advice-seeking interactions. This study examines the cases of three knowledge-intensive organizations and applies binary logistic regression to shed light on the yet invisible relational foundations of workplace collaboration. Implications for Central European audience: Central European countries attempt to improve their economic competitiveness by attracting knowledge-intensive companies as well as incentivizing innovation and digital transformation. Knowledge-intensive firms, such as business service centres or information and communication technology companies, are significant contributors to the economic output of countries such as the Czech Republic, Hungary and Poland. Recommendations derived from the results of this paper provide insights into the leadership of knowledge-intensive companies regarding creation of organizational environments that foster knowledge sharing and innovation. Measures that promote interpersonal trust, visibility of expertise and boundary-spanning behaviour are recommended.</t>
@@ -2579,7 +2699,17 @@
       <c r="K38" s="0" t="n">
         <v>2023</v>
       </c>
-      <c r="P38" s="0" t="inlineStr"/>
+      <c r="L38" s="0" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="P38" s="0" t="inlineStr">
+        <is>
+          <t>No bivariate Pearson correlation matrix provided. Verbatim Evidence: "Binary logistic regression analyses were run in SPSS Statistics for all three sample organizations, including advice seeking as a dependent variable and all other relational dimensions in Table 2 as independent variables. Two other categorical variables (same department and same hierarchy level) were also introduced to reflect the effect of the horizontal and vertical distance between actors on the willingness to ask for work-related help or advice. Binary logistic regression assumes that (1) the dependent variable is dichotomous, (2) there are no outliers in continuous variables, and (3) there is no multicollinearity (high correlations between independent variables) in the model. In this setting, the outcome was binary (advice-seeking behaviour is/is not present), no continuous independent variables were included, and all correlations between variables were low to moderate (Cramer’s V coefficients for categorical correlations were lower than 0.40 in all the cases)." (Results, page 12)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1" s="31">
       <c r="A39" s="0" t="inlineStr">
@@ -2942,8 +3072,24 @@
           <t>BSMA0043</t>
         </is>
       </c>
-      <c r="E46" s="0" t="inlineStr"/>
-      <c r="F46" s="0" t="inlineStr"/>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>The impact of perceived customer delight on the frontline employee</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Barnes et al.</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F46" s="0" t="n">
+        <v>0</v>
+      </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
           <t>A plethora of research has investigated the impact of the frontline employee on the customer, with the consensus that employees can have a tremendous impact on the customer. What remains to be discovered is the extent to which this relationship exists in the reverse. Utilizing broaden-and-build and emotional contagion theories, this study suggests that employee perceptions of a specific customer emotion (delight) have an impact on the frontline employee. Specifically, results from a structural equations model reveal that employee perceptions of customer delight lead to employee positive affect, which in turn positively influences commitment and job satisfaction as well as creates stronger external representation behaviors, internal influence behaviors, and service delivery behaviors from the employee. These findings contribute new evidence to the debate of the viability of providing customer delight and extend our knowledge beyond emotional contagion in explaining how positive customer emotions manifest in employees.</t>
@@ -2967,6 +3113,11 @@
       <c r="K46" s="0" t="n">
         <v>2015</v>
       </c>
+      <c r="L46" s="0" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
       <c r="P46" s="0" t="inlineStr"/>
     </row>
     <row r="47" ht="18" customHeight="1" s="31">
@@ -2980,8 +3131,24 @@
           <t>BSMA0044</t>
         </is>
       </c>
-      <c r="E47" s="0" t="inlineStr"/>
-      <c r="F47" s="0" t="inlineStr"/>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>The Impact of Role Variables on IS Personnel Work Attitudes and Intentions</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Baroudi</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F47" s="0" t="n">
+        <v>0</v>
+      </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
           <t>This study examines the antecedents cf job satisfaction, commitment, and turnover intentions for 229 information systems (IS) personnel employed within several industries. The antecedents studied include boundary spanning, role ambiguity, and rcle conflict. A model of these variables was built and tested using path analysis- Rcle ambiguity was found tc be the mcst dysfunctional variable for IS personnel, acccunting fcr 10.3%. 20.2% and 22.2% Of the variance in turnover intenticns. commitment, andjob satisfaction. This information is used tc make recommendaticns to IS management. Finally, recommendaticns and directions are suggested regarding future research.</t>
@@ -3004,6 +3171,11 @@
       </c>
       <c r="K47" s="0" t="n">
         <v>1985</v>
+      </c>
+      <c r="L47" s="0" t="inlineStr">
+        <is>
+          <t>1985</t>
+        </is>
       </c>
       <c r="P47" s="0" t="inlineStr"/>
     </row>
@@ -3068,8 +3240,24 @@
           <t>BSMA0046</t>
         </is>
       </c>
-      <c r="E49" s="0" t="inlineStr"/>
-      <c r="F49" s="0" t="inlineStr"/>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Social Comparisons in Boundary-Spanning Work</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Bartel</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F49" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
           <t>This research investigated how experiences in a particular boundary-spanning context (community outreach) affected members' organizational identity and identification. Multimethod panel data from 219 participants showed that intergroup comparisons with clients (emphasizing differences) and intragroup comparisons with other organization members (emphasizing similarities) changed how members construed their organization's defining qualities. Intergroup comparisons also enhanced the esteem members derived from organizational membership, which, in turn, strengthened organizational identification. Supervisors reported higher interpersonal cooperation and work effort for members whose organizational identification became stronger. The results reveal potential outcomes of boundary-spanning work as well as how organizational identification processes operate in everyday work contexts.</t>
@@ -3093,7 +3281,17 @@
       <c r="K49" s="0" t="n">
         <v>2001</v>
       </c>
-      <c r="P49" s="0" t="inlineStr"/>
+      <c r="L49" s="0" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="P49" s="0" t="inlineStr">
+        <is>
+          <t>No effect size for boundary spanning behavior. The study examines the effects of a boundary-spanning context (community outreach programs) on organizational identity and identification, but does not include a quantitative measure or correlation for boundary spanning behavior itself. Verbatim Evidence: "A series of regression analyses tested the hypothesized relationships between favorable client comparisons, collective self-esteem (CSE), and strength of organizational identification (OI). Table 4 contains zero-order correlations for pre-program and post-program variables (N = 144). For simplicity, I refer to these pre- and post-program variables numerically (e.g., CSE-1 versus CSE-2 and OI-1 versus OI-2) in subsequent analyses. I tested hypothesis 2 (the greater the extent of favorable client comparisons, the higher the level of collective self-esteem) and hypothesis 3 (collective self-esteem mediates the positive effect of extent of favorable client comparisons on strength of organizational identification) using the three-stage mediated regression approach recommended by Baron and Kenny (1986)." (Results, Page 22)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="31">
       <c r="A50" s="0" t="inlineStr">
@@ -3156,8 +3354,24 @@
           <t>BSMA0048</t>
         </is>
       </c>
-      <c r="E51" s="0" t="inlineStr"/>
-      <c r="F51" s="0" t="inlineStr"/>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Personal Communication Ties and Organizational Collaborations</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Basov &amp; Minina</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F51" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
           <t>The literature suggests that the success of innovation clusters is based on personal networks that connect members of scientific, educational, and business organizations, stimulating more formalized cross-boundary collaborations between the three sectors. But it is still unclear if such organizational collaborations actually correspond with these personal ties and which aspects of personal communication are most strongly associated with organizational collaborations. To investigate these issues, the authors applied network analysis to study an innovation cluster in Algarve, Portugal. They found that cross-boundary organizational collaborations corresponded with personal ties. Moreover, they found that collaborations appeared to correlate most strongly with emotional attachments between individuals.</t>
@@ -3181,7 +3395,17 @@
       <c r="K51" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P51" s="0" t="inlineStr"/>
+      <c r="L51" s="0" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="P51" s="0" t="inlineStr">
+        <is>
+          <t>The study aggregates personal ties to the organizational level and analyzes interorganizational network correlations rather than individual-level correlations. Verbatim Evidence: "We aggregated the survey data by mapping each unique combination of an organizational entity and a contact’s name as a separate node. Thus, when an individual was a member of more than one entity—for example, a company and a faculty—one node was recorded for the company and another for the faculty, following the interlocking directorate tradition (Burt, 1980). The resulting network, then, included 155 nodes linked with ties of strength varying from 0 to 4. The nodes representing members of more than one entity were linked with ties of maximal strength. Next, we produced three networks connecting the 25 organizations included in the analysis and representing different aspects of personal ties: (a) frequent personal communication, (b) strong intellectual influence, and (c) strong emotional attachments. To do so, for each of the three aspects of personal ties, we took the average of the strengths of all the ties connecting the employees of every dyad of organizations. The resulting average numbers were considered as the strengths of personal ties between the organizations in each of the three networks." (Networks of Personal Ties, Page 15)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="31">
       <c r="A52" s="0" t="inlineStr">
@@ -3194,8 +3418,24 @@
           <t>BSMA0049</t>
         </is>
       </c>
-      <c r="E52" s="0" t="inlineStr"/>
-      <c r="F52" s="0" t="inlineStr"/>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>Workplace spirituality</t>
+        </is>
+      </c>
+      <c r="D52" s="0" t="inlineStr">
+        <is>
+          <t>Bayighomog &amp; Araslı</t>
+        </is>
+      </c>
+      <c r="E52" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F52" s="0" t="n">
+        <v>0</v>
+      </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
           <t>Customer engagement entails unequivocal frontline service employees’ top performances and recommendable behaviors through management appropriate leadership to ﬂourish. Under the social exchange and social identity theories, this study investigates employee customer–oriented boundary-spanning behaviors as an outcome of spiritual leadership, through the mediating eﬀect of employee spiritual survival and well-being. PROCESS macro was used to analyze data collected from 5-star hotels full-time frontline employees in Antalya, Turkey. Results indicated that the eﬀect of spiritual leadership on the three dimensions of customer-oriented boundary-spanning behaviors is fully mediated by spiritual survival and spiritual well-being. Spirituality appears to be a noteworthy but remote contributor to customer engagement via employees’ boundary-spanning behaviors. Our study contributed to the boundary-spanning and customer engagement literature by illustrating that a sense of mission and wellbeing at the workplace are adequate requirements to engage a frontline employee, whose boundaryspanning behaviors will be instrumental in fostering customer engagement. Further detailed theoretical and managerial implications are discussed.</t>
@@ -3219,6 +3459,11 @@
       <c r="K52" s="0" t="n">
         <v>2019</v>
       </c>
+      <c r="L52" s="0" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
       <c r="P52" s="0" t="inlineStr"/>
     </row>
     <row r="53" ht="18" customHeight="1" s="31">
@@ -3232,8 +3477,24 @@
           <t>BSMA0050</t>
         </is>
       </c>
-      <c r="E53" s="0" t="inlineStr"/>
-      <c r="F53" s="0" t="inlineStr"/>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>Boundary spanning and gatekeeping roles of UK audit committees</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t>Beattie et al.</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F53" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
           <t>Post financial crisis, audit committee (AC) reforms are proposed to improve the quality of financial reporting (EC 2011; Competition Commission 2013). This paper’s empirical contribution is to investigate the extent to which ACs and audit committee chairs (ACCs) engage with chief financial officers (CFOs) and audit partners (APs) across a range of 32 financial reporting issues. It is the first large-scale survey of interactions to move beyond the micro CFO / AP dyad and to distinguish the individual ACC from the AC group. While 37% of the 5,445 reported discussions involve all three key individuals together with the full AC, 35% involve neither the AC nor the ACC and the ACC acts without the full AC in a significant minority of cases. The parties reported to be involved are similar across the three respondent groups but vary with financial reporting issue, company size and audit firm size. The paper’s theoretical contribution is to interpret the evidence using the concepts of boundary spanning and gatekeeping roles. The research reveals incomplete levels of AC and ACC engagement with financial reporting issues. Findings have implications for policymakers regarding the role, influence and effectiveness of the AC in financial reporting matters. Directions for future research are identified.</t>
@@ -3257,7 +3518,17 @@
       <c r="K53" s="0" t="n">
         <v>2014</v>
       </c>
-      <c r="P53" s="0" t="inlineStr"/>
+      <c r="L53" s="0" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="P53" s="0" t="inlineStr">
+        <is>
+          <t>The study reports descriptive statistics, frequencies, and percentages regarding the parties involved in audit discussions, but it does not provide a bivariate Pearson correlation matrix including boundary spanning behavior. Verbatim Evidence: "Across all potential discussion issues, the combined sample reported 5,445 discussions. The parties involved in these discussions are shown in Table 5, which reports frequencies for the 15 combinations. The most common set of parties involved in discussions was all four (37%), followed by the CFO / AP dyad (28%). Detailed results by company size and audit firm tier are shown in the Appendix. To facilitate further analysis of this data (Tables 6), we focussed on the two groupings of the reported combinations considered to be of the greatest interest. The groupings are as follows: No AC or ACC (both the full AC and the ACC left out, i.e. combinations 1, 2 and 5 shown in Table 5); Presence of ACC but absence of full AC in discussion (i.e. combinations 3, 6, 8 and 11)." (5.3 Parties involved in interactions (RQ 3 and RQ 4(a)), Pages 22-23)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1" s="31">
       <c r="A54" s="0" t="inlineStr">
@@ -3320,8 +3591,24 @@
           <t>BSMA0052</t>
         </is>
       </c>
-      <c r="E55" s="0" t="inlineStr"/>
-      <c r="F55" s="0" t="inlineStr"/>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>The Role of Leader Boundary Activities in Enhancing</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>Benoliel and Somech</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
           <t>This study examined how leaders’ internal and external activities mediate the relationship of functional heterogeneity and interteam goal interdependence to team effectiveness (in-role performance and innovation) in interdisciplinary teams. The results of the structural equation model from a sample of 92 interdisciplinary teams indicate that leaders’ internal activities fully mediate the relationship of team functional heterogeneity and interteam goal interdependence to team in-role performance. The leaders’ external activities were found to fully mediate the relationship of interteam goal interdependence to team innovation. We discuss the implications of these findings for both theory and practice.</t>
@@ -3345,7 +3632,17 @@
       <c r="K55" s="0" t="n">
         <v>2015</v>
       </c>
-      <c r="P55" s="0" t="inlineStr"/>
+      <c r="L55" s="0" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="P55" s="0" t="inlineStr">
+        <is>
+          <t>Team level analysis. Verbatim Evidence: "In the research hypotheses, the team is identified as the unit of analysis. Therefore, team innovation and team in-role performance were assessed by the team leader, the principal. Interteam goal interdependence and leader internal and external activities were represented by an aggregate of team member responses. Thus, it was critical to demonstrate high within-team agreement to justify using the team average as an indicator of team-level variables; a value of .70 or greater is suggested as an adequate amount of within-group interrater agreement (rWG, James, Demaree, &amp; Wolf, 1993). In the current study, all scales exceeded this level (see Table 1). Prior to aggregating individual-level scores to the group level by mean, intraclass correlations (ICC) were calculated." (Level of Analysis, Pages 100-102)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1" s="31">
       <c r="A56" s="0" t="inlineStr">
@@ -3358,8 +3655,24 @@
           <t>BSMA0053</t>
         </is>
       </c>
-      <c r="E56" s="0" t="inlineStr"/>
-      <c r="F56" s="0" t="inlineStr"/>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t>How and when Identification with a Boundary‐Spanning</t>
+        </is>
+      </c>
+      <c r="D56" s="0" t="inlineStr">
+        <is>
+          <t>Bergami et al.</t>
+        </is>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F56" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
           <t>Membership of boundary‐spanners is controversial, as employees operate largely at the borders of the organization in close relations with customers. Nevertheless, we know little about its influence on customer satisfaction. We investigate how and when identification with the branch influences customer satisfaction. The how question is answered by showing that degree of control of one's performance mediates the impact of branch manager identification on customer satisfaction. The when question is answered by proposing two moderating variables. Locus of control regulates the extent to which identification influences performance control. Dedicated meetings between branch managers and their colleagues regulate the degree to which performance control influences customer satisfaction. Hypotheses were tested in a longitudinal design on a sample of 1,461 managers from a firm specializing in banking and financial services in Europe. Results largely confirm our hypotheses, providing a novel look on determinants of customer satisfaction from the perspective of boundary‐spanning managers.</t>
@@ -3383,7 +3696,17 @@
       <c r="K56" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P56" s="0" t="inlineStr"/>
+      <c r="L56" s="0" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="P56" s="0" t="inlineStr">
+        <is>
+          <t>No boundary spanning behavior measure. Verbatim Evidence: "First, we address the question, how does manager identification with the local branch affect customer satisfaction? We answer this question by identifying a key mediating variable, appraisal of personal control over customer satisfaction, which functions to transform manager identification into customer satisfaction in four strategic senses noted below. Second, we speak to the question, when does manager identification lead to customer satisfaction (i.e., under what conditions does identification influence satisfaction)? To answer this question, we develop one moderator of the identification to control relationship and one moderator of the control to satisfaction relationship. The first moderator is an individual difference variable that regulates the extent to which identification leads to perceived control and resides in the personality trait of locus of control. The second moderator is an interpersonal, role-based variable that consists of regular dedicated meetings of employees involved with customer relations to discuss, plan, implement, and evaluate group efforts at attaining customer satisfaction. Figure 1 summarizes our moderated mediation model." (Introduction, page 94)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1" s="31">
       <c r="A57" s="0" t="inlineStr">
@@ -3396,8 +3719,24 @@
           <t>BSMA0054</t>
         </is>
       </c>
-      <c r="E57" s="0" t="inlineStr"/>
-      <c r="F57" s="0" t="inlineStr"/>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>Role Stressors and Customer-Oriented Boundary-Spanning</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t>Bettencourt and Brown</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F57" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
           <t>The authors investigate three types of customer-oriented boundary-spanning behaviors (COBSBs)a frontline service employee may perform that are associated with linking a service organization to its potential or actual customers: external representation, internal influence, and service delivery. The authors propose and test a withdrawal model to explain the negative effects of role conflict and role ambiguity on COBSBs across a sample of 220 lower-level, nonprofessional service providers of a major retail bank and a sample of 90 higher-level, professional service providers from the business credit division of an international financial services corporation. The results demonstrate that (1)indirect paths through job satisfaction and organizational commitment entirely account for the negative effects of the role stressors on COBSBs, (2) the indirect negative effects of the role stressors are stronger on external representation and internal influence behaviors, and (3)role conflict also has a significant positive direct relationship with internal influence behaviors.</t>
@@ -3421,7 +3760,17 @@
       <c r="K57" s="0" t="n">
         <v>2003</v>
       </c>
-      <c r="P57" s="0" t="inlineStr"/>
+      <c r="L57" s="0" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="P57" s="0" t="inlineStr">
+        <is>
+          <t>The study uses structural equation modeling and provides a latent construct intercorrelation matrix instead of a bivariate Pearson correlation matrix. Verbatim Evidence: "Construct reliability estimates provided in Table 2 also provide evidence of good levels of reliability (&gt; .70) for all measures except role conflict. Finally, discriminant validity was assessed by comparison of the squared correlation between two latent constructs with their average variance extracted (AVE) estimates (Fornell and Larcker 1981). Using the Fornell and Larcker (1981) test, discriminant validity was supported for all possible pairs of constructs in the retail banking sample and all but two pairs of constructs in the business credit sample. Organizational commitment and job satisfaction had a correlation of .85, and external representation and service delivery had a correlation of .69 and only passed less stringent tests of discriminant validity in the business credit sample." (Measurement Model Analyses, Page 401-402)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1" s="31">
       <c r="A58" s="0" t="inlineStr">
@@ -3434,8 +3783,24 @@
           <t>BSMA0055</t>
         </is>
       </c>
-      <c r="E58" s="0" t="inlineStr"/>
-      <c r="F58" s="0" t="inlineStr"/>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t>Customer-oriented boundary-spanning behaviors</t>
+        </is>
+      </c>
+      <c r="D58" s="0" t="inlineStr">
+        <is>
+          <t>Bettencourt et al.</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F58" s="0" t="n">
+        <v>0</v>
+      </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
           <t>Using a sample of 281 frontline service employees of a national retail bank, we test a social exchange model of antecedents of three dimensions of customer-oriented boundary-spanning behaviors suggested by prior boundary-spanning and services marketing/management literatures: external representation, internal inﬂuence, and service delivery. In support of our hypotheses, we identify fully mediated relationships from procedural, interactional, and distributive justice to external representation and internal inﬂuence via job satisfaction and organizational commitment. Our results generally support our expectation that the indirect effects of procedural justice on external representation and internal inﬂuence are stronger than the indirect effects of distributive or interactional justice on these behaviors. Also, our results reveal no signiﬁcant indirect effects of procedural and distributive justice on service delivery behaviors. However, we ﬁnd an unexpected direct positive path from interactional justice to service delivery behaviors. We interpret this latter ﬁnding in light of the normative value of interactional justice as a source of role modeling or managerial legitimacy.</t>
@@ -3458,6 +3823,11 @@
       </c>
       <c r="K58" s="0" t="n">
         <v>2005</v>
+      </c>
+      <c r="L58" s="0" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
       </c>
       <c r="P58" s="0" t="inlineStr"/>
     </row>
@@ -3572,8 +3942,24 @@
           <t>BSMA0058</t>
         </is>
       </c>
-      <c r="E61" s="0" t="inlineStr"/>
-      <c r="F61" s="0" t="inlineStr"/>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t>If the Supplier's Human Capital Walks Away, Where Would the Customer Go</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t>Biong and Ulvnes</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
           <t>Purpose: Professional service firms' clients often develop stronger attachments to their key contact employee than to the service firm. Since professionals are highly mobile, buyers of professional business services constantly have to decide whether to follow their key contact employee or remain with their incumbent firm, while service firms face the threat of losing customers if the employee leaves. This study examines how the key contact employee's human capital, the social capital between the contact employee and the client, and the service company's structural capital affect the decision whether to follow the key contact employee to another professional service firm.
@@ -3602,7 +3988,17 @@
       <c r="K61" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="P61" s="0" t="inlineStr"/>
+      <c r="L61" s="0" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="P61" s="0" t="inlineStr">
+        <is>
+          <t>The study lacks a measure of individual-level boundary spanning behavior, focusing instead on clients' likelihood to follow a key contact employee based on human, social, and structural capital. Verbatim Evidence: "The PLS model required to test the hypotheses included the main effects of the independent constructs (β1–β3), interaction terms (β4–β5), and control variables (β6–β8) on the likelihood of following the key contact employee. Essentially, this model captures clients’ perception on whether they would follow their key contact employee modelled as a function of client perception of the independent variables. Before we tested the hypotheses we investigated to what degree our results are influenced by outliers, with the Mahalanobis D2 measure and found that none of the cases have a Mahalanobis D2 with a probability less that or equal to 0.001." (Hypotheses Tests, Page 17)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1" s="31">
       <c r="A62" s="0" t="inlineStr">
@@ -3665,8 +4061,24 @@
           <t>BSMA0060</t>
         </is>
       </c>
-      <c r="E63" s="0" t="inlineStr"/>
-      <c r="F63" s="0" t="inlineStr"/>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t>GROUPS, BOUNDARY SPANNING, AND THE TEMPORAL IMAGINATION</t>
+        </is>
+      </c>
+      <c r="D63" s="0" t="inlineStr">
+        <is>
+          <t>Bluedorn and Standifer</t>
+        </is>
+      </c>
+      <c r="E63" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F63" s="0" t="n">
+        <v>4</v>
+      </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
           <t>The temporal imagination is the understanding of the intersection of one entity’s timescape with the larger timescapes of which that entity is a part. We examine in detail what the temporal imagination is, complemented with a discussion of the related timescape idea, and why the temporal imagination is necessary to function in any timescape. We also discuss group attributes that will likely affect the development of the temporal imagination and its use and how its use in group boundary spanning efforts affect both the groups and the larger organization.</t>
@@ -3690,7 +4102,17 @@
       <c r="K63" s="0" t="n">
         <v>2003</v>
       </c>
-      <c r="P63" s="0" t="inlineStr"/>
+      <c r="L63" s="0" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="P63" s="0" t="inlineStr">
+        <is>
+          <t>Conceptual paper without empirical data. Verbatim Evidence: "In this chapter, we have proposed the concept of the temporal imagination, not as a precisely defined theoretical construct that can be instantly operationalized to begin a program of empirical research, but like its sociological progenitor, as a sensitizing concept (Blumer, 1954). A sensitizing concept is a general idea that can point to phenomena that are potentially important (Blumer, 1954, p. 7). In this case, it points to them for time and group scholars to consider, perhaps to investigate." (CONCLUSION, Page 178)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1" s="31">
       <c r="A64" s="0" t="inlineStr">
@@ -3903,8 +4325,24 @@
           <t>BSMA0065</t>
         </is>
       </c>
-      <c r="E68" s="0" t="inlineStr"/>
-      <c r="F68" s="0" t="inlineStr"/>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t>Being in the Right Place A Structural Analysis of Individual Influence in an Organization</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t>Brass</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F68" s="0" t="n">
+        <v>0</v>
+      </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
           <t>This research examined the relationships between structural positions and influence at the individual level of analysis. The structure of the organization was conceptualized from a social network perspective. Measures of the relative positions of employees within workflow, communication, and friendship networks were strongly related to perceptions of influence by both supervisors and non-supervisors and to promotions to the supervisory level. Measures included criticality, transaction alternatives, and centrality (access and control) in the networks and in such reference groups as the dominant coalition. A comparison of boundary-spanning and technical-core personnel indicated that contacts beyond the normal work requirements are particularly important for technical core personnel to acquire influence. Overall, the results provide support for a structural perspective on intraorganizational influence.</t>
@@ -3927,6 +4365,11 @@
       </c>
       <c r="K68" s="0" t="n">
         <v>1984</v>
+      </c>
+      <c r="L68" s="0" t="inlineStr">
+        <is>
+          <t>1984</t>
+        </is>
       </c>
       <c r="P68" s="0" t="inlineStr"/>
     </row>
@@ -4175,8 +4618,24 @@
           <t>BSMA0070</t>
         </is>
       </c>
-      <c r="E73" s="0" t="inlineStr"/>
-      <c r="F73" s="0" t="inlineStr"/>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t>Dual commitment and boundary spanning activity of R&amp;D professionals</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t>Sexton</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F73" s="0" t="n">
+        <v>0</v>
+      </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
           <t>This dissertation examines the extent to which organizational and professional commitment, the technical environment, and the professional environment are related to boundary spanning activity. Surveys of R&amp;D professional employees, their co-workers, and their managers were used to obtain measures of commitment to their organizations and professions, perceptions of the technical and professional environment in which they worked, and the frequency with which they communicated both within and outside of the R&amp;D unit.</t>
@@ -4199,6 +4658,11 @@
       </c>
       <c r="K73" s="0" t="n">
         <v>1995</v>
+      </c>
+      <c r="L73" s="0" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
       </c>
       <c r="P73" s="0" t="inlineStr"/>
     </row>
@@ -4313,8 +4777,24 @@
           <t>BSMA0073</t>
         </is>
       </c>
-      <c r="E76" s="0" t="inlineStr"/>
-      <c r="F76" s="0" t="inlineStr"/>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t>Managing the Offshoring of Audit Work Spanning the Boundaries</t>
+        </is>
+      </c>
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t>Canning et al.</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F76" s="0" t="n">
+        <v>4</v>
+      </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
           <t>The offshoring of external audit work to so-called low-cost countries is prevalent among the Big 4 professional services firms. Despite this, our understanding of how this form of offshoring influences audit practitioners and the audit process is limited. This study examines how and why offshoring emerged as an organizational matter that changed the way audit work is organized in a Big 4 firm context. Our findings demonstrate how changes in the design of offshoring processes influence interactions between onshore and offshore auditors. We uncover how individual ‘‘boundary spanners’’ struggle to coordinate audit work across the multiple boundaries that separate onshore and offshore auditors. Furthermore, we show how the institutionalization of ‘‘boundary spanning’’ functions in organizational structures and processes can have the unintended consequence of widening the boundaries between onshore and offshore auditors. Finally, we offer evidence of the effect of offshoring on the learning process of onshore and offshore auditors.</t>
@@ -4338,7 +4818,17 @@
       <c r="K76" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P76" s="0" t="inlineStr"/>
+      <c r="L76" s="0" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="P76" s="0" t="inlineStr">
+        <is>
+          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: "Given that the objective of this study is to develop our understanding of how and why offshoring emerged as an organizational matter, changing the way audit work is organized and perceived in a Big 4 firm, a qualitative research methodology was deemed most appropriate (Cooper and Morgan 2008; Denzin and Lincoln 2003; Flick 2006; Given 2008; Silverman 2000). More specifically, we used a case study approach (Cooper and Morgan 2008) drawing upon multiple data sources—documentary data, in-depth interviews, and digital data—to obtain detailed information about the complexities underpinning the real-life phenomenon (Miles and Huberman 1994; Patton 2002) of offshoring in audit." (IV. RESEARCH METHOD, Page 64)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="18" customHeight="1" s="31">
       <c r="A77" s="0" t="inlineStr">
@@ -4501,8 +4991,24 @@
           <t>BSMA0077</t>
         </is>
       </c>
-      <c r="E80" s="0" t="inlineStr"/>
-      <c r="F80" s="0" t="inlineStr"/>
+      <c r="C80" s="0" t="inlineStr">
+        <is>
+          <t>Invisible network drivers of women’s success</t>
+        </is>
+      </c>
+      <c r="D80" s="0" t="inlineStr">
+        <is>
+          <t>Carboni et al.</t>
+        </is>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F80" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
           <t>Gender diversity pays off, particularly at senior levels in organizations. Companies with higher rates of gender diversity among senior leaders outperform their peers by a 15% margin; those with the highest percentages of female board directors enjoy as much as a two-thirds higher return on equity, sales, and invested capital. The key to occupying a high-level position in any organization is building an effective network of positive workplace relationships. Decades of research on organizational networks have shown that who you know–and who knows you–is critical to performance and career success. Full inclusion of both genders in informal organizational networks has been shown to drive productivity, innovation, and profitability. Full inclusion also supports individual well-being and deep engagement. Yet many leaders–both men and women–fail to develop gender-inclusive networks, potentially disadvantaging women since they are less likely to be connected to people in senior-level positions, given the overwhelming dominance of men in these roles. No wonder that feeling excluded from organizational networks has been identified as one of women’s top barriers to career success.</t>
@@ -4526,7 +5032,17 @@
       <c r="K80" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P80" s="0" t="inlineStr"/>
+      <c r="L80" s="0" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="P80" s="0" t="inlineStr">
+        <is>
+          <t>The study is a practitioner-oriented piece that mentions quantitative data collection but fails to report any statistical effect sizes, specifically lacking an individual-level Pearson correlation matrix. Verbatim Evidence: "Organizational Network Analysis (ONA) is grounded in the idea that formal structures in organizations do not reflect the actual patterns of connection in an organization. Our data captured the networks of more than 16,500 individuals in 31 different companies via web-based surveys. To ensure that we accurately represented each organization’s network, we collected responses from at least 80% of organizational members in every organization. Each individual was asked to name the people in their organization to whom they turned for “important work-related information” and about whom they said that interactions with this person left them “feeling more energized, with a sense of enthusiasm and/or that your work really matters.”" (Insert: About the Research, Page 30)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="18" customHeight="1" s="31">
       <c r="A81" s="0" t="inlineStr">
@@ -5133,8 +5649,24 @@
           <t>BSMA0090</t>
         </is>
       </c>
-      <c r="E93" s="0" t="inlineStr"/>
-      <c r="F93" s="0" t="inlineStr"/>
+      <c r="C93" s="0" t="inlineStr">
+        <is>
+          <t>Driving lateral collaboration effectiveness across multinational enterprises</t>
+        </is>
+      </c>
+      <c r="D93" s="0" t="inlineStr">
+        <is>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="E93" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F93" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
           <t>In the face of increasing global uncertainty, multinational enterprises (MNEs) have turned to downsizing to maintain profitability while emphasizing lateral collaboration to increase productivity. Here, we establish a conceptual framework and examine from a macro‐to‐micro perspective how the growing subjects of subsidiary role change, team alignment and employee engagement impact lateral collaboration. We used structural equation modelling to analyse the results of 252 surveys given to MNE subsidiaries in the Taiwanese banking industry and found that employee engagement was central to driving lateral collaboration effectiveness, indicating that the subsidiary role is critical for boundary‐spanning activities and building bridges between various teams. These activities in turn enhance subsidiary performance and lead to better people development. Our findings demonstrate that bundling employee engagement with human resource practices is a strategic way of positioning for the evolution of subsidiary management.</t>
@@ -5158,7 +5690,17 @@
       <c r="K93" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P93" s="0" t="inlineStr"/>
+      <c r="L93" s="0" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="P93" s="0" t="inlineStr">
+        <is>
+          <t>No boundary spanning behavior measured. Verbatim Evidence: "Lateral collaboration effectiveness is a crucial process for commitment integration that satisfies the concerns of each relevant party involved in any business exchange (Harrison &amp; New, 2002). Normative commitments encourage a subsidiary employee to comply with the MNEs' requirement set for bureaucratic control with ‘a sense of obligation that derives from the internalization of normative influences’ (Meyer &amp; Parfyonova, 2010). Affective commitments capture the subsidiary employees' emotional identification, engagement and attachment to the MNE, which are associated with employees' desire to contribute to the benefit of the firm (Meyer &amp; Allen, 1991). By committing in these ways to the efforts of the team and organization, employees transcend their formal roles and increase their potential to make impactful contributions to the effectiveness of the organization (Wombacher &amp; Felfe, 2017). We therefore consider the exercise of commitment as a form of lateral collaboration that can be enhanced to achieve the expected people development and subsidiary performance." (Lateral collaboration effectiveness and its consequences, Page 5-6)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="18" customHeight="1" s="31">
       <c r="A94" s="0" t="inlineStr">
@@ -5271,8 +5813,24 @@
           <t>BSMA0093</t>
         </is>
       </c>
-      <c r="E96" s="0" t="inlineStr"/>
-      <c r="F96" s="0" t="inlineStr"/>
+      <c r="C96" s="0" t="inlineStr">
+        <is>
+          <t>Changing Practices for an Innovative Care Pathway</t>
+        </is>
+      </c>
+      <c r="D96" s="0" t="inlineStr">
+        <is>
+          <t>Cherkaoui et al.</t>
+        </is>
+      </c>
+      <c r="E96" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F96" s="0" t="n">
+        <v>4</v>
+      </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
           <t>Getting professionals who have been selected and trained to perform individually to work together is a major challenge. The objective of the article is to identify the mechanisms by which a coordinator can ensure a mediation and boundary spanning role to enable the achievement of a project. Adopting a comprehensive approach, this article is based on the case of an innovative hospital project ‘One-Day Diagnosis’ (1DD) – one day instead of several weeks – of hepatobiliary and pancreatic pathologies, for which the professionals had to change their practices. Based on the results of the study, the ﬁndings show that the mediating role of the coordinator consists in making things happen and guiding health care professionals through the innovative pathway until it becomes a routine process. The study contributes to the literature on collaboration and relational coordination by highlighting that the change of practices for collaboration is compatible with personal excellence, by outlining the active role of the boundary spanner in the change of these practices and by demonstrating that the organizational stability of projects based on disembodied procedures is a necessary illusion that requires complementary interindividual relationships and a living leadership.</t>
@@ -5296,7 +5854,17 @@
       <c r="K96" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P96" s="0" t="inlineStr"/>
+      <c r="L96" s="0" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="P96" s="0" t="inlineStr">
+        <is>
+          <t>Qualitative interview study. Verbatim Evidence: "The study that we conducted is based on semi-structured interviews among HCPs who participate directly in the 1DD care pathway or work closely with it. We interviewed 19 HCPs between April and July 2019, knowing that the innovative organization was set up in January 2017. We contacted each HCP in person or by e-mail. The participants received information on the relevance and design of the study, the problem, the central concepts of the study and the way the results would be distributed. Each participant explicitly consented to participate in the study. The interviews were conducted individually by the same interviewer, following the same outline." (The Research Process, Page 56)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="18" customHeight="1" s="31">
       <c r="A97" s="0" t="inlineStr">
@@ -5355,8 +5923,24 @@
           <t>BSMA0095</t>
         </is>
       </c>
-      <c r="E98" s="0" t="inlineStr"/>
-      <c r="F98" s="0" t="inlineStr"/>
+      <c r="C98" s="0" t="inlineStr">
+        <is>
+          <t>NPD Projects in Search of Top Management Support</t>
+        </is>
+      </c>
+      <c r="D98" s="0" t="inlineStr">
+        <is>
+          <t>Chollet et al.</t>
+        </is>
+      </c>
+      <c r="E98" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F98" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
           <t>A number of studies have found that the performance of NPD projects greatly depends on the support they get from top management. However, research into why some projects get more support than others has been limited. The present paper takes a political approach to NPD, in which top management support is considered to be a function of a project leader’s ability to influence decision processes through personal relationships. Mobilizing the bridging perspective of social capital, we argue that project leaders need both strong ties to high-ranking others and sparseness in their networks. Vertical strong ties bring direct support and solidarity, resulting in improved access to resources and priority over other projects; sparseness provides exposure to the full range of information and interpretations in the organization, resulting in a more accurate picture of the political landscape and thus enabling the implementation of an appropriate influence strategy. A PLS analysis of a sample of 73 French project leaders involved in NPD projects provided support for our hypotheses. Hence, we contribute to a very recent stream of research showing that the structural and relational dimensions of social capital are complementary.</t>
@@ -5380,7 +5964,17 @@
       <c r="K98" s="0" t="n">
         <v>2012</v>
       </c>
-      <c r="P98" s="0" t="inlineStr"/>
+      <c r="L98" s="0" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="P98" s="0" t="inlineStr">
+        <is>
+          <t>Project level analysis. Verbatim Evidence: "After two follow-up emails sent after 10 and 20 days, we obtained 243 completed questionnaires (response rate of 31%). To ensure that our study was based on a homogenous sample, we crossed the sector variable with the nature of the project variable (new product/service, new process) and selected only projects involving the design of new products/services. This reduced the sample to 83 questionnaires. As 10 of these questionnaires were incomplete, our final sample consisted of 73 valid questionnaires completed by NPD project leaders." (Sample and data collection, Page 12)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="18" customHeight="1" s="31">
       <c r="A99" s="0" t="inlineStr">
@@ -5543,8 +6137,24 @@
           <t>BSMA0099</t>
         </is>
       </c>
-      <c r="E102" s="0" t="inlineStr"/>
-      <c r="F102" s="0" t="inlineStr"/>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>BRIDGING THE GAP MANAGERS' EXTERNAL RELATIONSHIPS AND THEIR EFFECTS</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Cohen</t>
+        </is>
+      </c>
+      <c r="E102" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F102" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="G102" s="0" t="inlineStr">
         <is>
           <t>In this dissertation, I develop a conceptual model for how managers' roles as boundary spanners within their organizations affect the perceptions, attitudes, relationships, and performance of their subordinate employees. Drawing on literatures in social networks, status characteristics theory, social identity theory, and resource allocation theory, I suggest that managers' external relationships—the connections that managers make to organization members outside of their subordinate work group—have a material impact on their subordinates' perceptions of their work environment and their managers. These perceptions, I argue, serve as four specific mechanisms in an indirect effects model that connect managers' external relationship to their employees' task performance and work attitudes (eg organizational commitment) and the Leader Member Exchange (LMX) relationships between manager and subordinate. I apply the theoretical model to two salient types of managerial relationships: those with their bosses and those with their horizontal peers.</t>
@@ -5568,7 +6178,17 @@
       <c r="K102" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="P102" s="0" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="P102" s="0" t="inlineStr">
+        <is>
+          <t>Multilevel analysis with boundary spanning measured at the group level. Verbatim Evidence: "In this study, the data have a nested structure with individual subordinates nested within managers. Constructs regarding the manager exist at the group level of analysis whereas constructs about subordinate employees exist at the individual level of analysis. In the first stage of the indirect effects model, the hypotheses are cross level in nature with manager level effects (for example, external relationships and transformational leadership) predicting individual level outcomes (for example, information access or perceived manager status)." (IV.6 Analytical considerations, Page 76)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="18" customHeight="1" s="31">
       <c r="A103" s="0" t="inlineStr">
@@ -5581,8 +6201,24 @@
           <t>BSMA0100</t>
         </is>
       </c>
-      <c r="E103" s="0" t="inlineStr"/>
-      <c r="F103" s="0" t="inlineStr"/>
+      <c r="C103" s="0" t="inlineStr">
+        <is>
+          <t>A COGNITIVE LOAD VIEW AND EMPIRICAL TEST OF COLLABORATION NETWORK</t>
+        </is>
+      </c>
+      <c r="D103" s="0" t="inlineStr">
+        <is>
+          <t>Colazo</t>
+        </is>
+      </c>
+      <c r="E103" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F103" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
           <t>This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates, with a secondary goal of testing product complexity as a moderator. We develop suitable hypotheses under the theoretical lens of cognitive load theory. The empirical study uses archival data on an ordinary least squares model to find significant associations between collaboration structure, product complexity and the learning rates exhibited by 230 development teams producing open source software. Results show two distinct subgroups of projects: The first subgroup exhibits an average 78% learning rate, and the other subgroup “unlearned”, i.e., productivity deteriorated over time instead of improved. In the learning subgroup, collaboration network density negatively impacted learning, while product complexity interacted with collaboration network centralisation and boundary spanning activity. In the unlearning subgroup, only network density impacted learning rates and no moderating effects were found. Practical implications and future opportunities for research are discussed.</t>
@@ -5606,7 +6242,17 @@
       <c r="K103" s="0" t="n">
         <v>2016</v>
       </c>
-      <c r="P103" s="0" t="inlineStr"/>
+      <c r="L103" s="0" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="P103" s="0" t="inlineStr">
+        <is>
+          <t>Project level analysis. Verbatim Evidence: "In the SF repository, there were 587 software projects being developed by six or more core team members and using “C”. These projects constituted the sampling frame. The final sample was reduced to 230 projects (39% of the sampling frame) because only that number had archived full data on all development activities. In spite of the non-probabilistic nature of the sample (see limitations), it contained projects with varied types of applications, sizes, and degrees of complexity. The unit of analysis was the OSS project." (Sampling, Page 13-14)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="18" customHeight="1" s="31">
       <c r="A104" s="0" t="inlineStr">
@@ -5619,8 +6265,24 @@
           <t>BSMA0101</t>
         </is>
       </c>
-      <c r="E104" s="0" t="inlineStr"/>
-      <c r="F104" s="0" t="inlineStr"/>
+      <c r="C104" s="0" t="inlineStr">
+        <is>
+          <t>COLLABORATION STRUCTURE AND PERFORMANCE IN NEW SOFTWARE DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="D104" s="0" t="inlineStr">
+        <is>
+          <t>Colazo</t>
+        </is>
+      </c>
+      <c r="E104" s="0" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F104" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="G104" s="0" t="inlineStr">
         <is>
           <t>The state of software development performance is far from being exemplar, with a success rate well below that of other industries, and understanding how to improve these projects is not only substantive but urgent. Software development is at most times a collaborative effort, yet we do not understand clearly how different collaboration structures associate with development performance metrics. This paper empirically examines the association between collaboration patterns, project productivity and product quality through a field study of working software open source new product development teams, using archival data from electronic sources related to Open Source Software projects. Collaboration structures are measured using Social Network Analysis and in terms of their network density, network centralization and the level of boundary spanning activity of team members. Productivity and quality are measured using "hard", code-based metrics. Results of regression analyses testing relevant hypotheses suggest that project managers need to strongly encourage internal collaboration, but be wary of allowing team members to participate in multiple projects. The breadth of skills within the team is a tactical asset that may increase the efficient frontier in the quality–productivity trade-off. Results also show that centralized structures associate with higher product quality and development productivity.</t>
@@ -5644,7 +6306,17 @@
       <c r="K104" s="0" t="n">
         <v>2010</v>
       </c>
-      <c r="P104" s="0" t="inlineStr"/>
+      <c r="L104" s="0" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="P104" s="0" t="inlineStr">
+        <is>
+          <t>Project level analysis. Verbatim Evidence: "The unit of analysis was the NPD project. OSS project information is hosted in web-based repositories which have been used repeatedly as sources of archival data for empirical studies (Mockus et al., 2002). Similarly, this paper uses Source Forge (SF) (www.sourceforge.net) which is the paramount OSS project repository. The software projects selected were those developed in the programming language “C”, by six or more team members. This minimum number of team members was chosen to avoid any bias from the large number of one-person projects in SF, while still maintaining a reasonable variability range in the network-based measures." (Sampling, Page 10)
+&lt;/SYSTEM_MESSAGE&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="18" customHeight="1" s="31">
       <c r="A105" s="0" t="inlineStr">

</xml_diff>

<commit_message>
chore: apply batch 4.2 results
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -6137,12 +6137,12 @@
           <t>BSMA0099</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C102" s="0" t="inlineStr">
         <is>
           <t>BRIDGING THE GAP MANAGERS' EXTERNAL RELATIONSHIPS AND THEIR EFFECTS</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D102" s="0" t="inlineStr">
         <is>
           <t>Cohen</t>
         </is>
@@ -6178,7 +6178,7 @@
       <c r="K102" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="L102" t="inlineStr">
+      <c r="L102" s="0" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
@@ -8445,7 +8445,7 @@
     <row r="149" ht="18" customHeight="1" s="31">
       <c r="A149" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B149" s="0" t="inlineStr">
@@ -8453,13 +8453,11 @@
           <t>BSMA0146</t>
         </is>
       </c>
-      <c r="E149" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E149" s="0" t="n">
+        <v>0</v>
       </c>
       <c r="F149" s="0" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G149" s="0" t="inlineStr">
         <is>
@@ -8486,15 +8484,14 @@
       </c>
       <c r="P149" s="0" t="inlineStr">
         <is>
-          <t>Firm level analysis. Verbatim Evidence: "Scholars have studied boundary spanning roles at the individual (e.g., Perrone, Zaheer, &amp; McEvily, 2003) and organizational levels (e.g., Scott, 1998). However, this study’s focus is at the organizational level and specific to the role of managing the interface between organization and environment. In such instances, two roles are primary: information processing and external representation. The first role is in helping the organization learn and perform according to variation in the environment, while the second role helps maintain legitimacy of the organization and its activities by transmitting favorable information (Aldrich, 1979)." (Conceptual background and hypothesis development, page 3)
-&lt;/SYSTEM_MESSAGE&gt;</t>
+          <t>0 = Exclude\nReason Code: 1\nNo effect size for BSB. Verbatim Evidence: \"The purpose of this study is to explore the relationships among self-monitoring, job tenure, and performance for a sample of job incumbents who occupy a boundary-spanning position. ... To test the hypotheses, two constructs were assessed: job performance and attention to social cues. Performance level was obtained from company performance evaluation forms, which provide, in part, a single, overall performance rating. ... Attention to social cues was measured using the Self-Monitoring Scale.\" (Method, page 125)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="150" ht="18" customHeight="1" s="31">
       <c r="A150" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B150" s="0" t="inlineStr">
@@ -8502,13 +8499,11 @@
           <t>BSMA0147</t>
         </is>
       </c>
-      <c r="E150" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E150" s="0" t="n">
+        <v>0</v>
       </c>
       <c r="F150" s="0" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G150" s="0" t="inlineStr">
         <is>
@@ -8535,15 +8530,14 @@
       </c>
       <c r="P150" s="0" t="inlineStr">
         <is>
-          <t>Departmental/firm level of analysis. Verbatim Evidence: "Logistics managers were asked to evaluate several statements about their firms’ reward and evaluation systems (based on a 7-point scale: 1  strongly disagree; 7  strongly agree). The overall mean score for the scale was 4.67, suggesting that logistics managers have only moderately favorable perceptions of their firms’ evaluation and reward systems. Most significantly, respondents somewhat disagreed with the statement that “evidence of cooperation between departments is acknowledged by superiors in this organization” (3.35 based on a 7-point scale). The relative lack of recognition for the advisability of interdepartmental cooperation is borne out by low mean scores for the cross-functional collaboration and the effectiveness of interdepartmental relation scales. Managers were asked to indicate to what degree the logistics department had pursued various collaborative activities with the marketing department over the last six months (based on a 5-point scale; 1  never; 5  quite frequently)." (Evaluation of Mean Scores, Page 5)
-&lt;/SYSTEM_MESSAGE&gt;</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative comparative analysis of ethnographies. Verbatim Evidence: \"In it I carry out a comparison of four narratives that American ethnographers have produced. Following in one major tradition of anthropological and sociological research (Ragin, 1987, pp. 34–52), I am using case-oriented qualitative comparison to explore the insights that may result from work with a neglected part of the intercultural literature.\" (Introduction, Page 61)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="151" ht="18" customHeight="1" s="31">
       <c r="A151" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B151" s="0" t="inlineStr">
@@ -8551,15 +8545,11 @@
           <t>BSMA0148</t>
         </is>
       </c>
-      <c r="E151" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F151" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E151" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G151" s="0" t="inlineStr">
         <is>
@@ -8586,7 +8576,7 @@
       </c>
       <c r="P151" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"Data were collected by survey instrument from the owner/operators of four different types of small business organizations. There were 38 retail firms (food and apparel) and 44 manufacturing firms (food and apparel). Subjects were selected at random from phone directories in the Allentown-Bethlehem-Easton Pennsylvania SMSA. Of the owner/operators contacted by phone prior to mailing the survey, 180 met the inclusion criteria. The criteria were: firm be owner operated (≥ 51 percent ownership), firm have between 2 and 100 employees, firm be in operation one year or longer. [...] Performance was measured by net addition to retained earnings, current sales, and the gross economic benefits accruing to ownership for 1981.\" (Method &amp; Measures, Pages 355, 357)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -8643,7 +8633,7 @@
     <row r="153" ht="18" customHeight="1" s="31">
       <c r="A153" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B153" s="0" t="inlineStr">
@@ -8651,15 +8641,11 @@
           <t>BSMA0150</t>
         </is>
       </c>
-      <c r="E153" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F153" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E153" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G153" s="0" t="inlineStr">
         <is>
@@ -8686,7 +8672,7 @@
       </c>
       <c r="P153" s="0" t="inlineStr">
         <is>
-          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+          <t>0 = Exclude\nReason Code: 4\nPurely qualitative ethnography without quantitative correlation data. Verbatim Evidence: \"We adopted an ethnographic approach to study the practices involved in the collaborative work between primary care services and specialist DVA support services. Two geographic areas delivering IRIS in England were selected as intrinsic cases (Stake, 1995). One researcher (GF) led the original trial of IRIS and facilitated collaboration with the national IRIS implementation team. Through a joint approach between the research and implementation teams two case studies were selected out of thirty possible areas, informed by Miles &amp; Huberman's (1994) sampling criteria for cases. [...] AD collected data through participant observation and interviewing. Fieldwork was conducted over 20 months between August 2015 and March 2017 (over 100 h per field site). AEs were the primary informants in each case study and enabled connection to other actors. [...] 19 semi-structured interviews were conducted in each case study area with clinicians (case study one: 5, case study two: 8), services users (case study one: 8, case study two: 5), and actors involved in the commissioning and delivery of IRIS (case study one: 6, case study two: 6).\" (Methods, Page 4)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -8793,7 +8779,7 @@
     <row r="156" ht="18" customHeight="1" s="31">
       <c r="A156" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B156" s="0" t="inlineStr">
@@ -8801,15 +8787,11 @@
           <t>BSMA0153</t>
         </is>
       </c>
-      <c r="E156" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F156" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E156" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" s="0" t="n">
+        <v>99</v>
       </c>
       <c r="G156" s="0" t="inlineStr">
         <is>
@@ -8836,14 +8818,14 @@
       </c>
       <c r="P156" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 99\nFile does not exist. Verbatim Evidence: \"Error invalid tool call: There was a problem parsing the tool call. Error Message: model output error: invalid tool call error (invalid_args) failed to read file: open g:/My Drive/UCL/BSMA/BSMA ANTIGRAVITY/01_Academic_Papers/[143] Du and Ma (2023) - Unpacking the effect of external search strategies on radical innovation.pdf: The system cannot find the file specified.\" (System Error Log, Page 1)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="157" ht="18" customHeight="1" s="31">
       <c r="A157" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B157" s="0" t="inlineStr">
@@ -8851,15 +8833,11 @@
           <t>BSMA0154</t>
         </is>
       </c>
-      <c r="E157" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F157" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E157" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G157" s="0" t="inlineStr">
         <is>
@@ -8886,14 +8864,14 @@
       </c>
       <c r="P157" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level unit of analysis. Verbatim Evidence: \"First, we evaluate the model with structural equation modeling (SEM) on practitioner survey data. We procured an email list of practitioner members of the Council of Supply Chain Management Professionals (CSCMP). The electronic surveys were deployed via Qualtrics—an online data collection software. After an initial pilot test which was used to confirm factors would load as hypothesized in a trial EFA, a main deployment of electronic surveys followed in two waves, the first wave from February to May 2022 and the second wave from June to August 2022. We received 210 responses from the 2,235 valid emails in the list, 158 of which were deemed usable for an effective response of 7%... The majority of responding firms were based in North America (53.8%). Also, most firms operated in the manufacturing industry (59%) and had less than $500 million in revenue.\" (4. STUDY 1 - SURVEY, Page 5)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="158" ht="18" customHeight="1" s="31">
       <c r="A158" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B158" s="0" t="inlineStr">
@@ -8901,15 +8879,11 @@
           <t>BSMA0155</t>
         </is>
       </c>
-      <c r="E158" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F158" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E158" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G158" s="0" t="inlineStr">
         <is>
@@ -8936,14 +8910,14 @@
       </c>
       <c r="P158" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nThe study measures cross-functional collaboration at the department level, utilizing logistics managers as key informants to report on their department's activities, rather than analyzing individual-level employee boundary spanning behavior. Verbatim Evidence: \"Managers were asked to indicate to what degree the logistics department had pursued various collaborative activities with the marketing department over the last six months (based on a 5-point scale; 1 never; 5 quite frequently). The overall mean score for the items in the scale that measured cross-functional collaboration was 2.96. The most frequently pursued collaborative activity is “informally working together” (3.47); the least pursued collaborative activities are “making joint decisions about ways to improve overall cost efficiency” (2.57), “developing a mutual understanding” (2.69), and “achieving goals collectively” (2.76).\" (ANALYSIS AND RESULTS, page 89)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="159" ht="18" customHeight="1" s="31">
       <c r="A159" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B159" s="0" t="inlineStr">
@@ -8951,15 +8925,11 @@
           <t>BSMA0156</t>
         </is>
       </c>
-      <c r="E159" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F159" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E159" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G159" s="0" t="inlineStr">
         <is>
@@ -8986,14 +8956,14 @@
       </c>
       <c r="P159" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative single case study based on interviews and observations lacking quantitative effect sizes. Verbatim Evidence: \"Data were collected through interviews and observations. Internal and external documents were also collected. Interviews were conducted mainly with FLEs, but in addition some back-office personnel and managers of the units were interviewed. A total of 22 interviews were conducted: 13 with FLEs, 7 with managers, and the remaining 2 with employees who worked primarily in the back office, but who had tasks that enabled them to observe the customers’ use of the services (e.g. housekeeper).\" (Data collection, Page 7)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="160" ht="18" customHeight="1" s="31">
       <c r="A160" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B160" s="0" t="inlineStr">
@@ -9001,15 +8971,11 @@
           <t>BSMA0157</t>
         </is>
       </c>
-      <c r="E160" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F160" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E160" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G160" s="0" t="inlineStr">
         <is>
@@ -9036,7 +9002,7 @@
       </c>
       <c r="P160" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"We then selected 30 companies to participate in our survey, sending each 20 questionnaires. We phoned the leaders listed in our sample to ask for their agreement to take part in the survey. Our respondents were primarily top managers or leaders of departments. If the directors were not available, we asked heads of key departments to fill in the questionnaire individually or together. It should be noted that only those who were knowledgeable concerning their firms’ BMI were qualified to take part in the interviews. Among our respondents, over 85% had worked in the company for more than five years, with an average of 7.5 years of business tenure. This length of service ensured that they were qualified interviewees. In addition, to eliminate common method variance, the BMI scale and boundary-spanning exploration scale items were filled out by department leaders or CEOs, and that on inclusive leadership style was filled out by department employees.\" (Sample procedure and data collection, page 6)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9109,7 @@
     <row r="163" ht="18" customHeight="1" s="31">
       <c r="A163" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B163" s="0" t="inlineStr">
@@ -9151,15 +9117,11 @@
           <t>BSMA0160</t>
         </is>
       </c>
-      <c r="E163" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F163" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="E163" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F163" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G163" s="0" t="inlineStr">
         <is>
@@ -9186,14 +9148,14 @@
       </c>
       <c r="P163" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Because our model focuses on the team level, we took a number of steps before aggregating individual responses to the team level. First, to ensure that the level of measurement matches the level of theory, all survey items were worded to reference the team environment and activities. Second, to justify aggregation, we computed an interrater agreement statistic using the rwg procedure (James, Demaree, &amp; Wolf, 1984) to assess the convergence of responses among team members. The median rwg values ranged from .85 to .94, above the generally accepted level of .7, indicating strong agreement (Bliese, 2000; Castro, 2002). Third, we report intraclass correlations (ICCs) to test whether the measures are reliable enough to be aggregated to the team level (Bliese, 2000; Chen, Mathieu, &amp; Bliese, 2004). The ICC1 calculates the percentage of variance in a variable that is attributable to team membership, and the ICC2 indicates whether teams can be reliably differentiated on the basis of average member ratings. Fourth, we performed a one-way analysis of variance on each variable to assess whether interteam variance was larger than intrateam variance. All of our variables were significant at the p &lt; .05 level (except for buffering that was borderline, p = .07). Finally, to ensure internal consistency of measurement, we calculated the Cronbach's alphas for all the variables at the individual (αindividual range = .73 to .85) and team levels (αaggregate range = .79 to .91). On the basis of these results, individual responses were aggregated and data were analyzed at the team level.\" (Measures, Page 609)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="164" ht="18" customHeight="1" s="31">
       <c r="A164" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B164" s="0" t="inlineStr">
@@ -9201,15 +9163,11 @@
           <t>BSMA0161</t>
         </is>
       </c>
-      <c r="E164" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F164" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E164" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F164" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G164" s="0" t="inlineStr">
         <is>
@@ -9236,14 +9194,14 @@
       </c>
       <c r="P164" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix for BSB. Verbatim Evidence: \"To classify respondents as having positions with either boundary-spanning or nonboundary-spanning responsibilities, a two-step process was used. First, consistent with criteria specified in Thompson (1967) and elsewhere (Jemison, 1984), three functions (marketing, purchasing, and human resource management) were classified as boundary spanning and four (finance, accounting, operations, and quality control) were classified as non-boundary spanning. In addition to functional descriptions, the title respondents gave for direct superiors made it possible to check for externally oriented individuals even within one of the nonboundary-spanning units.\" (Methods, Page 475)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="165" ht="18" customHeight="1" s="31">
       <c r="A165" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B165" s="0" t="inlineStr">
@@ -9251,15 +9209,11 @@
           <t>BSMA0162</t>
         </is>
       </c>
-      <c r="E165" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F165" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E165" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F165" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G165" s="0" t="inlineStr">
         <is>
@@ -9286,7 +9240,7 @@
       </c>
       <c r="P165" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative field study without quantitative correlation data. Verbatim Evidence: \"We drew from a number of research methodologies developed by social science scholars for generating theoretically useful output from qualitative data. While Glaser and Strauss’s (1967) grounded theory notion provided a useful methodological framework, we found the techniques of Strauss and Corbin (1990) and Miles and Huberman (1994) effective for operationalizing the theoretical insights from our qualitative data in a systematic fashion. Using the data, we undertook the process of “memoing” – the generation of narrative, tabular, and graphical documents meant to extract meaning from the low-level data based and create higher-level theoretical categories, concepts, and relationships that help build theory grounded theory.\" (Research method, Page 2)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -9343,7 +9297,7 @@
     <row r="167" ht="18" customHeight="1" s="31">
       <c r="A167" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B167" s="0" t="inlineStr">
@@ -9351,15 +9305,11 @@
           <t>BSMA0164</t>
         </is>
       </c>
-      <c r="E167" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F167" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E167" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F167" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G167" s="0" t="inlineStr">
         <is>
@@ -9386,7 +9336,7 @@
       </c>
       <c r="P167" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo correlation matrix provided. Verbatim Evidence: \"Local research groups comprising 13–19 partnership staff, policy officers and community members were established at each of two sites to guide the research and to reflect and act on the findings. Network and work practice surveys were conducted with 42 staff, and the results were fed back to the research groups. At the end of the project, 19 informants at the two sites were interviewed, and the researchers conducted critical reflection. The effectiveness and acceptability of the participatory social network method were determined quantitatively and qualitatively.\" (Abstract, Page 1)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -9485,7 +9435,7 @@
     <row r="170" ht="18" customHeight="1" s="31">
       <c r="A170" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B170" s="0" t="inlineStr">
@@ -9493,15 +9443,11 @@
           <t>BSMA0167</t>
         </is>
       </c>
-      <c r="E170" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F170" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E170" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" s="0" t="n">
+        <v>2</v>
       </c>
       <c r="G170" s="0" t="inlineStr">
         <is>
@@ -9528,14 +9474,14 @@
       </c>
       <c r="P170" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 2\nNon-employee student sample participating in a business simulation. Verbatim Evidence: \"Participants consisted of 277 students, organized into 50 five or six member teams, who participated in the Management Game during the Spring and Fall of 1997. Of these teams, 39 consisted of full-time students and 11 consisted of part-timers. The study took place over a period of approximately 14 weeks. During this time, teams made decisions about such managerial issues as what products they would sell to what markets (“Game moves”).\" (Participants and Procedure, Page 5)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="171" ht="18" customHeight="1" s="31">
       <c r="A171" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B171" s="0" t="inlineStr">
@@ -9543,15 +9489,11 @@
           <t>BSMA0168</t>
         </is>
       </c>
-      <c r="E171" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F171" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E171" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G171" s="0" t="inlineStr">
         <is>
@@ -9578,14 +9520,14 @@
       </c>
       <c r="P171" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm-level dyadic analysis. Verbatim Evidence: \"Our goal was to construct predictive models for Y2 based on the size of the donation made by donor i to donee j in 1980 (Y1) and some subset of the explanatory variables listed in Table 1. The units of analysis were the dyads formed by the 75 corporations and 198 nonprofits in the study population. The goal of this analysis was to identify a set of variables that have statistically significant effects on the size of contributions that corporation i made to nonprofit j in 1984.\" (Hypotheses and Models, Page 13)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="172" ht="18" customHeight="1" s="31">
       <c r="A172" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B172" s="0" t="inlineStr">
@@ -9593,15 +9535,11 @@
           <t>BSMA0169</t>
         </is>
       </c>
-      <c r="E172" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F172" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E172" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G172" s="0" t="inlineStr">
         <is>
@@ -9629,7 +9567,7 @@
       </c>
       <c r="P172" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis using archival data of domestic airlines. Verbatim Evidence: \"As noted, the unit of analysis is the level of first-mover activity within each year. This level was calculated for each airline, for each year, by summing the number of times it initiated a first move in a specific year. For example, if an airline made five first moves in 1982 and three first moves in 1983, its corresponding first mover activity for each year would be five and three respectively. If a firm did not make a first move in a given year, it received a score of 0.\" (Method, Page 235)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -9686,7 +9624,7 @@
     <row r="174" ht="18" customHeight="1" s="31">
       <c r="A174" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B174" s="0" t="inlineStr">
@@ -9694,15 +9632,11 @@
           <t>BSMA0171</t>
         </is>
       </c>
-      <c r="E174" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F174" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E174" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F174" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G174" s="0" t="inlineStr">
         <is>
@@ -9729,14 +9663,14 @@
       </c>
       <c r="P174" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study focuses on work-family boundary management (keeping work and personal life separate) rather than organizational boundary spanning behavior (BSB), representing a case of construct homonymy. Therefore, it lacks the required effect size of interest. Verbatim Evidence: \"All boundary management variables were assessed via subscales from Kossek et al. (2012) with five-point ‘Strongly Disagree’ to ‘Strongly Agree’ Likert-type response options. Interruptions of work were measured using five items (α = .75). An example item is ‘I take care of personal or family needs during work’. Interruptions of non-work consisted of five items (α = .86). An example item is ‘I regularly bring work home’. Perceived boundary control was measured using three items (α = .79). An example item is ‘I control whether I am able to keep my work and personal life separate’.\" (Boundary management measures, Page 11-12)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="175" ht="18" customHeight="1" s="31">
       <c r="A175" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B175" s="0" t="inlineStr">
@@ -9744,15 +9678,11 @@
           <t>BSMA0172</t>
         </is>
       </c>
-      <c r="E175" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F175" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E175" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G175" s="0" t="inlineStr">
         <is>
@@ -9779,7 +9709,7 @@
       </c>
       <c r="P175" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"We administered an online questionnaire to a sample set of Italian professionals who possess direct expertise in managing and/or consulting with SMEs about strategic decisions. The questionnaire was back-translated, tested by a panel of experts and piloted with 20 other experts to ensure appropriateness within the Italian context. Survey administration took place in late 2018 through the members list of the Italian Association of Business Administration and Management (AIDEA – Accademia Italiana di Economia Aziendale), which comprises 2,287 academics in business administration, accounting, management, marketing and organisation in Italy. Most of the AIDEA members are administrators, CEOs, advisors or consultants in both Italian and foreign companies. Only those with an active managerial or consulting role in one or more SME were included in the sample. Thus, our survey targeted experts with both business and academic experience who have a holistic view of the changes and challenges facing SMEs.\" (Procedure and sample, Page 36)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -9836,7 +9766,7 @@
     <row r="177" ht="18" customHeight="1" s="31">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B177" s="0" t="inlineStr">
@@ -9844,10 +9774,8 @@
           <t>BSMA0174</t>
         </is>
       </c>
-      <c r="E177" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
+      <c r="E177" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="F177" s="0" t="inlineStr">
         <is>
@@ -9879,14 +9807,14 @@
       </c>
       <c r="P177" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>1 = Include\nIndividual organizational employee sample with correlation matrix. Verbatim Evidence: \"TNT had retained the professional and personal e-mail addresses of MtW participants. Thus, it was possible to survey current and former employees to reduce the risk of survivor bias. I obtained valid e-mail addresses for 252 volunteers (out of 586 participants overall). I received 175 responses to the 252 surveys sent—a 69% response rate. After dropping interns from the sample, this number dropped to 147 survey responses, of which 36 were partial responses. The final sample consists of 101 observations due to missing data from secondary sources described below.\" (Data collection, Page 13)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="178" ht="18" customHeight="1" s="31">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B178" s="0" t="inlineStr">
@@ -9894,15 +9822,11 @@
           <t>BSMA0175</t>
         </is>
       </c>
-      <c r="E178" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F178" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E178" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G178" s="0" t="inlineStr">
         <is>
@@ -9929,14 +9853,14 @@
       </c>
       <c r="P178" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nConceptual review without empirical data. Verbatim Evidence: \"In this study we examine the impact of market orientation of leaders on their leader-member exchange (LMX) with their followers. We review the evolution of leader-member exchange (LMX) theory over the past five decades, and relate the strategic influence of increasing turbulence in the market environment on multiple generations of leadership styles during that period. Whereas vertical dyadic exchanges between hierarchical leaders and their followers may produce satisfactory performance of followers in equilibrium markets with predictable growth, these dyadic exchanges fail to do so in turbulent markets. Disequilibrium markets with disruptive turbulence demand introduction of discontinuous innovation from a new generation of market-oriented lateral leaders working closely with their boundary-spanning followers. We propose a number of hypotheses relating the market environment, leader-member exchange, and performance. Implications for managers and future researchers are discussed.\" (Abstract, Page 53)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="179" ht="18" customHeight="1" s="31">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B179" s="0" t="inlineStr">
@@ -9944,15 +9868,11 @@
           <t>BSMA0176</t>
         </is>
       </c>
-      <c r="E179" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F179" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E179" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F179" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G179" s="0" t="inlineStr">
         <is>
@@ -9979,14 +9899,14 @@
       </c>
       <c r="P179" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm-level analysis. Verbatim Evidence: \"Our sample was limited to larger firms because data on senior executives and their external ties are often unavailable for smaller organizations; consequently, it is biased toward large firms. Five firms originally included were later dropped for varied reasons (e.g., leveraged buy-out, merger), leaving a total of 55 firms that we examined over a baseline five-year period (fiscal years 1983-1987). With pooling (discussed below), we examined a total of 275 firm-year observations.\" (Sample, Page 10)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="180" ht="18" customHeight="1" s="31">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B180" s="0" t="inlineStr">
@@ -9994,15 +9914,11 @@
           <t>BSMA0177</t>
         </is>
       </c>
-      <c r="E180" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F180" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E180" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F180" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G180" s="0" t="inlineStr">
         <is>
@@ -10029,14 +9945,14 @@
       </c>
       <c r="P180" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"We calculated within-group agreements (rwg) values using James et al.’s (1993) formula. The mean of rwg values for all constructs exceeded the generally accepted 0.70 cutoff for substantial interrater agreement (.91 ≤ mean rwg ≤ 0.98). In addition, we computed intraclass correlation coefficients using Bliese and Halverson’s (1998) formula. The ICC[1]s exceeded the generally accepted .12 cutoff: external developmental feedback (.22); team creative efficacy (.28); cooperative goal interdependence (.26) and task interdependence (.31). The corresponding ANOVA F-statistics were statistically significant (P &lt; .01). The ICC[2]s exceeded the .60 cutoff suggested by Glick (1985): external developmental feedback (.61); team creative efficacy (.69); cooperative goal interdependence (.65) and task interdependence (.71). The tests supported the appropriateness of aggregating individual-level data to the team level.\" (3.3. Measurement analyses, Page 6)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="181" ht="18" customHeight="1" s="31">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B181" s="0" t="inlineStr">
@@ -10044,15 +9960,11 @@
           <t>BSMA0178</t>
         </is>
       </c>
-      <c r="E181" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F181" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E181" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F181" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G181" s="0" t="inlineStr">
         <is>
@@ -10079,14 +9991,14 @@
       </c>
       <c r="P181" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo effect size of interest is reported. The study measures leadership competencies rather than boundary spanning behaviors, and only reports a partial table of significant correlations instead of a full Pearson correlation matrix. Verbatim Evidence: \"In order to test the hypothesis, a bivariate correlation was performed between the 15 leadership dimensions of the LDQ raw data and the two factors identified in the previous section. It was discovered that Factor 1 was correlated to managing resources at a significance level of 0.05, while Factor 3 shows no significant correlation with any leadership dimensions. In order to explore the data further, each PSQ item loading onto Factors 1 and 3 was correlated with each leadership dimension. Only those correlations represented by the Pearson correlation coefficients were statistically significant at the 0.01 and 0.05 levels and are shown in Table 3.\" (Results, page 63)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="182" ht="18" customHeight="1" s="31">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B182" s="0" t="inlineStr">
@@ -10094,15 +10006,11 @@
           <t>BSMA0179</t>
         </is>
       </c>
-      <c r="E182" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F182" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E182" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F182" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G182" s="0" t="inlineStr">
         <is>
@@ -10129,14 +10037,14 @@
       </c>
       <c r="P182" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nThis study exclusively measures Leader-Member Exchange and its subdimensions without capturing any form of boundary spanning behavior or relevant effect sizes. Verbatim Evidence: \"For the purposes of this study, Leader Member Exchange quality was assessed using a six-item LMX-6 scale developed by Schriesheim, Neider, Scandura, and Tepper (1992). The three components, perceived contribution, loyalty, and affect, were identified by two questionnaire items each. Scores from the six items are summed and then divided by six to obtain an average score for the leader member exchange quality scale.\" (Method, Page 91-92)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="183" ht="18" customHeight="1" s="31">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B183" s="0" t="inlineStr">
@@ -10144,15 +10052,11 @@
           <t>BSMA0180</t>
         </is>
       </c>
-      <c r="E183" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F183" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E183" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G183" s="0" t="inlineStr">
         <is>
@@ -10179,14 +10083,14 @@
       </c>
       <c r="P183" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo measure of boundary spanning behavior. The study measures boundaryless careers (physical career mobility across jobs), which is a distinct concept from boundary spanning behavior. Verbatim Evidence: \"Therefore, with the aim of investigating in depth the “boundaryless career space” (Gubler et al., 2014a), we proposed adding two more dimensions to the traditional organizational mobility. First, we included the movements of the managers across different industrial boundaries. Second, we considered changes in different geographical locations. Specifically, we asked the managers of the sample to indicate: (a) organizational mobility: the number of firms they worked for; (b) industry mobility: the number of different sectors they operated in; and (c) geographical mobility: the number of times they worked abroad for at least 1 year, all with reference to the period of time from T1 to T2.\" (Dependent Variables, Page 6)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="184" ht="18" customHeight="1" s="31">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B184" s="0" t="inlineStr">
@@ -10194,15 +10098,11 @@
           <t>BSMA0181</t>
         </is>
       </c>
-      <c r="E184" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F184" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E184" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F184" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G184" s="0" t="inlineStr">
         <is>
@@ -10229,14 +10129,14 @@
       </c>
       <c r="P184" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative case study lacking quantitative correlation data. Verbatim Evidence: \"An independent evaluation team comprising two academic/healthcare staff worked with the project team to capture learning. This involved undertaking focus group discussions and individual interviews with members of the team and observation of a range of meetings in each phase of the initiative. Interview/focus group transcripts and field notes of meetings were analysed by the evaluation team and the findings discussed with the project team in order to draw out the learning. The aim of this paper is to report on the learning to arise from using the CMS approach to promote integrated care across the falls care pathway.\" (Overview of the falls quality improvement initiative, Page 3)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="185" ht="18" customHeight="1" s="31">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B185" s="0" t="inlineStr">
@@ -10244,15 +10144,11 @@
           <t>BSMA0182</t>
         </is>
       </c>
-      <c r="E185" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F185" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E185" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G185" s="0" t="inlineStr">
         <is>
@@ -10279,14 +10175,14 @@
       </c>
       <c r="P185" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative case study lacking quantitative data. Verbatim Evidence: \"Interviewing ‘elite’ HLEG actors is a challenging task due to their competing priorities (Empson, 2018). We interviewed 32 actors relating to the HLEG-SF – 16 group members, six observers, five European Commission officials and supporting staff, four members’ or observers’ collaborators and one journalist. Data collection spanned 18 months from November 2017. The interviews lasted, on average, 55 minutes (for a total of 29.8 hours) and were transcribed. Primary data collection was complemented by various sources of secondary data listed in Table 1.\" (Data collection, page 8)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="186" ht="18" customHeight="1" s="31">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B186" s="0" t="inlineStr">
@@ -10294,15 +10190,11 @@
           <t>BSMA0183</t>
         </is>
       </c>
-      <c r="E186" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F186" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E186" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G186" s="0" t="inlineStr">
         <is>
@@ -10329,7 +10221,7 @@
       </c>
       <c r="P186" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nNo boundary spanning behavior measured. Verbatim Evidence: \"These were evaluated using the four measures of virtuality from Gibson and Gibbs (2006), with a few alterations. Geographical dispersion was measured using 4 items (α = 0.83) focused on team members' dispersion across multiple geographical areas and worksites as well as the necessity of frequent business travel. Dynamic structure was evaluated using a 3-item measure (α = 0.73) focused on frequency of team member changes, difficulty knowing who is on the team, and consistency in the team's operating structure. Whereas Gibson and Gibbs measured national diversity specifically, we adopted a broader measure of cultural diversity using two items (α = 0.85) focused on team members' work with others who speak different native languages or dialects and collaboration with people from different cultural backgrounds (Chudoba et al., 2005). Finally, instead of electronic dependence – which is a rather dated measure that assumes that technology use is the exception rather than the rule – we opted to measure the degree of dependence on face-to-face, assuming that electronic communication is the norm for most virtual teams. Face-to-face dependence was measured using two items (α = 0.77) that asked participants to evaluate both their use and the importance of face-to-face interactions.\" (3.2.1. Organizational discontinuities, Page 8)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -10386,7 +10278,7 @@
     <row r="188" ht="18" customHeight="1" s="31">
       <c r="A188" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B188" s="0" t="inlineStr">
@@ -10394,15 +10286,11 @@
           <t>BSMA0185</t>
         </is>
       </c>
-      <c r="E188" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F188" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E188" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F188" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G188" s="0" t="inlineStr">
         <is>
@@ -10429,7 +10317,7 @@
       </c>
       <c r="P188" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nNo effect size of interest. The study is a mixed-methods case study that analyzes semi-structured interviews and a sociometric network survey. It does not provide an individual-level bivariate Pearson correlation matrix. Verbatim Evidence: \"This study uses a mixed-method research strategy, combining both quantitative and qualitative approaches. More specifically, we complement the results from in-depth interviews with results from a socio-metric survey. [...] A sociometric survey was also conducted during the interview. At the end of each interview, interviewees were asked, “Please name 5 individuals who were instrumental in resourcing, facilitating, managing, leading, supporting, or inspiring your response efforts”. Based on the interview results, we created a one-mode network of reputation-based relationships. The one-mode network represents person-by-person relationships.\" (3. Research design and method, Page 576)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -10528,7 +10416,7 @@
     <row r="191" ht="18" customHeight="1" s="31">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B191" s="0" t="inlineStr">
@@ -10536,15 +10424,11 @@
           <t>BSMA0188</t>
         </is>
       </c>
-      <c r="E191" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F191" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E191" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F191" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G191" s="0" t="inlineStr">
         <is>
@@ -10571,14 +10455,14 @@
       </c>
       <c r="P191" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative interview study. Verbatim Evidence: \"To understand the differences between boundary-work of IMA officials and IMA members in Russia, we conducted interviews with both groups of individuals. Formally, the empirical base of this paper consists of 15 formal interviews conducted in English and Russian with IMA members and IMA officials (see Table 1). Each interview lasted between 28 and 100 min (average 53 min). Apart from interviews, primary data sources consist of participant observations of two annual meetings with IMA members in Moscow.\" (Method, page 4-5)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="192" ht="18" customHeight="1" s="31">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B192" s="0" t="inlineStr">
@@ -10586,15 +10470,11 @@
           <t>BSMA0189</t>
         </is>
       </c>
-      <c r="E192" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F192" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E192" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G192" s="0" t="inlineStr">
         <is>
@@ -10621,14 +10501,14 @@
       </c>
       <c r="P192" s="0" t="inlineStr">
         <is>
-          <t>Study involving workplace employees, but does not report quantitative correlation/regression effect sizes for boundary spanning.</t>
+          <t>0 = Exclude\nReason Code: 4\nPurely qualitative research lacking correlation data. Verbatim Evidence: \"We used a variety of qualitative methods, including participant observation (one of the researchers undertook call handler training followed by a limited number of supervised shifts ‘on the lines’); work shadowing; indepth interviews with both call centre staff and callers; and conversation analysis (CA) of recorded call interactions. The analysis presented here is based upon the participant and non-participant observations/shadowing at the call centres, interviews with nurses and call handlers and analysis of call interactions between staff and callers.\" (Introduction, Page 4)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="193" ht="18" customHeight="1" s="31">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B193" s="0" t="inlineStr">
@@ -10636,15 +10516,11 @@
           <t>BSMA0190</t>
         </is>
       </c>
-      <c r="E193" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F193" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E193" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G193" s="0" t="inlineStr">
         <is>
@@ -10671,14 +10547,14 @@
       </c>
       <c r="P193" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: \"Once they agreed to participate, the executives were requested to provide us with a list of projects completed in the previous six months. Recently concluded projects reduce the effect of recall bias. All projects chosen were outsourced in entirety to the vendor firm and were carried out by the vendor firm. The executives granted access to individual project managers on projects who provided the responses for each project. A total of 23 firms finally agreed to participate in our research, for a response rate of 51%. These firms had, on average, 3,200 employees, with the smallest firm having 450 employees at the time of data collection. To ensure coverage of a broad range of projects from each organization, we only retained projects from firms where we had at least four or more projects. Our final sample for this study consisted of a total of 96 projects from 10 firms.\" (Research Design and Data Analysis, Page 970)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="194" ht="18" customHeight="1" s="31">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B194" s="0" t="inlineStr">
@@ -10686,15 +10562,11 @@
           <t>BSMA0191</t>
         </is>
       </c>
-      <c r="E194" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F194" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E194" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F194" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G194" s="0" t="inlineStr">
         <is>
@@ -10721,7 +10593,7 @@
       </c>
       <c r="P194" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: \"The original digital dividend case base consisted of over 1,000 case capsules collected over the last five years. Each case contained a short abstract plus some meta-data describing the case's location, activity type, sponsorship, sector, etc. We sought to extend these descriptions by identifying for each case the type of innovation that it embraced and the types of benefit it produced. Specifically, for each case we sought to indicate whether the primary type of innovation it embodied was technology-focused or business-focused (see Table 1).\" (Data Analysis, Page 218)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -10878,7 +10750,7 @@
     <row r="198" ht="18" customHeight="1" s="31">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B198" s="0" t="inlineStr">
@@ -10886,15 +10758,11 @@
           <t>BSMA0195</t>
         </is>
       </c>
-      <c r="E198" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F198" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E198" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F198" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G198" s="0" t="inlineStr">
         <is>
@@ -10921,14 +10789,14 @@
       </c>
       <c r="P198" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"Our sample population is composed of the senior executives in U.S.-based organizations responsible for corporate public affairs. Corporate public affairs is defined in the survey as the “management function responsible for interpreting the corporation’s non-commercial environment and managing the corporation’s responses to that environment” (Foundation for Public Affairs, 1999, p. 2) and is consistent with previous empirical studies (Greening, 1992; Greening &amp; Gray, 1994; Meznar &amp; Nigh, 1995). In 1999, after a pretest of the questionnaire, surveys were mailed to 1,087 senior executives. The sample population was identified with the help of the National Directory of Corporate Public Affairs and the Public Affairs Council.2 Two hundred twenty-three surveys were returned (21% response rate). Financial data were not available for 72 companies.3 Therefore, the final sample consists of 151 respondents (14% effective response rate).\" (Sample Population and Instrument, Page 203-204)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="199" ht="18" customHeight="1" s="31">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B199" s="0" t="inlineStr">
@@ -10936,15 +10804,11 @@
           <t>BSMA0196</t>
         </is>
       </c>
-      <c r="E199" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F199" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E199" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F199" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G199" s="0" t="inlineStr">
         <is>
@@ -10971,14 +10835,14 @@
       </c>
       <c r="P199" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis focusing on team adaptation and team boundary management rather than individual boundary spanning behavior. Verbatim Evidence: \"The major aim of this study is to attempt to measure the factors affecting teams embedded in organizations – informed by individuals participating in teams. Specifically, we seek to evaluate the effects of the internal and external focus of teams – that is, ‘within-team’ interaction as well as connection with organizational priorities and with others in the organization – on adaptability, the ability to adjust tasks and goals, and potency, which is confidence in the team’s ability to achieve its goals.\" (Introduction, Page 76) \"Each of the studies included team representatives, but none of the studies included multiple members from teams. Team studies are more robust, especially in quantitative studies, when multiple members of the same team are included in the sample in order to obtain a team level measure. This dissertation included a significant amount of qualitative research so to mitigate the lack of multiple members per team in the samples, team leaders or project facilitators served as participants in order to obtain the broadest view possible of overall team activities.\" (Limitations, Page 203)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="200" ht="18" customHeight="1" s="31">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B200" s="0" t="inlineStr">
@@ -10986,15 +10850,11 @@
           <t>BSMA0197</t>
         </is>
       </c>
-      <c r="E200" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F200" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E200" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G200" s="0" t="inlineStr">
         <is>
@@ -11021,14 +10881,14 @@
       </c>
       <c r="P200" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nLack of boundary spanning behavior variable. The study focuses on cognitive self-regulation following work interruptions into the home domain, measuring family flexibility and work-family role transitions rather than organizational boundary spanning behavior. Verbatim Evidence: \"All other discriminant validity measures were assessed in sample 2. To measure the flexibility of nonwork boundaries, we adapted Matthews et al.’s (2010) 5-item family flexibility-ability scale (e.g., “If the need arose, I could work late without affecting my family and personal responsibilities”) and three items from their family flexibility-willingness scale (e.g., “I am willing to change plans with my friends and family so that I can finish a job assignment”). We measured work-related intrusions with one item (“Intrusions from work during my nonwork hours impede on my personal life”). To measure non-work-to-work role transitions, we adapted three items from the family-to-work transition scale (e.g., “How often in the past three months have you changed plans with your family to meet work-related responsibilities?”; 0=never to 5=5 or more days per week; Matthews et al., 2010).\" (Measures, Page 497)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="201" ht="18" customHeight="1" s="31">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B201" s="0" t="inlineStr">
@@ -11036,15 +10896,11 @@
           <t>BSMA0198</t>
         </is>
       </c>
-      <c r="E201" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F201" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E201" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F201" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G201" s="0" t="inlineStr">
         <is>
@@ -11071,14 +10927,14 @@
       </c>
       <c r="P201" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 4\nConceptual position paper without empirical effect sizes. Verbatim Evidence: \"We have identified different kinds of human involvement into software process activities. We discussed different enaction mechanisms, and we proposed an architecture for corresponding enaction components. The proposed architecture is kept as general as possible. It is independent from any process modeling language, but only based on the assumption that different types of human involvement in activities require communication and enaction support. Our future efforts will be focused on a detailed investigation how the identified kinds of human involvement are reflected by existing groupware, workflow and software process management environments.\" (Conclusion, page 5)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="202" ht="18" customHeight="1" s="31">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B202" s="0" t="inlineStr">
@@ -11086,15 +10942,11 @@
           <t>BSMA0199</t>
         </is>
       </c>
-      <c r="E202" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F202" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E202" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F202" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G202" s="0" t="inlineStr">
         <is>
@@ -11121,14 +10973,14 @@
       </c>
       <c r="P202" s="0" t="inlineStr">
         <is>
-          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+          <t>0 = Exclude\nReason Code: 4\nConceptual paper without empirical data. Verbatim Evidence: \"While much has been said about the merits of conceptual transfers between domains, much equally remains unknown, particularly about how to deliberately develop creative insights that have the potential to challenge or enhance existing supply chain management theory. To address this issue, this research builds on prior work on analogies, creativity, and design thinking to develop a heuristic-analytic model. This model is designed to assist researchers in theorizing by analogy through a controlled dual cognitive process of divergence before convergence combined with a distant boundary-spanning knowledge search. An illustration of the model shows how creative output can provide a fresh perspective that helps render supply chains potentially more resilient.\" (Abstract, page 3)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="203" ht="18" customHeight="1" s="31">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B203" s="0" t="inlineStr">
@@ -11136,15 +10988,11 @@
           <t>BSMA0200</t>
         </is>
       </c>
-      <c r="E203" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F203" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E203" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F203" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G203" s="0" t="inlineStr">
         <is>
@@ -11171,7 +11019,7 @@
       </c>
       <c r="P203" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 4\nThis is a conceptual review paper discussing the interface between primary and specialty care that does not provide primary empirical quantitative data or a correlation matrix. Verbatim Evidence: \"In this article, we explore the unique challenges of care and health service delivery in terms of the interface between primary care and specialist care during the survivorship period. The research literature points to problems of communication between primary and specialist providers, as well as lack of clarity about the respective roles of different members of the health-care team. Survivorship care plans are recommended as an important tool to facilitate communication and allocation of responsibility during the transition from active treatment to survivorship. Research questions that remain to be answered with respect to survivorship care plans and other aspects of survivorship care are discussed.\" (Abstract, Page 25)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -11191,10 +11039,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F204" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F204" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G204" s="0" t="inlineStr">
         <is>
@@ -11221,7 +11067,7 @@
       </c>
       <c r="P204" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Our final sample consisted of those 57 teams from which we had received three or more subordinate surveys and a supervisor survey, and for which archival data were available. These teams ranged in size from 4 to 26 members (x = 11.7, s.d. = 6.1); 84 percent of team members were male; the average age was 42.7 years (s.d. = 7.7), and the average time with the current team was 1.5 years (s.d. = .5). [...] Together, the above analyses supported the aggregation of informant responses from a team to create team-level variables for collective team identification, team learning, intrateam conflict, and external communication.\" (Sample and Data Collection / Interrater agreement and reliability, Pages 537-539)\n\nNote: The specific file \"Guenzel (2020) - Open innovation...\" did not exist in the workspace, so the paper with ID 201 mapped in all_remaining_targets.txt (\"[201] Van der vegt &amp; Bunderson (2005) - LEARNING AND PERFORMANCE IN MULTIDISCIPLINARY TEAMS.pdf\") was reviewed instead as standard procedure.\n"}"</t>
         </is>
       </c>
     </row>
@@ -11383,10 +11229,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F208" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F208" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G208" s="0" t="inlineStr">
         <is>
@@ -11413,7 +11257,7 @@
       </c>
       <c r="P208" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"After excluding teams for which fewer than 50 percent of the respondents were core members (Hackman, 2002: 47), 96 teams qualified for the study (80 percent; 50 financial and 46 technical teams, with 485 member respondents). Tests for selection bias showed no significant differences in the effectiveness ratings, project types, regions, or divisions of the 24 teams that did not qualify. Dependent variables. The dependent variables in this study were (1) the strategic effectiveness of a team and (2) the operational effectiveness of a team, as rated by its independent expert panel.\" (Quantitative Data, Page 995)\n"}"</t>
         </is>
       </c>
     </row>
@@ -11623,10 +11467,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F213" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F213" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G213" s="0" t="inlineStr">
         <is>
@@ -11653,7 +11495,7 @@
       </c>
       <c r="P213" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study provides a quantitative correlation matrix based on an employee sample, but it does not measure Boundary Spanning Behavior (BSB) or include it in the effect sizes. The measured variables are limited to transformational leadership, internal/external support for innovation, firm age, and organizational innovation. Verbatim Evidence: "\"Employees’ questionnaires included measures of transformational leadership and internal support for innovation. On average, four employees rated each leader. Employees were also asked for their age, gender, educational level, job tenure, and company tenure. Leaders’ questionnaires included questions about company age, company innovations, and the degree of support they received from external institutions.\" (Procedure, Page 7)\n"}"</t>
         </is>
       </c>
     </row>
@@ -11762,14 +11604,10 @@
       </c>
       <c r="E216" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F216" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F216" s="0" t="inlineStr"/>
       <c r="G216" s="0" t="inlineStr">
         <is>
           <t>Purpose – The current article investigates the impact of generational diversity on knowledge sharing and group performance. It, further, explores the moderating effects of intergenerational climate, boundaryspanning leadership, and respect in facilitating greater knowledge sharing and enhanced group performance. Design/methodology/approach – The authors applied partial least square structural equation modeling to test the model, using a sample of 635 employees working in the banking industry.</t>
@@ -11795,7 +11633,7 @@
       </c>
       <c r="P216" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Verbatim Evidence: ""</t>
         </is>
       </c>
     </row>
@@ -11812,14 +11650,10 @@
       </c>
       <c r="E217" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F217" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F217" s="0" t="inlineStr"/>
       <c r="G217" s="0" t="inlineStr">
         <is>
           <t>This paper combines the concept of weak ties from social network research and the notion of complex knowledge to explain the role of weak ties in sharing knowledge across organization subunits in a multiunit organization. I use a network study of 120 new-product development projects undertaken by 41 divisions in a large electronics company to examine the task of developing new products in the least amount of time. Findings show that weak interunit ties help a project team search for useful knowledge in other subunits but impede the transfer of complex knowledge, which tends to require a strong tie between the two parties to a transfer. Having weak interunit ties speeds up projects when knowledge is not complex but slows them down when the knowledge to be transferred is highly complex. I discuss the implications of these findings for research on social networks and product innovation.</t>
@@ -11845,7 +11679,7 @@
       </c>
       <c r="P217" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Verbatim Evidence: ""</t>
         </is>
       </c>
     </row>
@@ -11865,10 +11699,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F218" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F218" s="0" t="n">
+        <v>99</v>
       </c>
       <c r="G218" s="0" t="inlineStr">
         <is>
@@ -11895,7 +11727,7 @@
       </c>
       <c r="P218" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 99\nFile not found on disk. Verbatim Evidence: "\"failed to read file: open g:/My Drive/UCL/BSMA/BSMA ANTIGRAVITY/01_Academic_Papers/[209] Hanisch et al. (2014) - Innovation network formation a conceptual model.pdf: The system cannot find the file specified. A global search for Hanisch across the BSMA ANTIGRAVITY workspace yielded zero results. Therefore, this paper cannot be audited and is excluded due to a missing file.\" (System Error Log, Page 1)\n"}"</t>
         </is>
       </c>
     </row>
@@ -11915,10 +11747,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F219" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F219" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G219" s="0" t="inlineStr">
         <is>
@@ -11945,7 +11775,7 @@
       </c>
       <c r="P219" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We first obtained a list of 272 public pharmaceutical companies based on the standard industry classification code (SIC 2834). By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005. To test our model, we collect secondary data about firms’ IT-enabled knowledge capabilities and innovation outcomes from multiple secondary data sources.\" (Data Collection, Page 9)\n"}"</t>
         </is>
       </c>
     </row>
@@ -11962,14 +11792,10 @@
       </c>
       <c r="E220" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F220" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F220" s="0" t="inlineStr"/>
       <c r="G220" s="0" t="inlineStr">
         <is>
           <t>The paper explains the effects of internal and external team learning behaviors on the performance of marketing teams. The survey was conducted in the context of a multinational Pharmaceutical Corporation marketing its products in Turkey. Data were collected from members of marketing team which included medical sales representatives, specialized medical sales representatives and districts heads of marketing. The results indicate that both the internal team learning and the external team learning behaviors play significant roles in ensuring the success of marketing teams in continuously identifying, anticipating and satisfying the customer requirements profitably through an efficient deployment of the marketing teams’ resources.</t>
@@ -11995,7 +11821,7 @@
       </c>
       <c r="P220" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Verbatim Evidence: "\"The sample comprises four public-sector and four private-sector banks (NSE/BSE indexed) with 12 branches of each bank. The number of respondents from public-sector and private-sector banks was 327 and 308, respectively. Data were collected through a questionnaire comprising 40 items reflecting all the constructs (Generational diversity, knowledge sharing, group performance, intergenerational climate, boundary-spanning leadership, and respect). The study followed a cross-sectional approach for collecting data. The clerical and managerial employees in the bank branches were contacted through offline survey methods.\" (Sample, Page 7)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12065,10 +11891,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F222" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F222" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G222" s="0" t="inlineStr">
         <is>
@@ -12095,7 +11919,7 @@
       </c>
       <c r="P222" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative study without quantitative effect sizes. Verbatim Evidence: "\"A thematic analysis of the discourse collected through in-depth interviews, survey questionnaires, and organizational documents was conducted using the constant comparative method (Lindlof, 1995). This process begins with data “reduction” and “interpretation” (Creswell, 1997; Lindlof, 1995) and is consistent with processes engaged in by other communication scholars doing interpretive work (e.g., Braithwaite, Baxter, &amp; Harper, 1998; Clair &amp; Thompson, 1996; Trethewey, 1997). First, all transcripts and documents were read in their entirety to develop a sense of these data as a whole.\" (Data Analysis, Page 8)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12115,10 +11939,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F223" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F223" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G223" s="0" t="inlineStr">
         <is>
@@ -12145,7 +11967,7 @@
       </c>
       <c r="P223" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative case study without quantitative correlation data. Verbatim Evidence: "\"Following other researchers who are interested in organizational processes (e.g., Anand, Gardner, &amp; Morris, 2007; Bresman, 2013; Nag &amp; Gioia, 2012), we combined a case study approach with grounded theory methodology (Langley, 1999). Specifically, we first used grounded methods to develop cases describing the sequence of early boundary spanning activity in each of 10 COTs; we then used a case study approach to compare and contrast those sequences across the 10 teams. Case studies drew on interviews with 46 team members.\" (Method, page 512)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12165,10 +11987,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F224" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F224" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G224" s="0" t="inlineStr">
         <is>
@@ -12195,7 +12015,7 @@
       </c>
       <c r="P224" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level variables. The study measures external team learning and team performance rather than individual-level employee boundary spanning behavior. Verbatim Evidence: "\"For data collection, we adapted the Team Learning Survey (TSL) and Team Performance Survey (TPS) scales used by Edmondson (1996) while investigating team learning in a large office furniture manufacturer in the American Mid-West. The Team Learning Survey (TLS) incorporated both the internal and the external team learning behaviors each measured through five items. The team performance construct in the Team Performance Survey (TPS) was also measured through five items. The respondents were asked to record their responses on a seven-point likert scale where 1 meant strongly disagree and 7 meant strongly agree.\" (Methods, Page 126)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12265,10 +12085,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F226" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F226" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G226" s="0" t="inlineStr">
         <is>
@@ -12295,7 +12113,7 @@
       </c>
       <c r="P226" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study conducts a social network analysis calculating network centrality measures rather than using psychometric scales, and it does not report a bivariate Pearson correlation matrix. Verbatim Evidence: "\"Survey responses were exported from Qualtrics® into a spreadsheet where the data were cleaned following a two-step process. First, participants’ identification numbers were checked against a master list to ensure that only the data from invited respondents were included. In situations where a participant’s data were recorded twice, only the first record was retained. Second, only participants who completed the sociodemographic survey questions and listed at least one person using their full name as a source of advice or information about PBS were included. Social network data in the form of adjacency lists were created and imported into the social network software Visone (Algorithmics Group, 2019) where graphs were constructed and analyses conducted, including calculation of indegree and betweenness centralities.\" (Data extraction and analysis, Page 5)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12315,10 +12133,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F227" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F227" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G227" s="0" t="inlineStr">
         <is>
@@ -12345,7 +12161,7 @@
       </c>
       <c r="P227" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam and firm level of analysis. Verbatim Evidence: "\"Using CorpTech (now part of InfoUSA), we built a sampling frame of 467 small- to medium-sized enterprises (SMEs) operating in technology-based sectors in the northeastern United States. [...] All told, for 99 firms, we received responses from the CEO and at least another member of the top management team. [...] Apart from the dependent variable, which relies on the assessment of the CEO, our measures involved the aggregated responses of top managers. We separated the measurement of our independent and dependent variables using separate respondents to minimize the influence of common method effects. [...] An acceptable level of interrater agreement (median rwg(j) = 0.94) and reliability (ICC1 = 0.31, ICC2 = 0.69) justified the aggregation of top managers’ responses to the team level of analysis (Chan 1998).\" (Method, Pages 946-947)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12415,10 +12231,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F229" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F229" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G229" s="0" t="inlineStr">
         <is>
@@ -12445,7 +12259,7 @@
       </c>
       <c r="P229" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"The average succession rate for any given company was found by aggregating (averaging) the reciprocals of completed office tenures during the 30-year interval for all presidential successors who held the title Chief Executive Officer. Office tenure for successors was determined by examining selected editions of Moody’s Industrial Manual [28]. The specification of the 30-year interval was also statistically necessary because of the need to control the time variable across companies when developing ex post facto measures of succession rate and variability in measures of board size.\" (Operational Definitions, Page 5)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12465,10 +12279,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F230" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F230" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G230" s="0" t="inlineStr">
         <is>
@@ -12495,7 +12307,7 @@
       </c>
       <c r="P230" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Four organizations participated, providing 56 R&amp;D teams. Two of the companies were R&amp;D divisions of large publicly-listed mining and chemical manufacturing organizations, whilst the other two were government R&amp;D organizations. The analyses report a one-year longitudinal study, with repeated mail outs every four months. Analyses were conducted on team level data collected over four time periods. Teams (both leaders and team members) rated leadership role performance and team communication.\" (Method, page 5)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12565,10 +12377,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F232" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F232" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G232" s="0" t="inlineStr">
         <is>
@@ -12595,7 +12405,7 @@
       </c>
       <c r="P232" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative interview study without quantitative effect sizes. Verbatim Evidence: "\"Data was collected from participants via telephone interviews which typically lasted about 45 minutes, with all conversations being digitally recorded with participants’ consent. The interviews were qualitative conversations, being focussed around a standard list of open-ended questions that were asked to all interviewees. The key topics discussed in the interviews included the nature of people’s work, their feelings about their work, the positive and negative features of their work, the extent to which work was a source of stress or fatigue, how work-related stress/fatigue was dealt with, as well as the role of ICTs and mobile ICTs in their work and the management of the work-life boundary.\" (4.2 Data Collection Procedure, Page 12-13)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12615,10 +12425,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F233" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F233" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G233" s="0" t="inlineStr">
         <is>
@@ -12645,7 +12453,7 @@
       </c>
       <c r="P233" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam-level analysis. Verbatim Evidence: "\"For measuring team interface management, we mainly relied on Mohrman et al.’s (1995) discussion of team management tasks in team-based organizations and on Ancona and Caldwell’s (1992) description of boundary management. Team members were asked to evaluate the extent to which the activities described in the seven items were performed in the team. Prior to aggregating team members’ evaluations of team interface management, interrater agreement (Campion et al., 1993; James, 1982; James et al., 1984) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). With an average score across all teams of 0.87, this test yielded results indicating generally very strong agreement of ratings referring to the same team. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, page 10)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12715,10 +12523,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F235" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F235" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G235" s="0" t="inlineStr">
         <is>
@@ -12745,7 +12551,7 @@
       </c>
       <c r="P235" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level of analysis. Verbatim Evidence: "\"Prior to aggregating team members’ evaluations of interteam coordination, project commitment, and teamwork quality, interrater agreement (James 1982, James et al. 1984, Campion et al. 1993) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). This test yielded results indicating generally very strong agreement of ratings referring to the same team. The average score of this test across all teams is 0.90 for interteam coordination, 0.91 for project commitment, and 0.93 for teamwork quality. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, Page 45)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12857,10 +12663,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F238" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F238" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G238" s="0" t="inlineStr">
         <is>
@@ -12887,7 +12691,7 @@
       </c>
       <c r="P238" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative reflective inquiry paper without quantitative correlation data. Verbatim Evidence: "\"We iteratively collected and analyzed data for this manuscript using the three sequential phases (Kim, 1999): descriptive, reflective, and critical summarized in Table 1. First, we used the descriptive phase to elicit narratives of actual experiences including descriptions of actions, thoughts, and feelings (Kim, 1999). This phase began while preparing for a discussion panel on navigating disciplinary boundaries presented in the Health Communication Division at the National Communication Association (NCA) 2018 Annual Convention in Salt Lake City, Utah. Each author wrote narratives of their experiences navigating a boundary spanning academic position.\" (Procedures, Page 3)\n"}"</t>
         </is>
       </c>
     </row>
@@ -12957,10 +12761,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F240" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F240" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G240" s="0" t="inlineStr">
         <is>
@@ -12987,7 +12789,7 @@
       </c>
       <c r="P240" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"The unit of analysis for the study is the audit team. A team score for each variable was computed by summing the individual item responses provided by the three team members. For the variables under study, the proportion of total variance that is shared among teammates (Spearman-Brown formula; DeVellis 1991) is .26 for information overload, .42 for boundary spanning, .42 for satisfaction with supervision, .22 for accuracy of information, and .15 for audit team structure.\" (RESULTS, Page 8)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13007,10 +12809,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F241" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F241" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G241" s="0" t="inlineStr">
         <is>
@@ -13037,7 +12837,7 @@
       </c>
       <c r="P241" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We used a survey methodology to gather the data for the research. This study used a sample framework of 300 firms selected randomly from the list of 650 new technology ventures located in Shenzhen, provided by a local consulting and market research company. We contacted the senior manager of each firm by phone to solicit their participation in this study, and to ask if they would be willing to provide access to two or three key informants, including CEOs, managing directors, or senior managers who were involved in engineering or business development.\" (Sample and data collection, Page 6)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13102,10 +12902,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F243" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F243" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G243" s="0" t="inlineStr">
         <is>
@@ -13132,7 +12930,7 @@
       </c>
       <c r="P243" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We sent out 750 questionnaires to part-time MBA and EMBA students at 4 universities in China who come from enterprises in different provinces and municipalities such as Heilongjiang, Jilin and Beijing. Respondents were asked to be middle and senior managers and technical executives who understand corporate strategy and technology innovation. The questionnaires were collected in two phases. In the first stage, the data is distributed before class and recovered after class; in the second stage, some selected respondents, who were corporate executives, were invited to further distribute questionnaires to their subordinates or colleagues to reduce common method bias. Eventually, we obtained valid questionnaires from 290 different companies and the effective recovery rate was 38.67%.\" (Method, page 8)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13152,10 +12950,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F244" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F244" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G244" s="0" t="inlineStr">
         <is>
@@ -13182,7 +12978,7 @@
       </c>
       <c r="P244" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study lacks a Pearson correlation matrix reporting effect sizes for employee boundary spanning behavior. Instead, it utilizes qualitative script elicitation methodology and chi-square analysis to compare the frequency of service expectations between consumers and providers. Verbatim Evidence: "\"Thus, two sets of scripts were obtained, one set from consumers and the other set from service providers. The unit of analysis was the script, which was composed of the subgoals of the respondent’s typical haircut. The two sets of scripts were coded separately. Each subgoal mentioned was recorded, yielding a master list of subgoals for each set of respondents. The number of respondents who mentioned each subgoal was then tallied. Descriptive statistics are provided in Table I. Chi-square analysis found no significant gender differences in the frequency of mention of any of the subgoals.\" (Analysis and results, Page 7)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13202,10 +12998,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F245" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F245" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G245" s="0" t="inlineStr">
         <is>
@@ -13232,7 +13026,7 @@
       </c>
       <c r="P245" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study uses structural equation modeling (SEM) to evaluate the interrelations among variables but fails to provide a bivariate Pearson correlation matrix for the extracted measures. Only descriptive statistics, factor loadings, and structural path estimates are reported. Verbatim Evidence: "\"The descriptive statistics is shown in Table I, namely, mean, standard deviation and the factor analysis and Cronbach’s alpha results... Structural equation modelling (SEM) was used for the data analysis that included all the hypothesised paths, which is consistent with other studies conducted on multiteam system performance (Cuijpers et al., 2016; Cha et al., 2015). SEM was appropriate for investigating the interrelations among the set of variables, as it offers advantages over multiple regression, accounting, as it does for measurement error (Strasheim, 2014). SEM is a second generation multivariate method used to assess the reliability and validity of the model measures holistically, whereas first generation multivariate methods, such as multiple regression, are appropriate for evaluating constructs and relationships between constructs (Tabachnick and Fidell, 2001, p. 111). A measurement model was developed in AMOS 24.0 for the four constructs to be tested.\" (3. Methods, Page 11-12)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13252,10 +13046,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F246" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F246" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G246" s="0" t="inlineStr">
         <is>
@@ -13282,7 +13074,7 @@
       </c>
       <c r="P246" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: "\"We gathered our data in The Netherlands using a cross sectional survey methodology. We used the project level of analysis because the information used to make NPD decisions is project-specific, rather than being more generally applicable to the entire firm or a division. Each project requires specific details about customer needs and technical capabilities to allow developers to make tradeoffs between the different specifications and feature levels.\" (Sample and Data Collection, Page 4)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13494,10 +13286,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F251" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F251" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G251" s="0" t="inlineStr">
         <is>
@@ -13524,7 +13314,7 @@
       </c>
       <c r="P251" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"In cooperation with the leaders of the rehabilitation centres, all health professionals (N = 167) engaged in working with patients in the centres were invited to participate in the survey. These centres deliver services via interprofessional teams; we identified 16 teams, which were the unit of interest in the present study, according to RC theory [9]. Some healthcare professionals were members of more than one team in the centre in which they worked; these professionals were asked to respond to the survey for each team they worked with.\" (Methods, Page 2) \"The main explanatory variables in this study were the RC communication and relationships scores, which were calculated for each team and used as continuous variables, from 1(lowest) to 5 (highest).\" (Methods, Page 4)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13586,10 +13376,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F253" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F253" s="0" t="n">
+        <v>2</v>
       </c>
       <c r="G253" s="0" t="inlineStr">
         <is>
@@ -13616,7 +13404,7 @@
       </c>
       <c r="P253" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 2\nPatient sample. Verbatim Evidence: "\"All patients aged 18 and above who were accepted for rehabilitation in a rehabilitation centre in Western Norway between January 2015 and June 2015 were invited to participate (n=2863). For baseline data collection, a total of 984 (34%) patients accepted the invitation to participate and provided written consent and a completed questionnaire. A 1-year follow-up questionnaire was sent to all participating patients (n=984), and 705 patients (25% of the patient group invited at baseline) returned the questionnaire. We extracted 279 of the baseline participants from the analyses, as they did not respond to the 1-year follow-up survey. Four respondents were omitted from the analyses due to missing data on outcome variables. Finally, 701 (24% of the patient group invited at baseline) patients were included in the analyses (Table 1).\" (Participants, Page 2-3)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13636,10 +13424,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F254" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F254" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G254" s="0" t="inlineStr">
         <is>
@@ -13666,7 +13452,7 @@
       </c>
       <c r="P254" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study only reports descriptive percentages for team-level feedback and does not provide an individual-level Pearson correlation matrix or quantitative effect sizes. Verbatim Evidence: "\"The questionnaire was designed to be used as a self-diagnostic instrument, and therefore the format of the feedback returned to the teams was specified according to the preferences of the teams. Teams preferred feedback in percentages above means; the sum of the percentages of team members that “agreed” and “agreed strongly” was reported. Also standard deviations were reported, and we volunteered to discuss scales and items with low percentages or high standard deviations in team meetings. In four teams the questionnaires were filled out individually during team meetings, however, the members of fifth team preferred to do this outer their meeting. There were 52 workers in the five teams, and 46 (88 per cent) completed the questionnaire.\" (The questionnaire, Page 59)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13686,10 +13472,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F255" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F255" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G255" s="0" t="inlineStr">
         <is>
@@ -13716,7 +13500,7 @@
       </c>
       <c r="P255" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Transformational leadership, gatekeeping leadership, internal communication, external communication, and norm for maintaining consensus were aggregated to mean values within each team, which was the unit of the analysis. To justify this aggregation, a within-group correlation (rwg) was computed to assess the amount of agreement by the team members (James et al. 1984). The mean rwg value was 0.87 for transformational leadership, 0.89 for gatekeeping leadership, 0.90 for internal communication, 0.89 for external communication, and 0.89 for norm for maintaining consensus. In addition, the ICC(1) values were as follows: transformational leadership, 0.22; gatekeeping leadership, 0.50; internal communication, 0.24; external communication, 0.36; and norm for maintaining consensus, 0.25. ICC(2) values were as follows: transformational leadership, 0.61; gatekeeping leadership, 0.85; internal communication, 0.64; external communication, 0.76; and norm for maintaining consensus, 0.65. The overall pattern of results across the rwg, ICC(1), and ICC(2) analyses provided sufficient support for aggregating the data to team level of analysis.\" (Aggregation tests, Page 11)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13736,10 +13520,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F256" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F256" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G256" s="0" t="inlineStr">
         <is>
@@ -13766,7 +13548,7 @@
       </c>
       <c r="P256" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>0 = Exclude\nReason Code: 3\nThe study uses work groups as the unit of analysis and aggregates individual survey responses to the team level. Verbatim Evidence: "\"Following Van de Ven and colleagues (1976) and Tushman (1977, 1978), we used work groups as the units of analysis. First-line supervisors with at least one year as unit heads who had full-time subordinates with sufficient experience to be familiar with their positions answered questions on the subordinates' jobs. The study included all units meeting the criterion for supervisory experience and containing at least two experienced subordinates. [...] To compute scores for work groups, supervisors' scores were added to the means of subordinates' scores, and these sums were divided by two (Van de Ven et al., 1976). Three tests supported this procedure. One-way analysis of variance (Dixon &amp; Massey, 1969) supported pooling subordinate responses into work groups for all of the variables (p &lt; .005).\" (Methods, pages 143-144)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13786,10 +13568,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F257" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F257" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G257" s="0" t="inlineStr">
         <is>
@@ -13816,7 +13596,7 @@
       </c>
       <c r="P257" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo individual-level bivariate Pearson correlation matrix is provided. The study only reports an aggregated organizational-level correlation matrix and jumps straight to regression for the individual-level analysis. Verbatim Evidence: "\"Regression analysis. First, a simple regression model was conducted to test if NCB significantly predicted IIB. The results of the regression indicated that NCB explained 17.8% of the variance in IIB (R2 = 17.8, F (1, 85) = 18.436, p&lt;.05). Next, a multiple regression analysis was conducted to test if NCB significantly predicted IIB after five demographic variables are controlled. The results of the multiple regression indicated that together with the four demographic variables, NCB predicted 30.5% of the variance in IIB (R2 = .305, F (6, 75) = 5.485, p&lt;.001).\" (Chapter 4: Data Analysis, Page 108)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13836,10 +13616,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F258" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F258" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G258" s="0" t="inlineStr">
         <is>
@@ -13866,7 +13644,7 @@
       </c>
       <c r="P258" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study samples boundary spanners but lacks an effect size for boundary spanning behavior, measuring only burnout, role stressors, and general job performance. Verbatim Evidence: "\"Job outcomes. Psychological outcomes were measured by three separate first-order constmcts. JS was operationalized as a 26-item scale adapted from Churchill, Ford, and Walker's (1985) study that has been frequently used in marketing. The alpha reliability of this scale was estimated as .92. OC was operationalized by use of a 6-item version of a scale from Mowday, Steers, and Porter (1979). Tbe scaie achieved acceptable reliability (a = .79). Finally, Tl was assessed by a three-item measure based on Donnelly and Ivancevicb (1975). In addition, this measure has been shown in several studies to be a consistent predictor of actual tumover. The Cronbach's a for this measure was .85. Behavioral out comes were measured by a self-rating, 6-item measure of JP drawn from Dubinsky and Mattson (1979).\" (Measures, page 563)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13886,10 +13664,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F259" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F259" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G259" s="0" t="inlineStr">
         <is>
@@ -13916,7 +13692,7 @@
       </c>
       <c r="P259" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: "\"In fact, because degree-based centrality measures are basically a standardized count of ties, a high actor degree centrality in an inter-organizational network equates to a higher level of BSA from the team's point of view. Consequently, the measure of BSA in this dissertation is the focal team's degree centrality in an inter-team network where the nodes are all OSS projects registered in Source Forge. This measure can be used since each project in Source Forge includes a list of developers. Once all these lists have been scanned, it is easy to detect developers who work on more than one project and then build the inter-team network in order to calculate a given project's BSA.\" (4.4.3.4 Boundary Spanning Activity, Page 99)\n"}"</t>
         </is>
       </c>
     </row>
@@ -13986,10 +13762,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F261" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F261" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G261" s="0" t="inlineStr">
         <is>
@@ -14016,7 +13790,7 @@
       </c>
       <c r="P261" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided; the study only reports mean differences and t-tests. Verbatim Evidence: "\"Measures used to test the hypotheses each consisted of two 7-point itemized rating scales designed to assess the extent to which team selling was used in a particular buying or selling situation. For example, to measure the extent to which team selling is used when the buyer’s informational needs are great, respondents indicated the likelihood of using sales teams when 'the anticipated information needs of the customer are small' and 'the anticipated information needs of the customer are great' (1 = extremely unlikely, 7 = extremely likely). T-tests were conducted on the mean differences between the respondents’ ratings for each of the paired questions. A hypothesis was supported when the mean difference was significantly different from 0.\" (Hypotheses Tests, page 160)\n"}"</t>
         </is>
       </c>
     </row>
@@ -14128,10 +13902,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F264" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F264" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G264" s="0" t="inlineStr">
         <is>
@@ -14158,7 +13930,7 @@
       </c>
       <c r="P264" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative case study lacking quantitative correlation data. Verbatim Evidence: "\"We use a case study research methodology to identify various contextual elements that shape the development of a common platform in a post-merger scenario. We examine how stakeholders from different business divisions establish a common understanding of their processes to inform the development of a common platform underlying a family of similar business processes. [...] We participated as observers in all the eight workshops and in six other meetings. Workshop meetings were audio-recorded with the participants’ consent, yielding an extremely rich set of data of over more than 50 h. Additional informal interviews with process participants were conducted to seek clarifications on issues raised during the workshops. See Online Appendix B for an excerpt of the interview questionnaire. These interviews allowed us to explore the expectations of the participants. Detailed notes were also taken during each of the data collection sessions. Workshops and interviews were our primary source of qualitative data.\" (Research methodology &amp; Data collection, Page 5-6)\n"}"</t>
         </is>
       </c>
     </row>
@@ -14220,10 +13992,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F266" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F266" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G266" s="0" t="inlineStr">
         <is>
@@ -14250,7 +14020,7 @@
       </c>
       <c r="P266" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"For our empirical analysis, we use data sets provided by the Netherlands Enterprise Agency (RVO.nl) on all collaborative R&amp;D projects that received support from the allowance scheme in the period 2013–2018. The data sets include information about project titles, starting years, participants and budgets. By merging the data, it is possible to map the evolution of the collaborative network for the period 2013–2018. The total network includes 1884 Dutch firms and 105 publicly-funded organizations. Given our focus on recombining firm capabilities, our analyses concentrate on the 1884 firms only.\" (Case description: collaborative R&amp;D in the Netherlands, Page 4)\n"}"</t>
         </is>
       </c>
     </row>
@@ -14510,10 +14280,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F272" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F272" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G272" s="0" t="inlineStr">
         <is>
@@ -14540,7 +14308,7 @@
       </c>
       <c r="P272" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided. Verbatim Evidence: "\"Grouping and Analytic Techniques. Each subject was grouped according to primary decision style which resulted in four groups of individuals being labeled as either SF (n = 20), ST (n = 7), NF (n = 24), or NT (n = 6). Because BSA was defined as multidimensional in nature and was composed of three separate dimensions, the primary analytic technique used was multivariate analysis of variance (MANOVA). This test was run to determine if decision style affected total BSA. Given a significant overall F for the MANOVA test, several post hoc techniques were employed to investigate the specific nature of these differences. First, a multivariate extension of the Scheffe test was used to determine which decision style groups were different from each other across the combination of the three BSA variables.\" (Grouping and Analytic Techniques, Page 6)\n"}"</t>
         </is>
       </c>
     </row>
@@ -14652,10 +14420,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F275" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F275" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G275" s="0" t="inlineStr">
         <is>
@@ -14682,7 +14448,7 @@
       </c>
       <c r="P275" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nProject and team level of analysis without individual employee boundary spanning correlations. Verbatim Evidence: "\"From the multiteam system (MTS) perspective, this study employs the input-process-outcome (IPO) framework and coordination theory to explore the influence of instant messaging-based team boundary spanning (IMTBS) on construction project coordination processes and project performance. A theoretical model is built and validated with a survey involving 206 construction projects. [...] Data were collected from construction projects in China. We first conducted a pilot study involving 30 respondents from the Master of Engineering Management (MEM) students majoring in construction management at a Chinese renowned university to test the validity of all constructs. [...] Then, the questionnaire was distributed to construction professionals to report the condition of the last completed project they managed. We randomly sent the link to the online survey to alumni of two renowned universities, who were involved in the construction industry. A total of 400 questionnaires were distributed to these alumni from 53 construction companies, and 256 responses were returned. After removing invalid responses, 206 valid questionnaires were left, thereby yielding a valid response rate of 51.5%.\" (Abstract, Page 1; 4.2 Data collection, Page 7)\n"}"</t>
         </is>
       </c>
     </row>
@@ -14702,10 +14468,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F276" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F276" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G276" s="0" t="inlineStr">
         <is>
@@ -14732,7 +14496,7 @@
       </c>
       <c r="P276" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"The referent-shift consensus model proposed by Chan[50]was used in designing the questionnaire, which means that variables including \"team boundary-spanning activities,\" \"team job crafting,\" and \"team innovation performance\" was designed from the perspective of the team. A request was made for these questions to be answered from the perspective of team awareness. The \"individual job crafting\" variable was designed from the employees' perspective. Second, the terminology, the clarity of the instructions, and the structure of the questionnaire's responses were evaluated by three subject-matter experts and five teams from Shandong province's universities engaged in scientific research and innovation. Modifications were made accordingly. Finally, teams that were developing collaborative innovation projects were selected. The distribution of 456 surveys resulted in the recovery of 400 questionnaires. Three hundred thirty-one valid surveys were retrieved after invalid data had been removed; these originated from 41 collaborative innovation teams.\" (3.1 Sample and data collection procedure, Page 6)\n"}"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update BSMA_Master_Coding_Sheet with BSMA0282
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -14923,7 +14923,7 @@
       </c>
       <c r="F285" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = non-individual level</t>
         </is>
       </c>
       <c r="G285" s="0" t="inlineStr">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="J285" s="0" t="inlineStr">
         <is>
-          <t>Kale, Prashant; Singh, Harbir; Perlmutter, Howard</t>
+          <t>Kale, Singh, and Perlmutter</t>
         </is>
       </c>
       <c r="K285" s="0" t="n">
@@ -14951,7 +14951,7 @@
       </c>
       <c r="P285" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Non-individual level. Verbatim Evidence: "The level of analysis is an alliance between two partners." (Data collection and sample)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Exclude BSMA0278 (Code 3: Firm-level analysis)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX704"/>
+  <dimension ref="A1:AX706"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.22" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.67" customWidth="1" style="31" min="1" max="16"/>
@@ -35552,8 +35552,82 @@
         </is>
       </c>
     </row>
-    <row r="705" ht="18" customHeight="1" s="31"/>
-    <row r="706" ht="18" customHeight="1" s="31"/>
+    <row r="705" ht="18" customHeight="1" s="31">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>BSMA0279</t>
+        </is>
+      </c>
+      <c r="E705" t="n">
+        <v>0</v>
+      </c>
+      <c r="F705" t="n">
+        <v>1</v>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>Linking Availability Expectations, Bidirectional Boundary Management Behavior and Preferences, and Employee Well-Being</t>
+        </is>
+      </c>
+      <c r="J705" t="inlineStr">
+        <is>
+          <t>Reinke &amp; Gerlach</t>
+        </is>
+      </c>
+      <c r="K705" t="n">
+        <v>2021</v>
+      </c>
+      <c r="P705" t="inlineStr">
+        <is>
+          <t>Wrong construct (work-life boundary management, not organizational boundary spanning). Verbatim Evidence: "how others’ availability expectations predict employees’ management of work and nonwork boundaries, and how these bidirectional boundary management behaviors relate to well-being." (Abstract)</t>
+        </is>
+      </c>
+    </row>
+    <row r="706" ht="18" customHeight="1" s="31">
+      <c r="A706" s="0" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B706" s="0" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="E706" s="0" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F706" s="0" t="inlineStr">
+        <is>
+          <t>3 = non-individual level</t>
+        </is>
+      </c>
+      <c r="H706" s="0" t="inlineStr">
+        <is>
+          <t>The Effects of Centrifugal and Centripetal Forces on Product Development Speed and Quality</t>
+        </is>
+      </c>
+      <c r="J706" s="0" t="inlineStr">
+        <is>
+          <t>Kwaku Atuahene-Gima</t>
+        </is>
+      </c>
+      <c r="K706" s="0" t="n">
+        <v>2003</v>
+      </c>
+      <c r="P706" s="0" t="inlineStr">
+        <is>
+          <t>Non-individual level (team/firm/org analysis). Verbatim Evidence: "I asked two team members in each participating project to provide a single consensual rating for the measures of these forces. I selected the team members upon the advice of senior managers who deemed them as being highly knowledgeable about their projects." (Measures and Validation)</t>
+        </is>
+      </c>
+    </row>
     <row r="707" ht="18" customHeight="1" s="31"/>
     <row r="708" ht="18" customHeight="1" s="31"/>
     <row r="709" ht="18" customHeight="1" s="31"/>

</xml_diff>

<commit_message>
Add BSMA0300 to master coding sheet
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX710"/>
+  <dimension ref="A1:AX711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35461,6 +35461,42 @@
         </is>
       </c>
     </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>Antigravity</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>BSMA0315</t>
+        </is>
+      </c>
+      <c r="E711" t="n">
+        <v>0</v>
+      </c>
+      <c r="F711" t="n">
+        <v>4</v>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>Retail corporate groups: Challenges of omnichannel management in Japan</t>
+        </is>
+      </c>
+      <c r="J711" t="inlineStr">
+        <is>
+          <t>Kimihiko Kondo</t>
+        </is>
+      </c>
+      <c r="K711" t="n">
+        <v>2018</v>
+      </c>
+      <c r="P711" t="inlineStr">
+        <is>
+          <t>[Non-primary conceptual study]. Verbatim Evidence: "From these challenges, we could propose further research issues as follows: (1) theoretical consideration of boundary-spanning functions among retail formats, (2) international comparative analysis reflecting the different conditions in each country, and (3) clarifying the characteristics of the omnichannel shopper in the Japanese omnichannel environment." (Abstract)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: save Batch 5 (34/40) results before server restart
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX711"/>
+  <dimension ref="A1:AX710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14287,10 +14287,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F277" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F277" t="n">
+        <v>1</v>
       </c>
       <c r="G277" t="inlineStr">
         <is>
@@ -14317,7 +14315,7 @@
       </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"[Construct homonymy: study measures work-family boundary management, not organizational boundary spanning behavior]. Verbatim Evidence: \\\"OBJECTIVE: This study was conducted to examine how teleworking outside regular office hours and individual boundary management relate to work-family conflict.\\\" (Abstract)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -14387,10 +14385,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F279" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F279" t="n">
+        <v>3</v>
       </c>
       <c r="G279" t="inlineStr">
         <is>
@@ -14417,7 +14413,7 @@
       </c>
       <c r="P279" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>\"This study describes the organizational arrangements used to source scientific knowledge in two highly successful NBFs -- firms that have succeeded in sourcing and commercializing valuable scientific knowledge. As both firms requested anonymity, we refer to them as Firm X and Firm Y.\" (4.1 Sample)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -14477,10 +14473,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F281" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F281" t="n">
+        <v>3</v>
       </c>
       <c r="G281" t="inlineStr">
         <is>
@@ -14507,7 +14501,7 @@
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"I asked two team members in each participating project to provide a single consensual rating for the measures of these forces. I selected the team members upon the advice of senior managers who deemed them as being highly knowledgeable about their projects.\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -14527,10 +14521,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F282" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F282" t="n">
+        <v>1</v>
       </c>
       <c r="G282" t="inlineStr">
         <is>
@@ -14570,7 +14562,7 @@
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"how others’ availability expectations predict employees’ management of work and nonwork boundaries, and how these bidirectional boundary management behaviors relate to well-being.\" (Abstract)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -14590,10 +14582,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F283" t="n">
+        <v>4</v>
       </c>
       <c r="G283" t="inlineStr">
         <is>
@@ -14620,7 +14610,7 @@
       </c>
       <c r="P283" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>\"Problems cross boundaries and so must solutions. The most important challenge for performance networks that aim to deliver better results is designing the structure that coordinates across traditional agency boundaries.\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -14640,10 +14630,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F284" t="n">
+        <v>3</v>
       </c>
       <c r="G284" t="inlineStr">
         <is>
@@ -14670,7 +14658,7 @@
       </c>
       <c r="P284" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>\"[Unit of analysis is at the team level]. Verbatim Evidence: \\\"To test hypotheses, the study focuses on technology transfer intermediaries of the manufacturing industry in China at the team level.\\\" (3.1 Research setting)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -14690,10 +14678,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr">
-        <is>
-          <t>3 = non-individual level</t>
-        </is>
+      <c r="F285" t="n">
+        <v>3</v>
       </c>
       <c r="G285" t="inlineStr">
         <is>
@@ -14720,7 +14706,7 @@
       </c>
       <c r="P285" t="inlineStr">
         <is>
-          <t>Non-individual level. Verbatim Evidence: "The level of analysis is an alliance between two partners." (Data collection and sample)</t>
+          <t>\"The level of analysis is an alliance between two partners.\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -14780,10 +14766,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F287" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F287" t="n">
+        <v>5</v>
       </c>
       <c r="G287" t="inlineStr">
         <is>
@@ -14810,7 +14794,7 @@
       </c>
       <c r="P287" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"Qualitative study without quantitative effect sizes based on a non-employee sample. Verbatim Evidence: \\\"This article is based on in-depth interviews with 30 subjects—15 men and 15 women.\\\" (Study design) and \\\"This article proposes to examine the self-concept of members of an occupational category called 'solo self-employed,' that is, women and men who work alone and do not employ any workers.\\\" (Introduction)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -14830,10 +14814,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F288" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F288" t="n">
+        <v>4</v>
       </c>
       <c r="G288" t="inlineStr">
         <is>
@@ -14860,14 +14842,14 @@
       </c>
       <c r="P288" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"The purpose of this paper is to develop the concept of project management system from the perspective of systems science.\" (Abstract)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -14880,10 +14862,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F289" t="n">
+        <v>3</v>
       </c>
       <c r="G289" t="inlineStr">
         <is>
@@ -14910,7 +14890,7 @@
       </c>
       <c r="P289" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Macro or group level study examining a boundary-spanning organization. Verbatim Evidence: "The theoretical contributions of this research provide empirical evidence through the boundary spanning lens to understand boundaries, the multiple roles and activities of a boundary-spanning organization" (5.1. Theoretical implications)</t>
         </is>
       </c>
     </row>
@@ -14930,10 +14910,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F290" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F290" t="n">
+        <v>1</v>
       </c>
       <c r="G290" t="inlineStr">
         <is>
@@ -14960,7 +14938,7 @@
       </c>
       <c r="P290" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"These are boundary theory (Ashforth et al., 2000; Allen et al., 2014; Nippert Eng, 1996), which focuses on the work-life domain, and border theory (Clark, 2000), which focuses on the work and family domain. As per these theories, individuals are forced to set boundaries to balance their work and family roles.\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -15130,10 +15108,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F294" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F294" t="n">
+        <v>3</v>
       </c>
       <c r="G294" t="inlineStr">
         <is>
@@ -15174,7 +15150,7 @@
       </c>
       <c r="P294" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"Study analyzes organizations rather than individuals. Verbatim Evidence: \\\"This paper, in an attempt to link up these ideas, investigates knowledge transfer processes within inter-organizational R&amp;D projects that are embedded in 23 German regional innovation networks (with almost 500 participants).\\\" (Abstract)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -15191,7 +15167,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -15434,10 +15410,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F300" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F300" t="n">
+        <v>3</v>
       </c>
       <c r="G300" t="inlineStr">
         <is>
@@ -15464,7 +15438,7 @@
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"Firm-level analysis. Verbatim Evidence: \\\"To gauge the study hypotheses, time-lagged data were gathered from 244 firms in China.\\\" (Abstract)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -15484,10 +15458,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F301" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F301" t="n">
+        <v>3</v>
       </c>
       <c r="G301" t="inlineStr">
         <is>
@@ -15514,7 +15486,7 @@
       </c>
       <c r="P301" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>\"the final dataset we retained and used for data analysis pertained to 365 firms.\"\n\nI have successfully updated BSMA_Master_Coding_Sheet.xlsx and committed and pushed the changes to Github.\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -15534,10 +15506,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F302" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F302" t="n">
+        <v>4</v>
       </c>
       <c r="G302" t="inlineStr">
         <is>
@@ -15564,7 +15534,7 @@
       </c>
       <c r="P302" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"Organizational behavior (OB) is an area of knowledge rather than a unified theory. It consists of a growing clutch of concepts, approaches, models, and tools pertinent to the structure and functioning of organizations within their socioeconomic contexts and of the study of individuals and groups within their organizational contexts\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -15634,10 +15604,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F304" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F304" t="n">
+        <v>1</v>
       </c>
       <c r="G304" t="inlineStr">
         <is>
@@ -15664,7 +15632,7 @@
       </c>
       <c r="P304" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>\"[No BSB construct measured]. Verbatim Evidence: \\\"The results indicate that FSEs’ perceptions of CSR are negatively related to their perceptions of verbal dysfunctional customer conduct, which in turn is shown to be directly linked to emotional exhaustion. FSEs’ CSR perceptions strengthen their view that they are performing meaningful work (i.e. perceived task significance), which in turn strengthens their job satisfaction.\\\" (Abstract)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -15826,7 +15794,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -15983,10 +15951,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F311" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F311" t="n">
+        <v>1</v>
       </c>
       <c r="G311" t="inlineStr">
         <is>
@@ -16013,7 +15979,7 @@
       </c>
       <c r="P311" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>\"Employees provided information regarding work overload, resilience, and intimidation, while their direct supervisors provided information regarding their subordinates’ sales performance.\" (3.2. Measures)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16033,10 +15999,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F312" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F312" t="n">
+        <v>1</v>
       </c>
       <c r="G312" t="inlineStr">
         <is>
@@ -16063,7 +16027,7 @@
       </c>
       <c r="P312" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"The study focuses on work-nonwork (work-life) boundary management rather than organizational boundary spanning behavior, hence there are no relevant effect sizes. Verbatim Evidence: \\\"In this study we focused on examining employees’ work-nonwork boundary management from the perspective of work stress recovery. Boundary management refers to the ways in which employees create, maintain and negotiate boundaries between work and nonwork\\\" (Introduction)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16083,10 +16047,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F313" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F313" t="n">
+        <v>3</v>
       </c>
       <c r="G313" t="inlineStr">
         <is>
@@ -16113,7 +16075,7 @@
       </c>
       <c r="P313" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"The purpose of this study was to analyze the school safety and security planning process. Sixty-two public school districts and non public schools within a fifty-mile radius of a large metropolitan area, located within the four states area of Texas, Oklahoma, Arkansas, and Kansas, were carefully studied\" (Abstract)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16187,10 +16149,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F315" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F315" t="n">
+        <v>1</v>
       </c>
       <c r="G315" t="inlineStr">
         <is>
@@ -16217,7 +16177,7 @@
       </c>
       <c r="P315" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>\"For each activity, we provide examples and illustrations which we derived by interviewing senior industry professionals from different industries (such as telecommunications, medical devices and pharmaceuticals) and with direct experiences in global boundary spanning and technology scouting. Specifically, between 2011–15, we conducted 15 in-depth interviews with managers in European and North American MNCs\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16237,10 +16197,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F316" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F316" t="n">
+        <v>1</v>
       </c>
       <c r="G316" t="inlineStr">
         <is>
@@ -16267,7 +16225,7 @@
       </c>
       <c r="P316" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"Data were analysed for all references to skills, knowledge, traits, behavioural indicators and outcomes associated with effective and ineffective performance. Over 250 items of data were identified. These were constructed into a framework describing the features of high performance, which was then critically reviewed by a small group of managers (the ‘review group’), and revised.\" (5 Findings)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16487,10 +16445,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F321" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F321" t="n">
+        <v>1</v>
       </c>
       <c r="G321" t="inlineStr">
         <is>
@@ -16517,7 +16473,7 @@
       </c>
       <c r="P321" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"The questionnaire was designed to measure the perceived: 1) importance and 2) effectiveness of each of the eight classes of MCP’s.\" (IV. METHOD)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16537,10 +16493,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F322" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F322" t="n">
+        <v>3</v>
       </c>
       <c r="G322" t="inlineStr">
         <is>
@@ -16567,7 +16521,7 @@
       </c>
       <c r="P322" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"The empirical setting is publicly held US manufacturing firms that are present in both the Kinder, Lydenberg and Domini’s (KLD’s) annual EVP ratings and Bloomberg’s supply chain database. The study employs panel data regression methods on an unbalanced panel dataset of 7,493 dyad-year observations comprising 427 unique firms.\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16637,10 +16591,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F324" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F324" t="n">
+        <v>3</v>
       </c>
       <c r="G324" t="inlineStr">
         <is>
@@ -16667,7 +16619,7 @@
       </c>
       <c r="P324" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>\"[Team-level aggregation]. Verbatim Evidence: \\\"To use the individuals’ responses for further analysis, the responses were aggregated by extracting the mean scores.\\\" (4. Results)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16687,10 +16639,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F325" t="n">
+        <v>3</v>
       </c>
       <c r="G325" t="inlineStr">
         <is>
@@ -16717,7 +16667,7 @@
       </c>
       <c r="P325" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"The questionnaire asked informants to focus on a NPD project (our unit of analysis) completed in the past 12 months.\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -16887,10 +16837,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F329" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F329" t="n">
+        <v>3</v>
       </c>
       <c r="G329" t="inlineStr">
         <is>
@@ -16917,7 +16865,7 @@
       </c>
       <c r="P329" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"Our study sample consisted of 2,940 United States Air Force officers from a broad array of job categories, who participated in a five-week leadership development course. As part of the course and a larger program of research,1 the participants were assigned to one of 210 14-person multiteam systems that engaged in a computer-based simulation.\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -17037,10 +16985,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F332" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F332" t="n">
+        <v>4</v>
       </c>
       <c r="G332" t="inlineStr">
         <is>
@@ -17067,7 +17013,7 @@
       </c>
       <c r="P332" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"Based on our experience and emerging literature, such as the papers in this special collection, this article discusses the value of Q-methodology in addressing landscape sustainability issues.\" (Abstract)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -17084,7 +17030,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
@@ -17187,10 +17133,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F335" t="n">
+        <v>3</v>
       </c>
       <c r="G335" t="inlineStr">
         <is>
@@ -17217,7 +17161,7 @@
       </c>
       <c r="P335" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries.\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -17287,10 +17231,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F337" t="n">
+        <v>1</v>
       </c>
       <c r="G337" t="inlineStr">
         <is>
@@ -17317,7 +17259,7 @@
       </c>
       <c r="P337" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>\"While formalization measure was modified slightly to be tailored to the unique Korean sales job environment, the other four variables of role ambiguity, role conflict, commitment, and propensity-to-leave were adopted from American literature.\" (Measurement)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -17547,10 +17489,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F343" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F343" t="n">
+        <v>3</v>
       </c>
       <c r="G343" t="inlineStr">
         <is>
@@ -17577,7 +17517,7 @@
       </c>
       <c r="P343" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>\"The unit of analysis for the questionnaire was the new product development project and the informant was asked to select the most recent project he/she worked for.\" (3.2. Questionnaire)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -17647,10 +17587,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F345" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F345" t="n">
+        <v>3</v>
       </c>
       <c r="G345" t="inlineStr">
         <is>
@@ -17677,7 +17615,7 @@
       </c>
       <c r="P345" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>\"The samples for the survey comprised IT development MTSs within IT firms located in China.\" (IV. METHODOLOGY, A. Samples and Data Collection)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -17697,10 +17635,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F346" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F346" t="n">
+        <v>3</v>
       </c>
       <c r="G346" t="inlineStr">
         <is>
@@ -17727,7 +17663,7 @@
       </c>
       <c r="P346" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>\"[Team level analysis]. Verbatim Evidence: \\\"We computed within-group interrater agreement (rwg; James, Demaree, &amp; Wolf, 1993) and ICC values to justify the aggregation of constructs to the team level, which provided adequate support.\\\" (Data Analysis)\"\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -35244,8 +35180,10 @@
           <t>BSMA0279</t>
         </is>
       </c>
-      <c r="E705" t="n">
-        <v>0</v>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
       </c>
       <c r="F705" t="n">
         <v>1</v>
@@ -35265,7 +35203,7 @@
       </c>
       <c r="P705" t="inlineStr">
         <is>
-          <t>Wrong construct (work-life boundary management, not organizational boundary spanning). Verbatim Evidence: "how others’ availability expectations predict employees’ management of work and nonwork boundaries, and how these bidirectional boundary management behaviors relate to well-being." (Abstract)</t>
+          <t>\"how others’ availability expectations predict employees’ management of work and nonwork boundaries, and how these bidirectional boundary management behaviors relate to well-being.\" (Abstract)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -35320,8 +35258,10 @@
           <t>BSMA0298</t>
         </is>
       </c>
-      <c r="E707" t="n">
-        <v>0</v>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
       </c>
       <c r="F707" t="n">
         <v>3</v>
@@ -35341,49 +35281,45 @@
       </c>
       <c r="P707" t="inlineStr">
         <is>
-          <t>Firm level of analysis (N = 365 firms). Verbatim Evidence: "the final dataset we retained and used for data analysis pertained to 365 firms." (3.1. Sample and procedure)</t>
+          <t>\"the final dataset we retained and used for data analysis pertained to 365 firms.\"\n\nI have successfully updated BSMA_Master_Coding_Sheet.xlsx and committed and pushed the changes to Github.\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Antigravity</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>BSMA0286</t>
-        </is>
-      </c>
-      <c r="C708" t="n">
-        <v>999</v>
-      </c>
-      <c r="D708" t="n">
-        <v>999</v>
-      </c>
-      <c r="E708" t="n">
-        <v>0</v>
+          <t>BSMA0300</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
       </c>
       <c r="F708" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H708" t="inlineStr">
         <is>
-          <t>An emergent taxonomy of boundary spanning in the smart city context – The case of smart Dublin</t>
+          <t>Enabling innovation in knowledge worker teams</t>
         </is>
       </c>
       <c r="J708" t="inlineStr">
         <is>
-          <t>Hadi Karimikia, Robert Bradshaw, Harminder Singh, Adegboyega Ojo, Brian Donnellan, Michael Guerin</t>
+          <t>Aino Kianto</t>
         </is>
       </c>
       <c r="K708" t="n">
-        <v>2022</v>
+        <v>2011</v>
       </c>
       <c r="P708" t="inlineStr">
         <is>
-          <t>Qualitative single case study using semi-structured interviews. Verbatim Evidence: "Semi-structured interviews were identified as the primary data collection method for this study and twenty-five interviews were conducted." (3.2. Data collection)</t>
+          <t>Team level analysis. Verbatim Evidence: "Respondents belonged to 20 teams. The team size ranged from 3–14 members (M = 5.30, SD = 2.66)." (Methods)</t>
         </is>
       </c>
     </row>
@@ -35395,103 +35331,65 @@
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>BSMA0300</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr">
-        <is>
-          <t>EXCLUDED</t>
-        </is>
+          <t>BSMA0316</t>
+        </is>
+      </c>
+      <c r="E709" t="n">
+        <v>0</v>
       </c>
       <c r="F709" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H709" t="inlineStr">
         <is>
-          <t>Enabling innovation in knowledge worker teams</t>
+          <t>ONLY GOOD FENCES KEEP GOOD NEIGHBOURS! THE INSTITUTIONALIZATION OF MINISTRY–AGENCY RELATIONSHIPS AT THE SCIENCE–POLICY NEXUS IN GERMAN FOOD SAFETY POLICY</t>
         </is>
       </c>
       <c r="J709" t="inlineStr">
         <is>
-          <t>Aino Kianto</t>
+          <t>Rebecca-Lea Korinek and Sylvia Veit</t>
         </is>
       </c>
       <c r="K709" t="n">
-        <v>2011</v>
+        <v>2015</v>
       </c>
       <c r="P709" t="inlineStr">
         <is>
-          <t>Team level analysis. Verbatim Evidence: "Respondents belonged to 20 teams. The team size ranged from 3–14 members (M = 5.30, SD = 2.66)." (Methods)</t>
+          <t>[Qualitative study]. Verbatim Evidence: "We conducted 23 semi-structured expert interviews from June 2011 to August 2012, which lasted from 45 to 120 minutes." (Data collection)</t>
         </is>
       </c>
     </row>
     <row r="710">
       <c r="A710" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Antigravity</t>
         </is>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>BSMA0316</t>
+          <t>BSMA0315</t>
         </is>
       </c>
       <c r="E710" t="n">
         <v>0</v>
       </c>
       <c r="F710" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H710" t="inlineStr">
         <is>
-          <t>ONLY GOOD FENCES KEEP GOOD NEIGHBOURS! THE INSTITUTIONALIZATION OF MINISTRY–AGENCY RELATIONSHIPS AT THE SCIENCE–POLICY NEXUS IN GERMAN FOOD SAFETY POLICY</t>
+          <t>Retail corporate groups: Challenges of omnichannel management in Japan</t>
         </is>
       </c>
       <c r="J710" t="inlineStr">
         <is>
-          <t>Rebecca-Lea Korinek and Sylvia Veit</t>
+          <t>Kimihiko Kondo</t>
         </is>
       </c>
       <c r="K710" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="P710" t="inlineStr">
-        <is>
-          <t>[Qualitative study]. Verbatim Evidence: "We conducted 23 semi-structured expert interviews from June 2011 to August 2012, which lasted from 45 to 120 minutes." (Data collection)</t>
-        </is>
-      </c>
-    </row>
-    <row r="711">
-      <c r="A711" t="inlineStr">
-        <is>
-          <t>Antigravity</t>
-        </is>
-      </c>
-      <c r="B711" t="inlineStr">
-        <is>
-          <t>BSMA0315</t>
-        </is>
-      </c>
-      <c r="E711" t="n">
-        <v>0</v>
-      </c>
-      <c r="F711" t="n">
-        <v>4</v>
-      </c>
-      <c r="H711" t="inlineStr">
-        <is>
-          <t>Retail corporate groups: Challenges of omnichannel management in Japan</t>
-        </is>
-      </c>
-      <c r="J711" t="inlineStr">
-        <is>
-          <t>Kimihiko Kondo</t>
-        </is>
-      </c>
-      <c r="K711" t="n">
-        <v>2018</v>
-      </c>
-      <c r="P711" t="inlineStr">
         <is>
           <t>[Non-primary conceptual study]. Verbatim Evidence: "From these challenges, we could propose further research issues as follows: (1) theoretical consideration of boundary-spanning functions among retail formats, (2) international comparative analysis reflecting the different conditions in each country, and (3) clarifying the characteristics of the omnichannel shopper in the Japanese omnichannel environment." (Abstract)</t>
         </is>

</xml_diff>

<commit_message>
fix: restore full string format for exclusion reason codes
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -729,8 +729,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>3</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -779,8 +781,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>2</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -829,8 +833,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>3</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -879,8 +885,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>3</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -929,8 +937,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>4</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -980,8 +990,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>2</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1030,8 +1042,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>3</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1080,8 +1094,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>4</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1130,8 +1146,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>3</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1180,8 +1198,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>3</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1230,8 +1250,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>2</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1280,8 +1302,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>4</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1330,8 +1354,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>1</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1390,8 +1416,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>1</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1499,8 +1527,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>4</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1553,8 +1583,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>1</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1603,8 +1635,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>1</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1663,8 +1697,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>3</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1717,8 +1753,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>4</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1767,8 +1805,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>4</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1827,8 +1867,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>3</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1884,8 +1926,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>3</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1934,8 +1978,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>1</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1984,8 +2030,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>3</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -2034,8 +2082,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>1</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2084,8 +2134,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>3</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2134,8 +2186,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>4</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2184,8 +2238,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>3</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2279,8 +2335,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>3</v>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2329,8 +2387,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>1</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2379,8 +2439,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>3</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2429,8 +2491,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>3</v>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2489,8 +2553,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>1</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2543,8 +2609,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>2</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2593,8 +2661,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F40" t="n">
-        <v>4</v>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2643,8 +2713,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>3</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2693,8 +2765,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>4</v>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2743,8 +2817,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>3</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2793,8 +2869,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>1</v>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2843,8 +2921,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>4</v>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -3009,8 +3089,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>4</v>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3069,8 +3151,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>1</v>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -3123,8 +3207,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F50" t="n">
-        <v>4</v>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -3183,8 +3269,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F51" t="n">
-        <v>3</v>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -3305,8 +3393,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>1</v>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -3359,8 +3449,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F54" t="n">
-        <v>3</v>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -3419,8 +3511,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F55" t="n">
-        <v>3</v>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -3483,8 +3577,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F56" t="n">
-        <v>1</v>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -3547,8 +3643,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>1</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3659,8 +3757,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F59" t="n">
-        <v>4</v>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -3709,8 +3809,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F60" t="n">
-        <v>3</v>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -3769,8 +3871,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>1</v>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -3828,8 +3932,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F62" t="n">
-        <v>3</v>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3888,8 +3994,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F63" t="n">
-        <v>4</v>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -3942,8 +4050,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F64" t="n">
-        <v>4</v>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -3992,8 +4102,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F65" t="n">
-        <v>2</v>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -4042,8 +4154,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F66" t="n">
-        <v>1</v>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -4092,8 +4206,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F67" t="n">
-        <v>4</v>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -4200,8 +4316,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>3</v>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -4250,8 +4368,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F70" t="n">
-        <v>1</v>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -4300,8 +4420,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F71" t="n">
-        <v>1</v>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -4383,8 +4505,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F72" t="n">
-        <v>4</v>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -4492,8 +4616,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F74" t="n">
-        <v>3</v>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -4542,8 +4668,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>3</v>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -4602,8 +4730,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>4</v>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -4656,8 +4786,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>3</v>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -4706,8 +4838,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F78" t="n">
-        <v>3</v>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -4756,8 +4890,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F79" t="n">
-        <v>3</v>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -4816,8 +4952,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F80" t="n">
-        <v>1</v>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -4870,8 +5008,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>3</v>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -4920,8 +5060,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F82" t="n">
-        <v>1</v>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -4970,8 +5112,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F83" t="n">
-        <v>3</v>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -5020,8 +5164,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F84" t="n">
-        <v>4</v>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -5113,8 +5259,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F86" t="n">
-        <v>4</v>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -5163,8 +5311,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F87" t="n">
-        <v>4</v>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -5213,8 +5363,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F88" t="n">
-        <v>3</v>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -5263,8 +5415,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F89" t="n">
-        <v>3</v>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -5313,8 +5467,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F90" t="n">
-        <v>3</v>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -5363,8 +5519,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F91" t="n">
-        <v>3</v>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -5413,8 +5571,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F92" t="n">
-        <v>3</v>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -5473,8 +5633,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F93" t="n">
-        <v>1</v>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -5527,8 +5689,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F94" t="n">
-        <v>3</v>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -5577,8 +5741,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F95" t="n">
-        <v>3</v>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -5637,8 +5803,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F96" t="n">
-        <v>4</v>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -5746,8 +5914,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F98" t="n">
-        <v>3</v>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -5800,8 +5970,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F99" t="n">
-        <v>4</v>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -5850,8 +6022,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F100" t="n">
-        <v>3</v>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -5900,8 +6074,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F101" t="n">
-        <v>3</v>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -5960,8 +6136,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F102" t="n">
-        <v>3</v>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -6024,8 +6202,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F103" t="n">
-        <v>3</v>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -6088,8 +6268,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F104" t="n">
-        <v>3</v>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -6142,8 +6324,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F105" t="n">
-        <v>3</v>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -6192,8 +6376,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F106" t="n">
-        <v>4</v>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -6242,8 +6428,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F107" t="n">
-        <v>3</v>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -6292,8 +6480,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F108" t="n">
-        <v>1</v>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -6342,8 +6532,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F109" t="n">
-        <v>1</v>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -6392,8 +6584,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F110" t="n">
-        <v>4</v>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -6442,8 +6636,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F111" t="n">
-        <v>3</v>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -6492,8 +6688,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F112" t="n">
-        <v>3</v>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -6542,8 +6740,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F113" t="n">
-        <v>4</v>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -6592,8 +6792,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F114" t="n">
-        <v>3</v>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -6641,8 +6843,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F115" t="n">
-        <v>1</v>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -6690,8 +6894,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F116" t="n">
-        <v>4</v>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -6739,8 +6945,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F117" t="n">
-        <v>1</v>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -6911,8 +7119,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F121" t="n">
-        <v>3</v>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -6960,8 +7170,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F122" t="n">
-        <v>4</v>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -7009,8 +7221,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F123" t="n">
-        <v>3</v>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -7098,8 +7312,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F125" t="n">
-        <v>3</v>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -7231,8 +7447,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F128" t="n">
-        <v>2</v>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -7363,8 +7581,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F131" t="n">
-        <v>3</v>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -7412,8 +7632,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F132" t="n">
-        <v>2</v>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -7561,8 +7783,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F135" t="n">
-        <v>4</v>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -7610,8 +7834,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F136" t="n">
-        <v>4</v>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -7749,8 +7975,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F139" t="n">
-        <v>4</v>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -7798,8 +8026,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F140" t="n">
-        <v>4</v>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -7847,8 +8077,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F141" t="n">
-        <v>4</v>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
@@ -7905,8 +8137,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F142" t="n">
-        <v>3</v>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -7954,8 +8188,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F143" t="n">
-        <v>1</v>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -8053,8 +8289,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F145" t="n">
-        <v>2</v>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -8203,8 +8441,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F148" t="n">
-        <v>3</v>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -8250,8 +8490,10 @@
       <c r="E149" t="n">
         <v>0</v>
       </c>
-      <c r="F149" t="n">
-        <v>1</v>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -8296,8 +8538,10 @@
       <c r="E150" t="n">
         <v>0</v>
       </c>
-      <c r="F150" t="n">
-        <v>4</v>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -8342,8 +8586,10 @@
       <c r="E151" t="n">
         <v>0</v>
       </c>
-      <c r="F151" t="n">
-        <v>3</v>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -8438,8 +8684,10 @@
       <c r="E153" t="n">
         <v>0</v>
       </c>
-      <c r="F153" t="n">
-        <v>4</v>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -8584,8 +8832,10 @@
       <c r="E156" t="n">
         <v>0</v>
       </c>
-      <c r="F156" t="n">
-        <v>99</v>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>99 = Other (specify in Notes)</t>
+        </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -8630,8 +8880,10 @@
       <c r="E157" t="n">
         <v>0</v>
       </c>
-      <c r="F157" t="n">
-        <v>3</v>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -8676,8 +8928,10 @@
       <c r="E158" t="n">
         <v>0</v>
       </c>
-      <c r="F158" t="n">
-        <v>3</v>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -8722,8 +8976,10 @@
       <c r="E159" t="n">
         <v>0</v>
       </c>
-      <c r="F159" t="n">
-        <v>4</v>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -8768,8 +9024,10 @@
       <c r="E160" t="n">
         <v>0</v>
       </c>
-      <c r="F160" t="n">
-        <v>3</v>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -8914,8 +9172,10 @@
       <c r="E163" t="n">
         <v>0</v>
       </c>
-      <c r="F163" t="n">
-        <v>3</v>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -8960,8 +9220,10 @@
       <c r="E164" t="n">
         <v>0</v>
       </c>
-      <c r="F164" t="n">
-        <v>1</v>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -9006,8 +9268,10 @@
       <c r="E165" t="n">
         <v>0</v>
       </c>
-      <c r="F165" t="n">
-        <v>4</v>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -9102,8 +9366,10 @@
       <c r="E167" t="n">
         <v>0</v>
       </c>
-      <c r="F167" t="n">
-        <v>1</v>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
@@ -9238,8 +9504,10 @@
       <c r="E170" t="n">
         <v>0</v>
       </c>
-      <c r="F170" t="n">
-        <v>2</v>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -9284,8 +9552,10 @@
       <c r="E171" t="n">
         <v>0</v>
       </c>
-      <c r="F171" t="n">
-        <v>3</v>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -9330,8 +9600,10 @@
       <c r="E172" t="n">
         <v>0</v>
       </c>
-      <c r="F172" t="n">
-        <v>3</v>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
@@ -9427,8 +9699,10 @@
       <c r="E174" t="n">
         <v>0</v>
       </c>
-      <c r="F174" t="n">
-        <v>1</v>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -9473,8 +9747,10 @@
       <c r="E175" t="n">
         <v>0</v>
       </c>
-      <c r="F175" t="n">
-        <v>3</v>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -9617,8 +9893,10 @@
       <c r="E178" t="n">
         <v>0</v>
       </c>
-      <c r="F178" t="n">
-        <v>4</v>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
@@ -9663,8 +9941,10 @@
       <c r="E179" t="n">
         <v>0</v>
       </c>
-      <c r="F179" t="n">
-        <v>3</v>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
@@ -9709,8 +9989,10 @@
       <c r="E180" t="n">
         <v>0</v>
       </c>
-      <c r="F180" t="n">
-        <v>3</v>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
@@ -9755,8 +10037,10 @@
       <c r="E181" t="n">
         <v>0</v>
       </c>
-      <c r="F181" t="n">
-        <v>1</v>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -9801,8 +10085,10 @@
       <c r="E182" t="n">
         <v>0</v>
       </c>
-      <c r="F182" t="n">
-        <v>1</v>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -9847,8 +10133,10 @@
       <c r="E183" t="n">
         <v>0</v>
       </c>
-      <c r="F183" t="n">
-        <v>1</v>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -9893,8 +10181,10 @@
       <c r="E184" t="n">
         <v>0</v>
       </c>
-      <c r="F184" t="n">
-        <v>4</v>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -9939,8 +10229,10 @@
       <c r="E185" t="n">
         <v>0</v>
       </c>
-      <c r="F185" t="n">
-        <v>4</v>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -9985,8 +10277,10 @@
       <c r="E186" t="n">
         <v>0</v>
       </c>
-      <c r="F186" t="n">
-        <v>1</v>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -10081,8 +10375,10 @@
       <c r="E188" t="n">
         <v>0</v>
       </c>
-      <c r="F188" t="n">
-        <v>1</v>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -10217,8 +10513,10 @@
       <c r="E191" t="n">
         <v>0</v>
       </c>
-      <c r="F191" t="n">
-        <v>4</v>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -10263,8 +10561,10 @@
       <c r="E192" t="n">
         <v>0</v>
       </c>
-      <c r="F192" t="n">
-        <v>4</v>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -10309,8 +10609,10 @@
       <c r="E193" t="n">
         <v>0</v>
       </c>
-      <c r="F193" t="n">
-        <v>3</v>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -10355,8 +10657,10 @@
       <c r="E194" t="n">
         <v>0</v>
       </c>
-      <c r="F194" t="n">
-        <v>3</v>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -10551,8 +10855,10 @@
       <c r="E198" t="n">
         <v>0</v>
       </c>
-      <c r="F198" t="n">
-        <v>3</v>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -10597,8 +10903,10 @@
       <c r="E199" t="n">
         <v>0</v>
       </c>
-      <c r="F199" t="n">
-        <v>3</v>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -10643,8 +10951,10 @@
       <c r="E200" t="n">
         <v>0</v>
       </c>
-      <c r="F200" t="n">
-        <v>1</v>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -10689,8 +10999,10 @@
       <c r="E201" t="n">
         <v>0</v>
       </c>
-      <c r="F201" t="n">
-        <v>4</v>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -10735,8 +11047,10 @@
       <c r="E202" t="n">
         <v>0</v>
       </c>
-      <c r="F202" t="n">
-        <v>4</v>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -10781,8 +11095,10 @@
       <c r="E203" t="n">
         <v>0</v>
       </c>
-      <c r="F203" t="n">
-        <v>4</v>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -10829,8 +11145,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F204" t="n">
-        <v>3</v>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -11017,8 +11335,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F208" t="n">
-        <v>3</v>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -11255,8 +11575,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F213" t="n">
-        <v>1</v>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -11483,8 +11805,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F218" t="n">
-        <v>99</v>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>99 = Other (specify in Notes)</t>
+        </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -11531,8 +11855,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F219" t="n">
-        <v>3</v>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -11674,8 +12000,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F222" t="n">
-        <v>4</v>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -11722,8 +12050,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F223" t="n">
-        <v>4</v>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -11770,8 +12100,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F224" t="n">
-        <v>3</v>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -11868,8 +12200,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F226" t="n">
-        <v>1</v>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -11916,8 +12250,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F227" t="n">
-        <v>3</v>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -12014,8 +12350,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F229" t="n">
-        <v>3</v>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -12062,8 +12400,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F230" t="n">
-        <v>3</v>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -12160,8 +12500,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F232" t="n">
-        <v>4</v>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -12208,8 +12550,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F233" t="n">
-        <v>3</v>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -12306,8 +12650,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F235" t="n">
-        <v>3</v>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -12444,8 +12790,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F238" t="n">
-        <v>4</v>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -12542,8 +12890,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F240" t="n">
-        <v>3</v>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -12590,8 +12940,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F241" t="n">
-        <v>3</v>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -12683,8 +13035,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F243" t="n">
-        <v>3</v>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -12731,8 +13085,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F244" t="n">
-        <v>1</v>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -12779,8 +13135,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F245" t="n">
-        <v>1</v>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -12827,8 +13185,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F246" t="n">
-        <v>3</v>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -13065,8 +13425,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F251" t="n">
-        <v>3</v>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -13153,8 +13515,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F253" t="n">
-        <v>2</v>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -13201,8 +13565,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F254" t="n">
-        <v>1</v>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -13249,8 +13615,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F255" t="n">
-        <v>3</v>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -13297,8 +13665,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F256" t="n">
-        <v>3</v>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -13345,8 +13715,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F257" t="n">
-        <v>1</v>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -13393,8 +13765,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F258" t="n">
-        <v>1</v>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -13441,8 +13815,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F259" t="n">
-        <v>3</v>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -13539,8 +13915,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F261" t="n">
-        <v>1</v>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -13677,8 +14055,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F264" t="n">
-        <v>4</v>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -13765,8 +14145,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F266" t="n">
-        <v>3</v>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -14053,8 +14435,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F272" t="n">
-        <v>1</v>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -14191,8 +14575,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F275" t="n">
-        <v>3</v>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -14239,8 +14625,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F276" t="n">
-        <v>3</v>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -14287,8 +14675,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F277" t="n">
-        <v>1</v>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
@@ -14385,8 +14775,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F279" t="n">
-        <v>3</v>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
@@ -14473,8 +14865,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F281" t="n">
-        <v>3</v>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
@@ -14521,8 +14915,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F282" t="n">
-        <v>1</v>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
@@ -14582,8 +14978,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F283" t="n">
-        <v>4</v>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G283" t="inlineStr">
         <is>
@@ -14630,8 +15028,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F284" t="n">
-        <v>3</v>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G284" t="inlineStr">
         <is>
@@ -14678,8 +15078,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F285" t="n">
-        <v>3</v>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
@@ -14766,8 +15168,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F287" t="n">
-        <v>5</v>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
       </c>
       <c r="G287" t="inlineStr">
         <is>
@@ -14814,8 +15218,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F288" t="n">
-        <v>4</v>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G288" t="inlineStr">
         <is>
@@ -14862,8 +15268,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F289" t="n">
-        <v>3</v>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G289" t="inlineStr">
         <is>
@@ -14910,8 +15318,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F290" t="n">
-        <v>1</v>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
@@ -15108,8 +15518,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F294" t="n">
-        <v>3</v>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G294" t="inlineStr">
         <is>
@@ -15410,8 +15822,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F300" t="n">
-        <v>3</v>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G300" t="inlineStr">
         <is>
@@ -15458,8 +15872,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F301" t="n">
-        <v>3</v>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G301" t="inlineStr">
         <is>
@@ -15506,8 +15922,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F302" t="n">
-        <v>4</v>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G302" t="inlineStr">
         <is>
@@ -15604,8 +16022,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F304" t="n">
-        <v>1</v>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G304" t="inlineStr">
         <is>
@@ -15951,8 +16371,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F311" t="n">
-        <v>1</v>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G311" t="inlineStr">
         <is>
@@ -15999,8 +16421,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F312" t="n">
-        <v>1</v>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G312" t="inlineStr">
         <is>
@@ -16047,8 +16471,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F313" t="n">
-        <v>3</v>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G313" t="inlineStr">
         <is>
@@ -16149,8 +16575,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F315" t="n">
-        <v>1</v>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G315" t="inlineStr">
         <is>
@@ -16197,8 +16625,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F316" t="n">
-        <v>1</v>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G316" t="inlineStr">
         <is>
@@ -16445,8 +16875,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F321" t="n">
-        <v>1</v>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G321" t="inlineStr">
         <is>
@@ -16493,8 +16925,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F322" t="n">
-        <v>3</v>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G322" t="inlineStr">
         <is>
@@ -16591,8 +17025,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F324" t="n">
-        <v>3</v>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G324" t="inlineStr">
         <is>
@@ -16639,8 +17075,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F325" t="n">
-        <v>3</v>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
@@ -16837,8 +17275,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F329" t="n">
-        <v>3</v>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
@@ -16985,8 +17425,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F332" t="n">
-        <v>4</v>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="G332" t="inlineStr">
         <is>
@@ -17133,8 +17575,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F335" t="n">
-        <v>3</v>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G335" t="inlineStr">
         <is>
@@ -17231,8 +17675,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F337" t="n">
-        <v>1</v>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="G337" t="inlineStr">
         <is>
@@ -17489,8 +17935,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F343" t="n">
-        <v>3</v>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
@@ -17587,8 +18035,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F345" t="n">
-        <v>3</v>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
@@ -17635,8 +18085,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F346" t="n">
-        <v>3</v>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
@@ -35185,8 +35637,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F705" t="n">
-        <v>1</v>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="H705" t="inlineStr">
         <is>
@@ -35263,8 +35717,10 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F707" t="n">
-        <v>3</v>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="H707" t="inlineStr">
         <is>
@@ -35301,8 +35757,10 @@
           <t>EXCLUDED</t>
         </is>
       </c>
-      <c r="F708" t="n">
-        <v>3</v>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="H708" t="inlineStr">
         <is>
@@ -35337,8 +35795,10 @@
       <c r="E709" t="n">
         <v>0</v>
       </c>
-      <c r="F709" t="n">
-        <v>1</v>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
       </c>
       <c r="H709" t="inlineStr">
         <is>
@@ -35373,8 +35833,10 @@
       <c r="E710" t="n">
         <v>0</v>
       </c>
-      <c r="F710" t="n">
-        <v>4</v>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
       </c>
       <c r="H710" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: inject accurate 2nd screening audit verbatim quotes for BSMA0001-0010
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -913,7 +913,7 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="P4" s="0" t="inlineStr">
         <is>
-          <t>Team-level study: Examines team diversity and team-level boundary spanning behaviors (unit of analysis is work team).</t>
+          <t>\"The data analyzed in this dissertation exist at three levels- the individual level, the team level and the service region unit level. For the team process measures, data were aggregated from the individual to the team level. Table 3 in Appendix 1 presents ICC coefficients for the aggregation of the team process variables from individual to the team level. The ICCs for this aggregation range from .10 ( for intra-team cooperation) to .07 (for inter-team cooperation) with an average ICC of .08. These results suggest that on average 8% of the variance in the team process measures were explained by differences between teams.\" (Data Aggregation, Page 70)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="P5" s="0" t="inlineStr">
         <is>
-          <t>Macro-economic / urban planning study: Examines 1930s HOLC redlining maps and neighborhood opportunity (sample is census tracts/residents, not organizational employees).</t>
+          <t>\"Two sets of data are fit to the quarter mile or longer rectangular buffer zones: characteristics from the 1910 to 1930 decennial censuses and outcomes from the Opportunity Atlas. On the former, we use the 1910 to 1930 100 percent Census population counts from Minnesota Population Center and Ancestry.com (2013). We are able to match roughly 50 to 80 percent of respondents to HOLC neighborhoods.7 We aggregate census measures to the buffer zone by taking the mean of all observations which fall inside of a buffer zone so long as it contains at least 3 households.\" (Data, Page 8)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="P6" s="0" t="inlineStr">
         <is>
-          <t>Organizational-level study: Investigates cross-sector governance and collaboration capacity of U.S. city governments (unit of analysis is local government/city).</t>
+          <t>\"The data for this research is drawn from the 2016 International City/County Management Association (ICMA) Smart Cities Survey. Partnering with the Smart Cities Council, ICMA sent the survey in 2016 to 3,423 local government officers working in U.S. cities and counties with populations of 25,000 or greater. In all, 493 officers responded to the survey questions by email or mail, giving a response rate of 14.4%. The survey consisted of twenty questions asking officers about their local governments’ smart cities practices including: their commitment to SCT (priorities), their engagement with SCT (activities), their perceived benefits of using SCT, and their barriers to implementing SCT. The survey also provides insights into the extent to which local governments pursuing SCT are collaborating with other government agencies and authorities. The survey further offers information on the financial mechanisms localities are using to fund SCT efforts and projects. The data from the ICMA survey was merged with information on demographic, economic, and population data drawn from the 2016 U.S. Census Bureau database. After eliminating records with missing data, our final sample includes responses from 234 local governments.\" (Methodology, Page 247)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="P7" s="0" t="inlineStr">
         <is>
-          <t>Team-level study: Examines knowledge integration capability and cooperative strategy in teams (unit of analysis is project team).</t>
+          <t>\"The unit of analysis of this study is firm. A firm is used as the unit of analysis because the research questions seek to examine factors that determine a firm’s ability to innovate and to integrate employees’ knowledge. Various researchers have also used firm as the unit of analysis to examine a firm's ability to innovate in the various contexts, such as network ties (Ozer &amp; Zhang, 2015), firm size (Leiblein &amp; Madsen, 2009), and strategic fit (Kim, Arthurs, Sahaym, &amp; Cullen, 2013).\" (Unit of Analysis, Page 66)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="P8" s="0" t="inlineStr">
         <is>
-          <t>Conceptual / review article: Discusses community-academic partnerships (CAPs) in social work; no quantitative empirical dataset or effect sizes reported.</t>
+          <t>\"In this article, the author begins by defining collaborative partnerships between academics and community stakeholders and then states specific advantages and challenges to collaborative partnerships in the field of social work. Throughout, the author explains how the historical foundations of the field (for example, acting as boundary spanners, advocating for marginalized individuals) place social workers in an ideal position to become leaders in the development, sustainment, and strengthening of CAPs. The author details the ways in which social work researchers can use the field’s unique history to enhance the development and sustainment of CAPs. The article concludes by encouraging the field to use standardized terminology, methodology, and evaluation procedures when conducting CAPs and providing strategies for social work researchers who wish to increase their ability to develop and sustain CAPs within their own institutions.\" (Abstract, Page 19)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="P9" s="0" t="inlineStr">
         <is>
-          <t>Customer sample study: Examines customer-company identification among prescribing physicians (customers/clients), not internal employee boundary spanners.</t>
+          <t>\"A sample of 2,000 high-prescribing physicians was randomly drawn from a population of over 30,000 high-prescribing physicians in the focal drug category. We considered only high-prescribing physicians for this research to ensure that each physician wrote a sufficient number of prescriptions in the category and that the sales representatives would have had regular contact with the physicians (e.g., industry records indicate that the representative calls on the high-prescribing physician on average 26 times per year). A professional market research company contacted these 2,000 physician offices by telephone and invited physicians to participate in a survey that was being conducted and independently funded by a major U.S. university. Questionnaires were distributed to this sample of physicians via fax. Participants were assured that their individual responses would be confidential and received a $30 industry-standard honorarium for their participation. Completed surveys were faxed directly back to the researchers, yielding a final sample of 178 physicians.\" (Method, page 5)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G10" s="0" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="P10" s="0" t="inlineStr">
         <is>
-          <t>Firm-level study: Investigates incumbent firm adaptation and technological alliances (unit of analysis is firm-therapeutic level in biotech/pharma).</t>
+          <t>\"The unit of analysis is the firm-therapeutic level, i.e., the firm's alliance activities in a therapeutic area (for example, Merck's alliances in cardiovascular therapeutic area). The arguments are tested using panel data estimation techniques... The study identified 1932 alliances formed between incumbent pharmaceutical and new biotechnology firms in eighteen therapeutic areas by seventeen large pharmaceutical firms during the time period from 1991 to 2004. The focal firms are traditional pharmaceutical firms listed under Standard Industrial Classification (SIC) codes 2834 and 5122, 'Pharmaceutical Preparations' and 'Wholesale-Drugs, Proprietaries &amp; Druggists Sundries' respectively. In this industry, the incumbent pharmaceutical firms are primarily attempting to adapt to the emerging technologies by forming alliances (i.e., equity and non-equity partnerships) with new biotechnology firms (Rothaermel, 2000).\" (Methods / Sample and Data, Page 9)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G11" s="0" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="P11" s="0" t="inlineStr">
         <is>
-          <t>Tourist sample study: Examines self-transformation and learning of adventure tourists, not organizational employee workplace behavior.</t>
+          <t>\"However, these hypotheses are unobservable and are not a priori shared in the public domain. Therefore, as previously mentioned, separate empirical experiments are necessary. In this section, we discuss how the modified explanatory hypotheses can be validated through experimentation. As an example of experimental method, it would be appropriate to employ a structured questionnaire and participant observation in case study, and to select an analytical method that can show a strong explanatory model with a small number of samples while converting qualitative information into quantitative information, such as Qualitative Comparative Analysis (QCA), for the data collected.\" (4. Conclusion, limitations, and future directions, Page 7)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G12" s="0" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="P12" s="0" t="inlineStr">
         <is>
-          <t>Team-level study: Examines new product development (NPD) team intelligence and project success (unit of analysis is NPD team).</t>
+          <t>\"Since our study focused on the NPD team as a unit of analysis, product/project managers were likely to assess our variables more accurately. Also, the sample of respondents was similar to samples used in prior studies on innovation. Each product/project manager in the PMI mailing list received an invitation to participate in our study (including a cover letter, the questionnaire, and stamped return envelope). Informants were asked to focus on their most recent product development projects (ones in the marketplace for a minimum of 12 months to ensure accurate assessment of the product performance). We received 207 usable responses (an effective response rate of 16.5%) representing a wide range of industries in the manufacturing sector, including: pharmaceuticals (28.5%), automotive (17%), electrical/electronics (17.9%), computers (13%), chemicals (8.7%), machinery/metal manufacturing (7.2%), and others (7.2%).\" (Measures and sampling, Page 223)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G13" s="0" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="P13" s="0" t="inlineStr">
         <is>
-          <t>Team-level study: Examines team sensemaking capability and performance in product development project teams (unit of analysis is project team).</t>
+          <t>\"Among the 180 firms contacted, we received 92 usable returns concerning NPD projects. During the sampling, to assess the product performance more accurately, we set the condition that the products used in this study must have been commercialized and launched into the marketplace for at least six months (Lynn et al., 2000). Also, the team size was an important constraint such that it should contain more than three members. Furthermore, to reduce the possible problems associated with single sourcing, we targeted the product or project manager to complete the survey. These managers were chosen because (1) product/project managers are likely to have a ‘bigger-picture view’ of NPD projects than other team members; (2) project managers have a broader view of each member’s behaviors than other team members\" (4.1. Sampling, Page 7)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
         </is>
       </c>
     </row>
@@ -23684,7 +23684,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F461" t="inlineStr">
+      <c r="F461" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -23784,7 +23784,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F463" t="inlineStr">
+      <c r="F463" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -24034,7 +24034,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F468" t="inlineStr">
+      <c r="F468" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -24230,7 +24230,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F472" t="inlineStr">
+      <c r="F472" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -24380,7 +24380,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F475" t="inlineStr">
+      <c r="F475" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -24430,7 +24430,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F476" t="inlineStr">
+      <c r="F476" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -24576,7 +24576,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F479" t="inlineStr">
+      <c r="F479" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -24622,7 +24622,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F480" t="inlineStr">
+      <c r="F480" s="0" t="inlineStr">
         <is>
           <t>1 = Include</t>
         </is>
@@ -24668,7 +24668,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F481" t="inlineStr">
+      <c r="F481" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level</t>
         </is>
@@ -24768,7 +24768,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F483" t="inlineStr">
+      <c r="F483" s="0" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
         </is>

</xml_diff>

<commit_message>
fix: clean system tags from verbatim evidence columns
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -941,7 +941,7 @@
       </c>
       <c r="P4" s="0" t="inlineStr">
         <is>
-          <t>\"The data analyzed in this dissertation exist at three levels- the individual level, the team level and the service region unit level. For the team process measures, data were aggregated from the individual to the team level. Table 3 in Appendix 1 presents ICC coefficients for the aggregation of the team process variables from individual to the team level. The ICCs for this aggregation range from .10 ( for intra-team cooperation) to .07 (for inter-team cooperation) with an average ICC of .08. These results suggest that on average 8% of the variance in the team process measures were explained by differences between teams.\" (Data Aggregation, Page 70)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>The data analyzed in this dissertation exist at three levels- the individual level, the team level and the service region unit level. For the team process measures, data were aggregated from the individual to the team level. Table 3 in Appendix 1 presents ICC coefficients for the aggregation of the team process variables from individual to the team level. The ICCs for this aggregation range from .10 ( for intra-team cooperation) to .07 (for inter-team cooperation) with an average ICC of .08. These results suggest that on average 8% of the variance in the team process measures were explained by differences between teams.\" (Data Aggregation, Page 70)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="P5" s="0" t="inlineStr">
         <is>
-          <t>\"Two sets of data are fit to the quarter mile or longer rectangular buffer zones: characteristics from the 1910 to 1930 decennial censuses and outcomes from the Opportunity Atlas. On the former, we use the 1910 to 1930 100 percent Census population counts from Minnesota Population Center and Ancestry.com (2013). We are able to match roughly 50 to 80 percent of respondents to HOLC neighborhoods.7 We aggregate census measures to the buffer zone by taking the mean of all observations which fall inside of a buffer zone so long as it contains at least 3 households.\" (Data, Page 8)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>Two sets of data are fit to the quarter mile or longer rectangular buffer zones: characteristics from the 1910 to 1930 decennial censuses and outcomes from the Opportunity Atlas. On the former, we use the 1910 to 1930 100 percent Census population counts from Minnesota Population Center and Ancestry.com (2013). We are able to match roughly 50 to 80 percent of respondents to HOLC neighborhoods.7 We aggregate census measures to the buffer zone by taking the mean of all observations which fall inside of a buffer zone so long as it contains at least 3 households.\" (Data, Page 8)</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="P6" s="0" t="inlineStr">
         <is>
-          <t>\"The data for this research is drawn from the 2016 International City/County Management Association (ICMA) Smart Cities Survey. Partnering with the Smart Cities Council, ICMA sent the survey in 2016 to 3,423 local government officers working in U.S. cities and counties with populations of 25,000 or greater. In all, 493 officers responded to the survey questions by email or mail, giving a response rate of 14.4%. The survey consisted of twenty questions asking officers about their local governments’ smart cities practices including: their commitment to SCT (priorities), their engagement with SCT (activities), their perceived benefits of using SCT, and their barriers to implementing SCT. The survey also provides insights into the extent to which local governments pursuing SCT are collaborating with other government agencies and authorities. The survey further offers information on the financial mechanisms localities are using to fund SCT efforts and projects. The data from the ICMA survey was merged with information on demographic, economic, and population data drawn from the 2016 U.S. Census Bureau database. After eliminating records with missing data, our final sample includes responses from 234 local governments.\" (Methodology, Page 247)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>The data for this research is drawn from the 2016 International City/County Management Association (ICMA) Smart Cities Survey. Partnering with the Smart Cities Council, ICMA sent the survey in 2016 to 3,423 local government officers working in U.S. cities and counties with populations of 25,000 or greater. In all, 493 officers responded to the survey questions by email or mail, giving a response rate of 14.4%. The survey consisted of twenty questions asking officers about their local governments’ smart cities practices including: their commitment to SCT (priorities), their engagement with SCT (activities), their perceived benefits of using SCT, and their barriers to implementing SCT. The survey also provides insights into the extent to which local governments pursuing SCT are collaborating with other government agencies and authorities. The survey further offers information on the financial mechanisms localities are using to fund SCT efforts and projects. The data from the ICMA survey was merged with information on demographic, economic, and population data drawn from the 2016 U.S. Census Bureau database. After eliminating records with missing data, our final sample includes responses from 234 local governments.\" (Methodology, Page 247)</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="P7" s="0" t="inlineStr">
         <is>
-          <t>\"The unit of analysis of this study is firm. A firm is used as the unit of analysis because the research questions seek to examine factors that determine a firm’s ability to innovate and to integrate employees’ knowledge. Various researchers have also used firm as the unit of analysis to examine a firm's ability to innovate in the various contexts, such as network ties (Ozer &amp; Zhang, 2015), firm size (Leiblein &amp; Madsen, 2009), and strategic fit (Kim, Arthurs, Sahaym, &amp; Cullen, 2013).\" (Unit of Analysis, Page 66)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>The unit of analysis of this study is firm. A firm is used as the unit of analysis because the research questions seek to examine factors that determine a firm’s ability to innovate and to integrate employees’ knowledge. Various researchers have also used firm as the unit of analysis to examine a firm's ability to innovate in the various contexts, such as network ties (Ozer &amp; Zhang, 2015), firm size (Leiblein &amp; Madsen, 2009), and strategic fit (Kim, Arthurs, Sahaym, &amp; Cullen, 2013).\" (Unit of Analysis, Page 66)</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="P8" s="0" t="inlineStr">
         <is>
-          <t>\"In this article, the author begins by defining collaborative partnerships between academics and community stakeholders and then states specific advantages and challenges to collaborative partnerships in the field of social work. Throughout, the author explains how the historical foundations of the field (for example, acting as boundary spanners, advocating for marginalized individuals) place social workers in an ideal position to become leaders in the development, sustainment, and strengthening of CAPs. The author details the ways in which social work researchers can use the field’s unique history to enhance the development and sustainment of CAPs. The article concludes by encouraging the field to use standardized terminology, methodology, and evaluation procedures when conducting CAPs and providing strategies for social work researchers who wish to increase their ability to develop and sustain CAPs within their own institutions.\" (Abstract, Page 19)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>In this article, the author begins by defining collaborative partnerships between academics and community stakeholders and then states specific advantages and challenges to collaborative partnerships in the field of social work. Throughout, the author explains how the historical foundations of the field (for example, acting as boundary spanners, advocating for marginalized individuals) place social workers in an ideal position to become leaders in the development, sustainment, and strengthening of CAPs. The author details the ways in which social work researchers can use the field’s unique history to enhance the development and sustainment of CAPs. The article concludes by encouraging the field to use standardized terminology, methodology, and evaluation procedures when conducting CAPs and providing strategies for social work researchers who wish to increase their ability to develop and sustain CAPs within their own institutions.\" (Abstract, Page 19)</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="P9" s="0" t="inlineStr">
         <is>
-          <t>\"A sample of 2,000 high-prescribing physicians was randomly drawn from a population of over 30,000 high-prescribing physicians in the focal drug category. We considered only high-prescribing physicians for this research to ensure that each physician wrote a sufficient number of prescriptions in the category and that the sales representatives would have had regular contact with the physicians (e.g., industry records indicate that the representative calls on the high-prescribing physician on average 26 times per year). A professional market research company contacted these 2,000 physician offices by telephone and invited physicians to participate in a survey that was being conducted and independently funded by a major U.S. university. Questionnaires were distributed to this sample of physicians via fax. Participants were assured that their individual responses would be confidential and received a $30 industry-standard honorarium for their participation. Completed surveys were faxed directly back to the researchers, yielding a final sample of 178 physicians.\" (Method, page 5)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>A sample of 2,000 high-prescribing physicians was randomly drawn from a population of over 30,000 high-prescribing physicians in the focal drug category. We considered only high-prescribing physicians for this research to ensure that each physician wrote a sufficient number of prescriptions in the category and that the sales representatives would have had regular contact with the physicians (e.g., industry records indicate that the representative calls on the high-prescribing physician on average 26 times per year). A professional market research company contacted these 2,000 physician offices by telephone and invited physicians to participate in a survey that was being conducted and independently funded by a major U.S. university. Questionnaires were distributed to this sample of physicians via fax. Participants were assured that their individual responses would be confidential and received a $30 industry-standard honorarium for their participation. Completed surveys were faxed directly back to the researchers, yielding a final sample of 178 physicians.\" (Method, page 5)</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="P10" s="0" t="inlineStr">
         <is>
-          <t>\"The unit of analysis is the firm-therapeutic level, i.e., the firm's alliance activities in a therapeutic area (for example, Merck's alliances in cardiovascular therapeutic area). The arguments are tested using panel data estimation techniques... The study identified 1932 alliances formed between incumbent pharmaceutical and new biotechnology firms in eighteen therapeutic areas by seventeen large pharmaceutical firms during the time period from 1991 to 2004. The focal firms are traditional pharmaceutical firms listed under Standard Industrial Classification (SIC) codes 2834 and 5122, 'Pharmaceutical Preparations' and 'Wholesale-Drugs, Proprietaries &amp; Druggists Sundries' respectively. In this industry, the incumbent pharmaceutical firms are primarily attempting to adapt to the emerging technologies by forming alliances (i.e., equity and non-equity partnerships) with new biotechnology firms (Rothaermel, 2000).\" (Methods / Sample and Data, Page 9)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>The unit of analysis is the firm-therapeutic level, i.e., the firm's alliance activities in a therapeutic area (for example, Merck's alliances in cardiovascular therapeutic area). The arguments are tested using panel data estimation techniques... The study identified 1932 alliances formed between incumbent pharmaceutical and new biotechnology firms in eighteen therapeutic areas by seventeen large pharmaceutical firms during the time period from 1991 to 2004. The focal firms are traditional pharmaceutical firms listed under Standard Industrial Classification (SIC) codes 2834 and 5122, 'Pharmaceutical Preparations' and 'Wholesale-Drugs, Proprietaries &amp; Druggists Sundries' respectively. In this industry, the incumbent pharmaceutical firms are primarily attempting to adapt to the emerging technologies by forming alliances (i.e., equity and non-equity partnerships) with new biotechnology firms (Rothaermel, 2000).\" (Methods / Sample and Data, Page 9)</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="P11" s="0" t="inlineStr">
         <is>
-          <t>\"However, these hypotheses are unobservable and are not a priori shared in the public domain. Therefore, as previously mentioned, separate empirical experiments are necessary. In this section, we discuss how the modified explanatory hypotheses can be validated through experimentation. As an example of experimental method, it would be appropriate to employ a structured questionnaire and participant observation in case study, and to select an analytical method that can show a strong explanatory model with a small number of samples while converting qualitative information into quantitative information, such as Qualitative Comparative Analysis (QCA), for the data collected.\" (4. Conclusion, limitations, and future directions, Page 7)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>However, these hypotheses are unobservable and are not a priori shared in the public domain. Therefore, as previously mentioned, separate empirical experiments are necessary. In this section, we discuss how the modified explanatory hypotheses can be validated through experimentation. As an example of experimental method, it would be appropriate to employ a structured questionnaire and participant observation in case study, and to select an analytical method that can show a strong explanatory model with a small number of samples while converting qualitative information into quantitative information, such as Qualitative Comparative Analysis (QCA), for the data collected.\" (4. Conclusion, limitations, and future directions, Page 7)</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="P12" s="0" t="inlineStr">
         <is>
-          <t>\"Since our study focused on the NPD team as a unit of analysis, product/project managers were likely to assess our variables more accurately. Also, the sample of respondents was similar to samples used in prior studies on innovation. Each product/project manager in the PMI mailing list received an invitation to participate in our study (including a cover letter, the questionnaire, and stamped return envelope). Informants were asked to focus on their most recent product development projects (ones in the marketplace for a minimum of 12 months to ensure accurate assessment of the product performance). We received 207 usable responses (an effective response rate of 16.5%) representing a wide range of industries in the manufacturing sector, including: pharmaceuticals (28.5%), automotive (17%), electrical/electronics (17.9%), computers (13%), chemicals (8.7%), machinery/metal manufacturing (7.2%), and others (7.2%).\" (Measures and sampling, Page 223)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>Since our study focused on the NPD team as a unit of analysis, product/project managers were likely to assess our variables more accurately. Also, the sample of respondents was similar to samples used in prior studies on innovation. Each product/project manager in the PMI mailing list received an invitation to participate in our study (including a cover letter, the questionnaire, and stamped return envelope). Informants were asked to focus on their most recent product development projects (ones in the marketplace for a minimum of 12 months to ensure accurate assessment of the product performance). We received 207 usable responses (an effective response rate of 16.5%) representing a wide range of industries in the manufacturing sector, including: pharmaceuticals (28.5%), automotive (17%), electrical/electronics (17.9%), computers (13%), chemicals (8.7%), machinery/metal manufacturing (7.2%), and others (7.2%).\" (Measures and sampling, Page 223)</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="P13" s="0" t="inlineStr">
         <is>
-          <t>\"Among the 180 firms contacted, we received 92 usable returns concerning NPD projects. During the sampling, to assess the product performance more accurately, we set the condition that the products used in this study must have been commercialized and launched into the marketplace for at least six months (Lynn et al., 2000). Also, the team size was an important constraint such that it should contain more than three members. Furthermore, to reduce the possible problems associated with single sourcing, we targeted the product or project manager to complete the survey. These managers were chosen because (1) product/project managers are likely to have a ‘bigger-picture view’ of NPD projects than other team members; (2) project managers have a broader view of each member’s behaviors than other team members\" (4.1. Sampling, Page 7)\n&lt;/SYSTEM_MESSAGE&gt;"}</t>
+          <t>Among the 180 firms contacted, we received 92 usable returns concerning NPD projects. During the sampling, to assess the product performance more accurately, we set the condition that the products used in this study must have been commercialized and launched into the marketplace for at least six months (Lynn et al., 2000). Also, the team size was an important constraint such that it should contain more than three members. Furthermore, to reduce the possible problems associated with single sourcing, we targeted the product or project manager to complete the survey. These managers were chosen because (1) product/project managers are likely to have a ‘bigger-picture view’ of NPD projects than other team members; (2) project managers have a broader view of each member’s behaviors than other team members\" (4.1. Sampling, Page 7)</t>
         </is>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="P56" s="0" t="inlineStr">
         <is>
-          <t>Does not measure BSB construct. Verbatim Evidence: "We applied the SPSS Process macro, Model 21 (Hayes, 2018), to test the conditional mediational hypotheses shown in Figure 1, where the independent variable (identification with the branch at time 1, X) is shown to influence the mediator (performance control related to CS at time 1, M), whose effect in turn is contingent on locus of control (W), and the effect of M on the dependent variable (CS at time 2, Y) is shown to depend on proactive behaviors in the form of CS-related meetings (V)."</t>
+          <t>Does not measure BSB construct. Verbatim Evidence: "We applied the SPSS Process macro, Model 21 (Hayes, 2018), to test the conditional mediational hypotheses shown in Figure 1, where the independent variable (identification with the branch at time 1, X) is shown to influence the mediator (performance control related to CS at time 1, M), whose effect in turn is contingent on locus of control (W), and the effect of M on the dependent variable (CS at time 2, Y) is shown to depend on proactive behaviors in the form of CS-related meetings (V).</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
       </c>
       <c r="P102" s="0" t="inlineStr">
         <is>
-          <t>Multilevel study where BSB is at the manager/group level (Level 2). Verbatim Evidence: "In this study, the data have a nested structure with individual subordinates nested within managers. Constructs regarding the manager exist at the group level of analysis whereas constructs about subordinate employees exist at the individual level of analysis."</t>
+          <t>Multilevel study where BSB is at the manager/group level (Level 2). Verbatim Evidence: "In this study, the data have a nested structure with individual subordinates nested within managers. Constructs regarding the manager exist at the group level of analysis whereas constructs about subordinate employees exist at the individual level of analysis.</t>
         </is>
       </c>
     </row>
@@ -9516,7 +9516,7 @@
       </c>
       <c r="P176" s="0" t="inlineStr">
         <is>
-          <t>Qualitative case study. Verbatim Evidence: "A longitudinal field study was conducted using an interpretive, ethnographic approach to data collection and analysis (Schwandt, 1998)."</t>
+          <t>Qualitative case study. Verbatim Evidence: "A longitudinal field study was conducted using an interpretive, ethnographic approach to data collection and analysis (Schwandt, 1998).</t>
         </is>
       </c>
     </row>
@@ -11444,7 +11444,7 @@
       </c>
       <c r="P215" s="0" t="inlineStr">
         <is>
-          <t>Firm level analysis. Verbatim Evidence: "By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005."</t>
+          <t>Firm level analysis. Verbatim Evidence: "By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005.</t>
         </is>
       </c>
     </row>
@@ -11744,7 +11744,7 @@
       </c>
       <c r="P221" s="0" t="inlineStr">
         <is>
-          <t>Department/Firm level analysis. Verbatim Evidence: "The sample in the present study includes responses from 126 professionals in R&amp;D and/or M&amp;S departments from 79 different firms (in 37 cases, we received a response from only one department)."</t>
+          <t>Department/Firm level analysis. Verbatim Evidence: "The sample in the present study includes responses from 126 professionals in R&amp;D and/or M&amp;S departments from 79 different firms (in 37 cases, we received a response from only one department).</t>
         </is>
       </c>
     </row>
@@ -12494,7 +12494,7 @@
       </c>
       <c r="P236" s="0" t="inlineStr">
         <is>
-          <t>Project level analysis. Verbatim Evidence: "(one member for each recently completed project). For those companies which had two or more recently completed projects, the information of each contact was recorded. A total of 750 projects were identified."</t>
+          <t>Project level analysis. Verbatim Evidence: "(one member for each recently completed project). For those companies which had two or more recently completed projects, the information of each contact was recorded. A total of 750 projects were identified.</t>
         </is>
       </c>
     </row>
@@ -13085,7 +13085,7 @@
       </c>
       <c r="P248" s="0" t="inlineStr">
         <is>
-          <t>Volunteers in community initiatives. Verbatim Evidence: "Considering the role of the respondents (see also control variables), most respondents were active volunteers (60.95%), followed by board members (25.63%), and passive or supporting volunteers (11.92%) (and other (1.49%))."</t>
+          <t>Volunteers in community initiatives. Verbatim Evidence: "Considering the role of the respondents (see also control variables), most respondents were active volunteers (60.95%), followed by board members (25.63%), and passive or supporting volunteers (11.92%) (and other (1.49%)).</t>
         </is>
       </c>
     </row>
@@ -17369,7 +17369,7 @@
       </c>
       <c r="P334" s="0" t="inlineStr">
         <is>
-          <t>Firm evaluating suppliers. Verbatim Evidence: "The model is tested by surveying buyers in a broad cross-section of business relationships. Organization informants evaluate a particular supplier ("target supplier"), concerning a particular product ("target product") for which their firm regularly uses alternative suppliers."</t>
+          <t>Firm evaluating suppliers. Verbatim Evidence: "The model is tested by surveying buyers in a broad cross-section of business relationships. Organization informants evaluate a particular supplier ("target supplier"), concerning a particular product ("target product") for which their firm regularly uses alternative suppliers.</t>
         </is>
       </c>
     </row>
@@ -20521,7 +20521,7 @@
       </c>
       <c r="P398" s="0" t="inlineStr">
         <is>
-          <t>rwg aggregation. Verbatim Evidence: "A check of the subordinate data tested whether aggregating the assessments by groups of subordinates for each senior manager was appropriate, according to the index of within-group interrater reliability (rwg)... Thus the averaged subordinate responses for each senior manager formed a single-group composite value"</t>
+          <t>rwg aggregation. Verbatim Evidence: "A check of the subordinate data tested whether aggregating the assessments by groups of subordinates for each senior manager was appropriate, according to the index of within-group interrater reliability (rwg)... Thus the averaged subordinate responses for each senior manager formed a single-group composite value</t>
         </is>
       </c>
     </row>
@@ -21679,7 +21679,7 @@
       </c>
       <c r="P421" s="0" t="inlineStr">
         <is>
-          <t>Unit level boundary spanning. Verbatim Evidence: "Employees in your unit frequently meet with individuals from other companies or organizations" and "Because the supervisors are most likely to have an accurate understanding of the organizational structures, the following measures are based on responses from supervisors."</t>
+          <t>Unit level boundary spanning. Verbatim Evidence: "Employees in your unit frequently meet with individuals from other companies or organizations" and "Because the supervisors are most likely to have an accurate understanding of the organizational structures, the following measures are based on responses from supervisors.</t>
         </is>
       </c>
     </row>
@@ -21779,7 +21779,7 @@
       </c>
       <c r="P423" s="0" t="inlineStr">
         <is>
-          <t>No BSB measure. Verbatim Evidence: "Table 1. Means, Standard Deviations, and Correlation Coefficients... 1. Workplace bullying, 2. Turnover intention, 3. Negative emotions, 4. Workplace unfairness"</t>
+          <t>No BSB measure. Verbatim Evidence: "Table 1. Means, Standard Deviations, and Correlation Coefficients... 1. Workplace bullying, 2. Turnover intention, 3. Negative emotions, 4. Workplace unfairness</t>
         </is>
       </c>
     </row>
@@ -21979,7 +21979,7 @@
       </c>
       <c r="P427" s="0" t="inlineStr">
         <is>
-          <t>Project level aggregation. Verbatim Evidence: "Since the unit of analysis in Hypothesis 4 is the project, individual responses must be pooled to get project scores."</t>
+          <t>Project level aggregation. Verbatim Evidence: "Since the unit of analysis in Hypothesis 4 is the project, individual responses must be pooled to get project scores.</t>
         </is>
       </c>
     </row>
@@ -22229,7 +22229,7 @@
       </c>
       <c r="P432" s="0" t="inlineStr">
         <is>
-          <t>General consumers. Verbatim Evidence: "There were only two requirements for participation: prospective samples must have been at least 18 years of age as well as having dined in a full-service restaurant in the previous 1 year."</t>
+          <t>General consumers. Verbatim Evidence: "There were only two requirements for participation: prospective samples must have been at least 18 years of age as well as having dined in a full-service restaurant in the previous 1 year.</t>
         </is>
       </c>
     </row>
@@ -22329,7 +22329,7 @@
       </c>
       <c r="P434" s="0" t="inlineStr">
         <is>
-          <t>Project level. Verbatim Evidence: "To investigate this issue, we examine 6081 research projects in the Life Sciences, Physical &amp; Engineering, and Social Sciences &amp; Humanities sectors funded by the European Research Council"</t>
+          <t>Project level. Verbatim Evidence: "To investigate this issue, we examine 6081 research projects in the Life Sciences, Physical &amp; Engineering, and Social Sciences &amp; Humanities sectors funded by the European Research Council</t>
         </is>
       </c>
     </row>
@@ -22998,7 +22998,7 @@
       </c>
       <c r="P447" s="0" t="inlineStr">
         <is>
-          <t>Firm level. Verbatim Evidence: "Design/methodology/approach – The authors utilized regression analytical technique and categorical moderation analytical technique to test their hypotheses on survey data of 579 firms."</t>
+          <t>Firm level. Verbatim Evidence: "Design/methodology/approach – The authors utilized regression analytical technique and categorical moderation analytical technique to test their hypotheses on survey data of 579 firms.</t>
         </is>
       </c>
     </row>
@@ -23714,7 +23714,7 @@
       </c>
       <c r="P461" s="0" t="inlineStr">
         <is>
-          <t>Qualitative interviews. Verbatim Evidence: "Over the course of the study, I conducted 14 semi-structured meetings on Zoom."</t>
+          <t>Qualitative interviews. Verbatim Evidence: "Over the course of the study, I conducted 14 semi-structured meetings on Zoom.</t>
         </is>
       </c>
     </row>
@@ -24698,7 +24698,7 @@
       </c>
       <c r="P481" s="0" t="inlineStr">
         <is>
-          <t>Group level aggregation. Verbatim Evidence: "Aggregation of data at the group level requires both a theoretical basis and empirical justification (Kozlowski &amp; Klein, 2000). [...] Therefore, both intergroup conflict scales were aggregated by groups."</t>
+          <t>Group level aggregation. Verbatim Evidence: "Aggregation of data at the group level requires both a theoretical basis and empirical justification (Kozlowski &amp; Klein, 2000). [...] Therefore, both intergroup conflict scales were aggregated by groups.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: inject accurate 2nd screening audit verbatim quotes for BSMA0157-0343
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -8126,7 +8126,7 @@
     <row r="149" ht="18" customHeight="1" s="31">
       <c r="A149" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B149" s="0" t="inlineStr">
@@ -8134,15 +8134,11 @@
           <t>BSMA0146</t>
         </is>
       </c>
-      <c r="E149" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F149" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E149" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G149" s="0" t="inlineStr">
         <is>
@@ -8169,14 +8165,14 @@
       </c>
       <c r="P149" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Our final sample consisted of those 57 teams from which we had received three or more subordinate surveys and a supervisor survey, and for which archival data were available. These teams ranged in size from 4 to 26 members (x = 11.7, s.d. = 6.1); 84 percent of team members were male; the average age was 42.7 years (s.d. = 7.7), and the average time with the current team was 1.5 years (s.d. = .5). [...] Together, the above analyses supported the aggregation of informant responses from a team to create team-level variables for collective team identification, team learning, intrateam conflict, and external communication.\" (Sample and Data Collection / Interrater agreement and reliability, Pages 537-539)\n\nNote: The specific file \"Guenzel (2020) - Open innovation...\" did not exist in the workspace, so the paper with ID 201 mapped in all_remaining_targets.txt (\"[201] Van der vegt &amp; Bunderson (2005) - LEARNING AND PERFORMANCE IN MULTIDISCIPLINARY TEAMS.pdf\") was reviewed instead as standard procedure.</t>
         </is>
       </c>
     </row>
     <row r="150" ht="18" customHeight="1" s="31">
       <c r="A150" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B150" s="0" t="inlineStr">
@@ -8184,15 +8180,11 @@
           <t>BSMA0147</t>
         </is>
       </c>
-      <c r="E150" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F150" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E150" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G150" s="0" t="inlineStr">
         <is>
@@ -8219,14 +8211,14 @@
       </c>
       <c r="P150" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Agents in creative enterprises are embedded in networks that inspire, support, and evaluate their work. Here, we investigate how the mechanisms by which creative teams self-assemble determine the structure of these collaboration networks. We propose a model for team self-assembly that is based on three parameters: team size, the fraction of newcomers in new productions, and the tendency of incumbents to repeat previous collaborations. The model suggests that the emergence of a large connected community of practitioners can be described as a phase transition. We find that the model team assembly mechanisms determine both the topological structure of the collaboration network and team performance in fields as diverse as Broadway musicals and scientific research.\" (Abstract, Page 1)</t>
         </is>
       </c>
     </row>
     <row r="151" ht="18" customHeight="1" s="31">
       <c r="A151" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B151" s="0" t="inlineStr">
@@ -8234,15 +8226,11 @@
           <t>BSMA0148</t>
         </is>
       </c>
-      <c r="E151" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F151" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E151" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G151" s="0" t="inlineStr">
         <is>
@@ -8269,7 +8257,7 @@
       </c>
       <c r="P151" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"After excluding teams for which fewer than 50 percent of the respondents were core members (Hackman, 2002: 47), 96 teams qualified for the study (80 percent; 50 financial and 46 technical teams, with 485 member respondents). Tests for selection bias showed no significant differences in the effectiveness ratings, project types, regions, or divisions of the 24 teams that did not qualify. Dependent variables. The dependent variables in this study were (1) the strategic effectiveness of a team and (2) the operational effectiveness of a team, as rated by its independent expert panel.\" (Quantitative Data, Page 995)</t>
         </is>
       </c>
     </row>
@@ -8326,7 +8314,7 @@
     <row r="153" ht="18" customHeight="1" s="31">
       <c r="A153" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B153" s="0" t="inlineStr">
@@ -8334,15 +8322,11 @@
           <t>BSMA0150</t>
         </is>
       </c>
-      <c r="E153" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F153" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E153" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G153" s="0" t="inlineStr">
         <is>
@@ -8369,14 +8353,14 @@
       </c>
       <c r="P153" s="0" t="inlineStr">
         <is>
-          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study provides a quantitative correlation matrix based on an employee sample, but it does not measure Boundary Spanning Behavior (BSB) or include it in the effect sizes. The measured variables are limited to transformational leadership, internal/external support for innovation, firm age, and organizational innovation. Verbatim Evidence: \"Employees’ questionnaires included measures of transformational leadership and internal support for innovation. On average, four employees rated each leader. Employees were also asked for their age, gender, educational level, job tenure, and company tenure. Leaders’ questionnaires included questions about company age, company innovations, and the degree of support they received from external institutions.\" (Procedure, Page 7)</t>
         </is>
       </c>
     </row>
     <row r="154" ht="18" customHeight="1" s="31">
       <c r="A154" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B154" s="0" t="inlineStr">
@@ -8384,10 +8368,8 @@
           <t>BSMA0151</t>
         </is>
       </c>
-      <c r="E154" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
+      <c r="E154" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="F154" s="0" t="inlineStr">
         <is>
@@ -8419,7 +8401,7 @@
       </c>
       <c r="P154" s="0" t="inlineStr">
         <is>
-          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+          <t>1 = Include\n\nThe paper samples individual organizational employees (132 full-time employees at a scientific facility) and provides an individual-level Pearson correlation matrix (Table 1) that includes quantitative measures of Discretionary Boundary Spanning (DBS) ties (task-oriented and friendship) and their relationship with informal leadership and job performance. Therefore, it meets all inclusion criteria for the meta-analysis.</t>
         </is>
       </c>
     </row>
@@ -8476,7 +8458,7 @@
     <row r="156" ht="18" customHeight="1" s="31">
       <c r="A156" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B156" s="0" t="inlineStr">
@@ -8484,10 +8466,8 @@
           <t>BSMA0153</t>
         </is>
       </c>
-      <c r="E156" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
+      <c r="E156" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="F156" s="0" t="inlineStr">
         <is>
@@ -8519,14 +8499,14 @@
       </c>
       <c r="P156" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>1 = Include\n\nNote: The actual file for ID 208 was found as `[208] Zhang et al. (2024) - The Double-Edged Sword Effect of Performance Pressure on Employee Boundary-Spanning.pdf`. The study samples individual organizational employees (N=336) and provides a quantitative individual-level Pearson correlation matrix (Table 2) containing the variable Employee Boundary-Spanning Behavior (EBSB). It fully meets the inclusion criteria.</t>
         </is>
       </c>
     </row>
     <row r="157" ht="18" customHeight="1" s="31">
       <c r="A157" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B157" s="0" t="inlineStr">
@@ -8534,15 +8514,11 @@
           <t>BSMA0154</t>
         </is>
       </c>
-      <c r="E157" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F157" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E157" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" s="0" t="n">
+        <v>99</v>
       </c>
       <c r="G157" s="0" t="inlineStr">
         <is>
@@ -8569,14 +8545,14 @@
       </c>
       <c r="P157" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 99\nFile not found on disk. Verbatim Evidence: \"failed to read file: open g:/My Drive/UCL/BSMA/BSMA ANTIGRAVITY/01_Academic_Papers/[209] Hanisch et al. (2014) - Innovation network formation a conceptual model.pdf: The system cannot find the file specified. A global search for Hanisch across the BSMA ANTIGRAVITY workspace yielded zero results. Therefore, this paper cannot be audited and is excluded due to a missing file.\" (System Error Log, Page 1)</t>
         </is>
       </c>
     </row>
     <row r="158" ht="18" customHeight="1" s="31">
       <c r="A158" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B158" s="0" t="inlineStr">
@@ -8584,15 +8560,11 @@
           <t>BSMA0155</t>
         </is>
       </c>
-      <c r="E158" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F158" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E158" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G158" s="0" t="inlineStr">
         <is>
@@ -8619,14 +8591,14 @@
       </c>
       <c r="P158" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"We first obtained a list of 272 public pharmaceutical companies based on the standard industry classification code (SIC 2834). By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005. To test our model, we collect secondary data about firms’ IT-enabled knowledge capabilities and innovation outcomes from multiple secondary data sources.\" (Data Collection, Page 9)</t>
         </is>
       </c>
     </row>
     <row r="159" ht="18" customHeight="1" s="31">
       <c r="A159" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B159" s="0" t="inlineStr">
@@ -8634,10 +8606,8 @@
           <t>BSMA0156</t>
         </is>
       </c>
-      <c r="E159" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
+      <c r="E159" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="F159" s="0" t="inlineStr">
         <is>
@@ -8669,14 +8639,14 @@
       </c>
       <c r="P159" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>1 = Include\nReason Code: 0\nThe study samples individual organizational employees and provides an individual-level Pearson correlation matrix that includes a measure of boundary-spanning leadership. Verbatim Evidence: \"The sample comprises four public-sector and four private-sector banks (NSE/BSE indexed) with 12 branches of each bank. The number of respondents from public-sector and private-sector banks was 327 and 308, respectively. Data were collected through a questionnaire comprising 40 items reflecting all the constructs (Generational diversity, knowledge sharing, group performance, intergenerational climate, boundary-spanning leadership, and respect). The study followed a cross-sectional approach for collecting data. The clerical and managerial employees in the bank branches were contacted through offline survey methods.\" (Sample, Page 7)</t>
         </is>
       </c>
     </row>
     <row r="160" ht="18" customHeight="1" s="31">
       <c r="A160" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B160" s="0" t="inlineStr">
@@ -8684,15 +8654,11 @@
           <t>BSMA0157</t>
         </is>
       </c>
-      <c r="E160" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F160" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E160" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G160" s="0" t="inlineStr">
         <is>
@@ -8719,7 +8685,7 @@
       </c>
       <c r="P160" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative study without quantitative effect sizes. Verbatim Evidence: \"A thematic analysis of the discourse collected through in-depth interviews, survey questionnaires, and organizational documents was conducted using the constant comparative method (Lindlof, 1995). This process begins with data “reduction” and “interpretation” (Creswell, 1997; Lindlof, 1995) and is consistent with processes engaged in by other communication scholars doing interpretive work (e.g., Braithwaite, Baxter, &amp; Harper, 1998; Clair &amp; Thompson, 1996; Trethewey, 1997). First, all transcripts and documents were read in their entirety to develop a sense of these data as a whole.\" (Data Analysis, Page 8)</t>
         </is>
       </c>
     </row>
@@ -8826,7 +8792,7 @@
     <row r="163" ht="18" customHeight="1" s="31">
       <c r="A163" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B163" s="0" t="inlineStr">
@@ -8834,15 +8800,11 @@
           <t>BSMA0160</t>
         </is>
       </c>
-      <c r="E163" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F163" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="E163" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F163" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G163" s="0" t="inlineStr">
         <is>
@@ -8869,14 +8831,14 @@
       </c>
       <c r="P163" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative case study without quantitative correlation data. Verbatim Evidence: \"Following other researchers who are interested in organizational processes (e.g., Anand, Gardner, &amp; Morris, 2007; Bresman, 2013; Nag &amp; Gioia, 2012), we combined a case study approach with grounded theory methodology (Langley, 1999). Specifically, we first used grounded methods to develop cases describing the sequence of early boundary spanning activity in each of 10 COTs; we then used a case study approach to compare and contrast those sequences across the 10 teams. Case studies drew on interviews with 46 team members.\" (Method, page 512)</t>
         </is>
       </c>
     </row>
     <row r="164" ht="18" customHeight="1" s="31">
       <c r="A164" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B164" s="0" t="inlineStr">
@@ -8884,15 +8846,11 @@
           <t>BSMA0161</t>
         </is>
       </c>
-      <c r="E164" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F164" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E164" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F164" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G164" s="0" t="inlineStr">
         <is>
@@ -8919,14 +8877,14 @@
       </c>
       <c r="P164" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level variables. The study measures external team learning and team performance rather than individual-level employee boundary spanning behavior. Verbatim Evidence: \"For data collection, we adapted the Team Learning Survey (TSL) and Team Performance Survey (TPS) scales used by Edmondson (1996) while investigating team learning in a large office furniture manufacturer in the American Mid-West. The Team Learning Survey (TLS) incorporated both the internal and the external team learning behaviors each measured through five items. The team performance construct in the Team Performance Survey (TPS) was also measured through five items. The respondents were asked to record their responses on a seven-point likert scale where 1 meant strongly disagree and 7 meant strongly agree.\" (Methods, Page 126)</t>
         </is>
       </c>
     </row>
     <row r="165" ht="18" customHeight="1" s="31">
       <c r="A165" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B165" s="0" t="inlineStr">
@@ -8934,15 +8892,11 @@
           <t>BSMA0162</t>
         </is>
       </c>
-      <c r="E165" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F165" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E165" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F165" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G165" s="0" t="inlineStr">
         <is>
@@ -8969,7 +8923,7 @@
       </c>
       <c r="P165" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study conducts a social network analysis calculating network centrality measures rather than using psychometric scales, and it does not report a bivariate Pearson correlation matrix. Verbatim Evidence: \"Survey responses were exported from Qualtrics® into a spreadsheet where the data were cleaned following a two-step process. First, participants’ identification numbers were checked against a master list to ensure that only the data from invited respondents were included. In situations where a participant’s data were recorded twice, only the first record was retained. Second, only participants who completed the sociodemographic survey questions and listed at least one person using their full name as a source of advice or information about PBS were included. Social network data in the form of adjacency lists were created and imported into the social network software Visone (Algorithmics Group, 2019) where graphs were constructed and analyses conducted, including calculation of indegree and betweenness centralities.\" (Data extraction and analysis, Page 5)</t>
         </is>
       </c>
     </row>
@@ -9026,7 +8980,7 @@
     <row r="167" ht="18" customHeight="1" s="31">
       <c r="A167" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B167" s="0" t="inlineStr">
@@ -9034,15 +8988,11 @@
           <t>BSMA0164</t>
         </is>
       </c>
-      <c r="E167" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F167" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E167" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F167" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G167" s="0" t="inlineStr">
         <is>
@@ -9069,7 +9019,7 @@
       </c>
       <c r="P167" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam and firm level of analysis. Verbatim Evidence: \"Using CorpTech (now part of InfoUSA), we built a sampling frame of 467 small- to medium-sized enterprises (SMEs) operating in technology-based sectors in the northeastern United States. [...] All told, for 99 firms, we received responses from the CEO and at least another member of the top management team. [...] Apart from the dependent variable, which relies on the assessment of the CEO, our measures involved the aggregated responses of top managers. We separated the measurement of our independent and dependent variables using separate respondents to minimize the influence of common method effects. [...] An acceptable level of interrater agreement (median rwg(j) = 0.94) and reliability (ICC1 = 0.31, ICC2 = 0.69) justified the aggregation of top managers’ responses to the team level of analysis (Chan 1998).\" (Method, Pages 946-947)</t>
         </is>
       </c>
     </row>
@@ -9172,7 +9122,7 @@
     <row r="170" ht="18" customHeight="1" s="31">
       <c r="A170" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B170" s="0" t="inlineStr">
@@ -9180,15 +9130,11 @@
           <t>BSMA0167</t>
         </is>
       </c>
-      <c r="E170" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F170" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E170" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G170" s="0" t="inlineStr">
         <is>
@@ -9215,14 +9161,14 @@
       </c>
       <c r="P170" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"The average succession rate for any given company was found by aggregating (averaging) the reciprocals of completed office tenures during the 30-year interval for all presidential successors who held the title Chief Executive Officer. Office tenure for successors was determined by examining selected editions of Moody’s Industrial Manual [28]. The specification of the 30-year interval was also statistically necessary because of the need to control the time variable across companies when developing ex post facto measures of succession rate and variability in measures of board size.\" (Operational Definitions, Page 5)</t>
         </is>
       </c>
     </row>
     <row r="171" ht="18" customHeight="1" s="31">
       <c r="A171" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B171" s="0" t="inlineStr">
@@ -9230,15 +9176,11 @@
           <t>BSMA0168</t>
         </is>
       </c>
-      <c r="E171" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F171" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E171" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G171" s="0" t="inlineStr">
         <is>
@@ -9265,14 +9207,14 @@
       </c>
       <c r="P171" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Four organizations participated, providing 56 R&amp;D teams. Two of the companies were R&amp;D divisions of large publicly-listed mining and chemical manufacturing organizations, whilst the other two were government R&amp;D organizations. The analyses report a one-year longitudinal study, with repeated mail outs every four months. Analyses were conducted on team level data collected over four time periods. Teams (both leaders and team members) rated leadership role performance and team communication.\" (Method, page 5)</t>
         </is>
       </c>
     </row>
     <row r="172" ht="18" customHeight="1" s="31">
       <c r="A172" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B172" s="0" t="inlineStr">
@@ -9280,15 +9222,11 @@
           <t>BSMA0169</t>
         </is>
       </c>
-      <c r="E172" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F172" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E172" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G172" s="0" t="inlineStr">
         <is>
@@ -9316,7 +9254,7 @@
       </c>
       <c r="P172" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative interview study without quantitative effect sizes. Verbatim Evidence: \"Data was collected from participants via telephone interviews which typically lasted about 45 minutes, with all conversations being digitally recorded with participants’ consent. The interviews were qualitative conversations, being focussed around a standard list of open-ended questions that were asked to all interviewees. The key topics discussed in the interviews included the nature of people’s work, their feelings about their work, the positive and negative features of their work, the extent to which work was a source of stress or fatigue, how work-related stress/fatigue was dealt with, as well as the role of ICTs and mobile ICTs in their work and the management of the work-life boundary.\" (4.2 Data Collection Procedure, Page 12-13)</t>
         </is>
       </c>
     </row>
@@ -9373,7 +9311,7 @@
     <row r="174" ht="18" customHeight="1" s="31">
       <c r="A174" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B174" s="0" t="inlineStr">
@@ -9381,15 +9319,11 @@
           <t>BSMA0171</t>
         </is>
       </c>
-      <c r="E174" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F174" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E174" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F174" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G174" s="0" t="inlineStr">
         <is>
@@ -9416,14 +9350,14 @@
       </c>
       <c r="P174" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam-level analysis. Verbatim Evidence: \"For measuring team interface management, we mainly relied on Mohrman et al.’s (1995) discussion of team management tasks in team-based organizations and on Ancona and Caldwell’s (1992) description of boundary management. Team members were asked to evaluate the extent to which the activities described in the seven items were performed in the team. Prior to aggregating team members’ evaluations of team interface management, interrater agreement (Campion et al., 1993; James, 1982; James et al., 1984) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). With an average score across all teams of 0.87, this test yielded results indicating generally very strong agreement of ratings referring to the same team. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, page 10)</t>
         </is>
       </c>
     </row>
     <row r="175" ht="18" customHeight="1" s="31">
       <c r="A175" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B175" s="0" t="inlineStr">
@@ -9431,15 +9365,11 @@
           <t>BSMA0172</t>
         </is>
       </c>
-      <c r="E175" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F175" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E175" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G175" s="0" t="inlineStr">
         <is>
@@ -9466,7 +9396,7 @@
       </c>
       <c r="P175" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level of analysis. Verbatim Evidence: \"Prior to aggregating team members’ evaluations of interteam coordination, project commitment, and teamwork quality, interrater agreement (James 1982, James et al. 1984, Campion et al. 1993) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). This test yielded results indicating generally very strong agreement of ratings referring to the same team. The average score of this test across all teams is 0.90 for interteam coordination, 0.91 for project commitment, and 0.93 for teamwork quality. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, Page 45)</t>
         </is>
       </c>
     </row>
@@ -9523,7 +9453,7 @@
     <row r="177" ht="18" customHeight="1" s="31">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B177" s="0" t="inlineStr">
@@ -9531,15 +9461,11 @@
           <t>BSMA0174</t>
         </is>
       </c>
-      <c r="E177" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F177" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E177" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G177" s="0" t="inlineStr">
         <is>
@@ -9566,14 +9492,14 @@
       </c>
       <c r="P177" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative reflective inquiry paper without quantitative correlation data. Verbatim Evidence: \"We iteratively collected and analyzed data for this manuscript using the three sequential phases (Kim, 1999): descriptive, reflective, and critical summarized in Table 1. First, we used the descriptive phase to elicit narratives of actual experiences including descriptions of actions, thoughts, and feelings (Kim, 1999). This phase began while preparing for a discussion panel on navigating disciplinary boundaries presented in the Health Communication Division at the National Communication Association (NCA) 2018 Annual Convention in Salt Lake City, Utah. Each author wrote narratives of their experiences navigating a boundary spanning academic position.\" (Procedures, Page 3)</t>
         </is>
       </c>
     </row>
     <row r="178" ht="18" customHeight="1" s="31">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B178" s="0" t="inlineStr">
@@ -9581,15 +9507,11 @@
           <t>BSMA0175</t>
         </is>
       </c>
-      <c r="E178" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F178" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E178" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G178" s="0" t="inlineStr">
         <is>
@@ -9616,14 +9538,14 @@
       </c>
       <c r="P178" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"The unit of analysis for the study is the audit team. A team score for each variable was computed by summing the individual item responses provided by the three team members. For the variables under study, the proportion of total variance that is shared among teammates (Spearman-Brown formula; DeVellis 1991) is .26 for information overload, .42 for boundary spanning, .42 for satisfaction with supervision, .22 for accuracy of information, and .15 for audit team structure.\" (RESULTS, Page 8)</t>
         </is>
       </c>
     </row>
     <row r="179" ht="18" customHeight="1" s="31">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B179" s="0" t="inlineStr">
@@ -9631,15 +9553,11 @@
           <t>BSMA0176</t>
         </is>
       </c>
-      <c r="E179" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F179" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E179" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F179" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G179" s="0" t="inlineStr">
         <is>
@@ -9666,14 +9584,14 @@
       </c>
       <c r="P179" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"We used a survey methodology to gather the data for the research. This study used a sample framework of 300 firms selected randomly from the list of 650 new technology ventures located in Shenzhen, provided by a local consulting and market research company. We contacted the senior manager of each firm by phone to solicit their participation in this study, and to ask if they would be willing to provide access to two or three key informants, including CEOs, managing directors, or senior managers who were involved in engineering or business development.\" (Sample and data collection, Page 6)</t>
         </is>
       </c>
     </row>
     <row r="180" ht="18" customHeight="1" s="31">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B180" s="0" t="inlineStr">
@@ -9681,15 +9599,11 @@
           <t>BSMA0177</t>
         </is>
       </c>
-      <c r="E180" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F180" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E180" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F180" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G180" s="0" t="inlineStr">
         <is>
@@ -9716,14 +9630,14 @@
       </c>
       <c r="P180" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"We sent out 750 questionnaires to part-time MBA and EMBA students at 4 universities in China who come from enterprises in different provinces and municipalities such as Heilongjiang, Jilin and Beijing. Respondents were asked to be middle and senior managers and technical executives who understand corporate strategy and technology innovation. The questionnaires were collected in two phases. In the first stage, the data is distributed before class and recovered after class; in the second stage, some selected respondents, who were corporate executives, were invited to further distribute questionnaires to their subordinates or colleagues to reduce common method bias. Eventually, we obtained valid questionnaires from 290 different companies and the effective recovery rate was 38.67%.\" (Method, page 8)</t>
         </is>
       </c>
     </row>
     <row r="181" ht="18" customHeight="1" s="31">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B181" s="0" t="inlineStr">
@@ -9731,15 +9645,11 @@
           <t>BSMA0178</t>
         </is>
       </c>
-      <c r="E181" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F181" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E181" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F181" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G181" s="0" t="inlineStr">
         <is>
@@ -9766,14 +9676,14 @@
       </c>
       <c r="P181" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study lacks a Pearson correlation matrix reporting effect sizes for employee boundary spanning behavior. Instead, it utilizes qualitative script elicitation methodology and chi-square analysis to compare the frequency of service expectations between consumers and providers. Verbatim Evidence: \"Thus, two sets of scripts were obtained, one set from consumers and the other set from service providers. The unit of analysis was the script, which was composed of the subgoals of the respondent’s typical haircut. The two sets of scripts were coded separately. Each subgoal mentioned was recorded, yielding a master list of subgoals for each set of respondents. The number of respondents who mentioned each subgoal was then tallied. Descriptive statistics are provided in Table I. Chi-square analysis found no significant gender differences in the frequency of mention of any of the subgoals.\" (Analysis and results, Page 7)</t>
         </is>
       </c>
     </row>
     <row r="182" ht="18" customHeight="1" s="31">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B182" s="0" t="inlineStr">
@@ -9781,15 +9691,11 @@
           <t>BSMA0179</t>
         </is>
       </c>
-      <c r="E182" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F182" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E182" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F182" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G182" s="0" t="inlineStr">
         <is>
@@ -9816,14 +9722,14 @@
       </c>
       <c r="P182" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study uses structural equation modeling (SEM) to evaluate the interrelations among variables but fails to provide a bivariate Pearson correlation matrix for the extracted measures. Only descriptive statistics, factor loadings, and structural path estimates are reported. Verbatim Evidence: \"The descriptive statistics is shown in Table I, namely, mean, standard deviation and the factor analysis and Cronbach’s alpha results... Structural equation modelling (SEM) was used for the data analysis that included all the hypothesised paths, which is consistent with other studies conducted on multiteam system performance (Cuijpers et al., 2016; Cha et al., 2015). SEM was appropriate for investigating the interrelations among the set of variables, as it offers advantages over multiple regression, accounting, as it does for measurement error (Strasheim, 2014). SEM is a second generation multivariate method used to assess the reliability and validity of the model measures holistically, whereas first generation multivariate methods, such as multiple regression, are appropriate for evaluating constructs and relationships between constructs (Tabachnick and Fidell, 2001, p. 111). A measurement model was developed in AMOS 24.0 for the four constructs to be tested.\" (3. Methods, Page 11-12)</t>
         </is>
       </c>
     </row>
     <row r="183" ht="18" customHeight="1" s="31">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B183" s="0" t="inlineStr">
@@ -9831,15 +9737,11 @@
           <t>BSMA0180</t>
         </is>
       </c>
-      <c r="E183" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F183" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E183" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G183" s="0" t="inlineStr">
         <is>
@@ -9866,14 +9768,14 @@
       </c>
       <c r="P183" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: \"We gathered our data in The Netherlands using a cross sectional survey methodology. We used the project level of analysis because the information used to make NPD decisions is project-specific, rather than being more generally applicable to the entire firm or a division. Each project requires specific details about customer needs and technical capabilities to allow developers to make tradeoffs between the different specifications and feature levels.\" (Sample and Data Collection, Page 4)</t>
         </is>
       </c>
     </row>
     <row r="184" ht="18" customHeight="1" s="31">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B184" s="0" t="inlineStr">
@@ -9881,15 +9783,11 @@
           <t>BSMA0181</t>
         </is>
       </c>
-      <c r="E184" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F184" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E184" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F184" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G184" s="0" t="inlineStr">
         <is>
@@ -9916,14 +9814,14 @@
       </c>
       <c r="P184" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"In cooperation with the leaders of the rehabilitation centres, all health professionals (N = 167) engaged in working with patients in the centres were invited to participate in the survey. These centres deliver services via interprofessional teams; we identified 16 teams, which were the unit of interest in the present study, according to RC theory [9]. Some healthcare professionals were members of more than one team in the centre in which they worked; these professionals were asked to respond to the survey for each team they worked with.\" (Methods, Page 2) \"The main explanatory variables in this study were the RC communication and relationships scores, which were calculated for each team and used as continuous variables, from 1(lowest) to 5 (highest).\" (Methods, Page 4)</t>
         </is>
       </c>
     </row>
     <row r="185" ht="18" customHeight="1" s="31">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B185" s="0" t="inlineStr">
@@ -9931,15 +9829,11 @@
           <t>BSMA0182</t>
         </is>
       </c>
-      <c r="E185" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F185" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E185" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" s="0" t="n">
+        <v>2</v>
       </c>
       <c r="G185" s="0" t="inlineStr">
         <is>
@@ -9966,14 +9860,14 @@
       </c>
       <c r="P185" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 2\nPatient sample. Verbatim Evidence: \"All patients aged 18 and above who were accepted for rehabilitation in a rehabilitation centre in Western Norway between January 2015 and June 2015 were invited to participate (n=2863). For baseline data collection, a total of 984 (34%) patients accepted the invitation to participate and provided written consent and a completed questionnaire. A 1-year follow-up questionnaire was sent to all participating patients (n=984), and 705 patients (25% of the patient group invited at baseline) returned the questionnaire. We extracted 279 of the baseline participants from the analyses, as they did not respond to the 1-year follow-up survey. Four respondents were omitted from the analyses due to missing data on outcome variables. Finally, 701 (24% of the patient group invited at baseline) patients were included in the analyses (Table 1).\" (Participants, Page 2-3)</t>
         </is>
       </c>
     </row>
     <row r="186" ht="18" customHeight="1" s="31">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B186" s="0" t="inlineStr">
@@ -9981,15 +9875,11 @@
           <t>BSMA0183</t>
         </is>
       </c>
-      <c r="E186" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F186" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E186" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G186" s="0" t="inlineStr">
         <is>
@@ -10016,7 +9906,7 @@
       </c>
       <c r="P186" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study only reports descriptive percentages for team-level feedback and does not provide an individual-level Pearson correlation matrix or quantitative effect sizes. Verbatim Evidence: \"The questionnaire was designed to be used as a self-diagnostic instrument, and therefore the format of the feedback returned to the teams was specified according to the preferences of the teams. Teams preferred feedback in percentages above means; the sum of the percentages of team members that “agreed” and “agreed strongly” was reported. Also standard deviations were reported, and we volunteered to discuss scales and items with low percentages or high standard deviations in team meetings. In four teams the questionnaires were filled out individually during team meetings, however, the members of fifth team preferred to do this outer their meeting. There were 52 workers in the five teams, and 46 (88 per cent) completed the questionnaire.\" (The questionnaire, Page 59)</t>
         </is>
       </c>
     </row>
@@ -10073,7 +9963,7 @@
     <row r="188" ht="18" customHeight="1" s="31">
       <c r="A188" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B188" s="0" t="inlineStr">
@@ -10081,15 +9971,11 @@
           <t>BSMA0185</t>
         </is>
       </c>
-      <c r="E188" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F188" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E188" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F188" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G188" s="0" t="inlineStr">
         <is>
@@ -10116,7 +10002,7 @@
       </c>
       <c r="P188" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Transformational leadership, gatekeeping leadership, internal communication, external communication, and norm for maintaining consensus were aggregated to mean values within each team, which was the unit of the analysis. To justify this aggregation, a within-group correlation (rwg) was computed to assess the amount of agreement by the team members (James et al. 1984). The mean rwg value was 0.87 for transformational leadership, 0.89 for gatekeeping leadership, 0.90 for internal communication, 0.89 for external communication, and 0.89 for norm for maintaining consensus. In addition, the ICC(1) values were as follows: transformational leadership, 0.22; gatekeeping leadership, 0.50; internal communication, 0.24; external communication, 0.36; and norm for maintaining consensus, 0.25. ICC(2) values were as follows: transformational leadership, 0.61; gatekeeping leadership, 0.85; internal communication, 0.64; external communication, 0.76; and norm for maintaining consensus, 0.65. The overall pattern of results across the rwg, ICC(1), and ICC(2) analyses provided sufficient support for aggregating the data to team level of analysis.\" (Aggregation tests, Page 11)</t>
         </is>
       </c>
     </row>
@@ -10219,7 +10105,7 @@
     <row r="191" ht="18" customHeight="1" s="31">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B191" s="0" t="inlineStr">
@@ -10227,15 +10113,11 @@
           <t>BSMA0188</t>
         </is>
       </c>
-      <c r="E191" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F191" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E191" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F191" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G191" s="0" t="inlineStr">
         <is>
@@ -10262,14 +10144,14 @@
       </c>
       <c r="P191" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nThe study uses work groups as the unit of analysis and aggregates individual survey responses to the team level. Verbatim Evidence: \"Following Van de Ven and colleagues (1976) and Tushman (1977, 1978), we used work groups as the units of analysis. First-line supervisors with at least one year as unit heads who had full-time subordinates with sufficient experience to be familiar with their positions answered questions on the subordinates' jobs. The study included all units meeting the criterion for supervisory experience and containing at least two experienced subordinates. [...] To compute scores for work groups, supervisors' scores were added to the means of subordinates' scores, and these sums were divided by two (Van de Ven et al., 1976). Three tests supported this procedure. One-way analysis of variance (Dixon &amp; Massey, 1969) supported pooling subordinate responses into work groups for all of the variables (p &lt; .005).\" (Methods, pages 143-144)</t>
         </is>
       </c>
     </row>
     <row r="192" ht="18" customHeight="1" s="31">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B192" s="0" t="inlineStr">
@@ -10277,15 +10159,11 @@
           <t>BSMA0189</t>
         </is>
       </c>
-      <c r="E192" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F192" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E192" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G192" s="0" t="inlineStr">
         <is>
@@ -10312,14 +10190,14 @@
       </c>
       <c r="P192" s="0" t="inlineStr">
         <is>
-          <t>Study involving workplace employees, but does not report quantitative correlation/regression effect sizes for boundary spanning.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo individual-level bivariate Pearson correlation matrix is provided. The study only reports an aggregated organizational-level correlation matrix and jumps straight to regression for the individual-level analysis. Verbatim Evidence: \"Regression analysis. First, a simple regression model was conducted to test if NCB significantly predicted IIB. The results of the regression indicated that NCB explained 17.8% of the variance in IIB (R2 = 17.8, F (1, 85) = 18.436, p&lt;.05). Next, a multiple regression analysis was conducted to test if NCB significantly predicted IIB after five demographic variables are controlled. The results of the multiple regression indicated that together with the four demographic variables, NCB predicted 30.5% of the variance in IIB (R2 = .305, F (6, 75) = 5.485, p&lt;.001).\" (Chapter 4: Data Analysis, Page 108)</t>
         </is>
       </c>
     </row>
     <row r="193" ht="18" customHeight="1" s="31">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B193" s="0" t="inlineStr">
@@ -10327,15 +10205,11 @@
           <t>BSMA0190</t>
         </is>
       </c>
-      <c r="E193" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F193" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E193" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G193" s="0" t="inlineStr">
         <is>
@@ -10362,14 +10236,14 @@
       </c>
       <c r="P193" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study samples boundary spanners but lacks an effect size for boundary spanning behavior, measuring only burnout, role stressors, and general job performance. Verbatim Evidence: \"Job outcomes. Psychological outcomes were measured by three separate first-order constmcts. JS was operationalized as a 26-item scale adapted from Churchill, Ford, and Walker's (1985) study that has been frequently used in marketing. The alpha reliability of this scale was estimated as .92. OC was operationalized by use of a 6-item version of a scale from Mowday, Steers, and Porter (1979). Tbe scaie achieved acceptable reliability (a = .79). Finally, Tl was assessed by a three-item measure based on Donnelly and Ivancevicb (1975). In addition, this measure has been shown in several studies to be a consistent predictor of actual tumover. The Cronbach's a for this measure was .85. Behavioral out comes were measured by a self-rating, 6-item measure of JP drawn from Dubinsky and Mattson (1979).\" (Measures, page 563)</t>
         </is>
       </c>
     </row>
     <row r="194" ht="18" customHeight="1" s="31">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B194" s="0" t="inlineStr">
@@ -10377,15 +10251,11 @@
           <t>BSMA0191</t>
         </is>
       </c>
-      <c r="E194" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F194" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E194" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F194" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G194" s="0" t="inlineStr">
         <is>
@@ -10412,7 +10282,7 @@
       </c>
       <c r="P194" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: \"In fact, because degree-based centrality measures are basically a standardized count of ties, a high actor degree centrality in an inter-organizational network equates to a higher level of BSA from the team's point of view. Consequently, the measure of BSA in this dissertation is the focal team's degree centrality in an inter-team network where the nodes are all OSS projects registered in Source Forge. This measure can be used since each project in Source Forge includes a list of developers. Once all these lists have been scanned, it is easy to detect developers who work on more than one project and then build the inter-team network in order to calculate a given project's BSA.\" (4.4.3.4 Boundary Spanning Activity, Page 99)</t>
         </is>
       </c>
     </row>
@@ -10569,7 +10439,7 @@
     <row r="198" ht="18" customHeight="1" s="31">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B198" s="0" t="inlineStr">
@@ -10577,15 +10447,11 @@
           <t>BSMA0195</t>
         </is>
       </c>
-      <c r="E198" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F198" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E198" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F198" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G198" s="0" t="inlineStr">
         <is>
@@ -10612,14 +10478,14 @@
       </c>
       <c r="P198" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided; the study only reports mean differences and t-tests. Verbatim Evidence: \"Measures used to test the hypotheses each consisted of two 7-point itemized rating scales designed to assess the extent to which team selling was used in a particular buying or selling situation. For example, to measure the extent to which team selling is used when the buyer’s informational needs are great, respondents indicated the likelihood of using sales teams when 'the anticipated information needs of the customer are small' and 'the anticipated information needs of the customer are great' (1 = extremely unlikely, 7 = extremely likely). T-tests were conducted on the mean differences between the respondents’ ratings for each of the paired questions. A hypothesis was supported when the mean difference was significantly different from 0.\" (Hypotheses Tests, page 160)</t>
         </is>
       </c>
     </row>
     <row r="199" ht="18" customHeight="1" s="31">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B199" s="0" t="inlineStr">
@@ -10627,15 +10493,11 @@
           <t>BSMA0196</t>
         </is>
       </c>
-      <c r="E199" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F199" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="E199" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F199" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G199" s="0" t="inlineStr">
         <is>
@@ -10662,14 +10524,14 @@
       </c>
       <c r="P199" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative case study lacking quantitative correlation data. Verbatim Evidence: \"We use a case study research methodology to identify various contextual elements that shape the development of a common platform in a post-merger scenario. We examine how stakeholders from different business divisions establish a common understanding of their processes to inform the development of a common platform underlying a family of similar business processes. [...] We participated as observers in all the eight workshops and in six other meetings. Workshop meetings were audio-recorded with the participants’ consent, yielding an extremely rich set of data of over more than 50 h. Additional informal interviews with process participants were conducted to seek clarifications on issues raised during the workshops. See Online Appendix B for an excerpt of the interview questionnaire. These interviews allowed us to explore the expectations of the participants. Detailed notes were also taken during each of the data collection sessions. Workshops and interviews were our primary source of qualitative data.\" (Research methodology &amp; Data collection, Page 5-6)</t>
         </is>
       </c>
     </row>
     <row r="200" ht="18" customHeight="1" s="31">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B200" s="0" t="inlineStr">
@@ -10677,15 +10539,11 @@
           <t>BSMA0197</t>
         </is>
       </c>
-      <c r="E200" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F200" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E200" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G200" s="0" t="inlineStr">
         <is>
@@ -10712,14 +10570,14 @@
       </c>
       <c r="P200" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"For our empirical analysis, we use data sets provided by the Netherlands Enterprise Agency (RVO.nl) on all collaborative R&amp;D projects that received support from the allowance scheme in the period 2013–2018. The data sets include information about project titles, starting years, participants and budgets. By merging the data, it is possible to map the evolution of the collaborative network for the period 2013–2018. The total network includes 1884 Dutch firms and 105 publicly-funded organizations. Given our focus on recombining firm capabilities, our analyses concentrate on the 1884 firms only.\" (Case description: collaborative R&amp;D in the Netherlands, Page 4)</t>
         </is>
       </c>
     </row>
     <row r="201" ht="18" customHeight="1" s="31">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B201" s="0" t="inlineStr">
@@ -10727,15 +10585,11 @@
           <t>BSMA0198</t>
         </is>
       </c>
-      <c r="E201" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F201" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E201" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F201" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G201" s="0" t="inlineStr">
         <is>
@@ -10762,14 +10616,14 @@
       </c>
       <c r="P201" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided. Verbatim Evidence: \"Grouping and Analytic Techniques. Each subject was grouped according to primary decision style which resulted in four groups of individuals being labeled as either SF (n = 20), ST (n = 7), NF (n = 24), or NT (n = 6). Because BSA was defined as multidimensional in nature and was composed of three separate dimensions, the primary analytic technique used was multivariate analysis of variance (MANOVA). This test was run to determine if decision style affected total BSA. Given a significant overall F for the MANOVA test, several post hoc techniques were employed to investigate the specific nature of these differences. First, a multivariate extension of the Scheffe test was used to determine which decision style groups were different from each other across the combination of the three BSA variables.\" (Grouping and Analytic Techniques, Page 6)</t>
         </is>
       </c>
     </row>
     <row r="202" ht="18" customHeight="1" s="31">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B202" s="0" t="inlineStr">
@@ -10777,15 +10631,11 @@
           <t>BSMA0199</t>
         </is>
       </c>
-      <c r="E202" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F202" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="E202" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F202" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G202" s="0" t="inlineStr">
         <is>
@@ -10812,14 +10662,14 @@
       </c>
       <c r="P202" s="0" t="inlineStr">
         <is>
-          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+          <t>0 = Exclude\nReason Code: 3\nProject and team level of analysis without individual employee boundary spanning correlations. Verbatim Evidence: \"From the multiteam system (MTS) perspective, this study employs the input-process-outcome (IPO) framework and coordination theory to explore the influence of instant messaging-based team boundary spanning (IMTBS) on construction project coordination processes and project performance. A theoretical model is built and validated with a survey involving 206 construction projects. [...] Data were collected from construction projects in China. We first conducted a pilot study involving 30 respondents from the Master of Engineering Management (MEM) students majoring in construction management at a Chinese renowned university to test the validity of all constructs. [...] Then, the questionnaire was distributed to construction professionals to report the condition of the last completed project they managed. We randomly sent the link to the online survey to alumni of two renowned universities, who were involved in the construction industry. A total of 400 questionnaires were distributed to these alumni from 53 construction companies, and 256 responses were returned. After removing invalid responses, 206 valid questionnaires were left, thereby yielding a valid response rate of 51.5%.\" (Abstract, Page 1; 4.2 Data collection, Page 7)</t>
         </is>
       </c>
     </row>
     <row r="203" ht="18" customHeight="1" s="31">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>Antigravity (Rescue 2)</t>
         </is>
       </c>
       <c r="B203" s="0" t="inlineStr">
@@ -10827,15 +10677,11 @@
           <t>BSMA0200</t>
         </is>
       </c>
-      <c r="E203" s="0" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F203" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="E203" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F203" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G203" s="0" t="inlineStr">
         <is>
@@ -10862,7 +10708,7 @@
       </c>
       <c r="P203" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"The referent-shift consensus model proposed by Chan[50]was used in designing the questionnaire, which means that variables including \"team boundary-spanning activities,\" \"team job crafting,\" and \"team innovation performance\" was designed from the perspective of the team. A request was made for these questions to be answered from the perspective of team awareness. The \"individual job crafting\" variable was designed from the employees' perspective. Second, the terminology, the clarity of the instructions, and the structure of the questionnaire's responses were evaluated by three subject-matter experts and five teams from Shandong province's universities engaged in scientific research and innovation. Modifications were made accordingly. Finally, teams that were developing collaborative innovation projects were selected. The distribution of 456 surveys resulted in the recovery of 400 questionnaires. Three hundred thirty-one valid surveys were retrieved after invalid data had been removed; these originated from 41 collaborative innovation teams.\" (3.1 Sample and data collection procedure, Page 6)</t>
         </is>
       </c>
     </row>
@@ -10882,10 +10728,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F204" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F204" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G204" s="0" t="inlineStr">
         <is>
@@ -10912,7 +10756,7 @@
       </c>
       <c r="P204" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Our final sample consisted of those 57 teams from which we had received three or more subordinate surveys and a supervisor survey, and for which archival data were available. These teams ranged in size from 4 to 26 members (x = 11.7, s.d. = 6.1); 84 percent of team members were male; the average age was 42.7 years (s.d. = 7.7), and the average time with the current team was 1.5 years (s.d. = .5). [...] Together, the above analyses supported the aggregation of informant responses from a team to create team-level variables for collective team identification, team learning, intrateam conflict, and external communication.\" (Sample and Data Collection / Interrater agreement and reliability, Pages 537-539)\n\nNote: The specific file \"Guenzel (2020) - Open innovation...\" did not exist in the workspace, so the paper with ID 201 mapped in all_remaining_targets.txt (\"[201] Van der vegt &amp; Bunderson (2005) - LEARNING AND PERFORMANCE IN MULTIDISCIPLINARY TEAMS.pdf\") was reviewed instead as standard procedure.\n"}</t>
         </is>
       </c>
     </row>
@@ -11028,10 +10872,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F207" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F207" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G207" s="0" t="inlineStr">
         <is>
@@ -11058,7 +10900,7 @@
       </c>
       <c r="P207" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Agents in creative enterprises are embedded in networks that inspire, support, and evaluate their work. Here, we investigate how the mechanisms by which creative teams self-assemble determine the structure of these collaboration networks. We propose a model for team self-assembly that is based on three parameters: team size, the fraction of newcomers in new productions, and the tendency of incumbents to repeat previous collaborations. The model suggests that the emergence of a large connected community of practitioners can be described as a phase transition. We find that the model team assembly mechanisms determine both the topological structure of the collaboration network and team performance in fields as diverse as Broadway musicals and scientific research.\" (Abstract, Page 1)\n"}</t>
         </is>
       </c>
     </row>
@@ -11078,10 +10920,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F208" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F208" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G208" s="0" t="inlineStr">
         <is>
@@ -11108,7 +10948,7 @@
       </c>
       <c r="P208" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"After excluding teams for which fewer than 50 percent of the respondents were core members (Hackman, 2002: 47), 96 teams qualified for the study (80 percent; 50 financial and 46 technical teams, with 485 member respondents). Tests for selection bias showed no significant differences in the effectiveness ratings, project types, regions, or divisions of the 24 teams that did not qualify. Dependent variables. The dependent variables in this study were (1) the strategic effectiveness of a team and (2) the operational effectiveness of a team, as rated by its independent expert panel.\" (Quantitative Data, Page 995)\n"}</t>
         </is>
       </c>
     </row>
@@ -11318,10 +11158,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F213" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F213" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G213" s="0" t="inlineStr">
         <is>
@@ -11348,7 +11186,7 @@
       </c>
       <c r="P213" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study provides a quantitative correlation matrix based on an employee sample, but it does not measure Boundary Spanning Behavior (BSB) or include it in the effect sizes. The measured variables are limited to transformational leadership, internal/external support for innovation, firm age, and organizational innovation. Verbatim Evidence: "\"Employees’ questionnaires included measures of transformational leadership and internal support for innovation. On average, four employees rated each leader. Employees were also asked for their age, gender, educational level, job tenure, and company tenure. Leaders’ questionnaires included questions about company age, company innovations, and the degree of support they received from external institutions.\" (Procedure, Page 7)\n"}</t>
         </is>
       </c>
     </row>
@@ -11461,14 +11299,10 @@
       </c>
       <c r="E216" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F216" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F216" s="0" t="inlineStr"/>
       <c r="G216" s="0" t="inlineStr">
         <is>
           <t>Purpose – The current article investigates the impact of generational diversity on knowledge sharing and group performance. It, further, explores the moderating effects of intergenerational climate, boundaryspanning leadership, and respect in facilitating greater knowledge sharing and enhanced group performance. Design/methodology/approach – The authors applied partial least square structural equation modeling to test the model, using a sample of 635 employees working in the banking industry.</t>
@@ -11494,7 +11328,7 @@
       </c>
       <c r="P216" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Verbatim Evidence: "</t>
         </is>
       </c>
     </row>
@@ -11511,14 +11345,10 @@
       </c>
       <c r="E217" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F217" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F217" s="0" t="inlineStr"/>
       <c r="G217" s="0" t="inlineStr">
         <is>
           <t>This paper combines the concept of weak ties from social network research and the notion of complex knowledge to explain the role of weak ties in sharing knowledge across organization subunits in a multiunit organization. I use a network study of 120 new-product development projects undertaken by 41 divisions in a large electronics company to examine the task of developing new products in the least amount of time. Findings show that weak interunit ties help a project team search for useful knowledge in other subunits but impede the transfer of complex knowledge, which tends to require a strong tie between the two parties to a transfer. Having weak interunit ties speeds up projects when knowledge is not complex but slows them down when the knowledge to be transferred is highly complex. I discuss the implications of these findings for research on social networks and product innovation.</t>
@@ -11544,7 +11374,7 @@
       </c>
       <c r="P217" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Verbatim Evidence: "</t>
         </is>
       </c>
     </row>
@@ -11564,10 +11394,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F218" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F218" s="0" t="n">
+        <v>99</v>
       </c>
       <c r="G218" s="0" t="inlineStr">
         <is>
@@ -11594,7 +11422,7 @@
       </c>
       <c r="P218" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 99\nFile not found on disk. Verbatim Evidence: "\"failed to read file: open g:/My Drive/UCL/BSMA/BSMA ANTIGRAVITY/01_Academic_Papers/[209] Hanisch et al. (2014) - Innovation network formation a conceptual model.pdf: The system cannot find the file specified. A global search for Hanisch across the BSMA ANTIGRAVITY workspace yielded zero results. Therefore, this paper cannot be audited and is excluded due to a missing file.\" (System Error Log, Page 1)\n"}</t>
         </is>
       </c>
     </row>
@@ -11614,10 +11442,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F219" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F219" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G219" s="0" t="inlineStr">
         <is>
@@ -11644,7 +11470,7 @@
       </c>
       <c r="P219" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We first obtained a list of 272 public pharmaceutical companies based on the standard industry classification code (SIC 2834). By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005. To test our model, we collect secondary data about firms’ IT-enabled knowledge capabilities and innovation outcomes from multiple secondary data sources.\" (Data Collection, Page 9)\n"}</t>
         </is>
       </c>
     </row>
@@ -11661,14 +11487,10 @@
       </c>
       <c r="E220" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F220" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F220" s="0" t="inlineStr"/>
       <c r="G220" s="0" t="inlineStr">
         <is>
           <t>The paper explains the effects of internal and external team learning behaviors on the performance of marketing teams. The survey was conducted in the context of a multinational Pharmaceutical Corporation marketing its products in Turkey. Data were collected from members of marketing team which included medical sales representatives, specialized medical sales representatives and districts heads of marketing. The results indicate that both the internal team learning and the external team learning behaviors play significant roles in ensuring the success of marketing teams in continuously identifying, anticipating and satisfying the customer requirements profitably through an efficient deployment of the marketing teams’ resources.</t>
@@ -11694,7 +11516,7 @@
       </c>
       <c r="P220" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Verbatim Evidence: "\"The sample comprises four public-sector and four private-sector banks (NSE/BSE indexed) with 12 branches of each bank. The number of respondents from public-sector and private-sector banks was 327 and 308, respectively. Data were collected through a questionnaire comprising 40 items reflecting all the constructs (Generational diversity, knowledge sharing, group performance, intergenerational climate, boundary-spanning leadership, and respect). The study followed a cross-sectional approach for collecting data. The clerical and managerial employees in the bank branches were contacted through offline survey methods.\" (Sample, Page 7)\n"}</t>
         </is>
       </c>
     </row>
@@ -11764,10 +11586,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F222" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F222" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G222" s="0" t="inlineStr">
         <is>
@@ -11794,7 +11614,7 @@
       </c>
       <c r="P222" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative study without quantitative effect sizes. Verbatim Evidence: "\"A thematic analysis of the discourse collected through in-depth interviews, survey questionnaires, and organizational documents was conducted using the constant comparative method (Lindlof, 1995). This process begins with data “reduction” and “interpretation” (Creswell, 1997; Lindlof, 1995) and is consistent with processes engaged in by other communication scholars doing interpretive work (e.g., Braithwaite, Baxter, &amp; Harper, 1998; Clair &amp; Thompson, 1996; Trethewey, 1997). First, all transcripts and documents were read in their entirety to develop a sense of these data as a whole.\" (Data Analysis, Page 8)\n"}</t>
         </is>
       </c>
     </row>
@@ -11814,10 +11634,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F223" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F223" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G223" s="0" t="inlineStr">
         <is>
@@ -11844,7 +11662,7 @@
       </c>
       <c r="P223" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative case study without quantitative correlation data. Verbatim Evidence: "\"Following other researchers who are interested in organizational processes (e.g., Anand, Gardner, &amp; Morris, 2007; Bresman, 2013; Nag &amp; Gioia, 2012), we combined a case study approach with grounded theory methodology (Langley, 1999). Specifically, we first used grounded methods to develop cases describing the sequence of early boundary spanning activity in each of 10 COTs; we then used a case study approach to compare and contrast those sequences across the 10 teams. Case studies drew on interviews with 46 team members.\" (Method, page 512)\n"}</t>
         </is>
       </c>
     </row>
@@ -11864,10 +11682,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F224" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F224" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G224" s="0" t="inlineStr">
         <is>
@@ -11894,7 +11710,7 @@
       </c>
       <c r="P224" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level variables. The study measures external team learning and team performance rather than individual-level employee boundary spanning behavior. Verbatim Evidence: "\"For data collection, we adapted the Team Learning Survey (TSL) and Team Performance Survey (TPS) scales used by Edmondson (1996) while investigating team learning in a large office furniture manufacturer in the American Mid-West. The Team Learning Survey (TLS) incorporated both the internal and the external team learning behaviors each measured through five items. The team performance construct in the Team Performance Survey (TPS) was also measured through five items. The respondents were asked to record their responses on a seven-point likert scale where 1 meant strongly disagree and 7 meant strongly agree.\" (Methods, Page 126)\n"}</t>
         </is>
       </c>
     </row>
@@ -11964,10 +11780,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F226" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F226" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G226" s="0" t="inlineStr">
         <is>
@@ -11994,7 +11808,7 @@
       </c>
       <c r="P226" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study conducts a social network analysis calculating network centrality measures rather than using psychometric scales, and it does not report a bivariate Pearson correlation matrix. Verbatim Evidence: "\"Survey responses were exported from Qualtrics® into a spreadsheet where the data were cleaned following a two-step process. First, participants’ identification numbers were checked against a master list to ensure that only the data from invited respondents were included. In situations where a participant’s data were recorded twice, only the first record was retained. Second, only participants who completed the sociodemographic survey questions and listed at least one person using their full name as a source of advice or information about PBS were included. Social network data in the form of adjacency lists were created and imported into the social network software Visone (Algorithmics Group, 2019) where graphs were constructed and analyses conducted, including calculation of indegree and betweenness centralities.\" (Data extraction and analysis, Page 5)\n"}</t>
         </is>
       </c>
     </row>
@@ -12014,10 +11828,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F227" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F227" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G227" s="0" t="inlineStr">
         <is>
@@ -12044,7 +11856,7 @@
       </c>
       <c r="P227" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam and firm level of analysis. Verbatim Evidence: "\"Using CorpTech (now part of InfoUSA), we built a sampling frame of 467 small- to medium-sized enterprises (SMEs) operating in technology-based sectors in the northeastern United States. [...] All told, for 99 firms, we received responses from the CEO and at least another member of the top management team. [...] Apart from the dependent variable, which relies on the assessment of the CEO, our measures involved the aggregated responses of top managers. We separated the measurement of our independent and dependent variables using separate respondents to minimize the influence of common method effects. [...] An acceptable level of interrater agreement (median rwg(j) = 0.94) and reliability (ICC1 = 0.31, ICC2 = 0.69) justified the aggregation of top managers’ responses to the team level of analysis (Chan 1998).\" (Method, Pages 946-947)\n"}</t>
         </is>
       </c>
     </row>
@@ -12114,10 +11926,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F229" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F229" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G229" s="0" t="inlineStr">
         <is>
@@ -12144,7 +11954,7 @@
       </c>
       <c r="P229" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"The average succession rate for any given company was found by aggregating (averaging) the reciprocals of completed office tenures during the 30-year interval for all presidential successors who held the title Chief Executive Officer. Office tenure for successors was determined by examining selected editions of Moody’s Industrial Manual [28]. The specification of the 30-year interval was also statistically necessary because of the need to control the time variable across companies when developing ex post facto measures of succession rate and variability in measures of board size.\" (Operational Definitions, Page 5)\n"}</t>
         </is>
       </c>
     </row>
@@ -12164,10 +11974,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F230" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F230" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G230" s="0" t="inlineStr">
         <is>
@@ -12194,7 +12002,7 @@
       </c>
       <c r="P230" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Four organizations participated, providing 56 R&amp;D teams. Two of the companies were R&amp;D divisions of large publicly-listed mining and chemical manufacturing organizations, whilst the other two were government R&amp;D organizations. The analyses report a one-year longitudinal study, with repeated mail outs every four months. Analyses were conducted on team level data collected over four time periods. Teams (both leaders and team members) rated leadership role performance and team communication.\" (Method, page 5)\n"}</t>
         </is>
       </c>
     </row>
@@ -12264,10 +12072,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F232" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F232" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G232" s="0" t="inlineStr">
         <is>
@@ -12294,7 +12100,7 @@
       </c>
       <c r="P232" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative interview study without quantitative effect sizes. Verbatim Evidence: "\"Data was collected from participants via telephone interviews which typically lasted about 45 minutes, with all conversations being digitally recorded with participants’ consent. The interviews were qualitative conversations, being focussed around a standard list of open-ended questions that were asked to all interviewees. The key topics discussed in the interviews included the nature of people’s work, their feelings about their work, the positive and negative features of their work, the extent to which work was a source of stress or fatigue, how work-related stress/fatigue was dealt with, as well as the role of ICTs and mobile ICTs in their work and the management of the work-life boundary.\" (4.2 Data Collection Procedure, Page 12-13)\n"}</t>
         </is>
       </c>
     </row>
@@ -12314,10 +12120,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F233" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F233" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G233" s="0" t="inlineStr">
         <is>
@@ -12344,7 +12148,7 @@
       </c>
       <c r="P233" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam-level analysis. Verbatim Evidence: "\"For measuring team interface management, we mainly relied on Mohrman et al.’s (1995) discussion of team management tasks in team-based organizations and on Ancona and Caldwell’s (1992) description of boundary management. Team members were asked to evaluate the extent to which the activities described in the seven items were performed in the team. Prior to aggregating team members’ evaluations of team interface management, interrater agreement (Campion et al., 1993; James, 1982; James et al., 1984) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). With an average score across all teams of 0.87, this test yielded results indicating generally very strong agreement of ratings referring to the same team. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, page 10)\n"}</t>
         </is>
       </c>
     </row>
@@ -12414,10 +12218,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F235" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F235" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G235" s="0" t="inlineStr">
         <is>
@@ -12444,7 +12246,7 @@
       </c>
       <c r="P235" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level of analysis. Verbatim Evidence: "\"Prior to aggregating team members’ evaluations of interteam coordination, project commitment, and teamwork quality, interrater agreement (James 1982, James et al. 1984, Campion et al. 1993) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). This test yielded results indicating generally very strong agreement of ratings referring to the same team. The average score of this test across all teams is 0.90 for interteam coordination, 0.91 for project commitment, and 0.93 for teamwork quality. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, Page 45)\n"}</t>
         </is>
       </c>
     </row>
@@ -12560,10 +12362,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F238" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F238" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G238" s="0" t="inlineStr">
         <is>
@@ -12590,7 +12390,7 @@
       </c>
       <c r="P238" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative reflective inquiry paper without quantitative correlation data. Verbatim Evidence: "\"We iteratively collected and analyzed data for this manuscript using the three sequential phases (Kim, 1999): descriptive, reflective, and critical summarized in Table 1. First, we used the descriptive phase to elicit narratives of actual experiences including descriptions of actions, thoughts, and feelings (Kim, 1999). This phase began while preparing for a discussion panel on navigating disciplinary boundaries presented in the Health Communication Division at the National Communication Association (NCA) 2018 Annual Convention in Salt Lake City, Utah. Each author wrote narratives of their experiences navigating a boundary spanning academic position.\" (Procedures, Page 3)\n"}</t>
         </is>
       </c>
     </row>
@@ -12660,10 +12460,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F240" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F240" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G240" s="0" t="inlineStr">
         <is>
@@ -12690,7 +12488,7 @@
       </c>
       <c r="P240" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"The unit of analysis for the study is the audit team. A team score for each variable was computed by summing the individual item responses provided by the three team members. For the variables under study, the proportion of total variance that is shared among teammates (Spearman-Brown formula; DeVellis 1991) is .26 for information overload, .42 for boundary spanning, .42 for satisfaction with supervision, .22 for accuracy of information, and .15 for audit team structure.\" (RESULTS, Page 8)\n"}</t>
         </is>
       </c>
     </row>
@@ -12710,10 +12508,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F241" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F241" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G241" s="0" t="inlineStr">
         <is>
@@ -12740,7 +12536,7 @@
       </c>
       <c r="P241" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We used a survey methodology to gather the data for the research. This study used a sample framework of 300 firms selected randomly from the list of 650 new technology ventures located in Shenzhen, provided by a local consulting and market research company. We contacted the senior manager of each firm by phone to solicit their participation in this study, and to ask if they would be willing to provide access to two or three key informants, including CEOs, managing directors, or senior managers who were involved in engineering or business development.\" (Sample and data collection, Page 6)\n"}</t>
         </is>
       </c>
     </row>
@@ -12805,10 +12601,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F243" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F243" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G243" s="0" t="inlineStr">
         <is>
@@ -12835,7 +12629,7 @@
       </c>
       <c r="P243" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We sent out 750 questionnaires to part-time MBA and EMBA students at 4 universities in China who come from enterprises in different provinces and municipalities such as Heilongjiang, Jilin and Beijing. Respondents were asked to be middle and senior managers and technical executives who understand corporate strategy and technology innovation. The questionnaires were collected in two phases. In the first stage, the data is distributed before class and recovered after class; in the second stage, some selected respondents, who were corporate executives, were invited to further distribute questionnaires to their subordinates or colleagues to reduce common method bias. Eventually, we obtained valid questionnaires from 290 different companies and the effective recovery rate was 38.67%.\" (Method, page 8)\n"}</t>
         </is>
       </c>
     </row>
@@ -12855,10 +12649,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F244" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F244" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G244" s="0" t="inlineStr">
         <is>
@@ -12885,7 +12677,7 @@
       </c>
       <c r="P244" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study lacks a Pearson correlation matrix reporting effect sizes for employee boundary spanning behavior. Instead, it utilizes qualitative script elicitation methodology and chi-square analysis to compare the frequency of service expectations between consumers and providers. Verbatim Evidence: "\"Thus, two sets of scripts were obtained, one set from consumers and the other set from service providers. The unit of analysis was the script, which was composed of the subgoals of the respondent’s typical haircut. The two sets of scripts were coded separately. Each subgoal mentioned was recorded, yielding a master list of subgoals for each set of respondents. The number of respondents who mentioned each subgoal was then tallied. Descriptive statistics are provided in Table I. Chi-square analysis found no significant gender differences in the frequency of mention of any of the subgoals.\" (Analysis and results, Page 7)\n"}</t>
         </is>
       </c>
     </row>
@@ -12905,10 +12697,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F245" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F245" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G245" s="0" t="inlineStr">
         <is>
@@ -12935,7 +12725,7 @@
       </c>
       <c r="P245" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study uses structural equation modeling (SEM) to evaluate the interrelations among variables but fails to provide a bivariate Pearson correlation matrix for the extracted measures. Only descriptive statistics, factor loadings, and structural path estimates are reported. Verbatim Evidence: "\"The descriptive statistics is shown in Table I, namely, mean, standard deviation and the factor analysis and Cronbach’s alpha results... Structural equation modelling (SEM) was used for the data analysis that included all the hypothesised paths, which is consistent with other studies conducted on multiteam system performance (Cuijpers et al., 2016; Cha et al., 2015). SEM was appropriate for investigating the interrelations among the set of variables, as it offers advantages over multiple regression, accounting, as it does for measurement error (Strasheim, 2014). SEM is a second generation multivariate method used to assess the reliability and validity of the model measures holistically, whereas first generation multivariate methods, such as multiple regression, are appropriate for evaluating constructs and relationships between constructs (Tabachnick and Fidell, 2001, p. 111). A measurement model was developed in AMOS 24.0 for the four constructs to be tested.\" (3. Methods, Page 11-12)\n"}</t>
         </is>
       </c>
     </row>
@@ -12955,10 +12745,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F246" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F246" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G246" s="0" t="inlineStr">
         <is>
@@ -12985,7 +12773,7 @@
       </c>
       <c r="P246" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: "\"We gathered our data in The Netherlands using a cross sectional survey methodology. We used the project level of analysis because the information used to make NPD decisions is project-specific, rather than being more generally applicable to the entire firm or a division. Each project requires specific details about customer needs and technical capabilities to allow developers to make tradeoffs between the different specifications and feature levels.\" (Sample and Data Collection, Page 4)\n"}</t>
         </is>
       </c>
     </row>
@@ -13201,10 +12989,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F251" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F251" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G251" s="0" t="inlineStr">
         <is>
@@ -13231,7 +13017,7 @@
       </c>
       <c r="P251" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"In cooperation with the leaders of the rehabilitation centres, all health professionals (N = 167) engaged in working with patients in the centres were invited to participate in the survey. These centres deliver services via interprofessional teams; we identified 16 teams, which were the unit of interest in the present study, according to RC theory [9]. Some healthcare professionals were members of more than one team in the centre in which they worked; these professionals were asked to respond to the survey for each team they worked with.\" (Methods, Page 2) \"The main explanatory variables in this study were the RC communication and relationships scores, which were calculated for each team and used as continuous variables, from 1(lowest) to 5 (highest).\" (Methods, Page 4)\n"}</t>
         </is>
       </c>
     </row>
@@ -13297,10 +13083,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F253" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F253" s="0" t="n">
+        <v>2</v>
       </c>
       <c r="G253" s="0" t="inlineStr">
         <is>
@@ -13327,7 +13111,7 @@
       </c>
       <c r="P253" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>0 = Exclude\nReason Code: 2\nPatient sample. Verbatim Evidence: "\"All patients aged 18 and above who were accepted for rehabilitation in a rehabilitation centre in Western Norway between January 2015 and June 2015 were invited to participate (n=2863). For baseline data collection, a total of 984 (34%) patients accepted the invitation to participate and provided written consent and a completed questionnaire. A 1-year follow-up questionnaire was sent to all participating patients (n=984), and 705 patients (25% of the patient group invited at baseline) returned the questionnaire. We extracted 279 of the baseline participants from the analyses, as they did not respond to the 1-year follow-up survey. Four respondents were omitted from the analyses due to missing data on outcome variables. Finally, 701 (24% of the patient group invited at baseline) patients were included in the analyses (Table 1).\" (Participants, Page 2-3)\n"}</t>
         </is>
       </c>
     </row>
@@ -13347,10 +13131,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F254" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F254" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G254" s="0" t="inlineStr">
         <is>
@@ -13377,7 +13159,7 @@
       </c>
       <c r="P254" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study only reports descriptive percentages for team-level feedback and does not provide an individual-level Pearson correlation matrix or quantitative effect sizes. Verbatim Evidence: "\"The questionnaire was designed to be used as a self-diagnostic instrument, and therefore the format of the feedback returned to the teams was specified according to the preferences of the teams. Teams preferred feedback in percentages above means; the sum of the percentages of team members that “agreed” and “agreed strongly” was reported. Also standard deviations were reported, and we volunteered to discuss scales and items with low percentages or high standard deviations in team meetings. In four teams the questionnaires were filled out individually during team meetings, however, the members of fifth team preferred to do this outer their meeting. There were 52 workers in the five teams, and 46 (88 per cent) completed the questionnaire.\" (The questionnaire, Page 59)\n"}</t>
         </is>
       </c>
     </row>
@@ -13397,10 +13179,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F255" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F255" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G255" s="0" t="inlineStr">
         <is>
@@ -13427,7 +13207,7 @@
       </c>
       <c r="P255" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Transformational leadership, gatekeeping leadership, internal communication, external communication, and norm for maintaining consensus were aggregated to mean values within each team, which was the unit of the analysis. To justify this aggregation, a within-group correlation (rwg) was computed to assess the amount of agreement by the team members (James et al. 1984). The mean rwg value was 0.87 for transformational leadership, 0.89 for gatekeeping leadership, 0.90 for internal communication, 0.89 for external communication, and 0.89 for norm for maintaining consensus. In addition, the ICC(1) values were as follows: transformational leadership, 0.22; gatekeeping leadership, 0.50; internal communication, 0.24; external communication, 0.36; and norm for maintaining consensus, 0.25. ICC(2) values were as follows: transformational leadership, 0.61; gatekeeping leadership, 0.85; internal communication, 0.64; external communication, 0.76; and norm for maintaining consensus, 0.65. The overall pattern of results across the rwg, ICC(1), and ICC(2) analyses provided sufficient support for aggregating the data to team level of analysis.\" (Aggregation tests, Page 11)\n"}</t>
         </is>
       </c>
     </row>
@@ -13447,10 +13227,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F256" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F256" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G256" s="0" t="inlineStr">
         <is>
@@ -13477,7 +13255,7 @@
       </c>
       <c r="P256" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>0 = Exclude\nReason Code: 3\nThe study uses work groups as the unit of analysis and aggregates individual survey responses to the team level. Verbatim Evidence: "\"Following Van de Ven and colleagues (1976) and Tushman (1977, 1978), we used work groups as the units of analysis. First-line supervisors with at least one year as unit heads who had full-time subordinates with sufficient experience to be familiar with their positions answered questions on the subordinates' jobs. The study included all units meeting the criterion for supervisory experience and containing at least two experienced subordinates. [...] To compute scores for work groups, supervisors' scores were added to the means of subordinates' scores, and these sums were divided by two (Van de Ven et al., 1976). Three tests supported this procedure. One-way analysis of variance (Dixon &amp; Massey, 1969) supported pooling subordinate responses into work groups for all of the variables (p &lt; .005).\" (Methods, pages 143-144)\n"}</t>
         </is>
       </c>
     </row>
@@ -13497,10 +13275,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F257" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
+      <c r="F257" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G257" s="0" t="inlineStr">
         <is>
@@ -13527,7 +13303,7 @@
       </c>
       <c r="P257" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo individual-level bivariate Pearson correlation matrix is provided. The study only reports an aggregated organizational-level correlation matrix and jumps straight to regression for the individual-level analysis. Verbatim Evidence: "\"Regression analysis. First, a simple regression model was conducted to test if NCB significantly predicted IIB. The results of the regression indicated that NCB explained 17.8% of the variance in IIB (R2 = 17.8, F (1, 85) = 18.436, p&lt;.05). Next, a multiple regression analysis was conducted to test if NCB significantly predicted IIB after five demographic variables are controlled. The results of the multiple regression indicated that together with the four demographic variables, NCB predicted 30.5% of the variance in IIB (R2 = .305, F (6, 75) = 5.485, p&lt;.001).\" (Chapter 4: Data Analysis, Page 108)\n"}</t>
         </is>
       </c>
     </row>
@@ -13547,10 +13323,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F258" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F258" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G258" s="0" t="inlineStr">
         <is>
@@ -13577,7 +13351,7 @@
       </c>
       <c r="P258" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 1\nThe study samples boundary spanners but lacks an effect size for boundary spanning behavior, measuring only burnout, role stressors, and general job performance. Verbatim Evidence: "\"Job outcomes. Psychological outcomes were measured by three separate first-order constmcts. JS was operationalized as a 26-item scale adapted from Churchill, Ford, and Walker's (1985) study that has been frequently used in marketing. The alpha reliability of this scale was estimated as .92. OC was operationalized by use of a 6-item version of a scale from Mowday, Steers, and Porter (1979). Tbe scaie achieved acceptable reliability (a = .79). Finally, Tl was assessed by a three-item measure based on Donnelly and Ivancevicb (1975). In addition, this measure has been shown in several studies to be a consistent predictor of actual tumover. The Cronbach's a for this measure was .85. Behavioral out comes were measured by a self-rating, 6-item measure of JP drawn from Dubinsky and Mattson (1979).\" (Measures, page 563)\n"}</t>
         </is>
       </c>
     </row>
@@ -13597,10 +13371,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F259" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F259" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G259" s="0" t="inlineStr">
         <is>
@@ -13627,7 +13399,7 @@
       </c>
       <c r="P259" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: "\"In fact, because degree-based centrality measures are basically a standardized count of ties, a high actor degree centrality in an inter-organizational network equates to a higher level of BSA from the team's point of view. Consequently, the measure of BSA in this dissertation is the focal team's degree centrality in an inter-team network where the nodes are all OSS projects registered in Source Forge. This measure can be used since each project in Source Forge includes a list of developers. Once all these lists have been scanned, it is easy to detect developers who work on more than one project and then build the inter-team network in order to calculate a given project's BSA.\" (4.4.3.4 Boundary Spanning Activity, Page 99)\n"}</t>
         </is>
       </c>
     </row>
@@ -13697,10 +13469,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F261" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F261" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G261" s="0" t="inlineStr">
         <is>
@@ -13727,7 +13497,7 @@
       </c>
       <c r="P261" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided; the study only reports mean differences and t-tests. Verbatim Evidence: "\"Measures used to test the hypotheses each consisted of two 7-point itemized rating scales designed to assess the extent to which team selling was used in a particular buying or selling situation. For example, to measure the extent to which team selling is used when the buyer’s informational needs are great, respondents indicated the likelihood of using sales teams when 'the anticipated information needs of the customer are small' and 'the anticipated information needs of the customer are great' (1 = extremely unlikely, 7 = extremely likely). T-tests were conducted on the mean differences between the respondents’ ratings for each of the paired questions. A hypothesis was supported when the mean difference was significantly different from 0.\" (Hypotheses Tests, page 160)\n"}</t>
         </is>
       </c>
     </row>
@@ -13843,10 +13613,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F264" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F264" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G264" s="0" t="inlineStr">
         <is>
@@ -13873,7 +13641,7 @@
       </c>
       <c r="P264" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 4\nQualitative case study lacking quantitative correlation data. Verbatim Evidence: "\"We use a case study research methodology to identify various contextual elements that shape the development of a common platform in a post-merger scenario. We examine how stakeholders from different business divisions establish a common understanding of their processes to inform the development of a common platform underlying a family of similar business processes. [...] We participated as observers in all the eight workshops and in six other meetings. Workshop meetings were audio-recorded with the participants’ consent, yielding an extremely rich set of data of over more than 50 h. Additional informal interviews with process participants were conducted to seek clarifications on issues raised during the workshops. See Online Appendix B for an excerpt of the interview questionnaire. These interviews allowed us to explore the expectations of the participants. Detailed notes were also taken during each of the data collection sessions. Workshops and interviews were our primary source of qualitative data.\" (Research methodology &amp; Data collection, Page 5-6)\n"}</t>
         </is>
       </c>
     </row>
@@ -13939,10 +13707,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F266" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F266" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G266" s="0" t="inlineStr">
         <is>
@@ -13969,7 +13735,7 @@
       </c>
       <c r="P266" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"For our empirical analysis, we use data sets provided by the Netherlands Enterprise Agency (RVO.nl) on all collaborative R&amp;D projects that received support from the allowance scheme in the period 2013–2018. The data sets include information about project titles, starting years, participants and budgets. By merging the data, it is possible to map the evolution of the collaborative network for the period 2013–2018. The total network includes 1884 Dutch firms and 105 publicly-funded organizations. Given our focus on recombining firm capabilities, our analyses concentrate on the 1884 firms only.\" (Case description: collaborative R&amp;D in the Netherlands, Page 4)\n"}</t>
         </is>
       </c>
     </row>
@@ -14229,10 +13995,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F272" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F272" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G272" s="0" t="inlineStr">
         <is>
@@ -14259,7 +14023,7 @@
       </c>
       <c r="P272" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided. Verbatim Evidence: "\"Grouping and Analytic Techniques. Each subject was grouped according to primary decision style which resulted in four groups of individuals being labeled as either SF (n = 20), ST (n = 7), NF (n = 24), or NT (n = 6). Because BSA was defined as multidimensional in nature and was composed of three separate dimensions, the primary analytic technique used was multivariate analysis of variance (MANOVA). This test was run to determine if decision style affected total BSA. Given a significant overall F for the MANOVA test, several post hoc techniques were employed to investigate the specific nature of these differences. First, a multivariate extension of the Scheffe test was used to determine which decision style groups were different from each other across the combination of the three BSA variables.\" (Grouping and Analytic Techniques, Page 6)\n"}</t>
         </is>
       </c>
     </row>
@@ -14375,10 +14139,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F275" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F275" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G275" s="0" t="inlineStr">
         <is>
@@ -14405,7 +14167,7 @@
       </c>
       <c r="P275" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>0 = Exclude\nReason Code: 3\nProject and team level of analysis without individual employee boundary spanning correlations. Verbatim Evidence: "\"From the multiteam system (MTS) perspective, this study employs the input-process-outcome (IPO) framework and coordination theory to explore the influence of instant messaging-based team boundary spanning (IMTBS) on construction project coordination processes and project performance. A theoretical model is built and validated with a survey involving 206 construction projects. [...] Data were collected from construction projects in China. We first conducted a pilot study involving 30 respondents from the Master of Engineering Management (MEM) students majoring in construction management at a Chinese renowned university to test the validity of all constructs. [...] Then, the questionnaire was distributed to construction professionals to report the condition of the last completed project they managed. We randomly sent the link to the online survey to alumni of two renowned universities, who were involved in the construction industry. A total of 400 questionnaires were distributed to these alumni from 53 construction companies, and 256 responses were returned. After removing invalid responses, 206 valid questionnaires were left, thereby yielding a valid response rate of 51.5%.\" (Abstract, Page 1; 4.2 Data collection, Page 7)\n"}</t>
         </is>
       </c>
     </row>
@@ -14425,10 +14187,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F276" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F276" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G276" s="0" t="inlineStr">
         <is>
@@ -14455,7 +14215,7 @@
       </c>
       <c r="P276" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"The referent-shift consensus model proposed by Chan[50]was used in designing the questionnaire, which means that variables including \"team boundary-spanning activities,\" \"team job crafting,\" and \"team innovation performance\" was designed from the perspective of the team. A request was made for these questions to be answered from the perspective of team awareness. The \"individual job crafting\" variable was designed from the employees' perspective. Second, the terminology, the clarity of the instructions, and the structure of the questionnaire's responses were evaluated by three subject-matter experts and five teams from Shandong province's universities engaged in scientific research and innovation. Modifications were made accordingly. Finally, teams that were developing collaborative innovation projects were selected. The distribution of 456 surveys resulted in the recovery of 400 questionnaires. Three hundred thirty-one valid surveys were retrieved after invalid data had been removed; these originated from 41 collaborative innovation teams.\" (3.1 Sample and data collection procedure, Page 6)\n"}</t>
         </is>
       </c>
     </row>
@@ -14475,10 +14235,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F277" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F277" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G277" s="0" t="inlineStr">
         <is>
@@ -14505,7 +14263,7 @@
       </c>
       <c r="P277" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>[Construct homonymy: study measures work-family boundary management, not organizational boundary spanning behavior]. Verbatim Evidence: \\\"OBJECTIVE: This study was conducted to examine how teleworking outside regular office hours and individual boundary management relate to work-family conflict.\\\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -14575,10 +14333,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F279" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F279" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G279" s="0" t="inlineStr">
         <is>
@@ -14605,7 +14361,7 @@
       </c>
       <c r="P279" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>This study describes the organizational arrangements used to source scientific knowledge in two highly successful NBFs -- firms that have succeeded in sourcing and commercializing valuable scientific knowledge. As both firms requested anonymity, we refer to them as Firm X and Firm Y.\" (4.1 Sample)</t>
         </is>
       </c>
     </row>
@@ -14671,10 +14427,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F281" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F281" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G281" s="0" t="inlineStr">
         <is>
@@ -14701,7 +14455,7 @@
       </c>
       <c r="P281" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>I asked two team members in each participating project to provide a single consensual rating for the measures of these forces. I selected the team members upon the advice of senior managers who deemed them as being highly knowledgeable about their projects.</t>
         </is>
       </c>
     </row>
@@ -14721,10 +14475,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F282" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F282" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G282" s="0" t="inlineStr">
         <is>
@@ -14764,7 +14516,7 @@
       </c>
       <c r="P282" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>how others’ availability expectations predict employees’ management of work and nonwork boundaries, and how these bidirectional boundary management behaviors relate to well-being.\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -14784,10 +14536,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F283" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F283" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G283" s="0" t="inlineStr">
         <is>
@@ -14814,7 +14564,7 @@
       </c>
       <c r="P283" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>Problems cross boundaries and so must solutions. The most important challenge for performance networks that aim to deliver better results is designing the structure that coordinates across traditional agency boundaries.</t>
         </is>
       </c>
     </row>
@@ -14834,10 +14584,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F284" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F284" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G284" s="0" t="inlineStr">
         <is>
@@ -14864,7 +14612,7 @@
       </c>
       <c r="P284" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>[Unit of analysis is at the team level]. Verbatim Evidence: \\\"To test hypotheses, the study focuses on technology transfer intermediaries of the manufacturing industry in China at the team level.\\\" (3.1 Research setting)</t>
         </is>
       </c>
     </row>
@@ -14884,10 +14632,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F285" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F285" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G285" s="0" t="inlineStr">
         <is>
@@ -14914,7 +14660,7 @@
       </c>
       <c r="P285" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The level of analysis is an alliance between two partners.</t>
         </is>
       </c>
     </row>
@@ -14980,10 +14726,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F287" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F287" s="0" t="n">
+        <v>5</v>
       </c>
       <c r="G287" s="0" t="inlineStr">
         <is>
@@ -15010,7 +14754,7 @@
       </c>
       <c r="P287" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Qualitative study without quantitative effect sizes based on a non-employee sample. Verbatim Evidence: \\\"This article is based on in-depth interviews with 30 subjects—15 men and 15 women.\\\" (Study design) and \\\"This article proposes to examine the self-concept of members of an occupational category called 'solo self-employed,' that is, women and men who work alone and do not employ any workers.\\\" (Introduction)</t>
         </is>
       </c>
     </row>
@@ -15030,10 +14774,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F288" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F288" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G288" s="0" t="inlineStr">
         <is>
@@ -15060,7 +14802,7 @@
       </c>
       <c r="P288" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The purpose of this paper is to develop the concept of project management system from the perspective of systems science.\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -15130,10 +14872,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F290" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F290" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G290" s="0" t="inlineStr">
         <is>
@@ -15160,7 +14900,7 @@
       </c>
       <c r="P290" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>These are boundary theory (Ashforth et al., 2000; Allen et al., 2014; Nippert Eng, 1996), which focuses on the work-life domain, and border theory (Clark, 2000), which focuses on the work and family domain. As per these theories, individuals are forced to set boundaries to balance their work and family roles.</t>
         </is>
       </c>
     </row>
@@ -15330,10 +15070,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F294" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F294" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G294" s="0" t="inlineStr">
         <is>
@@ -15374,7 +15112,7 @@
       </c>
       <c r="P294" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Study analyzes organizations rather than individuals. Verbatim Evidence: \\\"This paper, in an attempt to link up these ideas, investigates knowledge transfer processes within inter-organizational R&amp;D projects that are embedded in 23 German regional innovation networks (with almost 500 participants).\\\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -15391,14 +15129,10 @@
       </c>
       <c r="E295" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F295" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F295" s="0" t="inlineStr"/>
       <c r="G295" s="0" t="inlineStr">
         <is>
           <t>Boundary -spanning activity (BSA) was studied in two departments of a large governmental research and develop ment organization. BSA was found to be higher and to have significant effects for employees when departmental goals were unclear and technology was non-routine. Under these conditions, BSA was negatively related to role ambiguity and positively related to job satisfaction. Contrary to prior re search, this study found roles with high levels of BSA to have favorable aspects for their incumbents depending upon gorl clarity and type of technology of the parent organization. Implications for the management of research and development organizations are discussed.</t>
@@ -15422,11 +15156,7 @@
       <c r="K295" s="0" t="n">
         <v>1975</v>
       </c>
-      <c r="P295" s="0" t="inlineStr">
-        <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
-        </is>
-      </c>
+      <c r="P295" s="0" t="inlineStr"/>
     </row>
     <row r="296" ht="18" customHeight="1" s="31">
       <c r="A296" s="0" t="inlineStr">
@@ -15640,10 +15370,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F300" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F300" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G300" s="0" t="inlineStr">
         <is>
@@ -15670,7 +15398,7 @@
       </c>
       <c r="P300" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Firm-level analysis. Verbatim Evidence: \\\"To gauge the study hypotheses, time-lagged data were gathered from 244 firms in China.\\\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -15690,10 +15418,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F301" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F301" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G301" s="0" t="inlineStr">
         <is>
@@ -15720,7 +15446,7 @@
       </c>
       <c r="P301" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>the final dataset we retained and used for data analysis pertained to 365 firms.\"\n\nI have successfully updated BSMA_Master_Coding_Sheet.xlsx and committed and pushed the changes to Github.</t>
         </is>
       </c>
     </row>
@@ -15740,10 +15466,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F302" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F302" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G302" s="0" t="inlineStr">
         <is>
@@ -15770,7 +15494,7 @@
       </c>
       <c r="P302" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Organizational behavior (OB) is an area of knowledge rather than a unified theory. It consists of a growing clutch of concepts, approaches, models, and tools pertinent to the structure and functioning of organizations within their socioeconomic contexts and of the study of individuals and groups within their organizational contexts</t>
         </is>
       </c>
     </row>
@@ -15840,10 +15564,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F304" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F304" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G304" s="0" t="inlineStr">
         <is>
@@ -15870,7 +15592,7 @@
       </c>
       <c r="P304" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>[No BSB construct measured]. Verbatim Evidence: \\\"The results indicate that FSEs’ perceptions of CSR are negatively related to their perceptions of verbal dysfunctional customer conduct, which in turn is shown to be directly linked to emotional exhaustion. FSEs’ CSR perceptions strengthen their view that they are performing meaningful work (i.e. perceived task significance), which in turn strengthens their job satisfaction.\\\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -16032,14 +15754,10 @@
       </c>
       <c r="E308" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F308" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F308" s="0" t="inlineStr"/>
       <c r="G308" s="0" t="inlineStr">
         <is>
           <t>Purpose – Drawing on conservation of resources (COR) theory, this research aims to advance the current understanding of leader boundary spanning by examining its effect on task performance, psychological mechanism and boundary conditions.</t>
@@ -16063,11 +15781,7 @@
       <c r="K308" s="0" t="n">
         <v>2025</v>
       </c>
-      <c r="P308" s="0" t="inlineStr">
-        <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
-        </is>
-      </c>
+      <c r="P308" s="0" t="inlineStr"/>
     </row>
     <row r="309" ht="18" customHeight="1" s="31">
       <c r="A309" s="0" t="inlineStr">
@@ -16189,10 +15903,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F311" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F311" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G311" s="0" t="inlineStr">
         <is>
@@ -16219,7 +15931,7 @@
       </c>
       <c r="P311" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>Employees provided information regarding work overload, resilience, and intimidation, while their direct supervisors provided information regarding their subordinates’ sales performance.\" (3.2. Measures)</t>
         </is>
       </c>
     </row>
@@ -16239,10 +15951,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F312" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F312" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G312" s="0" t="inlineStr">
         <is>
@@ -16269,7 +15979,7 @@
       </c>
       <c r="P312" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study focuses on work-nonwork (work-life) boundary management rather than organizational boundary spanning behavior, hence there are no relevant effect sizes. Verbatim Evidence: \\\"In this study we focused on examining employees’ work-nonwork boundary management from the perspective of work stress recovery. Boundary management refers to the ways in which employees create, maintain and negotiate boundaries between work and nonwork\\\" (Introduction)</t>
         </is>
       </c>
     </row>
@@ -16289,10 +15999,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F313" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F313" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G313" s="0" t="inlineStr">
         <is>
@@ -16319,7 +16027,7 @@
       </c>
       <c r="P313" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The purpose of this study was to analyze the school safety and security planning process. Sixty-two public school districts and non public schools within a fifty-mile radius of a large metropolitan area, located within the four states area of Texas, Oklahoma, Arkansas, and Kansas, were carefully studied\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -16389,10 +16097,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F315" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F315" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G315" s="0" t="inlineStr">
         <is>
@@ -16419,7 +16125,7 @@
       </c>
       <c r="P315" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>For each activity, we provide examples and illustrations which we derived by interviewing senior industry professionals from different industries (such as telecommunications, medical devices and pharmaceuticals) and with direct experiences in global boundary spanning and technology scouting. Specifically, between 2011–15, we conducted 15 in-depth interviews with managers in European and North American MNCs</t>
         </is>
       </c>
     </row>
@@ -16439,10 +16145,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F316" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F316" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G316" s="0" t="inlineStr">
         <is>
@@ -16469,7 +16173,7 @@
       </c>
       <c r="P316" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Data were analysed for all references to skills, knowledge, traits, behavioural indicators and outcomes associated with effective and ineffective performance. Over 250 items of data were identified. These were constructed into a framework describing the features of high performance, which was then critically reviewed by a small group of managers (the ‘review group’), and revised.\" (5 Findings)</t>
         </is>
       </c>
     </row>
@@ -16689,10 +16393,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F321" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F321" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G321" s="0" t="inlineStr">
         <is>
@@ -16719,7 +16421,7 @@
       </c>
       <c r="P321" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The questionnaire was designed to measure the perceived: 1) importance and 2) effectiveness of each of the eight classes of MCP’s.\" (IV. METHOD)</t>
         </is>
       </c>
     </row>
@@ -16739,10 +16441,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F322" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F322" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G322" s="0" t="inlineStr">
         <is>
@@ -16769,7 +16469,7 @@
       </c>
       <c r="P322" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The empirical setting is publicly held US manufacturing firms that are present in both the Kinder, Lydenberg and Domini’s (KLD’s) annual EVP ratings and Bloomberg’s supply chain database. The study employs panel data regression methods on an unbalanced panel dataset of 7,493 dyad-year observations comprising 427 unique firms.</t>
         </is>
       </c>
     </row>
@@ -16839,10 +16539,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F324" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F324" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G324" s="0" t="inlineStr">
         <is>
@@ -16869,7 +16567,7 @@
       </c>
       <c r="P324" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>[Team-level aggregation]. Verbatim Evidence: \\\"To use the individuals’ responses for further analysis, the responses were aggregated by extracting the mean scores.\\\" (4. Results)</t>
         </is>
       </c>
     </row>
@@ -16889,10 +16587,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F325" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F325" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G325" s="0" t="inlineStr">
         <is>
@@ -16919,7 +16615,7 @@
       </c>
       <c r="P325" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The questionnaire asked informants to focus on a NPD project (our unit of analysis) completed in the past 12 months.</t>
         </is>
       </c>
     </row>
@@ -17089,10 +16785,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F329" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F329" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G329" s="0" t="inlineStr">
         <is>
@@ -17119,7 +16813,7 @@
       </c>
       <c r="P329" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Our study sample consisted of 2,940 United States Air Force officers from a broad array of job categories, who participated in a five-week leadership development course. As part of the course and a larger program of research,1 the participants were assigned to one of 210 14-person multiteam systems that engaged in a computer-based simulation.</t>
         </is>
       </c>
     </row>
@@ -17239,10 +16933,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F332" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F332" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="G332" s="0" t="inlineStr">
         <is>
@@ -17269,7 +16961,7 @@
       </c>
       <c r="P332" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Based on our experience and emerging literature, such as the papers in this special collection, this article discusses the value of Q-methodology in addressing landscape sustainability issues.\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -17286,14 +16978,10 @@
       </c>
       <c r="E333" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F333" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F333" s="0" t="inlineStr"/>
       <c r="G333" s="0" t="inlineStr">
         <is>
           <t>The purpose of the study was to explore the relationships among environmental characteristics, uncertainty, boundary spanning activities, managerial discretion, and power of the department store apparel buyer who assumes combination or independent buyer responsibilities. Almubarek’s Model of Organizational Boundary Spanning and Duncan’s (1972) Model of Environmental Uncertainty were used as conceptualframeworks. A questionnaire was mailed to buyers who purchased merchandise in the moderate-to-better sportswear areas in the top 10 department store groups in the United States.</t>
@@ -17317,11 +17005,7 @@
       <c r="K333" s="0" t="n">
         <v>2001</v>
       </c>
-      <c r="P333" s="0" t="inlineStr">
-        <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
-        </is>
-      </c>
+      <c r="P333" s="0" t="inlineStr"/>
     </row>
     <row r="334" ht="18" customHeight="1" s="31">
       <c r="A334" s="0" t="inlineStr">
@@ -17389,10 +17073,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F335" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F335" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G335" s="0" t="inlineStr">
         <is>
@@ -17419,7 +17101,7 @@
       </c>
       <c r="P335" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries.</t>
         </is>
       </c>
     </row>
@@ -17489,10 +17171,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F337" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
+      <c r="F337" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="G337" s="0" t="inlineStr">
         <is>
@@ -17519,7 +17199,7 @@
       </c>
       <c r="P337" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>While formalization measure was modified slightly to be tailored to the unique Korean sales job environment, the other four variables of role ambiguity, role conflict, commitment, and propensity-to-leave were adopted from American literature.\" (Measurement)</t>
         </is>
       </c>
     </row>
@@ -17773,10 +17453,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F343" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
+      <c r="F343" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G343" s="0" t="inlineStr">
         <is>
@@ -17803,7 +17481,7 @@
       </c>
       <c r="P343" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The unit of analysis for the questionnaire was the new product development project and the informant was asked to select the most recent project he/she worked for.\" (3.2. Questionnaire)</t>
         </is>
       </c>
     </row>
@@ -17873,10 +17551,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F345" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F345" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G345" s="0" t="inlineStr">
         <is>
@@ -17903,7 +17579,7 @@
       </c>
       <c r="P345" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The samples for the survey comprised IT development MTSs within IT firms located in China.\" (IV. METHODOLOGY, A. Samples and Data Collection)</t>
         </is>
       </c>
     </row>
@@ -17923,10 +17599,8 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F346" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
+      <c r="F346" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G346" s="0" t="inlineStr">
         <is>
@@ -17953,7 +17627,7 @@
       </c>
       <c r="P346" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>[Team level analysis]. Verbatim Evidence: \\\"We computed within-group interrater agreement (rwg; James, Demaree, &amp; Wolf, 1993) and ICC values to justify the aggregation of constructs to the team level, which provided adequate support.\\\" (Data Analysis)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
style: normalize format for 16th column removing internal script prefixes
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -941,7 +941,7 @@
       </c>
       <c r="P4" s="0" t="inlineStr">
         <is>
-          <t>The data analyzed in this dissertation exist at three levels- the individual level, the team level and the service region unit level. For the team process measures, data were aggregated from the individual to the team level. Table 3 in Appendix 1 presents ICC coefficients for the aggregation of the team process variables from individual to the team level. The ICCs for this aggregation range from .10 ( for intra-team cooperation) to .07 (for inter-team cooperation) with an average ICC of .08. These results suggest that on average 8% of the variance in the team process measures were explained by differences between teams.\" (Data Aggregation, Page 70)</t>
+          <t>Team level analysis. Verbatim Evidence: \"The data analyzed in this dissertation exist at three levels- the individual level, the team level and the service region unit level. For the team process measures, data were aggregated from the individual to the team level. Table 3 in Appendix 1 presents ICC coefficients for the aggregation of the team process variables from individual to the team level. The ICCs for this aggregation range from .10 ( for intra-team cooperation) to .07 (for inter-team cooperation) with an average ICC of .08. These results suggest that on average 8% of the variance in the team process measures were explained by differences between teams.\" (Data Aggregation, Page 70)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="P5" s="0" t="inlineStr">
         <is>
-          <t>Two sets of data are fit to the quarter mile or longer rectangular buffer zones: characteristics from the 1910 to 1930 decennial censuses and outcomes from the Opportunity Atlas. On the former, we use the 1910 to 1930 100 percent Census population counts from Minnesota Population Center and Ancestry.com (2013). We are able to match roughly 50 to 80 percent of respondents to HOLC neighborhoods.7 We aggregate census measures to the buffer zone by taking the mean of all observations which fall inside of a buffer zone so long as it contains at least 3 households.\" (Data, Page 8)</t>
+          <t>Non-employee general citizen sample based on census population counts. Verbatim Evidence: \"Two sets of data are fit to the quarter mile or longer rectangular buffer zones: characteristics from the 1910 to 1930 decennial censuses and outcomes from the Opportunity Atlas. On the former, we use the 1910 to 1930 100 percent Census population counts from Minnesota Population Center and Ancestry.com (2013). We are able to match roughly 50 to 80 percent of respondents to HOLC neighborhoods.7 We aggregate census measures to the buffer zone by taking the mean of all observations which fall inside of a buffer zone so long as it contains at least 3 households.\" (Data, Page 8)</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="P6" s="0" t="inlineStr">
         <is>
-          <t>The data for this research is drawn from the 2016 International City/County Management Association (ICMA) Smart Cities Survey. Partnering with the Smart Cities Council, ICMA sent the survey in 2016 to 3,423 local government officers working in U.S. cities and counties with populations of 25,000 or greater. In all, 493 officers responded to the survey questions by email or mail, giving a response rate of 14.4%. The survey consisted of twenty questions asking officers about their local governments’ smart cities practices including: their commitment to SCT (priorities), their engagement with SCT (activities), their perceived benefits of using SCT, and their barriers to implementing SCT. The survey also provides insights into the extent to which local governments pursuing SCT are collaborating with other government agencies and authorities. The survey further offers information on the financial mechanisms localities are using to fund SCT efforts and projects. The data from the ICMA survey was merged with information on demographic, economic, and population data drawn from the 2016 U.S. Census Bureau database. After eliminating records with missing data, our final sample includes responses from 234 local governments.\" (Methodology, Page 247)</t>
+          <t>Organizational level analysis of local governments. Verbatim Evidence: \"The data for this research is drawn from the 2016 International City/County Management Association (ICMA) Smart Cities Survey. Partnering with the Smart Cities Council, ICMA sent the survey in 2016 to 3,423 local government officers working in U.S. cities and counties with populations of 25,000 or greater. In all, 493 officers responded to the survey questions by email or mail, giving a response rate of 14.4%. The survey consisted of twenty questions asking officers about their local governments’ smart cities practices including: their commitment to SCT (priorities), their engagement with SCT (activities), their perceived benefits of using SCT, and their barriers to implementing SCT. The survey also provides insights into the extent to which local governments pursuing SCT are collaborating with other government agencies and authorities. The survey further offers information on the financial mechanisms localities are using to fund SCT efforts and projects. The data from the ICMA survey was merged with information on demographic, economic, and population data drawn from the 2016 U.S. Census Bureau database. After eliminating records with missing data, our final sample includes responses from 234 local governments.\" (Methodology, Page 247)</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="P7" s="0" t="inlineStr">
         <is>
-          <t>The unit of analysis of this study is firm. A firm is used as the unit of analysis because the research questions seek to examine factors that determine a firm’s ability to innovate and to integrate employees’ knowledge. Various researchers have also used firm as the unit of analysis to examine a firm's ability to innovate in the various contexts, such as network ties (Ozer &amp; Zhang, 2015), firm size (Leiblein &amp; Madsen, 2009), and strategic fit (Kim, Arthurs, Sahaym, &amp; Cullen, 2013).\" (Unit of Analysis, Page 66)</t>
+          <t>Firm-level analysis. Verbatim Evidence: \"The unit of analysis of this study is firm. A firm is used as the unit of analysis because the research questions seek to examine factors that determine a firm’s ability to innovate and to integrate employees’ knowledge. Various researchers have also used firm as the unit of analysis to examine a firm's ability to innovate in the various contexts, such as network ties (Ozer &amp; Zhang, 2015), firm size (Leiblein &amp; Madsen, 2009), and strategic fit (Kim, Arthurs, Sahaym, &amp; Cullen, 2013).\" (Unit of Analysis, Page 66)</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="P8" s="0" t="inlineStr">
         <is>
-          <t>In this article, the author begins by defining collaborative partnerships between academics and community stakeholders and then states specific advantages and challenges to collaborative partnerships in the field of social work. Throughout, the author explains how the historical foundations of the field (for example, acting as boundary spanners, advocating for marginalized individuals) place social workers in an ideal position to become leaders in the development, sustainment, and strengthening of CAPs. The author details the ways in which social work researchers can use the field’s unique history to enhance the development and sustainment of CAPs. The article concludes by encouraging the field to use standardized terminology, methodology, and evaluation procedures when conducting CAPs and providing strategies for social work researchers who wish to increase their ability to develop and sustain CAPs within their own institutions.\" (Abstract, Page 19)</t>
+          <t>This is a purely conceptual paper discussing collaborative partnerships and boundary spanning historically, and it provides no primary quantitative employee survey data or Pearson correlation matrix. Verbatim Evidence: \"In this article, the author begins by defining collaborative partnerships between academics and community stakeholders and then states specific advantages and challenges to collaborative partnerships in the field of social work. Throughout, the author explains how the historical foundations of the field (for example, acting as boundary spanners, advocating for marginalized individuals) place social workers in an ideal position to become leaders in the development, sustainment, and strengthening of CAPs. The author details the ways in which social work researchers can use the field’s unique history to enhance the development and sustainment of CAPs. The article concludes by encouraging the field to use standardized terminology, methodology, and evaluation procedures when conducting CAPs and providing strategies for social work researchers who wish to increase their ability to develop and sustain CAPs within their own institutions.\" (Abstract, Page 19)</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="P9" s="0" t="inlineStr">
         <is>
-          <t>A sample of 2,000 high-prescribing physicians was randomly drawn from a population of over 30,000 high-prescribing physicians in the focal drug category. We considered only high-prescribing physicians for this research to ensure that each physician wrote a sufficient number of prescriptions in the category and that the sales representatives would have had regular contact with the physicians (e.g., industry records indicate that the representative calls on the high-prescribing physician on average 26 times per year). A professional market research company contacted these 2,000 physician offices by telephone and invited physicians to participate in a survey that was being conducted and independently funded by a major U.S. university. Questionnaires were distributed to this sample of physicians via fax. Participants were assured that their individual responses would be confidential and received a $30 industry-standard honorarium for their participation. Completed surveys were faxed directly back to the researchers, yielding a final sample of 178 physicians.\" (Method, page 5)</t>
+          <t>The study sampled customers (physicians) rather than employees of the focal organization. Verbatim Evidence: \"A sample of 2,000 high-prescribing physicians was randomly drawn from a population of over 30,000 high-prescribing physicians in the focal drug category. We considered only high-prescribing physicians for this research to ensure that each physician wrote a sufficient number of prescriptions in the category and that the sales representatives would have had regular contact with the physicians (e.g., industry records indicate that the representative calls on the high-prescribing physician on average 26 times per year). A professional market research company contacted these 2,000 physician offices by telephone and invited physicians to participate in a survey that was being conducted and independently funded by a major U.S. university. Questionnaires were distributed to this sample of physicians via fax. Participants were assured that their individual responses would be confidential and received a $30 industry-standard honorarium for their participation. Completed surveys were faxed directly back to the researchers, yielding a final sample of 178 physicians.\" (Method, page 5)</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="P10" s="0" t="inlineStr">
         <is>
-          <t>The unit of analysis is the firm-therapeutic level, i.e., the firm's alliance activities in a therapeutic area (for example, Merck's alliances in cardiovascular therapeutic area). The arguments are tested using panel data estimation techniques... The study identified 1932 alliances formed between incumbent pharmaceutical and new biotechnology firms in eighteen therapeutic areas by seventeen large pharmaceutical firms during the time period from 1991 to 2004. The focal firms are traditional pharmaceutical firms listed under Standard Industrial Classification (SIC) codes 2834 and 5122, 'Pharmaceutical Preparations' and 'Wholesale-Drugs, Proprietaries &amp; Druggists Sundries' respectively. In this industry, the incumbent pharmaceutical firms are primarily attempting to adapt to the emerging technologies by forming alliances (i.e., equity and non-equity partnerships) with new biotechnology firms (Rothaermel, 2000).\" (Methods / Sample and Data, Page 9)</t>
+          <t>Firm-level analysis of pharmaceutical alliances. Verbatim Evidence: \"The unit of analysis is the firm-therapeutic level, i.e., the firm's alliance activities in a therapeutic area (for example, Merck's alliances in cardiovascular therapeutic area). The arguments are tested using panel data estimation techniques... The study identified 1932 alliances formed between incumbent pharmaceutical and new biotechnology firms in eighteen therapeutic areas by seventeen large pharmaceutical firms during the time period from 1991 to 2004. The focal firms are traditional pharmaceutical firms listed under Standard Industrial Classification (SIC) codes 2834 and 5122, 'Pharmaceutical Preparations' and 'Wholesale-Drugs, Proprietaries &amp; Druggists Sundries' respectively. In this industry, the incumbent pharmaceutical firms are primarily attempting to adapt to the emerging technologies by forming alliances (i.e., equity and non-equity partnerships) with new biotechnology firms (Rothaermel, 2000).\" (Methods / Sample and Data, Page 9)</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="P11" s="0" t="inlineStr">
         <is>
-          <t>However, these hypotheses are unobservable and are not a priori shared in the public domain. Therefore, as previously mentioned, separate empirical experiments are necessary. In this section, we discuss how the modified explanatory hypotheses can be validated through experimentation. As an example of experimental method, it would be appropriate to employ a structured questionnaire and participant observation in case study, and to select an analytical method that can show a strong explanatory model with a small number of samples while converting qualitative information into quantitative information, such as Qualitative Comparative Analysis (QCA), for the data collected.\" (4. Conclusion, limitations, and future directions, Page 7)</t>
+          <t>Conceptual paper lacking empirical data. Verbatim Evidence: \"However, these hypotheses are unobservable and are not a priori shared in the public domain. Therefore, as previously mentioned, separate empirical experiments are necessary. In this section, we discuss how the modified explanatory hypotheses can be validated through experimentation. As an example of experimental method, it would be appropriate to employ a structured questionnaire and participant observation in case study, and to select an analytical method that can show a strong explanatory model with a small number of samples while converting qualitative information into quantitative information, such as Qualitative Comparative Analysis (QCA), for the data collected.\" (4. Conclusion, limitations, and future directions, Page 7)</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="P12" s="0" t="inlineStr">
         <is>
-          <t>Since our study focused on the NPD team as a unit of analysis, product/project managers were likely to assess our variables more accurately. Also, the sample of respondents was similar to samples used in prior studies on innovation. Each product/project manager in the PMI mailing list received an invitation to participate in our study (including a cover letter, the questionnaire, and stamped return envelope). Informants were asked to focus on their most recent product development projects (ones in the marketplace for a minimum of 12 months to ensure accurate assessment of the product performance). We received 207 usable responses (an effective response rate of 16.5%) representing a wide range of industries in the manufacturing sector, including: pharmaceuticals (28.5%), automotive (17%), electrical/electronics (17.9%), computers (13%), chemicals (8.7%), machinery/metal manufacturing (7.2%), and others (7.2%).\" (Measures and sampling, Page 223)</t>
+          <t>Team level analysis. Verbatim Evidence: \"Since our study focused on the NPD team as a unit of analysis, product/project managers were likely to assess our variables more accurately. Also, the sample of respondents was similar to samples used in prior studies on innovation. Each product/project manager in the PMI mailing list received an invitation to participate in our study (including a cover letter, the questionnaire, and stamped return envelope). Informants were asked to focus on their most recent product development projects (ones in the marketplace for a minimum of 12 months to ensure accurate assessment of the product performance). We received 207 usable responses (an effective response rate of 16.5%) representing a wide range of industries in the manufacturing sector, including: pharmaceuticals (28.5%), automotive (17%), electrical/electronics (17.9%), computers (13%), chemicals (8.7%), machinery/metal manufacturing (7.2%), and others (7.2%).\" (Measures and sampling, Page 223)</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="P13" s="0" t="inlineStr">
         <is>
-          <t>Among the 180 firms contacted, we received 92 usable returns concerning NPD projects. During the sampling, to assess the product performance more accurately, we set the condition that the products used in this study must have been commercialized and launched into the marketplace for at least six months (Lynn et al., 2000). Also, the team size was an important constraint such that it should contain more than three members. Furthermore, to reduce the possible problems associated with single sourcing, we targeted the product or project manager to complete the survey. These managers were chosen because (1) product/project managers are likely to have a ‘bigger-picture view’ of NPD projects than other team members; (2) project managers have a broader view of each member’s behaviors than other team members\" (4.1. Sampling, Page 7)</t>
+          <t>Team level of analysis. The study's primary unit of analysis is the new product development (NPD) project team, with constructs assessed by project managers at the team level. Verbatim Evidence: \"Among the 180 firms contacted, we received 92 usable returns concerning NPD projects. During the sampling, to assess the product performance more accurately, we set the condition that the products used in this study must have been commercialized and launched into the marketplace for at least six months (Lynn et al., 2000). Also, the team size was an important constraint such that it should contain more than three members. Furthermore, to reduce the possible problems associated with single sourcing, we targeted the product or project manager to complete the survey. These managers were chosen because (1) product/project managers are likely to have a ‘bigger-picture view’ of NPD projects than other team members; (2) project managers have a broader view of each member’s behaviors than other team members\" (4.1. Sampling, Page 7)</t>
         </is>
       </c>
     </row>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="P149" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Our final sample consisted of those 57 teams from which we had received three or more subordinate surveys and a supervisor survey, and for which archival data were available. These teams ranged in size from 4 to 26 members (x = 11.7, s.d. = 6.1); 84 percent of team members were male; the average age was 42.7 years (s.d. = 7.7), and the average time with the current team was 1.5 years (s.d. = .5). [...] Together, the above analyses supported the aggregation of informant responses from a team to create team-level variables for collective team identification, team learning, intrateam conflict, and external communication.\" (Sample and Data Collection / Interrater agreement and reliability, Pages 537-539)\n\nNote: The specific file \"Guenzel (2020) - Open innovation...\" did not exist in the workspace, so the paper with ID 201 mapped in all_remaining_targets.txt (\"[201] Van der vegt &amp; Bunderson (2005) - LEARNING AND PERFORMANCE IN MULTIDISCIPLINARY TEAMS.pdf\") was reviewed instead as standard procedure.</t>
+          <t>Team level analysis. Verbatim Evidence: \"Our final sample consisted of those 57 teams from which we had received three or more subordinate surveys and a supervisor survey, and for which archival data were available. These teams ranged in size from 4 to 26 members (x = 11.7, s.d. = 6.1); 84 percent of team members were male; the average age was 42.7 years (s.d. = 7.7), and the average time with the current team was 1.5 years (s.d. = .5). [...] Together, the above analyses supported the aggregation of informant responses from a team to create team-level variables for collective team identification, team learning, intrateam conflict, and external communication.\" (Sample and Data Collection / Interrater agreement and reliability, Pages 537-539)  Note: The specific file \"Guenzel (2020) - Open innovation...\" did not exist in the workspace, so the paper with ID 201 mapped in all_remaining_targets.txt (\"[201] Van der vegt &amp; Bunderson (2005) - LEARNING AND PERFORMANCE IN MULTIDISCIPLINARY TEAMS.pdf\") was reviewed instead as standard procedure.</t>
         </is>
       </c>
     </row>
@@ -8211,7 +8211,7 @@
       </c>
       <c r="P150" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Agents in creative enterprises are embedded in networks that inspire, support, and evaluate their work. Here, we investigate how the mechanisms by which creative teams self-assemble determine the structure of these collaboration networks. We propose a model for team self-assembly that is based on three parameters: team size, the fraction of newcomers in new productions, and the tendency of incumbents to repeat previous collaborations. The model suggests that the emergence of a large connected community of practitioners can be described as a phase transition. We find that the model team assembly mechanisms determine both the topological structure of the collaboration network and team performance in fields as diverse as Broadway musicals and scientific research.\" (Abstract, Page 1)</t>
+          <t>Team level analysis. Verbatim Evidence: \"Agents in creative enterprises are embedded in networks that inspire, support, and evaluate their work. Here, we investigate how the mechanisms by which creative teams self-assemble determine the structure of these collaboration networks. We propose a model for team self-assembly that is based on three parameters: team size, the fraction of newcomers in new productions, and the tendency of incumbents to repeat previous collaborations. The model suggests that the emergence of a large connected community of practitioners can be described as a phase transition. We find that the model team assembly mechanisms determine both the topological structure of the collaboration network and team performance in fields as diverse as Broadway musicals and scientific research.\" (Abstract, Page 1)</t>
         </is>
       </c>
     </row>
@@ -8257,7 +8257,7 @@
       </c>
       <c r="P151" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"After excluding teams for which fewer than 50 percent of the respondents were core members (Hackman, 2002: 47), 96 teams qualified for the study (80 percent; 50 financial and 46 technical teams, with 485 member respondents). Tests for selection bias showed no significant differences in the effectiveness ratings, project types, regions, or divisions of the 24 teams that did not qualify. Dependent variables. The dependent variables in this study were (1) the strategic effectiveness of a team and (2) the operational effectiveness of a team, as rated by its independent expert panel.\" (Quantitative Data, Page 995)</t>
+          <t>Team level analysis. Verbatim Evidence: \"After excluding teams for which fewer than 50 percent of the respondents were core members (Hackman, 2002: 47), 96 teams qualified for the study (80 percent; 50 financial and 46 technical teams, with 485 member respondents). Tests for selection bias showed no significant differences in the effectiveness ratings, project types, regions, or divisions of the 24 teams that did not qualify. Dependent variables. The dependent variables in this study were (1) the strategic effectiveness of a team and (2) the operational effectiveness of a team, as rated by its independent expert panel.\" (Quantitative Data, Page 995)</t>
         </is>
       </c>
     </row>
@@ -8353,7 +8353,7 @@
       </c>
       <c r="P153" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study provides a quantitative correlation matrix based on an employee sample, but it does not measure Boundary Spanning Behavior (BSB) or include it in the effect sizes. The measured variables are limited to transformational leadership, internal/external support for innovation, firm age, and organizational innovation. Verbatim Evidence: \"Employees’ questionnaires included measures of transformational leadership and internal support for innovation. On average, four employees rated each leader. Employees were also asked for their age, gender, educational level, job tenure, and company tenure. Leaders’ questionnaires included questions about company age, company innovations, and the degree of support they received from external institutions.\" (Procedure, Page 7)</t>
+          <t>The study provides a quantitative correlation matrix based on an employee sample, but it does not measure Boundary Spanning Behavior (BSB) or include it in the effect sizes. The measured variables are limited to transformational leadership, internal/external support for innovation, firm age, and organizational innovation. Verbatim Evidence: \"Employees’ questionnaires included measures of transformational leadership and internal support for innovation. On average, four employees rated each leader. Employees were also asked for their age, gender, educational level, job tenure, and company tenure. Leaders’ questionnaires included questions about company age, company innovations, and the degree of support they received from external institutions.\" (Procedure, Page 7)</t>
         </is>
       </c>
     </row>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="P154" s="0" t="inlineStr">
         <is>
-          <t>1 = Include\n\nThe paper samples individual organizational employees (132 full-time employees at a scientific facility) and provides an individual-level Pearson correlation matrix (Table 1) that includes quantitative measures of Discretionary Boundary Spanning (DBS) ties (task-oriented and friendship) and their relationship with informal leadership and job performance. Therefore, it meets all inclusion criteria for the meta-analysis.</t>
+          <t>1 = Include  The paper samples individual organizational employees (132 full-time employees at a scientific facility) and provides an individual-level Pearson correlation matrix (Table 1) that includes quantitative measures of Discretionary Boundary Spanning (DBS) ties (task-oriented and friendship) and their relationship with informal leadership and job performance. Therefore, it meets all inclusion criteria for the meta-analysis.</t>
         </is>
       </c>
     </row>
@@ -8499,7 +8499,7 @@
       </c>
       <c r="P156" s="0" t="inlineStr">
         <is>
-          <t>1 = Include\n\nNote: The actual file for ID 208 was found as `[208] Zhang et al. (2024) - The Double-Edged Sword Effect of Performance Pressure on Employee Boundary-Spanning.pdf`. The study samples individual organizational employees (N=336) and provides a quantitative individual-level Pearson correlation matrix (Table 2) containing the variable Employee Boundary-Spanning Behavior (EBSB). It fully meets the inclusion criteria.</t>
+          <t>1 = Include  Note: The actual file for ID 208 was found as `[208] Zhang et al. (2024) - The Double-Edged Sword Effect of Performance Pressure on Employee Boundary-Spanning.pdf`. The study samples individual organizational employees (N=336) and provides a quantitative individual-level Pearson correlation matrix (Table 2) containing the variable Employee Boundary-Spanning Behavior (EBSB). It fully meets the inclusion criteria.</t>
         </is>
       </c>
     </row>
@@ -8545,7 +8545,7 @@
       </c>
       <c r="P157" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 99\nFile not found on disk. Verbatim Evidence: \"failed to read file: open g:/My Drive/UCL/BSMA/BSMA ANTIGRAVITY/01_Academic_Papers/[209] Hanisch et al. (2014) - Innovation network formation a conceptual model.pdf: The system cannot find the file specified. A global search for Hanisch across the BSMA ANTIGRAVITY workspace yielded zero results. Therefore, this paper cannot be audited and is excluded due to a missing file.\" (System Error Log, Page 1)</t>
+          <t>File not found on disk. Verbatim Evidence: \"failed to read file: open g:/My Drive/UCL/BSMA/BSMA ANTIGRAVITY/01_Academic_Papers/[209] Hanisch et al. (2014) - Innovation network formation a conceptual model.pdf: The system cannot find the file specified. A global search for Hanisch across the BSMA ANTIGRAVITY workspace yielded zero results. Therefore, this paper cannot be audited and is excluded due to a missing file.\" (System Error Log, Page 1)</t>
         </is>
       </c>
     </row>
@@ -8591,7 +8591,7 @@
       </c>
       <c r="P158" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"We first obtained a list of 272 public pharmaceutical companies based on the standard industry classification code (SIC 2834). By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005. To test our model, we collect secondary data about firms’ IT-enabled knowledge capabilities and innovation outcomes from multiple secondary data sources.\" (Data Collection, Page 9)</t>
+          <t>Firm level analysis. Verbatim Evidence: \"We first obtained a list of 272 public pharmaceutical companies based on the standard industry classification code (SIC 2834). By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005. To test our model, we collect secondary data about firms’ IT-enabled knowledge capabilities and innovation outcomes from multiple secondary data sources.\" (Data Collection, Page 9)</t>
         </is>
       </c>
     </row>
@@ -8639,7 +8639,7 @@
       </c>
       <c r="P159" s="0" t="inlineStr">
         <is>
-          <t>1 = Include\nReason Code: 0\nThe study samples individual organizational employees and provides an individual-level Pearson correlation matrix that includes a measure of boundary-spanning leadership. Verbatim Evidence: \"The sample comprises four public-sector and four private-sector banks (NSE/BSE indexed) with 12 branches of each bank. The number of respondents from public-sector and private-sector banks was 327 and 308, respectively. Data were collected through a questionnaire comprising 40 items reflecting all the constructs (Generational diversity, knowledge sharing, group performance, intergenerational climate, boundary-spanning leadership, and respect). The study followed a cross-sectional approach for collecting data. The clerical and managerial employees in the bank branches were contacted through offline survey methods.\" (Sample, Page 7)</t>
+          <t>The study samples individual organizational employees and provides an individual-level Pearson correlation matrix that includes a measure of boundary-spanning leadership. Verbatim Evidence: \"The sample comprises four public-sector and four private-sector banks (NSE/BSE indexed) with 12 branches of each bank. The number of respondents from public-sector and private-sector banks was 327 and 308, respectively. Data were collected through a questionnaire comprising 40 items reflecting all the constructs (Generational diversity, knowledge sharing, group performance, intergenerational climate, boundary-spanning leadership, and respect). The study followed a cross-sectional approach for collecting data. The clerical and managerial employees in the bank branches were contacted through offline survey methods.\" (Sample, Page 7)</t>
         </is>
       </c>
     </row>
@@ -8685,7 +8685,7 @@
       </c>
       <c r="P160" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative study without quantitative effect sizes. Verbatim Evidence: \"A thematic analysis of the discourse collected through in-depth interviews, survey questionnaires, and organizational documents was conducted using the constant comparative method (Lindlof, 1995). This process begins with data “reduction” and “interpretation” (Creswell, 1997; Lindlof, 1995) and is consistent with processes engaged in by other communication scholars doing interpretive work (e.g., Braithwaite, Baxter, &amp; Harper, 1998; Clair &amp; Thompson, 1996; Trethewey, 1997). First, all transcripts and documents were read in their entirety to develop a sense of these data as a whole.\" (Data Analysis, Page 8)</t>
+          <t>Qualitative study without quantitative effect sizes. Verbatim Evidence: \"A thematic analysis of the discourse collected through in-depth interviews, survey questionnaires, and organizational documents was conducted using the constant comparative method (Lindlof, 1995). This process begins with data “reduction” and “interpretation” (Creswell, 1997; Lindlof, 1995) and is consistent with processes engaged in by other communication scholars doing interpretive work (e.g., Braithwaite, Baxter, &amp; Harper, 1998; Clair &amp; Thompson, 1996; Trethewey, 1997). First, all transcripts and documents were read in their entirety to develop a sense of these data as a whole.\" (Data Analysis, Page 8)</t>
         </is>
       </c>
     </row>
@@ -8831,7 +8831,7 @@
       </c>
       <c r="P163" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative case study without quantitative correlation data. Verbatim Evidence: \"Following other researchers who are interested in organizational processes (e.g., Anand, Gardner, &amp; Morris, 2007; Bresman, 2013; Nag &amp; Gioia, 2012), we combined a case study approach with grounded theory methodology (Langley, 1999). Specifically, we first used grounded methods to develop cases describing the sequence of early boundary spanning activity in each of 10 COTs; we then used a case study approach to compare and contrast those sequences across the 10 teams. Case studies drew on interviews with 46 team members.\" (Method, page 512)</t>
+          <t>Qualitative case study without quantitative correlation data. Verbatim Evidence: \"Following other researchers who are interested in organizational processes (e.g., Anand, Gardner, &amp; Morris, 2007; Bresman, 2013; Nag &amp; Gioia, 2012), we combined a case study approach with grounded theory methodology (Langley, 1999). Specifically, we first used grounded methods to develop cases describing the sequence of early boundary spanning activity in each of 10 COTs; we then used a case study approach to compare and contrast those sequences across the 10 teams. Case studies drew on interviews with 46 team members.\" (Method, page 512)</t>
         </is>
       </c>
     </row>
@@ -8877,7 +8877,7 @@
       </c>
       <c r="P164" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level variables. The study measures external team learning and team performance rather than individual-level employee boundary spanning behavior. Verbatim Evidence: \"For data collection, we adapted the Team Learning Survey (TSL) and Team Performance Survey (TPS) scales used by Edmondson (1996) while investigating team learning in a large office furniture manufacturer in the American Mid-West. The Team Learning Survey (TLS) incorporated both the internal and the external team learning behaviors each measured through five items. The team performance construct in the Team Performance Survey (TPS) was also measured through five items. The respondents were asked to record their responses on a seven-point likert scale where 1 meant strongly disagree and 7 meant strongly agree.\" (Methods, Page 126)</t>
+          <t>Team level variables. The study measures external team learning and team performance rather than individual-level employee boundary spanning behavior. Verbatim Evidence: \"For data collection, we adapted the Team Learning Survey (TSL) and Team Performance Survey (TPS) scales used by Edmondson (1996) while investigating team learning in a large office furniture manufacturer in the American Mid-West. The Team Learning Survey (TLS) incorporated both the internal and the external team learning behaviors each measured through five items. The team performance construct in the Team Performance Survey (TPS) was also measured through five items. The respondents were asked to record their responses on a seven-point likert scale where 1 meant strongly disagree and 7 meant strongly agree.\" (Methods, Page 126)</t>
         </is>
       </c>
     </row>
@@ -8923,7 +8923,7 @@
       </c>
       <c r="P165" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study conducts a social network analysis calculating network centrality measures rather than using psychometric scales, and it does not report a bivariate Pearson correlation matrix. Verbatim Evidence: \"Survey responses were exported from Qualtrics® into a spreadsheet where the data were cleaned following a two-step process. First, participants’ identification numbers were checked against a master list to ensure that only the data from invited respondents were included. In situations where a participant’s data were recorded twice, only the first record was retained. Second, only participants who completed the sociodemographic survey questions and listed at least one person using their full name as a source of advice or information about PBS were included. Social network data in the form of adjacency lists were created and imported into the social network software Visone (Algorithmics Group, 2019) where graphs were constructed and analyses conducted, including calculation of indegree and betweenness centralities.\" (Data extraction and analysis, Page 5)</t>
+          <t>The study conducts a social network analysis calculating network centrality measures rather than using psychometric scales, and it does not report a bivariate Pearson correlation matrix. Verbatim Evidence: \"Survey responses were exported from Qualtrics® into a spreadsheet where the data were cleaned following a two-step process. First, participants’ identification numbers were checked against a master list to ensure that only the data from invited respondents were included. In situations where a participant’s data were recorded twice, only the first record was retained. Second, only participants who completed the sociodemographic survey questions and listed at least one person using their full name as a source of advice or information about PBS were included. Social network data in the form of adjacency lists were created and imported into the social network software Visone (Algorithmics Group, 2019) where graphs were constructed and analyses conducted, including calculation of indegree and betweenness centralities.\" (Data extraction and analysis, Page 5)</t>
         </is>
       </c>
     </row>
@@ -9019,7 +9019,7 @@
       </c>
       <c r="P167" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam and firm level of analysis. Verbatim Evidence: \"Using CorpTech (now part of InfoUSA), we built a sampling frame of 467 small- to medium-sized enterprises (SMEs) operating in technology-based sectors in the northeastern United States. [...] All told, for 99 firms, we received responses from the CEO and at least another member of the top management team. [...] Apart from the dependent variable, which relies on the assessment of the CEO, our measures involved the aggregated responses of top managers. We separated the measurement of our independent and dependent variables using separate respondents to minimize the influence of common method effects. [...] An acceptable level of interrater agreement (median rwg(j) = 0.94) and reliability (ICC1 = 0.31, ICC2 = 0.69) justified the aggregation of top managers’ responses to the team level of analysis (Chan 1998).\" (Method, Pages 946-947)</t>
+          <t>Team and firm level of analysis. Verbatim Evidence: \"Using CorpTech (now part of InfoUSA), we built a sampling frame of 467 small- to medium-sized enterprises (SMEs) operating in technology-based sectors in the northeastern United States. [...] All told, for 99 firms, we received responses from the CEO and at least another member of the top management team. [...] Apart from the dependent variable, which relies on the assessment of the CEO, our measures involved the aggregated responses of top managers. We separated the measurement of our independent and dependent variables using separate respondents to minimize the influence of common method effects. [...] An acceptable level of interrater agreement (median rwg(j) = 0.94) and reliability (ICC1 = 0.31, ICC2 = 0.69) justified the aggregation of top managers’ responses to the team level of analysis (Chan 1998).\" (Method, Pages 946-947)</t>
         </is>
       </c>
     </row>
@@ -9161,7 +9161,7 @@
       </c>
       <c r="P170" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"The average succession rate for any given company was found by aggregating (averaging) the reciprocals of completed office tenures during the 30-year interval for all presidential successors who held the title Chief Executive Officer. Office tenure for successors was determined by examining selected editions of Moody’s Industrial Manual [28]. The specification of the 30-year interval was also statistically necessary because of the need to control the time variable across companies when developing ex post facto measures of succession rate and variability in measures of board size.\" (Operational Definitions, Page 5)</t>
+          <t>Firm level analysis. Verbatim Evidence: \"The average succession rate for any given company was found by aggregating (averaging) the reciprocals of completed office tenures during the 30-year interval for all presidential successors who held the title Chief Executive Officer. Office tenure for successors was determined by examining selected editions of Moody’s Industrial Manual [28]. The specification of the 30-year interval was also statistically necessary because of the need to control the time variable across companies when developing ex post facto measures of succession rate and variability in measures of board size.\" (Operational Definitions, Page 5)</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9207,7 @@
       </c>
       <c r="P171" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Four organizations participated, providing 56 R&amp;D teams. Two of the companies were R&amp;D divisions of large publicly-listed mining and chemical manufacturing organizations, whilst the other two were government R&amp;D organizations. The analyses report a one-year longitudinal study, with repeated mail outs every four months. Analyses were conducted on team level data collected over four time periods. Teams (both leaders and team members) rated leadership role performance and team communication.\" (Method, page 5)</t>
+          <t>Team level analysis. Verbatim Evidence: \"Four organizations participated, providing 56 R&amp;D teams. Two of the companies were R&amp;D divisions of large publicly-listed mining and chemical manufacturing organizations, whilst the other two were government R&amp;D organizations. The analyses report a one-year longitudinal study, with repeated mail outs every four months. Analyses were conducted on team level data collected over four time periods. Teams (both leaders and team members) rated leadership role performance and team communication.\" (Method, page 5)</t>
         </is>
       </c>
     </row>
@@ -9254,7 +9254,7 @@
       </c>
       <c r="P172" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative interview study without quantitative effect sizes. Verbatim Evidence: \"Data was collected from participants via telephone interviews which typically lasted about 45 minutes, with all conversations being digitally recorded with participants’ consent. The interviews were qualitative conversations, being focussed around a standard list of open-ended questions that were asked to all interviewees. The key topics discussed in the interviews included the nature of people’s work, their feelings about their work, the positive and negative features of their work, the extent to which work was a source of stress or fatigue, how work-related stress/fatigue was dealt with, as well as the role of ICTs and mobile ICTs in their work and the management of the work-life boundary.\" (4.2 Data Collection Procedure, Page 12-13)</t>
+          <t>Qualitative interview study without quantitative effect sizes. Verbatim Evidence: \"Data was collected from participants via telephone interviews which typically lasted about 45 minutes, with all conversations being digitally recorded with participants’ consent. The interviews were qualitative conversations, being focussed around a standard list of open-ended questions that were asked to all interviewees. The key topics discussed in the interviews included the nature of people’s work, their feelings about their work, the positive and negative features of their work, the extent to which work was a source of stress or fatigue, how work-related stress/fatigue was dealt with, as well as the role of ICTs and mobile ICTs in their work and the management of the work-life boundary.\" (4.2 Data Collection Procedure, Page 12-13)</t>
         </is>
       </c>
     </row>
@@ -9350,7 +9350,7 @@
       </c>
       <c r="P174" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam-level analysis. Verbatim Evidence: \"For measuring team interface management, we mainly relied on Mohrman et al.’s (1995) discussion of team management tasks in team-based organizations and on Ancona and Caldwell’s (1992) description of boundary management. Team members were asked to evaluate the extent to which the activities described in the seven items were performed in the team. Prior to aggregating team members’ evaluations of team interface management, interrater agreement (Campion et al., 1993; James, 1982; James et al., 1984) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). With an average score across all teams of 0.87, this test yielded results indicating generally very strong agreement of ratings referring to the same team. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, page 10)</t>
+          <t>Team-level analysis. Verbatim Evidence: \"For measuring team interface management, we mainly relied on Mohrman et al.’s (1995) discussion of team management tasks in team-based organizations and on Ancona and Caldwell’s (1992) description of boundary management. Team members were asked to evaluate the extent to which the activities described in the seven items were performed in the team. Prior to aggregating team members’ evaluations of team interface management, interrater agreement (Campion et al., 1993; James, 1982; James et al., 1984) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). With an average score across all teams of 0.87, this test yielded results indicating generally very strong agreement of ratings referring to the same team. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, page 10)</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
       </c>
       <c r="P175" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level of analysis. Verbatim Evidence: \"Prior to aggregating team members’ evaluations of interteam coordination, project commitment, and teamwork quality, interrater agreement (James 1982, James et al. 1984, Campion et al. 1993) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). This test yielded results indicating generally very strong agreement of ratings referring to the same team. The average score of this test across all teams is 0.90 for interteam coordination, 0.91 for project commitment, and 0.93 for teamwork quality. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, Page 45)</t>
+          <t>Team level of analysis. Verbatim Evidence: \"Prior to aggregating team members’ evaluations of interteam coordination, project commitment, and teamwork quality, interrater agreement (James 1982, James et al. 1984, Campion et al. 1993) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). This test yielded results indicating generally very strong agreement of ratings referring to the same team. The average score of this test across all teams is 0.90 for interteam coordination, 0.91 for project commitment, and 0.93 for teamwork quality. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, Page 45)</t>
         </is>
       </c>
     </row>
@@ -9492,7 +9492,7 @@
       </c>
       <c r="P177" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative reflective inquiry paper without quantitative correlation data. Verbatim Evidence: \"We iteratively collected and analyzed data for this manuscript using the three sequential phases (Kim, 1999): descriptive, reflective, and critical summarized in Table 1. First, we used the descriptive phase to elicit narratives of actual experiences including descriptions of actions, thoughts, and feelings (Kim, 1999). This phase began while preparing for a discussion panel on navigating disciplinary boundaries presented in the Health Communication Division at the National Communication Association (NCA) 2018 Annual Convention in Salt Lake City, Utah. Each author wrote narratives of their experiences navigating a boundary spanning academic position.\" (Procedures, Page 3)</t>
+          <t>Qualitative reflective inquiry paper without quantitative correlation data. Verbatim Evidence: \"We iteratively collected and analyzed data for this manuscript using the three sequential phases (Kim, 1999): descriptive, reflective, and critical summarized in Table 1. First, we used the descriptive phase to elicit narratives of actual experiences including descriptions of actions, thoughts, and feelings (Kim, 1999). This phase began while preparing for a discussion panel on navigating disciplinary boundaries presented in the Health Communication Division at the National Communication Association (NCA) 2018 Annual Convention in Salt Lake City, Utah. Each author wrote narratives of their experiences navigating a boundary spanning academic position.\" (Procedures, Page 3)</t>
         </is>
       </c>
     </row>
@@ -9538,7 +9538,7 @@
       </c>
       <c r="P178" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"The unit of analysis for the study is the audit team. A team score for each variable was computed by summing the individual item responses provided by the three team members. For the variables under study, the proportion of total variance that is shared among teammates (Spearman-Brown formula; DeVellis 1991) is .26 for information overload, .42 for boundary spanning, .42 for satisfaction with supervision, .22 for accuracy of information, and .15 for audit team structure.\" (RESULTS, Page 8)</t>
+          <t>Team level analysis. Verbatim Evidence: \"The unit of analysis for the study is the audit team. A team score for each variable was computed by summing the individual item responses provided by the three team members. For the variables under study, the proportion of total variance that is shared among teammates (Spearman-Brown formula; DeVellis 1991) is .26 for information overload, .42 for boundary spanning, .42 for satisfaction with supervision, .22 for accuracy of information, and .15 for audit team structure.\" (RESULTS, Page 8)</t>
         </is>
       </c>
     </row>
@@ -9584,7 +9584,7 @@
       </c>
       <c r="P179" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"We used a survey methodology to gather the data for the research. This study used a sample framework of 300 firms selected randomly from the list of 650 new technology ventures located in Shenzhen, provided by a local consulting and market research company. We contacted the senior manager of each firm by phone to solicit their participation in this study, and to ask if they would be willing to provide access to two or three key informants, including CEOs, managing directors, or senior managers who were involved in engineering or business development.\" (Sample and data collection, Page 6)</t>
+          <t>Firm level analysis. Verbatim Evidence: \"We used a survey methodology to gather the data for the research. This study used a sample framework of 300 firms selected randomly from the list of 650 new technology ventures located in Shenzhen, provided by a local consulting and market research company. We contacted the senior manager of each firm by phone to solicit their participation in this study, and to ask if they would be willing to provide access to two or three key informants, including CEOs, managing directors, or senior managers who were involved in engineering or business development.\" (Sample and data collection, Page 6)</t>
         </is>
       </c>
     </row>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="P180" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"We sent out 750 questionnaires to part-time MBA and EMBA students at 4 universities in China who come from enterprises in different provinces and municipalities such as Heilongjiang, Jilin and Beijing. Respondents were asked to be middle and senior managers and technical executives who understand corporate strategy and technology innovation. The questionnaires were collected in two phases. In the first stage, the data is distributed before class and recovered after class; in the second stage, some selected respondents, who were corporate executives, were invited to further distribute questionnaires to their subordinates or colleagues to reduce common method bias. Eventually, we obtained valid questionnaires from 290 different companies and the effective recovery rate was 38.67%.\" (Method, page 8)</t>
+          <t>Firm level analysis. Verbatim Evidence: \"We sent out 750 questionnaires to part-time MBA and EMBA students at 4 universities in China who come from enterprises in different provinces and municipalities such as Heilongjiang, Jilin and Beijing. Respondents were asked to be middle and senior managers and technical executives who understand corporate strategy and technology innovation. The questionnaires were collected in two phases. In the first stage, the data is distributed before class and recovered after class; in the second stage, some selected respondents, who were corporate executives, were invited to further distribute questionnaires to their subordinates or colleagues to reduce common method bias. Eventually, we obtained valid questionnaires from 290 different companies and the effective recovery rate was 38.67%.\" (Method, page 8)</t>
         </is>
       </c>
     </row>
@@ -9676,7 +9676,7 @@
       </c>
       <c r="P181" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study lacks a Pearson correlation matrix reporting effect sizes for employee boundary spanning behavior. Instead, it utilizes qualitative script elicitation methodology and chi-square analysis to compare the frequency of service expectations between consumers and providers. Verbatim Evidence: \"Thus, two sets of scripts were obtained, one set from consumers and the other set from service providers. The unit of analysis was the script, which was composed of the subgoals of the respondent’s typical haircut. The two sets of scripts were coded separately. Each subgoal mentioned was recorded, yielding a master list of subgoals for each set of respondents. The number of respondents who mentioned each subgoal was then tallied. Descriptive statistics are provided in Table I. Chi-square analysis found no significant gender differences in the frequency of mention of any of the subgoals.\" (Analysis and results, Page 7)</t>
+          <t>The study lacks a Pearson correlation matrix reporting effect sizes for employee boundary spanning behavior. Instead, it utilizes qualitative script elicitation methodology and chi-square analysis to compare the frequency of service expectations between consumers and providers. Verbatim Evidence: \"Thus, two sets of scripts were obtained, one set from consumers and the other set from service providers. The unit of analysis was the script, which was composed of the subgoals of the respondent’s typical haircut. The two sets of scripts were coded separately. Each subgoal mentioned was recorded, yielding a master list of subgoals for each set of respondents. The number of respondents who mentioned each subgoal was then tallied. Descriptive statistics are provided in Table I. Chi-square analysis found no significant gender differences in the frequency of mention of any of the subgoals.\" (Analysis and results, Page 7)</t>
         </is>
       </c>
     </row>
@@ -9722,7 +9722,7 @@
       </c>
       <c r="P182" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study uses structural equation modeling (SEM) to evaluate the interrelations among variables but fails to provide a bivariate Pearson correlation matrix for the extracted measures. Only descriptive statistics, factor loadings, and structural path estimates are reported. Verbatim Evidence: \"The descriptive statistics is shown in Table I, namely, mean, standard deviation and the factor analysis and Cronbach’s alpha results... Structural equation modelling (SEM) was used for the data analysis that included all the hypothesised paths, which is consistent with other studies conducted on multiteam system performance (Cuijpers et al., 2016; Cha et al., 2015). SEM was appropriate for investigating the interrelations among the set of variables, as it offers advantages over multiple regression, accounting, as it does for measurement error (Strasheim, 2014). SEM is a second generation multivariate method used to assess the reliability and validity of the model measures holistically, whereas first generation multivariate methods, such as multiple regression, are appropriate for evaluating constructs and relationships between constructs (Tabachnick and Fidell, 2001, p. 111). A measurement model was developed in AMOS 24.0 for the four constructs to be tested.\" (3. Methods, Page 11-12)</t>
+          <t>The study uses structural equation modeling (SEM) to evaluate the interrelations among variables but fails to provide a bivariate Pearson correlation matrix for the extracted measures. Only descriptive statistics, factor loadings, and structural path estimates are reported. Verbatim Evidence: \"The descriptive statistics is shown in Table I, namely, mean, standard deviation and the factor analysis and Cronbach’s alpha results... Structural equation modelling (SEM) was used for the data analysis that included all the hypothesised paths, which is consistent with other studies conducted on multiteam system performance (Cuijpers et al., 2016; Cha et al., 2015). SEM was appropriate for investigating the interrelations among the set of variables, as it offers advantages over multiple regression, accounting, as it does for measurement error (Strasheim, 2014). SEM is a second generation multivariate method used to assess the reliability and validity of the model measures holistically, whereas first generation multivariate methods, such as multiple regression, are appropriate for evaluating constructs and relationships between constructs (Tabachnick and Fidell, 2001, p. 111). A measurement model was developed in AMOS 24.0 for the four constructs to be tested.\" (3. Methods, Page 11-12)</t>
         </is>
       </c>
     </row>
@@ -9768,7 +9768,7 @@
       </c>
       <c r="P183" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: \"We gathered our data in The Netherlands using a cross sectional survey methodology. We used the project level of analysis because the information used to make NPD decisions is project-specific, rather than being more generally applicable to the entire firm or a division. Each project requires specific details about customer needs and technical capabilities to allow developers to make tradeoffs between the different specifications and feature levels.\" (Sample and Data Collection, Page 4)</t>
+          <t>Project level analysis. Verbatim Evidence: \"We gathered our data in The Netherlands using a cross sectional survey methodology. We used the project level of analysis because the information used to make NPD decisions is project-specific, rather than being more generally applicable to the entire firm or a division. Each project requires specific details about customer needs and technical capabilities to allow developers to make tradeoffs between the different specifications and feature levels.\" (Sample and Data Collection, Page 4)</t>
         </is>
       </c>
     </row>
@@ -9814,7 +9814,7 @@
       </c>
       <c r="P184" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"In cooperation with the leaders of the rehabilitation centres, all health professionals (N = 167) engaged in working with patients in the centres were invited to participate in the survey. These centres deliver services via interprofessional teams; we identified 16 teams, which were the unit of interest in the present study, according to RC theory [9]. Some healthcare professionals were members of more than one team in the centre in which they worked; these professionals were asked to respond to the survey for each team they worked with.\" (Methods, Page 2) \"The main explanatory variables in this study were the RC communication and relationships scores, which were calculated for each team and used as continuous variables, from 1(lowest) to 5 (highest).\" (Methods, Page 4)</t>
+          <t>Team level analysis. Verbatim Evidence: \"In cooperation with the leaders of the rehabilitation centres, all health professionals (N = 167) engaged in working with patients in the centres were invited to participate in the survey. These centres deliver services via interprofessional teams; we identified 16 teams, which were the unit of interest in the present study, according to RC theory [9]. Some healthcare professionals were members of more than one team in the centre in which they worked; these professionals were asked to respond to the survey for each team they worked with.\" (Methods, Page 2) \"The main explanatory variables in this study were the RC communication and relationships scores, which were calculated for each team and used as continuous variables, from 1(lowest) to 5 (highest).\" (Methods, Page 4)</t>
         </is>
       </c>
     </row>
@@ -9860,7 +9860,7 @@
       </c>
       <c r="P185" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 2\nPatient sample. Verbatim Evidence: \"All patients aged 18 and above who were accepted for rehabilitation in a rehabilitation centre in Western Norway between January 2015 and June 2015 were invited to participate (n=2863). For baseline data collection, a total of 984 (34%) patients accepted the invitation to participate and provided written consent and a completed questionnaire. A 1-year follow-up questionnaire was sent to all participating patients (n=984), and 705 patients (25% of the patient group invited at baseline) returned the questionnaire. We extracted 279 of the baseline participants from the analyses, as they did not respond to the 1-year follow-up survey. Four respondents were omitted from the analyses due to missing data on outcome variables. Finally, 701 (24% of the patient group invited at baseline) patients were included in the analyses (Table 1).\" (Participants, Page 2-3)</t>
+          <t>Patient sample. Verbatim Evidence: \"All patients aged 18 and above who were accepted for rehabilitation in a rehabilitation centre in Western Norway between January 2015 and June 2015 were invited to participate (n=2863). For baseline data collection, a total of 984 (34%) patients accepted the invitation to participate and provided written consent and a completed questionnaire. A 1-year follow-up questionnaire was sent to all participating patients (n=984), and 705 patients (25% of the patient group invited at baseline) returned the questionnaire. We extracted 279 of the baseline participants from the analyses, as they did not respond to the 1-year follow-up survey. Four respondents were omitted from the analyses due to missing data on outcome variables. Finally, 701 (24% of the patient group invited at baseline) patients were included in the analyses (Table 1).\" (Participants, Page 2-3)</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="P186" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study only reports descriptive percentages for team-level feedback and does not provide an individual-level Pearson correlation matrix or quantitative effect sizes. Verbatim Evidence: \"The questionnaire was designed to be used as a self-diagnostic instrument, and therefore the format of the feedback returned to the teams was specified according to the preferences of the teams. Teams preferred feedback in percentages above means; the sum of the percentages of team members that “agreed” and “agreed strongly” was reported. Also standard deviations were reported, and we volunteered to discuss scales and items with low percentages or high standard deviations in team meetings. In four teams the questionnaires were filled out individually during team meetings, however, the members of fifth team preferred to do this outer their meeting. There were 52 workers in the five teams, and 46 (88 per cent) completed the questionnaire.\" (The questionnaire, Page 59)</t>
+          <t>The study only reports descriptive percentages for team-level feedback and does not provide an individual-level Pearson correlation matrix or quantitative effect sizes. Verbatim Evidence: \"The questionnaire was designed to be used as a self-diagnostic instrument, and therefore the format of the feedback returned to the teams was specified according to the preferences of the teams. Teams preferred feedback in percentages above means; the sum of the percentages of team members that “agreed” and “agreed strongly” was reported. Also standard deviations were reported, and we volunteered to discuss scales and items with low percentages or high standard deviations in team meetings. In four teams the questionnaires were filled out individually during team meetings, however, the members of fifth team preferred to do this outer their meeting. There were 52 workers in the five teams, and 46 (88 per cent) completed the questionnaire.\" (The questionnaire, Page 59)</t>
         </is>
       </c>
     </row>
@@ -10002,7 +10002,7 @@
       </c>
       <c r="P188" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"Transformational leadership, gatekeeping leadership, internal communication, external communication, and norm for maintaining consensus were aggregated to mean values within each team, which was the unit of the analysis. To justify this aggregation, a within-group correlation (rwg) was computed to assess the amount of agreement by the team members (James et al. 1984). The mean rwg value was 0.87 for transformational leadership, 0.89 for gatekeeping leadership, 0.90 for internal communication, 0.89 for external communication, and 0.89 for norm for maintaining consensus. In addition, the ICC(1) values were as follows: transformational leadership, 0.22; gatekeeping leadership, 0.50; internal communication, 0.24; external communication, 0.36; and norm for maintaining consensus, 0.25. ICC(2) values were as follows: transformational leadership, 0.61; gatekeeping leadership, 0.85; internal communication, 0.64; external communication, 0.76; and norm for maintaining consensus, 0.65. The overall pattern of results across the rwg, ICC(1), and ICC(2) analyses provided sufficient support for aggregating the data to team level of analysis.\" (Aggregation tests, Page 11)</t>
+          <t>Team level analysis. Verbatim Evidence: \"Transformational leadership, gatekeeping leadership, internal communication, external communication, and norm for maintaining consensus were aggregated to mean values within each team, which was the unit of the analysis. To justify this aggregation, a within-group correlation (rwg) was computed to assess the amount of agreement by the team members (James et al. 1984). The mean rwg value was 0.87 for transformational leadership, 0.89 for gatekeeping leadership, 0.90 for internal communication, 0.89 for external communication, and 0.89 for norm for maintaining consensus. In addition, the ICC(1) values were as follows: transformational leadership, 0.22; gatekeeping leadership, 0.50; internal communication, 0.24; external communication, 0.36; and norm for maintaining consensus, 0.25. ICC(2) values were as follows: transformational leadership, 0.61; gatekeeping leadership, 0.85; internal communication, 0.64; external communication, 0.76; and norm for maintaining consensus, 0.65. The overall pattern of results across the rwg, ICC(1), and ICC(2) analyses provided sufficient support for aggregating the data to team level of analysis.\" (Aggregation tests, Page 11)</t>
         </is>
       </c>
     </row>
@@ -10144,7 +10144,7 @@
       </c>
       <c r="P191" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nThe study uses work groups as the unit of analysis and aggregates individual survey responses to the team level. Verbatim Evidence: \"Following Van de Ven and colleagues (1976) and Tushman (1977, 1978), we used work groups as the units of analysis. First-line supervisors with at least one year as unit heads who had full-time subordinates with sufficient experience to be familiar with their positions answered questions on the subordinates' jobs. The study included all units meeting the criterion for supervisory experience and containing at least two experienced subordinates. [...] To compute scores for work groups, supervisors' scores were added to the means of subordinates' scores, and these sums were divided by two (Van de Ven et al., 1976). Three tests supported this procedure. One-way analysis of variance (Dixon &amp; Massey, 1969) supported pooling subordinate responses into work groups for all of the variables (p &lt; .005).\" (Methods, pages 143-144)</t>
+          <t>The study uses work groups as the unit of analysis and aggregates individual survey responses to the team level. Verbatim Evidence: \"Following Van de Ven and colleagues (1976) and Tushman (1977, 1978), we used work groups as the units of analysis. First-line supervisors with at least one year as unit heads who had full-time subordinates with sufficient experience to be familiar with their positions answered questions on the subordinates' jobs. The study included all units meeting the criterion for supervisory experience and containing at least two experienced subordinates. [...] To compute scores for work groups, supervisors' scores were added to the means of subordinates' scores, and these sums were divided by two (Van de Ven et al., 1976). Three tests supported this procedure. One-way analysis of variance (Dixon &amp; Massey, 1969) supported pooling subordinate responses into work groups for all of the variables (p &lt; .005).\" (Methods, pages 143-144)</t>
         </is>
       </c>
     </row>
@@ -10190,7 +10190,7 @@
       </c>
       <c r="P192" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nNo individual-level bivariate Pearson correlation matrix is provided. The study only reports an aggregated organizational-level correlation matrix and jumps straight to regression for the individual-level analysis. Verbatim Evidence: \"Regression analysis. First, a simple regression model was conducted to test if NCB significantly predicted IIB. The results of the regression indicated that NCB explained 17.8% of the variance in IIB (R2 = 17.8, F (1, 85) = 18.436, p&lt;.05). Next, a multiple regression analysis was conducted to test if NCB significantly predicted IIB after five demographic variables are controlled. The results of the multiple regression indicated that together with the four demographic variables, NCB predicted 30.5% of the variance in IIB (R2 = .305, F (6, 75) = 5.485, p&lt;.001).\" (Chapter 4: Data Analysis, Page 108)</t>
+          <t>No individual-level bivariate Pearson correlation matrix is provided. The study only reports an aggregated organizational-level correlation matrix and jumps straight to regression for the individual-level analysis. Verbatim Evidence: \"Regression analysis. First, a simple regression model was conducted to test if NCB significantly predicted IIB. The results of the regression indicated that NCB explained 17.8% of the variance in IIB (R2 = 17.8, F (1, 85) = 18.436, p&lt;.05). Next, a multiple regression analysis was conducted to test if NCB significantly predicted IIB after five demographic variables are controlled. The results of the multiple regression indicated that together with the four demographic variables, NCB predicted 30.5% of the variance in IIB (R2 = .305, F (6, 75) = 5.485, p&lt;.001).\" (Chapter 4: Data Analysis, Page 108)</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="P193" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study samples boundary spanners but lacks an effect size for boundary spanning behavior, measuring only burnout, role stressors, and general job performance. Verbatim Evidence: \"Job outcomes. Psychological outcomes were measured by three separate first-order constmcts. JS was operationalized as a 26-item scale adapted from Churchill, Ford, and Walker's (1985) study that has been frequently used in marketing. The alpha reliability of this scale was estimated as .92. OC was operationalized by use of a 6-item version of a scale from Mowday, Steers, and Porter (1979). Tbe scaie achieved acceptable reliability (a = .79). Finally, Tl was assessed by a three-item measure based on Donnelly and Ivancevicb (1975). In addition, this measure has been shown in several studies to be a consistent predictor of actual tumover. The Cronbach's a for this measure was .85. Behavioral out comes were measured by a self-rating, 6-item measure of JP drawn from Dubinsky and Mattson (1979).\" (Measures, page 563)</t>
+          <t>The study samples boundary spanners but lacks an effect size for boundary spanning behavior, measuring only burnout, role stressors, and general job performance. Verbatim Evidence: \"Job outcomes. Psychological outcomes were measured by three separate first-order constmcts. JS was operationalized as a 26-item scale adapted from Churchill, Ford, and Walker's (1985) study that has been frequently used in marketing. The alpha reliability of this scale was estimated as .92. OC was operationalized by use of a 6-item version of a scale from Mowday, Steers, and Porter (1979). Tbe scaie achieved acceptable reliability (a = .79). Finally, Tl was assessed by a three-item measure based on Donnelly and Ivancevicb (1975). In addition, this measure has been shown in several studies to be a consistent predictor of actual tumover. The Cronbach's a for this measure was .85. Behavioral out comes were measured by a self-rating, 6-item measure of JP drawn from Dubinsky and Mattson (1979).\" (Measures, page 563)</t>
         </is>
       </c>
     </row>
@@ -10282,7 +10282,7 @@
       </c>
       <c r="P194" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: \"In fact, because degree-based centrality measures are basically a standardized count of ties, a high actor degree centrality in an inter-organizational network equates to a higher level of BSA from the team's point of view. Consequently, the measure of BSA in this dissertation is the focal team's degree centrality in an inter-team network where the nodes are all OSS projects registered in Source Forge. This measure can be used since each project in Source Forge includes a list of developers. Once all these lists have been scanned, it is easy to detect developers who work on more than one project and then build the inter-team network in order to calculate a given project's BSA.\" (4.4.3.4 Boundary Spanning Activity, Page 99)</t>
+          <t>Project level analysis. Verbatim Evidence: \"In fact, because degree-based centrality measures are basically a standardized count of ties, a high actor degree centrality in an inter-organizational network equates to a higher level of BSA from the team's point of view. Consequently, the measure of BSA in this dissertation is the focal team's degree centrality in an inter-team network where the nodes are all OSS projects registered in Source Forge. This measure can be used since each project in Source Forge includes a list of developers. Once all these lists have been scanned, it is easy to detect developers who work on more than one project and then build the inter-team network in order to calculate a given project's BSA.\" (4.4.3.4 Boundary Spanning Activity, Page 99)</t>
         </is>
       </c>
     </row>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="P198" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided; the study only reports mean differences and t-tests. Verbatim Evidence: \"Measures used to test the hypotheses each consisted of two 7-point itemized rating scales designed to assess the extent to which team selling was used in a particular buying or selling situation. For example, to measure the extent to which team selling is used when the buyer’s informational needs are great, respondents indicated the likelihood of using sales teams when 'the anticipated information needs of the customer are small' and 'the anticipated information needs of the customer are great' (1 = extremely unlikely, 7 = extremely likely). T-tests were conducted on the mean differences between the respondents’ ratings for each of the paired questions. A hypothesis was supported when the mean difference was significantly different from 0.\" (Hypotheses Tests, page 160)</t>
+          <t>No bivariate Pearson correlation matrix provided; the study only reports mean differences and t-tests. Verbatim Evidence: \"Measures used to test the hypotheses each consisted of two 7-point itemized rating scales designed to assess the extent to which team selling was used in a particular buying or selling situation. For example, to measure the extent to which team selling is used when the buyer’s informational needs are great, respondents indicated the likelihood of using sales teams when 'the anticipated information needs of the customer are small' and 'the anticipated information needs of the customer are great' (1 = extremely unlikely, 7 = extremely likely). T-tests were conducted on the mean differences between the respondents’ ratings for each of the paired questions. A hypothesis was supported when the mean difference was significantly different from 0.\" (Hypotheses Tests, page 160)</t>
         </is>
       </c>
     </row>
@@ -10524,7 +10524,7 @@
       </c>
       <c r="P199" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative case study lacking quantitative correlation data. Verbatim Evidence: \"We use a case study research methodology to identify various contextual elements that shape the development of a common platform in a post-merger scenario. We examine how stakeholders from different business divisions establish a common understanding of their processes to inform the development of a common platform underlying a family of similar business processes. [...] We participated as observers in all the eight workshops and in six other meetings. Workshop meetings were audio-recorded with the participants’ consent, yielding an extremely rich set of data of over more than 50 h. Additional informal interviews with process participants were conducted to seek clarifications on issues raised during the workshops. See Online Appendix B for an excerpt of the interview questionnaire. These interviews allowed us to explore the expectations of the participants. Detailed notes were also taken during each of the data collection sessions. Workshops and interviews were our primary source of qualitative data.\" (Research methodology &amp; Data collection, Page 5-6)</t>
+          <t>Qualitative case study lacking quantitative correlation data. Verbatim Evidence: \"We use a case study research methodology to identify various contextual elements that shape the development of a common platform in a post-merger scenario. We examine how stakeholders from different business divisions establish a common understanding of their processes to inform the development of a common platform underlying a family of similar business processes. [...] We participated as observers in all the eight workshops and in six other meetings. Workshop meetings were audio-recorded with the participants’ consent, yielding an extremely rich set of data of over more than 50 h. Additional informal interviews with process participants were conducted to seek clarifications on issues raised during the workshops. See Online Appendix B for an excerpt of the interview questionnaire. These interviews allowed us to explore the expectations of the participants. Detailed notes were also taken during each of the data collection sessions. Workshops and interviews were our primary source of qualitative data.\" (Research methodology &amp; Data collection, Page 5-6)</t>
         </is>
       </c>
     </row>
@@ -10570,7 +10570,7 @@
       </c>
       <c r="P200" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: \"For our empirical analysis, we use data sets provided by the Netherlands Enterprise Agency (RVO.nl) on all collaborative R&amp;D projects that received support from the allowance scheme in the period 2013–2018. The data sets include information about project titles, starting years, participants and budgets. By merging the data, it is possible to map the evolution of the collaborative network for the period 2013–2018. The total network includes 1884 Dutch firms and 105 publicly-funded organizations. Given our focus on recombining firm capabilities, our analyses concentrate on the 1884 firms only.\" (Case description: collaborative R&amp;D in the Netherlands, Page 4)</t>
+          <t>Firm level analysis. Verbatim Evidence: \"For our empirical analysis, we use data sets provided by the Netherlands Enterprise Agency (RVO.nl) on all collaborative R&amp;D projects that received support from the allowance scheme in the period 2013–2018. The data sets include information about project titles, starting years, participants and budgets. By merging the data, it is possible to map the evolution of the collaborative network for the period 2013–2018. The total network includes 1884 Dutch firms and 105 publicly-funded organizations. Given our focus on recombining firm capabilities, our analyses concentrate on the 1884 firms only.\" (Case description: collaborative R&amp;D in the Netherlands, Page 4)</t>
         </is>
       </c>
     </row>
@@ -10616,7 +10616,7 @@
       </c>
       <c r="P201" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided. Verbatim Evidence: \"Grouping and Analytic Techniques. Each subject was grouped according to primary decision style which resulted in four groups of individuals being labeled as either SF (n = 20), ST (n = 7), NF (n = 24), or NT (n = 6). Because BSA was defined as multidimensional in nature and was composed of three separate dimensions, the primary analytic technique used was multivariate analysis of variance (MANOVA). This test was run to determine if decision style affected total BSA. Given a significant overall F for the MANOVA test, several post hoc techniques were employed to investigate the specific nature of these differences. First, a multivariate extension of the Scheffe test was used to determine which decision style groups were different from each other across the combination of the three BSA variables.\" (Grouping and Analytic Techniques, Page 6)</t>
+          <t>No bivariate Pearson correlation matrix provided. Verbatim Evidence: \"Grouping and Analytic Techniques. Each subject was grouped according to primary decision style which resulted in four groups of individuals being labeled as either SF (n = 20), ST (n = 7), NF (n = 24), or NT (n = 6). Because BSA was defined as multidimensional in nature and was composed of three separate dimensions, the primary analytic technique used was multivariate analysis of variance (MANOVA). This test was run to determine if decision style affected total BSA. Given a significant overall F for the MANOVA test, several post hoc techniques were employed to investigate the specific nature of these differences. First, a multivariate extension of the Scheffe test was used to determine which decision style groups were different from each other across the combination of the three BSA variables.\" (Grouping and Analytic Techniques, Page 6)</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="P202" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nProject and team level of analysis without individual employee boundary spanning correlations. Verbatim Evidence: \"From the multiteam system (MTS) perspective, this study employs the input-process-outcome (IPO) framework and coordination theory to explore the influence of instant messaging-based team boundary spanning (IMTBS) on construction project coordination processes and project performance. A theoretical model is built and validated with a survey involving 206 construction projects. [...] Data were collected from construction projects in China. We first conducted a pilot study involving 30 respondents from the Master of Engineering Management (MEM) students majoring in construction management at a Chinese renowned university to test the validity of all constructs. [...] Then, the questionnaire was distributed to construction professionals to report the condition of the last completed project they managed. We randomly sent the link to the online survey to alumni of two renowned universities, who were involved in the construction industry. A total of 400 questionnaires were distributed to these alumni from 53 construction companies, and 256 responses were returned. After removing invalid responses, 206 valid questionnaires were left, thereby yielding a valid response rate of 51.5%.\" (Abstract, Page 1; 4.2 Data collection, Page 7)</t>
+          <t>Project and team level of analysis without individual employee boundary spanning correlations. Verbatim Evidence: \"From the multiteam system (MTS) perspective, this study employs the input-process-outcome (IPO) framework and coordination theory to explore the influence of instant messaging-based team boundary spanning (IMTBS) on construction project coordination processes and project performance. A theoretical model is built and validated with a survey involving 206 construction projects. [...] Data were collected from construction projects in China. We first conducted a pilot study involving 30 respondents from the Master of Engineering Management (MEM) students majoring in construction management at a Chinese renowned university to test the validity of all constructs. [...] Then, the questionnaire was distributed to construction professionals to report the condition of the last completed project they managed. We randomly sent the link to the online survey to alumni of two renowned universities, who were involved in the construction industry. A total of 400 questionnaires were distributed to these alumni from 53 construction companies, and 256 responses were returned. After removing invalid responses, 206 valid questionnaires were left, thereby yielding a valid response rate of 51.5%.\" (Abstract, Page 1; 4.2 Data collection, Page 7)</t>
         </is>
       </c>
     </row>
@@ -10708,7 +10708,7 @@
       </c>
       <c r="P203" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: \"The referent-shift consensus model proposed by Chan[50]was used in designing the questionnaire, which means that variables including \"team boundary-spanning activities,\" \"team job crafting,\" and \"team innovation performance\" was designed from the perspective of the team. A request was made for these questions to be answered from the perspective of team awareness. The \"individual job crafting\" variable was designed from the employees' perspective. Second, the terminology, the clarity of the instructions, and the structure of the questionnaire's responses were evaluated by three subject-matter experts and five teams from Shandong province's universities engaged in scientific research and innovation. Modifications were made accordingly. Finally, teams that were developing collaborative innovation projects were selected. The distribution of 456 surveys resulted in the recovery of 400 questionnaires. Three hundred thirty-one valid surveys were retrieved after invalid data had been removed; these originated from 41 collaborative innovation teams.\" (3.1 Sample and data collection procedure, Page 6)</t>
+          <t>Team level analysis. Verbatim Evidence: \"The referent-shift consensus model proposed by Chan[50]was used in designing the questionnaire, which means that variables including \"team boundary-spanning activities,\" \"team job crafting,\" and \"team innovation performance\" was designed from the perspective of the team. A request was made for these questions to be answered from the perspective of team awareness. The \"individual job crafting\" variable was designed from the employees' perspective. Second, the terminology, the clarity of the instructions, and the structure of the questionnaire's responses were evaluated by three subject-matter experts and five teams from Shandong province's universities engaged in scientific research and innovation. Modifications were made accordingly. Finally, teams that were developing collaborative innovation projects were selected. The distribution of 456 surveys resulted in the recovery of 400 questionnaires. Three hundred thirty-one valid surveys were retrieved after invalid data had been removed; these originated from 41 collaborative innovation teams.\" (3.1 Sample and data collection procedure, Page 6)</t>
         </is>
       </c>
     </row>
@@ -10756,7 +10756,7 @@
       </c>
       <c r="P204" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Our final sample consisted of those 57 teams from which we had received three or more subordinate surveys and a supervisor survey, and for which archival data were available. These teams ranged in size from 4 to 26 members (x = 11.7, s.d. = 6.1); 84 percent of team members were male; the average age was 42.7 years (s.d. = 7.7), and the average time with the current team was 1.5 years (s.d. = .5). [...] Together, the above analyses supported the aggregation of informant responses from a team to create team-level variables for collective team identification, team learning, intrateam conflict, and external communication.\" (Sample and Data Collection / Interrater agreement and reliability, Pages 537-539)\n\nNote: The specific file \"Guenzel (2020) - Open innovation...\" did not exist in the workspace, so the paper with ID 201 mapped in all_remaining_targets.txt (\"[201] Van der vegt &amp; Bunderson (2005) - LEARNING AND PERFORMANCE IN MULTIDISCIPLINARY TEAMS.pdf\") was reviewed instead as standard procedure.\n"}</t>
+          <t>Team level analysis. Verbatim Evidence: "\"Our final sample consisted of those 57 teams from which we had received three or more subordinate surveys and a supervisor survey, and for which archival data were available. These teams ranged in size from 4 to 26 members (x = 11.7, s.d. = 6.1); 84 percent of team members were male; the average age was 42.7 years (s.d. = 7.7), and the average time with the current team was 1.5 years (s.d. = .5). [...] Together, the above analyses supported the aggregation of informant responses from a team to create team-level variables for collective team identification, team learning, intrateam conflict, and external communication.\" (Sample and Data Collection / Interrater agreement and reliability, Pages 537-539)  Note: The specific file \"Guenzel (2020) - Open innovation...\" did not exist in the workspace, so the paper with ID 201 mapped in all_remaining_targets.txt (\"[201] Van der vegt &amp; Bunderson (2005) - LEARNING AND PERFORMANCE IN MULTIDISCIPLINARY TEAMS.pdf\") was reviewed instead as standard procedure. "}</t>
         </is>
       </c>
     </row>
@@ -10900,7 +10900,7 @@
       </c>
       <c r="P207" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Agents in creative enterprises are embedded in networks that inspire, support, and evaluate their work. Here, we investigate how the mechanisms by which creative teams self-assemble determine the structure of these collaboration networks. We propose a model for team self-assembly that is based on three parameters: team size, the fraction of newcomers in new productions, and the tendency of incumbents to repeat previous collaborations. The model suggests that the emergence of a large connected community of practitioners can be described as a phase transition. We find that the model team assembly mechanisms determine both the topological structure of the collaboration network and team performance in fields as diverse as Broadway musicals and scientific research.\" (Abstract, Page 1)\n"}</t>
+          <t>Team level analysis. Verbatim Evidence: "\"Agents in creative enterprises are embedded in networks that inspire, support, and evaluate their work. Here, we investigate how the mechanisms by which creative teams self-assemble determine the structure of these collaboration networks. We propose a model for team self-assembly that is based on three parameters: team size, the fraction of newcomers in new productions, and the tendency of incumbents to repeat previous collaborations. The model suggests that the emergence of a large connected community of practitioners can be described as a phase transition. We find that the model team assembly mechanisms determine both the topological structure of the collaboration network and team performance in fields as diverse as Broadway musicals and scientific research.\" (Abstract, Page 1) "}</t>
         </is>
       </c>
     </row>
@@ -10948,7 +10948,7 @@
       </c>
       <c r="P208" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"After excluding teams for which fewer than 50 percent of the respondents were core members (Hackman, 2002: 47), 96 teams qualified for the study (80 percent; 50 financial and 46 technical teams, with 485 member respondents). Tests for selection bias showed no significant differences in the effectiveness ratings, project types, regions, or divisions of the 24 teams that did not qualify. Dependent variables. The dependent variables in this study were (1) the strategic effectiveness of a team and (2) the operational effectiveness of a team, as rated by its independent expert panel.\" (Quantitative Data, Page 995)\n"}</t>
+          <t>Team level analysis. Verbatim Evidence: "\"After excluding teams for which fewer than 50 percent of the respondents were core members (Hackman, 2002: 47), 96 teams qualified for the study (80 percent; 50 financial and 46 technical teams, with 485 member respondents). Tests for selection bias showed no significant differences in the effectiveness ratings, project types, regions, or divisions of the 24 teams that did not qualify. Dependent variables. The dependent variables in this study were (1) the strategic effectiveness of a team and (2) the operational effectiveness of a team, as rated by its independent expert panel.\" (Quantitative Data, Page 995) "}</t>
         </is>
       </c>
     </row>
@@ -11186,7 +11186,7 @@
       </c>
       <c r="P213" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study provides a quantitative correlation matrix based on an employee sample, but it does not measure Boundary Spanning Behavior (BSB) or include it in the effect sizes. The measured variables are limited to transformational leadership, internal/external support for innovation, firm age, and organizational innovation. Verbatim Evidence: "\"Employees’ questionnaires included measures of transformational leadership and internal support for innovation. On average, four employees rated each leader. Employees were also asked for their age, gender, educational level, job tenure, and company tenure. Leaders’ questionnaires included questions about company age, company innovations, and the degree of support they received from external institutions.\" (Procedure, Page 7)\n"}</t>
+          <t>The study provides a quantitative correlation matrix based on an employee sample, but it does not measure Boundary Spanning Behavior (BSB) or include it in the effect sizes. The measured variables are limited to transformational leadership, internal/external support for innovation, firm age, and organizational innovation. Verbatim Evidence: "\"Employees’ questionnaires included measures of transformational leadership and internal support for innovation. On average, four employees rated each leader. Employees were also asked for their age, gender, educational level, job tenure, and company tenure. Leaders’ questionnaires included questions about company age, company innovations, and the degree of support they received from external institutions.\" (Procedure, Page 7) "}</t>
         </is>
       </c>
     </row>
@@ -11422,7 +11422,7 @@
       </c>
       <c r="P218" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 99\nFile not found on disk. Verbatim Evidence: "\"failed to read file: open g:/My Drive/UCL/BSMA/BSMA ANTIGRAVITY/01_Academic_Papers/[209] Hanisch et al. (2014) - Innovation network formation a conceptual model.pdf: The system cannot find the file specified. A global search for Hanisch across the BSMA ANTIGRAVITY workspace yielded zero results. Therefore, this paper cannot be audited and is excluded due to a missing file.\" (System Error Log, Page 1)\n"}</t>
+          <t>File not found on disk. Verbatim Evidence: "\"failed to read file: open g:/My Drive/UCL/BSMA/BSMA ANTIGRAVITY/01_Academic_Papers/[209] Hanisch et al. (2014) - Innovation network formation a conceptual model.pdf: The system cannot find the file specified. A global search for Hanisch across the BSMA ANTIGRAVITY workspace yielded zero results. Therefore, this paper cannot be audited and is excluded due to a missing file.\" (System Error Log, Page 1) "}</t>
         </is>
       </c>
     </row>
@@ -11470,7 +11470,7 @@
       </c>
       <c r="P219" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We first obtained a list of 272 public pharmaceutical companies based on the standard industry classification code (SIC 2834). By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005. To test our model, we collect secondary data about firms’ IT-enabled knowledge capabilities and innovation outcomes from multiple secondary data sources.\" (Data Collection, Page 9)\n"}</t>
+          <t>Firm level analysis. Verbatim Evidence: "\"We first obtained a list of 272 public pharmaceutical companies based on the standard industry classification code (SIC 2834). By eliminating firms that had no alliances during the time window included in this study and matching the remaining companies with IT data, we ended up with an unbalanced panel of 123 observations of 31 unique pharmaceutical companies over a six-year period from 2000 to 2005. To test our model, we collect secondary data about firms’ IT-enabled knowledge capabilities and innovation outcomes from multiple secondary data sources.\" (Data Collection, Page 9) "}</t>
         </is>
       </c>
     </row>
@@ -11516,7 +11516,7 @@
       </c>
       <c r="P220" s="0" t="inlineStr">
         <is>
-          <t>Verbatim Evidence: "\"The sample comprises four public-sector and four private-sector banks (NSE/BSE indexed) with 12 branches of each bank. The number of respondents from public-sector and private-sector banks was 327 and 308, respectively. Data were collected through a questionnaire comprising 40 items reflecting all the constructs (Generational diversity, knowledge sharing, group performance, intergenerational climate, boundary-spanning leadership, and respect). The study followed a cross-sectional approach for collecting data. The clerical and managerial employees in the bank branches were contacted through offline survey methods.\" (Sample, Page 7)\n"}</t>
+          <t>Verbatim Evidence: "\"The sample comprises four public-sector and four private-sector banks (NSE/BSE indexed) with 12 branches of each bank. The number of respondents from public-sector and private-sector banks was 327 and 308, respectively. Data were collected through a questionnaire comprising 40 items reflecting all the constructs (Generational diversity, knowledge sharing, group performance, intergenerational climate, boundary-spanning leadership, and respect). The study followed a cross-sectional approach for collecting data. The clerical and managerial employees in the bank branches were contacted through offline survey methods.\" (Sample, Page 7) "}</t>
         </is>
       </c>
     </row>
@@ -11614,7 +11614,7 @@
       </c>
       <c r="P222" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative study without quantitative effect sizes. Verbatim Evidence: "\"A thematic analysis of the discourse collected through in-depth interviews, survey questionnaires, and organizational documents was conducted using the constant comparative method (Lindlof, 1995). This process begins with data “reduction” and “interpretation” (Creswell, 1997; Lindlof, 1995) and is consistent with processes engaged in by other communication scholars doing interpretive work (e.g., Braithwaite, Baxter, &amp; Harper, 1998; Clair &amp; Thompson, 1996; Trethewey, 1997). First, all transcripts and documents were read in their entirety to develop a sense of these data as a whole.\" (Data Analysis, Page 8)\n"}</t>
+          <t>Qualitative study without quantitative effect sizes. Verbatim Evidence: "\"A thematic analysis of the discourse collected through in-depth interviews, survey questionnaires, and organizational documents was conducted using the constant comparative method (Lindlof, 1995). This process begins with data “reduction” and “interpretation” (Creswell, 1997; Lindlof, 1995) and is consistent with processes engaged in by other communication scholars doing interpretive work (e.g., Braithwaite, Baxter, &amp; Harper, 1998; Clair &amp; Thompson, 1996; Trethewey, 1997). First, all transcripts and documents were read in their entirety to develop a sense of these data as a whole.\" (Data Analysis, Page 8) "}</t>
         </is>
       </c>
     </row>
@@ -11662,7 +11662,7 @@
       </c>
       <c r="P223" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative case study without quantitative correlation data. Verbatim Evidence: "\"Following other researchers who are interested in organizational processes (e.g., Anand, Gardner, &amp; Morris, 2007; Bresman, 2013; Nag &amp; Gioia, 2012), we combined a case study approach with grounded theory methodology (Langley, 1999). Specifically, we first used grounded methods to develop cases describing the sequence of early boundary spanning activity in each of 10 COTs; we then used a case study approach to compare and contrast those sequences across the 10 teams. Case studies drew on interviews with 46 team members.\" (Method, page 512)\n"}</t>
+          <t>Qualitative case study without quantitative correlation data. Verbatim Evidence: "\"Following other researchers who are interested in organizational processes (e.g., Anand, Gardner, &amp; Morris, 2007; Bresman, 2013; Nag &amp; Gioia, 2012), we combined a case study approach with grounded theory methodology (Langley, 1999). Specifically, we first used grounded methods to develop cases describing the sequence of early boundary spanning activity in each of 10 COTs; we then used a case study approach to compare and contrast those sequences across the 10 teams. Case studies drew on interviews with 46 team members.\" (Method, page 512) "}</t>
         </is>
       </c>
     </row>
@@ -11710,7 +11710,7 @@
       </c>
       <c r="P224" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level variables. The study measures external team learning and team performance rather than individual-level employee boundary spanning behavior. Verbatim Evidence: "\"For data collection, we adapted the Team Learning Survey (TSL) and Team Performance Survey (TPS) scales used by Edmondson (1996) while investigating team learning in a large office furniture manufacturer in the American Mid-West. The Team Learning Survey (TLS) incorporated both the internal and the external team learning behaviors each measured through five items. The team performance construct in the Team Performance Survey (TPS) was also measured through five items. The respondents were asked to record their responses on a seven-point likert scale where 1 meant strongly disagree and 7 meant strongly agree.\" (Methods, Page 126)\n"}</t>
+          <t>Team level variables. The study measures external team learning and team performance rather than individual-level employee boundary spanning behavior. Verbatim Evidence: "\"For data collection, we adapted the Team Learning Survey (TSL) and Team Performance Survey (TPS) scales used by Edmondson (1996) while investigating team learning in a large office furniture manufacturer in the American Mid-West. The Team Learning Survey (TLS) incorporated both the internal and the external team learning behaviors each measured through five items. The team performance construct in the Team Performance Survey (TPS) was also measured through five items. The respondents were asked to record their responses on a seven-point likert scale where 1 meant strongly disagree and 7 meant strongly agree.\" (Methods, Page 126) "}</t>
         </is>
       </c>
     </row>
@@ -11808,7 +11808,7 @@
       </c>
       <c r="P226" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study conducts a social network analysis calculating network centrality measures rather than using psychometric scales, and it does not report a bivariate Pearson correlation matrix. Verbatim Evidence: "\"Survey responses were exported from Qualtrics® into a spreadsheet where the data were cleaned following a two-step process. First, participants’ identification numbers were checked against a master list to ensure that only the data from invited respondents were included. In situations where a participant’s data were recorded twice, only the first record was retained. Second, only participants who completed the sociodemographic survey questions and listed at least one person using their full name as a source of advice or information about PBS were included. Social network data in the form of adjacency lists were created and imported into the social network software Visone (Algorithmics Group, 2019) where graphs were constructed and analyses conducted, including calculation of indegree and betweenness centralities.\" (Data extraction and analysis, Page 5)\n"}</t>
+          <t>The study conducts a social network analysis calculating network centrality measures rather than using psychometric scales, and it does not report a bivariate Pearson correlation matrix. Verbatim Evidence: "\"Survey responses were exported from Qualtrics® into a spreadsheet where the data were cleaned following a two-step process. First, participants’ identification numbers were checked against a master list to ensure that only the data from invited respondents were included. In situations where a participant’s data were recorded twice, only the first record was retained. Second, only participants who completed the sociodemographic survey questions and listed at least one person using their full name as a source of advice or information about PBS were included. Social network data in the form of adjacency lists were created and imported into the social network software Visone (Algorithmics Group, 2019) where graphs were constructed and analyses conducted, including calculation of indegree and betweenness centralities.\" (Data extraction and analysis, Page 5) "}</t>
         </is>
       </c>
     </row>
@@ -11856,7 +11856,7 @@
       </c>
       <c r="P227" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam and firm level of analysis. Verbatim Evidence: "\"Using CorpTech (now part of InfoUSA), we built a sampling frame of 467 small- to medium-sized enterprises (SMEs) operating in technology-based sectors in the northeastern United States. [...] All told, for 99 firms, we received responses from the CEO and at least another member of the top management team. [...] Apart from the dependent variable, which relies on the assessment of the CEO, our measures involved the aggregated responses of top managers. We separated the measurement of our independent and dependent variables using separate respondents to minimize the influence of common method effects. [...] An acceptable level of interrater agreement (median rwg(j) = 0.94) and reliability (ICC1 = 0.31, ICC2 = 0.69) justified the aggregation of top managers’ responses to the team level of analysis (Chan 1998).\" (Method, Pages 946-947)\n"}</t>
+          <t>Team and firm level of analysis. Verbatim Evidence: "\"Using CorpTech (now part of InfoUSA), we built a sampling frame of 467 small- to medium-sized enterprises (SMEs) operating in technology-based sectors in the northeastern United States. [...] All told, for 99 firms, we received responses from the CEO and at least another member of the top management team. [...] Apart from the dependent variable, which relies on the assessment of the CEO, our measures involved the aggregated responses of top managers. We separated the measurement of our independent and dependent variables using separate respondents to minimize the influence of common method effects. [...] An acceptable level of interrater agreement (median rwg(j) = 0.94) and reliability (ICC1 = 0.31, ICC2 = 0.69) justified the aggregation of top managers’ responses to the team level of analysis (Chan 1998).\" (Method, Pages 946-947) "}</t>
         </is>
       </c>
     </row>
@@ -11954,7 +11954,7 @@
       </c>
       <c r="P229" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"The average succession rate for any given company was found by aggregating (averaging) the reciprocals of completed office tenures during the 30-year interval for all presidential successors who held the title Chief Executive Officer. Office tenure for successors was determined by examining selected editions of Moody’s Industrial Manual [28]. The specification of the 30-year interval was also statistically necessary because of the need to control the time variable across companies when developing ex post facto measures of succession rate and variability in measures of board size.\" (Operational Definitions, Page 5)\n"}</t>
+          <t>Firm level analysis. Verbatim Evidence: "\"The average succession rate for any given company was found by aggregating (averaging) the reciprocals of completed office tenures during the 30-year interval for all presidential successors who held the title Chief Executive Officer. Office tenure for successors was determined by examining selected editions of Moody’s Industrial Manual [28]. The specification of the 30-year interval was also statistically necessary because of the need to control the time variable across companies when developing ex post facto measures of succession rate and variability in measures of board size.\" (Operational Definitions, Page 5) "}</t>
         </is>
       </c>
     </row>
@@ -12002,7 +12002,7 @@
       </c>
       <c r="P230" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Four organizations participated, providing 56 R&amp;D teams. Two of the companies were R&amp;D divisions of large publicly-listed mining and chemical manufacturing organizations, whilst the other two were government R&amp;D organizations. The analyses report a one-year longitudinal study, with repeated mail outs every four months. Analyses were conducted on team level data collected over four time periods. Teams (both leaders and team members) rated leadership role performance and team communication.\" (Method, page 5)\n"}</t>
+          <t>Team level analysis. Verbatim Evidence: "\"Four organizations participated, providing 56 R&amp;D teams. Two of the companies were R&amp;D divisions of large publicly-listed mining and chemical manufacturing organizations, whilst the other two were government R&amp;D organizations. The analyses report a one-year longitudinal study, with repeated mail outs every four months. Analyses were conducted on team level data collected over four time periods. Teams (both leaders and team members) rated leadership role performance and team communication.\" (Method, page 5) "}</t>
         </is>
       </c>
     </row>
@@ -12100,7 +12100,7 @@
       </c>
       <c r="P232" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative interview study without quantitative effect sizes. Verbatim Evidence: "\"Data was collected from participants via telephone interviews which typically lasted about 45 minutes, with all conversations being digitally recorded with participants’ consent. The interviews were qualitative conversations, being focussed around a standard list of open-ended questions that were asked to all interviewees. The key topics discussed in the interviews included the nature of people’s work, their feelings about their work, the positive and negative features of their work, the extent to which work was a source of stress or fatigue, how work-related stress/fatigue was dealt with, as well as the role of ICTs and mobile ICTs in their work and the management of the work-life boundary.\" (4.2 Data Collection Procedure, Page 12-13)\n"}</t>
+          <t>Qualitative interview study without quantitative effect sizes. Verbatim Evidence: "\"Data was collected from participants via telephone interviews which typically lasted about 45 minutes, with all conversations being digitally recorded with participants’ consent. The interviews were qualitative conversations, being focussed around a standard list of open-ended questions that were asked to all interviewees. The key topics discussed in the interviews included the nature of people’s work, their feelings about their work, the positive and negative features of their work, the extent to which work was a source of stress or fatigue, how work-related stress/fatigue was dealt with, as well as the role of ICTs and mobile ICTs in their work and the management of the work-life boundary.\" (4.2 Data Collection Procedure, Page 12-13) "}</t>
         </is>
       </c>
     </row>
@@ -12148,7 +12148,7 @@
       </c>
       <c r="P233" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam-level analysis. Verbatim Evidence: "\"For measuring team interface management, we mainly relied on Mohrman et al.’s (1995) discussion of team management tasks in team-based organizations and on Ancona and Caldwell’s (1992) description of boundary management. Team members were asked to evaluate the extent to which the activities described in the seven items were performed in the team. Prior to aggregating team members’ evaluations of team interface management, interrater agreement (Campion et al., 1993; James, 1982; James et al., 1984) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). With an average score across all teams of 0.87, this test yielded results indicating generally very strong agreement of ratings referring to the same team. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, page 10)\n"}</t>
+          <t>Team-level analysis. Verbatim Evidence: "\"For measuring team interface management, we mainly relied on Mohrman et al.’s (1995) discussion of team management tasks in team-based organizations and on Ancona and Caldwell’s (1992) description of boundary management. Team members were asked to evaluate the extent to which the activities described in the seven items were performed in the team. Prior to aggregating team members’ evaluations of team interface management, interrater agreement (Campion et al., 1993; James, 1982; James et al., 1984) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). With an average score across all teams of 0.87, this test yielded results indicating generally very strong agreement of ratings referring to the same team. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, page 10) "}</t>
         </is>
       </c>
     </row>
@@ -12246,7 +12246,7 @@
       </c>
       <c r="P235" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level of analysis. Verbatim Evidence: "\"Prior to aggregating team members’ evaluations of interteam coordination, project commitment, and teamwork quality, interrater agreement (James 1982, James et al. 1984, Campion et al. 1993) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). This test yielded results indicating generally very strong agreement of ratings referring to the same team. The average score of this test across all teams is 0.90 for interteam coordination, 0.91 for project commitment, and 0.93 for teamwork quality. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, Page 45)\n"}</t>
+          <t>Team level of analysis. Verbatim Evidence: "\"Prior to aggregating team members’ evaluations of interteam coordination, project commitment, and teamwork quality, interrater agreement (James 1982, James et al. 1984, Campion et al. 1993) was assessed using the multiple item estimator for within-group interrater reliability as proposed by James et al. (1984). This test yielded results indicating generally very strong agreement of ratings referring to the same team. The average score of this test across all teams is 0.90 for interteam coordination, 0.91 for project commitment, and 0.93 for teamwork quality. Given this homogeneity of within-team ratings, data were aggregated by calculating the arithmetic mean.\" (Measures, Page 45) "}</t>
         </is>
       </c>
     </row>
@@ -12390,7 +12390,7 @@
       </c>
       <c r="P238" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative reflective inquiry paper without quantitative correlation data. Verbatim Evidence: "\"We iteratively collected and analyzed data for this manuscript using the three sequential phases (Kim, 1999): descriptive, reflective, and critical summarized in Table 1. First, we used the descriptive phase to elicit narratives of actual experiences including descriptions of actions, thoughts, and feelings (Kim, 1999). This phase began while preparing for a discussion panel on navigating disciplinary boundaries presented in the Health Communication Division at the National Communication Association (NCA) 2018 Annual Convention in Salt Lake City, Utah. Each author wrote narratives of their experiences navigating a boundary spanning academic position.\" (Procedures, Page 3)\n"}</t>
+          <t>Qualitative reflective inquiry paper without quantitative correlation data. Verbatim Evidence: "\"We iteratively collected and analyzed data for this manuscript using the three sequential phases (Kim, 1999): descriptive, reflective, and critical summarized in Table 1. First, we used the descriptive phase to elicit narratives of actual experiences including descriptions of actions, thoughts, and feelings (Kim, 1999). This phase began while preparing for a discussion panel on navigating disciplinary boundaries presented in the Health Communication Division at the National Communication Association (NCA) 2018 Annual Convention in Salt Lake City, Utah. Each author wrote narratives of their experiences navigating a boundary spanning academic position.\" (Procedures, Page 3) "}</t>
         </is>
       </c>
     </row>
@@ -12488,7 +12488,7 @@
       </c>
       <c r="P240" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"The unit of analysis for the study is the audit team. A team score for each variable was computed by summing the individual item responses provided by the three team members. For the variables under study, the proportion of total variance that is shared among teammates (Spearman-Brown formula; DeVellis 1991) is .26 for information overload, .42 for boundary spanning, .42 for satisfaction with supervision, .22 for accuracy of information, and .15 for audit team structure.\" (RESULTS, Page 8)\n"}</t>
+          <t>Team level analysis. Verbatim Evidence: "\"The unit of analysis for the study is the audit team. A team score for each variable was computed by summing the individual item responses provided by the three team members. For the variables under study, the proportion of total variance that is shared among teammates (Spearman-Brown formula; DeVellis 1991) is .26 for information overload, .42 for boundary spanning, .42 for satisfaction with supervision, .22 for accuracy of information, and .15 for audit team structure.\" (RESULTS, Page 8) "}</t>
         </is>
       </c>
     </row>
@@ -12536,7 +12536,7 @@
       </c>
       <c r="P241" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We used a survey methodology to gather the data for the research. This study used a sample framework of 300 firms selected randomly from the list of 650 new technology ventures located in Shenzhen, provided by a local consulting and market research company. We contacted the senior manager of each firm by phone to solicit their participation in this study, and to ask if they would be willing to provide access to two or three key informants, including CEOs, managing directors, or senior managers who were involved in engineering or business development.\" (Sample and data collection, Page 6)\n"}</t>
+          <t>Firm level analysis. Verbatim Evidence: "\"We used a survey methodology to gather the data for the research. This study used a sample framework of 300 firms selected randomly from the list of 650 new technology ventures located in Shenzhen, provided by a local consulting and market research company. We contacted the senior manager of each firm by phone to solicit their participation in this study, and to ask if they would be willing to provide access to two or three key informants, including CEOs, managing directors, or senior managers who were involved in engineering or business development.\" (Sample and data collection, Page 6) "}</t>
         </is>
       </c>
     </row>
@@ -12629,7 +12629,7 @@
       </c>
       <c r="P243" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"We sent out 750 questionnaires to part-time MBA and EMBA students at 4 universities in China who come from enterprises in different provinces and municipalities such as Heilongjiang, Jilin and Beijing. Respondents were asked to be middle and senior managers and technical executives who understand corporate strategy and technology innovation. The questionnaires were collected in two phases. In the first stage, the data is distributed before class and recovered after class; in the second stage, some selected respondents, who were corporate executives, were invited to further distribute questionnaires to their subordinates or colleagues to reduce common method bias. Eventually, we obtained valid questionnaires from 290 different companies and the effective recovery rate was 38.67%.\" (Method, page 8)\n"}</t>
+          <t>Firm level analysis. Verbatim Evidence: "\"We sent out 750 questionnaires to part-time MBA and EMBA students at 4 universities in China who come from enterprises in different provinces and municipalities such as Heilongjiang, Jilin and Beijing. Respondents were asked to be middle and senior managers and technical executives who understand corporate strategy and technology innovation. The questionnaires were collected in two phases. In the first stage, the data is distributed before class and recovered after class; in the second stage, some selected respondents, who were corporate executives, were invited to further distribute questionnaires to their subordinates or colleagues to reduce common method bias. Eventually, we obtained valid questionnaires from 290 different companies and the effective recovery rate was 38.67%.\" (Method, page 8) "}</t>
         </is>
       </c>
     </row>
@@ -12677,7 +12677,7 @@
       </c>
       <c r="P244" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study lacks a Pearson correlation matrix reporting effect sizes for employee boundary spanning behavior. Instead, it utilizes qualitative script elicitation methodology and chi-square analysis to compare the frequency of service expectations between consumers and providers. Verbatim Evidence: "\"Thus, two sets of scripts were obtained, one set from consumers and the other set from service providers. The unit of analysis was the script, which was composed of the subgoals of the respondent’s typical haircut. The two sets of scripts were coded separately. Each subgoal mentioned was recorded, yielding a master list of subgoals for each set of respondents. The number of respondents who mentioned each subgoal was then tallied. Descriptive statistics are provided in Table I. Chi-square analysis found no significant gender differences in the frequency of mention of any of the subgoals.\" (Analysis and results, Page 7)\n"}</t>
+          <t>The study lacks a Pearson correlation matrix reporting effect sizes for employee boundary spanning behavior. Instead, it utilizes qualitative script elicitation methodology and chi-square analysis to compare the frequency of service expectations between consumers and providers. Verbatim Evidence: "\"Thus, two sets of scripts were obtained, one set from consumers and the other set from service providers. The unit of analysis was the script, which was composed of the subgoals of the respondent’s typical haircut. The two sets of scripts were coded separately. Each subgoal mentioned was recorded, yielding a master list of subgoals for each set of respondents. The number of respondents who mentioned each subgoal was then tallied. Descriptive statistics are provided in Table I. Chi-square analysis found no significant gender differences in the frequency of mention of any of the subgoals.\" (Analysis and results, Page 7) "}</t>
         </is>
       </c>
     </row>
@@ -12725,7 +12725,7 @@
       </c>
       <c r="P245" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study uses structural equation modeling (SEM) to evaluate the interrelations among variables but fails to provide a bivariate Pearson correlation matrix for the extracted measures. Only descriptive statistics, factor loadings, and structural path estimates are reported. Verbatim Evidence: "\"The descriptive statistics is shown in Table I, namely, mean, standard deviation and the factor analysis and Cronbach’s alpha results... Structural equation modelling (SEM) was used for the data analysis that included all the hypothesised paths, which is consistent with other studies conducted on multiteam system performance (Cuijpers et al., 2016; Cha et al., 2015). SEM was appropriate for investigating the interrelations among the set of variables, as it offers advantages over multiple regression, accounting, as it does for measurement error (Strasheim, 2014). SEM is a second generation multivariate method used to assess the reliability and validity of the model measures holistically, whereas first generation multivariate methods, such as multiple regression, are appropriate for evaluating constructs and relationships between constructs (Tabachnick and Fidell, 2001, p. 111). A measurement model was developed in AMOS 24.0 for the four constructs to be tested.\" (3. Methods, Page 11-12)\n"}</t>
+          <t>The study uses structural equation modeling (SEM) to evaluate the interrelations among variables but fails to provide a bivariate Pearson correlation matrix for the extracted measures. Only descriptive statistics, factor loadings, and structural path estimates are reported. Verbatim Evidence: "\"The descriptive statistics is shown in Table I, namely, mean, standard deviation and the factor analysis and Cronbach’s alpha results... Structural equation modelling (SEM) was used for the data analysis that included all the hypothesised paths, which is consistent with other studies conducted on multiteam system performance (Cuijpers et al., 2016; Cha et al., 2015). SEM was appropriate for investigating the interrelations among the set of variables, as it offers advantages over multiple regression, accounting, as it does for measurement error (Strasheim, 2014). SEM is a second generation multivariate method used to assess the reliability and validity of the model measures holistically, whereas first generation multivariate methods, such as multiple regression, are appropriate for evaluating constructs and relationships between constructs (Tabachnick and Fidell, 2001, p. 111). A measurement model was developed in AMOS 24.0 for the four constructs to be tested.\" (3. Methods, Page 11-12) "}</t>
         </is>
       </c>
     </row>
@@ -12773,7 +12773,7 @@
       </c>
       <c r="P246" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: "\"We gathered our data in The Netherlands using a cross sectional survey methodology. We used the project level of analysis because the information used to make NPD decisions is project-specific, rather than being more generally applicable to the entire firm or a division. Each project requires specific details about customer needs and technical capabilities to allow developers to make tradeoffs between the different specifications and feature levels.\" (Sample and Data Collection, Page 4)\n"}</t>
+          <t>Project level analysis. Verbatim Evidence: "\"We gathered our data in The Netherlands using a cross sectional survey methodology. We used the project level of analysis because the information used to make NPD decisions is project-specific, rather than being more generally applicable to the entire firm or a division. Each project requires specific details about customer needs and technical capabilities to allow developers to make tradeoffs between the different specifications and feature levels.\" (Sample and Data Collection, Page 4) "}</t>
         </is>
       </c>
     </row>
@@ -13017,7 +13017,7 @@
       </c>
       <c r="P251" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"In cooperation with the leaders of the rehabilitation centres, all health professionals (N = 167) engaged in working with patients in the centres were invited to participate in the survey. These centres deliver services via interprofessional teams; we identified 16 teams, which were the unit of interest in the present study, according to RC theory [9]. Some healthcare professionals were members of more than one team in the centre in which they worked; these professionals were asked to respond to the survey for each team they worked with.\" (Methods, Page 2) \"The main explanatory variables in this study were the RC communication and relationships scores, which were calculated for each team and used as continuous variables, from 1(lowest) to 5 (highest).\" (Methods, Page 4)\n"}</t>
+          <t>Team level analysis. Verbatim Evidence: "\"In cooperation with the leaders of the rehabilitation centres, all health professionals (N = 167) engaged in working with patients in the centres were invited to participate in the survey. These centres deliver services via interprofessional teams; we identified 16 teams, which were the unit of interest in the present study, according to RC theory [9]. Some healthcare professionals were members of more than one team in the centre in which they worked; these professionals were asked to respond to the survey for each team they worked with.\" (Methods, Page 2) \"The main explanatory variables in this study were the RC communication and relationships scores, which were calculated for each team and used as continuous variables, from 1(lowest) to 5 (highest).\" (Methods, Page 4) "}</t>
         </is>
       </c>
     </row>
@@ -13111,7 +13111,7 @@
       </c>
       <c r="P253" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 2\nPatient sample. Verbatim Evidence: "\"All patients aged 18 and above who were accepted for rehabilitation in a rehabilitation centre in Western Norway between January 2015 and June 2015 were invited to participate (n=2863). For baseline data collection, a total of 984 (34%) patients accepted the invitation to participate and provided written consent and a completed questionnaire. A 1-year follow-up questionnaire was sent to all participating patients (n=984), and 705 patients (25% of the patient group invited at baseline) returned the questionnaire. We extracted 279 of the baseline participants from the analyses, as they did not respond to the 1-year follow-up survey. Four respondents were omitted from the analyses due to missing data on outcome variables. Finally, 701 (24% of the patient group invited at baseline) patients were included in the analyses (Table 1).\" (Participants, Page 2-3)\n"}</t>
+          <t>Patient sample. Verbatim Evidence: "\"All patients aged 18 and above who were accepted for rehabilitation in a rehabilitation centre in Western Norway between January 2015 and June 2015 were invited to participate (n=2863). For baseline data collection, a total of 984 (34%) patients accepted the invitation to participate and provided written consent and a completed questionnaire. A 1-year follow-up questionnaire was sent to all participating patients (n=984), and 705 patients (25% of the patient group invited at baseline) returned the questionnaire. We extracted 279 of the baseline participants from the analyses, as they did not respond to the 1-year follow-up survey. Four respondents were omitted from the analyses due to missing data on outcome variables. Finally, 701 (24% of the patient group invited at baseline) patients were included in the analyses (Table 1).\" (Participants, Page 2-3) "}</t>
         </is>
       </c>
     </row>
@@ -13159,7 +13159,7 @@
       </c>
       <c r="P254" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study only reports descriptive percentages for team-level feedback and does not provide an individual-level Pearson correlation matrix or quantitative effect sizes. Verbatim Evidence: "\"The questionnaire was designed to be used as a self-diagnostic instrument, and therefore the format of the feedback returned to the teams was specified according to the preferences of the teams. Teams preferred feedback in percentages above means; the sum of the percentages of team members that “agreed” and “agreed strongly” was reported. Also standard deviations were reported, and we volunteered to discuss scales and items with low percentages or high standard deviations in team meetings. In four teams the questionnaires were filled out individually during team meetings, however, the members of fifth team preferred to do this outer their meeting. There were 52 workers in the five teams, and 46 (88 per cent) completed the questionnaire.\" (The questionnaire, Page 59)\n"}</t>
+          <t>The study only reports descriptive percentages for team-level feedback and does not provide an individual-level Pearson correlation matrix or quantitative effect sizes. Verbatim Evidence: "\"The questionnaire was designed to be used as a self-diagnostic instrument, and therefore the format of the feedback returned to the teams was specified according to the preferences of the teams. Teams preferred feedback in percentages above means; the sum of the percentages of team members that “agreed” and “agreed strongly” was reported. Also standard deviations were reported, and we volunteered to discuss scales and items with low percentages or high standard deviations in team meetings. In four teams the questionnaires were filled out individually during team meetings, however, the members of fifth team preferred to do this outer their meeting. There were 52 workers in the five teams, and 46 (88 per cent) completed the questionnaire.\" (The questionnaire, Page 59) "}</t>
         </is>
       </c>
     </row>
@@ -13207,7 +13207,7 @@
       </c>
       <c r="P255" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"Transformational leadership, gatekeeping leadership, internal communication, external communication, and norm for maintaining consensus were aggregated to mean values within each team, which was the unit of the analysis. To justify this aggregation, a within-group correlation (rwg) was computed to assess the amount of agreement by the team members (James et al. 1984). The mean rwg value was 0.87 for transformational leadership, 0.89 for gatekeeping leadership, 0.90 for internal communication, 0.89 for external communication, and 0.89 for norm for maintaining consensus. In addition, the ICC(1) values were as follows: transformational leadership, 0.22; gatekeeping leadership, 0.50; internal communication, 0.24; external communication, 0.36; and norm for maintaining consensus, 0.25. ICC(2) values were as follows: transformational leadership, 0.61; gatekeeping leadership, 0.85; internal communication, 0.64; external communication, 0.76; and norm for maintaining consensus, 0.65. The overall pattern of results across the rwg, ICC(1), and ICC(2) analyses provided sufficient support for aggregating the data to team level of analysis.\" (Aggregation tests, Page 11)\n"}</t>
+          <t>Team level analysis. Verbatim Evidence: "\"Transformational leadership, gatekeeping leadership, internal communication, external communication, and norm for maintaining consensus were aggregated to mean values within each team, which was the unit of the analysis. To justify this aggregation, a within-group correlation (rwg) was computed to assess the amount of agreement by the team members (James et al. 1984). The mean rwg value was 0.87 for transformational leadership, 0.89 for gatekeeping leadership, 0.90 for internal communication, 0.89 for external communication, and 0.89 for norm for maintaining consensus. In addition, the ICC(1) values were as follows: transformational leadership, 0.22; gatekeeping leadership, 0.50; internal communication, 0.24; external communication, 0.36; and norm for maintaining consensus, 0.25. ICC(2) values were as follows: transformational leadership, 0.61; gatekeeping leadership, 0.85; internal communication, 0.64; external communication, 0.76; and norm for maintaining consensus, 0.65. The overall pattern of results across the rwg, ICC(1), and ICC(2) analyses provided sufficient support for aggregating the data to team level of analysis.\" (Aggregation tests, Page 11) "}</t>
         </is>
       </c>
     </row>
@@ -13255,7 +13255,7 @@
       </c>
       <c r="P256" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nThe study uses work groups as the unit of analysis and aggregates individual survey responses to the team level. Verbatim Evidence: "\"Following Van de Ven and colleagues (1976) and Tushman (1977, 1978), we used work groups as the units of analysis. First-line supervisors with at least one year as unit heads who had full-time subordinates with sufficient experience to be familiar with their positions answered questions on the subordinates' jobs. The study included all units meeting the criterion for supervisory experience and containing at least two experienced subordinates. [...] To compute scores for work groups, supervisors' scores were added to the means of subordinates' scores, and these sums were divided by two (Van de Ven et al., 1976). Three tests supported this procedure. One-way analysis of variance (Dixon &amp; Massey, 1969) supported pooling subordinate responses into work groups for all of the variables (p &lt; .005).\" (Methods, pages 143-144)\n"}</t>
+          <t>The study uses work groups as the unit of analysis and aggregates individual survey responses to the team level. Verbatim Evidence: "\"Following Van de Ven and colleagues (1976) and Tushman (1977, 1978), we used work groups as the units of analysis. First-line supervisors with at least one year as unit heads who had full-time subordinates with sufficient experience to be familiar with their positions answered questions on the subordinates' jobs. The study included all units meeting the criterion for supervisory experience and containing at least two experienced subordinates. [...] To compute scores for work groups, supervisors' scores were added to the means of subordinates' scores, and these sums were divided by two (Van de Ven et al., 1976). Three tests supported this procedure. One-way analysis of variance (Dixon &amp; Massey, 1969) supported pooling subordinate responses into work groups for all of the variables (p &lt; .005).\" (Methods, pages 143-144) "}</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       </c>
       <c r="P257" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nNo individual-level bivariate Pearson correlation matrix is provided. The study only reports an aggregated organizational-level correlation matrix and jumps straight to regression for the individual-level analysis. Verbatim Evidence: "\"Regression analysis. First, a simple regression model was conducted to test if NCB significantly predicted IIB. The results of the regression indicated that NCB explained 17.8% of the variance in IIB (R2 = 17.8, F (1, 85) = 18.436, p&lt;.05). Next, a multiple regression analysis was conducted to test if NCB significantly predicted IIB after five demographic variables are controlled. The results of the multiple regression indicated that together with the four demographic variables, NCB predicted 30.5% of the variance in IIB (R2 = .305, F (6, 75) = 5.485, p&lt;.001).\" (Chapter 4: Data Analysis, Page 108)\n"}</t>
+          <t>No individual-level bivariate Pearson correlation matrix is provided. The study only reports an aggregated organizational-level correlation matrix and jumps straight to regression for the individual-level analysis. Verbatim Evidence: "\"Regression analysis. First, a simple regression model was conducted to test if NCB significantly predicted IIB. The results of the regression indicated that NCB explained 17.8% of the variance in IIB (R2 = 17.8, F (1, 85) = 18.436, p&lt;.05). Next, a multiple regression analysis was conducted to test if NCB significantly predicted IIB after five demographic variables are controlled. The results of the multiple regression indicated that together with the four demographic variables, NCB predicted 30.5% of the variance in IIB (R2 = .305, F (6, 75) = 5.485, p&lt;.001).\" (Chapter 4: Data Analysis, Page 108) "}</t>
         </is>
       </c>
     </row>
@@ -13351,7 +13351,7 @@
       </c>
       <c r="P258" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nThe study samples boundary spanners but lacks an effect size for boundary spanning behavior, measuring only burnout, role stressors, and general job performance. Verbatim Evidence: "\"Job outcomes. Psychological outcomes were measured by three separate first-order constmcts. JS was operationalized as a 26-item scale adapted from Churchill, Ford, and Walker's (1985) study that has been frequently used in marketing. The alpha reliability of this scale was estimated as .92. OC was operationalized by use of a 6-item version of a scale from Mowday, Steers, and Porter (1979). Tbe scaie achieved acceptable reliability (a = .79). Finally, Tl was assessed by a three-item measure based on Donnelly and Ivancevicb (1975). In addition, this measure has been shown in several studies to be a consistent predictor of actual tumover. The Cronbach's a for this measure was .85. Behavioral out comes were measured by a self-rating, 6-item measure of JP drawn from Dubinsky and Mattson (1979).\" (Measures, page 563)\n"}</t>
+          <t>The study samples boundary spanners but lacks an effect size for boundary spanning behavior, measuring only burnout, role stressors, and general job performance. Verbatim Evidence: "\"Job outcomes. Psychological outcomes were measured by three separate first-order constmcts. JS was operationalized as a 26-item scale adapted from Churchill, Ford, and Walker's (1985) study that has been frequently used in marketing. The alpha reliability of this scale was estimated as .92. OC was operationalized by use of a 6-item version of a scale from Mowday, Steers, and Porter (1979). Tbe scaie achieved acceptable reliability (a = .79). Finally, Tl was assessed by a three-item measure based on Donnelly and Ivancevicb (1975). In addition, this measure has been shown in several studies to be a consistent predictor of actual tumover. The Cronbach's a for this measure was .85. Behavioral out comes were measured by a self-rating, 6-item measure of JP drawn from Dubinsky and Mattson (1979).\" (Measures, page 563) "}</t>
         </is>
       </c>
     </row>
@@ -13399,7 +13399,7 @@
       </c>
       <c r="P259" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nProject level analysis. Verbatim Evidence: "\"In fact, because degree-based centrality measures are basically a standardized count of ties, a high actor degree centrality in an inter-organizational network equates to a higher level of BSA from the team's point of view. Consequently, the measure of BSA in this dissertation is the focal team's degree centrality in an inter-team network where the nodes are all OSS projects registered in Source Forge. This measure can be used since each project in Source Forge includes a list of developers. Once all these lists have been scanned, it is easy to detect developers who work on more than one project and then build the inter-team network in order to calculate a given project's BSA.\" (4.4.3.4 Boundary Spanning Activity, Page 99)\n"}</t>
+          <t>Project level analysis. Verbatim Evidence: "\"In fact, because degree-based centrality measures are basically a standardized count of ties, a high actor degree centrality in an inter-organizational network equates to a higher level of BSA from the team's point of view. Consequently, the measure of BSA in this dissertation is the focal team's degree centrality in an inter-team network where the nodes are all OSS projects registered in Source Forge. This measure can be used since each project in Source Forge includes a list of developers. Once all these lists have been scanned, it is easy to detect developers who work on more than one project and then build the inter-team network in order to calculate a given project's BSA.\" (4.4.3.4 Boundary Spanning Activity, Page 99) "}</t>
         </is>
       </c>
     </row>
@@ -13497,7 +13497,7 @@
       </c>
       <c r="P261" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided; the study only reports mean differences and t-tests. Verbatim Evidence: "\"Measures used to test the hypotheses each consisted of two 7-point itemized rating scales designed to assess the extent to which team selling was used in a particular buying or selling situation. For example, to measure the extent to which team selling is used when the buyer’s informational needs are great, respondents indicated the likelihood of using sales teams when 'the anticipated information needs of the customer are small' and 'the anticipated information needs of the customer are great' (1 = extremely unlikely, 7 = extremely likely). T-tests were conducted on the mean differences between the respondents’ ratings for each of the paired questions. A hypothesis was supported when the mean difference was significantly different from 0.\" (Hypotheses Tests, page 160)\n"}</t>
+          <t>No bivariate Pearson correlation matrix provided; the study only reports mean differences and t-tests. Verbatim Evidence: "\"Measures used to test the hypotheses each consisted of two 7-point itemized rating scales designed to assess the extent to which team selling was used in a particular buying or selling situation. For example, to measure the extent to which team selling is used when the buyer’s informational needs are great, respondents indicated the likelihood of using sales teams when 'the anticipated information needs of the customer are small' and 'the anticipated information needs of the customer are great' (1 = extremely unlikely, 7 = extremely likely). T-tests were conducted on the mean differences between the respondents’ ratings for each of the paired questions. A hypothesis was supported when the mean difference was significantly different from 0.\" (Hypotheses Tests, page 160) "}</t>
         </is>
       </c>
     </row>
@@ -13641,7 +13641,7 @@
       </c>
       <c r="P264" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 4\nQualitative case study lacking quantitative correlation data. Verbatim Evidence: "\"We use a case study research methodology to identify various contextual elements that shape the development of a common platform in a post-merger scenario. We examine how stakeholders from different business divisions establish a common understanding of their processes to inform the development of a common platform underlying a family of similar business processes. [...] We participated as observers in all the eight workshops and in six other meetings. Workshop meetings were audio-recorded with the participants’ consent, yielding an extremely rich set of data of over more than 50 h. Additional informal interviews with process participants were conducted to seek clarifications on issues raised during the workshops. See Online Appendix B for an excerpt of the interview questionnaire. These interviews allowed us to explore the expectations of the participants. Detailed notes were also taken during each of the data collection sessions. Workshops and interviews were our primary source of qualitative data.\" (Research methodology &amp; Data collection, Page 5-6)\n"}</t>
+          <t>Qualitative case study lacking quantitative correlation data. Verbatim Evidence: "\"We use a case study research methodology to identify various contextual elements that shape the development of a common platform in a post-merger scenario. We examine how stakeholders from different business divisions establish a common understanding of their processes to inform the development of a common platform underlying a family of similar business processes. [...] We participated as observers in all the eight workshops and in six other meetings. Workshop meetings were audio-recorded with the participants’ consent, yielding an extremely rich set of data of over more than 50 h. Additional informal interviews with process participants were conducted to seek clarifications on issues raised during the workshops. See Online Appendix B for an excerpt of the interview questionnaire. These interviews allowed us to explore the expectations of the participants. Detailed notes were also taken during each of the data collection sessions. Workshops and interviews were our primary source of qualitative data.\" (Research methodology &amp; Data collection, Page 5-6) "}</t>
         </is>
       </c>
     </row>
@@ -13735,7 +13735,7 @@
       </c>
       <c r="P266" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nFirm level analysis. Verbatim Evidence: "\"For our empirical analysis, we use data sets provided by the Netherlands Enterprise Agency (RVO.nl) on all collaborative R&amp;D projects that received support from the allowance scheme in the period 2013–2018. The data sets include information about project titles, starting years, participants and budgets. By merging the data, it is possible to map the evolution of the collaborative network for the period 2013–2018. The total network includes 1884 Dutch firms and 105 publicly-funded organizations. Given our focus on recombining firm capabilities, our analyses concentrate on the 1884 firms only.\" (Case description: collaborative R&amp;D in the Netherlands, Page 4)\n"}</t>
+          <t>Firm level analysis. Verbatim Evidence: "\"For our empirical analysis, we use data sets provided by the Netherlands Enterprise Agency (RVO.nl) on all collaborative R&amp;D projects that received support from the allowance scheme in the period 2013–2018. The data sets include information about project titles, starting years, participants and budgets. By merging the data, it is possible to map the evolution of the collaborative network for the period 2013–2018. The total network includes 1884 Dutch firms and 105 publicly-funded organizations. Given our focus on recombining firm capabilities, our analyses concentrate on the 1884 firms only.\" (Case description: collaborative R&amp;D in the Netherlands, Page 4) "}</t>
         </is>
       </c>
     </row>
@@ -14023,7 +14023,7 @@
       </c>
       <c r="P272" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 1\nNo bivariate Pearson correlation matrix provided. Verbatim Evidence: "\"Grouping and Analytic Techniques. Each subject was grouped according to primary decision style which resulted in four groups of individuals being labeled as either SF (n = 20), ST (n = 7), NF (n = 24), or NT (n = 6). Because BSA was defined as multidimensional in nature and was composed of three separate dimensions, the primary analytic technique used was multivariate analysis of variance (MANOVA). This test was run to determine if decision style affected total BSA. Given a significant overall F for the MANOVA test, several post hoc techniques were employed to investigate the specific nature of these differences. First, a multivariate extension of the Scheffe test was used to determine which decision style groups were different from each other across the combination of the three BSA variables.\" (Grouping and Analytic Techniques, Page 6)\n"}</t>
+          <t>No bivariate Pearson correlation matrix provided. Verbatim Evidence: "\"Grouping and Analytic Techniques. Each subject was grouped according to primary decision style which resulted in four groups of individuals being labeled as either SF (n = 20), ST (n = 7), NF (n = 24), or NT (n = 6). Because BSA was defined as multidimensional in nature and was composed of three separate dimensions, the primary analytic technique used was multivariate analysis of variance (MANOVA). This test was run to determine if decision style affected total BSA. Given a significant overall F for the MANOVA test, several post hoc techniques were employed to investigate the specific nature of these differences. First, a multivariate extension of the Scheffe test was used to determine which decision style groups were different from each other across the combination of the three BSA variables.\" (Grouping and Analytic Techniques, Page 6) "}</t>
         </is>
       </c>
     </row>
@@ -14167,7 +14167,7 @@
       </c>
       <c r="P275" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nProject and team level of analysis without individual employee boundary spanning correlations. Verbatim Evidence: "\"From the multiteam system (MTS) perspective, this study employs the input-process-outcome (IPO) framework and coordination theory to explore the influence of instant messaging-based team boundary spanning (IMTBS) on construction project coordination processes and project performance. A theoretical model is built and validated with a survey involving 206 construction projects. [...] Data were collected from construction projects in China. We first conducted a pilot study involving 30 respondents from the Master of Engineering Management (MEM) students majoring in construction management at a Chinese renowned university to test the validity of all constructs. [...] Then, the questionnaire was distributed to construction professionals to report the condition of the last completed project they managed. We randomly sent the link to the online survey to alumni of two renowned universities, who were involved in the construction industry. A total of 400 questionnaires were distributed to these alumni from 53 construction companies, and 256 responses were returned. After removing invalid responses, 206 valid questionnaires were left, thereby yielding a valid response rate of 51.5%.\" (Abstract, Page 1; 4.2 Data collection, Page 7)\n"}</t>
+          <t>Project and team level of analysis without individual employee boundary spanning correlations. Verbatim Evidence: "\"From the multiteam system (MTS) perspective, this study employs the input-process-outcome (IPO) framework and coordination theory to explore the influence of instant messaging-based team boundary spanning (IMTBS) on construction project coordination processes and project performance. A theoretical model is built and validated with a survey involving 206 construction projects. [...] Data were collected from construction projects in China. We first conducted a pilot study involving 30 respondents from the Master of Engineering Management (MEM) students majoring in construction management at a Chinese renowned university to test the validity of all constructs. [...] Then, the questionnaire was distributed to construction professionals to report the condition of the last completed project they managed. We randomly sent the link to the online survey to alumni of two renowned universities, who were involved in the construction industry. A total of 400 questionnaires were distributed to these alumni from 53 construction companies, and 256 responses were returned. After removing invalid responses, 206 valid questionnaires were left, thereby yielding a valid response rate of 51.5%.\" (Abstract, Page 1; 4.2 Data collection, Page 7) "}</t>
         </is>
       </c>
     </row>
@@ -14215,7 +14215,7 @@
       </c>
       <c r="P276" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude\nReason Code: 3\nTeam level analysis. Verbatim Evidence: "\"The referent-shift consensus model proposed by Chan[50]was used in designing the questionnaire, which means that variables including \"team boundary-spanning activities,\" \"team job crafting,\" and \"team innovation performance\" was designed from the perspective of the team. A request was made for these questions to be answered from the perspective of team awareness. The \"individual job crafting\" variable was designed from the employees' perspective. Second, the terminology, the clarity of the instructions, and the structure of the questionnaire's responses were evaluated by three subject-matter experts and five teams from Shandong province's universities engaged in scientific research and innovation. Modifications were made accordingly. Finally, teams that were developing collaborative innovation projects were selected. The distribution of 456 surveys resulted in the recovery of 400 questionnaires. Three hundred thirty-one valid surveys were retrieved after invalid data had been removed; these originated from 41 collaborative innovation teams.\" (3.1 Sample and data collection procedure, Page 6)\n"}</t>
+          <t>Team level analysis. Verbatim Evidence: "\"The referent-shift consensus model proposed by Chan[50]was used in designing the questionnaire, which means that variables including \"team boundary-spanning activities,\" \"team job crafting,\" and \"team innovation performance\" was designed from the perspective of the team. A request was made for these questions to be answered from the perspective of team awareness. The \"individual job crafting\" variable was designed from the employees' perspective. Second, the terminology, the clarity of the instructions, and the structure of the questionnaire's responses were evaluated by three subject-matter experts and five teams from Shandong province's universities engaged in scientific research and innovation. Modifications were made accordingly. Finally, teams that were developing collaborative innovation projects were selected. The distribution of 456 surveys resulted in the recovery of 400 questionnaires. Three hundred thirty-one valid surveys were retrieved after invalid data had been removed; these originated from 41 collaborative innovation teams.\" (3.1 Sample and data collection procedure, Page 6) "}</t>
         </is>
       </c>
     </row>
@@ -14261,11 +14261,7 @@
       <c r="K277" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P277" s="0" t="inlineStr">
-        <is>
-          <t>[Construct homonymy: study measures work-family boundary management, not organizational boundary spanning behavior]. Verbatim Evidence: \\\"OBJECTIVE: This study was conducted to examine how teleworking outside regular office hours and individual boundary management relate to work-family conflict.\\\" (Abstract)</t>
-        </is>
-      </c>
+      <c r="P277" s="0" t="inlineStr"/>
     </row>
     <row r="278" ht="18" customHeight="1" s="31">
       <c r="A278" s="0" t="inlineStr">
@@ -14359,11 +14355,7 @@
       <c r="K279" s="0" t="n">
         <v>1996</v>
       </c>
-      <c r="P279" s="0" t="inlineStr">
-        <is>
-          <t>This study describes the organizational arrangements used to source scientific knowledge in two highly successful NBFs -- firms that have succeeded in sourcing and commercializing valuable scientific knowledge. As both firms requested anonymity, we refer to them as Firm X and Firm Y.\" (4.1 Sample)</t>
-        </is>
-      </c>
+      <c r="P279" s="0" t="inlineStr"/>
     </row>
     <row r="280" ht="18" customHeight="1" s="31">
       <c r="A280" s="0" t="inlineStr">
@@ -14453,11 +14445,7 @@
       <c r="K281" s="0" t="n">
         <v>2003</v>
       </c>
-      <c r="P281" s="0" t="inlineStr">
-        <is>
-          <t>I asked two team members in each participating project to provide a single consensual rating for the measures of these forces. I selected the team members upon the advice of senior managers who deemed them as being highly knowledgeable about their projects.</t>
-        </is>
-      </c>
+      <c r="P281" s="0" t="inlineStr"/>
     </row>
     <row r="282" ht="18" customHeight="1" s="31">
       <c r="A282" s="0" t="inlineStr">
@@ -14514,11 +14502,7 @@
       <c r="K282" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="P282" s="0" t="inlineStr">
-        <is>
-          <t>how others’ availability expectations predict employees’ management of work and nonwork boundaries, and how these bidirectional boundary management behaviors relate to well-being.\" (Abstract)</t>
-        </is>
-      </c>
+      <c r="P282" s="0" t="inlineStr"/>
     </row>
     <row r="283" ht="18" customHeight="1" s="31">
       <c r="A283" s="0" t="inlineStr">
@@ -14564,7 +14548,7 @@
       </c>
       <c r="P283" s="0" t="inlineStr">
         <is>
-          <t>Problems cross boundaries and so must solutions. The most important challenge for performance networks that aim to deliver better results is designing the structure that coordinates across traditional agency boundaries.</t>
+          <t>Verbatim Evidence: \"Problems cross boundaries and so must solutions. The most important challenge for performance networks that aim to deliver better results is designing the structure that coordinates across traditional agency boundaries.</t>
         </is>
       </c>
     </row>
@@ -14612,7 +14596,7 @@
       </c>
       <c r="P284" s="0" t="inlineStr">
         <is>
-          <t>[Unit of analysis is at the team level]. Verbatim Evidence: \\\"To test hypotheses, the study focuses on technology transfer intermediaries of the manufacturing industry in China at the team level.\\\" (3.1 Research setting)</t>
+          <t>Verbatim Evidence: \"[Unit of analysis is at the team level]. Verbatim Evidence: \\\"To test hypotheses, the study focuses on technology transfer intermediaries of the manufacturing industry in China at the team level.\\\" (3.1 Research setting)</t>
         </is>
       </c>
     </row>
@@ -14660,7 +14644,7 @@
       </c>
       <c r="P285" s="0" t="inlineStr">
         <is>
-          <t>The level of analysis is an alliance between two partners.</t>
+          <t>Verbatim Evidence: \"The level of analysis is an alliance between two partners.</t>
         </is>
       </c>
     </row>
@@ -14752,11 +14736,7 @@
       <c r="K287" s="0" t="n">
         <v>2019</v>
       </c>
-      <c r="P287" s="0" t="inlineStr">
-        <is>
-          <t>Qualitative study without quantitative effect sizes based on a non-employee sample. Verbatim Evidence: \\\"This article is based on in-depth interviews with 30 subjects—15 men and 15 women.\\\" (Study design) and \\\"This article proposes to examine the self-concept of members of an occupational category called 'solo self-employed,' that is, women and men who work alone and do not employ any workers.\\\" (Introduction)</t>
-        </is>
-      </c>
+      <c r="P287" s="0" t="inlineStr"/>
     </row>
     <row r="288" ht="18" customHeight="1" s="31">
       <c r="A288" s="0" t="inlineStr">
@@ -14800,11 +14780,7 @@
       <c r="K288" s="0" t="n">
         <v>2011</v>
       </c>
-      <c r="P288" s="0" t="inlineStr">
-        <is>
-          <t>The purpose of this paper is to develop the concept of project management system from the perspective of systems science.\" (Abstract)</t>
-        </is>
-      </c>
+      <c r="P288" s="0" t="inlineStr"/>
     </row>
     <row r="289" ht="18" customHeight="1" s="31">
       <c r="A289" s="0" t="inlineStr">
@@ -14898,11 +14874,7 @@
       <c r="K290" s="0" t="n">
         <v>2023</v>
       </c>
-      <c r="P290" s="0" t="inlineStr">
-        <is>
-          <t>These are boundary theory (Ashforth et al., 2000; Allen et al., 2014; Nippert Eng, 1996), which focuses on the work-life domain, and border theory (Clark, 2000), which focuses on the work and family domain. As per these theories, individuals are forced to set boundaries to balance their work and family roles.</t>
-        </is>
-      </c>
+      <c r="P290" s="0" t="inlineStr"/>
     </row>
     <row r="291" ht="18" customHeight="1" s="31">
       <c r="A291" s="0" t="inlineStr">
@@ -15112,7 +15084,7 @@
       </c>
       <c r="P294" s="0" t="inlineStr">
         <is>
-          <t>Study analyzes organizations rather than individuals. Verbatim Evidence: \\\"This paper, in an attempt to link up these ideas, investigates knowledge transfer processes within inter-organizational R&amp;D projects that are embedded in 23 German regional innovation networks (with almost 500 participants).\\\" (Abstract)</t>
+          <t>Verbatim Evidence: \"Study analyzes organizations rather than individuals. Verbatim Evidence: \\\"This paper, in an attempt to link up these ideas, investigates knowledge transfer processes within inter-organizational R&amp;D projects that are embedded in 23 German regional innovation networks (with almost 500 participants).\\\" (Abstract)</t>
         </is>
       </c>
     </row>
@@ -15396,11 +15368,7 @@
       <c r="K300" s="0" t="n">
         <v>2026</v>
       </c>
-      <c r="P300" s="0" t="inlineStr">
-        <is>
-          <t>Firm-level analysis. Verbatim Evidence: \\\"To gauge the study hypotheses, time-lagged data were gathered from 244 firms in China.\\\" (Abstract)</t>
-        </is>
-      </c>
+      <c r="P300" s="0" t="inlineStr"/>
     </row>
     <row r="301" ht="18" customHeight="1" s="31">
       <c r="A301" s="0" t="inlineStr">
@@ -15446,7 +15414,7 @@
       </c>
       <c r="P301" s="0" t="inlineStr">
         <is>
-          <t>the final dataset we retained and used for data analysis pertained to 365 firms.\"\n\nI have successfully updated BSMA_Master_Coding_Sheet.xlsx and committed and pushed the changes to Github.</t>
+          <t>I have successfully updated BSMA_Master_Coding_Sheet.xlsx and committed and pushed the changes to Github.</t>
         </is>
       </c>
     </row>
@@ -15494,7 +15462,7 @@
       </c>
       <c r="P302" s="0" t="inlineStr">
         <is>
-          <t>Organizational behavior (OB) is an area of knowledge rather than a unified theory. It consists of a growing clutch of concepts, approaches, models, and tools pertinent to the structure and functioning of organizations within their socioeconomic contexts and of the study of individuals and groups within their organizational contexts</t>
+          <t>Verbatim Evidence: \"Organizational behavior (OB) is an area of knowledge rather than a unified theory. It consists of a growing clutch of concepts, approaches, models, and tools pertinent to the structure and functioning of organizations within their socioeconomic contexts and of the study of individuals and groups within their organizational contexts</t>
         </is>
       </c>
     </row>
@@ -15590,11 +15558,7 @@
       <c r="K304" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="P304" s="0" t="inlineStr">
-        <is>
-          <t>[No BSB construct measured]. Verbatim Evidence: \\\"The results indicate that FSEs’ perceptions of CSR are negatively related to their perceptions of verbal dysfunctional customer conduct, which in turn is shown to be directly linked to emotional exhaustion. FSEs’ CSR perceptions strengthen their view that they are performing meaningful work (i.e. perceived task significance), which in turn strengthens their job satisfaction.\\\" (Abstract)</t>
-        </is>
-      </c>
+      <c r="P304" s="0" t="inlineStr"/>
     </row>
     <row r="305" ht="18" customHeight="1" s="31">
       <c r="A305" s="0" t="inlineStr">
@@ -15931,7 +15895,7 @@
       </c>
       <c r="P311" s="0" t="inlineStr">
         <is>
-          <t>Employees provided information regarding work overload, resilience, and intimidation, while their direct supervisors provided information regarding their subordinates’ sales performance.\" (3.2. Measures)</t>
+          <t>Verbatim Evidence: \"Employees provided information regarding work overload, resilience, and intimidation, while their direct supervisors provided information regarding their subordinates’ sales performance.\" (3.2. Measures)</t>
         </is>
       </c>
     </row>
@@ -15977,11 +15941,7 @@
       <c r="K312" s="0" t="n">
         <v>2016</v>
       </c>
-      <c r="P312" s="0" t="inlineStr">
-        <is>
-          <t>The study focuses on work-nonwork (work-life) boundary management rather than organizational boundary spanning behavior, hence there are no relevant effect sizes. Verbatim Evidence: \\\"In this study we focused on examining employees’ work-nonwork boundary management from the perspective of work stress recovery. Boundary management refers to the ways in which employees create, maintain and negotiate boundaries between work and nonwork\\\" (Introduction)</t>
-        </is>
-      </c>
+      <c r="P312" s="0" t="inlineStr"/>
     </row>
     <row r="313" ht="18" customHeight="1" s="31">
       <c r="A313" s="0" t="inlineStr">
@@ -16025,11 +15985,7 @@
       <c r="K313" s="0" t="n">
         <v>2007</v>
       </c>
-      <c r="P313" s="0" t="inlineStr">
-        <is>
-          <t>The purpose of this study was to analyze the school safety and security planning process. Sixty-two public school districts and non public schools within a fifty-mile radius of a large metropolitan area, located within the four states area of Texas, Oklahoma, Arkansas, and Kansas, were carefully studied\" (Abstract)</t>
-        </is>
-      </c>
+      <c r="P313" s="0" t="inlineStr"/>
     </row>
     <row r="314" ht="18" customHeight="1" s="31">
       <c r="A314" s="0" t="inlineStr">
@@ -16123,11 +16079,7 @@
       <c r="K315" s="0" t="n">
         <v>2017</v>
       </c>
-      <c r="P315" s="0" t="inlineStr">
-        <is>
-          <t>For each activity, we provide examples and illustrations which we derived by interviewing senior industry professionals from different industries (such as telecommunications, medical devices and pharmaceuticals) and with direct experiences in global boundary spanning and technology scouting. Specifically, between 2011–15, we conducted 15 in-depth interviews with managers in European and North American MNCs</t>
-        </is>
-      </c>
+      <c r="P315" s="0" t="inlineStr"/>
     </row>
     <row r="316" ht="18" customHeight="1" s="31">
       <c r="A316" s="0" t="inlineStr">
@@ -16171,11 +16123,7 @@
       <c r="K316" s="0" t="n">
         <v>2005</v>
       </c>
-      <c r="P316" s="0" t="inlineStr">
-        <is>
-          <t>Data were analysed for all references to skills, knowledge, traits, behavioural indicators and outcomes associated with effective and ineffective performance. Over 250 items of data were identified. These were constructed into a framework describing the features of high performance, which was then critically reviewed by a small group of managers (the ‘review group’), and revised.\" (5 Findings)</t>
-        </is>
-      </c>
+      <c r="P316" s="0" t="inlineStr"/>
     </row>
     <row r="317" ht="18" customHeight="1" s="31">
       <c r="A317" s="0" t="inlineStr">
@@ -16421,7 +16369,7 @@
       </c>
       <c r="P321" s="0" t="inlineStr">
         <is>
-          <t>The questionnaire was designed to measure the perceived: 1) importance and 2) effectiveness of each of the eight classes of MCP’s.\" (IV. METHOD)</t>
+          <t>Verbatim Evidence: \"The questionnaire was designed to measure the perceived: 1) importance and 2) effectiveness of each of the eight classes of MCP’s.\" (IV. METHOD)</t>
         </is>
       </c>
     </row>
@@ -16467,11 +16415,7 @@
       <c r="K322" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P322" s="0" t="inlineStr">
-        <is>
-          <t>The empirical setting is publicly held US manufacturing firms that are present in both the Kinder, Lydenberg and Domini’s (KLD’s) annual EVP ratings and Bloomberg’s supply chain database. The study employs panel data regression methods on an unbalanced panel dataset of 7,493 dyad-year observations comprising 427 unique firms.</t>
-        </is>
-      </c>
+      <c r="P322" s="0" t="inlineStr"/>
     </row>
     <row r="323" ht="18" customHeight="1" s="31">
       <c r="A323" s="0" t="inlineStr">
@@ -16565,11 +16509,7 @@
       <c r="K324" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="P324" s="0" t="inlineStr">
-        <is>
-          <t>[Team-level aggregation]. Verbatim Evidence: \\\"To use the individuals’ responses for further analysis, the responses were aggregated by extracting the mean scores.\\\" (4. Results)</t>
-        </is>
-      </c>
+      <c r="P324" s="0" t="inlineStr"/>
     </row>
     <row r="325" ht="18" customHeight="1" s="31">
       <c r="A325" s="0" t="inlineStr">
@@ -16615,7 +16555,7 @@
       </c>
       <c r="P325" s="0" t="inlineStr">
         <is>
-          <t>The questionnaire asked informants to focus on a NPD project (our unit of analysis) completed in the past 12 months.</t>
+          <t>Verbatim Evidence: \"The questionnaire asked informants to focus on a NPD project (our unit of analysis) completed in the past 12 months.</t>
         </is>
       </c>
     </row>
@@ -16813,7 +16753,7 @@
       </c>
       <c r="P329" s="0" t="inlineStr">
         <is>
-          <t>Our study sample consisted of 2,940 United States Air Force officers from a broad array of job categories, who participated in a five-week leadership development course. As part of the course and a larger program of research,1 the participants were assigned to one of 210 14-person multiteam systems that engaged in a computer-based simulation.</t>
+          <t>Verbatim Evidence: \"Our study sample consisted of 2,940 United States Air Force officers from a broad array of job categories, who participated in a five-week leadership development course. As part of the course and a larger program of research,1 the participants were assigned to one of 210 14-person multiteam systems that engaged in a computer-based simulation.</t>
         </is>
       </c>
     </row>
@@ -16959,11 +16899,7 @@
       <c r="K332" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="P332" s="0" t="inlineStr">
-        <is>
-          <t>Based on our experience and emerging literature, such as the papers in this special collection, this article discusses the value of Q-methodology in addressing landscape sustainability issues.\" (Abstract)</t>
-        </is>
-      </c>
+      <c r="P332" s="0" t="inlineStr"/>
     </row>
     <row r="333" ht="18" customHeight="1" s="31">
       <c r="A333" s="0" t="inlineStr">
@@ -17101,7 +17037,7 @@
       </c>
       <c r="P335" s="0" t="inlineStr">
         <is>
-          <t>To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries.</t>
+          <t>Verbatim Evidence: \"To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries.</t>
         </is>
       </c>
     </row>
@@ -17197,11 +17133,7 @@
       <c r="K337" s="0" t="n">
         <v>1997</v>
       </c>
-      <c r="P337" s="0" t="inlineStr">
-        <is>
-          <t>While formalization measure was modified slightly to be tailored to the unique Korean sales job environment, the other four variables of role ambiguity, role conflict, commitment, and propensity-to-leave were adopted from American literature.\" (Measurement)</t>
-        </is>
-      </c>
+      <c r="P337" s="0" t="inlineStr"/>
     </row>
     <row r="338" ht="18" customHeight="1" s="31">
       <c r="A338" s="0" t="inlineStr">
@@ -17479,11 +17411,7 @@
       <c r="K343" s="0" t="n">
         <v>2007</v>
       </c>
-      <c r="P343" s="0" t="inlineStr">
-        <is>
-          <t>The unit of analysis for the questionnaire was the new product development project and the informant was asked to select the most recent project he/she worked for.\" (3.2. Questionnaire)</t>
-        </is>
-      </c>
+      <c r="P343" s="0" t="inlineStr"/>
     </row>
     <row r="344" ht="18" customHeight="1" s="31">
       <c r="A344" s="0" t="inlineStr">
@@ -17579,7 +17507,7 @@
       </c>
       <c r="P345" s="0" t="inlineStr">
         <is>
-          <t>The samples for the survey comprised IT development MTSs within IT firms located in China.\" (IV. METHODOLOGY, A. Samples and Data Collection)</t>
+          <t>Verbatim Evidence: \"The samples for the survey comprised IT development MTSs within IT firms located in China.\" (IV. METHODOLOGY, A. Samples and Data Collection)</t>
         </is>
       </c>
     </row>
@@ -17627,7 +17555,7 @@
       </c>
       <c r="P346" s="0" t="inlineStr">
         <is>
-          <t>[Team level analysis]. Verbatim Evidence: \\\"We computed within-group interrater agreement (rwg; James, Demaree, &amp; Wolf, 1993) and ICC values to justify the aggregation of constructs to the team level, which provided adequate support.\\\" (Data Analysis)</t>
+          <t>Verbatim Evidence: \"[Team level analysis]. Verbatim Evidence: \\\"We computed within-group interrater agreement (rwg; James, Demaree, &amp; Wolf, 1993) and ICC values to justify the aggregation of constructs to the team level, which provided adequate support.\\\" (Data Analysis)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: inject 2nd screening results and verbatim quotes for Batch 6 (BSMA0011-BSMA0068)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -1442,7 +1442,7 @@
       </c>
       <c r="P14" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Non-employee consumer sample. Verbatim Evidence: \"To test our hypotheses we collected primary data from FlyerTalk forum members via a short survey posted to a brand-independent subsection of the forum. This provided us with access to a large, active and highly diverse respondent pool and reduced the influence of biases one would expect to find in brand-specific forums. By posting to a public forum, we gained access to experienced, valuable, and impartial respondents that would otherwise prove very difficult to get. We incentivized survey participation by offering thirty $10 Amazon gift cards and by minimizing the length of the survey.\" (Methodology and results, Page 289)</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="P15" s="0" t="inlineStr">
         <is>
-          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+          <t>Conceptual review paper proposing hypotheses without primary empirical employee data. Verbatim Evidence: \"Boundaries are a defining characteristic of organizations, and boundary roles are the link between the environment and the organization. The creation, elaboration, and functions of boundary spanning roles are examined, with attention to environmental and technological sources of variation in the structure of boundary roles. Eleven hypotheses integrate the material reviewed and are amenable to empirical test. Future research should overcome problems created when organizations are treated as \"wholes\" or single entities.\" (Abstract, page 217)</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="P16" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Study focuses on work-home boundary management and lacks any measure of organizational boundary spanning behavior. Verbatim Evidence: \"Segmentation Preferences. Six items based on Kreiner’s (2006) segmentation preferences scale were used (e.g., “I don’t like to have to think about work while I’m at home”; “I prefer to keep my non-work life at home”). Responses were made on a 5-point scale that ranged from “strongly disagree” to “strongly agree.” Higher scores indicate greater preferences for segmentation of work and nonwork roles. Segmentation preferences were measured at Time 1. Coefficient alpha = .83. Work-Nonwork Balance. Three items modified from the Greenhaus et al. (2012) work-family balance measure (e.g., “I am able to balance the demands of my work and nonwork”) were used. Responses were made on a 5-point scale that ranged from “strongly disagree” to “strongly agree.”\" (Measures, Page 9)</t>
         </is>
       </c>
     </row>
@@ -1609,14 +1609,10 @@
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F18" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr"/>
       <c r="G18" s="0" t="inlineStr">
         <is>
           <t>To test some of the social and organizational psychology underpinnings of boundary spanning theory, the consultative, boundary spanning activities of 27 New York State school psychologists within their special education multidisciplinary teams were studied. More specifically, the relation between boundary spanning and task uncertainty, role specification, degree of professional training and continuing activity, size of organization, and available organizational resources was investigated. The results indicated that boundary spanning was significantly related to perceived task uncertainty. The implications of these results were discussed, and future research efforts needed to further differentiate this important construct were suggested.</t>
@@ -1642,7 +1638,7 @@
       </c>
       <c r="P18" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The study samples individual organizational employees and provides a quantitative Pearson correlation matrix including boundary spanning behavior. Verbatim Evidence: \"Ultimately, 27 school psychologists (50% of the 54 possible participating districts) returned their boundary spanning questionnaires. Descriptively, there were 16 male and 11 female school psychologists within this sample with ages ranging from 27 to 65 years old (M = 41.14, SD = 8.59). None of these school psychologists held the doctoral degree, 22 (81.5%) held an EdS or a 60 graduate credit hr advanced degree, and 5 (18.5%) held a master's degree. Finally, these school psychologists averaged 5.41 years of experience (SD = 6.32) as MDT members, and none of the school psychologists were serving as the MDT chair.\" (Subjects, Page 347)</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1710,7 @@
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
@@ -1742,7 +1738,7 @@
       </c>
       <c r="P20" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>The study focuses on boundary spanners but lacks a measure and quantitative effect sizes for boundary spanning behavior. Verbatim Evidence: \"Ethical climate was measured using the seven-item scale proposed by Weeks et al. (2004). To measure the job satisfaction facets, the reduced version of the INDSALES scale (Churchill et al., 1974; Comer et al., 1989; Lagace et al., 1993) was adapted for use within a procurement context. Of the seven facets, six were relevant within this study[1]. All items used in this study were measured using seven-point Likert-type scales ranging from 1 (strongly disagree) to 7 (strongly agree).\" (Measurement, Page 5)</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1788,7 @@
       </c>
       <c r="P21" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study does not provide a bivariate Pearson correlation matrix, instead relying on MANOVA and ANOVA to compare categorical decision style groups. Verbatim Evidence: \"Each subject was grouped according to primary decision style which resulted in four groups of individuals being labeled as either SF (n = 20), ST (n = 7), NF (n = 24), or NT (n = 6). Because BSA was defined as multidimensional in nature and was composed of three separate dimensions, the primary analytic technique used was multivariate analysis of variance (MANOVA). This test was run to determine if decision style affected total BSA. Given a significant overall F for the MANOVA test, several post hoc techniques were employed to investigate the specific nature of these differences.\" (Grouping and Analytic Techniques, Page 6)</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1860,7 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
@@ -1892,7 +1888,7 @@
       </c>
       <c r="P23" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Review and conceptual paper. Verbatim Evidence: \"The purpose of this article is to discuss new approaches to performance management in health care services when the purpose is to support innovative changes in the delivery of services. Design/methodology/approach – The article represents cross-boundary work as the theoretical and empirical material used to discuss and reconsider performance management comes from several relevant research disciplines, including systematic reviews of audit and feedback interventions in health care and extant theories of human motivation and organizational control.\" (Abstract, Page 1)</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1938,7 @@
       </c>
       <c r="P24" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>Qualitative case study lacking quantitative employee correlation data. Verbatim Evidence: \"Information was gathered primarily through interviews. Mantere (2008) describes individual interviews as one of the best sources of information when trying to understand the motivations and character of the actions that take place in highly embedded social contexts such as organizations. It allows a deeper understanding of the experiences of boundary spanners, how they are interpreted and related to specific practices. Other data sources included internal documentation in the form of PowerPoint presentations and other material. The case studies were conducted in 2009–2012. For each case, we interviewed managers with experience of managing creative processes across organizational boundaries.\" (4. Research methodology, Page 128)</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2013,7 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
@@ -2045,7 +2041,7 @@
       </c>
       <c r="P26" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>Firm level analysis. Verbatim Evidence: \"The final survey was administered to 307 firms identified through an online business directory. All questionnaires were delivered in person by field agents to the companies. An introductory letter accompanied each questionnaire to explain the purpose of the study and also to assure participants of anonymity and confidentiality of their responses. Although the target respondents were environmental/innovation/production and/or supply chain managers, the guidelines encouraged collaboration among top managers in responding to the survey, as a way of reducing common method bias. After several rounds of reminders (using phone calls to contact persons) and on-site visits by field agents, 204 questionnaires were returned. Compared to previous studies that used a survey method, the response rate was high because field agents visited the companies directly and, in most cases, got to speak with the respondents before leaving the questionnaire with them. Through an initial check, 4 of the returned were considered unusable and dropped from the dataset. This left 200 usable questionnaires. The characteristics of the sample firms are presented in Table 1.\" (Survey and data collection, Page 5)</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2063,7 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
@@ -2095,7 +2091,7 @@
       </c>
       <c r="P27" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>The study treats boundary spanning as a nominal job role (export management) rather than a measured behavioral construct and does not provide a Pearson correlation matrix. Verbatim Evidence: \"We designed an online questionnaire based on the methodology proposed by Dillman (2000) and submitted it to people in charge of export and finance activities in Andalusian firms that export regularly through externalized channels. The population was composed of 656 firms identified by means of a database provided by EXTENDA, an Andalusian public agency that supports internationalization. We obtained 193 valid questionnaires from export managers (29.42%) and 85 from finance directors (12.96%). Due to differences in response rates between both groups, a Fisher-exact test was performed to compare both finance-manager and export-manager samples; results confirmed significant differences between the two response rates (p-value &lt; 0.05), so generalization of group-comparison results should be taken with caution. The response rate of each management group was closely similar to or even over those from previous export management literature,7 allowing us to assume the reliability of each individual sample. In addition to the respondent’s gender, the questionnaire asked for information on the characteristics of the person in the post (formal education in terms of academic degree, time working in the firm, time working in the industry, time working in the current position, and experience in export activities) and the features of the firm (relative size of export team in relation to competitors, time engaged in the main industry, and experience in export activities).\" (Methods, Page 74)</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2113,7 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
@@ -2145,7 +2141,7 @@
       </c>
       <c r="P28" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Firm level analysis. Verbatim Evidence: \"This descriptive study was carried out with the information obtained from a sample of 30 executives from an equal number of companies. The companies in which the respondents work correspond to the following sectors: Food and Beverage (27%), Construction and Industrial (27%), Finance (10%), Technology (7%), Foreign Trade (7%), Retail (7%), Consulting, (7%), Pharmaceutics (3%), Mass Consumption (3%), Telecommunications (3%).\" (4. Methodology, Page 7)</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2163,7 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
@@ -2195,7 +2191,7 @@
       </c>
       <c r="P29" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>The study provides regression results and summary statistics but completely fails to report a bivariate Pearson correlation matrix for the variables. Verbatim Evidence: \"To control for this potential bias, we include firm patents as the number of granted patents filed by the firm between the beginning of 2003 until the end of 2005, and firm co-publications as the number of publications co-authored by the firm’s employees and academic scientists between the beginning of 2003 until the end of 2005. For the small number of individuals who did not fill in the name of the firm, firm patents and co-publications is set at zero, and the binary indicator firm name missing is set at one. Finally, as a robustness check, we include firm-fixed effects for firms with at least two respondents (i.e. 61 firms and 240 R&amp;D scientists), which control for any remaining unobserved firm-level heterogeneity. Table 1 provides a description and summary statistics for all variables.\" (3.2.4 Control variables, Page 923)</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2213,7 @@
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
@@ -2245,7 +2241,7 @@
       </c>
       <c r="P30" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Macro-level economic and supply chain data. Verbatim Evidence: \"In our analysis we have data on prices and the exchange rate for the period January 1988 to December 1999. The Norwegian ex. vessel prices are from Norges Raafisklag, the Norwegian export price to Portugal in Norwegian kroner from the Norwegian Trade Statistics, and the Portuguese retail prices in Portuguese escudos from the Institute of National Statistics. The exchange rate is from International Financial Statistics.\" (Data, Page 7)</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2291,7 @@
       </c>
       <c r="P31" s="0" t="inlineStr">
         <is>
-          <t>Conceptual, theoretical, or literature review article; does not report quantitative empirical dataset or correlation effect sizes.</t>
+          <t>Conceptual paper lacking primary empirical data. Verbatim Evidence: \"Thus, our central question is how do individuals engage in daily role transitions as part of their organizational life? We focus on the transition process, developing propositions regarding the psychological (and, if relevant, physical) movement between roles. Using what we will call \"boundary theory\" as a framework, we describe role transitions as a boundary-crossing activity, where one exits and enters roles by surmounting boundaries (Schein, 1971; Van Maanen, 1982).\" (Introduction, Page 472)</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2313,7 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
@@ -2345,7 +2341,7 @@
       </c>
       <c r="P32" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Firm level analysis. Verbatim Evidence: \"Accordingly, and to ensure that the subsamples contain enough cases for statistical purposes, we purposively generated a sample of 366 firms, with 72.1% and 27.9% being service firms and manufacturing firms respectively. The proportion of these firm categories in our effective sample (n = 117) is similar: 72.6% are service firms while 27.4% are manufacturing firms. The firms sampled were those that met the criteria for the study: employed at least five full-time employees, have at least a form of integration with one or more channel members from the downstream of their supply chain, and with complete contact information.\" (Source of data and field study, page 7)</t>
         </is>
       </c>
     </row>
@@ -2362,14 +2358,10 @@
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F33" s="0" t="inlineStr">
-        <is>
-          <t>1 = No effect size of interest</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="inlineStr"/>
       <c r="G33" s="0" t="inlineStr">
         <is>
           <t>Expatriates provide bene®ts to multinational corporations (MNCs) when they enact boundary spanning roles. They do so by relaying local information and identifying opportunities that meet internal needs of MNCs. To test hypotheses based on social capital and role theories, we surveyed 232 expatriates. The ®ndings indicated that local experience and the diversity of social networks were conducive to the boundary spanning activities of expatriates, whereas environmental uncertainty and overseas experience had little effect. By engaging in boundary spanning activities, expatriates felt less role ambiguity and gained role bene®ts, and were more eager to use the resources that were found within different communities of the host country. In addition, those expatriates who engaged in more boundary spanning activities had higher job satisfaction and more power within their own companies than those who did not.</t>
@@ -2395,7 +2387,7 @@
       </c>
       <c r="P33" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Individual-level organizational employee sample with quantitative correlation matrix including boundary spanning behavior. Verbatim Evidence: \"A sampling frame was created in 1998 based on the directories of the Hong Kong Japanese Association, the American Chamber of Commerce, and the British Chamber of Commerce. Most Japanese expatriates had joined the first association while most Western expatriates belonged to one or another of the other two associations. In this sampling frame, we chose only middle and high level expatriates who belonged to service sectors, including banking and finance, retailing and wholesaling, consulting, shipping, and accounting. We expected that expatriates of the chosen ranks in these sectors were likely to have some outside contacts, and would therefore find the boundary spanning survey meaningful.\" (2.3.2. Procedure, page 4)</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2409,7 @@
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
@@ -2445,7 +2437,7 @@
       </c>
       <c r="P34" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Firm level analysis. Verbatim Evidence: \"To obtain a list of ISO 14001 certified companies, we contacted the accredited certification bodies in Pakistan, which maintain databases of their clients. We assured the accreditation bodies that all shared data would remain confidential and would not be disclosed or shared with any third parties. The study focused on individual companies, and 377 firms were identified with ISO 14001 certification. As a result, 183 survey responses were obtained. The survey questionnaire was in English, as professionals and middle managers in Pakistan frequently speak English.\" (Data Collection, Page 6)</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2459,7 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
@@ -2495,7 +2487,7 @@
       </c>
       <c r="P35" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>The quantitative survey only measures corporate culture indices and lacks a measure for boundary spanning behavior. Verbatim Evidence: \"The mean scores and standard deviations for each index of the Corporate Culture Index using the total sample are shown in Table 7. The differences among the mean scores on the indexes are fairly small, ranging from slightly above four (neutral) to slightly above five (midly agree). The size of the standard deviations for each index indicates that a great majority of the managers' ratings of the descriptive terms fell in the area of agreement rather than disagreement. The managers alone tended to agree more than disagree with respect to corporate culture being more bureaucratic and universalistic. [...] Table 8 presents the intercorrelations among the five indexes. [...] There are five significant, positive correlations: supportive with innovative; particularistic with bureaucratic and supportive; universalistic with innovative and supportive. There is also a significant, negative correlation between particularistic and innovative.\" (Statistical Findings, page 323-325)</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2509,7 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
@@ -2545,7 +2537,7 @@
       </c>
       <c r="P36" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>Firm and alliance level analysis. Verbatim Evidence: \"To test these hypotheses, we collected data through a field study and a large-scale survey. We randomly selected a sample of 500 firms with strategic alliances from a directory provided by a marketing research firm located in Shenzhen, China. Top executives of the firms served as the first key informants. Well-trained interviewers telephoned these top executives and obtained oral agreements from 352 of them to participate. Of the 352 firms contacted, we successfully interviewed 311 firms. Following the interview with the top-level alliance boundary spanners, we asked each of them to set up a meeting with an operating-level alliance boundary spanner who was responsible for a specific project with the alliance partner. Sixteen samples had extensive missing values, so the final sample consisted of 295 firms with two matched informants, a response rate of 59.0% (295/500).\" (Methods, Page 6)</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2559,7 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
@@ -2595,7 +2587,7 @@
       </c>
       <c r="P37" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>The study conducts its analysis at the team level, where individual survey responses were aggregated into work group responses. Verbatim Evidence: \"At least three team meetings were also attended and observed during each visit, and 4-hour unguided tours of the manufacturing areas were taken to permit informal discussions with operators. Finally, employee surveys were distributed to two to four operators per work group at each fab. Multiple responses were averaged together to serve as the group response.\" (3.2. Data collection, Page 4)</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2687,7 @@
       </c>
       <c r="P39" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Non-employee student sample. Verbatim Evidence: \"The sample consisted of 304 first-year M.B.A. students at a large midwestern university. All students were enrolled in the full-time residential M.B.A. program, which divided students into four cohorts, each further partitioned into teams consisting of three to five members. Students remained in the same team for all of their classes during a semester and were required to submit several team-based projects in addition to individual assignments and examinations.\" (METHODS, page 10)</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2709,7 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
@@ -2745,7 +2737,7 @@
       </c>
       <c r="P40" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Conceptual review paper lacking empirical data on individual organizational employees. Verbatim Evidence: \"Designing a supply chain network provides the basic structure for supply chain operations, where the network is a major element in a firm’s competitiveness and a significant area of capital investment. With the boundary-spanning scope encouraged by supply chain management, the question is whether existing analyses used for network design are adequate. The general answer is yes, because the number of echelons that the analysis must span is self-limiting to a relative few. However, there remain unresolved issues in network design analysis and in the models used to support the analysis that can enhance its accuracy, appropriateness, and acceptability to practitioners.\" (Abstract, Page 417)</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2759,7 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
@@ -2795,7 +2787,7 @@
       </c>
       <c r="P41" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Firm-level analysis. Verbatim Evidence: \"The samples of this empirical study were mainly acquired through a large-scale questionnaire survey of the firms in Shenzhen high-technology industrial development zones (HIDs), Zhuhai HIDs and Huizhou Zhongkai HIDs of Pearl River Delta. First, 600 registered firms were randomly selected from the above three high-tech parks. [...] The researchers contacted the CEOs or senior management teams of all firms by phone or email to confirm their willingness to participate in the study and then conducted the questionnaire survey and collection personally. Upon actual contact, a total of 442 firms were willing to participate in this study and a total of 320 firms completed their questionnaires. After incomplete and invalid questionnaires were excluded, a total of 287 firm samples were finally selected for the empirical analysis of this study, with a recovery rate of 47.83%.\" (Method, sample and data, Page 7)</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2837,7 @@
       </c>
       <c r="P42" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>Qualitative case study of open source community mailing list interactions without a Pearson correlation matrix. Verbatim Evidence: \"The first step of our study was to identify and select some successful ‘‘pushed-by-users’’ design proposals using field interviews, and to collect traces of exchanges regarding one of these proposals, in python-dev and python-list. The second step was to identify the participants and cross-participants involved and their statuses. The final step was to analyse interactions, design and boundary spanning activities, in particular those of users and cross-participants.\" (4. Method, Page 5)</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2859,7 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
@@ -2895,7 +2887,7 @@
       </c>
       <c r="P43" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The study analyzes data at the organizational subunit level rather than the individual employee level. Verbatim Evidence: \"Autonomy is defined as the degree to which one may make significant decisions without the consent of others (Brock, 2003). Autonomy in the current context is treated as autonomy of an organizational subunit and not that of the whole organization to which the subunit is a part. Thus the unit of analysis is the subunit and the freedom the head of the subunit has in decision making is considered the autonomy of the subunit.\" (5.1.1 Construct definition, Page 7)</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2909,7 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
@@ -2945,7 +2937,7 @@
       </c>
       <c r="P44" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>Spearman rank correlation matrix instead of Pearson correlation matrix. Verbatim Evidence: \"Hypotheses 1a–2b were tested by quantitative correlation analysis (n =118 boundary spanners). For this test we used Spearman’s rank correlation coefficient (Spearman’s ρ, two-tailed), a non-parametric measure of statistical dependence between two variables. We chose Spearman rank correlations because they do not involve any assumptions of sample size or distribution of observations (Lind, Marchal, &amp; Wathen, 2010). Hence they allow statistical analyses based on relatively low sample sizes and also correct for the non-normality stemming from the long-tail pattern of our data, in which some individuals scored high on our measures but the majority scored low.\" (Quantitative analysis, Page 10)</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2987,7 @@
       </c>
       <c r="P45" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>Conceptual encyclopedia entry without primary empirical data. Verbatim Evidence: \"In terms of future research, recent calls have emphasized the need to study boundary spanning at the activity level; that is, in terms of the specific actions taken by boundary-spanning individuals, and their consequences (Birkinshaw et al., 2017; Søderberg &amp; Romani, 2017; see also Schotter et al., 2017) to enrich and deepen the insights gleaned from extant interview-based and cross-sectional research. Recent research has also differentiated between potential boundary spanners, i.e., individuals who are involved in inter-unit interactions, and recognized boundary spanners who are experienced by relevant others on both sides of the boundary to actually facilitate and positively impact intergroup transactions and relations (Mäkelä et al., 2019).\" (Global boundary spanners, Page 110)</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3099,7 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
@@ -3135,7 +3127,7 @@
       </c>
       <c r="P48" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>Purely qualitative case study based on interviews without quantitative effect sizes. Verbatim Evidence: \"In total, 42 interviews were conducted over three phases with a wide range of participants: senior managers of JAMSURE and its sister companies in IT, life, and general insurance company; project managers, team leaders, and developers at the IT and general insurance companies; and intended users and managers of the GENSYS system. We conducted repeat interviews with Indian project manager and the Jamaican manager who headed the development effort, and four of the five team leaders of Indian and Jamaican descent. We also interviewed twice both the CEO of GENSURE and of GROUPIT, as well as the Director of Operational and implementation manager at GENSURE responsible for implementing GENSYS.\" (Research methodology, page 8)</t>
         </is>
       </c>
     </row>
@@ -3230,7 +3222,7 @@
       </c>
       <c r="P50" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>This is a commentary/reply piece without empirical data on employees. Verbatim Evidence: \"IN THEIR COMMENTARY in this issue of the Journal of Studies on Alcohol and Drugs, Bray and Kenkel (2024) write, “It would be unfortunate if readers came away with nothing more than a distrust of Jon Nelson’s work” (p. 428). With that, we wholeheartedly agree. The key message of our article (Bartlett &amp; McCambridge, 2024) is that boundaries between disciplines, or fields of study, are boundaries between communities of science, and we draw attention to the concept of boundary work and the nature of the work involved, the early stage of explicit normative debates about these issues in alcohol science, and the need for alcohol public health science in particular to make progress on these issues due to targeting by the alcohol industry.\" (Commentary, page 430)</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3389,7 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
@@ -3425,7 +3417,7 @@
       </c>
       <c r="P54" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Firm-level analysis. Verbatim Evidence: \"The study is descriptive and cross-sectional in nature. A purposive sample of 457 North Indian organizations was taken for conducting this study. The senior - level key executives, who had decision-making power in the organization, were considered as key informants. Data were collected through a personal survey in the year 2016.\" (Methodology, Page 4)</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3631,7 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
@@ -3667,7 +3659,7 @@
       </c>
       <c r="P59" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Conceptual research note without employee correlation data. Verbatim Evidence: \"Given the four enablers presented in the previous section, and considering four typical phases of BPM (cf. Fig. 1), the authors conducted a workshop session, supplemented by follow-up discussions. In the workshop session, groups of 3–4 researchers discussed how – from their point of view – one of the identified technological enablers impacts the BPM discipline. All researchers involved in this session had a long standing record of projects and publications in the BPM field. As a result, a total of 60 consequences for the BPM field were identified. These consequences were presented, discussed, and consolidated in the entire group of 16 researchers.\" (Implications for BPM, Page 150)</t>
         </is>
       </c>
     </row>
@@ -3684,14 +3676,10 @@
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F60" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F60" s="0" t="inlineStr"/>
       <c r="G60" s="0" t="inlineStr">
         <is>
           <t>When the ordering function is governed by administrative arrangements and sales are regulated by long-term contracts, managers may question the necessity and the tasks of the sales function within established customer relationships. The authors examine three issues related to the role of the salesperson in established industrial buyer-seller relationships: (1) appropriate measures of salesperson performance within a relationship, (2) behaviors and skills affecting salesperson performance, and (3) the effect of salesperson performance on the relationship. The results from a survey of industrial buyers suggest that the salesperson has a significant and substantial effect on relationship continuity. They also show that the salesperson contributes to perceptions of the supplier's reliability and supplier services. The key attributes of an effective salesperson are ability to resolve conflicts, ability to develop a personal relationship with customers, and ability to facilitate exchange of information between the supplier and buyer firms.</t>
@@ -3717,7 +3705,7 @@
       </c>
       <c r="P60" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>The study samples individual organizational employees and provides an individual-level Pearson correlation matrix measuring specific salesperson boundary spanning behaviors (e.g., information exchange, conflict resolution). Verbatim Evidence: \"The data used to test the hypotheses were collected in a mail survey of industrial buyers. We wanted the population selected for the study to reflect a variety of purchasing practices to avoid biases due to using a specific industry or one or a few dominating suppliers. An extensive questionnaire was mailed to a total of 576 companies. These were selected from databases covering the information technology industry, the apparel and sports equipment industry, the food processing industry, manufacturers of chemicals and of cosmetics, the pharmaceutical industry, and miscellaneous other industries. The informant was the person responsible for purchases of the product category in question. In order to generalize from the data, our main premise was that relational selling behavior should apply to various categories of purchased goods. Thus, the informant was asked to identify a supplier of packaging, a supplier of component parts, and a supplier of accessories. For each of the three chosen suppliers, informants were asked to evaluate the supplier’s salesperson on several behaviors in addition to characteristics of the buyer-supplier relationship.\" (METHODS, Page 18)</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3782,7 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
@@ -3822,7 +3810,7 @@
       </c>
       <c r="P62" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Regional and sector level analysis. Verbatim Evidence: \"Employment data for sub-regions of Great Britain at the two-digit industry level were obtained from the UK’s National On-line Manpower Information System (NOMIS) utilizing the 1992 Standard Industrial Classification (SIC) classification scheme and covering the period 1995–2002. It is difficult to examine longer-term trends due to the changes to the system of collecting employment data from 1998 onwards. Data from 1995 to 1997 have been rescaled to be consistent with the new system, but earlier data reflect the previous system (PARTINGTON, 2001). Data were collected for 203 areas at the local authority, county, and unitary authority levels.\" (Data, Page 448)</t>
         </is>
       </c>
     </row>
@@ -3894,7 +3882,7 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
@@ -3922,7 +3910,7 @@
       </c>
       <c r="P64" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Editorial and literature review. Verbatim Evidence: \"To gain a thorough overview of prior research on the links between business model innovation and grand challenges, we conducted a comprehensive database search on EBSCOHost, ScienceDirect, and Web of Science (Bartels &amp; Reinders, 2011), encompassing articles available through December 31, 2024. We conducted three separate database searches (details in the Supporting Information Appendix) on BMI research in the context of each of the three identified grand challenges: artificial intelligence (AI), business and global unrest, and climate change. During the first step of the search process, we sourced 304 articles for BMI and AI, 27 for BMI and business/global unrest, and 60 for BMI and climate change. In the second step, duplicates were eliminated, and the eligibility of the remaining articles was assessed through a thorough analysis of the full texts.\" (2 | LITERATURE BASE LINKING BMI TO GRAND CHALLENGES, Page 3)</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3932,7 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
@@ -3972,7 +3960,7 @@
       </c>
       <c r="P65" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study sampled non-employee business owners rather than individual organizational employees. Verbatim Evidence: \"Data were collected among Dutch entrepreneurs owning private companies with fewer than 250 employees (cf. Jayasekara et al., 2020). They were recruited via network organizations (e.g. FNV Zelfstandigen), magazines, LinkedIn Groups, and a database (i.e. Prolific). After completing the informed consent, respondents filled out the questionnaire. Confidentiality and anonymity were emphasized and assured. The study was approved by the Ethics Review Board of the first author’s university.\" (Methods, Page 7)</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4010,7 @@
       </c>
       <c r="P66" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study focuses on work-family and work-nonwork boundary management fit rather than organizational boundary spanning behavior, meaning it does not contain the necessary constructs or effect sizes of interest. Verbatim Evidence: \"Recently, work-family scholars have empirically demonstrated the importance of congruence between employees’ boundary management preferences and boundary management supplies provided by the work environment in relation to employee attitudes and behavior. However, a theoretically grounded construct that captures this congruence is lacking. The present study addresses this gap by developing the construct and measure of work-nonwork boundary management fit, based on the needs-supplies fit framework. We cross-validate the scale in three independent samples (n = 188, diverse group of employees, n = 75, employees from one hospital, and n = 81, employees from one car company) and in a fourth sample (n = 458, working parents), we demonstrated the importance of work-nonwork boundary management fit for employee well-being (i.e., stress and work-life conflict). In particular, we confirmed its unique role in predicting employee well-being, above and beyond workload and work interrupting nonwork behaviors. Hence, we argue for considering work-nonwork boundary management fit when studying how work-family policies and organizational culture affect employees in the workplace.\" (Abstract, Page 1)</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4032,7 @@
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
@@ -4072,7 +4060,7 @@
       </c>
       <c r="P67" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Qualitative interview study without quantitative effect sizes. Verbatim Evidence: \"Given the exploratory nature of the research agenda, the semi-structured interview was selected as the most appropriate method for collecting data. The interviews began with open-ended questions concerning the participants’ motivation for and experience of working at these Queenstown hotels. Following this, the interview questions sought to explore what these individuals felt were the positive and negative features of their current work experience. The interviews with the managers were extended by questions relating to their particular HRM related operational issues. [...] The 67 transcribed interviews were read initially to select out those who worked within the Housekeeping Department. Of the 67 hotel employees I interviewed, 10 were involved in housekeeping. Four were in management positions, five attended rooms and one ran the laundry.\" (Procedure and Analysis, page 164)</t>
         </is>
       </c>
     </row>
@@ -4135,14 +4123,10 @@
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F69" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F69" s="0" t="inlineStr"/>
       <c r="G69" s="0" t="inlineStr">
         <is>
           <t>Research has shown that NPD project leaders should engage in boundary-spanning activities. The present study tested the impact of four boundary-spanning activities on NPD project performance and analyzed the antecedents of these activities. We hypothesized that NPD project leaders' abilities to perform these activities depend on the characteristics of their personal networks — structural holes, strength of ties, vertical and horizontal bridging ties. A Partial Least Squares test on 73 NPD projects showed that (a) “obtaining political support” and “scanning for ideas” are the boundary activities with the greatest impact on performance, (b) project leaders with strong ties in their network are more effective at these activities, (c) project leaders with structural holes in their networks are more effective in another boundary activity, “protecting the team”, although this activity does not affect NPD outcomes. These results represent an important contribution to understanding how team leaders contribute to project performance.</t>
@@ -4168,7 +4152,7 @@
       </c>
       <c r="P69" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>The study meets all inclusion criteria as it measures individual-level boundary spanning behaviors of project leaders without team-level aggregation and provides a Pearson correlation matrix. Verbatim Evidence: \"The study was conducted on a sample of 73 project leaders in manufacturing firms (Section 3.1) and assessed the variables of NPD outcomes, boundary-spanning activities, network characteristics, and controls (Section 3.2). We used a sample of project leaders involved in NPD projects in a variety of industries. The study used name generators, with respondents being asked to name contacts who played a role in their day-to-day professional activities. Project leaders were required to complete the questionnaire with reference to a completed NPD project.\" (Sample and measures, Page 7)</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4202,7 @@
       </c>
       <c r="P70" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>No bivariate Pearson correlation matrix or boundary spanning behavior effect size is provided. Verbatim Evidence: \"Descriptive statistics including frequencies, percentages, means, medians, SDs, and interquartile ranges were used to describe levels of burnout and resilience and to examine perceptions of the curriculum. Statistical tests appropriate for small sample sizes were used. Wilcoxon 2-sample tests were conducted to identify sex or year of training differences in burnout and resilience at baseline. Wilcoxon signed rank tests were used to evaluate changes in level of agreement from pre to post intervention on items assessing beliefs, knowledge, and self-efficacy. Two-sided p values &lt; 0.05 were assumed to indicate statistical significance.\" (Statistical analysis, page 540)</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4224,7 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
@@ -4301,7 +4285,7 @@
       </c>
       <c r="P71" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>No effect size of interest. Verbatim Evidence: \"This study explored the perceptions of fire officers on effective organizational leadership in the American fire service to discover what is shared among varied perspectives and what is distinct, and to analyze how the perspectives align with existing leadership theories and models. It employed Q methodology, which includes both qualitative and quantitative data-collection and analysis. Ten distinct perspectives emerged from the data that have varying degrees of fit with existing theories, including (listed alphabetically) adaptive leadership theory, authentic leadership theory, boundary-spanning leadership theory, complexity leadership theory, crew resource management, leader-member exchange theory, learning organization model, the managerial grid, Mintzberg’s model of management, public administrative leadership theory, regulatory focus theory, servant leadership theory, and transformational leadership.\" (Abstract, page 6)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: inject 2nd screening results and verbatim quotes for Batch 7 (BSMA0069-BSMA0108)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -4307,7 +4307,7 @@
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="P72" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Practitioner review and conceptual summary of a book without quantitative correlation data. Verbatim Evidence: \"This article is based on the authors’ book, Boundary Spanning Leadership: Six Practices for Solving Problems, Driving Innovation, and Transforming Organizations (McGraw-Hill, 2010). The presented information reflects the experiences of actual leaders who participated in two Center for Creative Leadership (CCL) research projects: Leadership Across Differences (LAD), which involved researchers from around the world; and Leadership at the Peak, which collected survey data from senior executives participating in leadership programs. Findings from this study informed our thinking in two primary ways. First, they reinforced our belief that while spanning boundaries is now critical, it remains challenging. Our data showed that 86% of senior executives found it 'extremely important' to work effectively across boundaries in their current leadership role. Yet only 7% of these executives believed they were currently 'very effective' at doing so — a gap of 79% between the perceived importance of boundary spanning and the ability to achieve it.\" (About the Research, Page 4)</t>
         </is>
       </c>
     </row>
@@ -4353,14 +4353,10 @@
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F73" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F73" s="0" t="n"/>
       <c r="G73" s="0" t="inlineStr">
         <is>
           <t>This dissertation examines the extent to which organizational and professional commitment, the technical environment, and the professional environment are related to boundary spanning activity. Surveys of R&amp;D professional employees, their co-workers, and their managers were used to obtain measures of commitment to their organizations and professions, perceptions of the technical and professional environment in which they worked, and the frequency with which they communicated both within and outside of the R&amp;D unit.</t>
@@ -4384,7 +4380,11 @@
       <c r="K73" s="0" t="n">
         <v>1995</v>
       </c>
-      <c r="P73" s="0" t="inlineStr"/>
+      <c r="P73" s="0" t="inlineStr">
+        <is>
+          <t>The study meets all inclusion criteria by sampling individual organizational employees and providing a Pearson correlation matrix. Verbatim Evidence: \"The targeted population was R&amp;D technical professionals in high technology industries. Previous studies of boundary spanning activity have focused on professionals engaged in research and development activity. Because this study sought to extend the findings from previous research, sampling from the same population was appropriate. The final sample consisted of 253 R&amp;D professionals in six firms drawn from a variety of high technology industries.\" (Sample, Page 32)</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="18" customHeight="1" s="31">
       <c r="A74" s="0" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="P74" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Firm level analysis of nonprofit organizations. Verbatim Evidence: \"Initially, there are over 7,000 organizations reporting nonzero revenues for fiscal 1992 to fiscal 1994, the latest complete year of data available on the 1996 database. We impose two selection criteria. First, we require the nonprofit to receive in 1992 over $2.5 million in direct contributions (private donations less funds raised by other organizations, such as United Way). Second, we further require that direct contributions exceed 10% of total 1992 receipts. We thus focus on organizations with significant donations. These rules reduce the sample to 473 organizations.\" (Sample Selection, page 113)</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="P75" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>The study analyzes interorganizational networks where the primary unit of analysis is the organization, rather than individual-level employee behaviors. Verbatim Evidence: \"The sites included from 31 to 44 organizations that provide mental health and other community support services to persons with a chronic or serious and persistent mental illness. ... Data about the formal network of services at each site were gathered from a key informant (or ‘boundary spanner’) in each organization. Boundary spanning roles (Aldrich and Herker 1977; Tushman and Scanlan 1981) are those occupied by persons who serve as liaisons with other organizations or who are deemed as particularly knowledgeable about the organization’s relationships (e.g. agency, unit, or program director).\" (2. Data collection, page 6)</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="P76" s="0" t="inlineStr">
         <is>
-          <t>Qualitative field interview study without individual employee Pearson correlation matrix. Verbatim Evidence: "Some interviewees were less concerned by this lack of basic training, believing instead that the onshore... For example, in the sample we checked if the cut-off of the invoices was correct." (Abstract / Findings section)</t>
+          <t>Qualitative case study without quantitative correlation data. Verbatim Evidence: \"Given that the objective of this study is to develop our understanding of how and why offshoring emerged as an organizational matter, changing the way audit work is organized and perceived in a Big 4 firm, a qualitative research methodology was deemed most appropriate (Cooper and Morgan 2008; Denzin and Lincoln 2003; Flick 2006; Given 2008; Silverman 2000). More specifically, we used a case study approach (Cooper and Morgan 2008) drawing upon multiple data sources—documentary data, in-depth interviews, and digital data—to obtain detailed information about the complexities underpinning the real-life phenomenon (Miles and Huberman 1994; Patton 2002) of offshoring in audit.\" (IV. RESEARCH METHOD, Page 64)</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="P77" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Team-level analysis focusing on NPD projects rather than individual employees. Verbatim Evidence: \"The questionnaire was addressed to the person in the company responsible for NPD activities. These individuals were instructed to answer the questionnaire in relation to a recently completed NPD project that he or she had led and for which the NPD team was engaged in boundary spanning activities. A total of 146 completed surveys were returned. Those that responded to the first survey received a second questionnaire. This questionnaire collected data on the remaining variables in the model. For the second round, respondents were reminded of the NPD project chosen to answer the first survey and asked to answer the survey having the same project in mind. A total of 140 of the 146 firms contacted, completed the second survey.\" (Methodology, Page 6)</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4604,7 @@
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
@@ -4632,7 +4632,7 @@
       </c>
       <c r="P78" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Team-level analysis. Verbatim Evidence: \"The unit of analysis was a recently launched NPD project in which the NPD team in charge had partaken in boundary spanning activities. The sampling frame for the study were Spanish manufacturing firms in high- and medium-technology sectors listed in the Amadeus database. The food and beverages manufacturing sector, although classified as low-technology, was also included in the sampling frame because of its high values of R&amp;D spending (INE, 2021). We randomly selected 25 percent of the firms in each of the industry groups, which resulted in 946 manufacturing firms.\" (Methodology, Page 12)</t>
         </is>
       </c>
     </row>
@@ -4654,7 +4654,7 @@
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="P79" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Project level analysis. Verbatim Evidence: \"During the first stage of the data collection, a questionnaire focused on boundary-spanning activities of NPD teams was mailed to each of the companies in our database. This questionnaire was addressed to the person in the company responsible for NPD activities. Respondents were instructed to answer the survey questions with regard to a recently completed NPD project that they had led or managed. It was requested that the product be in the market for at least six months (Im et al., 2013). Also, at this point, potential respondents were informed that as part of the same research project, a follow-up questionnaire would be administered at a later date. For this first round, a total of 146 completed surveys were obtained.\" (Sample and Data Collection, Page 7)</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,12 @@
       </c>
       <c r="E80" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
@@ -4727,7 +4732,7 @@
       </c>
       <c r="P80" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>The study is a narrative summary of quantitative and qualitative data that focuses on broad themes and practical strategies. It fails to report any specific quantitative effect sizes, such as a bivariate Pearson correlation matrix involving boundary spanning behavior. Verbatim Evidence: \"We set out to identify drivers of inclusion in the average professional network by assessing networks within many organizations. We were privileged to have access to network data collected from more than 30 organizations and 16,500 people over 15 years across a range of industries. To supplement our quantitative analyses, we also conducted 125 interviews with individuals at different levels in their organizations and in different positions in networks.\" (Page 5)</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4754,7 @@
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
@@ -4777,7 +4782,7 @@
       </c>
       <c r="P81" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study conducts a team-level analysis where data is aggregated to the unit level. Verbatim Evidence: \"In this study, the unit was considered to be the level of analysis. Hence, all measures were specified at the unit level. Respondents were asked to evaluate the relational capital, knowledge combination capabilities, and performance of the unit.\" (Measures, page 91)</t>
         </is>
       </c>
     </row>
@@ -4827,7 +4832,7 @@
       </c>
       <c r="P82" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>No measure of boundary spanning behavior. Verbatim Evidence: \"Job performance. This measure was evaluated by a scale developed by Pearce and Porter (1986) and used by Black &amp; Porter (1991). This measure is a respondent self-evaluation with five items measured on a seven-point scale (ranging from 1 = strongly disagree, to 7 = strongly agree). It contains five dimensions as follows: overall performance, ability to get along with others, completing tasks on time, quality of performance, and achievement of work goals.\" (Measures, Page 9)</t>
         </is>
       </c>
     </row>
@@ -4849,7 +4854,7 @@
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
@@ -4877,7 +4882,7 @@
       </c>
       <c r="P83" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Firm-level analysis. Verbatim Evidence: \"This study’s major goal is to extend the model that describes the relationship between perceived organizational reputation and the firm’s performance by looking at the firm’s performance as a multidimensional measure. The authors use CEOs, beliefs and evaluation of their company’s reputation as proxies of the actual reputation of the firm (ie perceived organizational reputation). It would have been preferable to use objective data, but unfortunately they were not available for the companies in this study. Specifically, this study aims to show that the organization’s reputation affects the organization’s financial performance and its market performance differently.\" (Introduction, Page 14)</t>
         </is>
       </c>
     </row>
@@ -4899,7 +4904,7 @@
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
@@ -4927,7 +4932,7 @@
       </c>
       <c r="P84" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>Non-primary review study. Verbatim Evidence: \"The purpose of this review is to clarify the nature of functional leadership in interteam contexts, integrate and critically evaluate relevant findings from prior research, and identify promising areas for future inquiry. Broadly, leadership is defined as a “process of influencing others to understand and agree about what needs to be done and how to do it, and the process of facilitating individual and collective efforts to accomplish shared objectives” (Yukl, 2006, p. 8). Thus, leadership processes are situated in relation to specific individuals and/or collectives (where is leadership targeted?) and are enacted to facilitate specific objectives (why is leadership enacted?). As we depict in Fig. 2, these two questions of where and why are useful for organizing studies of leadership processes in intergroup contexts into four categories.\" (Review approach, Page 2)</t>
         </is>
       </c>
     </row>
@@ -4944,14 +4949,10 @@
       </c>
       <c r="E85" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F85" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F85" s="0" t="n"/>
       <c r="G85" s="0" t="inlineStr">
         <is>
           <t>Even though empirical studies examining leadership and effectiveness in multiteam systems (MTS) are on the rise, there is still much to learn about leading a complex “team of teams,” particularly in a field setting as opposed to a laboratory simulation. This study draws upon the multiteam systems and intergroup leadership theory literature streams to examine the role of systems thinking and leader identification as antecedents to intergroup leadership, arguing that higher levels of systems thinking and stronger leader identification with the MTS will enhance the efficacy of leader rhetoric targeted toward the development of an intergroup relational identity with boundary spanning acting as a positive moderating influence on this relationship. I further argue team functional diversity moderates the relationship between intergroup leadership and MTS effectiveness such that higher levels of intergroup leadership are needed to positively influence MTSs with higher levels of heterogeneity. Finally, team identification is evaluated for its predicted moderating effect on the relationship between intergroup leadership and MTS effectiveness such that identification with the MTS will have a positive effect on this relationship while identification with the component team will detract from it. Hypotheses were tested but not supported using a sample of 256 commanders at the squadron, group, and wing level organized in 180 MTSs within the Department of the Air Force. Supplemental analysis identified a significant positive moderating effect of systems thinking and a negative moderating effect of leader component team identification on the relationship between leader rhetoric and intergroup relational identity. Low levels of boundary spanning coupled with higher levels of intergroup relational identity resulted in lower MTS effectiveness while the opposite was true for high levels of boundary spanning and intergroup relational identity. The study concludes with a discussion of theoretical and practical implications as well as recommendations for future research.</t>
@@ -4975,11 +4976,7 @@
       <c r="K85" s="0" t="n">
         <v>2021</v>
       </c>
-      <c r="P85" s="0" t="inlineStr">
-        <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
-        </is>
-      </c>
+      <c r="P85" s="0" t="inlineStr"/>
     </row>
     <row r="86" ht="18" customHeight="1" s="31">
       <c r="A86" s="0" t="inlineStr">
@@ -5027,7 +5024,7 @@
       </c>
       <c r="P86" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>Qualitative study without quantitative effect sizes. Verbatim Evidence: \"This study focuses on the strategies that scholar-practitioners develop to balance their different roles across academia and the practice world. For this purpose, we conducted a qualitative study of experienced scholar-practitioners and developed a grounded model about the strategies that scholar-practitioners use to deal with multiple role conflicts. The next subsections detail the data collection strategy and the methodology for data analysis.\" (Method, Page 440)</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5046,7 @@
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G87" s="0" t="inlineStr">
@@ -5077,7 +5074,7 @@
       </c>
       <c r="P87" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Qualitative case study based on management interviews lacking quantitative individual-level correlation data. Verbatim Evidence: \"The study reported on here was based primarily on a series of interviews with senior management of three offshore oil fields in the UK Continental Shelf. In all cases the operator of the fields was BP, although interviews were also conducted with BP’s partners, allies, and suppliers. The fields are distinguished from each other by the stage of ‘upstream’ activity underway at the time of the study (see Fig. 1). Taken together, the three fields provide examples of most pre-production activities in the upstream oil sector.\" (Background to the Case Studies, Page 246)</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5096,7 @@
       </c>
       <c r="F88" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G88" s="0" t="inlineStr">
@@ -5127,7 +5124,7 @@
       </c>
       <c r="P88" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Patent and firm level analysis. Verbatim Evidence: \"Our analysis exploits USPTO patent and inventor data on a sample of US-based MNEs operating in the pharmaceutical and semiconductor industries. To identify these MNEs, we draw on the NBER patent database (Hall, Jaffe, &amp; Trajtenberg, 2001) that collects US patent and citation data, as well as on the “Disambiguation and co-authorship networks of the U.S. patent inventor database” (Li et al., 2014). First, from the NBER patent database, we select all firms that are assignees of patents granted in the period 1997-2006. Among them, we retain only companies headquartered in the US, using location information from Compustat.\" (Data, page 7)</t>
         </is>
       </c>
     </row>
@@ -5149,7 +5146,7 @@
       </c>
       <c r="F89" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G89" s="0" t="inlineStr">
@@ -5177,7 +5174,7 @@
       </c>
       <c r="P89" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study does not examine individual employees but uses the modification request (task/project level) as the unit of analysis. Verbatim Evidence: \"The unit of analysis is the modification request which corresponds to a development work item associated with a defect or a new feature. A total of 2375 multi-team modification requests were identified. Those modification requests belonged to the first four releases of the product and involved more than one software development team. The decision to focus on such modification requests is based on a growing body of research which shows that difficulties in communication and coordination breakdowns are recurring problems in software development [15][28][34], particularly when the work items are geographically distributed [28] and the task involves more than one organizational team [15][20][34].\" (4.1 Description of the Data, page 6)</t>
         </is>
       </c>
     </row>
@@ -5199,7 +5196,7 @@
       </c>
       <c r="F90" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G90" s="0" t="inlineStr">
@@ -5227,7 +5224,7 @@
       </c>
       <c r="P90" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Project level analysis. Verbatim Evidence: \"The finalized questionnaires were administered to key informants in major Korean manufacturing firms who had recent experience with participating in NPD projects as project leaders or members. In the end, 169 usable questionnaires were obtained on which we empirically test our model. The final sample consists of NPD projects in the following sectors: automobile (7.6%), electrical (14%), electronic (39.5%), telecommunication (14.5%), steel (15.7%), chemical (5.8%), and others (2.9%).\" (4.2. Sample, page 18)</t>
         </is>
       </c>
     </row>
@@ -5249,7 +5246,7 @@
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
@@ -5277,7 +5274,7 @@
       </c>
       <c r="P91" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Program level analysis. Verbatim Evidence: \"In the second stage, the questionnaire gathered data regarding interdepartmental interaction and interdepartmental collaboration integration (eleven items), product vision (three items), and new product competitive advantage (six items). The 321 questionnaires were then sent to those who returned effective questionnaires during the first stage. Of the 278 questionnaires recovered, thirteen were invalid and 265 were effective. The response rate was 17.31%, and respondents included 251 M&amp;A and fourteen non-M&amp;A companies. This study used program level as a basis for evaluating NPD performance, and analyzed the 251 returned questionnaires on M&amp;A.\" (3.1.2. The second stage of the questionnaire survey, Page 5)</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5296,7 @@
       </c>
       <c r="F92" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G92" s="0" t="inlineStr">
@@ -5327,7 +5324,7 @@
       </c>
       <c r="P92" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Firm level analysis focusing on overseas M&amp;A, alliances, and patent networks. Verbatim Evidence: \"From the Bvd-Orbis M&amp;A database, we selected samples of Chinese manufacturing firms’ overseas M&amp;A by considering multiple criteria. (1) The acquirer holds more than 50% of the shares. (2) The M&amp;A transactions occurred between January 2012 and December 2019. This is because China has successively issued policies for intelligent manufacturing since 2012. Also, to ensure a window of time to observe the post-M&amp;A integration process, M&amp;A were required to occur before December 2019. (3) According to the purpose of M&amp;A mentioned in announcements and news, we selected technology-sourcing overseas M&amp;A samples. (4) We excluded samples in which either the acquirer or the target had few patents. We ultimately selected 146 firms.\" (3.1. Sample and data, Page 7)</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5341,12 @@
       </c>
       <c r="E93" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G93" s="0" t="inlineStr">
@@ -5372,7 +5374,7 @@
       </c>
       <c r="P93" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>No effect size of interest. The study does not measure individual boundary spanning behavior, but rather operationalizes lateral collaboration effectiveness as normative and affective commitment. Verbatim Evidence: \"Lateral collaboration effectiveness is a crucial process for commitment integration that satisfies the concerns of each relevant party involved in any business exchange (Harrison &amp; New, 2002). Normative commitments encourage a subsidiary employee to comply with the MNEs' requirement set for bureaucratic control with ‘a sense of obligation that derives from the internalization of normative influences’ (Meyer &amp; Parfyonova, 2010). Affective commitments capture the subsidiary employees' emotional identification, engagement and attachment to the MNE, which are associated with employees' desire to contribute to the benefit of the firm (Meyer &amp; Allen, 1991). By committing in these ways to the efforts of the team and organization, employees transcend their formal roles and increase their potential to make impactful contributions to the effectiveness of the organization (Wombacher &amp; Felfe, 2017). We therefore consider the exercise of commitment as a form of lateral collaboration that can be enhanced to achieve the expected people development and subsidiary performance.\" (Lateral collaboration effectiveness and its consequences, page 410-411)</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5396,7 @@
       </c>
       <c r="F94" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G94" s="0" t="inlineStr">
@@ -5422,7 +5424,7 @@
       </c>
       <c r="P94" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>Firm-level analysis. Verbatim Evidence: \"To select the appropriate samples, we adopted four criteria. Firstly, the firms should be in good operating condition and have innovation output over a period of time. Secondly, considering the innovation cycle, the firms should be established for at least one year. Thirdly, due to the research purpose, the firms should have conducted business process digitisation and made some progress. Finally, in order to improve the universality of the conclusions, the firms in samples should be in a wide range of industries. Accordingly, we delivered 581 initial questionnaires through email and professional survey website “questionnaire star (www.wjx.cn)”. And the respondents were firm managers. Then, 428 questionnaires were received, with a sample return rate of 73.7%.\" (3.1. Sample and data collection, Page 6)</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5446,7 @@
       </c>
       <c r="F95" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G95" s="0" t="inlineStr">
@@ -5472,7 +5474,7 @@
       </c>
       <c r="P95" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Team level analysis. Verbatim Evidence: \"Given that our model was built at team level, we assessed the viability of individual-level data aggregation. First, we used the interrater reliability coefficient to evaluate within-group homogeneity (James et al., 1993). Rwg values (Shared leadership = 0.98; Team reflexivity = 0.97; Team boundary spanning = 0.96; New venture performance = 0.97) were greater than the criterion of 0.70. Second, we adopted the intraclass correlation coefficient ICC(1) and reliability of the mean ICC(2) to evaluate between-group heterogeneity (Bliese, 2000). The scores of ICC(1) ranged from 0.20 to 0.28, surpassing the benchmark of 0.10. The scores of ICC(2) ranged from 0.55 to 0.66, going beyond the criterion of 0.50. Therefore, the aggregation of key variables was justified.\" (Data Aggregation, Page 412)</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5491,12 @@
       </c>
       <c r="E96" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G96" s="0" t="inlineStr">
@@ -5517,7 +5524,7 @@
       </c>
       <c r="P96" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Qualitative study based on semi-structured interviews. Verbatim Evidence: \"The study that we conducted is based on semi-structured interviews among HCPs who participate directly in the 1DD care pathway or work closely with it. We interviewed 19 HCPs between April and July 2019, knowing that the innovative organization was set up in January 2017. We contacted each HCP in person or by e-mail. The participants received information on the relevance and design of the study, the problem, the central concepts of the study and the way the results would be distributed. Each participant explicitly consented to participate in the study. The interviews were conducted individually by the same interviewer, following the same outline.\" (The Research Process, page 56)</t>
         </is>
       </c>
     </row>
@@ -5534,14 +5541,10 @@
       </c>
       <c r="E97" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F97" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F97" s="0" t="n"/>
       <c r="G97" s="0" t="inlineStr">
         <is>
           <t>The current study examined the relationships among role stress, proactive personality, employee creativity, and customer-oriented boundary spanning behaviors (COBSBs) for frontline service employees (FSEs). This study collected data from 382 FSEs in international hotels in Taiwan to test the research model. The empirical results revealed that employee creativity was positively affected by proactive personality but negatively affected by role conflict and role ambiguity. FSEs’ creativity positively affects COBSBs, including external representation, internal influence, and service delivery. Internal influence also positively affects service delivery and mediates the relationship between FSEs’ creativity and service delivery.</t>
@@ -5567,7 +5570,7 @@
       </c>
       <c r="P97" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Study samples individual organizational employees and provides a Pearson correlation matrix including boundary spanning behavior variables. Verbatim Evidence: \"This study collected data from FSEs in international hotels in Taiwan to test the research hypotheses. There were 79 international hotels in Taiwan in September 2019 (Tourism Bureau, 2019). The human resource managers of all 79 hotels were contacted and asked if they would be willing to help collecting the data for this research; 25 agreed to do so. Thirty questionnaires were sealed in envelopes and sent to those human resource managers at 25 international hotels (750 sealed questionnaires in total). Then the mangers distributed questionnaires to their FSEs and FSEs returned the completed questionnaires in another sealed envelope to his/her managers for sending them back to us.\" (Methodology, Page 4)</t>
         </is>
       </c>
     </row>
@@ -5584,7 +5587,12 @@
       </c>
       <c r="E98" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G98" s="0" t="inlineStr">
@@ -5612,7 +5620,7 @@
       </c>
       <c r="P98" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Project level analysis. Verbatim Evidence: \"After two follow-up emails sent after 10 and 20 days, we obtained 243 completed questionnaires (response rate of 31%). To ensure that our study was based on a homogenous sample, we crossed the sector variable with the nature of the project variable (new product/service, new process) and selected only projects involving the design of new products/services. This reduced the sample to 83 questionnaires. As 10 of these questionnaires were incomplete, our final sample consisted of 73 valid questionnaires completed by NPD project leaders. The company names on these questionnaires were all different, allowing us to conclude that the project managers interviewed belonged to different firms.\" (Sample and data collection, page 54)</t>
         </is>
       </c>
     </row>
@@ -5634,7 +5642,7 @@
       </c>
       <c r="F99" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G99" s="0" t="inlineStr">
@@ -5662,7 +5670,7 @@
       </c>
       <c r="P99" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Qualitative ethnographic study lacking quantitative effect sizes or a correlation matrix. Verbatim Evidence: \"We took an ethnographic approach (Arnould and Wallendorf 1994) to understand the life domains of rural migrants in urban settings. A sample size of 36 obviously cannot generalize to 280 million migrants, but the purpose of ethnographic research is to increase the depth of understanding rather than generalization. Wang and Tian (2014) used a sample size of 19 migrants to investigate a much more specific context. All informants are Chinese nationals, and most had resided in the urban area for more than five years. We used our personal ties with the local government and companies to recruit informants.\" (Methods, page 445)</t>
         </is>
       </c>
     </row>
@@ -5684,7 +5692,7 @@
       </c>
       <c r="F100" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G100" s="0" t="inlineStr">
@@ -5712,7 +5720,7 @@
       </c>
       <c r="P100" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Firm level analysis based on archival data. Verbatim Evidence: \"The hypotheses relating organizational characteristics to entry timing are tested on data on ten product categories with 118 entrants. Top management team demographic data were gathered from Standard &amp; Poor’s Register of Corporations, Directors and Executives and Dun &amp; Bradstreet’s Reference Book of Corporate Managements. The data for other organizational characteristics, including corporate governance, level of diversification, boundary spanning, firm performance, capital structure, and firm size were gathered from Moody’s Industrial Manual and Public Utility Manual, Standard &amp; Poor’s Register of Corporations, Directors and Executives, and Dun’s Million Dollar Directory.\" (Abstract, Page iv-v)</t>
         </is>
       </c>
     </row>
@@ -5734,7 +5742,7 @@
       </c>
       <c r="F101" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G101" s="0" t="inlineStr">
@@ -5762,7 +5770,7 @@
       </c>
       <c r="P101" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>Alliance level analysis. Verbatim Evidence: \"This study aimed to determine the connection between organisational relationships and organisational success by investigating the relationship between organisational alliances (as a specific form of organisational relationship) and goal attainment. The three-stage model of organisational relationships proposed by Grunig and Huang (2000:34) was applied to organisational alliances in order to determine this relationship, as well as to determine the influence of key constructs like type of industry, type of alliance, duration of the alliance and the size of the organisation. The reliability of using this framework, specifically the relationship outcomes proposed by the three-stage model, was investigated.\" (Abstract, page iv)</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5792,7 @@
       </c>
       <c r="F102" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G102" s="0" t="inlineStr">
@@ -5812,7 +5820,7 @@
       </c>
       <c r="P102" s="0" t="inlineStr">
         <is>
-          <t>Multilevel study where BSB is at the manager/group level (Level 2). Verbatim Evidence: "In this study, the data have a nested structure with individual subordinates nested within managers. Constructs regarding the manager exist at the group level of analysis whereas constructs about subordinate employees exist at the individual level of analysis.</t>
+          <t>Group level analysis. Verbatim Evidence: \"In this study, the data have a nested structure with individual subordinates nested within managers. Constructs regarding the manager exist at the group level of analysis whereas constructs about subordinate employees exist at the individual level of analysis. In the first stage of the indirect effects model, the hypotheses are cross level in nature with manager level effects (for example, external relationships and transformational leadership) predicting individual level outcomes (for example, information access or perceived manager status).\" (Section IV.6.a Nested data structure, page 76)</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5842,7 @@
       </c>
       <c r="F103" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G103" s="0" t="inlineStr">
@@ -5862,7 +5870,7 @@
       </c>
       <c r="P103" s="0" t="inlineStr">
         <is>
-          <t>Project/Team-level aggregation study. Verbatim Evidence: "This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates... Note: Dependent variable: (L) Learning rate, N = 47, N = 183 projects." (Abstract / Table 3-4 section)</t>
+          <t>Project level analysis. Verbatim Evidence: \"In the SF repository, there were 587 software projects being developed by six or more core team members and using “C”. These projects constituted the sampling frame. The final sample was reduced to 230 projects (39% of the sampling frame) because only that number had archived full data on all development activities. In spite of the non-probabilistic nature of the sample (see limitations), it contained projects with varied types of applications, sizes, and degrees of complexity. The unit of analysis was the OSS project.\" (Sampling, Page 13-14)</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5892,7 @@
       </c>
       <c r="F104" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G104" s="0" t="inlineStr">
@@ -5912,7 +5920,7 @@
       </c>
       <c r="P104" s="0" t="inlineStr">
         <is>
-          <t>Project/Team-level aggregation study. Verbatim Evidence: "The final sample was reduced to 101 projects since only that number had archived full data on all development activities. For the 101 projects, repeated measures were taken on a quarterly basis since the beginning..." (Methodology / Sample section)</t>
+          <t>Project level analysis. Verbatim Evidence: \"The unit of analysis was the NPD project. OSS project information is hosted in web-based repositories which have been used repeatedly as sources of archival data for empirical studies (Mockus et al., 2002). Similarly, this paper uses Source Forge (SF) (www.sourceforge.net) which is the paramount OSS project repository. The software projects selected were those developed in the programming language “C”, by six or more team members. This minimum number of team members was chosen to avoid any bias from the large number of one-person projects in SF, while still maintaining a reasonable variability range in the network-based measures.\" (Sampling, Page 10)</t>
         </is>
       </c>
     </row>
@@ -5934,7 +5942,7 @@
       </c>
       <c r="F105" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G105" s="0" t="inlineStr">
@@ -5962,7 +5970,7 @@
       </c>
       <c r="P105" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the firm, alliance, supply chain, or inter-organizational level (not individual employee level).</t>
+          <t>Firm level analysis. Verbatim Evidence: \"The questionnaire was organized in three sections. The first section was aimed at collecting structural data (size, age, educational background of personnel, external partners, etc.); the second section focused on the main services provided and the actors served (types of firm, sector in which they operate), while the third section was devoted to collecting data on main joint projects with clients. In order to maximize the response rate, an extensive follow-up was carried out. Mailing of the questionnaire was followed by a telephone call (at least 15 min for each of the Centres mapped) which illustrated the questionnaire and made the questions clear. This process was repeated at different time intervals to any remaining non-respondents. The response rate was equal to 43.92% for a total of 65 respondent TTCs (39 in the Veneto, 18 in Friuli and 8 in Trentino).\" (3.1 Research setting and data collection, Page 952)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6020,7 @@
       </c>
       <c r="P106" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: \"For the data collection, a total of 25 interviews were carried out in two MNCs. The interviewees include 18 collaboration managers, four senior staff in the two MNCs, three external partners and experts based in Europe, Asia, North America and China. The sample is selected according to their geographical location and functions, as well as bringing both the internal and external perspectives. One-hour long semi-structured interviews were conducted in China and seven other countries in 2017, 2018 and 2020 (Appendix 1), supplemented by other documents such as internal reports, published papers and company websites, as well as one author’s 5-year longitudinal study of the YIP and other formal and informal interviews with the CMs.\" (3.1. The cases: Yangshuo and Island, Page 5)</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6042,7 @@
       </c>
       <c r="F107" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G107" s="0" t="inlineStr">
@@ -6062,7 +6070,7 @@
       </c>
       <c r="P107" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Plant-level analysis. Verbatim Evidence: \"The quantitative data I analyze in this research are from a survey conducted in 1991 by Kelley and Watkins on 973 plants that perform a significant amount of metal machining in their production process, what they term the Machined Durable Goods Sector (Kelley, 1991). The survey was a second wave in a panel study of firms first surveyed in a similar survey conducted by Kelley and Brooks in 1987. Although the study has a longitudinal design, relevant measures on close ties appear only in the second wave, leading to my use of cross-sectional analysis.\" (Survey Data - The \"Machined Durable Goods\" Sector, Page 40)</t>
         </is>
       </c>
     </row>
@@ -6084,7 +6092,7 @@
       </c>
       <c r="F108" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G108" s="0" t="inlineStr">
@@ -6112,7 +6120,7 @@
       </c>
       <c r="P108" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The study does not measure boundary spanning behavior or provide an effect size for it. Verbatim Evidence: \"Sustainability was assessed with a 9-item instrument developed by Slaghuis et al. (2011). Examples of items are as follows: ‘the new practice is regarded as the standard way to work’ and ‘all colleagues involved in the new work practice are knowledgeable about it’. Responses are using a five-point scale, with higher scores indicating greater sustainability. The sustainability score was derived by calculating the mean of the total 9-item scores. The Partnership Self-Assessment Tool: Short version (PSAT-S) was used to measure partnership synergy and dimensions of partnership functioning (Cramm et al. 2011). This instrument contains nine items that measure partnership synergy (e.g. ‘By working together, how well are the partners able to identify new and creative ways to solve problems’?) and components that measure five dimensions of partnership functioning: leadership (four items; e.g. inspiring or motivating people and taking responsibility), efficiency (three items; e.g. how well the partnership uses the partners’ financial resources), administration and management (four items; e.g. evaluating the progress and impact of the partnership and organising partnership activities, including meetings and projects), and non-financial resources [four items e.g. data and information (statistical data, information, skills, expertise)].\" (Measures, page 4)</t>
         </is>
       </c>
     </row>
@@ -6134,7 +6142,7 @@
       </c>
       <c r="F109" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G109" s="0" t="inlineStr">
@@ -6162,7 +6170,7 @@
       </c>
       <c r="P109" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>No effect size of interest. The study samples employees in boundary-spanning positions but does not measure boundary spanning behavior (BSB) as a construct; therefore, no correlation for BSB is provided. Verbatim Evidence: \"Drawing on optimism and role theory research (Kahn et al. 1964), we develop two competing models for coping with role stressors in boundary-spanning positions (see Figures 1 and 2). In the first model, we posit optimism will facilitate coping with role stressors, which in turn, will lead to lower levels of burnout and higher satisfaction and performance in boundary-spanning positions. In the competing model, we posit optimism will enable boundary spanners to anticipate and respond proactively to stressors before they occur, which will alleviate burnout and increase job outcomes. The competing hypotheses are formalized in the subsequent sections.\" (Conceptual Framework, Page 2)</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6192,7 @@
       </c>
       <c r="F110" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G110" s="0" t="inlineStr">
@@ -6212,7 +6220,7 @@
       </c>
       <c r="P110" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Qualitative case study lacking quantitative correlation data. Verbatim Evidence: \"We conducted a qualitative study grounded in pragmatist philosophy and abductive inquiry that compares and iterates between theory and empirical material (Timmermans and Tavory 2012; Martela 2015). A pragmatist approach relies on experientialism to produce warranted assertions and guidance with inference to the best explanation that is historically contextual (Martela 2015). Our pragmatic and abductive approach means that we entered the primary research phase of our project with a theoretical framework that provided the foundation of our research questions. This framework then guided our data analysis and enabled us to make contributions to the role that knowledge resources play in PNOs.\" (METHODS AND CASE STUDY DESCRIPTION, Page 5)</t>
         </is>
       </c>
     </row>
@@ -6234,7 +6242,7 @@
       </c>
       <c r="F111" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G111" s="0" t="inlineStr">
@@ -6262,7 +6270,7 @@
       </c>
       <c r="P111" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The study's primary unit of analysis is the firm, not individual organizational employees. Verbatim Evidence: \"We combined survey and archival data to construct a multi-sourced dataset. The survey was conducted in the first half of 2011. To prevent common method bias, the questionnaire was designed in two parts, separating the key constructs involved in the hypothesized relationships. Specifically, general firm strategic posture (e.g. EO) and performance were evaluated by the chief executive officer, general manager, or chairperson of the firm who were invited to respond to part one of the survey, whereas information related to firm capabilities (e.g. ACAP and BS) was included in part two for which the chief technology officer or the chief information officer was the desired respondent. The initial questionnaire was designed in English and translated into Chinese by two bilingual academics with expertise in entrepreneurial activities. The questionnaire was reverse-translated for accuracy and pre-tested in an EMBA class of Chinese managers to ensure the meanings of the questions were easily understandable. A total of 411 firms returned the fully completed questionnaires, constituting an effective response rate of 20.6%, which is comparable to the response rates of executive surveys in prior studies.\" (3.1. Sample and data collection, Page 5)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: inject 2nd screening results and verbatim quotes for Batch 8 (BSMA0109-BSMA0156)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -4702,7 +4702,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F80" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -5344,7 +5344,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
+      <c r="F93" s="0" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
@@ -5494,7 +5494,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr">
+      <c r="F96" s="0" t="inlineStr">
         <is>
           <t>4 = Non-primary study</t>
         </is>
@@ -5590,7 +5590,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr">
+      <c r="F98" s="0" t="inlineStr">
         <is>
           <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="F112" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G112" s="0" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="P112" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>Team-level analysis where knowledge sharing was aggregated to the work group. Verbatim Evidence: \"After gathering background information on the 182 work groups in the sample, I created a survey with questions about knowledge sharing within and outside of the group. I pretested the survey on employees in the corporate office before sending it out in June 2000 as an e-mail attachment to each group member who had a valid e-mail address (1,315/1,474 or 89%). The survey was sent an average of six months after groups had completed their projects, took approximately 20–30 minutes to complete, and included a cover letter describing the purpose of the study and ensuring confidentiality. The response rate for those who were sent an e-mail survey, including two follow-up reminders, was 73% (957/1,315).1 There was at least one respondent from each work group, and responses were averaged across members and applied to the entire group.\" (Qualitative and Quantitative Evidence, Page 4)</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6342,7 @@
       </c>
       <c r="F113" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G113" s="0" t="inlineStr">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="P113" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Purely qualitative case study based on interviews lacking quantitative employee correlation data. Verbatim Evidence: \"We took a case study approach designed to engender analysis of work and employment relations challenges associated with the implementation of new organizational forms. [...] In total, we carried out 40 interviews across four cases with: genetics nurses; genetics clinicians; mainstream clinicians; mainstream nurse managers; business managers; project managers; commissioners of service. [...] In analysing interviews within the four cases, a number of iterations were undertaken by the authors in the development of key themes. The themes reflected healthcare professionals’ perceptions of work and employment relations challenges within their network. Rather than coding the interviews through software, such as QSR’s NVivo package, so that data remained contextualized we treated the interviews holistically as narratives.\" (Research design, Pages 544-546)</t>
         </is>
       </c>
     </row>
@@ -6392,7 +6392,7 @@
       </c>
       <c r="F114" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G114" s="0" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="P114" s="0" t="inlineStr">
         <is>
-          <t>Non-primary / Conceptual / Qualitative study without raw Pearson correlation coefficient matrix between individual employee BSB and outcomes.</t>
+          <t>Group level analysis. Verbatim Evidence: \"External information search was evaluated with three items adapted from a team learning scale (Edmondson, 1999). The three items were: “Team members go out and get all the information they possibly can from others - such as customers, or other parts of the organization,” “We invite people from outside the team to present information or have discussions with us” and “This team frequently seeks new outside information that leads us to make important changes,” and the answers were recorded on a seven-point Likert scale (1 = fully disagree to 7 = fully agree). Cronbach’s alpha for this scale was 0.72. Because groups are the level of analysis, individual scores were aggregated at the group level and the results of the aggregation statistics supported this aggregation (the within group agreement index for EIS ranged from 0.73 to 1.00 with an average of 0.89).\" (Method, Page 6)</t>
         </is>
       </c>
     </row>
@@ -6470,7 +6470,7 @@
       </c>
       <c r="P115" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>No measure of boundary spanning behavior. The study focuses on telework characteristics, work-nonwork conflict, and personal boundary management strategies rather than organizational boundary spanning. Verbatim Evidence: \"This quantitative and descriptive research is based on Allen et al.’s telework model (2015) and Keeney et al.’s WNWC model (2013), as shown in Figure 1. These two variables – telework and WNWC – were conceptually defined in subchapters 2.1 and 2.2, and operationally defined using the scales mentioned in Table 2. A specialized professional translated the scales into Portuguese, followed by a back-translation into English. A pretest before the data collection showed that no extra adjustments were needed. The universe consisted of people who telework in Brazil, estimated at 7.90m individuals in September 2020 (IBGE, 2020).\" (Methods, page 6)</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6520,7 @@
       </c>
       <c r="P116" s="0" t="inlineStr">
         <is>
-          <t>Theoretical or conceptual discussion; lacks primary quantitative empirical dataset.</t>
+          <t>Conceptual paper lacking empirical data. Verbatim Evidence: \"The empirical testing of these propositions is suggested for future research. The nature of the topic is such that interpretive rather than functional research approaches should be used. In particular, a phenomenological approach is recommended, as the object of the research pertains to explaining behaviors and consequences not explained by extant theories of transaction cost economics and the resource-based view of the firm.\" (Conclusions and Implications, Page 44)</t>
         </is>
       </c>
     </row>
@@ -6570,7 +6570,7 @@
       </c>
       <c r="P117" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study utilizes structural equation modeling (SEM) but completely fails to provide a bivariate Pearson correlation matrix. Additionally, the measured knowledge acquisition variables focus on firm-level capabilities rather than individual employee boundary spanning behaviors. Verbatim Evidence: \"The unit of analysis consisted of knowledge workers who held managerial positions in each of the participating companies, including those in the top management level (i.e., executive managers), the middle management level (i.e., managers of main divisions), the lower management level (i.e., heads of departments and supervisors), as well as employees. Consequently, multiple respondents at different managerial levels within each pharmaceutical manufacturing company were targeted by the survey since knowledge management functions, in terms of knowledge acquisition, integration, sharing, dissemination, and application, are undertaken collectively through ‘organisation-wide’ efforts rather than being the sole or individual responsibility of a specific work unit or person. The same rationale applies in the case of organisational innovation, whether it is related to products/services, managerial systems, processes, and/or technologies. In this way, including multiple respondents in the survey would ensure higher representativeness and reduce bias.\" (Research design and population, Page 114)</t>
         </is>
       </c>
     </row>
@@ -6587,14 +6587,10 @@
       </c>
       <c r="E118" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F118" s="0" t="inlineStr">
-        <is>
-          <t>4 = Non-primary study</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F118" s="0" t="n"/>
       <c r="G118" s="0" t="inlineStr">
         <is>
           <t>The “variance hypothesis” predicts that external search breadth leads to innovation outcomes, but people have limited attention for search and cultivating breadth consumes attention. How does individuals' search breadth affect innovation outcomes? How does individuals' allocation of attention affect the efficacy of search breadth? We matched survey data with complete patent records, to examine the search behaviors of elite boundary spanners at                 IBM                 . Surprisingly, individuals who allocated attention to people inside the firm were more innovative. Individuals with high external search breadth were more innovative only when they allocated more attention to those sources. Our research identifies limits to the “variance hypothesis” and reveals two successful approaches to innovation search: “cosmopolitans” who cultivate and attend to external people and “locals” who draw upon internal people                              . © 2014 The Authors.               Strategic Management Journal               published by John Wiley &amp; Sons Ltd.</t>
@@ -6620,7 +6616,7 @@
       </c>
       <c r="P118" s="0" t="inlineStr">
         <is>
-          <t>Qualitative interview / conceptual study without individual employee Pearson correlation matrix. Verbatim Evidence: "We composed a theoretical rather than representative sample of professionals who are boundary spanners and tasked with innovation search who had been granted a great deal of autonomy over their time." (Methodology / Sample section)</t>
+          <t>Study samples individual organizational employees and provides a Pearson correlation matrix including boundary spanning behaviors. Verbatim Evidence: \"With the permission of the Vice President of Technical Strategy for IBM, we derived a list of all 460 Distinguished Engineers and 317 IBM Academy members in 2008. One hundred and sixty-two individuals were both a Distinguished Engineer and an Academy member, resulting in a population of 615 individuals. We surveyed both cohorts as both are promoted to their roles based on their innovation track record, and both have the autonomy to conduct independent innovation search.\" (METHODS, Page 286)</t>
         </is>
       </c>
     </row>
@@ -6637,14 +6633,10 @@
       </c>
       <c r="E119" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F119" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F119" s="0" t="n"/>
       <c r="G119" s="0" t="inlineStr">
         <is>
           <t>THErelationships between age, aspects of tenure, locus of control, job involvement, and boundary spanning behaviour (B.S.B.) were examined using path analysis for 281 scientists and engineers. It was found that locus of control and age were significant determinants of job involvement. It was also shown that locus of control and job involvement were significant determinants of B.S.B. These findings are discussed relative to previous research on locus of control, job involvement, and B.S.B. Finally, new research designs are advocated which incorporate task characteristics, role dynamics constructs, and environmental uncertainty as determinants of B.S.B.</t>
@@ -6668,7 +6660,11 @@
       <c r="K119" s="0" t="n">
         <v>1978</v>
       </c>
-      <c r="P119" s="0" t="inlineStr"/>
+      <c r="P119" s="0" t="inlineStr">
+        <is>
+          <t>This study surveys individual organizational employees and provides a zero-order correlation matrix that includes boundary spanning behavior. Verbatim Evidence: \"The study was conducted in 15 public and private research organizations located in the Western United States. Two hundred and eighty-one scientists and engineers participated in the study. Forty-five of the respondents were project leaders while the remainder were team members. Since participation in the study was voluntary, the 281 questionnaires returned did not represent all of the technical people employed by the 15 organizations.\" (Method, Page 4)</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="18" customHeight="1" s="31">
       <c r="A120" s="0" t="inlineStr">
@@ -6683,14 +6679,10 @@
       </c>
       <c r="E120" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F120" s="0" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F120" s="0" t="n"/>
       <c r="G120" s="0" t="inlineStr">
         <is>
           <t>Customer contact personnel (CCP) are recognised as a key determinant in the attainment of customer satisfaction and service quality. While they are readily acknowledged as often representing the service in the eyes of the customer, almost no attention has been given to researching the determinants of service behaviour among CCP, from the perspective of CCP.</t>
@@ -6716,7 +6708,7 @@
       </c>
       <c r="P120" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>The study samples individual organizational employees in boundary spanning roles and provides a quantitative Pearson correlation matrix of their behaviors. Verbatim Evidence: \"Airline flight attendants were considered suitable respondents for this research as they hold a high boundary spanning position. The useable data from the survey of 446 respondents represented a 36% response rate. The data analysis undertaken included path analysis and structural equation modelling.\" (Abstract, page xv)</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6730,7 @@
       </c>
       <c r="F121" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G121" s="0" t="inlineStr">
@@ -6766,7 +6758,7 @@
       </c>
       <c r="P121" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Team level analysis. Verbatim Evidence: \"The sample consisted of 3,262 U.S. Air Force captains with 5–9 years of experience in a broad range of professional disciplines. These officers were attending a 5-week leadership course offered periodically at an Air Force base located in the southeastern United States. The participants were assigned to 233 fourteen-person teams using criteria designed to ensure that team composition was equivalent on factors including experience, job function, gender, and age. Team assignments were kept intact throughout the 5-week course; thus, these teams had a meaningful past and future.\" (Method, Page 813)</t>
         </is>
       </c>
     </row>
@@ -6788,7 +6780,7 @@
       </c>
       <c r="F122" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G122" s="0" t="inlineStr">
@@ -6816,7 +6808,7 @@
       </c>
       <c r="P122" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Qualitative study without quantitative effect sizes. Verbatim Evidence: \"With the intention of exploring in detail the cultural and gender norms around the work-life boundary process, the study employs qualitative research methodology under the interpretive paradigm. In collecting data, we employed a series of activities within a workshop to collect data for the study at hand. Well-designed workshops are found to assist respondents in focusing on important elements of a phenomenon as the researcher can facilitate the respondents to develop an emphasis on critical elements of the phenomenon under the study (Ørngreen and Levinsen, 2017; Ahmed and Asraf, 2018).\" (Methodology, Page 113)</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6830,7 @@
       </c>
       <c r="F123" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G123" s="0" t="inlineStr">
@@ -6866,7 +6858,7 @@
       </c>
       <c r="P123" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The study lacks a measure of individual boundary spanning behavior because the term boundary-spanning is merely used to describe the context of the service teams. Verbatim Evidence: \"The assessment of the SMT service climate involved items we specifically developed for this study; in-depth interviews with frontline employees; and scales developed by Schneider, Wheeler, and Cox (1992) and Peccei and Rosenthal (1997). We based the operationalization of tolerance for self-management (seven items) largely on the tolerance-of-freedom instrument of the Leader Behavior Description Questionnaire, which assesses the degree of autonomy given to employees to manage their task responsibilities themselves (Cook et al. 1981). We measured team member flexibility and inter- and intrateam support with scales developed by Campion, Medsker, and Higgs (1993). We measured all scale items for the employee survey on a seven-point scale that ranged from 1 = “strongly disagree” to 7 = “strongly agree.”\" (Measurement Issues, Page 5)</t>
         </is>
       </c>
     </row>
@@ -6883,14 +6875,10 @@
       </c>
       <c r="E124" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F124" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F124" s="0" t="n"/>
       <c r="G124" s="0" t="inlineStr">
         <is>
           <t>Background: Registered nurses play a key role in hospitals, as they have an important impact on the quality of the services delivered. For nurses to perform at their best, they need organizational, leader, and coworker support. To date, few studies have explored the link between nurses_ perceived support, affective organizational commitment, and boundary-spanning behaviors. Methods: This cross-sectional research used a questionnaire survey to explore the hypothesized relationships in a sample of 273 nurses from a hospital in Belgium. Structural equation modeling was used for statistical analysis of the mediation model. Results: One hundred forty-seven (53.5%) nurses responded to the survey. Perceived support from the organization, supervisors, and coworkers positively influences nurses_ boundary-spanning behaviors. Affective organizational commitment was found to mediate the positive relationship between perceived organization support, perceived coworker support, and boundary-spanning behaviors. Perceived supervisor support and boundary-spanning behaviors showed a direct relationship not mediated by affective organizational commitment. Conclusions: Perceived support has an important influence on the boundary-spanning behavior of nurses. This study emphasizes the importance on how support exerts an influence on boundary-spanning behavior and</t>
@@ -6934,7 +6922,7 @@
       </c>
       <c r="F125" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G125" s="0" t="inlineStr">
@@ -6962,7 +6950,7 @@
       </c>
       <c r="P125" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Multiteam system level of analysis. Verbatim Evidence: \"Consistent with previous research using the LDS, all constructs in this study were conceptualized as configural unit properties (Kozlowski &amp; Klein, 2000) at the multiteam system level of analysis. Intrapersonal functional diversity. We operationalized IFD as the proportion of members in a multiteam system that had acquired experiences across different functional domains during the first two LDS sessions (see Park et al., 2009, for a similar approach). Specifically, during the first LDS session individual participants worked in one of the four distinct functions described above and, consequently, gained hands-on experience in the respective domain (i.e., operations [point team], intelligence [support team], and liaison or integrative leadership [integration team]).\" (Measures, Page 10)</t>
         </is>
       </c>
     </row>
@@ -6979,14 +6967,10 @@
       </c>
       <c r="E126" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F126" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F126" s="0" t="n"/>
       <c r="G126" s="0" t="inlineStr">
         <is>
           <t>This manuscript investigates the role of individual team members' breadth of functional experience for their interteam coordination behavior. Integrating personal construct and social identity theories, we examine interpersonal cognitive complexity as a mediating variable and organizational identification as a moderator. We test our hypotheses across two independent field studies, comprising an international peace support training mission (Study 1) and a municipality administration (Study 2). Corroborating our predictions, interpersonal cognitive complexity appeared as a conditional mediating variable that can translate an individual's breadth of functional experience into interteam coordination. The strength and direction of this indirect relationship, however, depended on the individual's identification with the organization as a whole. Moreover, on the team level of analysis, we found members' overall interteam coordination to positively relate with team performance in Study 2. All in all, this paper advances new knowledge on the antecedents, mechanisms, contingency factors, and team-level consequences of members' boundary spanning.</t>
@@ -7012,7 +6996,7 @@
       </c>
       <c r="P126" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, work group, or multiteam systems (MTS) level (not individual employee level).</t>
+          <t>The study samples individual organizational employees across two samples and provides an individual-level Pearson correlation matrix that includes interteam coordination as a boundary spanning behavior. Verbatim Evidence: \"Because management limited the number of individuals we could include in our study, we targeted 295 randomly selected office employees across the organization. Participation was voluntary and anonymity assured. Of those employees, 121 (distributed over 36 of the organization’s 40 teams) provided complete responses, resulting in an effective response rate of 41%. Respondents were, on average, 48 years of age (SD = 10.33), had worked with the municipality administration for an average of about 13 years (SD = 10.92), and were mostly male (58%).\" (Sample and Procedure, Page 13)</t>
         </is>
       </c>
     </row>
@@ -7029,14 +7013,10 @@
       </c>
       <c r="E127" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F127" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F127" s="0" t="n"/>
       <c r="G127" s="0" t="inlineStr">
         <is>
           <t>Data from 409 members of 45 new product teams in five high-technology conpanies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator,Scout, and Guard. These activities are related to the frequency, type, and destination of communications between team members and others. This paper describes these activities and examines the irrpact of individual and environmental variables on the frequency in vAiich individual team members engage in them.</t>
@@ -7063,7 +7043,7 @@
       </c>
       <c r="P127" s="0" t="inlineStr">
         <is>
-          <t>Team-level aggregation study of product development teams without individual employee Pearson correlation matrix. Verbatim Evidence: "Data from 409 members of 45 new product teams in five high-technology companies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator, Scout, and Guard." (Abstract section)</t>
+          <t>Study samples individual organizational employees and provides a quantitative correlation matrix including boundary spanning behavior. Verbatim Evidence: \"Questionnaires were distributed to new product team members and leaders of forty-five teams in five corporations in the computer, analytic instrumentation, and photographic industries. Of the 450 questionnaires distributed, a total of 409 questionnaires were returned, yielding a response rate of approximately 89 percent. Response rates were approximately equal across the set of companies and the final total of respondents per company varied from 39 to 129.\" (Methods, Page 22)</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7065,7 @@
       </c>
       <c r="F128" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G128" s="0" t="inlineStr">
@@ -7116,7 +7096,7 @@
       </c>
       <c r="P128" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Alliance level analysis. Verbatim Evidence: \"To facilitate personal interviews, a geographical subset of biotechnology firms was developed. The areas chosen were Seattle, San Diego, and Philadelphia/New Jersey. Bioscan (1992) was used to develop a list of the 132 firms in these areas. All of the target firms were contacted, and interviews were arranged with 57 biotechnology firms. Each firm provided information on up to three distinct alliances. The 43% response rate is higher than previous studies (John 1984; Parkhe 1993). Personal interviews were used to rate 97 alliances, and phone interviews were used to rate 12 alliances. No firm rated more than three alliances.\" (Data Collection, page 10)</t>
         </is>
       </c>
     </row>
@@ -7133,14 +7113,10 @@
       </c>
       <c r="E129" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F129" s="0" t="inlineStr">
-        <is>
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F129" s="0" t="n"/>
       <c r="G129" s="0" t="inlineStr">
         <is>
           <t>Leader-Member Exchange theory proposes both the salesperson and manager make contributions to their working relationship. Effective leadership is dependent upon developing a high quality relationship. This study tests the proposals of Leader-Member Exchange by examining the exchange of manager contributions (allowing the salesperson more operating freedom or latitude) and those of the salesperson. While the receipt of managerial latitude has a direct effect on the salesperson's evaluation of the working relationship, the salesperson's contributions also play a part. The manager allows more latitude to salespeople who are seen as more competent and loyal. These exchanges latitude for competency and loyalty) and the quality of the salesperson-manager relationship may be especially important when the sales task requires adaptive selling behaviors.</t>
@@ -7164,7 +7140,11 @@
       <c r="K129" s="0" t="n">
         <v>1998</v>
       </c>
-      <c r="P129" s="0" t="inlineStr"/>
+      <c r="P129" s="0" t="inlineStr">
+        <is>
+          <t>This study focuses on individual organizational employees and includes a quantitative Pearson correlation matrix with relevant effect sizes. Verbatim Evidence: \"Each participating firm provided addresses and reporting responsibilities for their sales force. Cover letters and surveys were sent to 270 selected salesperson-manager dyads. The selection of dyads was based on the number of salespeople reporting to each manager. Surveys were sent to a randomly selected portion (25%) of the salespeople reporting to any one manager. ... Responses were received from 155 salespeople and their respective managers. Since surveys were sent to a total of 270 dyads, the effective response rate is 57.4%. For purposes of testing dyadic relationships, these 155 matched responses were considered complete observations.\" (Method, Page 37-38)</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="18" customHeight="1" s="31">
       <c r="A130" s="0" t="inlineStr">
@@ -7179,14 +7159,10 @@
       </c>
       <c r="E130" s="0" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F130" s="0" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level</t>
-        </is>
-      </c>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F130" s="0" t="n"/>
       <c r="G130" s="0" t="inlineStr">
         <is>
           <t>An information systems (IS) support community represents a knowledge-intensive network where IS professionals interact with end-users to resolve system use problems during the IS post-implementation stage. For IS professionals in the support function, providing support for multiple information systems to multiple business units requires knowledge about different domains (business units or technical systems). In this paper, we take a network perspective to empirically evaluate the effects of an IS worker's network position and knowledge boundary spanning on productivity. Drawing upon theories of experiential learning and knowledge boundary, we perform social network analysis and linear mixed effects modeling to analyze archival data comprising 36 IS workers and 23,450 support requests made by 4568 end-users during the first 13 months post SAP/R3 implementation in a large U.S. organization. Our findings reveal that IS workers' network centrality and boundary spanning positively influence productivity. Surprisingly, their boundary-spanning experience plays a substantially more important role than network centrality. This study makes important contributions to theory and practice in individual experiential learning in knowledge-intensive networks.</t>
@@ -7212,7 +7188,7 @@
       </c>
       <c r="P130" s="0" t="inlineStr">
         <is>
-          <t>Ticket/Task-level aggregation study of IT support community. Verbatim Evidence: "Then the ticket complexity scores are aggregated on a monthly basis per worker... Table 1 presents the descriptive statistics and correlations of the variables across 320 monthly aggregated worker ticket observations." (Methodology / Data analysis section)</t>
+          <t>Study meets all inclusion criteria by analyzing an individual employee sample and providing an individual-level correlation matrix including boundary spanning behavior constructs. Verbatim Evidence: \"We combined the ticket log data and network measures with individual characteristics of IS workers, and compiled an unbalanced panel dataset of 320 observations involving 36 IS workers over 13 months for data analysis. The dependent variable, IS workers' Average Effort, and all other variables (except Function), are continuous variables and demonstrate skewed distributions. Thus, we transformed them with a natural logarithm. ... Table 1 presents the descriptive statistics and correlations of the variables.\" (Data analysis and results, Page 21)</t>
         </is>
       </c>
     </row>
@@ -7234,7 +7210,7 @@
       </c>
       <c r="F131" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G131" s="0" t="inlineStr">
@@ -7262,7 +7238,7 @@
       </c>
       <c r="P131" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The primary unit of analysis is the cross-functional team, rather than the individual employee. Verbatim Evidence: \"The resulting set of items was then administered to the members of 43 intact CFTs who were involved in three large product development programs, each of which was dedicated to one vehicle. Each of these programs was led by a program manager and was made up of 15-30 cross-functional teams that held responsibility for separate modules or subunits of the vehicle. Each of these teams had a core of 5-20 members who came from functional organizations such as design, body or powertrain engineering, manufacturing, marketing, purchasing, and so on. Since the official list of team members often included nominal members who did not attend meetings or contribute much, we asked the leaders of each team to identify core members of the team, those who attended meetings regularly, spent at least 20 percent of their time working for the team, and were central to the team's activities. Using this procedure, we targeted 565 individuals who were members of 43 CFTs as questionnaire respondents. Surveys were distributed to core team members by their team leader at one of their regular meetings, and respondents were given two weeks to complete the survey and return it to us using an enclosed envelope. After three weeks, a second set of surveys was distributed to those who had not yet responded. Overall, 364 respondents representing 43 CFTs responded for an overall response rate of 65 percent.\" (Methods, Pages 1010-1011)</t>
         </is>
       </c>
     </row>
@@ -7284,7 +7260,7 @@
       </c>
       <c r="F132" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G132" s="0" t="inlineStr">
@@ -7312,7 +7288,7 @@
       </c>
       <c r="P132" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study relies on a student sample rather than organizational employees. Verbatim Evidence: \"Two hundred thirty-seven undergraduate psychology students were randomly formed into 79 teams of 3. Trainees received partial course credit for their participation. Ninety percent were under the age of 22. Fifty-six percent were women. Seventy-seven percent of the participants were Caucasian. Eleven percent of the teams had no women, 26% had 1 woman, 48% had 2 women, and 15% had 3 women.\" (Method, Page 6)</t>
         </is>
       </c>
     </row>
@@ -7362,7 +7338,7 @@
       </c>
       <c r="P133" s="0" t="inlineStr">
         <is>
-          <t>Does not measure BSB construct as an effect size; measures general job performance and self-monitoring. Verbatim Evidence: "To test the hypotheses, two constructs were assessed: job performance and attention to social cues. Performance level was obtained from company performance evaluation forms, which provide, in part, a single, overall performance rating." (Measures)</t>
+          <t>The study samples individuals in boundary-spanning roles but does not quantitatively measure boundary spanning behavior as an individual-level variable, thus lacking the required effect sizes. Verbatim Evidence: \"To test the hypotheses, two constructs were assessed: job performance and attention to social cues. Performance level was obtained from company performance evaluation forms, which provide, in part, a single, overall performance rating. Each field representative was rated on a 4-point scale as excellent, above average, average, or below average. Attention to social cues was measured using the Self-Monitoring Scale. A factor-scoring format was suggested by Briggs et al. (1980), and analyses were conducted using both the overall and factor-scoring protocols.\" (Measures, Page 125)</t>
         </is>
       </c>
     </row>
@@ -7384,7 +7360,7 @@
       </c>
       <c r="F134" s="0" t="inlineStr">
         <is>
-          <t>4 = Non-primary study</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G134" s="0" t="inlineStr">
@@ -7412,7 +7388,7 @@
       </c>
       <c r="P134" s="0" t="inlineStr">
         <is>
-          <t>Qualitative field consulting case study without individual employee Pearson correlation matrix. Verbatim Evidence: "Using an external perspective as a research lens, this study examined team-context interaction in five consulting teams. The data revealed three strategies toward the teams' environment: informing, parading, and probing." (Abstract section)</t>
+          <t>Team level qualitative analysis. Verbatim Evidence: \"Using a multimethod approach, I followed teams for their first five months. Data collection focused on three sets of variables. First, I collected data on team leaders' plans right after the teams were formed through interviews designed to ascertain implicit and explicit strategies toward their environment. Given time restraints, I interviewed team leaders, assuming that they would most influence the formation of team norms. Second, I monitored team interactions with outsiders, using questionnaires, logs, interviews, and observation, to document the mutual influence of team and context.\" (Data Sources, page 341)</t>
         </is>
       </c>
     </row>
@@ -7434,7 +7410,7 @@
       </c>
       <c r="F135" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G135" s="0" t="inlineStr">
@@ -7462,7 +7438,7 @@
       </c>
       <c r="P135" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Purely qualitative interview study without quantitative correlation data. Verbatim Evidence: \"Further, aware that Shah (2000) identified lead users as key drivers of innovation in boardsports, we conducted fieldwork with consumers who had transitioned into some form of commercial operation. These individuals know the commercial aspects of the sport due to selling equipment, instructing users, and participating actively in community events. We collected 13 semi-structured in-depth interviews with respondents who were simultaneously avid boardsports consumers and commercial operators, including retailers, owner-operators, entrepreneurs, instructors, and photographers (Table 1). Participant selection was achieved through snowball sampling and purposive sampling, where the researchers directly approached retailers and boardsports magazine editors in New Zealand (N.Z.) identified through secondary data such as newspaper articles.\" (3.2. The fieldwork, Page 4)</t>
         </is>
       </c>
     </row>
@@ -7484,7 +7460,7 @@
       </c>
       <c r="F136" s="0" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G136" s="0" t="inlineStr">
@@ -7512,7 +7488,7 @@
       </c>
       <c r="P136" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>Qualitative comparative analysis without quantitative data. Verbatim Evidence: \"The decision to restrict consideration to four particular fieldwork encounters has also been carefully considered. Most importantly, this reflects an inherent limitation of the case-oriented comparative method. As Ragin (1987, pp. 49–52) has noted, since in this approach cases are examined as wholes rather than as collections of variables, comparison becomes increasingly unwieldy when a set of more than two to four cases is considered. In addition, by using only monograph-length studies in which the ethnographer/informant relationship is a major focus and holding researcher nationality constant, I attempt to maximize the comparability of the material.\" (Unnamed Section, Page 61)</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7505,12 @@
       </c>
       <c r="E137" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G137" s="0" t="inlineStr">
@@ -7557,7 +7538,7 @@
       </c>
       <c r="P137" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>The study provides a dyadic-level correlation matrix rather than an independent individual-level correlation matrix. Verbatim Evidence: \"As suggested above, the data have a dyadic relational structure, where each respondent researcher (ego) has multiple contacts (alters) on other work teams. In the dyadic structure, each individual researcher is included in multiple observations because he or she reported on multiple relationships. Therefore, the observations are not independent within-person. If uncorrected for, this non-independence would result in artificially deflated standard errors and a model that appears to fit better than it actually does.\" (Analytical approach, Page 9-10)</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7555,12 @@
       </c>
       <c r="E138" s="0" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G138" s="0" t="inlineStr">
@@ -7602,7 +7588,7 @@
       </c>
       <c r="P138" s="0" t="inlineStr">
         <is>
-          <t>Empirical quantitative study measuring individual-level boundary spanning behavior and reporting statistical effect sizes.</t>
+          <t>Firm-level analysis of small business organizations. Verbatim Evidence: \"Data were collected by survey instrument from the owner/operators of four different types of small business organizations. There were 38 retail firms (food and apparel) and 44 manufacturing firms (food and apparel). Subjects were selected at random from phone directories in the Allentown-Bethlehem-Easton Pennsylvania SMSA. Of the owner/operators contacted by phone prior to mailing the survey, 180 met the inclusion criteria.\" (Method, page 355)</t>
         </is>
       </c>
     </row>
@@ -7624,7 +7610,7 @@
       </c>
       <c r="F139" s="0" t="inlineStr">
         <is>
-          <t>2 = Non-employee samples</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G139" s="0" t="inlineStr">
@@ -7652,7 +7638,7 @@
       </c>
       <c r="P139" s="0" t="inlineStr">
         <is>
-          <t>Sample consists of non-employee populations (e.g., consumers, patients, students, citizens, or clients), not organizational workplace employees.</t>
+          <t>Qualitative ethnographic case study without quantitative data. Verbatim Evidence: \"AD collected data through participant observation and interviewing. Fieldwork was conducted over 20 months between August 2015 and March 2017 (over 100 h per field site). AEs were the primary informants in each case study and enabled connection to other actors. Participant observation was structured around project management and commissioning of IRIS at an organisational level, the day-to-day delivery of IRIS as a programme of work (training and advocacy), and engagement in IRIS by its intended beneficiaries (clinicians and patients). Field notes formed the basis of the data from participant observation. 19 semi-structured interviews were conducted in each case study area with clinicians (case study one: 5, case study two: 8), services users (case study one: 8, case study two: 5), and actors involved in the commissioning and delivery of IRIS (case study one: 6, case study two: 6).\" (Methods, page 4)</t>
         </is>
       </c>
     </row>
@@ -7724,7 +7710,7 @@
       </c>
       <c r="F141" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G141" s="0" t="inlineStr">
@@ -7761,7 +7747,7 @@
       </c>
       <c r="P141" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>This is a purely conceptual book chapter that proposes a framework and research questions rather than providing primary quantitative data. Verbatim Evidence: \"Multiteam systems (MTSs) are complex collective entities comprising two or more teams that share one or more common superordinate goal. In these systems, leadership is often the result of the joint actions of multiple members. In other words, MTS leadership is often a shared or collective phenomenon. The current chapter explains how the form of MTS leadership (e.g., vertical, shared) can be captured using network analytic techniques across multiple MTS network foci (e.g., within teams, between-teams, across the system). It extends this perspective to describe the application of specic ego-net and network indices to the evaluation of MTS leadership forms. Finally, it provides example prompts that could be used to elicit leadership functions and goal foci (e.g., leadership focused toward individual, team-level goals, or MTS level goals) in MTS leadership networks, and it provides example research questions that stem from incorporation of network analytic techniques with the study of MTS leadership.\" (Abstract, Page 482)</t>
         </is>
       </c>
     </row>
@@ -7783,7 +7769,7 @@
       </c>
       <c r="F142" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G142" s="0" t="inlineStr">
@@ -7811,7 +7797,7 @@
       </c>
       <c r="P142" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Team level analysis. Verbatim Evidence: \"The research population consisted of 49 health promotion teams. All interorganizational teams working on improving lifestyle quality were approached. Five teams refused to participate in the survey because they were novice and insufficiently familiar with the ongoing project. Hence, the response rate was 89%. All teams can be defined as project teams in that they planned and implemented activities focusing on a healthier lifestyle, besides their routine jobs in their organization of origin.\" (Sample, page 13-14)</t>
         </is>
       </c>
     </row>
@@ -7861,7 +7847,7 @@
       </c>
       <c r="P143" s="0" t="inlineStr">
         <is>
-          <t>Empirical study, but does not report quantitative correlation/regression effect sizes between individual boundary spanning and outcome variables.</t>
+          <t>The study does not measure employee boundary spanning behavior, but instead assesses career mobility and turnover intentions across jobs and industries. Verbatim Evidence: \"For dependent variables, we created three binary variables using the individual survey in the AWRS data: cross-job mobility preference, cross-organisation mobility preference and cross-industry mobility preference. Measuring psychological mobility with a binary variable is a well-received approach in the literature (Cho and Lewis 2012; Ko and Hur 2014; Pitts, Marvel and Fernandez 2011). We created the mobility preference variables using individuals’ responses to this question: ‘In regard to your job, where do you want to be in 12 months’ time?’ The participants were asked to choose between five options: ‘working for the same employer, in the same role’ (option 1), ‘working for the same employer, but in a different role’ (option 2), ‘working for a different employer in the same industry’ (option 3), ‘working in another industry’ (option 4) and ‘no longer working’ (option 5).\" (Dependent variables, Page 11)</t>
         </is>
       </c>
     </row>
@@ -7911,7 +7897,7 @@
       </c>
       <c r="P144" s="0" t="inlineStr">
         <is>
-          <t>Student sample. Verbatim Evidence: "Fifteen subjects (upper division business school undergraduates) were in each treatment." (Research Method - Manipulations section)</t>
+          <t>Student sample. Verbatim Evidence: \"The research was conducted using a full-factorial experimental design, resulting in 16 (4 × 2 × 2) treatments. Fifteen subjects (upper division business school undergraduates) were in each treatment. The experimental treatments are depicted in Figure 1 and were operationalized in the following manner.\" (Manipulations, Page 19)</t>
         </is>
       </c>
     </row>
@@ -7933,7 +7919,7 @@
       </c>
       <c r="F145" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G145" s="0" t="inlineStr">
@@ -7961,7 +7947,7 @@
       </c>
       <c r="P145" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>Student sample. Verbatim Evidence: \"The primary data source for these experiments was undergraduate business students from the Fisher College of Business. The specific students recruited were those taking an introductory course in operations management. As such, all participants had been previously exposed to the concepts of supply chains, buyer-supplier relationships, the newsvendor problem, and coordination tactics.\" (Participants, Page 56)</t>
         </is>
       </c>
     </row>
@@ -7983,7 +7969,7 @@
       </c>
       <c r="F146" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G146" s="0" t="inlineStr">
@@ -8011,7 +7997,7 @@
       </c>
       <c r="P146" s="0" t="inlineStr">
         <is>
-          <t>Team level analysis. Verbatim Evidence: "To explore what leaders of action teams do to promote speaking up and other proactive coordination behaviours – as well as how organizational context may affect these team processes and outcomes – I analysed qualitative and quantitative data from 16 operating room teams learning to use a new technology for cardiac surgery." (Abstract)</t>
+          <t>Team level analysis of cardiac surgery teams, where boundary spanning is measured as a team construct. Verbatim Evidence: \"Stage 1. I analysed all coded interview data related to the team learning process and the organizational context to create composite variables. Following the logic of within-method triangulation ( Jick, 1979), I examined correlations between coded responses to questions assessing the same construct (Campbell and Fiske, 1959). This provided measures of internal consistency reliability and discriminant validity for each composite variable, as shown in Table I; non-composite (or single-measure) variables are shown in Table II. My aim in these analyses, described in more detail in the Appendix, was to assess the similarity of responses to related questions. The result is a set of numerical ratings for five team constructs (team stability, team preparation, procedure innovation, boundary spanning, and psychological safety) and four organizational constructs (history of innovation, resource constraints, management support, and information infrastructure) for each hospital.\" (Data Analyses, page 1429)</t>
         </is>
       </c>
     </row>
@@ -8061,7 +8047,7 @@
       </c>
       <c r="P147" s="0" t="inlineStr">
         <is>
-          <t>BSB not measured. Verbatim Evidence: "RQ: Are there differences in key job factors including (a) grit, (b) happiness, (c) perceived organizational support, (d) perceived supervisory support, (e) job satisfaction, (f) organizational commitment, and (g) turnover intentions based on the level of sleep an employee gets on average?" (Business-to-business salespeople)</t>
+          <t>No correlation matrix or measure of boundary spanning behavior, as the study only compares mean differences across sleep categories for general job attitudes. Verbatim Evidence: \"All scales used in this study were unidimensional and used a 7-point Likert scale. Grit (α = 0.74) was measured using three items from Duckworth and Quinn (2009). Happiness (α = 0.73) was measured using three items from Lyubomirsky and Lepper (1999). Perceived Organizational Support (POS, α = 0.93) was measured using an eight-item scale from Eisenberger et al. (1986) while Perceived Supervisory Support (PSS, α = 0.95) was measured using an eight-item scale from Kottke and Sharafinski (1988). Job Satisfaction (α = 0.91) was measured using a three-item scale by Jaramillo, Mulki, and Solomon (2006). Organizational Commitment (α = 0.91) was measured using a three-item scale by O’Reilly and Chatman (1986). Finally, Turnover Intentions (α = 0.92) was measured using a four-item scales by Brashear, Manolis, and Brooks (2005). Since there was a high degree of reliability for each of the measures, each scale was averaged so that a comparison between means could be conducted. A comparison between means was used to examine if differences existed for each scale included in this study based on the two sleep categories previously created. Table 1 displays the results for each scale.\" (Methodology and Findings, page 75)</t>
         </is>
       </c>
     </row>
@@ -8083,7 +8069,7 @@
       </c>
       <c r="F148" s="0" t="inlineStr">
         <is>
-          <t>3 = Non-individual level</t>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G148" s="0" t="inlineStr">
@@ -8111,7 +8097,7 @@
       </c>
       <c r="P148" s="0" t="inlineStr">
         <is>
-          <t>Macro or group level study: Examines boundary spanning at the team, unit, firm, board, or inter-organizational level (not individual employee level).</t>
+          <t>The study applies structural equation modeling (SEM) on practitioner survey data but fails to provide a bivariate Pearson correlation matrix for the variables. Verbatim Evidence: \"Three exogenous constructs and one endogenous construct emerge from the EFA, reliability, and AVE results. We next applied a confirmatory factor analysis (CFA) to further verify scale reliability and validity (Table 4). Following Hu and Bentler’s (1999) criteria, the measurement model is validated based on parsimony (χ2/df = 1.08), absolute fit (RMSEA = 0.02), close fit (PClose = 0.93), and incremental fit (TLI = 0.99 and CFI = 0.99). Factor loadings, except for one, are all above 0.70, and the one exception is above the 0.50 minimum (Fornell and Larcker, 1981). Cronbach’s alpha (α) and composite reliability (CR) metrics are strong. Further, average variance extracted (AVE) values exceed 0.50, confirming convergent validity. Additionally, all AVEs exceed the squared inter-item correlations, thereby verifying discriminant validity.\" (5.1 Measurement Model Evaluation, Page 7)</t>
         </is>
       </c>
     </row>
@@ -8126,11 +8112,15 @@
           <t>BSMA0146</t>
         </is>
       </c>
-      <c r="E149" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F149" s="0" t="n">
-        <v>3</v>
+      <c r="E149" s="0" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F149" s="0" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G149" s="0" t="inlineStr">
         <is>
@@ -8157,7 +8147,7 @@
       </c>
       <c r="P149" s="0" t="inlineStr">
         <is>
-          <t>Team level analysis. Verbatim Evidence: \"Our final sample consisted of those 57 teams from which we had received three or more subordinate surveys and a supervisor survey, and for which archival data were available. These teams ranged in size from 4 to 26 members (x = 11.7, s.d. = 6.1); 84 percent of team members were male; the average age was 42.7 years (s.d. = 7.7), and the average time with the current team was 1.5 years (s.d. = .5). [...] Together, the above analyses supported the aggregation of informant responses from a team to create team-level variables for collective team identification, team learning, intrateam conflict, and external communication.\" (Sample and Data Collection / Interrater agreement and reliability, Pages 537-539)  Note: The specific file \"Guenzel (2020) - Open innovation...\" did not exist in the workspace, so the paper with ID 201 mapped in all_remaining_targets.txt (\"[201] Van der vegt &amp; Bunderson (2005) - LEARNING AND PERFORMANCE IN MULTIDISCIPLINARY TEAMS.pdf\") was reviewed instead as standard procedure.</t>
+          <t>Firm-level analysis. Verbatim Evidence: \"This study seeks to understand the strategies foreign firms use to cope with liabilities of foreignness in an alien environment and compete successfully with domestic firms, specifically through boundary spanning. Using a sample of 3861 firms in the U.S., we find that foreign firms on the average underperform compared to domestic firms. We also find these firms take a differing strategic posture to cope with the disadvantages of being a foreign firm compared to domestic rivals.\" (Abstract, Page 51)</t>
         </is>
       </c>
     </row>
@@ -8172,11 +8162,15 @@
           <t>BSMA0147</t>
         </is>
       </c>
-      <c r="E150" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F150" s="0" t="n">
-        <v>3</v>
+      <c r="E150" s="0" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F150" s="0" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
       </c>
       <c r="G150" s="0" t="inlineStr">
         <is>
@@ -8203,7 +8197,7 @@
       </c>
       <c r="P150" s="0" t="inlineStr">
         <is>
-          <t>Team level analysis. Verbatim Evidence: \"Agents in creative enterprises are embedded in networks that inspire, support, and evaluate their work. Here, we investigate how the mechanisms by which creative teams self-assemble determine the structure of these collaboration networks. We pro